<commit_message>
chore: injected validation 2 batches 2-4 (47 papers)
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -3045,6 +3045,16 @@
           <t>BSMA0042</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr">
         <is>
           <t>Book chapter</t>
@@ -3068,6 +3078,11 @@
       <c r="K45" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Non-primary study; it is an encyclopedia entry providing a conceptual overview without any primary quantitative empirical data.. Verbatim Evidence: [Publication Type]. Verbatim Evidence: "[Header] &lt;Encyclopedia of international strategic management&gt;" "[Introduction] &lt;Research on boundary spanners, like other research on individuals in MNEs (see the entry expatriation), subsequently bifurcated into two distinct streams.&gt;"</t>
         </is>
       </c>
     </row>
@@ -3082,6 +3097,16 @@
           <t>BSMA0043</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr">
         <is>
           <t>A plethora of research has investigated the impact of the frontline employee on the customer, with the consensus that employees can have a tremendous impact on the customer. What remains to be discovered is the extent to which this relationship exists in the reverse. Utilizing broaden-and-build and emotional contagion theories, this study suggests that employee perceptions of a specific customer emotion (delight) have an impact on the frontline employee. Specifically, results from a structural equations model reveal that employee perceptions of customer delight lead to employee positive affect, which in turn positively influences commitment and job satisfaction as well as creates stronger external representation behaviors, internal influence behaviors, and service delivery behaviors from the employee. These findings contribute new evidence to the debate of the viability of providing customer delight and extend our knowledge beyond emotional contagion in explaining how positive customer emotions manifest in employees.</t>
@@ -3105,6 +3130,11 @@
       <c r="K46" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Study includes valid customer-oriented boundary-spanning behaviors (external representation, internal influence) at the individual employee level with an extractable correlation matrix.. Verbatim Evidence: [4.1. Research context and sample] "The final sample size was 431, including 183 respondents from Group 1, 138 from Group 2, and 110 from Group 3 of Bowen's taxonomy." [4.2. Measures] "The customer-oriented boundary-spanning behaviors were measured using three components previously employed in service research (Bettencourt &amp; Brown, 2003). External representation behaviors were measured using a three-item scale designed to capture the extent to which an employee is a vocal advocate to outsiders of the organization's image, goods, and services. Internal influence behaviors were measured with a three-item scale intended to measure the extent to which a person takes individual initiative in communicating to the firm and coworkers about ways to improve service delivery by the organization, co-workers, and oneself." [Table 2] "Means, standard deviations (SD) and correlations."</t>
         </is>
       </c>
     </row>
@@ -3119,6 +3149,16 @@
           <t>BSMA0044</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr">
         <is>
           <t>This study examines the antecedents cf job satisfaction, commitment, and turnover intentions for 229 information systems (IS) personnel employed within several industries. The antecedents studied include boundary spanning, role ambiguity, and rcle conflict. A model of these variables was built and tested using path analysis- Rcle ambiguity was found tc be the mcst dysfunctional variable for IS personnel, acccunting fcr 10.3%. 20.2% and 22.2% Of the variance in turnover intenticns. commitment, andjob satisfaction. This information is used tc make recommendaticns to IS management. Finally, recommendaticns and directions are suggested regarding future research.</t>
@@ -3142,6 +3182,11 @@
       <c r="K47" t="inlineStr">
         <is>
           <t>1985</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Valid study measuring individual-level boundary spanning activities (intra- and inter-organizational) using the Miles and Perrault scale. Zero-order correlations are provided in Table 6.. Verbatim Evidence: [Sample] "Nine companies from the New York/Boston area participated in the study, with data collected from a total of 229 individuals. The study participants included applications programmers, programmer/analysts, analysts, and project leaders in centralized IS groups." [Measures] "Boundary spanning refers to the individual's crossing of intradepartmental and interorganizational boundaries in order to perform his/her job [2, 42]." "To gather boundary spanning data a measure developed by Miles and Perrault [25] was adapted and used. The Miles and Perrault scale measures the boundary spanning activities of laboratory research and development personnel. For use in the IS personnel setting, it was necessary to generalize the questionnaire by replacing all references to the laboratory setting with non-situation-specific terminology." [Results] "Table 6. Reconstructed Correlations ... [provides Original Correlation]"</t>
         </is>
       </c>
     </row>
@@ -3156,6 +3201,16 @@
           <t>BSMA0045</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
         <is>
           <t>This article examines the evolving use of boundary objects in cross-cultural software teams. Our field study of a Jamaican-Indian team examines the use of software specifications and project management tools as boundary objects in facilitating sharing across knowledge boundaries.We examine how and why the role and use of boundary objects may facilitate collaboration across knowledge boundaries at one time and contribute to conflict at other times. We unpack the interacting elements that both facilitate and constrain knowledge sharing, and trigger conflicts at different stages of the software team development. Specifically, we found that the use of boundary objects at transitions involving definitional control and the subsequent redistribution of power/authority may inhibit knowledge sharing. The subsequent reifying of cultural boundaries along with negative stereotyping led to relational conflict, through a process we call culturizing, as cross-cultural differences emerged as problematic for team dynamics.</t>
@@ -3179,6 +3234,11 @@
       <c r="K48" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Qualitative study without extractable quantitative effect sizes. Verbatim Evidence: [Research methodology] "Case studies are the preferred research strategy for a process study when an in-depth understanding of phenomena is needed (Eisenhardt, 1989)." [Research methodology] "We conducted a two-year longitudinal case study of cross-cultural software development for a general insurance system across three phases." [Data collection and analysis] "In total, 42 interviews were conducted over three phases with a wide range of participants: senior managers of JAMSURE and its sister companies in IT, life, and general insurance company; project managers, team leaders, and developers at the IT and general insurance companies; and intended users and managers of the GENSYS system."</t>
         </is>
       </c>
     </row>
@@ -3193,6 +3253,16 @@
           <t>BSMA0046</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
           <t>This research investigated how experiences in a particular boundary-spanning context (community outreach) affected members' organizational identity and identification. Multimethod panel data from 219 participants showed that intergroup comparisons with clients (emphasizing differences) and intragroup comparisons with other organization members (emphasizing similarities) changed how members construed their organization's defining qualities. Intergroup comparisons also enhanced the esteem members derived from organizational membership, which, in turn, strengthened organizational identification. Supervisors reported higher interpersonal cooperation and work effort for members whose organizational identification became stronger. The results reveal potential outcomes of boundary-spanning work as well as how organizational identification processes operate in everyday work contexts.</t>
@@ -3216,6 +3286,11 @@
       <c r="K49" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>No effect size of interest. Measures community outreach experience (volunteering days) and social comparisons in a 'boundary-spanning context', lacking a valid measure of purposive boundary-spanning behavior.. Verbatim Evidence: [Abstract / Discussion] "This study makes a first attempt to document the psychological experiences of members who find themselves in boundary-spanning contexts by focusing on changes in organizational identification that accompany changes in contexts and social interaction partners." [Method] "To test the hypotheses, I collected data from organization members who performed community outreach for the Pillsbury Company, headquartered in Minneapolis, MN." [Method] "Four programs constitute the heart of Pillsbury's community outreach initiatives. The first program consists of business and elementary school partnerships... The second program aims to help at-risk children improve their reading skills... The third program is a partnership with a service agency that delivers midday meals... The fourth program involves an international nonprofit organization dedicated to building homes" [Measures] "Because the sample contained both novice and seasoned participants, I also controlled for prior experience in company-sponsored community outreach projects (measured as the average number of service days the previous year) to avoid potential confounds."</t>
         </is>
       </c>
     </row>
@@ -3230,6 +3305,16 @@
           <t>BSMA0047</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -3253,6 +3338,11 @@
       <c r="K50" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Multiple reasons [Code 1, Code 2, Code 4]. This is a non-empirical commentary/reply discussing disciplinary boundaries and conflicts of interest in alcohol public health science. It contains no empirical data, sample, or quantitative effect sizes.. Verbatim Evidence: [Commentary lacking empirical data]. Verbatim Evidence: "[Page 1] IN THEIR COMMENTARY in this issue of the Journal of Studies on Alcohol and Drugs, Bray and Kenkel (2024) write, “It would be unfortunate if readers came away with nothing more than a distrust of Jon Nelson’s work” (p. 428). With that, we wholeheartedly agree. The key message of our article (Bartlett &amp; McCambridge, 2024) is that boundaries between disciplines, or fields of study, are boundaries between communities of science, and we draw attention to the concept of boundary work and the nature of the work involved, the early stage of explicit normative debates about these issues in alcohol science, and the need for alcohol public health science in particular to make progress on these issues due to targeting by the alcohol industry."</t>
         </is>
       </c>
     </row>
@@ -3267,6 +3357,16 @@
           <t>BSMA0048</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
         <is>
           <t>The literature suggests that the success of innovation clusters is based on personal networks that connect members of scientific, educational, and business organizations, stimulating more formalized cross-boundary collaborations between the three sectors. But it is still unclear if such organizational collaborations actually correspond with these personal ties and which aspects of personal communication are most strongly associated with organizational collaborations. To investigate these issues, the authors applied network analysis to study an innovation cluster in Algarve, Portugal. They found that cross-boundary organizational collaborations corresponded with personal ties. Moreover, they found that collaborations appeared to correlate most strongly with emotional attachments between individuals.</t>
@@ -3290,6 +3390,11 @@
       <c r="K51" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Non-individual level (QAP network correlations at the organizational dyad level). Verbatim Evidence: [Method and Data] "The empirical study included three steps: (a) mapping and analyzing the organizational collaboration network, (b) mapping and analyzing the personal networks, and (c) analyzing the correlations between organizational collaborations and personal networks." [Network of Organizational Collaboration] "The network of organizational collaboration between science, education, and business that we examine here includes 25 nodes across the three sectors" [Networks of Personal Ties] "We aggregated the survey data by mapping each unique combination of an organizational entity and a contact’s name as a separate node." [Networks of Personal Ties] "Next, we produced three networks connecting the 25 organizations included in the analysis and representing different aspects of personal ties" [Correlations Between Networks of Personal Ties and Organizational Collaborations] "To check for correlations between organizational and personal networks in the Algarve maritime cluster, we applied the QAP correlation (Hubert &amp; Schultz, 1976) to the pairs of networks."</t>
         </is>
       </c>
     </row>
@@ -3304,6 +3409,16 @@
           <t>BSMA0049</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr">
         <is>
           <t>Customer engagement entails unequivocal frontline service employees’ top performances and recommendable behaviors through management appropriate leadership to ﬂourish. Under the social exchange and social identity theories, this study investigates employee customer–oriented boundary-spanning behaviors as an outcome of spiritual leadership, through the mediating eﬀect of employee spiritual survival and well-being. PROCESS macro was used to analyze data collected from 5-star hotels full-time frontline employees in Antalya, Turkey. Results indicated that the eﬀect of spiritual leadership on the three dimensions of customer-oriented boundary-spanning behaviors is fully mediated by spiritual survival and spiritual well-being. Spirituality appears to be a noteworthy but remote contributor to customer engagement via employees’ boundary-spanning behaviors. Our study contributed to the boundary-spanning and customer engagement literature by illustrating that a sense of mission and wellbeing at the workplace are adequate requirements to engage a frontline employee, whose boundaryspanning behaviors will be instrumental in fostering customer engagement. Further detailed theoretical and managerial implications are discussed.</t>
@@ -3327,6 +3442,11 @@
       <c r="K52" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix.. Verbatim Evidence: [Reason summary] The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix. Verbatim Evidence: "[Sampling and data collection procedure] The research team received approval from 14 hotels’ Management to collect data from their FLEs." "[Sampling and data collection procedure] At time II 309 questionnaires were redistributed, and 250 responses were used after deletion of unusable and incomplete questionnaires." "[Measures] Staffs’ COBSBs were assessed with the scale developed by Bettencourt et al. (2005) that measures service delivery with 5 items, internal influence and external representation with both 4 items." "[Results] Table 2. Intercorrelations and discriminant validity criterion."</t>
         </is>
       </c>
     </row>
@@ -3341,6 +3461,16 @@
           <t>BSMA0050</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr">
         <is>
           <t>Post financial crisis, audit committee (AC) reforms are proposed to improve the quality of financial reporting (EC 2011; Competition Commission 2013). This paper’s empirical contribution is to investigate the extent to which ACs and audit committee chairs (ACCs) engage with chief financial officers (CFOs) and audit partners (APs) across a range of 32 financial reporting issues. It is the first large-scale survey of interactions to move beyond the micro CFO / AP dyad and to distinguish the individual ACC from the AC group. While 37% of the 5,445 reported discussions involve all three key individuals together with the full AC, 35% involve neither the AC nor the ACC and the ACC acts without the full AC in a significant minority of cases. The parties reported to be involved are similar across the three respondent groups but vary with financial reporting issue, company size and audit firm size. The paper’s theoretical contribution is to interpret the evidence using the concepts of boundary spanning and gatekeeping roles. The research reveals incomplete levels of AC and ACC engagement with financial reporting issues. Findings have implications for policymakers regarding the role, influence and effectiveness of the AC in financial reporting matters. Directions for future research are identified.</t>
@@ -3364,6 +3494,11 @@
       <c r="K53" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>No correlation matrix or extractable effect sizes (descriptive survey); data analyzed at the discussion/interaction level (N=5,445 discussions) violating independence.. Verbatim Evidence: [5. RESULTS AND DISCUSSION] "Across all potential discussion issues, the combined sample reported 5,445 discussions. The parties involved in these discussions are shown in Table 5, which reports frequencies for the 15 combinations." [4. METHODS] "The present study utilises experiential questionnaires which ask expert respondents about specific events they have encountered (Gibbins and Qu 2005)."</t>
         </is>
       </c>
     </row>
@@ -3378,6 +3513,16 @@
           <t>BSMA0051</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>The proactiveness - business performance relationship was examined in this study by adopting a descriptive and crosssectional research design. Structural equation modeling was applied on a purposive sample of 457 North Indian firms to assess the impact of proactiveness on business performance. Moderating effect of environmental turbulence on proactiveness – business performance relationship was also assessed. The study found proactiveness as a significant predictor of business performance. The study revealed that firms operating in a dynamic environment were likely to be benefitted more from the pursuit of proactiveness. The findings provoke managers and entrepreneurs to adopt forwardlooking and opportunity-seeking perspectives to achieve robust business performance. Managers of Indian firms can draw insights from this study and can better decide the strategic posture of their firms.</t>
@@ -3401,6 +3546,11 @@
       <c r="K54" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Measures firm-level proactiveness, not individual BSB.. Verbatim Evidence: [Methodology] "A purposive sample of 457 North Indian organizations was taken for conducting this study. The senior - level key executives, who had decision-making power in the organization, were considered as key informants." [Appendix Table A1] "In dealing with its competitors, my firm typically initiates actions which competitors respond to." [Appendix Table A1] "My firm actively collects and evaluates information on consumer needs and preferences."</t>
         </is>
       </c>
     </row>
@@ -3415,6 +3565,16 @@
           <t>BSMA0052</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr">
         <is>
           <t>This study examined how leaders’ internal and external activities mediate the relationship of functional heterogeneity and interteam goal interdependence to team effectiveness (in-role performance and innovation) in interdisciplinary teams. The results of the structural equation model from a sample of 92 interdisciplinary teams indicate that leaders’ internal activities fully mediate the relationship of team functional heterogeneity and interteam goal interdependence to team in-role performance. The leaders’ external activities were found to fully mediate the relationship of interteam goal interdependence to team innovation. We discuss the implications of these findings for both theory and practice.</t>
@@ -3438,6 +3598,11 @@
       <c r="K55" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Valid measurement of Leader Boundary Spanning Behavior (scouting, persuading) with real employee sample and extractable correlation matrix.. Verbatim Evidence: [Sample] "Data were collected from 92 management teams from 92 public educational organizations in Israel." [Sample] "School administrators, usually the principal, typically serve as the leaders of these teams." [Measures] "external scouting (six items, for example, “How often does the leader seek information and advice from peers for the team’s benefit,” α = .89); external persuading (seven items, for example, “How often does the leader act as a representative of the team with parts of the school environment” [parents, educational ministry, district], α = .92)" [Correlation Matrix] "Table 1. Descriptive Statistics and Intercorrelation Matrix for Study Variables, N = 92."</t>
         </is>
       </c>
     </row>
@@ -3452,6 +3617,16 @@
           <t>BSMA0053</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>Membership of boundary‐spanners is controversial, as employees operate largely at the borders of the organization in close relations with customers. Nevertheless, we know little about its influence on customer satisfaction. We investigate how and when identification with the branch influences customer satisfaction. The how question is answered by showing that degree of control of one's performance mediates the impact of branch manager identification on customer satisfaction. The when question is answered by proposing two moderating variables. Locus of control regulates the extent to which identification influences performance control. Dedicated meetings between branch managers and their colleagues regulate the degree to which performance control influences customer satisfaction. Hypotheses were tested in a longitudinal design on a sample of 1,461 managers from a firm specializing in banking and financial services in Europe. Results largely confirm our hypotheses, providing a novel look on determinants of customer satisfaction from the perspective of boundary‐spanning managers.</t>
@@ -3475,6 +3650,11 @@
       <c r="K56" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>No measure of Boundary Spanning Behavior (BSB). The study surveys boundary spanners (bank managers) but only measures Branch identification, Locus of control, Performance control, and internal CS-related meetings with branch colleagues.. Verbatim Evidence: [Abstract] "Membership of boundary-spanners is controversial, as employees operate largely at the borders of the organization in close relations with customers. Nevertheless, we know little about its influence on customer satisfaction. We investigate how and when identification with the branch influences customer satisfaction." [Measures] "Branch manager identification (t1). Two items were used to measure identification with the branch (Bergami and Bagozzi, 2000)." [Measures] "CS-related meetings (t1). Two items were used to assess CS-related meetings between managers and colleagues. One item asked, ‘How many times during the last month did you discuss CS-related topics or issues with your Bank Manager?’ (i.e., the supervisor). The second one asked: ‘How many times during the last month did you discuss CS related topics or issues with your colleagues in the branch?’"</t>
         </is>
       </c>
     </row>
@@ -3489,6 +3669,16 @@
           <t>BSMA0054</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
           <t>The authors investigate three types of customer-oriented boundary-spanning behaviors (COBSBs)a frontline service employee may perform that are associated with linking a service organization to its potential or actual customers: external representation, internal influence, and service delivery. The authors propose and test a withdrawal model to explain the negative effects of role conflict and role ambiguity on COBSBs across a sample of 220 lower-level, nonprofessional service providers of a major retail bank and a sample of 90 higher-level, professional service providers from the business credit division of an international financial services corporation. The results demonstrate that (1)indirect paths through job satisfaction and organizational commitment entirely account for the negative effects of the role stressors on COBSBs, (2) the indirect negative effects of the role stressors are stronger on external representation and internal influence behaviors, and (3)role conflict also has a significant positive direct relationship with internal influence behaviors.</t>
@@ -3512,6 +3702,11 @@
       <c r="K57" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Meets all inclusion criteria. The study measures Customer-Oriented Boundary-Spanning Behaviors (COBSBs) in two samples of frontline service employees and provides zero-order latent correlations.. Verbatim Evidence: [Sample] "Retail banking. Our first sample consisted of boundary-spanning service employees of a major, multistate retail bank." [Sample] "It was possible to match 220 completed employee surveys with a manager rating of COBSBs." [Sample] "Business credit. Our second sample consisted of professional boundary-spanning service providers of the business credit division of an international financial services corporation." [Sample] "It was possible to match 90 employee surveys with a manager rating of COBSBs." [Measures] "The COBSB measures were administered to both the FSEs and their managers in each sample, and the average of these responses on an item-by-item basis was used to represent the three COBSB constructs in the hypothesis tests."</t>
         </is>
       </c>
     </row>
@@ -3526,6 +3721,16 @@
           <t>BSMA0055</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
           <t>Using a sample of 281 frontline service employees of a national retail bank, we test a social exchange model of antecedents of three dimensions of customer-oriented boundary-spanning behaviors suggested by prior boundary-spanning and services marketing/management literatures: external representation, internal inﬂuence, and service delivery. In support of our hypotheses, we identify fully mediated relationships from procedural, interactional, and distributive justice to external representation and internal inﬂuence via job satisfaction and organizational commitment. Our results generally support our expectation that the indirect effects of procedural justice on external representation and internal inﬂuence are stronger than the indirect effects of distributive or interactional justice on these behaviors. Also, our results reveal no signiﬁcant indirect effects of procedural and distributive justice on service delivery behaviors. However, we ﬁnd an unexpected direct positive path from interactional justice to service delivery behaviors. We interpret this latter ﬁnding in light of the normative value of interactional justice as a source of role modeling or managerial legitimacy.</t>
@@ -3549,6 +3754,11 @@
       <c r="K58" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>The study meets all inclusion criteria. It measures individual-level customer-oriented boundary-spanning behaviors (external representation and internal influence) among 281 frontline service employees and provides a latent correlation matrix.. Verbatim Evidence: The study meets all inclusion criteria. Verbatim Evidence: "[Conceptual background] Drawing from this research, we investigate three types of behaviors the FSE may perform that are associated with linking the organization to its potential or actual customers (cf. Bettencourt &amp; Brown 2003; Bettencourt et al. 2001): (1) external representation, being vocal advocates to outsiders of the organization’s image, goods, and services (cf. Bowen &amp; Schneider 1985), (2) internal inﬂuence, taking individual initiative in communications to the ﬁrm and co-workers to improve service delivery by the organization, co-workers, and oneself (cf. Schneider &amp; Bowen 1984; Zeithaml et al. 1988), and (3) service delivery, serving customers in a conscientious, responsive, ﬂexible, and courteous manner (cf. Parasuraman et al. 1988)." "[Sample and procedure] A sample of FSEs of a major, multi-state retail bank was used to test the hypotheses." "[Sample and procedure] In total, 656 customer service employees were surveyed across 40 branches, representing an entire region of the bank." "[Sample and procedure] Of the employee responses, it was possible to match 281 with a manager rating of COBSBs." "[Results] Table 2 reports Cronbach alpha internal consistency reliabilities, average shared variance estimates, and latent construct intercorrelations."</t>
         </is>
       </c>
     </row>
@@ -3563,6 +3773,16 @@
           <t>BSMA0056</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
           <t>Abstract                            Business Process Management is a boundary-spanning discipline that aligns operational capabilities and technology to design and manage business processes. The               Digital Transformation               has enabled human actors, information systems, and smart products to interact with each other via multiple digital channels. The emergence of this hyper-connected world greatly leverages the prospects of business processes – but also boosts their complexity to a new level. We need to discuss how the BPM discipline can find new ways for identifying, analyzing, designing, implementing, executing, and monitoring business processes. In this research note, selected transformative trends are explored and their impact on current theories and IT artifacts in the BPM discipline is discussed to stimulate transformative thinking and prospective research in this field.</t>
@@ -3586,6 +3806,11 @@
       <c r="K59" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] Conceptual research note about Business Process Management lacking primary empirical data and a measure of interpersonal BSB.. Verbatim Evidence: [Reason summary] This is a conceptual research note discussing Business Process Management as a discipline, rather than an empirical study measuring interpersonal boundary spanning behavior. Verbatim Evidence: "[Abstract] Business Process Management is a boundary-spanning discipline that aligns operational capabilities and technology to design and manage business processes." [Abstract] "In this research note, selected transformative trends are explored and their impact on current theories and IT artifacts in the BPM discipline is discussed to stimulate transformative thinking and prospective research in this field."</t>
         </is>
       </c>
     </row>
@@ -3635,6 +3860,16 @@
       <c r="B61" t="inlineStr">
         <is>
           <t>BSMA0058</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3667,6 +3902,11 @@
           <t>2011</t>
         </is>
       </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Study measures Human Capital, Social Capital, and firm structural capital rather than Boundary Spanning Behavior (Code 1), and is conducted at the inter-firm B2B relationship level where informants evaluate their supplier agency (Code 3).. Verbatim Evidence: [Reason summary] Study measures Human Capital, Social Capital, and firm structural capital rather than Boundary Spanning Behavior (Code 1), and is conducted at the inter-firm B2B relationship level where informants evaluate their supplier agency (Code 3). Verbatim Evidence: "[Abstract] Methodology /approach: The model is tested on a sample of 120 organizational buyers of advertising services by using partial last squares, a structural equation modelling technique." "[Appendix] Imagine a situation when your key contact employee in agency XYZ leaves to join another agency or to start a new agency. Based on your relationship with agency XYZ and with your contact employee, you have to make a decision whether your company would follow the contact employee to the new agency or remain as a customer in agency XYZ." "[Appendix] Agency XYZ has devoted significant resources to gain insight into our company's market situation."</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3679,6 +3919,16 @@
           <t>BSMA0059</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr">
         <is>
           <t>B ishop P. and G ripaios P. Spatial externalities, relatedness and sector employment growth in Great Britain, Regional Studies. This paper examines the impact of externalities on employment growth in sub-regions of Great Britain by estimating ordinary least-squares (OLS) and maximum likelihood spatial models at the two-digit level for 23 sectors. Issues arising from relatedness, sector differences, competition, cross-boundary spillovers, and spatial autocorrelation are explicitly addressed. Results indicate that specialization has a generally negative impact on growth, whilst the impact of diversity is heterogeneous across sectors and strong local competition has a typically positive impact. The results question the merits of policies primarily aimed at promoting regional specialization and suggest that diversity, local competition, and sector heterogeneity are important policy issues.</t>
@@ -3702,6 +3952,11 @@
       <c r="K62" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Macro-economic study analyzing aggregate employment data at the regional level (203 administrative areas) rather than individual employees.. Verbatim Evidence: [Abstract] "This paper examines the impact of externalities on employment growth in sub-regions of Great Britain by estimating ordinary least-squares (OLS) and maximum likelihood spatial models at the two-digit level for 23 sectors." [Methodology] "data for sub-regions of Great Britain at the two-digit industry level were obtained from the UK’s National On-line Manpower Information System (NOMIS) utilizing the 1992 Standard Industrial Classi-ﬁcation (SIC) classiﬁcation scheme and covering the period 1995–2002." [Methodology] "Data were collected for 203 areas at the local authority, county, and unitary authority levels. These areas are administrative units and vary from large, densely populated urban regions to smaller, rural sub-regions."</t>
         </is>
       </c>
     </row>
@@ -3716,6 +3971,16 @@
           <t>BSMA0060</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr">
         <is>
           <t>The temporal imagination is the understanding of the intersection of one entity’s timescape with the larger timescapes of which that entity is a part. We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape. We also discuss group attributes that will likely affect the development of the temporal imagination and its use and how its use in group boundary spanning efforts affect both the groups and the larger organization.</t>
@@ -3739,6 +4004,11 @@
       <c r="K63" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Conceptual book chapter with no primary quantitative data.. Verbatim Evidence: [Abstract] "The temporal imagination is the understanding of the intersection of one entity's timescape with the larger timescapes of which that entity is a part. We examine in detail what the temporal imagination is, complemented with a discussion of the related timescape idea, and why the temporal imagination is necessary to function in any timescape." [Introduction] "The entity can be an individual, a group, or an entire organization, but this chapter focuses on boundary spanning groups and their parent organizations. Several attributes of boundary spanning groups that are likely to influence the quality of the group's temporal imagination are then presented and analyzed (group diversity, shared mental models within the group, longevity, and autonomy)."</t>
         </is>
       </c>
     </row>
@@ -3753,6 +4023,16 @@
           <t>BSMA0061</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr">
         <is>
           <t>Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed “ABC” classification and “BMI-GC” concept. Highlighting BMI's role as a boundary-spanning, collaborative approach to innovation, we demonstrate its potential to drive sustainable solutions by rethinking value creation, delivery, and capture mechanisms. We examine how BMI may foster resilience and help firms and organizations adapt to global volatility, integrate ethical AI, and advance sustainability in business ecosystems. We offer a roadmap for future inquiry into BMI-GC, including measurement and assessment, digital transformation, and collaborative ecosystems. By embracing these research pathways, scholars can contribute to a deeper theoretical and practical understanding of BMI to address grand challenges.</t>
@@ -3776,6 +4056,11 @@
       <c r="K64" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Non-primary study (Editorial for a Special Section). Verbatim Evidence: [Page 1] "EDITORIAL Innovating for impact: Harnessing business model innovation to tackle grand challenges" [Abstract] "Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed “ABC” classification and “BMI-GC” concept." [Introduction] "Our objective with this Special Section is to link our improved conceptual and empirical understanding of business models with the important notion of grand challenges, the urgency of which has become increasingly apparent."</t>
         </is>
       </c>
     </row>
@@ -3790,6 +4075,16 @@
           <t>BSMA0062</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
           <t>Purpose – This study adopts a person-centered perspective to explore how entrepreneurs combine multiple proactive behavioral strategies across the business, personal and business-environment domains. We research whether certain combinations of proactive behavioral strategies (i.e. seeking resources, optimizing demands, seeking challenges, idea generation, environmental exploration, network crafting, self-insight and boundary management) relate to well-being and business performance. Moreover, we investigate whether entrepreneurs’ daily use of these strategies aligns with their general profiles.</t>
@@ -3813,6 +4108,11 @@
       <c r="K65" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Multiple reasons [Code 1 &amp; Code 2]: Sample consists of independent entrepreneurs rather than organizational employees, and no zero-order correlation matrix is provided.. Verbatim Evidence: [Methods] "Data were collected among Dutch entrepreneurs owning private companies with fewer than 250 employees (cf. Jayasekara et al., 2020). They were recruited via network organizations (e.g. FNV Zelfstandigen), magazines, LinkedIn Groups, and a database (i.e. Prolific)." [Methods] "We examined cross-sectional data from 2021–2023, with 286 entrepreneurs completing the general survey."</t>
         </is>
       </c>
     </row>
@@ -3827,6 +4127,16 @@
           <t>BSMA0063</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>Recently, work-family scholars have empirically demonstrated the importance of congruence between employees' boundary management preferences and boundary management supplies provided by the work environment in relation to employee attitudes and behavior. However, a theoretically grounded construct that captures this congruence is lacking. The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. We cross-validate the scale in three independent samples (n = 188, diverse group of employees, n = 75, employees from one hospital, and n = 81, employees from one car company) and in a fourth sample (n = 458, working parents), we demonstrated the importance of work-nonwork boundary management fit for employee well-being (i.e., stress and work-life conflict). In particular, we confirmed its unique role in predicting employee well-being, above and beyond workload and work interrupting nonwork behaviors. Hence, we argue for considering work-nonwork boundary management fit when studying how work-family policies and organizational culture affect employees in the workplace.</t>
@@ -3850,6 +4160,11 @@
       <c r="K66" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>The study focuses on work-nonwork (work-family) boundary management rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: [Abstract] The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. [Introduction] Research devoted to the interplay of work and nonwork (e.g., family and leisure) life continues to flourish, as “balancing” both roles becomes a vital concern to an increasing proportion of employees that engages in multiple roles (Kelly et al., 2008; Allen and Martin, 2017).</t>
         </is>
       </c>
     </row>
@@ -3864,6 +4179,16 @@
           <t>BSMA0064</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>Context is an important but largely ignored dimension of quality service encounters. This paper contributes to the hospitality service industries literature by examining how the front-of-house and backof-house boundary work (Nippert-Eng 1996, 2003) engaged by Room Attendants working within the hotel guest room space impact on the hospitality impression management performed. Qualitative data from fieldwork engaging with hotel employees located within the tourist resort of Queenstown New Zealand are used to explore the multiple fronts on which the front-of-house and back-of-house boundaries are simultaneously negotiated. The results suggest that Room Attendants negotiate the front-ofhouse and back-of-house boundary through objects – such as the guest room and articles belonging to the guest – and aspects of self – such as impression management, safety, socialising and self-responsibility for room checking. The results support the importance of considering context when seeking to understand the complexities associated with the (re)production of a reliably positive service encounter.</t>
@@ -3887,6 +4212,11 @@
       <c r="K67" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Qualitative study without quantitative effect sizes. Verbatim Evidence: [Qualitative study exclusion]. Verbatim Evidence: "[Abstract] Qualitative data from fieldwork engaging with hotel employees located within the tourist resort of Queenstown New Zealand are used to explore the multiple fronts on which the front-of-house and back-of-house boundaries are simultaneously negotiated." "[Procedure] Given the exploratory nature of the research agenda, the semi-structured interview was selected as the most appropriate method for collecting data." "[Analysis] The 67 transcribed interviews were read initially to select out those who worked within the Housekeeping Department."</t>
         </is>
       </c>
     </row>
@@ -3938,6 +4268,16 @@
           <t>BSMA0066</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr">
         <is>
           <t>Research has shown that NPD project leaders should engage in boundary-spanning activities. The present study tested the impact of four boundary-spanning activities on NPD project performance and analyzed the antecedents of these activities. We hypothesized that NPD project leaders' abilities to perform these activities depend on the characteristics of their personal networks — structural holes, strength of ties, vertical and horizontal bridging ties. A Partial Least Squares test on 73 NPD projects showed that (a) “obtaining political support” and “scanning for ideas” are the boundary activities with the greatest impact on performance, (b) project leaders with strong ties in their network are more effective at these activities, (c) project leaders with structural holes in their networks are more effective in another boundary activity, “protecting the team”, although this activity does not affect NPD outcomes. These results represent an important contribution to understanding how team leaders contribute to project performance.</t>
@@ -3961,6 +4301,11 @@
       <c r="K69" t="inlineStr">
         <is>
           <t>2012</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Valid measurement of individual-level boundary spanning behavior by project leaders, providing a correlation matrix.. Verbatim Evidence: [Sample] "The study was conducted on a sample of 73 project leaders in manufacturing firms" [Sample] "our final sample consisted of 73 valid questionnaires for project leaders in the manufacturing sector." [Construct] "The four boundary-spanning activity measures (coordinating with external actors, scanning for ideas and information, obtaining political support and protecting the team) were based on previous research (Ancona and Caldwell, 1992; Faraj and Yan, 2009)." [Measures] "During the project, to what extent did you manage to... Scan the environment to get information on market trends"</t>
         </is>
       </c>
     </row>
@@ -3975,6 +4320,16 @@
           <t>BSMA0067</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G70" t="inlineStr">
         <is>
           <t>Objective To evaluate feasibility and acceptability of a health professional resilience skills training program with neurology residents. Methods The curriculum consists of ﬁve 1-hour-long modules that included the following skills: reﬂective narrative practices, emotion regulation, communication with highly distressed individuals, boundary management, and the identiﬁcation of depression and trauma. Using a web-based survey tool, we administered the Brief Resilience Scale (BRS) and Abbreviated Maslach Burnout Inventory (aMBI) at baseline, in addition to a pre- and post-survey assessing change in beliefs and self-eﬃcacy, as well as satisfaction with the intervention. Means were compared using the Wilcoxon rank-sum and signed rank tests. Results Twenty-two residents representing each year of training completed the pre-survey; 41% were women. Subscale scores on the aMBI revealed that 50% had moderate or high emotional exhaustion, 41% had moderate depersonalization, and 37% had moderate or low personal accomplishment, though 77.3% reported high career satisfaction. Female residents had lower scores on the BRS (mean 3.26 vs 3.88, p &lt; 0.05), though scores on aMBI subscales did not diﬀer by sex. Scores did not diﬀer by year of training. Sixteen residents completed both the pre- and post-survey. Signiﬁcant increases were detected in 4 of 9 self-eﬃcacy statements. Seventy-one percent of residents were satisﬁed or extremely satisﬁed with the training. Conclusions Residents were satisﬁed with the curriculum and reported improved ability to identify and cope with work-related stress. Further study is needed to evaluate the inﬂuence of skills adoption and practice on resilience and burnout.</t>
@@ -3998,6 +4353,11 @@
       <c r="K70" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>The study evaluates a resilience training module on 'boundary management' (setting professional limits with patients), which is not boundary spanning behavior. It also lacks a zero-order correlation matrix.. Verbatim Evidence: [Abstract] "The curriculum consists of five 1-hour-long modules that included the following skills: reflective narrative practices, emotion regulation, communication with highly distressed individuals, boundary management, and the identification of depression and trauma." [Methods] "Boundary management: This module provided a review of why boundary management is important, encouraged residents to discuss their related skills and challenges, and instructed residents on effective techniques, including management of patients who request nonstandard care. Residents practiced these skills." [Results] "Twenty-two residents completed a pre-survey and 17 completed a post-survey."</t>
         </is>
       </c>
     </row>
@@ -4010,6 +4370,16 @@
       <c r="B71" t="inlineStr">
         <is>
           <t>BSMA0068</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4070,6 +4440,11 @@
           <t>2017</t>
         </is>
       </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Study uses Q methodology to identify subjective perspectives on leadership (including boundary-spanning leadership theory); it does not provide zero-order effect sizes between BSB and other constructs.. Verbatim Evidence: [Abstract] This study explored the perceptions of fire officers on effective organizational leadership in the American fire service to discover what is shared among varied perspectives and what is distinct, and to analyze how the perspectives align with existing leadership theories and models. It employed Q methodology, which includes both qualitative and quantitative data-collection and analysis. Ten distinct perspectives emerged from the data that have varying degrees of fit with existing theories, including (listed alphabetically) adaptive leadership theory, authentic leadership theory, boundary-spanning leadership theory, complexity leadership theory, crew resource management, leader-member exchange theory, learning organization model, the managerial grid, Mintzberg's model of management, public administrative leadership theory, regulatory focus theory, servant leadership theory, and transformational leadership. [Appendix J] Intercorrelation Matrix Between Sorts, Sorts 1 - 16</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4082,6 +4457,16 @@
           <t>BSMA0069</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
         <is>
           <t>As Thomas Friedman so persuasively argued in his book The World is Flat, 1 a significant effect of globalization is a leveling of the playing field for many of the competitors in today’s worldwide markets. Technological innovations have revolutionized the workplace, bringing the competitive power of emerging economies’ fast-growth organizations into closer alignment with their developed-world counterparts. Paradoxically, at the same time that these developments have made doing business across borders easier, relational barriers—obstacles to productive human interactions—not only remain largely unchanged but in some cases have deepened.
@@ -4108,6 +4493,11 @@
           <t>2011</t>
         </is>
       </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] Practitioner article based on a book; lacks quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [ABOUT THE RESEARCH] "This article is based on the authors’ book, Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations (McGraw-Hill, 2010)." [REFERENCES] "2. This article is primarily based on C. Ernst and D. Chrobot-Mason, “Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations” (New York: McGraw-Hill, 2010)."</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4120,6 +4510,16 @@
           <t>BSMA0070</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr">
         <is>
           <t>This dissertation examines the extent to which organizational and professional commitment, the technical environment, and the professional environment are related to boundary spanning activity. Surveys of R&amp;D professional employees, their co-workers, and their managers were used to obtain measures of commitment to their organizations and professions, perceptions of the technical and professional environment in which they worked, and the frequency with which they communicated both within and outside of the R&amp;D unit.</t>
@@ -4143,6 +4543,11 @@
       <c r="K73" t="inlineStr">
         <is>
           <t>1995</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Measures mere communication frequency rather than purposive boundary spanning behavior.. Verbatim Evidence: [Measures] "Extraunit communication frequency is the frequency of oral, work-related communication with categories of individuals outside the subject’s subunit." [Appendix V: Survey Materials] "How often have you discussed technical issues encountered in your current work over the past month, either face to face or by phone, with each person on the list?" [Appendix V: Survey Materials] "Over the past month how often have you discussed work-related issues with the following in personnel in your company?"</t>
         </is>
       </c>
     </row>
@@ -4157,6 +4562,16 @@
           <t>BSMA0071</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr">
         <is>
           <t>We study the relation between stability of the nonproﬁt organization’s environment and its board structure and the impact of this relation on organizational performance from the perspectives of both Agency Theory and Resource Dependence (Boundary Spanning) Theory. The impact of board characteristics on organizational performance is contextual. Speciﬁcally, we predict and show for a sample of U.S. nonproﬁts that board mechanisms related to monitoring are more likely to be effective for stable organizations, whereas board mechanisms related to boundary spanning are more effective for less stable organizations. We ﬁnd that the two theories are complementary and address different aspects of nonproﬁt performance, but the results are statistically stronger and more often consistent with resource dependence than with agency theory. Overall, this study supports Miller-Millesen’s (Nonproﬁt and Voluntary Sector Quarterly, 32: 521–547 2003) contention that, because the nonproﬁt environment is often more complex and heterogeneous than the for-proﬁt world, no one theory describes all tasks of nonproﬁt boards.</t>
@@ -4180,6 +4595,11 @@
       <c r="K74" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Non-individual level analysis. The unit of analysis is nonprofit organizations, and it examines board-level boundary spanning and organizational performance.. Verbatim Evidence: [Abstract] "We study the relation between stability of the nonprofit organization's environment and its board structure and the impact of this relation on organizational performance from the perspectives of both Agency Theory and Resource Dependence (Boundary Spanning) Theory." [Introduction] "This study employs a sample of operating public charities to test hypotheses suggested by both Agency Theory and Resource Dependence Theory regarding the relation between board characteristics and two different measures of organizational performance." [Sample Selection] "The sample of 123 publicly supported organizations that responded..."</t>
         </is>
       </c>
     </row>
@@ -4194,6 +4614,16 @@
           <t>BSMA0072</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
         <is>
           <t>Although network analysis is becoming a more viable and informative methodology for the study of interorganizational behavior, issues involving the accuracy and reliability of self-reported or ‘cognitive’ network data are still unresolved. Two networks based on information and coordination relationships in each of four major cities are examined. Reliability of responses is assessed as the percent of confirmed relationships between agency respondents and by correlating the extent of agreement in each network. In addition, two possible measurement errors are examined: systematic errors which are network-independent and idiosyncratic errors which are network-dependent. These errors are assessed through correlational analyses of the intensity of an organization's relationships with the number of its relationships that are confirmed in each network. Also systematic errors are accounted for by calculating the proportion of confirmed relationships within the different response categories used to judge the strength of relationship between ego organizations in the network. It is concluded that boundary spanning personnel of organizations can provide fairly reliable responses to network generated questions, but that errors in the data tend to be systematic in the way that prior studies of interpersonal cognitive networks report.</t>
@@ -4217,6 +4647,11 @@
       <c r="K75" t="inlineStr">
         <is>
           <t>1993</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>The study uses key informants as proxies to report on inter-organizational (agency-level) networks (violating Code 3) and lacks a correlation matrix with extractable individual-level effect sizes (violating Code 1).. Verbatim Evidence: [2. Data collection] "Data about the formal network of services at each site were gathered from a key informant (or 'boundary spanner') in each organization." [2. Data collection] "the interviewer oriented the respondent to the format and content of a self-administered questionnaire containing 16 questions about the relationships between the respondent's organization and each of the other organizations in the community support system." [3. Measurement] "The first asks respondents: 'To what extent does your agency receive information for coordination, control, planning, or evaluation purposes from this agency?' A second asks: 'How well coordinated are the activities of your agency with those of this other agency?'"</t>
         </is>
       </c>
     </row>
@@ -4231,6 +4666,16 @@
           <t>BSMA0073</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr">
         <is>
           <t>The offshoring of external audit work to so-called low-cost countries is prevalent among the Big 4 professional services firms. Despite this, our understanding of how this form of offshoring influences audit practitioners and the audit process is limited. This study examines how and why offshoring emerged as an organizational matter that changed the way audit work is organized in a Big 4 firm context. Our findings demonstrate how changes in the design of offshoring processes influence interactions between onshore and offshore auditors. We uncover how individual ‘‘boundary spanners’’ struggle to coordinate audit work across the multiple boundaries that separate onshore and offshore auditors. Furthermore, we show how the institutionalization of ‘‘boundary spanning’’ functions in organizational structures and processes can have the unintended consequence of widening the boundaries between onshore and offshore auditors. Finally, we offer evidence of the effect of offshoring on the learning process of onshore and offshore auditors.</t>
@@ -4254,6 +4699,11 @@
       <c r="K76" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Methodology] "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000)." [Methodology] "More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sources—documentary data, in-depth interviews, and digital data—to obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit."</t>
         </is>
       </c>
     </row>
@@ -4268,6 +4718,16 @@
           <t>BSMA0074</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr">
         <is>
           <t>Despite the relevance of team boundary spanning in new product development (NPD), there is great deal we still do not know about these activities. For example, little is known about how these activities affect the development of team identification, an important emergent state with critical implications for new product performance. This study extends our understanding of this topic by exploring the relationship between team boundary spanning and team identification. This relationship is examined via the intervening mechanisms of team potency and team boundedness and the moderating effect of intra-team communication. Data from a time-lagged survey study of 140 NPD projects revealed that team potency and team boundedness, respectively, positively and negatively mediate the relationship between team boundary spanning and team identification. Intra-team communication was found to reduce the negative effect of team boundary spanning on team boundedness.</t>
@@ -4291,6 +4751,11 @@
       <c r="K77" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Team-level analysis and key informant proxy reporting on team boundary spanning.. Verbatim Evidence: [Methodology] &lt;The data for this study were drawn from Spanish manufacturing firms in five high-technology and medium-technology sectors&gt; [Methodology] &lt;The questionnaire was addressed to the person in the company responsible for NPD activities. These individuals were instructed to answer the questionnaire in relation to a recently completed NPD project that he or she had led and for which the NPD team was engaged in boundary spanning activities.&gt; [Measurement scales] &lt;Project leader or team members talked up the NPD project to individuals or groups in the company.&gt;</t>
         </is>
       </c>
     </row>
@@ -4305,6 +4770,16 @@
           <t>BSMA0075</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr">
         <is>
           <t>In today’s highly interconnected, uncertain, and dynamic business environment, team boundary spanning has become an important determinant of the performance of new product development (NPD) projects. Despite the positive evidence supporting the use of boundary spanning activities by NPD teams, little is still known about how boundary spanning teams become high-performance teams. The current study advances research on this subject by examining the mediating effect of team potency on the relationship between team boundary spanning and new product performance, as well as the moderating effects of team size and functional diversity on the relationship between team boundary spanning and team potency. Data from a time-lagged survey study of 140 NPD projects found that team boundary spanning can promote team potency which, in turn, results in greater product quality and new product creativity. The positive effect of team boundary spanning on team potency was found to be more pronounced for NPD teams of medium size and high levels of functional diversity.</t>
@@ -4328,6 +4803,11 @@
       <c r="K78" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Non-individual level (team analysis). Verbatim Evidence: [Methodology] "The unit of analysis was a recently launched NPD project in which the NPD team in charge had partaken in boundary spanning activities." [Methodology] "Thus, the study's sample consists of 140 NPD projects, each one from a different company."</t>
         </is>
       </c>
     </row>
@@ -4342,6 +4822,16 @@
           <t>BSMA0076</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G79" t="inlineStr">
         <is>
           <t>Although team boundary spanning is conducive to achieving new product (NP) competitive advantage, these actions may not always deliver the expected performance. The current study makes an initial attempt to examine factors that undermine team boundary spanning positive effects on NP competitive advantage by proposing and testing a negative moderating effect of team social cohesion on the relationship between team boundary spanning and NP competitive advantage. Furthermore, the current study expects team social cohesion to have a stronger negative moderating effect on the relationship between team boundary spanning and NP competitive advantage when external task interdependence and project newness are high than when they are low. Data for this study come from 140 NPD projects developed and commercialized by Spanish manufacturing firms in high‐ and medium‐high‐technology sectors. The study’s results reveal a positive effect of team boundary spanning on NP competitive advantage. Furthermore, high levels of team social cohesion are shown to reduce the positive effect of team boundary spanning on NP competitive advantage. Finally, we found that project newness and external task interdependence accentuate the negative moderating effect of team social cohesion on the relationship between team boundary spanning and NP competitive advantage. The current study makes several contributions to the literature. First, findings from this study give us new insights into the significance of team boundary spanning to the success of NPs by revealing that boundary‐spanning activities are beneficial to achieving NP competitive advantage. Second, the study departs from existing research in that it exposes a dark side of team social cohesion for NPD teams engaged in boundary spanning activities. Last, the study expands extant research by proposing and demonstrating that project newness and external task interdependence bring about situations in which external groups present a threat to the collective identity of socially cohesive groups.</t>
@@ -4365,6 +4855,11 @@
       <c r="K79" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=140 NPD projects/teams). Verbatim Evidence: [Abstract] "Data for this study come from 140 NPD projects developed and commercialized by Spanish manufacturing firms in high- and medium-high-technology sectors." [Sample and Data Collection] "Respondents were instructed to answer the survey questions with regard to a recently completed NPD project that they had led or managed." [Table 2] "I_AMB1: Project leader or team members talked up the NPD project to individuals or groups in the company."</t>
         </is>
       </c>
     </row>
@@ -4379,6 +4874,16 @@
           <t>BSMA0077</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr">
         <is>
           <t>Gender diversity pays off, particularly at senior levels in organizations. Companies with higher rates of gender diversity among senior leaders outperform their peers by a 15% margin; those with the highest percentages of female board directors enjoy as much as a two-thirds higher return on equity, sales, and invested capital. The key to occupying a high-level position in any organization is building an effective network of positive workplace relationships. Decades of research on organizational networks have shown that who you know–and who knows you–is critical to performance and career success. Full inclusion of both genders in informal organizational networks has been shown to drive productivity, innovation, and profitability. Full inclusion also supports individual well-being and deep engagement. Yet many leaders–both men and women–fail to develop gender-inclusive networks, potentially disadvantaging women since they are less likely to be connected to people in senior-level positions, given the overwhelming dominance of men in these roles. No wonder that feeling excluded from organizational networks has been identified as one of women’s top barriers to career success.</t>
@@ -4402,6 +4907,11 @@
       <c r="K80" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Practitioner/qualitative summary lacking formal correlation matrices or extractable quantitative effect sizes.. Verbatim Evidence: [Methodology] "We were privileged to have access to network data collected from more than 30 organizations and 16,500 people over 15 years across a range of industries. To supplement our quantitative analyses, we also conducted 125 interviews with individuals at different levels in their organizations and in different positions in networks." [Methodology] "These data were organized into matrices and analyzed statistically. To complement our quantitative findings, we also interviewed 125 individuals in these organizations. These semi-structured hour-long interviews included open-ended questions... Transcripts were analyzed to identify themes, patterns, and examples."</t>
         </is>
       </c>
     </row>
@@ -4416,6 +4926,16 @@
           <t>BSMA0078</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr">
         <is>
           <t>Abstract             The defense industry in Israel has long been considered a critical platform for the development of the high‐technology sector. This study examines the importance of knowledge combination capability work units build through social relationships to enhance their performance. Specifically, we probe how both intraunit relational capital (within a unit) and interunit relational capital (across units) enable units to build knowledge combination capabilities and how such capabilities affect their performance. Data collected from senior managers in 122 knowledge units indicate that: (1) both intra‐ and interunit relational capital are positively related to knowledge combination capability; (2) knowledge combination capability is positively associated with enhanced unit performance; (3) knowledge combination capability fully mediates the relationship between interunit relational capital and unit performance; and (4) intraunit relational capital impacts both directly and indirectly (through knowledge combination capability) on unit performance. The findings suggest that interunit relational capital entails greater variation in knowledge stocks and thus may lead to more radical innovation than intra‐relational capital that entails more similar knowledge bases and, thus, produces more incremental innovations. Copyright © 2009 Strategic Management Society.</t>
@@ -4439,6 +4959,11 @@
       <c r="K81" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Sample and data collection] "Overall, we received usable data from 244 respondents in 122 units, yielding a response rate of 76.7 percent." [Measures] "In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit." [Level of analysis] "We performed three tests to determine whether the data should be aggregated to the unit level (see Table 1)." [RESULTS] "Table 2. Means, standard deviations, and Pearson’s correlations between research variables... N = 122"</t>
         </is>
       </c>
     </row>
@@ -4453,6 +4978,16 @@
           <t>BSMA0079</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G82" t="inlineStr">
         <is>
           <t>This study examines the relationships between joint work commitments, job satisfaction, and job performance of lawyers employed by private law firms in Israel. Based on Morrow’s (1993) concept of five universal forms of commitment, their interrelationship was tested with respect to the commitment model of Randall and Cote (1991), which appeared to show in previous studies (Cohen, 1999, 2000) a better fit compared to other models. In addition, the study examined the relationship between the commitment model and work attitude and outcome, namely, job satisfaction and job performance. The results show that the commitment model of Randall and Cote was almost fully supported, except for the relationship between job involvement and continuance commitment. This relationship is better understood via career commitment. An interesting finding of this study is that job satisfaction has a mediating role in the relationship between joint work commitment and job performance. The article concludes with suggestions regarding further investigation of the interrelationships between work commitment constructs, and the relationship between joint commitment forms, job satisfaction, and job performance.</t>
@@ -4476,6 +5011,11 @@
       <c r="K82" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>No boundary spanning behavior construct measured. The study measures work commitment forms, job satisfaction, and job performance.. Verbatim Evidence: [Abstract] "This study examines the relationships between joint work commitments, job satisfaction, and job performance of lawyers employed by private law firms in Israel." [The Conceptual Framework] "The model investigates the relationships between five forms of work commitment, job satisfaction and job performance."</t>
         </is>
       </c>
     </row>
@@ -4490,6 +5030,16 @@
           <t>BSMA0080</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr">
         <is>
           <t>This study analyzes the complex set of relationships among perceived organizational reputation, ﬁrm’s quality of products/services, customers’ satisfaction and multiple performance measures. A path analysis shows that reputation is inﬂuenced by customers’ satisfaction, which is a mediator in the relationship between the ﬁrm’s quality of products/services and reputation. Reputation is associated with the ﬁrm’s growth and accumulation of customers’ orders, but is not directly associated with market share, proﬁtability and ﬁnancial strength. Market share inﬂuences a ﬁrm’s profitability and is a function of the ﬁrm’s growth and accumulation of customers’ orders, but it has no inﬂuence on the ﬁrm’s ﬁnancial strength.</t>
@@ -4513,6 +5063,11 @@
       <c r="K83" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Multiple reasons [Code 1 &amp; Code 3]: The study does not measure boundary spanning behavior, focusing instead on organizational reputation and product quality, and the unit of analysis is the firm (N=86 industrial enterprises) with the CEO acting as a key informant.. Verbatim Evidence: [Participants and Data Collection] "The data used in this study were taken from a comprehensive research project that evaluated organizational competencies (organizational communication, organizational culture, internal control and others) of Kibbutz-owned industrial enterprises." [Participants and Data Collection] "A questionnaire to the enterprise’s CEO was mailed from and returned to a university address, using a self-addressed reply envelope." [Participants and Data Collection] "Due to missing data, only 86 questionnaires were usable for this study." [Measures] "The study analyzed the relations between measures of quality of products/services, customers’ satisfaction, perceived organizational reputation and performance measures of the industrial enterprises in the sample."</t>
         </is>
       </c>
     </row>
@@ -4527,6 +5082,16 @@
           <t>BSMA0081</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G84" t="inlineStr">
         <is>
           <t>Research on team leadership has primarily focused on leadership processes targeted within teams, in support of team objectives. Yet, teams are open systems that interact with other teams to achieve proximal as well as distal goals. This review clariﬁes that deﬁning ‘what’ constitutes functionally eﬀective leadership in interteam contexts requires greater precision with regard to where (within teams, across teams) and why (team goals, system goals) leadership processes are enacted, as well as greater consideration of when and among whom leadership processes arise. We begin by synthesizing ﬁndings from empirical studies published over the past 30 years that shed light on questions of what, where, why, when, and who related to interteam leadership and end by providing three overarching recommendations for how research should proceed in order to provide a more comprehensive picture of leadership in interteam contexts.</t>
@@ -4550,6 +5115,11 @@
       <c r="K84" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] Non-primary study (Literature review) lacking primary quantitative effect sizes.. Verbatim Evidence: [Abstract] "This review clarifies that defining ‘what’ constitutes functionally effective leadership in interteam contexts requires greater precision with regard to where (within teams, across teams) and why (team goals, system goals) leadership processes are enacted, as well as greater consideration of when and among whom leadership processes arise." [Review approach] "The purpose of this review is to clarify the nature of functional leadership in interteam contexts, integrate and critically evaluate relevant findings from prior research, and identify promising areas for future inquiry." [Review approach] "In the final step of our process, the full text of each article was reviewed carefully by the authorship team to confirm its relevance to this review based on the inclusion criteria described previously. This vetting process resulted in a smaller subset of 160 articles."</t>
         </is>
       </c>
     </row>
@@ -4564,6 +5134,16 @@
           <t>BSMA0082</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G85" t="inlineStr">
         <is>
           <t>Even though empirical studies examining leadership and effectiveness in multiteam systems (MTS) are on the rise, there is still much to learn about leading a complex “team of teams,” particularly in a field setting as opposed to a laboratory simulation. This study draws upon the multiteam systems and intergroup leadership theory literature streams to examine the role of systems thinking and leader identification as antecedents to intergroup leadership, arguing that higher levels of systems thinking and stronger leader identification with the MTS will enhance the efficacy of leader rhetoric targeted toward the development of an intergroup relational identity with boundary spanning acting as a positive moderating influence on this relationship. I further argue team functional diversity moderates the relationship between intergroup leadership and MTS effectiveness such that higher levels of intergroup leadership are needed to positively influence MTSs with higher levels of heterogeneity. Finally, team identification is evaluated for its predicted moderating effect on the relationship between intergroup leadership and MTS effectiveness such that identification with the MTS will have a positive effect on this relationship while identification with the component team will detract from it. Hypotheses were tested but not supported using a sample of 256 commanders at the squadron, group, and wing level organized in 180 MTSs within the Department of the Air Force. Supplemental analysis identified a significant positive moderating effect of systems thinking and a negative moderating effect of leader component team identification on the relationship between leader rhetoric and intergroup relational identity. Low levels of boundary spanning coupled with higher levels of intergroup relational identity resulted in lower MTS effectiveness while the opposite was true for high levels of boundary spanning and intergroup relational identity. The study concludes with a discussion of theoretical and practical implications as well as recommendations for future research.</t>
@@ -4587,6 +5167,11 @@
       <c r="K85" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Included. The study examines individual-level boundary spanning among Air Force commanders and provides an extractable zero-order correlation matrix.. Verbatim Evidence: [Sample] "The final survey contact list included 18,713 Department of the Air Force individuals who, as of 31 May 2020: 1) occupied active-duty numbered flight, squadron, group, and wing commander positions; 2) supervised wing or direct-report group commanders as a NAF/Center-level commander or higher; or 3) were supervised by the probable commander of a unit." [Individual Level] "The study population of 256 cases thus had 100% participation in the survey and both the supervisor and subordinates assessed the commander’s unit on MTS effectiveness and the commander on leader rhetoric and intergroup relational identity, respectively." [BSB Measure] "Boundary Spanning. Boundary spanning was measured as a self-assessment using the 4-item empirically validated scale developed by Faraj and Yan (2009) adapted from a team focus to an individual assessment and modified for an Air Force setting. For example, the item “To what extent does the team encourage its members to solicit information and resources from elsewhere in and/or beyond the division?” was modified to read “To what extent do I solicit information and resources from elsewhere in and/or beyond my unit?”"</t>
         </is>
       </c>
     </row>
@@ -4601,6 +5186,16 @@
           <t>BSMA0083</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr">
         <is>
           <t>This study investigates the relationship between multiple role management strategies and knowledge spillovers across roles. We focus on a particular category of boundary-spanning professionals, the scholar-practitioners—professionals who work across the boundaries of academic and practice worlds—and apply a role theory lens to study (a) the sources of interrole conflict they experience at role boundaries, (b) the strategies of multiple role management they enact, and (c) the knowledge spillovers associated to such strategies. We develop a grounded model that describes three role management strategies, which occupy different positions on a role separation–integration continuum, and generate different mechanisms of knowledge spillover. Our study sheds light on the understudied relationship between role management strategies and knowledge consequences, and the type of tensions individuals experience in this process. In addition, we discuss how the strategic management of teaching, research, and practical application roles can help bridge academic and managerial practice worlds.</t>
@@ -4624,6 +5219,11 @@
       <c r="K86" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Qualitative study (grounded theory) lacking quantitative effect sizes.. Verbatim Evidence: [Method] "For this purpose, we conducted a qualitative study of experienced scholar-practitioners and developed a grounded model about the strategies that scholar-practitioners use to deal with multiple role conflicts." [Data Collection] "The final sample consists of 16 scholar-practitioners ranging from 10 to 50 years of practical experience (see Table 1)." [Data Analysis] "We performed data analysis using the consolidated theory of Strauss and Corbin (1990) to develop a grounded model of how scholar-practitioners manage multiple professional roles."</t>
         </is>
       </c>
     </row>
@@ -4638,6 +5238,16 @@
           <t>BSMA0084</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr">
         <is>
           <t>Since the collapse of the price of crude oil in the mid 1980s, some participants in the sector have overhauled their approach to learning for strategic advantage. The management teams dealing with the projects discussed here demonstrated an awareness that learning can be a core rigidity as well as a core competence, and set about institutionalizing new learning. The speed of learning was an important determinant of success, leading to substantial increases in project NPVs and a rapid reinvestment in the learning capabilities themselves. Learning about `boundary management' helps to distinguish areas where internal learning could develop proprietary competitive advantage, from those areas where valuable learning might best be achieved through alliance.</t>
@@ -4661,6 +5271,11 @@
       <c r="K87" t="inlineStr">
         <is>
           <t>1999</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [Background to the Case Studies] "The study reported on here was based primarily on a series of interviews with senior management of three offshore oil fields in the UK Continental Shelf. In all cases the operator of the fields was BP, although interviews were also conducted with BP's partners, allies, and suppliers."</t>
         </is>
       </c>
     </row>
@@ -4712,6 +5327,16 @@
           <t>BSMA0086</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G89" t="inlineStr">
         <is>
           <t>The identification and management of work dependencies is a fundamental challenge in software development organizations. This paper argues that modularization, the traditional technique intended to reduce interdependencies among components of a system, has serious limitations in the context of software development. We build on the idea of congruence, proposed in our prior work, to examine the relationship between the structure of technical and work dependencies and the impact of dependencies on software development productivity. Our empirical evaluation of the congruence framework showed that when developers’ coordination patterns are congruent with their coordination needs, the resolution time of modification requests was significantly reduced. Furthermore, our analysis highlights the importance of identifying the “right” set of technical dependencies that drive the coordination requirements among software developers. Call and data dependencies appear to have far less impact than logical dependencies.</t>
@@ -4735,6 +5360,11 @@
       <c r="K89" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>No BSB measured and unit of analysis is modification requests (tasks), not individuals [Code 1 &amp; Code 3].. Verbatim Evidence: [Method] "The unit of analysis is the modification request which corresponds to a development work item associated with a defect or a new feature. A total of 2375 multi-team modification requests were identified." [Measures] "Congruence Measures: The data for building the Coordination Requirements matrix (equation 1) was extracted from several data sources such as the modification request reports, the version control system as well as the software code itself." [Results] "Table 1: Effects on Resolution Time (FCT method) ... N 2375"</t>
         </is>
       </c>
     </row>
@@ -4749,6 +5379,16 @@
           <t>BSMA0087</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
           <t>Prior research on the impact of organizational memory on new product success has divergent perspectives. Such inconsistency has accrued mainly from not considering memory's multifaceted aspects, which interact with specific project characteristics. This paper tries to sort out this paradox by proposing that project innovativeness moderates the relationship among variables of organizational memory and new product success. An empirical study of 169 NPD projects of Korean manufacturing firms finds that memory sharing and the use of external information and formal procedures enhance new product success, whereas organizational memory has no effect. Project innovativeness is found to moderate memory's effect, despite some tradeoffs. As innovativeness increases, the effect of organizational memory and use of external information become stronger whereas the effect of memory sharing and use of formal procedures weaken. This suggests that firms must activate organizational memory more carefully according to project characteristics and the memory level to maximize its positive effects.</t>
@@ -4772,6 +5412,11 @@
       <c r="K90" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Team/Project level analysis (N=169 NPD projects) with key informant rating the team. Verbatim Evidence: [4.2. Sample] "The finalized questionnaires were administered to key informants in major Korean manufacturing firms who had recent experience with participating in NPD projects as project leaders or members. In the end, 169 usable questionnaires were obtained on which we empirically test our model." [Appendix A. Measures] "During the project, project team -Regularly discussed with customers -Systematically acquired external technological and market information -Consulted regularly outside experts -Conducted systematic benchmarking"</t>
         </is>
       </c>
     </row>
@@ -4786,6 +5431,16 @@
           <t>BSMA0088</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G91" t="inlineStr">
         <is>
           <t>This study investigates how post-M&amp;A interdepartmental integration affects the efficiency and effectiveness of new product development (NPD).The total sample size was 251 respondents. Confirmatory factor analysis (CFA) and structural equation modeling (SEM) were used for statistical analysis. Analytical results indicate that, although collaboration interdepartmental integration positively correlates with product vision, interaction interdepartmental interaction integration does not reach a significant level. Despite the fact that some interaction is essential when developing new product competitive advantage (NPCA), such interaction does not necessarily achieve success. Further, product vision positively correlates with new product competitive advantage and NPD performance, and new product competitive advantage positively correlates with NPD performance. In addition, an examination of the mediation effect in terms of Sobel t-test reveals that product vision is a significant mediator for the influence of interdepartmental integration on new product competitive advantage, while the new product competitive advantage is also a significant mediator for the influence of interdepartmental integration on NPD performance. Moreover, this study provides a framework for managing post-M&amp;A integration and closes with a discussion of the theoretical and practical implications of the research findings.</t>
@@ -4809,6 +5464,11 @@
       <c r="K91" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Non-individual level of analysis (Proxy Guardrail). Respondents act as key informants to evaluate interdepartmental integration at the department/program level.. Verbatim Evidence: [Section 3.1.2] "This study used program level as a basis for evaluating NPD performance, and analyzed the 251 returned questionnaires on M&amp;A." [Appendix A] "For the team members involved in post-M&amp;A interdepartmental integration, the purpose of the questions listed below is to estimate the level of understanding what degree did your department interact with other department in regards to the below activities." [Appendix A] "Respondents were asked to assess the degree to which their department and other departments achieved collective goals, had mutual understanding, informally worked together, shared the same company vision, and shared ideas, information, and/or resources."</t>
         </is>
       </c>
     </row>
@@ -4823,6 +5483,16 @@
           <t>BSMA0089</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
           <t>Digital transformation accelerates the boundary reshaping of firms’ R&amp;D cooperation and knowledge bases, bringing opportunities for breakthrough innovation following overseas mergers and acquisitions (M&amp;A). Unlike previous studies that have focused separately on digital transformation and overseas M&amp;A integration, this paper aims to explore their synergy effects on firms’ breakthrough innovation from a boundary-spanning perspective. Based on samples of Chinese manufacturing firms’ technology-sourcing overseas M&amp;A from 2012 to 2019, our empirical results show that boundary spanning in R&amp;D cooperation networks and knowledge networks mediate the synergy effects of digital transformation and appropriate overseas M&amp;A integration on firms’ breakthrough innovation. This paper not only complements recent studies that combine digital transformation and boundary-spanning theories, but also provides a deeper understanding of the relationship between boundary spanning and breakthrough innovation in the digital context. It offers important theoretical and practical insights into overseas M&amp;A and innovation in the digital era.</t>
@@ -4846,6 +5516,11 @@
       <c r="K92" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] Archival firm-level data on M&amp;A, alliances, and patents without individual employee surveys.. Verbatim Evidence: [Method] "From the Bvd-Orbis M&amp;A database, we selected samples of Chinese manufacturing firms’ overseas M&amp;A by considering multiple criteria. (1) The acquirer holds more than 50% of the shares. (2) The M&amp;A transactions occurred between January 2012 and December 2019." [Method] "We ultimately selected 146 firms." [Dependent variable] "Breakthrough innovation (BI). We relied on two patent-based measures to capture breakthrough innovation. The data was obtained from the Incopat patent database." [Mediating variables] "Boundary spanning in R&amp;D cooperation networks (BSCN). We employed a snowball method to collect R&amp;D cooperation, alliance, and joint patent application information of the acquirer, the target firm, and firms that had those relationships with the merging parties three years before and after the M&amp;A. These data came from the SDC alliance database, corporate annual reports, Lexis–Nexis database, and Incopat database."</t>
         </is>
       </c>
     </row>
@@ -4860,6 +5535,16 @@
           <t>BSMA0090</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr">
         <is>
           <t>In the face of increasing global uncertainty, multinational enterprises (MNEs) have turned to downsizing to maintain profitability while emphasizing lateral collaboration to increase productivity. Here, we establish a conceptual framework and examine from a macro‐to‐micro perspective how the growing subjects of subsidiary role change, team alignment and employee engagement impact lateral collaboration. We used structural equation modelling to analyse the results of 252 surveys given to MNE subsidiaries in the Taiwanese banking industry and found that employee engagement was central to driving lateral collaboration effectiveness, indicating that the subsidiary role is critical for boundary‐spanning activities and building bridges between various teams. These activities in turn enhance subsidiary performance and lead to better people development. Our findings demonstrate that bundling employee engagement with human resource practices is a strategic way of positioning for the evolution of subsidiary management.</t>
@@ -4883,6 +5568,11 @@
       <c r="K93" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Excluded under Code 1 as the study measures lateral collaboration effectiveness via normative and affective commitment, and team alignment via formal/informal structural coordination, rather than individual purposive boundary-spanning behavior.. Verbatim Evidence: [Sample] "The data for our study was garnered from MNE subsidiaries in the Taiwanese banking industry including Citibank, HSBC, Standard Chartered Bank, DBS and ANZ... We e-mailed a 5-point Likert scale questionnaire to 650 employees with the title of Manager and above to these five selected international banks... we ended up with 252 valid responses" [Constructs] "Our study examines how the antecedents of lateral collaboration, subsidiary role change, team alignment and employee engagement, can gauge the health of an organization... It also exploits the consequent relationship between lateral collaboration effectiveness, subsidiary performance and people development." [Measurement 1] "We therefore consider the exercise of commitment as a form of lateral collaboration that can be enhanced to achieve the expected people development and subsidiary performance." [Measurement 2] "L21 You trust other colleagues know their works and can play their roles. L22 You feel collective ownership is our responsibility." [Measurement 3] "A21 You are requested to participate the conference call with RHQ or HQ periodically. A22 HQ or RHQ will visit your subsidiary regularly."</t>
         </is>
       </c>
     </row>
@@ -4897,6 +5587,16 @@
           <t>BSMA0091</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G94" t="inlineStr">
         <is>
           <t>This paper investigates the impact of boundary-spanning search on innovation performance, with knowledge recombination as the underlying mechanism. It also explores the contingent eﬀect of in house training of employees by considering not invented here syndrome derived from attitude theory, and examines communication investment as a second-order moderator. We test the hypotheses based on a sample of 184 Hong Kong manufacturing ﬁrms. The results show that boundary-spanning search is positively related to innovation performance, which is negatively moderated by in house training of employees. Moreover, communication investment has a suppressing eﬀect on the moderating role of in house training of employees. This paper highlights the not invented here syndrome and its mechanism of attitude theory to examine the contingent eﬀects, providing insights for managers to balance among in house training of employees, communication investment, and boundary-spanning search to enhance innovation performance.</t>
@@ -4920,6 +5620,11 @@
       <c r="K94" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Firm-level analysis with manager acting as a proxy informant for the organization. Verbatim Evidence: [Methodology] To select the appropriate samples, we adopted four criteria. Firstly, the firms should be in good operating condition and have innovation output over a period of time. Secondly, considering the innovation cycle, the firms should be established for at least one year. ... And the respondents were firm managers. [Measures] boundary-spanning search was measured by five items: “In our firm, we search for knowledge disclosed from patent gazette”, “In our firm, we search for knowledge from technology licensing”, “In our firm, we search for knowledge from research institutions, universities or colleges”, “In our firm, we search for knowledge from industry exhibitions”, “In our firm, we search for knowledge from technical publications and technical conferences”.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -3825,6 +3825,16 @@
           <t>BSMA0057</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr">
         <is>
           <t>When the ordering function is governed by administrative arrangements and sales are regulated by long-term contracts, managers may question the necessity and the tasks of the sales function within established customer relationships. The authors examine three issues related to the role of the salesperson in established industrial buyer-seller relationships: (1) appropriate measures of salesperson performance within a relationship, (2) behaviors and skills affecting salesperson performance, and (3) the effect of salesperson performance on the relationship. The results from a survey of industrial buyers suggest that the salesperson has a significant and substantial effect on relationship continuity. They also show that the salesperson contributes to perceptions of the supplier's reliability and supplier services. The key attributes of an effective salesperson are ability to resolve conflicts, ability to develop a personal relationship with customers, and ability to facilitate exchange of information between the supplier and buyer firms.</t>
@@ -3848,6 +3858,11 @@
       <c r="K60" t="inlineStr">
         <is>
           <t>1997</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Relationship-level analysis (Dyadic data). Verbatim Evidence: [METHODS] "The data used to test the hypotheses were collected in a mail survey of industrial buyers." [METHODS] "This procedure produced completed questionnaires from 126 companies (a response rate of 22%)." [METHODS] "A total sample of 279 relationships was collected. Thus, on average each informant evaluated about two relationships."</t>
         </is>
       </c>
     </row>
@@ -4231,6 +4246,16 @@
           <t>BSMA0065</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr">
         <is>
           <t>This research examined the relationships between structural positions and influence at the individual level of analysis. The structure of the organization was conceptualized from a social network perspective. Measures of the relative positions of employees within workflow, communication, and friendship networks were strongly related to perceptions of influence by both supervisors and non-supervisors and to promotions to the supervisory level. Measures included criticality, transaction alternatives, and centrality (access and control) in the networks and in such reference groups as the dominant coalition. A comparison of boundary-spanning and technical-core personnel indicated that contacts beyond the normal work requirements are particularly important for technical core personnel to acquire influence. Overall, the results provide support for a structural perspective on intraorganizational influence.</t>
@@ -4254,6 +4279,11 @@
       <c r="K68" t="inlineStr">
         <is>
           <t>1984</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Included as valid intra-organizational BSB per Rule 17 and Rule 18.. Verbatim Evidence: [Participants] "One hundred forty (87.5 percent response rate) full-time, nonsupervisory employees completed a questionnaire administered by the researcher." [Measures] "Contacts beyond the workflow. Separate measures of contacts with others were calculated for the communication network and friendship network. This was done by counting the number of direct relationships between a focal person and persons who were not members of the focal person's immediate workgroup nor persons with whom the focal person was required to interact in performing normal work functions." [Results] "Table 2 presents the zero-order correlations between each of the structural measures and the influence measures."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected straggler results
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -5320,6 +5320,16 @@
           <t>BSMA0085</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr">
         <is>
           <t>Adopting a microfoundations approach to the analysis of intra-multinational enterprise (MNE) knowledge integration, we focus on mobile inventors and their boundary-spanning experience. Using inventor-patent data on US-based MNEs, we show that intra-organizational cross-border mobility and inter-organizational mobility have respectively a positive and a negative effect on knowledge integration. Cross-border mobility within the MNE enables the temporary co-location of mobile inventors in different units, facilitating the dissemination of their knowledge within the MNE. Conversely, “job-hopping” inventors may remain organizational outsiders, which hinders their ability to foster intra-MNE knowledge integration.</t>
@@ -5343,6 +5353,11 @@
       <c r="K88" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] Uses secondary patent/inventor data (bibliometrics) instead of primary employee surveys, and analyzes knowledge integration at the firm/patent level.. Verbatim Evidence: [Title] "Knowledge integration in multinational enterprises: The role of inventors crossing national and organizational boundaries"</t>
         </is>
       </c>
     </row>
@@ -8643,6 +8658,12 @@
           <t>BSMA0172</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>The digital era is radically changing our societies and how ﬁrms do business. Innovating the business model has become a fundamental capability to survive competition, particularly for small and mediumsized enterprises (SMEs). This study investigates the digital-era role of boundary management capabilities in the processes of Business Model Innovation (BMI) in SMEs. Structural Equation Modelling is adopted to analyse data from a survey of 250 Italian experts who possess direct research and consulting experience with SMEs. Our ﬁndings reveal that digitalisation and ﬁrms’ boundaries aﬀect BMI in SMEs. Moreover, our results demonstrate how boundary management, speciﬁcally its technological and relational aspects, directly impacts BMI and mediates the relationship between boundary size and BMI. The study also oﬀers important theoretical and practical insights, calling on scholars and managers to give more attention to the boundary management of SMEs in order to support BMI.</t>
@@ -8666,6 +8687,11 @@
       <c r="K175" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8680,6 +8706,12 @@
           <t>BSMA0173</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>This study investigated how a project group deals with the contradiction between distributed knowledge in boundary-spanning collaborative processes and the expectation that software systems will provide unified, codified knowledge. It employed an ethnographic, interpretive approach to examine the ways in which relevant knowledge was presented, recognized, shared or otherwise managed during a project concerned with the joint design of business process and IT systems change. Developing a group understanding of how to manage sensemaking and expertise across salient knowledge boundaries were discovered to be central to perceptions of project completion. Four stages of this development were identified. The contribution of this paper is to propose these stages as the basis for boundary-spanning group management approaches and to suggest ways of progressing the complexities of communication, consensus-building, information exchange, problem-formulation and solution-brokering that are fundamental to collaboration in IS definition. These processes are normally taken for granted, rationalized or ignored by managers of IT-related organizational change. The use of specific types of boundary-object may aid in managing such processes explicitly and ensuring rapid progress. Thus the findings have significant implications for research and practice in other forms of boundary-spanning group collaboration, such as organizational innovation and problem-solving.</t>
@@ -8703,6 +8735,11 @@
       <c r="K176" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8717,6 +8754,12 @@
           <t>BSMA0174</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>Research Summary: This paper builds theoretical arguments and shows empirical evidence of the direct benefits and indirect costs of corporate volunteering in developing countries. Spanning corporate and humanitarian sectors to work in challenging environments should activate motivational and learning benefits for participating employees. However, results from a field study of a 10-year partnership between logistics provider TNT and the United Nations World Food Program show that such boundary-spanning corporate social responsibility (CSR) can be a double-edged sword. Task interdependence with nonprofit peers while volunteering strengthens employees' partnership identification and institutional learning. However, institutional learning triggers identity strain (associated with attrition) when they return, unless firms foster a sense that they recognize CSR experiences as valuable. The findings inform the behavioral and microfoundations of the potential consequences of CSR.</t>
@@ -8740,6 +8783,11 @@
       <c r="K177" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8754,6 +8802,12 @@
           <t>BSMA0175</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>In this study we examine the impact of market orientation of leaders on their leader-member exchange (IMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the exist five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.</t>
@@ -8777,6 +8831,11 @@
       <c r="K178" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8791,6 +8850,12 @@
           <t>BSMA0176</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>We examine the extent to which executives' boundary spanning relations inside and outside their industry affect organizational strategy and performance. We posit that the informational and social influences of external ties will be reflected in the degree to which the organization's strategy conforms to or deviates from the central tendencies of its industry and that the alignment of executives' external ties with the firm's strategy will be beneficial to firm performance. Using a multiyear sample of firms in the branded foods and computer industries, we find that executives' intraindustry ties are related to strategic conformity, that extraindustry ties are associated with the adoption of deviant strategies, and that alignment of executives' external ties with the informational requirements of the firm's strategy enhances organizational performance. Our results also show that a unique or differentiated strategy is not universally advantageous and that the benefits accruing from strategic conformity are especially strong in the more uncertain computer industry.</t>
@@ -8814,6 +8879,11 @@
       <c r="K179" t="inlineStr">
         <is>
           <t>1997</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8828,6 +8898,12 @@
           <t>BSMA0177</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>The relationship between external communication and R&amp;D team creativity has received increasing attention in the R&amp;D management literature. However, little is known about the motivational mechanism between the two. We propose a second‐stage moderation model based on social cognitive theory to explain whether, how and when R&amp;D team’s external developmental feedback motivates its creativity. Using the data gathered from 452 R&amp;D team members and 84 supervisors in a time‐lagged field study, we found external developmental feedback had a positive effect on R&amp;D team creativity via increasing team creative efficacy. Further, conditional indirect effect analyses found that a high level of cooperative goal interdependence strengthened the positive effect of team creative efficacy on R&amp;D team creativity and the mediating effect of team creative efficacy between external developmental feedback and R&amp;D team creativity.</t>
@@ -8851,6 +8927,11 @@
       <c r="K180" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8865,6 +8946,12 @@
           <t>BSMA0178</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -8888,6 +8975,11 @@
       <c r="K181" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8902,6 +8994,12 @@
           <t>BSMA0179</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -8925,6 +9023,11 @@
       <c r="K182" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -8976,6 +9079,12 @@
           <t>BSMA0181</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>Aim: To identify learning from a clinical microsystems (CMS) quality improvement initiative to develop a more integrated service across a falls care pathway spanning community and hospital services. Background: Falls present a major challenge to healthcare providers internationally as populations age. A review of the falls care pathway in Sheffield, United Kingdom, identified that pathway implementation was constrained by inconsistent coordination and integration at the hospital–community interface. Approach: The initiative utilised the CMS quality improvement approach and comprised three phases. Phase 1 focussed on developing a climate for change through engaging stakeholders across the existing pathway and coaching frontline teams operating as microsystems in quality improvement. Phase 2 involved initiating change by working at the mesosystem level to identify priorities for improvement and undertake tests of change. Phase 3 engaged decision makers at the macrosystem level from across the wider pathway in achieving change identified in earlier phases of the initiative. Findings: The initiative was successful in delivering change in relation to key aspects of the pathway, engaging frontline staff and decision makers from different services within the pathway, and in building quality improvement capability within the workforce. Viewing the pathway as a series of interrelated CMS enabled stakeholders to understand the complex nature of the pathway and to target key areas for change. Particular challenges encountered arose from organisational reconfiguration and cross-boundary working. Conclusion: CMS quality improvement methodology may be a useful approach to promoting integration across a care pathway. Using a CMS approach contributed towards clinical and professional integration of some aspects of the service. Recognition of the pathway operating at meso- and macrosystem levels fostered wider stakeholder engagement with the potential of improving integration of care across a range of health and care providers involved in the pathway.</t>
@@ -8999,6 +9108,11 @@
       <c r="K184" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11603,6 +11717,12 @@
           <t>BSMA0252</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>Marketing boundary spanners—especially customer service representatives—are notably susceptible to burnout. The authors define the burnout construct and develop hypotheses to examine if burnout acts as a partial mediator between role stressors and key behavioral and psychological job outcomes. Responses from 377 customer service representatives reveal that burnout levels are high relative to other burnout-prone occupations (e.g., police, nursing) and that burnout has consistent, significant, and dysfunctional effects on their behavioral and psychological outcomes. Moreover, burnout mediates the negative effects of role stressors on job outcomes, whereas the positive effects of role stressors are unmediated.</t>
@@ -11626,6 +11746,11 @@
       <c r="K255" t="inlineStr">
         <is>
           <t>1994</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14594,6 +14719,12 @@
           <t>BSMA0332</t>
         </is>
       </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>Science parks are a type of organizational sponsorship initiative aimed at generating resource-munificent environments through the provision of bridging and buffering services. While extant research has studied the relationship between these services and firm outcomes, it has neglected to provide insights into when tenant firms utilize these services to a greater or lesser extent. Our study evaluates science parks’ buffering mechanism and identifies firm-level characteristics affecting tenants’ use intensity of buffering services. To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries. Taking a resource dependence perspective, our findings indicate that tenants’ managerial resources (particularly top management team size and functional experience) and boundary-spanning capacity jointly determine the extent to which firms rely upon the science park’s buffering mechanism. This study contributes to the organizational sponsorship, resource dependence, and science park literatures, as well as has important practical implications.</t>
@@ -14617,6 +14748,11 @@
       <c r="K335" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14631,6 +14767,12 @@
           <t>BSMA0333</t>
         </is>
       </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>Purpose – As teams are built around specialized and different knowledge, they need to regulate their knowledge boundaries to exchange their specialized knowledge with other teams and to protect the value of such specialized knowledge. However, prior studies focus primarily on boundary spanning and imply that boundaries are obstacles to sharing knowledge. To ﬁll this research gap, this study aims to indicate the importance of knowledge protection regulation, an activity that sets an adequate boundary for protecting knowledge, and investigate the factors that facilitate knowledge protection regulation and its consequences.</t>
@@ -14654,6 +14796,11 @@
       <c r="K336" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14705,6 +14852,12 @@
           <t>BSMA0335</t>
         </is>
       </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the effects of relationship bonds on the psychological response and behavior of bank employees based on the job demands–resources theory. Specifically, it examines the effects of relationship bonds in terms of person–job (P–J) fit, emotional exhaustion, job satisfaction and boundary-spanning behaviors, all of which comprise the behavioral dimensions of bank employees. In addition, the study examines how the resiliency of bank employees influences their emotional exhaustion and determines whether a moderating effect related to emotional exhaustion exists.</t>
@@ -14728,6 +14881,11 @@
       <c r="K338" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P338" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14779,6 +14937,16 @@
           <t>BSMA0337</t>
         </is>
       </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G340" t="inlineStr">
         <is>
           <t>This research examines the effect an Information Systems (IS) development team has on end-users’ perceptions of system quality and system benefits by transferring relevant knowledge through inter- and intra-firm boundaries. The research context is the prevalent partnership in which an external consultant with relevant expertise leads a client team to undertake an IS project. A high-level research model that depicts dynamics among team competence (for knowledge transfer), consultant partnership (with the project team), knowledge transfer (through inter- and intra-firm boundaries), and project success is proposed grounded on the theory of boundary spanning. Key indicators of team competence and consultant partnership are derived from existing studies. With expected multiplicity in the conceptual dimensions of team competence and consultant partnership, they are designated as second-order constructs with first-order manifest variables. User perceptions of the post-implementation quality and benefits of an information system serve as project success variables. Relevant hypotheses propose dynamics among the studied constructs. Survey data are gathered from both system developers and end-users, and the integrity of the research model and corresponding hypotheses are empirically tested with structural equation modeling. Data analysis confirmed the importance of knowledge transfer for the post-implementation success of an IS project.</t>
@@ -14802,6 +14970,11 @@
       <c r="K340" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14816,6 +14989,12 @@
           <t>BSMA0338</t>
         </is>
       </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -14839,6 +15018,11 @@
       <c r="K341" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P341" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14890,6 +15074,12 @@
           <t>BSMA0340</t>
         </is>
       </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>Innovation is a risky business. Notwithstanding the attention in research on the determinants of innovation success, the estimates of the extremely high failure rates (ranging from 40% to 90%) have not come down. As a result, new approaches have to be found to address the issues that prevent organizations from reaching innovation success over a longer period of time. In this study, Signal Detection Theory (SDT) is introduced to show that it may be less important to improve innovation practices in companies, than it is to change the nature of the projects that enter the corporate innovation funnel. In our empirical study of 44 innovation projects in the pharmaceutical and electronics industry, we show that pursuing more noisy signals (uncertain technological and market opportunities) is currently beneficial for innovation success. In general, companies allocate too few resources to noisy innovation opportunities. Interestingly, we find a positive, and not an inverted U-shaped, relationship between noise/signal ratios and innovation success. This indicates that there are almost no companies that take too much risk in the current competitive environment and that many can gain from increasing their noise tolerance. The implications from this study are quite counter-intuitive in a sense that ‘risk’ is not the cause of the innovation problems, but may be a solution.</t>
@@ -14913,6 +15103,11 @@
       <c r="K343" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14927,6 +15122,12 @@
           <t>BSMA0341</t>
         </is>
       </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to provide a novel way of thinking about firm internationalization. We offer a stylized view of family firms as internationalizers who choose to engage in “boundary-spanning” across global product markets while engaging in “boundary-buffering” to insulate themselves from global financial markets.</t>
@@ -14950,6 +15151,11 @@
       <c r="K344" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14964,6 +15170,12 @@
           <t>BSMA0342</t>
         </is>
       </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>Multiteam systems (MTSs) have been increasingly adopted as an organizational form to manage large-scale projects. However, new product development (NPD) in the MTSs structure entails challenges with respect to achieving efﬁciency due to interteam coordination challenges. Shared mental models (SMMs) within a single team have been found to facilitate intrateam coordination; however, further exploration is needed as to whether SMMs within MTSs can improve interteam coordination among component teams and, if so, what mechanisms underlie this. The present article examines the theoretical underpinning of the impacts of SMMs among component team leaders on MTSs’ NPD efﬁciency, and further considers the impact of external conditions of requirement uncertainty, the most common external situation during NPD. Using survey data from 110 information technology development MTSs and drawing on boundary management perspective, the results reveal that SMMs among component team leaders positively affect NPD efﬁciency by managing the MTSs boundary, i.e., through boundary entrainment and boundary buffering activities at the system level. In addition, we ﬁnd that requirement uncertainty plays a vital role in determining the nature of this relationship. Taken together, our ﬁndings highlight the importance of the role of SMMs among component team leaders in facilitating NPD efﬁciency in MTSs settings.</t>
@@ -14987,6 +15199,11 @@
       <c r="K345" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study analyzes data at the Multi-Team System (MTS) level (N=110 MTSs), measuring system-level boundary management activities rather than individual-level employee boundary spanning behavior.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15001,6 +15218,12 @@
           <t>BSMA0343</t>
         </is>
       </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>Past research on team boundary work has focused on a “cold,” information-exchange perspective to explain why boundary activities affect team innovation. Although the theory is widely accepted, empirical studies on the actual mechanism are scant and produce inconsistent results. Drawing from Interaction Ritual Theory (Collins, 2004), we propose a “warm,” affective perspective that emphasizes team emotional energy - a shared feeling of enthusiasm among team members - as a mechanism linking boundary work and team innovation. Moreover, we examine a theory-driven contextual factor -team role overload - that modifies the hypothesized mediated relationship. Based on field data from four different sources of 89 automotive research and development teams (comprising 724 employees, 89 direct supervisors and 18 managers), we found that both team boundary-spanning and boundary-buffering activities are associated with higher levels of team emotional energy, which, in turn, are related to greater levels of team innovation. Moreover, the mediated relationship of boundary-buffering activities, team emotional energy and team innovation is moderated by team role overload, such that the mediated relationship is stronger when team role overload is higher. Our study contributes to the literature by broadening our understanding of why boundary work is effective and when it matters most.</t>
@@ -15024,6 +15247,11 @@
       <c r="K346" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15038,6 +15266,12 @@
           <t>BSMA0344</t>
         </is>
       </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr">
         <is>
           <t>Drawing from team-level job demands-resources theory, we hypothesize that team workload demands moderate the positive link between team boundary work (i.e., boundary spanning and boundary buffering) and team effectiveness (i.e., team innovation and team performance), such that boundary work is more beneficial for team effectiveness when teams face higher team workload demands. Furthermore, we predict that this interaction occurs through increased team vigor, where team vigor is defined as an affective emergent state characterized by positive valences and high activation levels experienced by team members. We largely find support for our model across two field studies: a cross-sectional survey using three independent data sources (89 automotive research and development teams, including 724 team members, 89 team leaders and 18 managers) and a time-lagged survey using two independent data sources (139 teams working in a Chinese utility company, including 640 team members and 139 team leaders). Our article contributes to team research by broadening our understanding of when and how team boundary work is associated with greater team effectiveness.</t>
@@ -15061,6 +15295,11 @@
       <c r="K347" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15075,6 +15314,12 @@
           <t>BSMA0345</t>
         </is>
       </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>Boundary spanning activity Is conceived of as an intervening variable between organization structure and perceived environmental uncertainty. This is because boundary spanners operate at the skin of the organization and hence their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relationships between perceived environmental uncertainty, organization structure, and boundary spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relationships were found between all three variables. Partial relationships indicated that PEtJ does not influence the boundary spanning-structure relationship, but structure reduces the PEtJ-boundary spanning relationship to zero, and boundary spanning reduces the structurePEU relationship to zero. Thus, not only is the boundary spanning as an intervening variable supported, but results suggest that causality in the Btructure-PEU relationship may be in the direction of structure to PEU rather than current contingency notions of PEU effecting structure.</t>
@@ -15098,6 +15343,11 @@
       <c r="K348" t="inlineStr">
         <is>
           <t>1976</t>
+        </is>
+      </c>
+      <c r="P348" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15112,6 +15362,12 @@
           <t>BSMA0346</t>
         </is>
       </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>Boundary-spanning activity is conceived of as an intervening variable between organization structure and perceived environmental uncertainty (PEU). This is due primarily because, since boundary spanners operate at the skin of the organization, their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relations between PEU, organization structure, and boundary-spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relations were found between all three variables. Partial relations indicated that PEU does not influence the relationship of boundary spanning to structure but structure reduces the relationship of PEU to boundary spanning to zero, and boundary spanning reduces the relationship between structure and PEU to zero. Thus, not only is the notion of boundary spanning as an intervening variable supported, but results suggest that causality in the relationship between structure and PEU may be from structure to PEU rather than current contingency notions of PEU affecting structure.</t>
@@ -15135,6 +15391,11 @@
       <c r="K349" t="inlineStr">
         <is>
           <t>1977</t>
+        </is>
+      </c>
+      <c r="P349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15149,6 +15410,12 @@
           <t>BSMA0347</t>
         </is>
       </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>Building on the theories of knowledge recombination, we argue that the external acquisition of technologies acts as a boundary spanning mechanism that impacts on the recipient firm’ subsequent technology development. The effect is moderated by two additional mechanisms, namely the retention of star scientists and the experience in upstream strategic alliances. We tested our hypotheses on a sample of 6208 USPTO patented technologies acquired by 350 biotechnology firms over the period 1980–2012. Findings reveal an inverted U-shaped effect of the pioneering nature of the acquired technology on firm’s subsequent developments, in terms of (self) citations of firm’s subsequent patents to the acquired one. Moreover, the main relationship is negatively moderated by the retention of star scientists, while the experience in upstream alliances demonstrates to be a positive moderator.</t>
@@ -15172,6 +15439,11 @@
       <c r="K350" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P350" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15186,6 +15458,12 @@
           <t>BSMA0348</t>
         </is>
       </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>Successful product development requires managing tensions—coping with fluctuating contingencies to foster innovation and efficiency. To investigate this challenge, we explored the nature, dynamics, and impacts of contrasting project management styles. Our conceptual framework details emergent and planned styles. Following 80 projects over two-year periods, we find that these styles offer disparate but interwoven approaches to monitoring, evaluation, and control activities; use of these activities fluctuates over time; a paradoxical blend of styles enhances performance; and uncertainty moderates project management-performance relationships.</t>
@@ -15209,6 +15487,11 @@
       <c r="K351" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16074,6 +16357,16 @@
           <t>BSMA0372</t>
         </is>
       </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G375" t="inlineStr">
         <is>
           <t>In this paper we present a study of the structure of three lead firm‐network relationships at two points in time. Using data on companies in the packaging machine industry, we study the process of vertical disintegration and focus on the ability to coordinate competencies and combine knowledge across corporate boundaries. We argue that the capability to interact with other companies—which we call relational capability—accelerates the lead firm’s knowledge access and transfer with relevant effects on company growth and innovativeness. This study provides evidence that interfirm networks can be shaped and deliberately designed: over time managers develop a specialized supplier network and build a narrower and more competitive set of core competencies. The ability to integrate knowledge residing both inside and outside the firm’s boundaries emerges as a distinctive organizational capability. Our main goal is to contribute to the current discussion of cooperative ties and dynamic aspects of interfirm networks, adding new dimensions to resource‐based and knowledge‐based interpretations of company performance.</t>
@@ -16097,6 +16390,11 @@
       <c r="K375" t="inlineStr">
         <is>
           <t>1999</t>
+        </is>
+      </c>
+      <c r="P375" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16111,6 +16409,16 @@
           <t>BSMA0373</t>
         </is>
       </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G376" t="inlineStr">
         <is>
           <t>Research on the district’s role in fostering improvements affecting student learning is still in its infancy. Since the early 1990s, when school districts were often viewed as a waste of time and money (Chubb and Moe 1990), the winds have shifted, with states and districts expected to promote coherence and accountability in the loosely coupled US school system (Boyd and Crowson 1981). The articles in this issue not only expand middle-level theories concerning how these enlarged responsibilities and roles may develop but also add empirical meat to expectations in state and federal accountability policies. As advertised, the articles represent a “first installment” on a needed scholarly dialogue. Let me further the dialogue by suggesting topics for additional investigation arising from their work.</t>
@@ -16134,6 +16442,11 @@
       <c r="K376" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P376" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16185,6 +16498,12 @@
           <t>BSMA0375</t>
         </is>
       </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr"/>
       <c r="G378" t="inlineStr">
         <is>
           <t>A central focus of cross-cultural management research is how individuals and organizations differ across national cultures and how that fundamentally shapes their thoughts and actions and serves as a unit of identification. In this article, we critically reconsider the essential categorical nature of culture, problematizing categorization and questioning national culture as the primary basis of differentiation. We draw on intersectionality, an approach that helps understand how multiple categories are experienced by the individual, and on relationality, an approach that conceptualizes people, organizations, and their actions within dynamic patterns of relations and cultural meanings. Both approaches challenge the primacy, unity, and separateness of any given category, the a priori determination of categories (and associated boundaries) in research, and the nature and stability of boundaries. Based on this we advance notions of boundary work and boundary shifting that help explore how today’s sociocultural groups and categories, and the boundaries that separate them, emerge and change. We conclude that, while the extant crosscultural literature has come far in identifying differences, relationality and intersectionality can enable cross-cultural scholars to engage in research practice that better reflects the complexities of sociocultural life. We contribute to theory by suggesting why and how these two approaches can be used to explore complex cross-cultural management phenomena.</t>
@@ -16208,6 +16527,11 @@
       <c r="K378" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16222,6 +16546,12 @@
           <t>BSMA0376</t>
         </is>
       </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr"/>
       <c r="G379" t="inlineStr">
         <is>
           <t>The paper explores how formal leaders make sense of and deal with autonomy of knowledge-workers. Based on interviews, I suggest that leaders make sense of knowledge-workers’ autonomy as ranging from perfectly autonomous to too autonomous to less independent to acting childish. This ambiguity was dealt with by making sense of leading as ranging from facilitative and supportive approaches to more controlling, even reprimanding acts. This empirical investigation of constructions of ‘leader/ship’ and ‘followers’ contributes to leader/ship-follower/ship literature. The paper’s contribution to theory lies in the notion of situated ambiguity; a way to understand the emerging way through which formal leaders navigate and smoothly move between their own diﬀering perspectives, diﬀerent practical situations, various culturally acceptable understandings of leaders and knowledgeworkers.</t>
@@ -16245,6 +16575,11 @@
       <c r="K379" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17576,6 +17911,12 @@
           <t>BSMA0412</t>
         </is>
       </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>The purpose of this research is to determine the description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, to determine and analyze the influence of Emotional Dissonance on Service Sabotage, to determine and analyze the influence of Emotional Intelligence on Service Sabotage, and to determine and analyze the influence of Emotional Exhaustion on Service Sabotage. The population in this study were all employees of the Grand Mercure Hotel Kemayoran Jakarta. In this research, a quantitative method approach was used with a survey and a sample of 225 people was obtained using a purposive sampling technique. Survey research is carried out by distributing questionnaires. Previously, the questionnaire was tested for validity and reliability first. The data analysis technique in this research uses descriptive analysis and linear regression analysis. Description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, most of whom are male, most employees are under 35 years old, and most employees have worked at the hotel for 0-2 years. The results of this research explain that Emotional Dissonance has a positive and significant effect on Service Sabotage with p-value of 0.012. Emotional Intelligence has a negative and significant effect on Service Sabotage with p-value of 0.023. Emotional Exhaustion has a positive and significant effect on Service Sabotage with p-value of 0.045.</t>
@@ -17599,6 +17940,11 @@
       <c r="K415" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17650,6 +17996,12 @@
           <t>BSMA0414</t>
         </is>
       </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>Intergroup knowledge integration, that is the acquisition, processing, and utilization of knowledge across group boundaries, is a critical source of competitive advantage in modern organizations. Prior research has highlighted the important role of boundary spanning knowledge exchange for intergroup knowledge integration, neglecting, however, the question of what makes individual boundary spanners more effective in fostering intergroup knowledge integration. Integrating boundary spanning literature with theories of group information processing, we hypothesize that the effect of individual boundary spanning ties on intergroup knowledge integration depends on the boundary spanners’ levels of metaknowledge, i.e., knowledge of who knows what in their respective groups, and proactivity. We find general support for our predictions in a study of 457 engineering consultants nested in 22 interdependent business units within an organization. Additional criterion analyses confirm the material importance of intergroup knowledge integration for group performance. Our findings have implications for literatures on intergroup effectiveness, team cognition, and proactivity.</t>
@@ -17673,6 +18025,11 @@
       <c r="K417" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17687,6 +18044,12 @@
           <t>BSMA0415</t>
         </is>
       </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr">
         <is>
           <t>Drawing upon the theory of gender frame, the research on gender in science, and social network studies, this paper focuses on the social mechanism of collaboration, speciﬁcally the boundary-spanning collaboration, to understand the gender gap in academic patenting in the U.S. Correspondingly, the author developed a few hypotheses for empirical testing. The results show that, else being equal, only collaboration with industry would signiﬁcantly increase the probability of patenting for female academic scientists, but this helps explain considerable difference in patenting between female and male academics. The ﬁndings are discussed along with the limitations and policy implications at the end.</t>
@@ -17710,6 +18073,11 @@
       <c r="K418" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17724,6 +18092,12 @@
           <t>BSMA0416</t>
         </is>
       </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their boundaries in ways that complement their preferences.</t>
@@ -17747,6 +18121,11 @@
       <c r="K419" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study focuses on work-family/work-life role segmentation preferences and boundary management between work and home domains, rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17761,6 +18140,12 @@
           <t>BSMA0417</t>
         </is>
       </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>Background Increasing role complexity has intensiﬁed the boundary spanning functions of managers. Because work demands and scope vary by management position, time in staff contact rather than span may better explain managersÕ capacity to support staff. Methods A descriptive, correlational design was used to collect cross-sectional survey and prospective work log and administrative data from a convenience sample of 558 nurses in 51 clinical areas and 31 front-line nurse managers from four acute care hospitals in 2007–2008. Data were analysed using hierarchical linear modelling. Results Span, but not time in staff contact, interacted with leadership and operational hours to explain supervision satisfaction. Conclusions With compressed operational hours, supervision satisfaction was lower with highly transformational leadership in combination with wider spans. With extended operational hours, supervision satisfaction was higher with highly transformational leadership, and this effect was more pronounced under wider spans. Implications for Nursing Management Operational hours, which inﬂuence the managerÕs daily span (average number of direct report staff working per weekday), should be factored into the design of front-line management positions.</t>
@@ -17784,6 +18169,11 @@
       <c r="K420" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study conceptually frames front-line managers as boundary spanners but does not measure the behavioral construct of boundary spanning behavior (BSB). Instead, it measures structural variables (span of control) and 'time in staff contact' (mere interaction time without specifying purposive boundary-spanning actions), alongside transformational leadership. Under Rule 18, variables measuring mere communication frequency or time without specifying purposive action are invalid. Thus, the study lacks a valid effect size of interest.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17835,6 +18225,16 @@
           <t>BSMA0419</t>
         </is>
       </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
       <c r="G422" t="inlineStr">
         <is>
           <t>This paper develops and tests a theoretical model of the relationships among environmental interdependence, environmental uncertainty, and boundary-spanning activities. Drawing from the strategic choice literature, a decision variable labeled influence on organizational decision was incorporated as a moderator. Results supported the environmental interdependence-environmental uncertainty-boundary-spanning activities relationships, but the individual influence variable failed to emerge as a moderator.</t>
@@ -17858,6 +18258,11 @@
       <c r="K422" t="inlineStr">
         <is>
           <t>1987</t>
+        </is>
+      </c>
+      <c r="P422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17872,6 +18277,12 @@
           <t>BSMA0420</t>
         </is>
       </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>Background: Emotions play a central role in how employees respond to workplace bullying, influencing both their well-being and organizational outcomes. The purpose of the current study was to examine how workplace bullying and turnover intention are related to negative emotions and workplace unfairness. Methods: The research involved collecting data from 269 boundary-spanning bank workers (call center workers, frontline office staff, and customer service representatives) who experienced bullying. A moderated mediation was tested using Model 7 of the Process macro. The relationship between workplace bullying and turnover intention was analyzed, emphasizing the moderating effect of workplace unfairness and the mediating role of negative emotions. Results: The results validated the model, showing that an increase in negative emotions and workplace unfairness promotes the link between workplace bullying and the intention to leave. Increased negative emotions and perceived workplace unfairness amplified the relationship between workplace bullying and turnover intention. Conclusions: The findings underscored the cumulative risk of bullying environments for employee well-being and retention, providing practical recommendations for HRM and leadership strategies to cultivate healthier, more inclusive workplace settings. This study adds to the bullying–turnover literature by examining the joint role of negative emotions and workplace unfairness in a moderated mediation framework. The study connects these findings to sustainable labor management, emphasizing both theoretical and practical implications for organizations.</t>
@@ -17895,6 +18306,11 @@
       <c r="K423" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17909,6 +18325,12 @@
           <t>BSMA0421</t>
         </is>
       </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
           <t>It is widely recognized that new product development (NPD) is a highly interdependent process, yet efforts to empirically model the interdependence and examine its effect on ﬁrm performance are scarce. Our study addresses this research gap. We model ﬁrms’ abilities to collectively collaborate with suppliers, customers, and internal employee teams in NPD as collaborative competence and examine its impact on project and market performance. Using responses collected from 189 NPD managers, we ﬁnd empirical evidence for collaborative competence and its differential impact on project and market performance. Speciﬁcally, we ﬁnd that collaborative competence has a direct impact on project performance, but its impact on market performance is indirect, mediated through project performance. The results have signiﬁcant managerial implications; achieving superior market performance from inter- and intra-organizational involvement is contingent on achieving superior project performance, and companies that fail to achieve desired project performance outcomes will also fail in achieving market performance goals.</t>
@@ -17932,6 +18354,11 @@
       <c r="K424" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The unit of analysis is the product development project (N=189 projects/plants), and the product development managers act as key informants reporting on project-level collaborative practices rather than their own individual boundary spanning behavior. Survey items use 'We' or team-level referents.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17946,6 +18373,12 @@
           <t>BSMA0422</t>
         </is>
       </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>Abstract             In organizational contexts, professional boundaries serve a dual purpose by distinguishing various professions from one another and regulating access to power, status, and rewards. Individuals operating within professions in which such boundaries are not clearly or explicitly defined face the risk of compromising their status and autonomy. However, they possess the agency to actively define their profession and enhance its standing among both internal and external stakeholders. This study explores how homeroom teachers in the Israeli education system—recognized as a distinct occupation within the broader teaching profession—engage in boundary work to form and define their professional group. Our findings reveal that (1) homeroom teachers employ adaptable boundary work strategies, tailored to their interactions with different key stakeholders. Specifically, they (a) define boundaries to clarify, for themselves, the parameters of their own roles; (b) balance boundaries with partners inside the school (administrators and subject teachers) to facilitate day-to-day collaboration while simultaneously asserting their own roles; and (c) orchestrate boundaries when interacting with external partners (students’ parents), acknowledging the distinction between roles while primarily seeking to foster effective joint work towards the common goal of helping students succeed. (2) Despite the diversity in their approaches, all homeroom teachers exhibit a unique expertise, allowing them to combine boundary-setting with inclusivity, highlighting the dynamic and interactive nature of the boundary work process. This dual nature enhances the effectiveness of communication and collaboration within the educational system, molding the role of homeroom teachers as a distinct professional group.</t>
@@ -17969,6 +18402,11 @@
       <c r="K425" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -22121,6 +22559,16 @@
           <t>BSMA0533</t>
         </is>
       </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G536" t="inlineStr">
         <is>
           <t>Many firms actively disclose research findings in scientific peer-reviewed journals. The literature highlights several potential benefits of such scientific boundary-spanning activities, including privileged access to academic information networks. However, scientific disclosure may lead to unintended knowledge spillovers. It remains unclear whether active engagement in science leads to higher returns. This paper investigates the impact of scientific activities on the firm’s market value, using accounting data for U.S. firms and matched patent and scientific publication data. We find evidence for the positive impact of scientific publications on a firm’s market value beyond the effects of research and development, patent stocks, and patent quality, and also document heterogeneity with respect to this impact between different industrial sectors.             This paper was accepted by David Hsu, entrepreneurship and innovation.</t>
@@ -22144,6 +22592,11 @@
       <c r="K536" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P536" t="inlineStr">
+        <is>
+          <t>Firm-level analysis of scientific publications using accounting and patent databases lacking individual employee samples [Code 2 &amp; Code 3].. Verbatim Evidence: [Abstract] "Thispaper investigatesthe impactofscientific activities onthefirm'smarket value, using accountingdataforU.S.firms andmatched patentandscientific publication data." [Introduction] "Ourempirical analysisusesfirm-level information fromtheCompustat database andmatched scientificpublication andpatentdataforarepresentativesampleof1,739stockmarketlistedfirms(9,920 firm-year observations) fromallhigh-technologysectors,coveringtheperiod1996-2006."</t>
         </is>
       </c>
     </row>
@@ -22158,6 +22611,16 @@
           <t>BSMA0534</t>
         </is>
       </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G537" t="inlineStr">
         <is>
           <t>This paper proposes a radical empirical look on the concrete activities of project managers involved in creative projects, with a speciﬁc focus on ‘‘non-administrative’’ issues. Through four case studies in the video-game industry, multimedia, advertising and a circus, we propose an integrated synthesis of what creative project managers actually do. Beyond analytical, cognitive, psychological, symbolic and discursive activities, we identify four sets of activities carefully coined to acknowledge the everyday work of project manager involved in creative projects. We suggest that this project manager acts as a sense-maker, a web-weaver, a game-master and a ﬂowbalancer. This empirical ‘‘picture’’ raises questions on the technical and theoretical focus of research in project management where creativity is an utmost strategic issue.</t>
@@ -22181,6 +22644,11 @@
       <c r="K537" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P537" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Abstract] "This paper proposes a radical empirical look on the concrete activities of project managers involved in creative projects, with a speciﬁc focus on ‘‘non-administrative’’ issues. Through four case studies in the video-game industry, multimedia, advertising and a circus, we propose an integrated synthesis of what creative project managers actually do." [Research method] "This is a cases study based research which derives from an exploratory ethnographic ﬁeld study on the video-game industry in the tradition of grounded theory [43,44] and qualitative research on emergent phenomena [45–47] ."</t>
         </is>
       </c>
     </row>
@@ -22232,6 +22700,16 @@
           <t>BSMA0536</t>
         </is>
       </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G539" t="inlineStr">
         <is>
           <t>To successfully satisfy large customers and meet financial objectives, dedicated sales teams need to manage two boundaries: a boundary within the selling firm and one with the customer organization. However, little is known about the process of managing these multiple boundaries. This study integrates job demands-resource theory with research on key account management and sales teams to examine (1) the main effect of customer boundary spanning on perceived customer satisfaction and team performance and (2) the moderating role of within-firm coordination activities at three levels: top management, cross-functional, and within-team. An empirical test of the model with data from 167 sales teams finds that the interaction between customer boundary spanning and within-firm coordination activities has opposite effects on perceived customer satisfaction and team performance outcomes. The results are robust to endogeneity and heteroskedasticity concerns.</t>
@@ -22255,6 +22733,11 @@
       <c r="K539" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P539" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=167 sales teams). Verbatim Evidence: [Method] The firm collected the data by sending a survey to 201 United States-based dedicated sales teams of a large multinational firm. The data were made available to us after being aggregated to the team level. [Method] The end result was a total of 167 usable surveys. [Table 1] N=167.</t>
         </is>
       </c>
     </row>
@@ -22269,6 +22752,16 @@
           <t>BSMA0537</t>
         </is>
       </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="G540" t="inlineStr">
         <is>
           <t>This dissertation investigated the effects of intrinsic and extrinsic motivational orientations in a boundary spanning model of retail buyers. Contributions of the dissertation to the field of marketing include the following: First, a boundary spanning/role stress model was tested in the context of retail buyers. No previous work has empirically or conceptually investigated the ability of a boundary spanning/role stress model to explain retail buyers' work-related attitudes. Second, the boundary spanning/role stress model was extended with the inclusion of accumulated role benefits. Previous role stress studies consider only negative role perceptions; accumulated role benefits examines positive role perceptions. Third, the boundary spanning/role stress model considers only external influences of role set members on a role incumbent. In doing so, the model neglects the influence of the individual who is perceiving and interpreting these stimuli. To capture individual differences, effects of intrinsic and extrinsic motivational orientations of the buyers were tested in the model. Finally, scales were developed to measure intrinsic motivational orientations, extrinsic motivational orientations, boundary spanning beliefs, and accumulated role benefits.</t>
@@ -22292,6 +22785,11 @@
       <c r="K540" t="inlineStr">
         <is>
           <t>1988</t>
+        </is>
+      </c>
+      <c r="P540" t="inlineStr">
+        <is>
+          <t>Included. The study examines individual-level boundary spanning behaviors (beliefs) of retail buyers and provides a zero-order correlation matrix.. Verbatim Evidence: [Sample] "The sample frame was Sheldon's Retail Directory (1986), which lists buyer names, store affiliations with addresses, and type of merchandise bought for department stores, chain stores, and specialty stores." [Methodology] "305 of the original 700 buyers sampled responded to the survey, for a response rate of 43.6%." [Measures] "Three positively worded items address beliefs about external boundary spanning: item Q51 states, "I spend at least half my time dealing with people who work for other companies"; item Q34 states, "Getting my job done often depends on the activities of people who don't even work for my company"; and item Q7 states, "I regularly communicate with employees of other companies in order to get my job done."" [Data] "Table 4-17 Descriptive Statistics for Summated Scales: Matrix of Correlations, 1-Tailed Sig, N of cases"</t>
         </is>
       </c>
     </row>
@@ -22306,6 +22804,16 @@
           <t>BSMA0538</t>
         </is>
       </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G541" t="inlineStr">
         <is>
           <t>A widely-cited proposition in boundary theory states that it is difficult for individuals to transition between roles, especially when these roles are highly segmented. Surprisingly, this hypothesis has not been directly tested. We provide an empirical test of these propositions and draw from the self-regulation literature to expand boundary theory in exploring how episodes of cognitive role transitions impact job performance. We propose that cognitive role transitioning is cognitively demanding, which consumes the limited executive control resources that facilitate effective job performance. In a multilevel study of 619 employees providing 4371 episodes, we observed that work-to-family cognitive role transitioning was negatively related to job performance, and this effect was mediated by self-regulatory depletion. Although individuals with greater role integration were somewhat more likely to experience cognitive role transitions than those with segmented roles, these individuals were also buffered from the self-regulatory depletion that impairs effective job performance. Overall, these findings suggest that integration, rather than segmentation, may be a better long-term boundary management strategy for minimizing self-regulatory depletion and maintaining higher levels of job performance during inevitable work–family role transitions.</t>
@@ -22329,6 +22837,11 @@
       <c r="K541" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P541" t="inlineStr">
+        <is>
+          <t>Work-Family construct homonymy.. Verbatim Evidence: [Abstract] "we observed that work-to-family cognitive role transitioning was negatively related to job performance" [Method] "We used data from the Sloan 500 Family Study (Schneider and Waite, 2008) to test our hypotheses." "The 500 Family Study targeted middle-class, dual-earner families, including mothers, fathers and children sampled from communities dispersed across the United States." [Measures] "Work-to-family cognitive role transition episodes were measured dichotomously where participants were assigned a 0 if no role transition occurred or a 1 if a role transition episode was present." "Cognitive role transition episodes were coded as 1 if a participant was thinking about family-related content."</t>
         </is>
       </c>
     </row>
@@ -22343,6 +22856,16 @@
           <t>BSMA0539</t>
         </is>
       </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G542" t="inlineStr">
         <is>
           <t>Purpose – Boundary-spanning managers need to recognize, learn and implement external knowledge while balancing the conflicts emerging from new and existing knowledge. The authors’ study explores how a paradox mindset (PM) and a learning focus [learning goal orientation (LGO)] promote two managerial capabilities: absorptive capacity (ACAP) and ambidexterity. The authors’ study explores the inter-relationship between the mindsets and the capabilities required for innovative work behavior.</t>
@@ -22366,6 +22889,11 @@
       <c r="K542" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P542" t="inlineStr">
+        <is>
+          <t>No effect size of interest; boundary spanning is used as a sample inclusion criterion rather than a measured construct in the correlation matrix.. Verbatim Evidence: [Methodology] "We targeted technology managers who act as boundary spanners and were directly involved in activities related to R&amp;D, product development and management, marketing and quality assurance departments of the firm." [Methodology] "The initial part of the questionnaire asked each respondent whether they were involved in boundary-spanning activities in the last three years. We eliminated 14 responses from further analysis because of the absence of boundary-spanning roles or missing data." [Table 2] "Mean SD AVE CA CR LGO PM IAC IA"</t>
         </is>
       </c>
     </row>
@@ -22417,6 +22945,16 @@
           <t>BSMA0541</t>
         </is>
       </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G544" t="inlineStr">
         <is>
           <t>This empirical research compared job characteristics and organizational climate in the private and public sectors. Perceptions and satisfaction of 240 top managers from a variety of private and public organizations in Israel were compared. The hypotheses tested were that (a) performance-based rewards and (b) policies that promote efficiency would be significantly more prevalent in private sector organizations and (c) that higher levels of satisfaction would be expressed by managers in the private sector. Two-way analyses of variance, private versus public and production versus service organizations, were performed. Results yielded significant main effects for sector of ownership and provided strong support for the three hypotheses of the research. Interaction effects in specific scales were also in the hypothesized direction, revealing that the private/public sector differences are further amplified in service organizations. The relation of the findings of this research to those of comparable studies in the United States are discussed.</t>
@@ -22440,6 +22978,11 @@
       <c r="K544" t="inlineStr">
         <is>
           <t>1986</t>
+        </is>
+      </c>
+      <c r="P544" t="inlineStr">
+        <is>
+          <t>The study does not measure boundary spanning behavior (BSB). It focuses on job characteristics and organizational climate.. Verbatim Evidence: [Measures] "Two questionnaires were used for the collection of the data for this research, one addressing job characteristics, the other organizational climate." [Measures] "The job characteristics questionnaire consisted of 20 items." [Measures] "These included job reward policies, interpersonal job aspects, and training opportunities." [Measures] "The Organizational Climate Questionnaire consisted of 19 items." [Measures] "These pertained to policies of improvement of methods and efficiency, participation, reward structure, consideration, and decision making practices"</t>
         </is>
       </c>
     </row>
@@ -22454,6 +22997,16 @@
           <t>BSMA0542</t>
         </is>
       </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G545" t="inlineStr">
         <is>
           <t>The purpose of this study is to broaden our understanding of team boundary activities in promoting team innovation. The model examines the mediating role of boundary activities in the relationship between the structural variables of inter-team goal interdependence and team functional heterogeneity and team innovation. Sixty teams from high-technology companies were studied involving 196 team members and their 60 corresponding team leaders and unit managers to whom the leaders report. Results identified two dimensions of boundary activities: boundary-loosening activities and boundary-tightening activities. Overall, the results of the structural equation model confirmed the mediating role of team boundary activity. The results indicated a positive relationship between the two structural variables and boundary-loosening activities, a negative relationship between functional heterogeneity and boundary-tightening activities, and a positive relationship between the two dimensions of boundary activities and team innovation. Implications, limitations, and directions for further research on team boundary activities are discussed.</t>
@@ -22477,6 +23030,11 @@
       <c r="K545" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P545" t="inlineStr">
+        <is>
+          <t>Team Level Aggregation (N = 60 teams). Verbatim Evidence: [Sample] "Sixty product development teams were recruited from different high-technology companies in Israel, specializing in telecommunications, computer software, computer hardware, and semiconductors." [Level of Analysis] "In the present study, the unit of analysis was the team. All the hypotheses referred to the team and such study variables as boundary activities and inter-team goal interdependence were framed at the team level, and aggregated to team level." [Correlation Matrix] "Table 1. Means, Standard Deviations, and Correlation Matrix of Study’s Variables (N = 60)."</t>
         </is>
       </c>
     </row>
@@ -22491,6 +23049,16 @@
           <t>BSMA0543</t>
         </is>
       </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G546" t="inlineStr">
         <is>
           <t>Boundary‐spanning individuals (BSIs) play a critical role in supply chain management, especially in small and medium‐sized enterprises (SMEs) where interactions with buyers and suppliers can depend heavily on just a few individuals. This study, utilizing data from Korean manufacturing‐sector SMEs, explores whether cooperative social value orientations of SMEs' BSIs influence the effects of collaborative buyer‐supplier initiatives. The results suggested that the performance implication of decision‐sharing initiative increases when BSIs have a high level of cooperative social value orientation. However, it also negatively moderates the relationship between risk/benefit sharing (involving financial losses or gains) and performance suggesting possible negative side effects. However, we found that such orientation also negatively moderates the relationship between risk/benefit sharing (involving direct financial losses or gains) and relationship performance suggesting possible negative side effects.</t>
@@ -22514,6 +23082,11 @@
       <c r="K546" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P546" t="inlineStr">
+        <is>
+          <t>Excluded due to multiple reasons: [Code 1 &amp; Code 3]. The study uses individuals as proxy informants for firm-level supply chain initiatives, and the individual-level measure is a personality trait/orientation rather than actual boundary-spanning behavior.. Verbatim Evidence: [Theoretical Development] Tangpong, Hung, and Ro (2010) conceptualize this particular disposition in the buyer-supplier setting as “cooperativeness”; an example is the personality trait that entails acting toward others in tolerant, empathetic, supportive, and compassionate ways for mutual benefit. [Appendix] I am willing to share risks and benefits with my partners. [Research Methods] We selected 2,000 SMEs identified from the Korean Chamber of Commerce and Industry Directory, and to ensure that our respondents were in boundary-spanning roles in their companies, included a covering letter asking that the questionnaire be completed by BSIs such as sales managers. [Appendix] My company shares operational information with our partners. [Appendix] My company does strategic supply-chain planning jointly with our partners.</t>
         </is>
       </c>
     </row>
@@ -22528,6 +23101,16 @@
           <t>BSMA0544</t>
         </is>
       </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G547" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to explore the potential contribution of inter-unit network structure and intraunit task environment to the overall knowledge management (KM) effectiveness of an organization through different KM strategies.</t>
@@ -22551,6 +23134,11 @@
       <c r="K547" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P547" t="inlineStr">
+        <is>
+          <t>The study analyzes boundary-spanning network variables (degree centrality and structural holes) at the work unit level (N=20), which violates the individual-level requirement [Code 3]. Additionally, the individual-level analysis (N=84) focuses on general knowledge management strategies (personalization and codification) which do not measure purposive boundary spanning behavior [Code 1].. Verbatim Evidence: [3.4 Levels of analysis] "The unit of analysis is individual for intra-unit analysis (H3-H6). All task-related and KM-related measures were measured at the individual level. For inter-unit analysis (H1 and H2), the unit of analysis is at the work unit level." [3. Research methodology] "As a result, 20 leader responses and 84 member responses were used in the data analysis." [Appendix 1. Instruments] "Personalization strategy TO1 Making face-to-face social interactions to exchange knowledge."</t>
         </is>
       </c>
     </row>
@@ -22602,6 +23190,16 @@
           <t>BSMA0546</t>
         </is>
       </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G549" t="inlineStr">
         <is>
           <t>Wildfire is a cross-boundary, collective action issue. Previous research has demonstrated the importance of collaborative relationships in wildfire for purposes such as increasing capacity, trading information, and facilitating landscape-scale mitigation projects. However, a stakeholder’s location in social networks, as well as personal factors, may impact their collaboration. Furthermore, stakeholders must prioritize their own organizational goals and responsibilities, which may differ from those of their collaborators. I used interview and survey methods to investigate these questions in the context of wildfire management professionals in northwestern Wyoming. For the interviews, I selected 12 individuals with high betweenness centrality who were involved in wildfire management in different organizations and locations throughout the study area. I used semi-structured interviews and asked participants to describe how they use collaboration to accomplish both collective and organizational goals for wildfire management. I found that managers’ answers to this question could be divided into four themes:(1) Deciding when collaboration is and isn’t the right tool,(2) Utilizing jurisdictional and organizational differences,(3) Finding or designing multi-benefit projects, and (4) Choosing collaborators and building relationships. For the survey, I used chain referral sampling and asked about managers’ participation in 8 collaborative actions, as well as their scope and focus of work, their gender, their role in wildfire management, who they worked with most frequently. I then modeled managers’ participation in the collaborative actions using betweenness centrality, gender, focus, scale, and role as predictors. I found that higher betweenness centrality, a focus on wildfire, and working at the scale of multiple communities or jurisdictions all increased collaboration. Holding the self-identified roles of coordinating across jurisdictions or interests, engaging with landowners, providing leadership or authority, and responding to emergencies also increased collaboration. When all of the variables were combined in a single model, I found that working at the multiple community or jurisdiction scale and holding engaging, coordinating, or responding roles had the most significant impact on collaborative action in a combined model. I found that managers who identified as women had lower collaborative scores, possibly as a result of gender bias in the natural resource and wildfire fields. I also found that men were much more likely to nominate other men in the chain referral portion of the survey, suggesting that gender bias may influence research using this method.</t>
@@ -22625,6 +23223,11 @@
       <c r="K549" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P549" t="inlineStr">
+        <is>
+          <t>No correlation matrix or extractable zero-order effect size (reports only GLMs with McFadden's pseudo-R^2). Verbatim Evidence: [Methods] "I then constructed 5 generalized linear models (GLMs) to understand the influence of social network position and personal factors on collaborative behavior." [Results] "I ran five different generalized linear models (GLM) with CS as the dependent variable, using the “quasibinomial” family to account for CS being a proportion." [Results] "Table 4. Results of 5 GLMs predicting influence of variables on Collaborative Score (CS)."</t>
         </is>
       </c>
     </row>
@@ -22639,6 +23242,16 @@
           <t>BSMA0547</t>
         </is>
       </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G550" t="inlineStr">
         <is>
           <t>Purpose – This study aims to develop and test a new formative theory of coping intelligence (CI). It asserts that problem- and emotion-focused coping strategies contribute differently to the overall CI latent construct, which, in turn, relates to three outcome variables – job satisfaction, life satisfaction and sales commission.</t>
@@ -22662,6 +23275,11 @@
       <c r="K550" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P550" t="inlineStr">
+        <is>
+          <t>No effect size of interest. Measures coping strategies rather than boundary spanning behavior.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] The study collected data from multiple sources: survey data from 452 boundary-spanning salespeople and sales commission from a company’s personnel record." "[Methodology] For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)." "[Appendix] Problem-focused coping (CI-P) I try to work more efficiently. I devote more time and energy to my job. I decide what I think should be done and explain this to the people who are affected."</t>
         </is>
       </c>
     </row>
@@ -22676,6 +23294,16 @@
           <t>BSMA0548</t>
         </is>
       </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G551" t="inlineStr">
         <is>
           <t>In this study, we develop a new theoretical framework of Coping Intelligence (CI) which examines relationships between coping strategies and organizational commitment among boundary spanning employees. We collected data from 452 boundary spanning salespeople using multiple sources. Results demonstrate that a formative model of Coping Intelligence (CI) is superior to a reﬂective model and that problem-focused coping contributes to CI which, in turn, is related to affective and normative commitment. Further, our more parsimonious formative model illustrates that positive problem-focused coping and negative emotion-focused coping contribute to both affective and normative commitment. After controlling for gender and salespeople’s commission (from company’s personnel record) in separate analyses, results remain signiﬁcant. We provide additional insights: Females are likely to use emotion-focused coping than males, but gender is not related to organizational commitment. Salespeople’s commission is positively related to both affective and normative commitment but unrelated to coping strategies. We shed new lights on boundary spanning employees’ Coping Intelligence and organizational commitment and offer theoretical, empirical, and practical implications to coping strategies and business ethics.</t>
@@ -22699,6 +23327,11 @@
       <c r="K551" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P551" t="inlineStr">
+        <is>
+          <t>The study surveys boundary-spanning employees (salespeople) but does not measure Boundary Spanning Behavior (BSB) as a variable. It only measures coping strategies and organizational commitment.. Verbatim Evidence: [Abstract] "We collected data from 452 boundary spanning salespeople using multiple sources." [Measure] "The components of Coping Intelligence, problem-focused coping (CI-P), action-focused coping (CI-A), and emotion-focused coping (CI-E), were measured using 33 items adapted from Folkman and Lazarus (1988) Ways of Coping Checklist." [Measure] "We used Meyer et al. (1993) organizational commitment scale to measure affective (OC-A), continuance (OC-C), and normative (OC-N) commitment."</t>
         </is>
       </c>
     </row>
@@ -22713,6 +23346,16 @@
           <t>BSMA0549</t>
         </is>
       </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G552" t="inlineStr">
         <is>
           <t>The current study draws upon socialization theory to investigate both antecedents and outcomes of support service utilization within a sales employee context. Research indicates high performing, in contrast to low performing, salespeople may be more adept at discerning the ways in which an organization’s support services can be useful to them. The empirical results obtained from sales personnel of a financial services firm suggest that effective socialization/communication is important in securing an employee’s reliance upon organizational support. Further, high-performing salespeople are more proactive and instrumental in relation to utilization of support services, while low-performing salespeople are more passive and conforming in interfacing with support. Implications to both practice and research are discussed.</t>
@@ -22736,6 +23379,11 @@
       <c r="K552" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P552" t="inlineStr">
+        <is>
+          <t>The study does not measure boundary spanning behavior. It focuses on the consumption of organizationally provided support services, measuring variables such as reliance on support-service provider, satisfaction with support-service outcome, and communication frequency.. Verbatim Evidence: [Sample and data collection] &lt;The firm identified 1524 salespeople for whom a new office had been opened within the previous 3 years.&gt; [Measures] &lt;The constructs used to test our hypotheses were all measured with multiple-item, seven-point scales (see Table 1 for a listing of scale items).&gt; [Conceptual model and hypotheses] &lt;We propose that sales employees derive value from OPS in two ways: 1) through feelings of satisfaction with the OPS outcomes and, 2) through reliance on the OPS provider to produce the service, rather than self-production, which would direct employees’ time and effort toward nonproductive activities as opposed to value creation through customer interaction (Arndt &amp; Harkins, 2013).&gt; [Managerial implications] &lt;Customer expectations about receiving the full array of services of these boundary spanners is formed by the firm’s and/or competitor’s marketing communications.&gt;</t>
         </is>
       </c>
     </row>
@@ -22750,6 +23398,16 @@
           <t>BSMA0550</t>
         </is>
       </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G553" t="inlineStr">
         <is>
           <t>Within business-to-business relationship marketing, boundary-spanning representatives play a crucial role in establishing and maintaining positive relations between their organizations. Spirituality, a workplace individual-level variable, is proposed to significantly influence buyer representatives’ relationship formation with their seller counterparts, which subsequently affects the relationship development between organizations. Here we identify aspects of spirituality within buyer representatives and present a conceptual framework that delineates the impact of spirituality upon individual perceptions of relational constructs such as trust and commitment. Structural equation modeling analyses support the inclusion of spirituality as a relevant construct in relationship marketing research. In addition, because cultural differences are known to exist regarding the role of spirituality, the impact of spirituality upon perception within relationship marketing is addressed with data collected from both American and Chinese buying representatives. The results indicate that spirituality is significantly related to perceptions about communication, commitment, and shared values for both sets of participants.</t>
@@ -22773,6 +23431,11 @@
       <c r="K553" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P553" t="inlineStr">
+        <is>
+          <t>The study refers to 'boundary-spanning representatives' but does not measure Boundary Spanning Behavior (BSB), focusing instead on spirituality. Additionally, the respondent acts as a proxy informant evaluating inter-firm relationships ('my firm'), and the study lacks a correlation matrix.. Verbatim Evidence: [Multiple reasons: Code 1 no BSB measure, Code 3 firm-level proxy informant]. Verbatim Evidence: "[Abstract] Within business-to-business relationship marketing, boundary-spanning representatives play a crucial role in establishing and maintaining positive relations between their organizations." "[Measures] The measures used in this study were all adaptations of existing measures in the literature." "[Measures] Spirituality was measured using questions adapted from Ashmos and Duchon’s (2000) spirituality scale and questions regarding “sense of community” from a scale in Milliman et al. (2003)." "[Appendix] 1. The relationship that my firm has with this company is something we are very committed to." "[Appendix] 2. The relationship that my firm has with this company deserves our firm’s maximum effort to maintain."</t>
         </is>
       </c>
     </row>
@@ -22787,6 +23450,16 @@
           <t>BSMA0551</t>
         </is>
       </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G554" t="inlineStr">
         <is>
           <t>Abstract             This article examines the frequently cited argument that coordination issues in humanitarian relief can be addressed more effectively with greater centralized authority and argues for a new conceptualization of aid delivery. The former position suggests a hierarchical, top‐down view of the humanitarian relief theater, while this analysis contends that the relief implementation structure may be better conceived as consisting of a network of loosely coupled semiautonomous organizations (Weick, 1976). A network approach allows examination of aid coordination dynamics at multiple levels of analysis: individual (professional and personal), organizational and interorganizational (operational), and strategic (structural/contextual). So viewed, factors that influence relief delivery, including contextual or strategic conditions and organization‐scale concerns, may either encourage or dissuade coordination across institutional boundaries. We argue that trust is a key precondition to coordination and that its extension is in turn conditioned by a number of strategic and operating‐level factors. We concentrate on operational coordination, as strategic concerns are not often open to the control of lone organizational actors. Our analysis rests in part on in‐depth interviews (each consisted of open‐ended questions and lasted an average of ninety to one hundred minutes) with a small sample of experienced international nongovernmental organization relief professionals who were engaged in aid efforts in Kosovo following the 1999 intervention by the North Atlantic Treaty Organization in that region.</t>
@@ -22810,6 +23483,11 @@
       <c r="K554" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P554" t="inlineStr">
+        <is>
+          <t>Qualitative study (interviews) lacking extractable quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [Abstract] Our analysis rests in part on in-depth interviews (each consisted of open-ended questions and lasted an average of ninety to one hundred minutes) with a small sample of experienced international nongovernmental organization relief professionals who were engaged in aid efforts in Kosovo following the 1999 intervention by the North Atlantic Treaty Organization in that region. [Methodology] To begin to explore empirically the utility of this conceptualization of relief efforts, we conducted lengthy open-ended interviews with a small sample (N = 5) of experienced INGO professionals and leaders who were deployed in the Kosovo region in the late summer of 1999. [Methodology] We tape-recorded and transcribed each interview. On average, each session lasted about ninety to one hundred minutes.</t>
         </is>
       </c>
     </row>
@@ -25122,6 +25800,12 @@
           <t>BSMA0613</t>
         </is>
       </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate the individual effects of boundary-spanning search from suppliers (supplier-side search (SS)). It is proposed that SS contributes to innovation ambidexterity (IA) and then business performance (BP). Further, this paper includes buyer–supplier relationships (BSRs) and competitive intensity (CI) as moderators to clarify boundary conditions.</t>
@@ -25145,6 +25829,11 @@
       <c r="K616" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P616" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -25159,6 +25848,12 @@
           <t>BSMA0614</t>
         </is>
       </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -25182,6 +25877,11 @@
       <c r="K617" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P617" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26602,6 +27302,12 @@
           <t>BSMA0653</t>
         </is>
       </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry. Using a multiyear sample of ﬁrms from the computer industry, we found that intra-industry trade-association ties of top managers led to the adoption of a resource-imitation strategy by late movers while extra-industry importation and professional-association ties led to the adoption of a resource-substitution strategy. We also found that trade association ties had a negative effect on the performance of late movers using resource-substitution, while top managers’ service on other ﬁrms’ boards had a positive inﬂuence on the performance of those ﬁrms. Our ﬁndings not only conﬁrm the importance of the role of ﬁt in strategy and performance, but they also highlight the importance of the management and control of boundary-spanning activities.</t>
@@ -26625,6 +27331,11 @@
       <c r="K656" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P656" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26639,6 +27350,16 @@
           <t>BSMA0654</t>
         </is>
       </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="G657" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate the effect of social undermining on the service employees’ boundary-spanning behavior though perceived ﬁt with job (P-J ﬁt). This study also aims to examine the moderating role of ethical climate in the relationship between service employees’ perceived ﬁt with job (P-J ﬁt) and boundary-spanning behavior.</t>
@@ -26662,6 +27383,11 @@
       <c r="K657" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P657" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26676,6 +27402,12 @@
           <t>BSMA0655</t>
         </is>
       </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr"/>
       <c r="G658" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this model is to explain how person – organization fit (P – O fit) and competitive intensity, conceptualized as a job resource and a job demand, respectively, ultimately affect the development of frontline employee boundary-spanning behavior (BSB).</t>
@@ -26699,6 +27431,11 @@
       <c r="K658" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P658" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26713,6 +27450,12 @@
           <t>BSMA0656</t>
         </is>
       </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr">
         <is>
           <t>Individuals in work teams frequently cross boundaries across teams, often by using information and communication technologies (ICTs). The current study investigates the effects of members’ boundary work and the visibility affordance of teams’ ICTs on Transactive Memory Systems (TMS) in teams. Survey data from 212 fulltime employees whose work hours were divided between multiple teams reveals that boundary spanning enhances the focal team’s TMS specialization and credibility and negatively inﬂuences TMS coordination. Additionally, boundary reinforcement positively affects TMS credibility and coordination. The visibility affordance has a direct positive effect on all three dimensions of TMS and a moderating effect for boundary reinforcement such that higher visibility overrides the positive direct effect of boundary reinforcement on TMS. These ﬁndings suggest that different types of boundary work contribute to different dimensions of TMS and that teams might consider prioritizing the use of ICTs with high visibility to enhance their TMS.</t>
@@ -26736,6 +27479,11 @@
       <c r="K659" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P659" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26750,6 +27498,16 @@
           <t>BSMA0657</t>
         </is>
       </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G660" t="inlineStr">
         <is>
           <t>When Leaders Use Self-Uncertainty Strategically: Consequences for Intergroup Leadership and Identity Confirmation Dynamics By Alison Young Claremont Graduate University: 2023 Framed by the social identity theory of leadership, one question that is beginning to receive attention is how intergroup leaders can lead across distinct subgroups and improve intersubgroup relations without provoking social identity-related concerns (e.g., subgroup identity distinctiveness threat). Past studies have found that leaders can use their rhetoric and boundary spanning behavior to meet their members’ identity needs and garner support. In addition, the self-uncertainty literature has suggested that leaders can strategically elevate and resolve members’ self-uncertainty through their rhetoric. The current research proposed that members who felt uncertain about their subgroup’s identity would have more favorable evaluations of the intergroup leader and perceptions of the out-subgroup if the leader confirmed their subgroup identity and/or was a blended boundary spanner. Members’ identity-uncertainty and subgroup identity validation have yet to be jointly examined in the context of intergroup leadership. Study 1 (N = 214) showed that those with high identity centrality had more positive leader evaluations and out-subgroup perceptions. Study 2 (N = 248) showed that those with greater subgroup identity-uncertainty who received a message from their leader that confirmed their subgroup identity had more positive out-subgroup perceptions; however, a person’s level of subgroup identity-uncertainty led to differential perceptions depending on the leader’s boundary spanning behavior. Implications and future directions are discussed.</t>
@@ -26773,6 +27531,11 @@
       <c r="K660" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P660" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26787,6 +27550,12 @@
           <t>BSMA0658</t>
         </is>
       </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>This study examines how deans and associate deans of a group from similar universities use networking. Specifically, we consider whether the deans, traditionally considered to perform boundary-spanning functions, make more use of external networking than do the associate deans, who are their subordinates. We examine the relationship between accuracy in perceiving a network and influence in the network. Finally, we consider the relationship between reports of networking outside the sample and influence within the sample. We find support for our first two propositions and raise several issues related to our final one.</t>
@@ -26810,6 +27579,11 @@
       <c r="K661" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P661" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26824,6 +27598,12 @@
           <t>BSMA0659</t>
         </is>
       </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr"/>
       <c r="G662" t="inlineStr">
         <is>
           <t>This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of noncore firms operating in the context of sustainable development. The dynamic nature of technological innovation, exacerbated by market flattening and the challenges posed by the COVID-19 pandemic, has compelled small and medium-sized enterprises (SMEs) to seek innovative breakthroughs. Cooperative innovation emerges as a strategic avenue for SMEs to mitigate risks and enhance their willingness to innovate. However, non-core firms often encounter technological and market disadvantages, hindering innovation efforts. This study explores how boundary-spanning knowledge search, which bridges the gap between non-core firms and the external environment, influences cooperative innovation. Furthermore, the research delves into the mediating role of both potential and actual absorptive capacity in the relationship between boundaryspanning knowledge search and cooperative innovation performance. Empirical findings indicate that boundary-spanning knowledge searches positively impact cooperative innovation, with technological and market knowledge searches yield significant results. Moreover, absorptive capacity exhibits a dual mechanism, directly influencing cooperative innovation and mediating the relationship between knowledge search and performance. This paper extends existing research by focusing on non-core firms within the sustainable development context, offering valuable insights for SMEs seeking innovative strategies. It also highlights the diverse pathways through which boundary-spanning knowledge search affects cooperative innovation. These findings offer practical implications for enhancing non-core firms’ innovation capabilities, including encouraging proactive knowledge search and developing absorptive capacity-inducing mechanisms through employee training and information platforms.</t>
@@ -26847,6 +27627,11 @@
       <c r="K662" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P662" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26861,6 +27646,12 @@
           <t>BSMA0660</t>
         </is>
       </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr"/>
       <c r="G663" t="inlineStr">
         <is>
           <t>This paper examines the influence of boundary-spanning knowledge search on cooperative innovation performance and explores the moderating role of innovation passion in Chinese firms. We collected 229 valid responses from Chinese firms participating in collaborative innovation projects and applied confirmatory factor analysis to test the reliability and validity of the constructs, multiple stepwise regressions to verify the direct effect, and the PROCESS macro to test the moderating effect. The results show that all three dimensions of boundary-spanning knowledge search (i.e. network capability, IT capability, and absorptive capacity) positively affect cooperative innovation performance. Harmonious innovation passion positively moderates the relationship between network capability and cooperative innovation performance. In contrast, compulsive innovation passion plays a negative moderating role in the relationship between absorptive capacity and cooperative innovation performance. This study further enriches and extends the theoretical framework of cooperative innovation performance by emphasizing the impact of the three dimensions of boundary-spanning knowledge search.</t>
@@ -26884,6 +27675,11 @@
       <c r="K663" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P663" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26935,6 +27731,12 @@
           <t>BSMA0662</t>
         </is>
       </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>Local government or better known as the local authority vested with the power to plan, develop, and regulate businesses in the area within its jurisdiction plays a significant role in creating a conducive environment for businesses to grow and flourish. In playing this role, employees in local authority must possess a certain degree of innovative work behavior. This paper reports on a study that investigated innovative work behavior orientation among employees of the local government. A total of 100 employees of a local city council responded to a self-administered questionnaire on innovative work behavior. The results revealed that respondents scored a moderate high orientation on the innovative work behavior scale.</t>
@@ -26958,6 +27760,11 @@
       <c r="K665" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P665" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28100,6 +28907,12 @@
           <t>BSMA0693</t>
         </is>
       </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr"/>
       <c r="G696" t="inlineStr">
         <is>
           <t>Purpose – Business model innovation (BMI) is an important channel of enterprise innovation, and BMI’s antecedents have attracted extensive attention. The purpose of this paper is to address a substantial gap in the extant literature by developing a moderate model to explain the effects of boundary-spanning search on BMI as well as whether and how innovative cognitive imprinting (ICI) and environmental dynamics (ED) affect the above relationship.</t>
@@ -28123,6 +28936,11 @@
       <c r="K696" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P696" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28137,6 +28955,12 @@
           <t>BSMA0694</t>
         </is>
       </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>Based on organizational learning theory, the influence of the transactive memory system of the top management team on business model innovation is discussed, as is the impact of different dimensions of boundary-spanning search on different business model innovation attributes when attention distribution is taken into account. Meanwhile, the moderating effects of environmental dynamism are considered. Regression and bootstrap analysis are used to test hypotheses. The results based on empirical research show that the transactive memory system has a positive effect on the dual attributes of business model innovation; acute boundary-spanning search and concentrated boundary-spanning search affect novelty-centered business model innovation and efficiencycentered business model innovation, respectively, and play mediating roles. Meanwhile, environmental dynamism positively moderates the relationship between acute boundary-spanning search and novelty-centered business model innovation, but negatively moderates the relationship between concentrated boundaryspanning and business efficiency-centered model innovation efficiency.</t>
@@ -28160,6 +28984,11 @@
       <c r="K697" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P697" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team/firm level of analysis. The study analyzes boundary spanning at the Top Management Team (TMT) / firm level, utilizing aggregated team data and firm-level referents ('We').. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28174,6 +29003,16 @@
           <t>BSMA0695</t>
         </is>
       </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G698" t="inlineStr">
         <is>
           <t>Due to their distinctive features, multiteam systems (MTSs) face significant coordination challenges—both within component teams and across the larger system. Despite the benefits of informal mechanisms of coordination for knowledge-based work, there is considerable ambiguity regarding their effects in MTSs. To resolve this ambiguity, we build and test theory about how interpersonal interactions among MTS members serve as an informal coordination mechanism that facilitates team and system functioning. Integrating MTS research with insights from the team boundary spanning literature, we argue that the degree to which MTS members balance their interactions with members of their own component team (i.e., intrateam interactions) and with the members of other teams in the system (i.e., interteam interactions) shapes team- and system-level performance. The findings of a multimethod study of 44 MTSs composed of 295 teams and 930 members show that as interteam interactions exceed intrateam interactions, team conflict arises and detracts from component team performance. At the system level, a balance between intrateam and interteam interactions enhances system success. Our findings advance understanding of MTSs by highlighting how informal coordination mechanisms enable MTSs to overcome their coordination challenges and address the unique performance tension between component teams and the larger system.</t>
@@ -28197,6 +29036,11 @@
       <c r="K698" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P698" t="inlineStr">
+        <is>
+          <t>Team and system-level analysis (N=268 teams, N=44 systems). Verbatim Evidence: [Abstract] The findings of a multimethod study of 44 MTSs composed of 295 teams and 930 members show that as interteam interactions exceed intrateam interactions, team conflict arises and detracts from component team performance. At the system level, a balance between intrateam and interteam interactions enhances system success. [Results] Tables 1 and 2 provide descriptive statistics for and intercorrelations among study variables at the team level and the system level, respectively. [Table 1] Notes: Entries are bivariate correlations. n=268 teams nested within 44 systems.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results part 1
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -9039,7 +9039,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Even though, over the last two decades, the boundaryless career concept has stimulated a wide theoretical debate, scholars have recently claimed that research on the competencies that are necessary for managing a cross-boundary career is still incomplete. Similarly, the literature on emotional and social competencies has demonstrated how they predict work performance across industries and jobs but has neglected their inﬂuence in explaining the individual’s mobility across boundaries and their impact on career success. This study aims to ﬁll these gaps by examining the effects of emotional and social competencies on boundaryless career and on objective career success. By analyzing a sample of 142 managers over a period of 8 years, we found evidence that emotional competencies positively inﬂuence the propensity of an individual to undertake physical career mobility and that career advancements are related to the possession of social competencies and depend on the adoption of boundaryless career paths. This study also provides a contribution in terms of the evaluation of the emotional and social competencies demonstrated by an individual and of the operationalization of the measurement of boundaryless career paths, considering three facets of the physical mobility construct (organizational, industrial, and geographical boundaries).</t>
@@ -9134,7 +9133,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>To explain how multistakeholder groups organize democratic deliberations about complex sustainability issues, organizational scholars have focused on the key role of deliberative capacity, which encompasses the dimensions of inclusiveness, authenticity and consequentiality. However, the tensions inherent to the search of these three dimensions have been overlooked. In this paper, we argue that focusing on how spaces for deliberation are designed can help one understand how to manage such tensions. We identified the boundary work practices that shape the design of deliberative spaces and generate deliberative capacity properties in a high-level expert group (HLEG) launched by the European Commission about sustainable finance regulation. Our results show how these boundary work practices help balance deliberative tensions. We advance deliberation studies by conceptualizing deliberative boundary work, explaining how deliberative capacity is spatially generated and showing how deliberative tensions are balanced. We also contribute to boundary work theory by making explicit the deliberative nature of configuring boundary work and showing its relevancy to regulatory settings.</t>
@@ -9182,7 +9180,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>Global offshoring has become a key strategy for international staffing, especially in the software industry. Global software teams engage in boundary spanning activities that may help MNEs achieve international connectivity and cope with external disruptions through their use of virtual work. However, offshoring IT professionals who bridge these boundaries in offshoring MNEs must contend with discontinuities, or perceived disruptions in expected communication flows, which impact their job satisfaction. Drawing on survey data from 193 professional consultants from an IT services offshoring MNE located primarily in Eastern Europe and working for a U.S. client, we test a model grounded in Organizational Discontinuity Theory. We find that potential discontinuities arising from the virtual work environment have no impact on the job satisfaction of offshoring IT professionals, but that those who experience team-level continuities of identification and shared vision are more satisfied with their jobs. Our findings suggest that virtual work may have become normalized such that it is not problematic in and of itself, and that fostering connectivity in boundary spanning global teams may be beneficial for MNEs. Our findings have important implications for MNEs managing disruptions created by global work arrangements as well as exogenous disruptions.</t>
@@ -9230,7 +9227,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>Acknowledgements: This research was funded by NSF grant #0422676 and #0726798 as well as support provided by the University of California, Irvine Center for Research on Information Technology in Organizations. The authors would like to acknowledge the helpful comments provided by Christopher Earley, Mark Griffin, John Mathieu, and Jone Pearce; assistance in data collection provided by Diaky Diaz, Christopher Reisdel and Bettina Wolf; and the generous time invested by all the film makers and film viewers who participated in the study.</t>
@@ -9273,6 +9269,12 @@
           <t>BSMA0185</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -9296,6 +9298,11 @@
       <c r="K188" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -9347,6 +9354,12 @@
           <t>BSMA0187</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -9370,6 +9383,11 @@
       <c r="K190" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11804,7 +11822,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -11852,7 +11869,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>Because of their boundary-spanning nature, manufacturers’ representatives frequently are involved in team selling. The results from a survey of 362 manufacturers’ representatives indicates that team selling is more likely to be used by manufacturers’ representatives when the customer faces a first-time buy of a complex product, when the information needs of the customer are great, when the account requires special treatment, and when a number of people are involved in the decision to buy. In addition, team selling is more likely when the potential sale is large for the representative firm and when the product is new to the representative’s product line.</t>
@@ -11900,7 +11916,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>With congeneric mergers, which involve firms with interrelated but not identical business lines that develop diverse products and services, a major challenge for organizations is the development of a common platform that fulfills similar business functions across multiple divisions. Through a field study of a postmerger common platform development initiative, we develop a framework that highlights how environmental and organizational contexts shape the process of common platform development (CPD). Our study provides an account of how the focal organization transitioned to a platform-based approach by achieving a balance between stable and flexible aspects of the common platform through negotiations among the divisions acquired through mergers and acquisitions. These negotiations were enabled through various boundary-spanning activities and the guided successive enrichment of boundary objects used in CPD process. European Journal of Information Systems (2015) 24(2), 159–177.</t>
@@ -11943,6 +11958,12 @@
           <t>BSMA0256</t>
         </is>
       </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>Two main targets of contemporary preferential innovation policy support, especially in Europe, are key enabling technologies (KETs) and innovation ‘missions’ focused on solving societal challenges. Both topics are associated with uniting disparate sets of capabilities, either by driving technology-based innovation into various application domains or by eliciting interdisciplinary and cross-sectoral solutions to urgent societal demands. In this study we assess to what extent pre-commercial R&amp;D collaborations span geographic and cognitive boundaries. We analyze firm-level tie formation in Dutch collaborative R&amp;D projects initiated in the period 2013–2018. Gravity models reveal that, while results for geographic proximity are mixed, some KET types are indeed related to projects in which cognitive proximity is significantly less relevant for tie formation. This contrasts with the findings for projects that retroactively received a mission label. Projects on health and care missions, and especially energy transition and sustainability missions, instead spur collaborations between cognitively proximate firms. The latter suggests that without additional policy intervention, such projects might interconnect similar rather than dissimilar knowledge bases. We conclude by discussing research and policy implications.</t>
@@ -11966,6 +11987,11 @@
       <c r="K259" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11980,6 +12006,12 @@
           <t>BSMA0257</t>
         </is>
       </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -12003,6 +12035,11 @@
       <c r="K260" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12017,6 +12054,12 @@
           <t>BSMA0258</t>
         </is>
       </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>This study investigated the effects of small business owner decision styles on the search for external assistance information, community information, and competitor information. Results confirmed the existence of decision style differences in selection of boundary spanning activities. A conclusion is drawn that small business owners use preferred sources for gathering information related to business operations, but need to utilize additional sources to ensure a comprehensive boundary spanning role. Ways to enhance boundary spanning activities are provided</t>
@@ -12040,6 +12083,11 @@
       <c r="K261" t="inlineStr">
         <is>
           <t>1990</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14964,6 +15012,12 @@
           <t>BSMA0336</t>
         </is>
       </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -14987,6 +15041,11 @@
       <c r="K339" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15105,7 +15164,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>Improving performance often requires creative ideas in extreme work settings like health care. Frontline workers are promising sources of creative ideas. The authors assert that their job dissatisfaction is positively associated with creativity in health care settings because negative emotion spurs creativity when tied to engaging work and that characteristics such as shorter tenure, greater role centrality, and high boundary spanning can strengthen this relationship. The authors find supporting evidence in data on ideas generated over 18 months by health professionals in 12 clinics.</t>
@@ -15576,7 +15634,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>Boundary spanning has been proven to have positive implications for innovation performance; yet, some individuals are less boundary-spanning than others. Drawing on the attachment theory and organizational support theory, this study develops a multi-level theoretical model to investigate how individuals’ attachment insecurity influences boundaryspanning behavior through self-efficacy and the moderating role of organizational support climate. To validate the proposed model, we adopted a survey research, and collected data from NPD project teams in China. The results revealed that both insecure attachment styles were associated with lower levels of individual boundary-spanning behavior, and self-efficacy partially mediated these relationships. Moreover, organizational support climate played a moderating role in the relationship between attachment anxiety and boundary-spanning behavior. With a high level of support climate, the negative impact of attachment anxiety on boundary-spanning behavior was weakened. This elucidates the role of individual affective motivation and team shared perceptions in shaping individual externally focused behavior.</t>
@@ -15708,6 +15765,12 @@
           <t>BSMA0352</t>
         </is>
       </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -15731,6 +15794,11 @@
       <c r="K355" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P355" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16552,6 +16620,12 @@
           <t>BSMA0374</t>
         </is>
       </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>Based on the social identity theory, this study investigates whether and how employee perceptions of corporate environmental behavior (CEB) influence the realization of an organization's internal value. Using employees' organizational citizenship behavior (OCB) as a direct agent for corporate internal value, the current study constructs a theoretical model of perceived CEB and OCB, with work meaningfulness and person–organization (P-O) value fit serving as mediator and moderator, respectively. After analyzing 235 questionnaire samples, we discovered that the perceived CEB positively influenced OCB via work meaningfulness and that this positive effect was strengthened by a greater P-O value fit. These findings suggest that in the process of motivating employees to implement OCB, firms should address the significance of internal driving roles of work meaningfulness and boundary-spanning roles of P-O value fit in order to enhance corporate internal value and correct managers' misconceptions about the value of CEB.</t>
@@ -16575,6 +16649,11 @@
       <c r="K377" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P377" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16757,6 +16836,12 @@
           <t>BSMA0379</t>
         </is>
       </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>Building on the “loose coupling” logic, this study examines the importance of boundary spanners' shared perceptions of procedural justice in cross-cultural cooperative alliances. I argue that alliance profitability is higher when both parties perceive high rather than low procedural justice. Profitability is also higher when both parties' perceptions are high than when one party perceives high procedural justice but the other perceives low procedural justice. Shared justice perceptions become even more important for alliance profitability when the cultural distance between partners is high or when the industry of operation is uncertain. Analysis of 124 cross-cultural alliances in China supports these propositions.</t>
@@ -16780,6 +16865,11 @@
       <c r="K382" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16794,6 +16884,12 @@
           <t>BSMA0380</t>
         </is>
       </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>This study extends research on strategic alliances by exploring independent and combined effects of distributive, procedural, and interactional justice in these alliances. An integrated framework links cooperation payoffs with organizational justice as perceived by boundary-spanning alliance executives, through whom justice perceptions become parent actions. Analysis of 127 alliances demonstrates that when goal differences between parties are high, the joint effect on alliance performance of procedural and distributive justice is significantly positive. When interactional justice is high, procedural justice exerts a stronger performance effect. This perspective enriches alliance research, especially regarding procedural formalization, incentive structure, and interparty attachment.</t>
@@ -16817,6 +16913,11 @@
       <c r="K383" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16831,6 +16932,12 @@
           <t>BSMA0381</t>
         </is>
       </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -16854,6 +16961,11 @@
       <c r="K384" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18047,6 +18159,12 @@
           <t>BSMA0413</t>
         </is>
       </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -18070,6 +18188,11 @@
       <c r="K416" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18272,6 +18395,12 @@
           <t>BSMA0418</t>
         </is>
       </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>This dissertation investigates factors that influence efforts by lower-level employees to initiate organizational change and innovation from the bottom up. Specifically, I attempt to reconcile competing theories regarding the effects of structural and social integration on individual innovation efforts. One theoretical view posits that integration provides information, ideas, and motivation necessary for innovation. An alternative view is that integration constrains individuals and routines, and thereby hinders innovation efforts. Drawing on both theoretical perspectives, I predict the effects of distinct types of structural integration (eg, centralization, cross-unit integration, boundary spanning) and social integration determinants (eg, geographic dispersion, decision process involvement, workplace network size) on the likelihood of individual innovation efforts among lower-level employees. I also consider the effects of interactions of social and structural integration with individual characteristics (ie, personality, and experience) on innovation efforts. I test these predictions using survey data collected from interns and supervisors in the context of MBA and undergraduate internships. Analyses demonstrate that several aspects of structural integration do influence the levels of individual innovation efforts. For example, centralization and boundary spanning levels of the work unit have inverse U-shaped relationships with the level of innovation effort. These findings suggest that for certain types of innovation, structural integration can constrain efforts at the extremes (very high or low) and facilitate efforts at modest levels of integration. Predicted social integration effects are largely non-significant, suggesting the need for further consideration and alternative empirical tests of such effects. Nevertheless, the structural integration findings reaffirm the need to bring together both theoretical perspectives (ie, the view that integration fosters innovation efforts, and the alternative view that isolation and independence are necessary for innovation). By empirically demonstrating that distinct types of integration have unique, yet theoretically consistent effects on several different classes of individual innovation efforts (both process and strategy related), this study contributes to efforts to reconcile these competing theories. Additionally, this research enhances our understanding of a class of little-studied behaviors that play a potentially important role in autonomous strategic change and organizational learning.</t>
@@ -18295,6 +18424,11 @@
       <c r="K421" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18507,7 +18641,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
           <t>Recent research has emphasized cross functional integration as a key facilitator of success in new product development (NPD) projects. This dissertation developed and tested a model using supply chain integration as a key enabler influencing both planning of the new product and execution of the development process in NPD projects. Supply chain integration was operationalized to include cross functional (for example, between design and manufacturing) and boundary spanning integration mechanisms (such as supplier integration). Product concept effectiveness (a construct capturing the planning of the new product), and development process performance (a construct measuring the execution of new product development process) were theorized to influence overall project success. Hypotheses drawn from this framework were tested on a multi-industry sample (electronics, communications, semiconductors, and computers) of firms. Data analysis was conducted using regression analyses, partial correlations, confirmatory factor analyses and structural equation modeling.</t>
@@ -18592,7 +18725,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
           <t>Mentoring is a valuable resource that enhances outcomes like career success. Applying conservation of resources theory, we examine the interaction effects of workers’ management aspirations and lengthy career interruption(s) on the mentoring-career success relationship. Utilizing 259 older professional workers, we test these relationships with both cross-sectional and time-separated data. Although the pattern of results was similar when comparing the crosssectional data to the time-separated data, we found that relationships were stronger within the cross-sectional data, resulting in the support of two additional hypotheses. With the timeseparated data, we found evidence of a three-way interaction. Speciﬁcally, mentoring is more valuable for the perceived career success of workers with higher management aspirations who had not experienced a lengthy career interruption than it is for workers with higher management aspirations who had experienced a lengthy career interruption or for workers with lower management aspirations regardless of whether they had experienced a career interruption.</t>
@@ -18635,6 +18767,16 @@
           <t>BSMA0426</t>
         </is>
       </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G429" t="inlineStr">
         <is>
           <t>Rudy Moenaert, William Souder, Arnoud De Meyer, and Dirk Deschoolmeester report the results of their study of forty technologically innovative Belgian companies to examine the interaction between marketing and R&amp;D. They studied one commercially successful and one commercially unsuccessful technological product innovation project in each participating company and collected data from one marketing and one R&amp;D respondent per project. Communication flows between marketing and R&amp;D are increased under conditions involving formalization of projects, decentralization, positive inter-functional climate, and role flexibility.</t>
@@ -18658,6 +18800,11 @@
       <c r="K429" t="inlineStr">
         <is>
           <t>1994</t>
+        </is>
+      </c>
+      <c r="P429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18672,6 +18819,12 @@
           <t>BSMA0427</t>
         </is>
       </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>Urban metabolism approaches are increasingly becoming relevant in providing pathways to sustainable development. The ways through which urban green infrastructures are planned and designed can influence resource flows in cities. Yet, little is known about the agency and contributions of landscape architects and spatial planners as curators of urban greenery, in facilitating circular resource flows, and accelerating the transition to a circular economy. This paper offers an empirical inquiry into the understanding and use of metabolic approaches in spatial planning and design practices. Through a multi-method approach and the use of boundary spanning as an analytical lens, we identify different modes of agency of spatial practitioners in enhancing resource efficiency across the life stages of urban landscape projects. Results show that while the ‘urban metabolism’ concept is not widely used by practitioners, its relevance to planning and designing green infrastructure for sustainable resource flows is well understood. Additionally, we highlight existing barriers including policy constraints in engaging with metabolic approaches and offer recommendations to facilitate a resource-sensitive turn in planning and designing urban landscapes. This study highlights important contributions of design practice to an expanding discourse of urban metabolism, including policy reforms for enabling circular resource flows in cities.</t>
@@ -18695,6 +18848,11 @@
       <c r="K430" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21137,7 +21295,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>Abstract             In this study, we analyse the discursive strategies of professionalization used by psychology in Spain during its professionalization phase in the health sector in the early twenty-first century. Our primary focus is the conflict with political regulators and other healthcare professions after the Ley de Ordenación de Profesiones Sanitarias (Healthcare Professions Act) came into effect, since this Act calls into question the extent to which psychology can be viewed as health care. We use discourse analysis to determine the discursive structure of the conflict, which has an interprofessional dimension, as well as the professionalization and social closure strategies of psychology within the framework of professional relationships (boundary work). We argue that understanding this conflict requires viewing it as part of the European and international regulation context of healthcare professions. Highlighted in the analysis is the emergence of two psychology discourses divided into four modes of enunciation (professionalizing, cultural, scientific, and political–economic). Among other aspects, the conclusions focus on the dual interprofessional and intraprofessional nature of the conflict and evidence of a dual closure in psychology. The latter’s professionalization strategies in the sector occasionally resemble those employed by nursing, although at other times they are similar to those followed by some paramedical professions.</t>
@@ -21180,6 +21337,16 @@
           <t>BSMA0493</t>
         </is>
       </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G496" t="inlineStr">
         <is>
           <t>No Abstract</t>
@@ -21203,6 +21370,11 @@
       <c r="K496" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P496" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21217,6 +21389,12 @@
           <t>BSMA0494</t>
         </is>
       </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -21240,6 +21418,11 @@
       <c r="K497" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P497" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -22636,6 +22819,16 @@
           <t>BSMA0532</t>
         </is>
       </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G535" t="inlineStr">
         <is>
           <t>Information processing theory suggests the need for different types of integration mechanisms in R &amp; D project management depending on levels of uncertainty and equivocality. This paper examines the use of these mechanisms and their links to project performance in a sample of 121 R &amp; D projects in a large research laboratory. Overall, it is found that formal leadership, planning and process specification, and to a lesser extent information technology use are related to project performance while the positive effects of horizontal structures are apparently balanced out by their costs. The integration mechanisms studied act on performance partly through their effect on horizontal communications. Modest support was found for the contingency hypotheses derived from information processing theory. It appears that managers adjusted their use of horizontal structures, planning and process specification, and informal leadership to project uncertainty but not to project equivocality. The positive effects of horizontal communications on performance were found to be greatest under high project equivocality as would be predicted by information processing arguments. Moreover, with the exception of formal leadership, the use of integration mechanisms did not enhance performance in contexts of low uncertainty and low equivocality. q 2000 Elsevier Science B.V. All rights reserved.</t>
@@ -22659,6 +22852,13 @@
       <c r="K535" t="inlineStr">
         <is>
           <t>2000</t>
+        </is>
+      </c>
+      <c r="P535" t="inlineStr">
+        <is>
+          <t>Excluded because the unit of analysis is the project (N=121) and the variables measure team/project-level integration mechanisms rather than individual-level boundary spanning behavior.. Verbatim Evidence: [Methodology] &lt;The sample consisted of 121 different R&amp;D projects from 13 research units&gt; [Methodology] &lt;Respondents usually completed the questionnaire for two projects&gt; [Appendix A] &lt;Horizontal structures: `` To what extent were the following decision-making mecha -
+nisms used? ''
+Steering committee&gt;</t>
         </is>
       </c>
     </row>
@@ -22777,6 +22977,16 @@
           <t>BSMA0535</t>
         </is>
       </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G538" t="inlineStr">
         <is>
           <t>Manufacturers are often placing their intellectual property (IP) at risk by outsourcing to suppliers in countries with weak IP rights. Thus, understanding how to safeguard their IP from poaching, which is a supplier's unauthorized use of a buyer's proprietary information, is of critical practical importance for manufacturers that outsource to suppliers in countries with weak IP rights. To investigate this phenomenon, we use dyadic data from globally dispersed manufacturer–supplier relationships to examine how the IP rights of a supplier's location affects poaching and how IP rights influence the effectiveness of two transactional characteristics—supplier idiosyncratic investments and media‐rich communication—on poaching. We examine these two transaction characteristics because they are representative of two forms of safeguards which create self‐enforcing agreements that do not require legal enforcement—economic and relational. We find that the strength of IP rights not only has a direct effect on poaching, but it also influences the relationships for both transaction characteristics. Intriguingly, when IP rights are weak, we find that not only are supplier idiosyncratic investments less effective in reducing poaching, but increases in these investments are associated with an increase in poaching. This finding illustrates that the strength of IP rights is a determinant of the degree to which supplier idiosyncratic investments are transaction specific. For suppliers in countries with weak IP rights, media‐rich communication is found to be more effective in reducing poaching. This finding illustrates the importance of manufacturers’ boundary spanners in building relationships with suppliers in countries with weak IP rights.</t>
@@ -22800,6 +23010,11 @@
       <c r="K538" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P538" t="inlineStr">
+        <is>
+          <t>Excluded due to multiple reasons: the unit of analysis is the manufacturer-supplier dyad (Code 3), and the boundary-spanning proxy merely measures communication frequency (Code 1).. Verbatim Evidence: [4.1. Data Collection and Sample Characteristics] "The unit of analysis for this study is a manufacturer (buyer)–supplier dyad." [4.1. Data Collection and Sample Characteristics] "The respondents answered questions regarding the overall relationship between the two firms, including listing all of the buyer plant locations that received products from the supplier." [Appendix A: Survey Questions] "Media-Rich Communication (Source = Buyer) (1 = Never; 2 = Annually; 3 = Semi-annually; 4 = Quarterly; 5 = Monthly; 6 = Weekly; 7 = Daily) How often do personnel from your firm and &lt;&lt;SUPPLIER&gt;&gt; communicate using the following methods. . . PC1 Face-to-face PC3 Telephone"</t>
         </is>
       </c>
     </row>
@@ -23735,6 +23950,16 @@
           <t>BSMA0554</t>
         </is>
       </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G557" t="inlineStr">
         <is>
           <t>Extant research has largely ignored the phenomenon of interorganizational teams, which consist of members from both supplier and customer companies. This study examines the degree to which team interorganizationality influences team performance in a business-to-business context. On the basis of resource-dependence theory and boundary theory, the author argues that team interorganizationality positively influences team effectiveness, particularly when uncertainty is high. The hypotheses testing is based on multiple informant data collected from members and leaders of 225 teams in various industries. The results show the positive influence of team interorganizationality on team effectiveness. In addition, uncertainty-related moderator variables (company-related, market-related, and technological uncertainty) strengthen the link between team interorganizationality and team effectiveness.</t>
@@ -23758,6 +23983,11 @@
       <c r="K557" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P557" t="inlineStr">
+        <is>
+          <t>Team level of analysis (N = 161 teams) measuring team interorganizationality rather than individual-level boundary spanning behavior.. Verbatim Evidence: [Framework and Hypotheses] "The unit of analysis for this study was a customer-related team in a B2B setting." [Sample and Data Collection] "The final sample therefore contained 161 teams, each of which provided at least two team-member evaluations and one team-leader evaluation, for 691 total respondents, or an average number of respondents per team of 4.29." [Measure Development and Assessment] "The results supported the plan to average data obtained from respondents within a team."</t>
         </is>
       </c>
     </row>
@@ -23772,6 +24002,16 @@
           <t>BSMA0555</t>
         </is>
       </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G558" t="inlineStr">
         <is>
           <t>Purpose – Boundary-spanning exploration through establishing alliances is an effective strategy to explore technologies beyond local search in innovating firms. The purpose of this paper is to argue that it is useful to make a distinction in boundary-spanning exploration between what a firm learns from its alliance partners (explorative learning from partners (ELP)) and what it learns from other organisations (explorative learning from non-partners (ELN)).</t>
@@ -23795,6 +24035,11 @@
       <c r="K558" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P558" t="inlineStr">
+        <is>
+          <t>Firm-level analysis using patent and alliance database data instead of individual employee survey data; does not measure interpersonal boundary spanning behavior [Code 1, Code 2, &amp; Code 3].. Verbatim Evidence: [5. Data and variables] &lt;We constructed a panel data set covering the population of ASIC producers over the period 1987–2000.&gt; [5. Data and variables] &lt;In order to measure the technological knowledge base of the ASIC producers, we draw on patent data from the US Patent and Trademark Office.&gt; [5.3 Variables] &lt;ELP is calculated as the sum of patents successfully applied for by the focal firm in each year[3], which have at least one citation to its alliance partners’ prior patents, but no citations to its own prior patents.&gt;</t>
         </is>
       </c>
     </row>
@@ -23807,6 +24052,16 @@
       <c r="B559" t="inlineStr">
         <is>
           <t>BSMA0556</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
         </is>
       </c>
       <c r="G559" t="inlineStr">
@@ -23843,6 +24098,11 @@
       <c r="K559" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P559" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] Non-primary study (Literature Review). Verbatim Evidence: [Abstract] This chapter reviews literatures from organizational psychology and management to assess the impact of member diversity on project team performance. [Literature Review on the Two Types of Functional Diversity in Project Teams] A total of 22 empirical studies that examined the two functional diversity categories in the project team context were identified (see Table 13.1 for the summary of the identified studies).</t>
         </is>
       </c>
     </row>
@@ -26058,7 +26318,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr">
         <is>
           <t>This study utilizes network exploitation and exploration theory to distinguish the exploitative and exploratory mechanisms (government support and boundary-spanning learning, respectively) that convert political ties into firm innovativeness. It also examines the moderating roles market uncertainty plays in how political ties influence firm innovativeness. An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness. Market uncertainty negatively moderates the impact of political ties on boundary-spanning learning but does not significantly moderate their impact on government support. Moreover, market uncertainty moderates the impact of government support on firm innovativeness negatively but moderates the impacts of boundary-spanning learning on firm innovativeness positively. This study theorizes two mediating factors for how firms exploit and explore their political ties to increase their innovativeness and enriches the knowledge of how market uncertainty affects the relationship between political ties and innovation.</t>
@@ -26106,7 +26365,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F619" t="inlineStr"/>
       <c r="G619" t="inlineStr">
         <is>
           <t>Organizational values and beliefs significantly influence employee decision making and behavior and manifest themselves as multiple climates existing within a single organization. A subset of organizational climate is an ethical climate, embodying normative values and beliefs involving moral issues shared by the employees of the organization. Reseachers have found multiple ethical climates present in an organization.</t>
@@ -26154,7 +26412,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F620" t="inlineStr"/>
       <c r="G620" t="inlineStr">
         <is>
           <t>Boundary‐spanning communication has been found to be important to various types of organizations and groups as a source of new information and awareness of environmental changes. Although the importance of formal, public channels in building the knowledge base of a field has long been recognized, most studies of boundary‐spanning activity have been limited to direct, personal (informal) communication. This study examines both informal and formal communication patterns of three groups in order to determine whether, in fact, a variety of media are used in boundary‐spanning communication. The groups selected were the members of three professions which fill intermediary positions between the creators and consumers of cultural products; one located in academia and two in the private sector. Major findings were that: (1) A boundary‐spanning structure linking 82.2% of the survey respondents was composed of both informal and formal media. (2) The professions differed in which type of channel was most heavily used, but were similar in their perceptions of the importance of the channels. (3) Individuals central to the informal part of the structure were also more likely to use the formal parts of the structure. (4) Boundary‐spanning media were among the five most frequently cited media for all three of the professions.</t>
@@ -26234,6 +26491,12 @@
           <t>BSMA0619</t>
         </is>
       </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -26257,6 +26520,11 @@
       <c r="K622" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P622" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -27878,6 +28146,12 @@
           <t>BSMA0661</t>
         </is>
       </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -27901,6 +28175,11 @@
       <c r="K664" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P664" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28036,6 +28315,12 @@
           <t>BSMA0665</t>
         </is>
       </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr"/>
       <c r="G668" t="inlineStr">
         <is>
           <t>Innovation is a key driver for organizations to survive and thrive in increasingly hyper-competitive markets. This study investigates the effects of boundary-spanning search on innovation capability. Speciﬁcally, it examines the mediating and moderating effects of network ties and absorptive capacity on boundary-spanning search and innovation in Chinese companies. We constructed a theoretical model of an organization’s boundary-spanning search and innovation capability and distributed a survey questionnaire to a sample of speciﬁc industries with upstream and downstream relations in Sichuan Province in China for their responses. Results from the study reveal that boundary-spanning search has a positive and signiﬁcant impact on innovation capability as well as a positive moderating effect on absorptive capacity and innovation capability. This paper shows that enterprises need to continuously focus on exploring networking opportunities in direct and indirect ways to get access to effective ﬂow and diffusion of resources, which in turn can enhance innovation capability.</t>
@@ -28059,6 +28344,11 @@
       <c r="K668" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P668" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28073,6 +28363,12 @@
           <t>BSMA0666</t>
         </is>
       </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>Due to their complexity and high social impact, urban infrastructure projects often face challenges in managing the design decision-making processes across disparate disciplinary and knowledge domain boundaries. This paper introduces the notion of design boundary dynamics to describe the various cross-boundary coordination phenomena associated with organising the design of infrastructure projects. Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project. Findings illustrate the entangled processes, through which the disciplinary, knowledge-domain and stage-based design boundaries emerged as a result of unfolding project practices. Paper identifies the key role of resource allocation constraints, path dependency of project decisions, and problem-solving nature of design and concludes with strategic recommendations for upstream operational integration to mitigate the impact of design boundary dynamics on infrastructure projects.</t>
@@ -28096,6 +28392,11 @@
       <c r="K669" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P669" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28184,6 +28485,12 @@
           <t>BSMA0669</t>
         </is>
       </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -28207,6 +28514,11 @@
       <c r="K672" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P672" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29236,6 +29548,12 @@
           <t>BSMA0696</t>
         </is>
       </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr"/>
       <c r="G699" t="inlineStr">
         <is>
           <t>Although the information‐seeking literature has tended to focus upon the selection and use of inanimate objects as information sources, this research follows the more recent trend of investigating how individuals evaluate and use interpersonal information sources. By drawing from the structural, relational, and cognitive elements of social capital theory to inform antecedents to information quality and source accessibility, a research model is developed and tested. For interpersonal information sources, information quality is the key determinant of source use. Perceptions of information quality and accessibility of an interpersonal source are shown to be influenced by boundary spanning, transactive memory, and content type. Implications and prescriptions for future research are discussed.</t>
@@ -29259,6 +29577,11 @@
       <c r="K699" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P699" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29278,7 +29601,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
         <is>
           <t>This study adopts a temporal perspective to investigate how boundary spanners can increase the inflow of external knowledge by engaging with both external and internal parties. We add to prior work on knowledge transfer by shifting the focus from engagement levels to investigating engagement dynamics, especially the degree of switching between external and internal engagement across consecutive time periods. Drawing from a cognitive perspective, we argue that switching strongly between engagement types is associated with a segmented knowledge structure that enables quick and efficient categorical processing when knowledge can simply be “channeled” from source to recipient units. In contrast, weak or no switching is associated with a blended knowledge structure and more reflective processing, which is particularly helpful when knowledge transfer requires more translation and transformation. Correspondingly, we adopt a contingency perspective and theorize that the cognitive advantages associated with stronger versus weaker switching weigh differently, contingent on the stickiness of knowledge to be transferred and the nature of boundary-spanning activities that vary in importance over time. Fixed effects models of eight waves of original survey data reveal that, in line with our theorizing, the association between switching and knowledge transfer becomes increasingly negative (1) the more boundary spanners access knowledge that is transspecialist in nature, (2) the greater the organizational distance between source and recipient units, and (3) in later phases of the boundary-spanning process.</t>
@@ -29395,6 +29717,12 @@
           <t>BSMA0700</t>
         </is>
       </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr"/>
       <c r="G703" t="inlineStr">
         <is>
           <t>We propose and test a framework that describes the relationship between network structures and job performance. We provide an integration of the current conceptualizations of social capital as they pertain to job performance outcomes by taking a multi-dimensional view of job performance. We break down job performance into creativity, decision-making, task execution, and teamwork, and distinguish the effect of structural holes within and across the organizational boundary on these four job performance domains. In an analysis of 318 managers, we ﬁnd that networks rich in structural holes that cross the organizational boundary had a positive association with creativity and decision-making, whereas networks with few structural holes within the organization had a positive association with task execution and teamwork. We discuss the theoretical implications for integrating the social capital, boundary spanning, and network structure literatures, as well as the practical beneﬁts of giving much more precise advice to managers and employees regarding how to use networks to improve performance at work.</t>
@@ -29418,6 +29746,11 @@
       <c r="K703" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P703" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results part 2
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -9274,7 +9274,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -9359,7 +9358,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -10290,6 +10288,12 @@
           <t>BSMA0212</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Innovation is considered the engine for firm growth. Especially innovations, through recombining seemingly unrelated knowledge streams, can have groundbreaking impact and lead to sustained competitive advantage. To generate such innovation, firms often need to go beyond their existing technological or geographical boundaries to identify and integrate novel knowledge elements. This article refers to firms’ knowledge activities of drawing upon distant knowledge (i.e., knowledge from dissimilar technological domains or distant geographical regions) to create novel technological solutions, as innovation through boundary spanning. Aiming to investigate the roles of information technology (IT) in facilitating innovation through boundary spanning, we collected data from the pharmaceutical industry over a six-year period to test the research model. The data analysis results indicate that IT supports boundary-spanning activities in firm innovation and different IT-enabled knowledge capabilities affect boundary-spanning innovation differently.</t>
@@ -10313,6 +10317,11 @@
       <c r="K215" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10364,6 +10373,12 @@
           <t>BSMA0214</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -10387,6 +10402,11 @@
       <c r="K217" t="inlineStr">
         <is>
           <t>1999</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11963,7 +11983,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>Two main targets of contemporary preferential innovation policy support, especially in Europe, are key enabling technologies (KETs) and innovation ‘missions’ focused on solving societal challenges. Both topics are associated with uniting disparate sets of capabilities, either by driving technology-based innovation into various application domains or by eliciting interdisciplinary and cross-sectoral solutions to urgent societal demands. In this study we assess to what extent pre-commercial R&amp;D collaborations span geographic and cognitive boundaries. We analyze firm-level tie formation in Dutch collaborative R&amp;D projects initiated in the period 2013–2018. Gravity models reveal that, while results for geographic proximity are mixed, some KET types are indeed related to projects in which cognitive proximity is significantly less relevant for tie formation. This contrasts with the findings for projects that retroactively received a mission label. Projects on health and care missions, and especially energy transition and sustainability missions, instead spur collaborations between cognitively proximate firms. The latter suggests that without additional policy intervention, such projects might interconnect similar rather than dissimilar knowledge bases. We conclude by discussing research and policy implications.</t>
@@ -12011,7 +12030,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -12059,7 +12077,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>This study investigated the effects of small business owner decision styles on the search for external assistance information, community information, and competitor information. Results confirmed the existence of decision style differences in selection of boundary spanning activities. A conclusion is drawn that small business owners use preferred sources for gathering information related to business operations, but need to utilize additional sources to ensure a comprehensive boundary spanning role. Ways to enhance boundary spanning activities are provided</t>
@@ -12102,6 +12119,12 @@
           <t>BSMA0259</t>
         </is>
       </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>The influence of boundary spanning roles on strategic decision-making was explored in a field study in fifteen organizations. Results support the importance of boundary spanning roles in the strategic decision-making process and the relationship of technology to the differential strategic decision-making influence of different boundary spanning roles.</t>
@@ -12125,6 +12148,11 @@
       <c r="K262" t="inlineStr">
         <is>
           <t>1984</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12139,6 +12167,12 @@
           <t>BSMA0260</t>
         </is>
       </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>The impact of perceived environmental demands on the roles and job satisfaction of the school psychologist in rural school systems was explored. Superintendents rated their perceptions of the community context and the psychologist’s involvement in interagency linking functions. School psychologists rated their performance of boundary-spanning functions and their job perceptions. Results indicated that certain perceived environmental pressures are related to the performance of boundaryspanning activities. Those who performed boundary-spanning functions are more satisfied with their jobs and more influential in determining their roles.</t>
@@ -12162,6 +12196,11 @@
       <c r="K263" t="inlineStr">
         <is>
           <t>1984</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13424,6 +13463,12 @@
           <t>BSMA0294</t>
         </is>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -13447,6 +13492,11 @@
       <c r="K297" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15017,7 +15067,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -15728,6 +15777,12 @@
           <t>BSMA0351</t>
         </is>
       </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>From a knowledge-based perspective, this paper highlights the need for a framework linking perceived competition of the industry and ﬁrms’ strategic location choices of external knowledge search and examines whether the perceived competition increases the propensity of cluster ﬁrms to search more widely from extra-cluster knowledge sources than intra-cluster knowledge sources. Furthermore, we emphasise that cluster ﬁrms with varying degrees of tacitness in their knowledge base might respond to such competition diﬀerently when conducting external knowledge search activities. Using a sample of 310 cluster ﬁrms in the Zhejiang Province of China, we ﬁnd that the cluster ﬁrm would increase the propensity for more geographic boundary-spanning search relative to local search while under the pressure of competition. Moreover, the positive relationship between perceived competition and the propensity towards geographic knowledge search is weaker when the tacitness of the cluster ﬁrm’s knowledge base is higher. The ﬁndings contribute to the understanding of the relationship between competition and the choice of location strategies in external knowledge search.</t>
@@ -15751,6 +15806,11 @@
       <c r="K354" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P354" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15770,7 +15830,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -16625,7 +16684,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>Based on the social identity theory, this study investigates whether and how employee perceptions of corporate environmental behavior (CEB) influence the realization of an organization's internal value. Using employees' organizational citizenship behavior (OCB) as a direct agent for corporate internal value, the current study constructs a theoretical model of perceived CEB and OCB, with work meaningfulness and person–organization (P-O) value fit serving as mediator and moderator, respectively. After analyzing 235 questionnaire samples, we discovered that the perceived CEB positively influenced OCB via work meaningfulness and that this positive effect was strengthened by a greater P-O value fit. These findings suggest that in the process of motivating employees to implement OCB, firms should address the significance of internal driving roles of work meaningfulness and boundary-spanning roles of P-O value fit in order to enhance corporate internal value and correct managers' misconceptions about the value of CEB.</t>
@@ -16841,7 +16899,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>Building on the “loose coupling” logic, this study examines the importance of boundary spanners' shared perceptions of procedural justice in cross-cultural cooperative alliances. I argue that alliance profitability is higher when both parties perceive high rather than low procedural justice. Profitability is also higher when both parties' perceptions are high than when one party perceives high procedural justice but the other perceives low procedural justice. Shared justice perceptions become even more important for alliance profitability when the cultural distance between partners is high or when the industry of operation is uncertain. Analysis of 124 cross-cultural alliances in China supports these propositions.</t>
@@ -16889,7 +16946,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>This study extends research on strategic alliances by exploring independent and combined effects of distributive, procedural, and interactional justice in these alliances. An integrated framework links cooperation payoffs with organizational justice as perceived by boundary-spanning alliance executives, through whom justice perceptions become parent actions. Analysis of 127 alliances demonstrates that when goal differences between parties are high, the joint effect on alliance performance of procedural and distributive justice is significantly positive. When interactional justice is high, procedural justice exerts a stronger performance effect. This perspective enriches alliance research, especially regarding procedural formalization, incentive structure, and interparty attachment.</t>
@@ -16937,7 +16993,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -18164,7 +18219,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -18400,7 +18454,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>This dissertation investigates factors that influence efforts by lower-level employees to initiate organizational change and innovation from the bottom up. Specifically, I attempt to reconcile competing theories regarding the effects of structural and social integration on individual innovation efforts. One theoretical view posits that integration provides information, ideas, and motivation necessary for innovation. An alternative view is that integration constrains individuals and routines, and thereby hinders innovation efforts. Drawing on both theoretical perspectives, I predict the effects of distinct types of structural integration (eg, centralization, cross-unit integration, boundary spanning) and social integration determinants (eg, geographic dispersion, decision process involvement, workplace network size) on the likelihood of individual innovation efforts among lower-level employees. I also consider the effects of interactions of social and structural integration with individual characteristics (ie, personality, and experience) on innovation efforts. I test these predictions using survey data collected from interns and supervisors in the context of MBA and undergraduate internships. Analyses demonstrate that several aspects of structural integration do influence the levels of individual innovation efforts. For example, centralization and boundary spanning levels of the work unit have inverse U-shaped relationships with the level of innovation effort. These findings suggest that for certain types of innovation, structural integration can constrain efforts at the extremes (very high or low) and facilitate efforts at modest levels of integration. Predicted social integration effects are largely non-significant, suggesting the need for further consideration and alternative empirical tests of such effects. Nevertheless, the structural integration findings reaffirm the need to bring together both theoretical perspectives (ie, the view that integration fosters innovation efforts, and the alternative view that isolation and independence are necessary for innovation). By empirically demonstrating that distinct types of integration have unique, yet theoretically consistent effects on several different classes of individual innovation efforts (both process and strategy related), this study contributes to efforts to reconcile these competing theories. Additionally, this research enhances our understanding of a class of little-studied behaviors that play a potentially important role in autonomous strategic change and organizational learning.</t>
@@ -18683,6 +18736,16 @@
           <t>BSMA0424</t>
         </is>
       </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G427" t="inlineStr">
         <is>
           <t>The research described in this article focuses on one important aspect of the innovation process - the need for the innovating system to gather information from and transmit information to several external information areas. Special boundary roles evolve in the organization's communication network to fulfill the essential function of linking the organization's internal network to external sources of information. These boundary roles occur at several organizational boundaries, and their distribution within the organization is contingent on the nature of the organization's work. This research supports literature on boundary spanning in general and highlights the importance of boundary roles in the process of innovation.</t>
@@ -18706,6 +18769,11 @@
       <c r="K427" t="inlineStr">
         <is>
           <t>1977</t>
+        </is>
+      </c>
+      <c r="P427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18824,7 +18892,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>Urban metabolism approaches are increasingly becoming relevant in providing pathways to sustainable development. The ways through which urban green infrastructures are planned and designed can influence resource flows in cities. Yet, little is known about the agency and contributions of landscape architects and spatial planners as curators of urban greenery, in facilitating circular resource flows, and accelerating the transition to a circular economy. This paper offers an empirical inquiry into the understanding and use of metabolic approaches in spatial planning and design practices. Through a multi-method approach and the use of boundary spanning as an analytical lens, we identify different modes of agency of spatial practitioners in enhancing resource efficiency across the life stages of urban landscape projects. Results show that while the ‘urban metabolism’ concept is not widely used by practitioners, its relevance to planning and designing green infrastructure for sustainable resource flows is well understood. Additionally, we highlight existing barriers including policy constraints in engaging with metabolic approaches and offer recommendations to facilitate a resource-sensitive turn in planning and designing urban landscapes. This study highlights important contributions of design practice to an expanding discourse of urban metabolism, including policy reforms for enabling circular resource flows in cities.</t>
@@ -18867,6 +18934,12 @@
           <t>BSMA0428</t>
         </is>
       </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -18890,6 +18963,11 @@
       <c r="K431" t="inlineStr">
         <is>
           <t>1996</t>
+        </is>
+      </c>
+      <c r="P431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study analyzes data at the firm level, using CEOs as key informants to evaluate firm-level functional capabilities (logistics, production, marketing) and business performance, rather than measuring individual-level interpersonal boundary spanning behavior.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21394,7 +21472,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -21437,6 +21514,12 @@
           <t>BSMA0495</t>
         </is>
       </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
           <t>Process Management Programs (PMPs) rely heavily on the standardization of activities to improve organizational efficiency and reliability. Standardization, however, can lead to rigidity and inertia, which may eventually inhibit exploration and innovation. While scholars have provided cognitive and routine-based arguments to cope with this dilemma, the fact that standardization is a social process that requires collaboration between individuals has been overlooked. In this paper, we propose that standardization can improve a team’s social capital and thereby facilitate the activities that enable exploration. Specifically, we hypothesize that standardization relates positively to external communication, psychological safety, and the perception of support for innovation in operational teams. These three social capital attributes mediate the relationship between standardization and exploration. We tested this multilevel mediation model by analysing 431 members of 62 operational teams in a large multinational mining company that had recently implemented a Process Management Program (Lean Management). Our multilevel mediation results confirmed that standardisation promoted exploration by enhancing the teams’ social capital. For robustness we tested our model with a second survey of 450 workers of different companies and obtained similar results. Therefore, we propose that the productivity dilemma can be balanced by improving operational teams’ social capital.</t>
@@ -21460,6 +21543,11 @@
       <c r="K498" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P498" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -24117,6 +24205,16 @@
           <t>BSMA0557</t>
         </is>
       </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G560" t="inlineStr">
         <is>
           <t>Project value creation faces tensions between the project owner and the outsourced project manager, particularly in their crossorganizational and cross-temporal interactions. The interplay between cross-organizational and cross-temporal interactions brings signiﬁcant challenges to value creation. Therefore, this research aims to explore these cross-boundary tensions between the project owner and project manager in value creation. Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions. This research identiﬁed four dimensions of cross-boundary tension: (1) structural tension between empowerment and control, (2) priority tension between short-term and long-term, (3) communication tension between convergence and divergence, and (4) involvement tension between assistance and intervention. This research could theoretically contribute to value creation from the owner–manager cross-boundary tension perspective and extend the scope of the temporal boundary. Additionally, it provides practical guidance for professionals to understand the implications of tensions and strike the right balance for optimal value creation.</t>
@@ -24140,6 +24238,11 @@
       <c r="K560" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P560" t="inlineStr">
+        <is>
+          <t>Qualitative/Q-methodology study lacking extractable zero-order effect sizes and measuring cross-boundary tensions rather than boundary spanning behavior.. Verbatim Evidence: [Abstract] "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions." [Step 1: Interviews and Q Statements] "They were asked to respond to questions related to cross-boundary tensions, for example: “What do you believe are the biggest barriers to interaction between project owners and project managers across organizations and stages in the process of achieving project objectives?”" [Step 2: Q Surveys] "Between July and December 2023, 20 participants were invited to rank-order 20 Q statements, presented on cards, in a quasinormal distribution (see Figure 3)."</t>
         </is>
       </c>
     </row>
@@ -26454,6 +26557,12 @@
           <t>BSMA0618</t>
         </is>
       </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>Research-practice partnerships (RPPs) offer promising approaches to improve educational outcomes. Navigating boundaries between contexts is essential for RPP effectiveness, yet much work remains to establish a conceptual framework of boundary spanning in partnerships. Our longitudinal comparative case study draws from our experiences as graduate student boundary spanners in three long-term partnerships to examine boundary spanning roles in RPPs, with particular attention to the ways in which power permeates partnership work. Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums: institutional focus, task orientation, expertise, partnership disposition, and agency. Our roles were shaped by the organizational, cultural, relational, and historical features of the partnerships and contexts of interaction. We aim to promote the development of effective RPP strategies by leveraging the perspectives and positionality of graduate students in order to advance understanding of boundary spanning roles.</t>
@@ -26477,6 +26586,11 @@
       <c r="K621" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P621" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26496,7 +26610,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -28151,7 +28264,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -28320,7 +28432,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F668" t="inlineStr"/>
       <c r="G668" t="inlineStr">
         <is>
           <t>Innovation is a key driver for organizations to survive and thrive in increasingly hyper-competitive markets. This study investigates the effects of boundary-spanning search on innovation capability. Speciﬁcally, it examines the mediating and moderating effects of network ties and absorptive capacity on boundary-spanning search and innovation in Chinese companies. We constructed a theoretical model of an organization’s boundary-spanning search and innovation capability and distributed a survey questionnaire to a sample of speciﬁc industries with upstream and downstream relations in Sichuan Province in China for their responses. Results from the study reveal that boundary-spanning search has a positive and signiﬁcant impact on innovation capability as well as a positive moderating effect on absorptive capacity and innovation capability. This paper shows that enterprises need to continuously focus on exploring networking opportunities in direct and indirect ways to get access to effective ﬂow and diffusion of resources, which in turn can enhance innovation capability.</t>
@@ -28368,7 +28479,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>Due to their complexity and high social impact, urban infrastructure projects often face challenges in managing the design decision-making processes across disparate disciplinary and knowledge domain boundaries. This paper introduces the notion of design boundary dynamics to describe the various cross-boundary coordination phenomena associated with organising the design of infrastructure projects. Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project. Findings illustrate the entangled processes, through which the disciplinary, knowledge-domain and stage-based design boundaries emerged as a result of unfolding project practices. Paper identifies the key role of resource allocation constraints, path dependency of project decisions, and problem-solving nature of design and concludes with strategic recommendations for upstream operational integration to mitigate the impact of design boundary dynamics on infrastructure projects.</t>
@@ -28490,7 +28600,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -28570,6 +28679,12 @@
           <t>BSMA0671</t>
         </is>
       </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -28593,6 +28708,11 @@
       <c r="K674" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P674" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29553,7 +29673,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F699" t="inlineStr"/>
       <c r="G699" t="inlineStr">
         <is>
           <t>Although the information‐seeking literature has tended to focus upon the selection and use of inanimate objects as information sources, this research follows the more recent trend of investigating how individuals evaluate and use interpersonal information sources. By drawing from the structural, relational, and cognitive elements of social capital theory to inform antecedents to information quality and source accessibility, a research model is developed and tested. For interpersonal information sources, information quality is the key determinant of source use. Perceptions of information quality and accessibility of an interpersonal source are shown to be influenced by boundary spanning, transactive memory, and content type. Implications and prescriptions for future research are discussed.</t>
@@ -29680,6 +29799,12 @@
           <t>BSMA0699</t>
         </is>
       </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>
@@ -29703,6 +29828,11 @@
       <c r="K702" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P702" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29722,7 +29852,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F703" t="inlineStr"/>
       <c r="G703" t="inlineStr">
         <is>
           <t>We propose and test a framework that describes the relationship between network structures and job performance. We provide an integration of the current conceptualizations of social capital as they pertain to job performance outcomes by taking a multi-dimensional view of job performance. We break down job performance into creativity, decision-making, task execution, and teamwork, and distinguish the effect of structural holes within and across the organizational boundary on these four job performance domains. In an analysis of 318 managers, we ﬁnd that networks rich in structural holes that cross the organizational boundary had a positive association with creativity and decision-making, whereas networks with few structural holes within the organization had a positive association with task execution and teamwork. We discuss the theoretical implications for integrating the social capital, boundary spanning, and network structure literatures, as well as the practical beneﬁts of giving much more precise advice to managers and employees regarding how to use networks to improve performance at work.</t>
@@ -29765,6 +29894,12 @@
           <t>BSMA0701</t>
         </is>
       </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>
@@ -29788,6 +29923,11 @@
       <c r="K704" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P704" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results part 3
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -10293,7 +10293,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Innovation is considered the engine for firm growth. Especially innovations, through recombining seemingly unrelated knowledge streams, can have groundbreaking impact and lead to sustained competitive advantage. To generate such innovation, firms often need to go beyond their existing technological or geographical boundaries to identify and integrate novel knowledge elements. This article refers to firms’ knowledge activities of drawing upon distant knowledge (i.e., knowledge from dissimilar technological domains or distant geographical regions) to create novel technological solutions, as innovation through boundary spanning. Aiming to investigate the roles of information technology (IT) in facilitating innovation through boundary spanning, we collected data from the pharmaceutical industry over a six-year period to test the research model. The data analysis results indicate that IT supports boundary-spanning activities in firm innovation and different IT-enabled knowledge capabilities affect boundary-spanning innovation differently.</t>
@@ -10378,7 +10377,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -12124,7 +12122,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>The influence of boundary spanning roles on strategic decision-making was explored in a field study in fifteen organizations. Results support the importance of boundary spanning roles in the strategic decision-making process and the relationship of technology to the differential strategic decision-making influence of different boundary spanning roles.</t>
@@ -12172,7 +12169,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>The impact of perceived environmental demands on the roles and job satisfaction of the school psychologist in rural school systems was explored. Superintendents rated their perceptions of the community context and the psychologist’s involvement in interagency linking functions. School psychologists rated their performance of boundary-spanning functions and their job perceptions. Results indicated that certain perceived environmental pressures are related to the performance of boundaryspanning activities. Those who performed boundary-spanning functions are more satisfied with their jobs and more influential in determining their roles.</t>
@@ -13468,7 +13464,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -15782,7 +15777,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>From a knowledge-based perspective, this paper highlights the need for a framework linking perceived competition of the industry and ﬁrms’ strategic location choices of external knowledge search and examines whether the perceived competition increases the propensity of cluster ﬁrms to search more widely from extra-cluster knowledge sources than intra-cluster knowledge sources. Furthermore, we emphasise that cluster ﬁrms with varying degrees of tacitness in their knowledge base might respond to such competition diﬀerently when conducting external knowledge search activities. Using a sample of 310 cluster ﬁrms in the Zhejiang Province of China, we ﬁnd that the cluster ﬁrm would increase the propensity for more geographic boundary-spanning search relative to local search while under the pressure of competition. Moreover, the positive relationship between perceived competition and the propensity towards geographic knowledge search is weaker when the tacitness of the cluster ﬁrm’s knowledge base is higher. The ﬁndings contribute to the understanding of the relationship between competition and the choice of location strategies in external knowledge search.</t>
@@ -18939,7 +18933,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -21519,7 +21512,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
           <t>Process Management Programs (PMPs) rely heavily on the standardization of activities to improve organizational efficiency and reliability. Standardization, however, can lead to rigidity and inertia, which may eventually inhibit exploration and innovation. While scholars have provided cognitive and routine-based arguments to cope with this dilemma, the fact that standardization is a social process that requires collaboration between individuals has been overlooked. In this paper, we propose that standardization can improve a team’s social capital and thereby facilitate the activities that enable exploration. Specifically, we hypothesize that standardization relates positively to external communication, psychological safety, and the perception of support for innovation in operational teams. These three social capital attributes mediate the relationship between standardization and exploration. We tested this multilevel mediation model by analysing 431 members of 62 operational teams in a large multinational mining company that had recently implemented a Process Management Program (Lean Management). Our multilevel mediation results confirmed that standardisation promoted exploration by enhancing the teams’ social capital. For robustness we tested our model with a second survey of 450 workers of different companies and obtained similar results. Therefore, we propose that the productivity dilemma can be balanced by improving operational teams’ social capital.</t>
@@ -26562,7 +26554,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>Research-practice partnerships (RPPs) offer promising approaches to improve educational outcomes. Navigating boundaries between contexts is essential for RPP effectiveness, yet much work remains to establish a conceptual framework of boundary spanning in partnerships. Our longitudinal comparative case study draws from our experiences as graduate student boundary spanners in three long-term partnerships to examine boundary spanning roles in RPPs, with particular attention to the ways in which power permeates partnership work. Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums: institutional focus, task orientation, expertise, partnership disposition, and agency. Our roles were shaped by the organizational, cultural, relational, and historical features of the partnerships and contexts of interaction. We aim to promote the development of effective RPP strategies by leveraging the perspectives and positionality of graduate students in order to advance understanding of boundary spanning roles.</t>
@@ -28684,7 +28675,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -29804,7 +29794,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>
@@ -29899,7 +29888,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results part 8
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -18975,6 +18975,16 @@
           <t>BSMA0429</t>
         </is>
       </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G432" t="inlineStr">
         <is>
           <t>Success in the restaurant industry is, in part, determined by boundary spanning service providers’ ability to manage their emotions with the goal of providing excellent service while simultaneously authentically displaying the proper emotions to connect with the guest. How men and women respond to these displays of emotion is of interest, as previous scholars have demonstrated perceptions and reactions to service delivery diﬀer across genders. This study utilized a between subject quasi-experimental design manipulating each one of the independent variables (gender, emotional labor, and service quality) in a dichotomous fashion for each scenario. The dependent variables measured were satisfaction and loyalty. The results indicated that women are more receptive to deep acting than are their male counterparts, and are thus, more likely to be loyal to an organization if deep acting is employed. How to encourage deep acting among foodservice providers is discussed.</t>
@@ -18998,6 +19008,11 @@
       <c r="K432" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 6
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -7583,6 +7583,16 @@
           <t>BSMA0132</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G135" t="inlineStr">
         <is>
           <t>The market-shaping literature recognizes that consumers are actors who can shape markets. However, research into the mechanisms of consumption-driven market-shaping is only emerging. This paper shows that one way in which consumers shape markets is through boundary work, as consumers make, break, and re-make the boundaries among multiple markets. Empirically, this paper investigates how user innovation practices catalyzed the formation of four boardsport markets: surfing, kitesurfing, windsurfing, and stand-up-paddling. The findings show that consumers shape markets in three steps: (1) generating local variations of consumption practices; (2) imposing order and coherence to intermediate frames; and (3) channeling creative consumption practices into market formation. This paper contributes to the market-shaping literature by conceptualizing how consumers splinter an existing singular market into new markets. We coin the term ‘market bifurcations’ to describe how a singular, seemingly cohesive consumer practice breaks down, splintering into several local variations, which can then catalyze the formation of new markets.</t>
@@ -7606,6 +7616,11 @@
       <c r="K135" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Qualitative study on market boundaries (construct homonymy) lacking quantitative effect sizes.. Verbatim Evidence: [Abstract] "This paper shows that one way in which consumers shape markets is through boundary work, as consumers make, break, and re-make the boundaries among multiple markets." [Method] "We collected 13 semi-structured in-depth interviews with respondents who were simultaneously avid boardsports consumers and commercial operators, including retailers, owner-operators, entrepreneurs, instructors, and photographers (Table 1)."</t>
         </is>
       </c>
     </row>
@@ -7620,6 +7635,16 @@
           <t>BSMA0133</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
           <t>An intriguing window on Japanese/American intercultural relations can be found in American ethnographers’ in-depth accounts of their diﬃculties with Japanese informants. Although the literature contains excellent self-analyses of this kind, this body of data has yet to be mined for general lessons regarding communication between Americans and Japanese. This paper addresses that gap by comparing several reﬂexive accounts of doing ethnography in Japan: Matthews Hamabata’s Crested Kimono, Gail Bernstein’s Haruko’s World, Liza Dalby’s Geisha, and Crafting Selves by Dorinne Kondo. Examining the barriers to Japanese/American communication through this special lens reveals a complicated picture. On the one hand, familiar factors, such as the universalism of Americans, their emphasis upon individual autonomy in social relations, and the Japanese matrix of constantly shifting in-group/outgroup relations are often the dominant inﬂuences on intercultural interactions. Yet, on the other hand, situational contexts and the value orientations and political commitments of the actors clearly do modify the expression of such factors and sometimes even reverse the expected outcomes. The present approach facilitates the representation of these complex relationships. A qualitative analysis in which an objectively framed comparison aimed at generalization rests upon the non-reiﬁed foundation of several reﬂexive ethnographies, shows promise as one strategy for transcending the stalemate between traditional group-based interpretations of culture and more recent approaches stressing individual agency and internal cultural diversity. This paper also illustrates some advantages of an anthropological approach to communication between the members of two cultures whose diﬀerences have long been a focus of interculturalist research and examines implications for models of collectivist and individualist cultures. r 2002 Elsevier Science Ltd. All rights reserved.</t>
@@ -7643,6 +7668,11 @@
       <c r="K136" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Qualitative study of cultural boundaries lacking quantitative effect sizes.. Verbatim Evidence: [Abstract] "A qualitative analysis in which an objectively framed comparison aimed at generalization rests upon the non-reified foundation of several reflexive ethnographies, shows promise as one strategy for transcending the stalemate between traditional group-based interpretations of culture and more recent approaches stressing individual agency and internal cultural diversity." [Introduction] "In it I carry out a comparison of four narratives that American ethnographers have produced."</t>
         </is>
       </c>
     </row>
@@ -7731,6 +7761,16 @@
           <t>BSMA0136</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G139" t="inlineStr">
         <is>
           <t>Improving access to support for people experiencing domestic violence and abuse requires better connections between healthcare services and specialist domestic violence and abuse (DVA) support agencies. We examined the work involved in restructuring the relationship between primary care and specialist DVA support services. This was part of a broader study of the implementation of a general practice DVA training and support programme (IRIS). We conducted an ethnography in two diﬀerent UK areas where the IRIS programme was being delivered. We investigated the work done by specialist DVA workers (Advocate Educators) in the dual role of providing training to GPs and advocacy support to patients. Drawing on concepts of boundary actors and boundary objects, we examined how interactions between clinicians and patients changed after the introduction of the IRIS programme. The referral pathway emerged as a boundary object, meeting a shared ambition of general practitioners and patients to distribute responsibility for addressing DVA. However, maintaining this as a boundary object-in-use required signiﬁcant, and often unseen, work on the part of the Advocate Educator as boundary spanner. Our study contributes to scholarship on boundary work by highlighting the role of marginal boundary actors in maintaining the use of boundary objects among disparate groups.</t>
@@ -7754,6 +7794,11 @@
       <c r="K139" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Qualitative study (ethnography and interviews) lacking quantitative effect sizes.. Verbatim Evidence: [3. Methods] "We adopted an ethnographic approach to study the practices involved in the collaborative work between primary care services and specialist DVA support services." [3. Methods] "AD collected data through participant observation and interviewing." [3. Methods] "19 semi-structured interviews were conducted in each case study area with clinicians (case study one: 5, case study two: 8), services users (case study one: 8, case study two: 5), and actors involved in the commissioning and delivery of IRIS (case study one: 6, case study two: 6)."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 7
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -7687,6 +7687,16 @@
           <t>BSMA0134</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G137" t="inlineStr">
         <is>
           <t>Social ties to colleagues on other work teams can spur creative ideas and workplace innovation by exposing an individual to diverse knowledge. However, for external knowledge to be recombined into innovation, the knowledge must first be recognized as potentially valuable. Going beyond traditional structural explanations, we predict that the use of diverse knowledge to generate creative ideas and solutions will depend in part on employees’ psychological attachment to the organizational groups to which they belong, i.e., their social identity, and the strength of their social ties. We test our hypotheses in an R&amp;D division of a global hightechnology firm, finding that social identity influences the creative generativity of boundary-spanning ties. Specifically, stronger team identity renders interactions with colleagues on other work teams less generative of creative ideas, while identification with an overarching, superordinate group (e.g., a division) enhances creative generativity. We also hypothesize and find that tie strength attenuates the negative effect of team identity.</t>
@@ -7710,6 +7720,11 @@
       <c r="K137" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>The study analyzes data at the dyad/relationship level (N=673 ties reported by 87 individuals), violating statistical independence for individual-level effect sizes.. Verbatim Evidence: [Data and Methods] "The survey yielded 87 complete responses, for a response rate of 73.7%." [Data and Methods] "Because of missing data, the total usable sample is composed of 673 boundary-spanning relationships." [Analytical approach] "As suggested above, the data have a dyadic relational structure, where each respondent researcher (ego) has multiple contacts (alters) on other work teams." [Analytical approach] "In the dyadic structure, each individual researcher is included in multiple observations because he or she reported on multiple relationships." [Analytical approach] "Therefore, the observations are not independent within-person."</t>
         </is>
       </c>
     </row>
@@ -7724,6 +7739,16 @@
           <t>BSMA0135</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G138" t="inlineStr">
         <is>
           <t>The boundary spanning activity of the entrepreneur is used to examine the strategic management process in small business. In a sample of 82 owner/operators, intensive boundary spanning activity was strongly related to organizational performance, and information processing capability significantly affected the performance-boundary spanning relationship.</t>
@@ -7747,6 +7772,11 @@
       <c r="K138" t="inlineStr">
         <is>
           <t>1984</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Excluded under Code 5 [Code 1 &amp; Code 2] due to the use of an independent entrepreneur sample (owner/operators) rather than embedded employees, and because the boundary spanning measure merely assesses time spent and contact frequency without capturing intentional boundary-spanning actions.. Verbatim Evidence: [Sample] &lt;Data were collected by survey instrument from the owner/operators of four different types of small business organizations.&gt; [Sample] &lt;The focus of this study is on the strategic behavior of the owner/operator of the small business organization, the entrepreneur.&gt; [Measures] &lt;Subjects were asked to record the number of hours and the number of contacts they had in an average week with each of nine categories of environmental constituencies.&gt; [Measures] &lt;The sum of the hours spent in these activities divided by the number of hours worked per week is a measure of how intensive the owner/operator's boundary spanning activity is: the percentage of work time spent in boundary spanning activity.&gt;</t>
         </is>
       </c>
     </row>
@@ -7896,6 +7926,16 @@
           <t>BSMA0139</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G142" t="inlineStr">
         <is>
           <t>Interorganizational teams are rapidly becoming more prevalent as a means to improve organizations' responsiveness. To achieve their objective, interorganizational teams must engage in extensive amounts of boundary spanning activity. This study juxtaposed three structural variables, namely team informational diversity, team boundedness, and extrateam links, in an integrated model aimed at promoting our understanding of how to increase interorganizational team boundary spanning activity and its effectiveness. The model was tested with 49 health promotion teams. Our findings indicated that three types of boundary spanning—scouting, ambassadorial, and coordinating—were positively associated with interorganizational team effectiveness. In addition, for team informational diversity, team boundedness, and extrateam links, scouting and ambassadorial activities fully mediated their relationships with team effectiveness; for team boundedness, coordinating activity also fully mediated its relationship with team effectiveness. These findings highlight the importance of incorporating structural considerations into the management of interorganizational teams.</t>
@@ -7919,6 +7959,11 @@
       <c r="K142" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Excluded because the unit of analysis is the team (N=49 health promotion teams) rather than the individual employee.. Verbatim Evidence: [Method - Sample] &lt;The research population consisted of 49 health promotion teams.&gt; [Method - Measures] &lt;I tested for the homogeneity of responses at the unit level by calculating the rwg coefficients (James, Demaree, &amp; Wolf, 1984) for each of the four boundary activities for each of the 49 participating interorganizational teams.&gt; [Results] &lt;TABLE 1 Intercorrelation matrix of study variables&gt; &lt;N = 49.&gt;</t>
         </is>
       </c>
     </row>
@@ -7933,6 +7978,16 @@
           <t>BSMA0140</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G143" t="inlineStr">
         <is>
           <t>The role of gender in career mobility is a major practical and scholarly concern. Drawing on boundaryless career literature and social role theory, we examined whether gender influences employees' psychological mobility, whether this influence varies depending on the nature of career boundaries (the boundaries of job, organisation and industry) and whether it is contingent on organisational or occupational characteristics. We conducted cross‐classified multilevel analyses on 3,527 Australian employees nested within 725 organisations and 43 occupations. The results suggest that females show higher mobility preferences than males when it comes to crossing industries but not changing organisations or jobs. However, their preference for crossing career boundaries is significantly reduced when their organisation has a strong presence of female leadership. We also find that in female‐dominated occupations, females show a higher cross‐organisational mobility preference than males, while in male‐dominated occupations, females show a lower cross‐organisational mobility preference.</t>
@@ -7956,6 +8011,11 @@
       <c r="K143" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Construct Homonymy (Boundaryless Career). The study measures cross-boundary mobility preferences (career mobility / turnover intention) across jobs, organizations, and industries, not interpersonal Boundary Spanning Behavior.. Verbatim Evidence: [Introduction] "First, we take into account the multiplicity of career boundaries (job, organisation and industry), refining the understanding of ‘boundary’ in boundaryless careers (Inkson et al. 2012)." [Measures] "For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference." [Measures] "We created the mobility preference variables using individuals’ responses to this question: ‘In regard to your job, where do you want to be in 12 months’ time?’"</t>
         </is>
       </c>
     </row>
@@ -7970,6 +8030,16 @@
           <t>BSMA0141</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G144" t="inlineStr">
         <is>
           <t>Managing a complex, boundary‐spanning function to maximize its contribution to the firm can be a challenging task. This research is concerned with providing management with increased understanding of the effects of different ways of managing a function, especially a significant boundary‐spanning operation. Conducted in the context of a procurement function, through a laboratory experiment, explores the impact of performance measures, interaction with other internal organizations and access to information about external events on an individual′s decision making and “comfort level”. Results indicate that the performance measurement system determines an individual′s decision‐making performance. The broader, more effectiveness‐oriented measures also tend to make the individuals more confident and satisfied with their operating environment and decisions. The availability of interaction with other internal organizations and the access to information about external events impact on an individual′s decisions but have relatively little effect on his/her comfort level.</t>
@@ -7993,6 +8063,11 @@
       <c r="K144" t="inlineStr">
         <is>
           <t>1994</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 2] Laboratory experiment using a student sample (business school undergraduates) and reporting no zero-order correlation matrix.. Verbatim Evidence: [Manipulations] "The research was conducted using a full-factorial experimental design, resulting in 16 (4 × 2 × 2) treatments." [Manipulations] "Fifteen subjects (upper division business school undergraduates) were in each treatment."</t>
         </is>
       </c>
     </row>
@@ -8007,6 +8082,16 @@
           <t>BSMA0142</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G145" t="inlineStr">
         <is>
           <t>A psychological contract is composed of an individual’s belief regarding the reciprocal obligations that exist between that individual and another entity with which that person is engaged. Psychological contracts are important in many business relationships, such as those between a buyer and supplier. The perceptions held by one individual may not be congruent with those of the other, in which case conflict may arise within the relationship. We introduce to the operations and supply chain literatures a comprehensive view of the theory of psychological contracts, which with few exceptions has largely been omitted from research regarding inter-firm relationships. This research investigates the processes by which individuals manage conflict in inter-firm relationships, and the extent to which decisions at both tactical and strategic levels are influenced by the experience of psychological contract violation. At the tactical level, we seek to understand how the daily operational decisions that individuals make are affected by psychological contract violation, particularly when sub-optimal decision-making is observed. At the strategic level, we consider the circumstances under which relational versus written contractual governance mechanisms are leveraged in response to conflict, and how the experience of psychological contract violation may influence these broader,firm-level decisions. Our research plan uses two different methodological approaches in investigating these issues. First, to evaluate tactical behaviors, we employ an experiment. The goal of the experiment is to determine specifically how economic decisions made by those in boundary-spanning roles deviate from optimal in response to conflict and how these behaviors are influenced by the experience of psychological contract violation. To this end, we employ a 2x2x2 factorial design in which violation timing, severity, and attribution are investigated. The experiment was accompanied by an exit survey which served to assess the experience of psychological contract violation and related issues of trust and fairness. Data from 295 subjects were included in our analysis. We observe a main effect of severity occurring during the violation, and main effects of time and attribution are evident in post-violation periods. We tie these phenomena to the psychological constructs under study. Second, in order to investigate strategic-level decisions, we propose administration of an industry survey to purchasing and sales managers. The survey will allow us to more broadly characterize types of conflict experienced in inter-firm relationships and the contractual governance mechanisms leveraged in response. Models useful for investigating these issues are developed and discussed, and a survey instrument is presented. The work presented in this dissertation is among the first to incorporate both individual-level and firm-level contracts into an investigation of tactical and strategic conflict response and resolution analysis within buyer-supplier exchange relationships.</t>
@@ -8030,6 +8115,11 @@
       <c r="K145" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 2] The study uses a laboratory experiment with an undergraduate student sample and measures economic decisions (order quantity) and psychological contract violation rather than boundary spanning behavior. The industry survey in Chapter 4 is only proposed and contains no empirical data.. Verbatim Evidence: [Abstract] "The goal of the experiment is to determine specifically how economic decisions made by those in boundary-spanning roles deviate from optimal in response to conflict and how these behaviors are influenced by the experience of psychological contract violation." [Participants] "The primary data source for these experiments was undergraduate business students from the Fisher College of Business." [Participants] "A total of 304 undergraduates participated in our experiment sessions, which were conducted between May 7th and May 21st, 2010." [The Industry Survey] "The effort expended so far has focused on model development and instrument design, and the resulting survey instrument represents the key contribution of the survey to our body of work thus far."</t>
         </is>
       </c>
     </row>
@@ -8044,6 +8134,16 @@
           <t>BSMA0143</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G146" t="inlineStr">
         <is>
           <t>ABSTRACT               This paper examines learning in interdisciplinary action teams. Research on team effectiveness has focused primarily on single‐discipline teams engaged in routine production tasks and, less often, on interdisciplinary teams engaged in discussion and management rather than action. The resulting models do not explain differences in learning in interdisciplinary action teams. Members of these teams must coordinate action in uncertain, fast‐paced situations, and the extent to which they are comfortable speaking up with observations, questions, and concerns may critically influence team outcomes. To explore what leaders of action teams do to promote speaking up and other proactive coordination behaviours – as well as how organizational context may affect these team processes and outcomes – I analysed qualitative and quantitative data from 16 operating room teams learning to use a new technology for cardiac surgery. Team leader coaching, ease of speaking up, and boundary spanning were associated with successful technology implementation. The most effective leaders helped teams learn by communicating a motivating rationale for change and by minimizing concerns about power and status differences to promote speaking up in the service of learning.</t>
@@ -8067,6 +8167,11 @@
       <c r="K146" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Non-individual level analysis (team level, N=16 teams). Verbatim Evidence: [Research Design] The sample consisted of 16 cardiac surgery teams selected to ensure differences in geography and innovation history from the approximately 150 US hospitals that had purchased the technology. [Data Analyses] The result is a set of numerical ratings for five team constructs (team stability, team preparation, procedure innovation, boundary spanning, and psychological safety) and four organizational constructs (history of innovation, resource constraints, management support, and information infrastructure) for each hospital.</t>
         </is>
       </c>
     </row>
@@ -8118,6 +8223,16 @@
           <t>BSMA0145</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G148" t="inlineStr">
         <is>
           <t>Organizations are increasingly applying artificial intelligence (AI) in interorganizational systems (IOS) to mitigate demand and supply disruptions. This shift towards AI to enhance supply chain agility capabilities automates some tasks previously undertaken by boundary-spanning employees who serve as critical informational and influential links with supply chain partners. Given limited related research, we investigate the impact of AI not only on the potential displacement of boundary-spanning employee roles but also on subsequent supply chain agility. Leveraging dynamic capabilities and social network theories, we first conducted interviews with supply chain executives to develop a practitioner survey. Following a mixedmethods approach, we next applied structural equation modeling to this survey data and then probed further via follow-up interviews. The results reveal that despite displacing some employees, the use of AI in IOS enhances the remaining operational and strategic roles of the boundary-spanning employees to enrich supply chain agility. The ensuing theoretical and managerial contributions emphasize the essential role of boundaryspanning employees as part of a hybrid human-AI solution, providing insight into the need for an optimal human/AI balance in the supply chain to cope with dynamic marketplaces.</t>
@@ -8141,6 +8256,11 @@
       <c r="K148" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Firm-level analysis using proxy informants and no extractable correlation matrix [Code 1 &amp; Code 3]. Verbatim Evidence: [Code 3: Proxy Informants] &lt;In the survey, participants were asked to consider one specific supply chain partner when responding.&gt; [Code 3: Grammatical Subject 'We'] &lt;We depend on BSE to regularly exchange information or resources with partners&gt; [Code 3: Firm Level] &lt;The majority of responding firms were based in North America (53.8%). Also, most firms operated in the manufacturing industry (59%) and had less than $500 million in revenue.&gt;</t>
         </is>
       </c>
     </row>
@@ -8155,6 +8275,16 @@
           <t>BSMA0146</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G149" t="inlineStr">
         <is>
           <t>While anecdotal and research evidence exists supporting the difﬁculties faced by foreign ﬁrms in host nation environments due to liability of foreignness, it is clear that many foreign ﬁrms have been successfully operating in the U.S. over the years. This study seeks to understand the strategies foreign ﬁrms use to cope with liabilities of foreignness in an alien environment and compete successfully with domestic ﬁrms, speciﬁcally through boundary spanning. Using a sample of 3861 ﬁrms in the U.S., we ﬁnd that foreign ﬁrms on the average underperform compared to domestic ﬁrms. We also ﬁnd these ﬁrms take a differing strategic posture to cope with the disadvantages of being a foreign ﬁrm compared to domestic rivals. Multiple mediation models indicate that once this strategic posture of foreign ﬁrms is controlled for, performance differentials do not exist between foreign and domestic ﬁrms.</t>
@@ -8178,6 +8308,11 @@
       <c r="K149" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] The study analyzes firm-level secondary data from the NAIC database (N=3861 firms) rather than individual employee behavior. It explicitly focuses on organizational-level boundary spanning.. Verbatim Evidence: [Abstract] "Using a sample of 3861 firms in the U.S., we find that foreign firms on the average underperform compared to domestic firms." [2. Conceptual background and hypothesis development] "Scholars have studied boundary spanning roles at the individual (e.g., Perrone, Zaheer, &amp; McEvily, 2003) and organizational levels (e.g., Scott, 1998). However, this study’s focus is at the organizational level and specific to the role of managing the interface between organization and environment." [3.1. Data sources] "This study used two sources of data, namely the National Association of Insurance Commissioners (NAIC) database and Best’s Rating guide."</t>
         </is>
       </c>
     </row>
@@ -8192,6 +8327,16 @@
           <t>BSMA0147</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G150" t="inlineStr">
         <is>
           <t>Currently, little is known about the internal (intrafirm) behaviors that may positively affect collaborative marketing/logistics integration, or about the benefits that may be associated with making these considerable investments. In short, what should firms be doing to promote marketing/logistics collaborative integration? What is the potential payoff? This paper addresses these questions by examining relationships between the organization's evaluation and reward system, cross-functional collaboration, effective marketing/logistics interdepartmental integration, and distribution service performance.</t>
@@ -8215,6 +8360,11 @@
       <c r="K150" t="inlineStr">
         <is>
           <t>2000</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Proxy Informant Trap: The survey measures department-level interdepartmental relations using the individual manager as a key informant.. Verbatim Evidence: [Sample Design] "The sampling frame consisted of logistics managers employed by U.S.-based manufacturers listed in the Council of Logistics Management (CLM) membership roster, where 2,046 potential candidates were identified." [Table 2] "During the past six months, how often did the logistics department engage in the following activities with the marketing department? (5-point scale: 1 = never; 5 = quite frequently)"</t>
         </is>
       </c>
     </row>
@@ -8303,6 +8453,16 @@
           <t>BSMA0150</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G153" t="inlineStr">
         <is>
           <t>Why do so many organizations fail to respond to crises effectively, and what can be done to improve their crisis response? We aim to address these questions by developing a typology of boundaries that can help us understand and better prepare for future crises. Building on the existing literature on crisis management and boundaries, our typology seeks to address the critique of current crisis management models, such as these being too prescriptive and placing too much emphasis on assumptions that only the decisions made by the crisis management team (i.e., centralized decisions) will impact the crisis response. We address this critique by elaborating on four categories of boundaries that are relevant to manage crisis response, such as physical, mental, social, and temporal. Examples of these boundaries could include access to properties (physical), interpreting whether a crisis is happening (mental), shifting relationship dynamics (social), and the urgency of response time to a crisis (temporal). Our typology offers a lens to consider crisis management by taking into consideration the complexities and nuances that linear crisis management models have not yet adequately addressed. We argue that by identifying, defining, and understanding different configurations of boundaries, one can better manage crises toward a desired outcome.</t>
@@ -8326,6 +8486,11 @@
       <c r="K153" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] The article is a theoretical/conceptual paper proposing a typology of boundaries in crisis management. It contains no primary quantitative empirical data or extractable effect sizes.. Verbatim Evidence: [Abstract] "We aim to address these questions by developing a typology of boundaries that can help us understand and better prepare for future crises." [Abstract] "Building on the existing literature on crisis management and boundaries, our typology seeks to address the critique of current crisis management models, such as these being too prescriptive and placing too much emphasis on assumptions that only the decisions made by the crisis management team (i.e., centralized decisions) will impact the crisis response." [Discussion] "This paper aimed to propose and develop a typology of boundaries in crisis management, which moves away from prescriptive planning and views crisis management as a process of understanding and managing intersecting and interacting boundaries."</t>
         </is>
       </c>
     </row>
@@ -8340,6 +8505,16 @@
           <t>BSMA0151</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G154" t="inlineStr">
         <is>
           <t>The literature on interorganizational relationships has explored them at the organizational level and ignored interpersonal relationships. This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in business–to–business (B2B) interorganizational relationships, pointing out directions for future research. The review was carried out in ten steps, separated into three phases encompassing planning, collecting, and synthesizing data, and disclosing the results. The study assesses 3,156 published articles, and 45 of them addressed the theme of boundary spanners in B2B interorganizational relationships. These articles were analyzed, identifying their characteristics and the evolution of research through time. The definitions of interpersonal and interorganizational relationships were compared, observing how the literature has addressed the interdependency between these relationships. Also, the concepts and roles assigned to boundary spanners were analyzed, leading to an integrated framework of the existing literature on the theme. Finally, suggestions for future research are presented, followed by this review’s implications and limitations.</t>
@@ -8363,6 +8538,11 @@
       <c r="K154" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Systematic literature review, no primary effect sizes.. Verbatim Evidence: [Abstract] This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in business–to–business (B2B) interorganizational relationships, pointing out directions for future research. [Methodology] A systematic literature review allows the synthesizing of results and evidence from existing studies and producing new knowledge.</t>
         </is>
       </c>
     </row>
@@ -8451,6 +8631,16 @@
           <t>BSMA0154</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G157" t="inlineStr">
         <is>
           <t>The purpose of this article is to promote an open systems perspective on team research. The authors develop a model of team boundary activities: boundary spanning, buffering, and reinforcement. The model examines the relationship between these boundary activities and team performance, the moderating effects of organizational contextual factors, and the mediating effect of team psychological safety on the boundary work–performance relationship. These relationships were empirically tested with data collected from 64 software development teams. Boundary spanning, buffering, and boundary reinforcement were found to relate to team performance and psychological safety. Both relationships are moderated by the team’s task uncertainty and resource scarcity. The implications of the findings are offered for future research and practice.</t>
@@ -8474,6 +8664,11 @@
       <c r="K157" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Measures] "Because our model focuses on the team level, we took a number of steps before aggregating individual responses to the team level." [Measures] "On the basis of these results, individual responses were aggregated and data were analyzed at the team level." [Results] "Because our actual sample contained 64 teams, the sample-size requirement was adequately met."</t>
         </is>
       </c>
     </row>
@@ -8525,6 +8720,16 @@
           <t>BSMA0156</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G159" t="inlineStr">
         <is>
           <t>Top management teams (TMTs) interact with key external stakeholders through boundary spanning, often by holding outside directorships. Yet research suggests these activities have an equivocal relationship with firm financial performance. Although outside directorships promise informational benefits (i.e., the social network perspective), they also present challenges in the form of managerial opportunism (i.e., the agency perspective). Here, we adopt a contingency perspective to reconcile these perspectives, investigating the moderating role of cohesion, or the degree to which team members mutually support and get along with one another. We argue that boundary spanning will yield performance benefits for TMTs with high cohesion, because their increased commitment to the team will enable members to use their external relationships for the benefit of their firms. However, we also identify a boundary condition for this effect based on structural position in the TMT: that cohesion is especially relevant when proportionally more non-chief executive officer (CEO) TMT members span boundaries than CEOs span boundaries. Results from an archival study of TMTs using q-sort methodology provide support for these predictions.</t>
@@ -8548,6 +8753,11 @@
       <c r="K159" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Team/Firm-level analysis of TMT outside directorships (N = 48 teams). Verbatim Evidence: [Data and Sample] "Our sample was taken from a larger study of leadership teams of large pub-licly traded organizations and consisted of 48 TMTs." [Variables] "To assess TMT boundary spanning, we adapted measures used in previous research on boundary spanning in the form of outside direc-torships" [Variables] "First, we counted and summed the number of outside ties for each TMT member in each year and averaged them over the Group Dynamic Q-sort (GDQ) time period." [Results] "Note. N = 48 teams; CEO = chief executive officer; TMT = top management team;"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 8
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -7843,6 +7843,16 @@
           <t>BSMA0137</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G140" t="inlineStr">
         <is>
           <t>Multinational companies (MNC) are facing increasing pressure in the marketplace. It is up to MNC leaders to engage the resources available to them to ensure these firms remain competitive and avoid organizational decline. A hallmark MNC business model competitive advantage is organizational effectiveness in promoting collaboration and cooperation across organizational and environmental boundaries. Boundary crossing actors and the activities they pursue are valuable resources residing at the core of the MNC business model and hence constitute a key element of the firm’s competitive advantage. The purpose of this research is to investigate how MNC leaders can engage these resources for organizational benefit. The research question asked and answered in this study is, How can MNC leaders bolster organizational effectiveness using boundary activity resource (re) combination and control? The organizational control theory lens is used to guide this research. Using the principles of evidence-based management, a systematic review of evidence from 2002 to 2022 was conducted. The systematic review process included a systematic search for evidence including gathering input from subject matter experts and a critical assessment and quality appraisal of the evidence sources. Subsequently, the sources were subjected to an analysis and synthesis in search of emergent themes related to the research question. The research showed that organizational climate, knowledge management, and individual idiosyncrasies (combined with role idiosyncrasies) have considerable implications for leaders in the decision-making process. Although each element is important on its own, the totality of the evidence suggests it is the holistic combination of all four elements that can lead to promotion of boundary activities and hence enhancement of organizational effectiveness. Furthermore, it is an MNC leader’s responsibility to ensure an organizational climate conducive to boundary crossing activities is created and maintained for these elements to work. The recommendations resulting from the research are that MNC leaders must prioritize boundary actors and activities as core organizational value drivers, core boundary crossing competencies have to be built out, and once constructed, these competencies have to be entrenched in the organization’s compositional mechanisms and be monitored and maintained for them to remain effective.</t>
@@ -7866,6 +7876,11 @@
       <c r="K140" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Non-primary study (Systematic review). Verbatim Evidence: [Abstract] "Using the principles of evidence-based management, a systematic review of evidence from 2002 to 2022 was conducted." [Chapter 3: Method] "A qualitative systematic review (SR) was conducted to answer the research question: How can MNC leaders bolster organizational effectiveness using boundary spanning resource (re)combination and control?" [Review Design and Methodology] "Scholars define a SR as a review of existing research; hence, SR methodology is neither primary or empirical in nature and can be viewed as secondary research (Gough et al., 2017)."</t>
         </is>
       </c>
     </row>
@@ -7878,6 +7893,16 @@
       <c r="B141" t="inlineStr">
         <is>
           <t>BSMA0138</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -7914,6 +7939,11 @@
           <t>2014</t>
         </is>
       </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Non-primary conceptual/theoretical chapter proposing a network perspective on multiteam system leadership, lacking empirical data and effect sizes.. Verbatim Evidence: [Non-primary study]. Verbatim Evidence: "[Abstract] The current chapter explains how the form of MTS leadership (e.g., vertical, shared) can be captured using network analytic techniques across multiple MTS network foci (e.g., within teams, between-teams, across the system)." "[Introduction] In the reminder of this chapter, we advance a framework to study MTS leadership from a network perspective."</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -8186,6 +8216,16 @@
           <t>BSMA0144</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G147" t="inlineStr">
         <is>
           <t>Purpose: Sleep deprivation among employees has become commonplace in the workforce. In the United States, the number of hours individuals sleep per night has declined by an hour and a half per night since the 1960s. As of 2005, seventy-four percent of individuals were getting less than eight hours of sleep per night on weekdays. There are negative ramifications to the organization when employees are sleep deprived such as lost productivity, increased accident rate, and increased absenteeism.</t>
@@ -8209,6 +8249,11 @@
       <c r="K147" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>No effect size of interest. The study does not measure Boundary Spanning Behavior, but merely examines the effect of sleep duration on job factors among salespeople, whom they describe conceptually as 'boundary spanning employees'.. Verbatim Evidence: [Abstract] "Because of these distinctive roles, this study examines if differences based on sleep duration exist for business-to-business sales employees for two individual and five organizational factors." [Abstract] "The two individual factors consisted of grit and happiness while the five organizational factors consisted of perceived organizational support, perceived supervisory support, job satisfaction, organizational commitment, and turnover intentions." [Abstract] "For example, business-to-business sales employees are boundary spanning employees that are responsible for generating revenue for the organization."</t>
         </is>
       </c>
     </row>
@@ -8416,6 +8461,16 @@
           <t>BSMA0149</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr">
         <is>
           <t>This article aims for a deeper understanding of front-line employees (FLEs) and their boundary-spanning role in service organizations’ innovation processes from the vantage points of creativity and service innovation theory. It explores in particular FLEs’ processes of creativity by focusing on how ideas emerge and how these ideas are further managed in the organizations’ innovation processes. It draws on an in-depth empirical study of three units at a large spa and resort hotel. The article demonstrates how FLEs’ ideas are related to the assimilation and utilization of knowledge gained in the customer–supplier interface. Furthermore, it introduces the concept of ‘management by weaving’, which encompasses the middle managers’ roles in the complexity of leading diverse innovation processes in the service organization. By having the roles of facilitator, gatekeeper, and translator, middle managers hold the key position for letting FLEs play the role as innovators.</t>
@@ -8439,6 +8494,11 @@
       <c r="K152" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Qualitative study without extractable effect sizes. Verbatim Evidence: [Method] A single-case study was conducted owing to the need to carry out a comprehensive study where the data would make it possible to makecomparisons within a single organization, instead of comparisons between cases (Stake, 2003 ; Yin, 2009 ). [Data collection] Data were collected through interviews and observations. Internal and external documents were also collected. Interviews were conducted mainly with FLEs, but in addition someback-office personnel and managers of the units were interviewed.</t>
         </is>
       </c>
     </row>
@@ -8594,6 +8654,16 @@
           <t>BSMA0153</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G156" t="inlineStr">
         <is>
           <t>Purpose – To better understand factors that lead to business model innovation (BMI) in organizations, this study argues that inclusive leadership is the primary source that motivates employee engagement in boundaryspanning activities, which fosters BMI by generating and integrating employee knowledge through boundaryspanning exploration.</t>
@@ -8617,6 +8687,11 @@
       <c r="K156" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Firm-level construct measured via proxy informants. Verbatim Evidence: [Methodology] "We then selected 30 companies to participate in our survey, sending each 20 questionnaires." [Methodology] "Our respondents were primarily top managers or leaders of departments." [Methodology] "It should be noted that only those who were knowledgeable concerning their firms’ BMI were qualified to take part in the interviews." [Methodology] "In addition, to eliminate common method variance, the BMI scale and boundary-spanning exploration scale items were filled out by department leaders or CEOs, and that on inclusive leadership style was filled out by department employees." [Methodology] "This paper measures boundary-spanning exploration of technical knowledge and market knowledge using the scale developed by Sidhu et al. (2007), which has been widely recognized by scholars." [Literature review and hypotheses development] "Laursen and Salte (2006) observed that boundary-spanning exploration guides enterprises to search for new ideas and knowledge; in the process of BMI, a greater breadth of partner enterprises with which to interact leads to better innovation outcomes."</t>
         </is>
       </c>
     </row>
@@ -8683,6 +8758,16 @@
           <t>BSMA0155</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G158" t="inlineStr">
         <is>
           <t>Boundary work, or task-related activities with external actors, has been shown to positively influence small group performance. However, these "external activities" may also detract from important internal group processes that help groups function. This research examines the puzzle of how groups can perform external activities without compromising their internal group dynamics. I explore how groups perform boundary work and consider the effectiveness of different methods of boundary work from a group identity perspective. Using both qualitative and quantitative methods in experimental and field-based settings, I compare and contrast boundary work that involves sending group members outside the group boundary to interact with external actors individually (i.e., an outward-bound approach), with an inward-bound approach, which entails inviting outsiders in to provide information, resources, or support to the group as a whole. Across four studies, I find that an inward-bound approach to boundary work strengthens group identity and subsequent group satisfaction and viability (Studies 1, 2 and 4), an outward-bound approach used in combination with an inward-bound approach can positively influence task performance and group satisfaction and viability (Study 4), and that an initially weak group identity leads group members to choose an inward-bound approach over an outward-bound approach when interacting with outsiders (Studies 1, 3 and 4). The main contributions of this work are 1) delineating different ways in which groups interact with outsiders, 2) considering the nature of the relationships between boundary work methods and group identity, and 3) investigating the consequences of performing these methods of boundary work using multiple criteria of group effectiveness. Findings converge to reveal that inward boundary work is an important phenomenon for organizational groups. Ultimately, this research offers a more nuanced view of the external perspective of small groups by suggesting that the ways in which groups interact with outsiders are both multidimensional and consequential.</t>
@@ -8706,6 +8791,11 @@
       <c r="K158" t="inlineStr">
         <is>
           <t>2030</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=65 groups) and student sample (MBA student groups).. Verbatim Evidence: [Chapter 4: Longitudinal Field Study] "To understand the relationships between boundary work, group identity, and effectiveness among interacting groups, I conducted a longitudinal study of MBA student groups at a graduate business school in the United Kingdom. The sample consisted of 65 teams of five to seven members each." [Chapter 4: Longitudinal Field Study] "To test the hypotheses I used ordinary least squares regression with variables measured or calculated at the group level." [Chapter 4: Longitudinal Field Study] "Table 4.2. Means, Standard Deviations, and Correlations among Study Variablesa. ... aSample size ranged from 58 to 65 (groups) because of missing data."</t>
         </is>
       </c>
     </row>
@@ -8772,6 +8862,16 @@
           <t>BSMA0157</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G160" t="inlineStr">
         <is>
           <t>Multiteam systems are increasingly used by organizations, but are difficult to coordinate effectively. Building from theory on representational gaps, we explain why coordination between teams in multiteam systems can be hindered by inconsistencies that exist between them regarding the definition of shared problems. We argue that frame-of-reference training, an intervention that is theorized to reduce representational gaps, can facilitate coordination and subsequent performance in multiteam systems. We studied the effects of frame-of-reference training on multiteam system coordination and performance in 249 multiteam systems comprised of specialized teams. Supporting our expectations, we found that: (a) frame-of-reference training had a positive effect on multiteam system performance by enhancing between-team coordination; (b) within-team coordination improved the relationship between frame-of-reference training and between-team coordination, ultimately improving multiteam system performance; and (c) the patterns by which within-team coordination leveraged our intervention depended on teams’ specific functions. Our findings extend representational gaps theory, highlight the interdependencies between team-level and system-level coordination, and demonstrate the utility of frame-of-reference training in a new setting.</t>
@@ -8795,6 +8895,11 @@
       <c r="K160" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Non-individual level of analysis (multiteam system).. Verbatim Evidence: [Sample and Task] "A total of 3,486 officers were randomly assigned to one of 249 14-person multiteam systems for the entire five-week course, such that each multiteam system was comparable with respect to members’ ability, gender, experience, age, and vocational specialty." [Measures] "We measured between-team coordination behaviorally as the number of missions sent to targets on the COP with a confidence rating indicated (i.e., missions sent to targets with ratings of “1” through “4”; missions with confidence ratings of “0” were excluded; see Appendix C)." [Table 1] "Notes: n = 249; observations are multiteam systems of 14 members each."</t>
         </is>
       </c>
     </row>
@@ -8809,6 +8914,16 @@
           <t>BSMA0158</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr">
         <is>
           <t>Purpose: This study is designed to respond to repeated calls for research on sales person retentionby building upon a mature research stream to identify ways to reduce turnover in boundary spanning employees and the resultant effect it has on organizational productivity. Specifically, this research draws on the Job Demands-Resources model to explore the effect of employee perceptions of firm market orientation as a way to reduce role stressors and subsequently turnover intentions. It also looks at employee traits that may serve as a buffer to the role stress to turnover intentions link and can be part of the hiring selection process (in this case grit). In so doing, this research uses a sample of early career salespeople to examine the effects of a firm’s market orientation (MO) and selective hiring for specific traits (level of grit) on a salesperson’s intention to quit using Job Demand-Resources as a framework.</t>
@@ -8832,6 +8947,11 @@
       <c r="K161" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>The study surveys boundary-spanning employees (salespeople) but does not measure Boundary Spanning Behavior (BSB) as a construct. Instead, it measures their perceptions of the firm's market orientation, role conflict, role ambiguity, grit, job satisfaction, and turnover intentions.. Verbatim Evidence: [Sample] "A Qualtrics survey panel was selected as the sample for this study with the sample consisting of 260 respondents who were employed full-time and worked in either B2B or B2C sales as boundary-spanning employees." [Constructs] "Market orientation was measured on a 14-item scale originally constructed by Narver and Slater (1995)) and adapted by Hooley et al. (2000)." [Constructs] "Role conflict (eight items) and role ambiguity (six items) scales were adapted from Rizzo, House, and Lirtzman (1970)." [Findings] "The supported hypotheses of a significant negative relationship between (1) market orientation and role ambiguity, (2) the negative relationships between role conflict and ambiguity and job satisfaction and (3) the negative relationship between job satisfaction and turnover intentions all reinforce the conceptualization of market orientation as a job resource."</t>
         </is>
       </c>
     </row>
@@ -8846,6 +8966,16 @@
           <t>BSMA0159</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G162" t="inlineStr">
         <is>
           <t>What types of human and social capital identify the emergence of leaders of open innovation communities? Consistent with the norms of an engineering culture, we find that future leaders must first make strong technical contributions. Beyond technical contributions, they must then integrate their communities in order to mobilize volunteers and avoid the ever-present danger of forking and balkanization. This is enabled by two correlated but distinct social positions: social brokerage and boundary spanning between technological areas. An inherent lack of trust associated with brokerage positions can be overcome through physical interaction. Boundary spanners do not suffer this handicap and are much more likely than brokers to advance to leadership. The research separates the influence of human and social capital on promotion, and highlights previously unexamined differences between brokerage- and boundary-spanning positions. Longitudinal analyses of careers within the Internet Engineering Task Force community from 1986–2002 support the arguments.</t>
@@ -8869,6 +8999,11 @@
       <c r="K162" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>Excluded due to multiple reasons [Code 1 &amp; Code 2]: The study uses invalid structural network variables based on bibliometric data (Burt's constraint and publication counts) rather than purposive boundary-spanning behavior, and the sample consists of unpaid volunteers in an open innovation community rather than organizational employees.. Verbatim Evidence: [Variables] "Social Brokerage measures the opposite of individual constraint, where constraint measures the extent to which ego has ties with few alters and those alters have ties between them (Burt 1992). We enter the negative of constraint (Equation (1)) as our measure of brokering." [Variables] "Spans 1 boundary indicates that an engineer published within two working groups; Spans 2+ boundaries indicates that a subject published in three or more working groups." [Open Innovation Communities and the IETF] "We define an open innovation community as a group of unpaid volunteers who work informally, attempt to keep their processes of innovation public and available to any qualified contributor, and seek to distribute their work at no charge. While we induct theory from many open innovation communities, we test our hypotheses with a specific data set culled from the archives of the IETF, with the dependent variable as time to appointment as a working group leader within the IETF." [Evidence] "We draw data primarily from the published proceedings of the IETF’s triannual meetings from its inception in 1986 until 2002, and from the organization’s RFC (request for comments) publication series over the same time period."</t>
         </is>
       </c>
     </row>
@@ -8883,6 +9018,16 @@
           <t>BSMA0160</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G163" t="inlineStr">
         <is>
           <t>In the water and energy sectors, projects geared towards new forms of cross-sectoral functioning have boomed in most European countries over the past decade, and have deeply transformed the ecology of urban services. These projects are often considered as an answer to a rising challenge affecting numerous traditional utilities: the unforeseen urban change relating to shifting (i.e. declining) demand patterns that are undermining traditional models of infrastructure management. The development of cross-sectoral strategies is considered a way both to tackle the attrition of traditional sources of revenue and to develop greener infrastructure systems by enhancing their efficiency level, often in line with low-carbon programmes implemented by national or local governments. The appeal lies in a fairly static perception of infrastructure management and technological change. Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the company’s transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities. Various facets of such ‘boundary work’ are analysed, focusing on organisational and financial aspects to reveal the new sites of tensions and negotiations between sectors, but also on the material component of these cross-sectoral projects through the case of one such nexus programme, a waste-toenergy programme. This programme embodies the potential contradictions between the call for reduced use of resources (i.e. the production of less waste) and the development of new urban technical systems relying primarily on those same resources.</t>
@@ -8906,6 +9051,11 @@
       <c r="K163" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>Qualitative ethnographic case study lacking an extractable quantitative effect size or correlation matrix.. Verbatim Evidence: [Abstract] "Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the company’s transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities." [Methodological aspects: Embedded in a utility] "To flesh out the reorganisation of a municipal utility and better capture the ‘socio-technical geometry of powers in town’ (Graham and Marvin, 2001), I decided to immerse myself directly in this technical world by being embedded within the teams of infrastructure management of a German multi-utility."</t>
         </is>
       </c>
     </row>
@@ -8920,6 +9070,16 @@
           <t>BSMA0161</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G164" t="inlineStr">
         <is>
           <t>This study investigated relationships between middle managers’ formal position, their strategic influence and organizational performance. Among the 259 middle managers represented in the study, managers with formal positions in boundaryspanning sub-units reported higher levels of strategic influence activity than others. At the organizational level of analysis, the study found that firm performance was associated with more uniform levels of downward strategic influence, and more varied levels of upward influence among middle management cohorts. The findings suggest that middle managers’ strategic influence arises from their ability to mediate between internal and external selection environments. In addition, positive effects on organizational performance appear to depend on: (1) whether the overall pattern of upward influence is conducive to shifts in the network centrality of individual managers; and (2) whether the pattern of downward influence is consistent with an appropriate balance between the organization’s need for control and flexibility.</t>
@@ -8943,6 +9103,11 @@
       <c r="K164" t="inlineStr">
         <is>
           <t>1997</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>The study does not measure Boundary Spanning Behavior as an interpersonal behavioral construct. It uses the manager's formal organizational role (department type, e.g., marketing vs. finance) as a structural proxy for boundary-spanning position.. Verbatim Evidence: [Participants] "A questionnaire on managers’ involvement in their organization’s strategy process was responded to by 259 middle managers from 25 organizations representing a wide variety of industries." [Measures] "Therefore, our measure of boundary spanning was based on functional descriptions of sub-units and formal organizational roles." [Measures] "First, consistent with criteria specified in Thompson (1967) and elsewhere (Jemison, 1984), three functions (marketing, purchasing, and human resource management) were classified as boundary spanning and four (finance, accounting, operations, and quality control) were classified as non-boundary spanning."</t>
         </is>
       </c>
     </row>
@@ -8957,6 +9122,16 @@
           <t>BSMA0162</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G165" t="inlineStr">
         <is>
           <t>Self-assessment is increasingly prevalent in many organizations. Although managers perceive self-assessment as internally driven, the well-known link between organizational activities and the external environment suggests that outside forces play a signiﬁcant role. This investigation explores the external motivators of self-assessment through a ﬁeld study of 14 organizations. Five factors were found to link the conduct of self-assessment to the external environment: availability of an externally developed or sponsored model, presence of a boundary spanning individual, afﬁliation with professional and trade associations, pressure from powerful external entities, and potential for external reward or recognition. These ﬁndings suggest that self-assessment is driven signiﬁcantly by forces external to the organization. How these external factors combine to form the context of self-assessment may affect the outcomes of the project.</t>
@@ -8980,6 +9155,11 @@
       <c r="K165" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Qualitative field study conducted at the organizational level without extractable effect sizes.. Verbatim Evidence: [Abstract] "This investigation explores the external motivators of self-assessment through a field study of 14 organizations." [Research method] "The research was carried out in 14 organizations." [Research method] "While Glaser and Strauss’s (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion."</t>
         </is>
       </c>
     </row>
@@ -8994,6 +9174,16 @@
           <t>BSMA0163</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G166" t="inlineStr">
         <is>
           <t>In this paper we test the hypothesis that boundary spanning is a differentiated function that is not necessarily performed by one person, as assumed in much previous research. Using longitudinal network data collected during labor negotiations, we found that some individuals on the bargaining teams ("representatives") broker ties toward their opponents, while others ("gatekeepers") broker ties from their opponents; and some broker task-oriented ties (measured by flows of advice), while others broker socioemotional ties (measured by flows of trust). Differentiation of trust and advice brokerage roles was strong throughout the negotiations, while differentiation of representative and gatekeeper roles became more distinct as the contract deadline (and increased potential for role conflict) neared. This analytic distinction suggests that role conflict must be examined differently, both conceptually and methodologically, and widens the range of options available for managing potential role conflicts.</t>
@@ -9017,6 +9207,11 @@
       <c r="K166" t="inlineStr">
         <is>
           <t>1992</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>The study only reports correlations among mathematical network properties (structural brokerage roles, indegree, outdegree, centrality) derived from the same sociomatrices. It does not measure any substantive psychological or behavioral antecedents or outcomes (e.g., role conflict is theorized but not measured), providing no effect sizes of interest.. Verbatim Evidence: [The study lacks substantive effect sizes, only correlating network metrics with other network metrics.] Verbatim Evidence: "[Network Indices] From these data, separate sociomatrices for trust and advice were constructed for each time period on which there were data." [Network Indices] "Using this data, raw brokerage scores were calculated, following Gould and Fernandez (1989)." [RESULTS] "The relationship between brokerage scores and embeddedness can be seen in Table 3, which displays the zero-order correlations of the various brokerage scores with the appropriate measures for indegree and outdegree."</t>
         </is>
       </c>
     </row>
@@ -9031,6 +9226,16 @@
           <t>BSMA0164</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G167" t="inlineStr">
         <is>
           <t>Background: While participatory social network analysis can help health service partnerships to solve problems, little is known about its acceptability in cross-cultural settings. We conducted two case studies of chronic illness service partnerships in 2007 and 2008 to determine whether participatory research incorporating social network analysis is acceptable for problem-solving in Australian Aboriginal health service delivery. Methods: Local research groups comprising 13–19 partnership staff, policy officers and community members were established at each of two sites to guide the research and to reflect and act on the findings. Network and work practice surveys were conducted with 42 staff, and the results were fed back to the research groups. At the end of the project, 19 informants at the two sites were interviewed, and the researchers conducted critical reflection. The effectiveness and acceptability of the participatory social network method were determined quantitatively and qualitatively. Results: Participants in both local research groups considered that the network survey had accurately described the links between workers related to the exchange of clinical and cultural information, team care relationships, involvement in service management and planning and involvement in policy development. This revealed the function of the teams and the roles of workers in each partnership. Aboriginal workers had a high number of direct links in the exchange of cultural information, illustrating their role as the cultural resource, whereas they had fewer direct links with other network members on clinical information exchange and team care. The problem of their current and future roles was discussed inside and outside the local research groups. According to the interview informants the participatory network analysis had opened the way for problem-solving by “putting issues on the table”. While there were confronting and ethically challenging aspects, these informants considered that with flexibility of data collection to account for the preferences of Aboriginal members, then the method was appropriate in cross-cultural contexts for the difficult discussions that are needed to improve partnerships. Conclusion: Critical reflection showed that the preconditions for difficult discussions are, first, that partners have the capacity to engage in such discussions, second, that partners assess whether the effort required for these discussions is balanced by the benefits they gain from the partnership, and, third, that “boundary spanning” staff can facilitate commitment to partnership goals.</t>
@@ -9054,6 +9259,11 @@
       <c r="K167" t="inlineStr">
         <is>
           <t>2012</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>No effect size of interest. The study is a participatory case study reporting qualitative findings and descriptive network link means without a formal correlation matrix or extractable zero-order effect sizes.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] We conducted two case studies of chronic illness service partnerships in 2007 and 2008 to determine whether participatory research incorporating social network analysis is acceptable for problem-solving in Australian Aboriginal health service delivery." "[Survey] For the network component of the survey, we used the social network analysis technique described by Fried [37] and by Provan [21]." "[Results] The tables provide summary measures of the different types of links. The main finding from the data in Table 5 was a dense network of workers linked on the exchange of team care but a much less dense network of workers linked on the exchange of management and planning or policy development."</t>
         </is>
       </c>
     </row>
@@ -9068,6 +9278,16 @@
           <t>BSMA0165</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G168" t="inlineStr">
         <is>
           <t>This paper reports on an important subgroup of international boundary-spanners – immigrants and second or third generation migrants from the MNC’s home country living in the subsidiary host country. We take as our example the Nikkeijin (Japanese immigrants and their descendants) in Brazil. Such bicultural people are a largely unexplored source of boundary-spanning internationally competent talent for multinational enterprises. Using two different surveys, we ﬁnd that this group is recognized as a source of talent by Japanese MNCs, but that their HRM practices are not appropriate to attract and use them in their global talent management programmes.</t>
@@ -9091,6 +9311,11 @@
       <c r="K168" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>No effect size of interest. The study does not report a correlation matrix or any zero-order correlational effect sizes (r). It only reports means, t-tests, and factor loadings regarding language proficiency, traits, and HRM perceptions.. Verbatim Evidence: [Abstract] "Using two different surveys, we find that this group is recognized as a source of talent by Japanese MNCs, but that their HRM practices are not appropriate to attract and use them in their global talent management programmes." [Methodology] "These hypotheses are tested through two surveys: The first of these was a survey of Japanese-affiliates in Brazil, the second survey was of the Nikkeijin (Japanese Brazilians) themselves." [Methodology] "Five-point Likert scales were used for those questions (Appendix A)." [Methodology] "Additionally, t-tests were performed to measure the differences between the manufacturing and non-manufacturing sectors."</t>
         </is>
       </c>
     </row>
@@ -9142,6 +9367,16 @@
           <t>BSMA0167</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G170" t="inlineStr">
         <is>
           <t>The god of this paper is to iden@ the communication tactics that tiow management teams to successtiy coordinate without becoming overloaded, and to see whether successti coordination and fidom from overload independently Muence team pefiormance. We found that how much teams comnumicatti, what they communicated abou~ and the technologies they used to communicate prdlcted coordination and overload. Team coordination but not overload prdlcted team SUWSS.</t>
@@ -9165,6 +9400,11 @@
       <c r="K170" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Excluded due to multiple reasons: student sample (Management Game), team-level analysis, and measures team coordination/communication frequency rather than individual boundary spanning behavior.. Verbatim Evidence: [Excluded due to student sample, team-level analysis, and lack of valid BSB measure]. Verbatim Evidence: "[Participants and Procedure] Participants consisted of 277 students, organized into 50 five or six member teams, who participated in the Management Game during the Spring and Fall of 1997." "[Abstract] The goal of this paper is to identify the communication tactics that allow management teams to coordinate successfully without becoming overloaded and to see whether successful coordination and freedom from overload independently influence team performance." "[RESULTS] We used two measures of team performance in our analyses."</t>
         </is>
       </c>
     </row>
@@ -9179,6 +9419,16 @@
           <t>BSMA0168</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G171" t="inlineStr">
         <is>
           <t>The paper explores DiMaggio and Powell's thesis that under conditions of uncertainty organizational decision makers will mimic the behavior of other organizations in their environment. We add to their discussion by positing that managers are especially likely to mimic the behavior of organizations to which they have some type of network tie via boundary-spanning personnel. Data are presented on the charitable contributions of 75 business corporations to 198 nonprofit organizations in the Minneapolis-St. Paul metropolitan area in 1980 and 1984. Using logistic regression models, we found that a firm is likely to give more money to a nonprofit that was previously funded by companies whose CEOs and/or giving officers are known personally by the firm's boundary-spanning personnel. Firms are also likely to give greater contributions to a nonprofit that is viewed more favorably by the local philanthropic elite. We also found that a nonprofit is likely to receive more money from a corporation that previously gave money to nonprofits whose directors sit on the nonprofit's board. We concluded that managers utilize the information gathered through extraorganizational, interpersonal networks to make decisions on how to relate to other organizations in their task environment and achieve organizational ends.</t>
@@ -9202,6 +9452,11 @@
       <c r="K171" t="inlineStr">
         <is>
           <t>1989</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Firm and dyad-level analysis predicting corporate charitable contributions rather than individual boundary spanning behavior.. Verbatim Evidence: [Abstract] "Data are presented on the charitable contributions of 75 business corporations to 198 nonprofit organizations in the Minneapolis-St. Paul metropolitan area in 1980 and 1984." [Method] "Transactions between corporations and nonprofits. In the course of the 1981 and 1985 interviews we asked the administrator of each nonprofit to look at a list of all the publicly held firms in the metro area for 1980 and 1984, respectively, and to tell us the amount of corporate contributions his or her organization received from each." [Hypotheses and Models] "The units of analysis were the dyads formed by the 75 corporations and 198 nonprofits in the study population. The goal of this analysis was to identify a set of variables that have statistically significant effects on the size of contributions that corporation i made to nonprofit j in 1984."</t>
         </is>
       </c>
     </row>
@@ -9254,6 +9509,16 @@
           <t>BSMA0170</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G173" t="inlineStr">
         <is>
           <t>Purpose – More enterprises adopt open innovation by breaking technological or organizational boundaries to seek internal and external knowledge when they face a fiercely competitive environment, complex market demands, and increasingly rapid technological change. In this context, a knowledge search strategy is regarded as an effective means of obtaining inside and outside resources and an important way to break the innovation bottleneck. Moreover, information technology (IT) is deemed an important asset for sourcing knowledge, whereas absorptive capacity is seen as an indispensable ability for utilizing novel knowledge. Thus, this paper aims to test the role of knowledge search in open innovation and examine the mediating effect of absorptive capacity and the moderating effect of IT capability.</t>
@@ -9277,6 +9542,11 @@
       <c r="K173" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N=1,088 firms) using top managers as proxy informants for the establishment's knowledge search.. Verbatim Evidence: [Firm-level analysis and proxy informants]. Verbatim Evidence: "[Abstract] Using a sample of 1,088 Chinese firms’ data collected by the World Bank in 2012, this paper employs logistic regression to test the hypotheses." "[Method] Following a two-stage procedure, a screening phase over the phone and a face-to-face interview with the top manager of each establishment, the data is collected between December 2011 and February 2013." "[Measurement] In the questionnaire, the item “in what ways has this establishment introduced new products or services and new or improved process?” is used for identifying knowledge search."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 9
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -9330,6 +9330,12 @@
           <t>BSMA0166</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -9353,6 +9359,11 @@
       <c r="K169" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Included. The study provides a correlation matrix for individual-level boundary spanning behavior (acting as a bridge person) of Japanese self-initiated expatriates as rated by their supervisors.. Verbatim Evidence: [Sample] "We collected the evaluations of 91 Japanese SIEs which cover 57% of the total Japanese SIEs employed." [Measure] "Respondents were asked about the extent to which each SIE acts as a bridge between Japanese AEs and Chinese employees as well as between the Chinese operation and the headquarters in Japan." [Correlation Matrix] "Appendix 3: Descriptive statistics (Mean and Standard Deviation) and correlations of variables"</t>
         </is>
       </c>
     </row>
@@ -9471,6 +9482,16 @@
           <t>BSMA0169</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G172" t="inlineStr">
         <is>
           <t>The present study examines a set of organizational predictors of first moves. More specifically, the study employed organizational information-processing theory to derive a set of hypotheses relating organizational characteristics to the level of first- mover activity. This archival study used a pooled cross section-time series data set of domestic airlines over an 8-year period.
@@ -9495,6 +9516,11 @@
       <c r="K172" t="inlineStr">
         <is>
           <t>1992</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] Archival firm-level data of domestic airlines, not an individual-level employee sample.. Verbatim Evidence: [Code 2 &amp; Code 3] Archival firm-level data of domestic airlines, not an individual-level employee sample. Verbatim Evidence: "[Abstract] This archival study used a pooled cross section-time series data set of domestic airlines over an 8-year period." "[Method] As noted, the unit of analysis is the level of first-mover activity within each year. This level was calculated for each airline. for each year, by summing the number of times it initiated a first move in a specific year." "[Method] There were 197 observations in this study" "[Method] More specifically, the amount of boundary spanning was measured by the number of marketing vice-presidents as a percent of total vice-presidents and expenditures for promotion as a percent of sales."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 10
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -8424,6 +8424,16 @@
           <t>BSMA0148</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G151" t="inlineStr">
         <is>
           <t>Although cross-functional integration is important for research and development (R&amp;D), research about implications of cross-functional integration has been rather sparse. In new product development (NPD), no study to date has examined intrafirm as well as interfirm integration of key functions such as intrafirm R&amp;D–marketing–production together with interfirm integration of host R&amp;D–partner R&amp;D. Such marketing and operations interface contributes to a better understanding of how operational and marketing activities impact on competitiveness and firm performance. This study collected data from 202 electronics manufacturing firms operating in an emerging economy, mainland China and Hong Kong with international R&amp;D partnerships. The findings indicate that a high level of R&amp;D integration between firms improved NPD performance when cross-functional integration is based on existing rather than new product configurations and key technologies. Interestingly, in high distance situations, cross-functional integration in the production validation stage generated NPD success. The findings show that high environmental uncertainties lead to a high level of host and partner firms R&amp;D integration. However, product newness has no significant effects on R&amp;D integration in any of the NPD stages.</t>
@@ -8447,6 +8457,11 @@
       <c r="K151" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Firm-level analysis / Proxy informants rating firm inter-organizational partnerships and intra-firm project integration. Verbatim Evidence: [Methodology] "The ﬁnal sampling frame of the study consisted of 731 ﬁrms." [Methodology] "The study targeted two key informants for each ﬁrm to reduce the threat of common method variance" [Methodology] "The overall number of usable responses was 202 complete cases or approximately 27% response rate." [Measures] "–What is the approximate working hour overlap between your company and the foreign company?" [Measures] "–Jointly discuss customer's requirements at the beginning of the project."</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9350,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -9587,6 +9601,16 @@
           <t>BSMA0171</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G174" t="inlineStr">
         <is>
           <t>With an increasing overlap between the work and non‐work domain, more research is needed to understand the factors that relate to how individuals manage their boundaries across multiple roles (i.e., work roles, family roles). Using a sample of 498 individuals, we explored the relationships between personality, O*NET job characteristic variables, and boundary management styles. Results revealed that job responsibility and work structure related to cross‐role interruptions and work identity centrality. Further, conscientiousness was related to greater perceptions of boundary control, family identity centrality, and fewer interruptions of work, while neuroticism was related to fewer interruptions of non‐work. Finally, the present findings replicated four of six defined boundary management styles put forth in prior research. Theoretical and practical implications are discussed.                                         Practitioner points                                                                        Individuals may differ in how they enact boundaries between work and non‐work as related to their individual personality.                                                           The job in which one works may relate to the manner in which boundaries between work and non‐work are managed.                                                           Organizational efforts to help employees with boundary management may be improved if job context and employee individual differences are noted and accommodated.</t>
@@ -9610,6 +9634,11 @@
       <c r="K174" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Work-Family Boundary Management Trap. Verbatim Evidence: [Construct Homonymy Trap] Verbatim Evidence: "[Abstract] With an increasing overlap between the work and non-work domain, more research is needed to understand the factors that relate to how individuals manage their boundaries across multiple roles (i.e., work roles, family roles)." "[Participants] With respect to employment status, 94.8% reported full-time employment, while the remaining 5.2% reported part-time employment."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 11
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -8632,6 +8632,16 @@
           <t>BSMA0152</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G155" t="inlineStr">
         <is>
           <t>Purpose – Prior studies have largely overlooked the potentially negative consequences of a buyer’s relational capital (RC) with a supplier for supply-side resilience, assuming a positive linear relationship between the constructs. Meanwhile, the focus of research has been at an organisational level without incorporating the role of boundary spanning individuals at the interface between buyer and supplier. Drawing on social capital and boundary spanning theory, the purpose of this paper is to: re-examine the relationship between RC and supply-side resilience, challenging the linear assumption; and investigate how both the strength and diversity of a boundary spanner’s ties moderate this relationship.</t>
@@ -8655,6 +8665,11 @@
       <c r="K155" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Firm-level analysis of buyer-supplier relationships; measures structural network diversity (Blau's index) and communication frequency rather than purposive boundary spanning behavior.. Verbatim Evidence: [Section 3.1] "Our hypotheses were assessed using a survey-based approach in the context of an ongoing BSR, where the buyer reported on its fourth largest supplier." [Section 3.1] "An electronic survey was used where the initial sample consisted of 1,641 manufacturing firms (SIC codes 20–51) listed by Dun and Bradstreet." [Section 3.1] "The total number of completed and useful responses received was 248" [Table III] "RC3. My company's business relationship with this supplier is characterised by high levels of respect" [Section 3.4.2] "For BSPTs, we followed Collins and Clark (2003) by asking respondents to identify the number of contacts in each of seven categories of actors ... in the corresponding supplier organisation. Tie diversity was then measured using Blau's (1977) index of diversity" [Section 3.4.2] "Interaction frequency was measured as the average number of times per month that an individual in the buyer firm interacted with their identified contacts within the supplier."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 12
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -1727,7 +1727,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Qualitative study (autoethnography) lacking extractable quantitative effect sizes.. Verbatim Evidence: [Abstract] "The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro’s anti-doping policy with WADA." [3.2. Collaborative Autoethnography] "Qualitative in nature, autoethnography is a method that shifts the attention from the perceived reality of research participants to the researcher him/herself (as a subject), thereby giving them a voice towards explaining the phenomenon under study in a self-reflective and often critical, fashion (Ellis &amp; Bochner, 2000)."</t>
+          <t>Qualitative study (autoethnography) lacking extractable quantitative effect sizes.. Verbatim Evidence: [Abstract] "The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegroâs anti-doping policy with WADA." [3.2. Collaborative Autoethnography] "Qualitative in nature, autoethnography is a method that shifts the attention from the perceived reality of research participants to the researcher him/herself (as a subject), thereby giving them a voice towards explaining the phenomenon under study in a self-reflective and often critical, fashion (Ellis &amp; Bochner, 2000)."</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>[Code 4 &amp; Code 3 &amp; Code 1] Conceptual paper on macro-level supply chain network design.. Verbatim Evidence: [Conceptual study on supply chain network design]. Verbatim Evidence: "[Abstract] Designing a supply chain network provides the basic structure for supply chain operations, where the network is a ma-jor element in a ﬁrm’s competitiveness and a signiﬁcant area ofcapital investment." "[1. Introduction] In this article, the impact of the supply chain move-ment on facility location analysis will be examined tosee the challenges posed to traditional location method-ology."</t>
+          <t>[Code 4 &amp; Code 3 &amp; Code 1] Conceptual paper on macro-level supply chain network design.. Verbatim Evidence: [Conceptual study on supply chain network design]. Verbatim Evidence: "[Abstract] Designing a supply chain network provides the basic structure for supply chain operations, where the network is a ma-jor element in a ï¬rmâs competitiveness and a signiï¬cant area ofcapital investment." "[1. Introduction] In this article, the impact of the supply chain move-ment on facility location analysis will be examined tosee the challenges posed to traditional location method-ology."</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix.. Verbatim Evidence: [Reason summary] The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix. Verbatim Evidence: "[Sampling and data collection procedure] The research team received approval from 14 hotels’ Management to collect data from their FLEs." "[Sampling and data collection procedure] At time II 309 questionnaires were redistributed, and 250 responses were used after deletion of unusable and incomplete questionnaires." "[Measures] Staffs’ COBSBs were assessed with the scale developed by Bettencourt et al. (2005) that measures service delivery with 5 items, internal influence and external representation with both 4 items." "[Results] Table 2. Intercorrelations and discriminant validity criterion."</t>
+          <t>The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix.. Verbatim Evidence: [Reason summary] The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix. Verbatim Evidence: "[Sampling and data collection procedure] The research team received approval from 14 hotelsâ Management to collect data from their FLEs." "[Sampling and data collection procedure] At time II 309 questionnaires were redistributed, and 250 responses were used after deletion of unusable and incomplete questionnaires." "[Measures] Staffsâ COBSBs were assessed with the scale developed by Bettencourt et al. (2005) that measures service delivery with 5 items, internal influence and external representation with both 4 items." "[Results] Table 2. Intercorrelations and discriminant validity criterion."</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Valid measurement of Leader Boundary Spanning Behavior (scouting, persuading) with real employee sample and extractable correlation matrix.. Verbatim Evidence: [Sample] "Data were collected from 92 management teams from 92 public educational organizations in Israel." [Sample] "School administrators, usually the principal, typically serve as the leaders of these teams." [Measures] "external scouting (six items, for example, “How often does the leader seek information and advice from peers for the team’s benefit,” α = .89); external persuading (seven items, for example, “How often does the leader act as a representative of the team with parts of the school environment” [parents, educational ministry, district], α = .92)" [Correlation Matrix] "Table 1. Descriptive Statistics and Intercorrelation Matrix for Study Variables, N = 92."</t>
+          <t>Valid measurement of Leader Boundary Spanning Behavior (scouting, persuading) with real employee sample and extractable correlation matrix.. Verbatim Evidence: [Sample] "Data were collected from 92 management teams from 92 public educational organizations in Israel." [Sample] "School administrators, usually the principal, typically serve as the leaders of these teams." [Measures] "external scouting (six items, for example, âHow often does the leader seek information and advice from peers for the teamâs benefit,â Î± = .89); external persuading (seven items, for example, âHow often does the leader act as a representative of the team with parts of the school environmentâ [parents, educational ministry, district], Î± = .92)" [Correlation Matrix] "Table 1. Descriptive Statistics and Intercorrelation Matrix for Study Variables, N = 92."</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Methodology] "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000)." [Methodology] "More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sources—documentary data, in-depth interviews, and digital data—to obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit."</t>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Methodology] "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000)." [Methodology] "More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sourcesâdocumentary data, in-depth interviews, and digital dataâto obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit."</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Sample and data collection] "Overall, we received usable data from 244 respondents in 122 units, yielding a response rate of 76.7 percent." [Measures] "In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit." [Level of analysis] "We performed three tests to determine whether the data should be aggregated to the unit level (see Table 1)." [RESULTS] "Table 2. Means, standard deviations, and Pearson’s correlations between research variables... N = 122"</t>
+          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Sample and data collection] "Overall, we received usable data from 244 respondents in 122 units, yielding a response rate of 76.7 percent." [Measures] "In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit." [Level of analysis] "We performed three tests to determine whether the data should be aggregated to the unit level (see Table 1)." [RESULTS] "Table 2. Means, standard deviations, and Pearsonâs correlations between research variables... N = 122"</t>
         </is>
       </c>
     </row>
@@ -5689,6 +5689,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>While there is a burgeoning trend to recognize leadership as an important enabler of new venture development and growth, scant research has explored the performance mechanisms of shared leadership in the entrepreneurial context. Based on the information processing perspective, we propose a moderated mediation model to examine how shared leadership in entrepreneurial teams advance new venture performance by identifying team reflexivity as a pivotal mediator and team boundary spanning as a crucial contingency. The data set from a cross-industry sample of 94 entrepreneurial teams indicated that shared leadership exerts a positive indirect influence on new venture performance via team reflexivity; and team boundary spanning moderates such indirect influence. Finally, how our findings contribute to the entrepreneurship, leadership, team research, and managerial practice are discussed.</t>
@@ -5830,6 +5831,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>A number of studies have found that the performance of NPD projects greatly depends on the support they get from top management. However, research into why some projects get more support than others has been limited. The present paper takes a political approach to NPD, in which top management support is considered to be a function of a project leader’s ability to influence decision processes through personal relationships. Mobilizing the bridging perspective of social capital, we argue that project leaders need both strong ties to high-ranking others and sparseness in their networks. Vertical strong ties bring direct support and solidarity, resulting in improved access to resources and priority over other projects; sparseness provides exposure to the full range of information and interpretations in the organization, resulting in a more accurate picture of the political landscape and thus enabling the implementation of an appropriate influence strategy. A PLS analysis of a sample of 73 French project leaders involved in NPD projects provided support for our hypotheses. Hence, we contribute to a very recent stream of research showing that the structural and relational dimensions of social capital are complementary.</t>
@@ -6211,6 +6213,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>This paper contributes to open innovation (OI) and boundary spanning literatures by providing a first understanding of industry‐based boundary spanners in university‐industry (U‐I) collaboration through case studies of Chinese multinational corporations (MNCs) and their international OI platforms. Organisational roles created by these platforms within the MNCs and their activity of bridging between organisations are examined. The analysis of 25 in‐depth interviews in two MNCs located in eight countries, along with internal documents, sheds light on U‐I collaboration practices implemented by Chinese MNCs. Two new boundary spanning roles are identified:               Dual Cultural Bridger               – as these OI platforms bridge organisational and national cultural gaps to prevent and solve problems in the collaborative process; and               International Network Enhancer               – as these OI platforms act as trust building and local knowledge listening posts for the MNC’s global network. Managerial and policy implications are provided.</t>
@@ -6404,6 +6407,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>In this paper, we highlight the networked context of the professions. In particular, we indicate that neo-classical professionals tend to work across organizational boundaries in project teams, often to meet the needs of clients and the wider society. However, little is known about the resources that professionals draw on to meet immediate, fast paced, client demands in project network organizations (PNOs). We pinpoint how knowledge resources, human, social and organizational capital enable professionals to produce outputs at a fast pace/tempo. Temporality emerged as an unexpected but key issue in our empirical research and we explore this further here. First, we put forward how professional work organization(s) has changed by focusing on the boundaries of organizations, and how this is often temporary and project-driven. Second, we use the speciﬁc lens of knowledge resources which are drawn upon to enable networked working and ask the question: which knowledge resources enable professionals to work at a fast pace within networks? Third, appreciative of the vast literature on temporary and networked organizations in professional work, our focus is beyond a single profession or organization, and hence, we build upon the prior research on PNOs. We do this by drawing on empirical data of a humanitarian aid project networked organization (HN) that upscales across its network at high speed, often within days, to generate funds for humanitarian disasters in order to save lives.</t>
@@ -6451,6 +6455,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>This research examines the mechanisms through which entrepreneurial orientation (EO) aﬀects ﬁrm performance in an emerging market context. We argue that EO drives ﬁrms to develop the dynamic capabilities of absorptive capacity (ACAP) and boundary-spanning (BS), and that these capabilities enhance ﬁrm performance. Moreover, the eﬀectiveness of these knowledge- and network-based dynamic capabilities in mediating the EOperformance relationship is contingent on the institutional conditions ﬁrms are exposed to. We test our hypotheses using multi-sourced data on Chinese high-tech ﬁrms in business-to-business (B2B) markets. Our results show that ACAP and BS mediate the positive eﬀect of EO on ﬁrm performance, and that as the development of market-supporting institutions improves, the mediating eﬀect of ACAP becomes stronger while that of BS weakens.</t>
@@ -6498,6 +6503,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Effective work groups engage in external knowledge sharing—the exchange of information, know-how, and feedback with customers, organizational experts, and others outside of the group. This paper argues that the value of external knowledge sharing increases when work groups are more structurally diverse. A structurally diverse work group is one in which the members, by virtue of their different organizational affiliations, roles, or positions, can expose the group to unique sources of knowledge. It is hypothesized that if members of structurally diverse work groups engage in external knowledge sharing, their performance will improve because of this active exchange of knowledge through unique external sources. A field study of 182 work groups in a Fortune 500 telecommunications firm operationalizes structural diversity as member differences in geographic locations, functional assignments, reporting managers, and business units, as indicated by corporate database records. External knowledge sharing was measured with group member surveys and performance was assessed using senior executive ratings. Ordered logit analyses showed that external knowledge sharing was more strongly associated with performance when work groups were more structurally diverse. Implications for theory and practice around the integration of work groups and social networks are addressed.</t>
@@ -6545,6 +6551,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>Our study responds to a call for research to integrate institutional, organizational and individual levels of analysis in examining the implications for work and employment relations of new organizational forms. We empirically examine the implementation of network forms of genetics healthcare delivery that cross organizational and professional boundaries. We highlight that less powerful professional groups may find difficulty in enacting boundary-spanning roles associated with new organizational forms. This is due, first, to inconsistency of government policy, which fragments organizations. Second, professional institutions sustain professional hierarchy and power differentials.</t>
@@ -6592,6 +6599,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to test the inﬂuence of external information search (EIS) on knowledge elaboration and group cognitive complexity (GCC) under the moderating effect of absorptive capacity (AC is indicated by prior knowledge base and gender diversity).</t>
@@ -6738,6 +6746,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>The aim of this research is to empirically investigate the relationships among the three vital knowledge management processes of acquisition, integration and application, and their effects on organisational innovation in the pharmaceutical manufacturing industry in Jordan; a knowledge-intensive business service (KIBS) sector. Structural equation modelling findings show an excellent fit among all these processes and innovation, with positive and significant relationships. Moreover, knowledge integration and knowledge application emerged as having strong and significant mediation effects upon the relationship between knowledge acquisition and innovation. As such, an organisation’s innovation efforts would significantly benefit from the synergistic effects of properly integrating and applying externally acquired knowledge. The findings make a valuable contribution to pharmaceutical knowledge management and innovation literature, especially in an era of open innovation. Pharmaceutical companies are advised to focus on developing proficient assimilation and application capabilities in order for acquired knowledge to have notable effects on their innovation performance.</t>
@@ -6832,6 +6841,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6926,6 +6936,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>This study investigated coordinated action in multiteam systems employing 233 correspondent systems, comprising 3 highly specialized 6-person teams, that were engaged in an exercise that was simultaneously “laboratory-like” and “field-like.” It enriches multiteam system theory through the combination of theoretical perspectives from the team and the large organization literatures, underscores the differential impact of large size and modular organization by specialization, and demonstrates that conventional wisdom regarding effective coordination in traditional teams and large organizations does not always transfer to multiteam systems. We empirically show that coordination enacted across team boundaries at the component team level can be detrimental to performance and that coordinated actions enacted by component team boundary spanners and system leadership positively impact system performance only when these actions are centered around the component team most critical to addressing the demands of the task environment.</t>
@@ -7020,6 +7031,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>In this article, the authors examine antecedents and consequences of the service climate in boundary-spanning self-managing teams (SMTs) that deliver financial services. Using data from members of 61 SMTs and their customers, the authors show a differential impact of the SMT service climate on various marketing performance measures. Furthermore, they obtain support for independent group-level effects of intrateam support and team member flexibility on employee perceptions of the SMT service climate. Both effects are persistent over time and demonstrate that collective perceptions in the SMT have incremental value in the explanation of the service climate.</t>
@@ -7306,6 +7318,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -7400,6 +7413,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>This article develops a framework for studying cross-functional teams in organizations that focuses on three domains: organizational context, internal process, and outcome measures. The framework was developed from qualitative data from over 200 individual and group interviews, written descriptions, and team observations. We then operationally defined this model through a set of questionnaire items and validated it through quantitative analysis of data from 565 members of cross-functional teams. The resulting framework provides a base for the future study of cross-functional teams.</t>
@@ -7447,6 +7461,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>When working as a member of a team, individuals must make decisions concerning the allocation of resources (eg, effort) toward individual goals and team goals. As a result, individual and team goals, and feedback related to progress toward these goals, should be potent levers for affecting resource allocation decisions. This research develops a multilevel, multiple-goal model of individual and team regulatory processes that affect the allocation of resources across individual and team goals resulting in individual and team performance. On the basis of this model, predictions concerning the impact of individual and team performance feedback are examined empirically to evaluate the model and to understand the influence of feedback on regulatory processes and resource allocation. Two hundred thirty-seven participants were randomly formed into 79 teams of 3 that performed a simulated radar task that required teamwork. Results support the model and the predicted role of feedback in affecting the allocation of resources when individuals strive to accomplish both individual and team goals.</t>
@@ -8045,7 +8060,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>Construct Homonymy (Boundaryless Career). The study measures cross-boundary mobility preferences (career mobility / turnover intention) across jobs, organizations, and industries, not interpersonal Boundary Spanning Behavior.. Verbatim Evidence: [Introduction] "First, we take into account the multiplicity of career boundaries (job, organisation and industry), refining the understanding of ‘boundary’ in boundaryless careers (Inkson et al. 2012)." [Measures] "For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference." [Measures] "We created the mobility preference variables using individuals’ responses to this question: ‘In regard to your job, where do you want to be in 12 months’ time?’"</t>
+          <t>Construct Homonymy (Boundaryless Career). The study measures cross-boundary mobility preferences (career mobility / turnover intention) across jobs, organizations, and industries, not interpersonal Boundary Spanning Behavior.. Verbatim Evidence: [Introduction] "First, we take into account the multiplicity of career boundaries (job, organisation and industry), refining the understanding of âboundaryâ in boundaryless careers (Inkson et al. 2012)." [Measures] "For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference." [Measures] "We created the mobility preference variables using individualsâ responses to this question: âIn regard to your job, where do you want to be in 12 monthsâ time?â"</t>
         </is>
       </c>
     </row>
@@ -8461,7 +8476,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>Firm-level analysis / Proxy informants rating firm inter-organizational partnerships and intra-firm project integration. Verbatim Evidence: [Methodology] "The ﬁnal sampling frame of the study consisted of 731 ﬁrms." [Methodology] "The study targeted two key informants for each ﬁrm to reduce the threat of common method variance" [Methodology] "The overall number of usable responses was 202 complete cases or approximately 27% response rate." [Measures] "–What is the approximate working hour overlap between your company and the foreign company?" [Measures] "–Jointly discuss customer's requirements at the beginning of the project."</t>
+          <t>Firm-level analysis / Proxy informants rating firm inter-organizational partnerships and intra-firm project integration. Verbatim Evidence: [Methodology] "The ï¬nal sampling frame of the study consisted of 731 ï¬rms." [Methodology] "The study targeted two key informants for each ï¬rm to reduce the threat of common method variance" [Methodology] "The overall number of usable responses was 202 complete cases or approximately 27% response rate." [Measures] "âWhat is the approximate working hour overlap between your company and the foreign company?" [Measures] "âJointly discuss customer's requirements at the beginning of the project."</t>
         </is>
       </c>
     </row>
@@ -8617,7 +8632,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>Systematic literature review, no primary effect sizes.. Verbatim Evidence: [Abstract] This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in business–to–business (B2B) interorganizational relationships, pointing out directions for future research. [Methodology] A systematic literature review allows the synthesizing of results and evidence from existing studies and producing new knowledge.</t>
+          <t>Systematic literature review, no primary effect sizes.. Verbatim Evidence: [Abstract] This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in businessâtoâbusiness (B2B) interorganizational relationships, pointing out directions for future research. [Methodology] A systematic literature review allows the synthesizing of results and evidence from existing studies and producing new knowledge.</t>
         </is>
       </c>
     </row>
@@ -9085,7 +9100,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>Qualitative ethnographic case study lacking an extractable quantitative effect size or correlation matrix.. Verbatim Evidence: [Abstract] "Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the company’s transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities." [Methodological aspects: Embedded in a utility] "To flesh out the reorganisation of a municipal utility and better capture the ‘socio-technical geometry of powers in town’ (Graham and Marvin, 2001), I decided to immerse myself directly in this technical world by being embedded within the teams of infrastructure management of a German multi-utility."</t>
+          <t>Qualitative ethnographic case study lacking an extractable quantitative effect size or correlation matrix.. Verbatim Evidence: [Abstract] "Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the companyâs transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities." [Methodological aspects: Embedded in a utility] "To flesh out the reorganisation of a municipal utility and better capture the âsocio-technical geometry of powers in townâ (Graham and Marvin, 2001), I decided to immerse myself directly in this technical world by being embedded within the teams of infrastructure management of a German multi-utility."</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9204,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 3] Qualitative field study conducted at the organizational level without extractable effect sizes.. Verbatim Evidence: [Abstract] "This investigation explores the external motivators of self-assessment through a field study of 14 organizations." [Research method] "The research was carried out in 14 organizations." [Research method] "While Glaser and Strauss’s (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion."</t>
+          <t>[Code 1 &amp; Code 3] Qualitative field study conducted at the organizational level without extractable effect sizes.. Verbatim Evidence: [Abstract] "This investigation explores the external motivators of self-assessment through a field study of 14 organizations." [Research method] "The research was carried out in 14 organizations." [Research method] "While Glaser and Straussâs (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion."</t>
         </is>
       </c>
     </row>
@@ -9365,6 +9380,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -9720,6 +9736,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>This study investigated how a project group deals with the contradiction between distributed knowledge in boundary-spanning collaborative processes and the expectation that software systems will provide unified, codified knowledge. It employed an ethnographic, interpretive approach to examine the ways in which relevant knowledge was presented, recognized, shared or otherwise managed during a project concerned with the joint design of business process and IT systems change. Developing a group understanding of how to manage sensemaking and expertise across salient knowledge boundaries were discovered to be central to perceptions of project completion. Four stages of this development were identified. The contribution of this paper is to propose these stages as the basis for boundary-spanning group management approaches and to suggest ways of progressing the complexities of communication, consensus-building, information exchange, problem-formulation and solution-brokering that are fundamental to collaboration in IS definition. These processes are normally taken for granted, rationalized or ignored by managers of IT-related organizational change. The use of specific types of boundary-object may aid in managing such processes explicitly and ensuring rapid progress. Thus the findings have significant implications for research and practice in other forms of boundary-spanning group collaboration, such as organizational innovation and problem-solving.</t>
@@ -10002,6 +10019,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -10190,6 +10208,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>Global offshoring has become a key strategy for international staffing, especially in the software industry. Global software teams engage in boundary spanning activities that may help MNEs achieve international connectivity and cope with external disruptions through their use of virtual work. However, offshoring IT professionals who bridge these boundaries in offshoring MNEs must contend with discontinuities, or perceived disruptions in expected communication flows, which impact their job satisfaction. Drawing on survey data from 193 professional consultants from an IT services offshoring MNE located primarily in Eastern Europe and working for a U.S. client, we test a model grounded in Organizational Discontinuity Theory. We find that potential discontinuities arising from the virtual work environment have no impact on the job satisfaction of offshoring IT professionals, but that those who experience team-level continuities of identification and shared vision are more satisfied with their jobs. Our findings suggest that virtual work may have become normalized such that it is not problematic in and of itself, and that fostering connectivity in boundary spanning global teams may be beneficial for MNEs. Our findings have important implications for MNEs managing disruptions created by global work arrangements as well as exogenous disruptions.</t>
@@ -10237,6 +10256,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>Acknowledgements: This research was funded by NSF grant #0422676 and #0726798 as well as support provided by the University of California, Irvine Center for Research on Information Technology in Organizations. The authors would like to acknowledge the helpful comments provided by Christopher Earley, Mark Griffin, John Mathieu, and Jone Pearce; assistance in data collection provided by Diaky Diaz, Christopher Reisdel and Bettina Wolf; and the generous time invested by all the film makers and film viewers who participated in the study.</t>
@@ -10368,6 +10388,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -12991,6 +13012,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>Two main targets of contemporary preferential innovation policy support, especially in Europe, are key enabling technologies (KETs) and innovation ‘missions’ focused on solving societal challenges. Both topics are associated with uniting disparate sets of capabilities, either by driving technology-based innovation into various application domains or by eliciting interdisciplinary and cross-sectoral solutions to urgent societal demands. In this study we assess to what extent pre-commercial R&amp;D collaborations span geographic and cognitive boundaries. We analyze firm-level tie formation in Dutch collaborative R&amp;D projects initiated in the period 2013–2018. Gravity models reveal that, while results for geographic proximity are mixed, some KET types are indeed related to projects in which cognitive proximity is significantly less relevant for tie formation. This contrasts with the findings for projects that retroactively received a mission label. Projects on health and care missions, and especially energy transition and sustainability missions, instead spur collaborations between cognitively proximate firms. The latter suggests that without additional policy intervention, such projects might interconnect similar rather than dissimilar knowledge bases. We conclude by discussing research and policy implications.</t>
@@ -13038,6 +13060,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -15894,6 +15917,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>Science parks are a type of organizational sponsorship initiative aimed at generating resource-munificent environments through the provision of bridging and buffering services. While extant research has studied the relationship between these services and firm outcomes, it has neglected to provide insights into when tenant firms utilize these services to a greater or lesser extent. Our study evaluates science parks’ buffering mechanism and identifies firm-level characteristics affecting tenants’ use intensity of buffering services. To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries. Taking a resource dependence perspective, our findings indicate that tenants’ managerial resources (particularly top management team size and functional experience) and boundary-spanning capacity jointly determine the extent to which firms rely upon the science park’s buffering mechanism. This study contributes to the organizational sponsorship, resource dependence, and science park literatures, as well as has important practical implications.</t>
@@ -16025,6 +16049,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the effects of relationship bonds on the psychological response and behavior of bank employees based on the job demands–resources theory. Specifically, it examines the effects of relationship bonds in terms of person–job (P–J) fit, emotional exhaustion, job satisfaction and boundary-spanning behaviors, all of which comprise the behavioral dimensions of bank employees. In addition, the study examines how the resiliency of bank employees influences their emotional exhaustion and determines whether a moderating effect related to emotional exhaustion exists.</t>
@@ -16072,6 +16097,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -16265,6 +16291,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>Innovation is a risky business. Notwithstanding the attention in research on the determinants of innovation success, the estimates of the extremely high failure rates (ranging from 40% to 90%) have not come down. As a result, new approaches have to be found to address the issues that prevent organizations from reaching innovation success over a longer period of time. In this study, Signal Detection Theory (SDT) is introduced to show that it may be less important to improve innovation practices in companies, than it is to change the nature of the projects that enter the corporate innovation funnel. In our empirical study of 44 innovation projects in the pharmaceutical and electronics industry, we show that pursuing more noisy signals (uncertain technological and market opportunities) is currently beneficial for innovation success. In general, companies allocate too few resources to noisy innovation opportunities. Interestingly, we find a positive, and not an inverted U-shaped, relationship between noise/signal ratios and innovation success. This indicates that there are almost no companies that take too much risk in the current competitive environment and that many can gain from increasing their noise tolerance. The implications from this study are quite counter-intuitive in a sense that ‘risk’ is not the cause of the innovation problems, but may be a solution.</t>
@@ -16406,6 +16433,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>Past research on team boundary work has focused on a “cold,” information-exchange perspective to explain why boundary activities affect team innovation. Although the theory is widely accepted, empirical studies on the actual mechanism are scant and produce inconsistent results. Drawing from Interaction Ritual Theory (Collins, 2004), we propose a “warm,” affective perspective that emphasizes team emotional energy - a shared feeling of enthusiasm among team members - as a mechanism linking boundary work and team innovation. Moreover, we examine a theory-driven contextual factor -team role overload - that modifies the hypothesized mediated relationship. Based on field data from four different sources of 89 automotive research and development teams (comprising 724 employees, 89 direct supervisors and 18 managers), we found that both team boundary-spanning and boundary-buffering activities are associated with higher levels of team emotional energy, which, in turn, are related to greater levels of team innovation. Moreover, the mediated relationship of boundary-buffering activities, team emotional energy and team innovation is moderated by team role overload, such that the mediated relationship is stronger when team role overload is higher. Our study contributes to the literature by broadening our understanding of why boundary work is effective and when it matters most.</t>
@@ -16500,6 +16528,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>Boundary spanning activity Is conceived of as an intervening variable between organization structure and perceived environmental uncertainty. This is because boundary spanners operate at the skin of the organization and hence their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relationships between perceived environmental uncertainty, organization structure, and boundary spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relationships were found between all three variables. Partial relationships indicated that PEtJ does not influence the boundary spanning-structure relationship, but structure reduces the PEtJ-boundary spanning relationship to zero, and boundary spanning reduces the structurePEU relationship to zero. Thus, not only is the boundary spanning as an intervening variable supported, but results suggest that causality in the Btructure-PEU relationship may be in the direction of structure to PEU rather than current contingency notions of PEU effecting structure.</t>
@@ -16547,6 +16576,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>Boundary-spanning activity is conceived of as an intervening variable between organization structure and perceived environmental uncertainty (PEU). This is due primarily because, since boundary spanners operate at the skin of the organization, their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relations between PEU, organization structure, and boundary-spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relations were found between all three variables. Partial relations indicated that PEU does not influence the relationship of boundary spanning to structure but structure reduces the relationship of PEU to boundary spanning to zero, and boundary spanning reduces the relationship between structure and PEU to zero. Thus, not only is the notion of boundary spanning as an intervening variable supported, but results suggest that causality in the relationship between structure and PEU may be from structure to PEU rather than current contingency notions of PEU affecting structure.</t>
@@ -16594,6 +16624,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>Building on the theories of knowledge recombination, we argue that the external acquisition of technologies acts as a boundary spanning mechanism that impacts on the recipient firm’ subsequent technology development. The effect is moderated by two additional mechanisms, namely the retention of star scientists and the experience in upstream strategic alliances. We tested our hypotheses on a sample of 6208 USPTO patented technologies acquired by 350 biotechnology firms over the period 1980–2012. Findings reveal an inverted U-shaped effect of the pioneering nature of the acquired technology on firm’s subsequent developments, in terms of (self) citations of firm’s subsequent patents to the acquired one. Moreover, the main relationship is negatively moderated by the retention of star scientists, while the experience in upstream alliances demonstrates to be a positive moderator.</t>
@@ -16641,6 +16672,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>Successful product development requires managing tensions—coping with fluctuating contingencies to foster innovation and efficiency. To investigate this challenge, we explored the nature, dynamics, and impacts of contrasting project management styles. Our conceptual framework details emergent and planned styles. Following 80 projects over two-year periods, we find that these styles offer disparate but interwoven approaches to monitoring, evaluation, and control activities; use of these activities fluctuates over time; a paradoxical blend of styles enhances performance; and uncertainty moderates project management-performance relationships.</t>
@@ -16688,6 +16720,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>Boundary spanning has been proven to have positive implications for innovation performance; yet, some individuals are less boundary-spanning than others. Drawing on the attachment theory and organizational support theory, this study develops a multi-level theoretical model to investigate how individuals’ attachment insecurity influences boundaryspanning behavior through self-efficacy and the moderating role of organizational support climate. To validate the proposed model, we adopted a survey research, and collected data from NPD project teams in China. The results revealed that both insecure attachment styles were associated with lower levels of individual boundary-spanning behavior, and self-efficacy partially mediated these relationships. Moreover, organizational support climate played a moderating role in the relationship between attachment anxiety and boundary-spanning behavior. With a high level of support climate, the negative impact of attachment anxiety on boundary-spanning behavior was weakened. This elucidates the role of individual affective motivation and team shared perceptions in shaping individual externally focused behavior.</t>
@@ -16787,6 +16820,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>From a knowledge-based perspective, this paper highlights the need for a framework linking perceived competition of the industry and ﬁrms’ strategic location choices of external knowledge search and examines whether the perceived competition increases the propensity of cluster ﬁrms to search more widely from extra-cluster knowledge sources than intra-cluster knowledge sources. Furthermore, we emphasise that cluster ﬁrms with varying degrees of tacitness in their knowledge base might respond to such competition diﬀerently when conducting external knowledge search activities. Using a sample of 310 cluster ﬁrms in the Zhejiang Province of China, we ﬁnd that the cluster ﬁrm would increase the propensity for more geographic boundary-spanning search relative to local search while under the pressure of competition. Moreover, the positive relationship between perceived competition and the propensity towards geographic knowledge search is weaker when the tacitness of the cluster ﬁrm’s knowledge base is higher. The ﬁndings contribute to the understanding of the relationship between competition and the choice of location strategies in external knowledge search.</t>
@@ -17688,6 +17722,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>Based on the social identity theory, this study investigates whether and how employee perceptions of corporate environmental behavior (CEB) influence the realization of an organization's internal value. Using employees' organizational citizenship behavior (OCB) as a direct agent for corporate internal value, the current study constructs a theoretical model of perceived CEB and OCB, with work meaningfulness and person–organization (P-O) value fit serving as mediator and moderator, respectively. After analyzing 235 questionnaire samples, we discovered that the perceived CEB positively influenced OCB via work meaningfulness and that this positive effect was strengthened by a greater P-O value fit. These findings suggest that in the process of motivating employees to implement OCB, firms should address the significance of internal driving roles of work meaningfulness and boundary-spanning roles of P-O value fit in order to enhance corporate internal value and correct managers' misconceptions about the value of CEB.</t>
@@ -17735,6 +17770,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F378" t="inlineStr"/>
       <c r="G378" t="inlineStr">
         <is>
           <t>A central focus of cross-cultural management research is how individuals and organizations differ across national cultures and how that fundamentally shapes their thoughts and actions and serves as a unit of identification. In this article, we critically reconsider the essential categorical nature of culture, problematizing categorization and questioning national culture as the primary basis of differentiation. We draw on intersectionality, an approach that helps understand how multiple categories are experienced by the individual, and on relationality, an approach that conceptualizes people, organizations, and their actions within dynamic patterns of relations and cultural meanings. Both approaches challenge the primacy, unity, and separateness of any given category, the a priori determination of categories (and associated boundaries) in research, and the nature and stability of boundaries. Based on this we advance notions of boundary work and boundary shifting that help explore how today’s sociocultural groups and categories, and the boundaries that separate them, emerge and change. We conclude that, while the extant crosscultural literature has come far in identifying differences, relationality and intersectionality can enable cross-cultural scholars to engage in research practice that better reflects the complexities of sociocultural life. We contribute to theory by suggesting why and how these two approaches can be used to explore complex cross-cultural management phenomena.</t>
@@ -17782,6 +17818,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F379" t="inlineStr"/>
       <c r="G379" t="inlineStr">
         <is>
           <t>The paper explores how formal leaders make sense of and deal with autonomy of knowledge-workers. Based on interviews, I suggest that leaders make sense of knowledge-workers’ autonomy as ranging from perfectly autonomous to too autonomous to less independent to acting childish. This ambiguity was dealt with by making sense of leading as ranging from facilitative and supportive approaches to more controlling, even reprimanding acts. This empirical investigation of constructions of ‘leader/ship’ and ‘followers’ contributes to leader/ship-follower/ship literature. The paper’s contribution to theory lies in the notion of situated ambiguity; a way to understand the emerging way through which formal leaders navigate and smoothly move between their own diﬀering perspectives, diﬀerent practical situations, various culturally acceptable understandings of leaders and knowledgeworkers.</t>
@@ -17903,6 +17940,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>Building on the “loose coupling” logic, this study examines the importance of boundary spanners' shared perceptions of procedural justice in cross-cultural cooperative alliances. I argue that alliance profitability is higher when both parties perceive high rather than low procedural justice. Profitability is also higher when both parties' perceptions are high than when one party perceives high procedural justice but the other perceives low procedural justice. Shared justice perceptions become even more important for alliance profitability when the cultural distance between partners is high or when the industry of operation is uncertain. Analysis of 124 cross-cultural alliances in China supports these propositions.</t>
@@ -17950,6 +17988,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>This study extends research on strategic alliances by exploring independent and combined effects of distributive, procedural, and interactional justice in these alliances. An integrated framework links cooperation payoffs with organizational justice as perceived by boundary-spanning alliance executives, through whom justice perceptions become parent actions. Analysis of 127 alliances demonstrates that when goal differences between parties are high, the joint effect on alliance performance of procedural and distributive justice is significantly positive. When interactional justice is high, procedural justice exerts a stronger performance effect. This perspective enriches alliance research, especially regarding procedural formalization, incentive structure, and interparty attachment.</t>
@@ -17997,6 +18036,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19176,6 +19216,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>The purpose of this research is to determine the description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, to determine and analyze the influence of Emotional Dissonance on Service Sabotage, to determine and analyze the influence of Emotional Intelligence on Service Sabotage, and to determine and analyze the influence of Emotional Exhaustion on Service Sabotage. The population in this study were all employees of the Grand Mercure Hotel Kemayoran Jakarta. In this research, a quantitative method approach was used with a survey and a sample of 225 people was obtained using a purposive sampling technique. Survey research is carried out by distributing questionnaires. Previously, the questionnaire was tested for validity and reliability first. The data analysis technique in this research uses descriptive analysis and linear regression analysis. Description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, most of whom are male, most employees are under 35 years old, and most employees have worked at the hotel for 0-2 years. The results of this research explain that Emotional Dissonance has a positive and significant effect on Service Sabotage with p-value of 0.012. Emotional Intelligence has a negative and significant effect on Service Sabotage with p-value of 0.023. Emotional Exhaustion has a positive and significant effect on Service Sabotage with p-value of 0.045.</t>
@@ -19270,6 +19311,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>Intergroup knowledge integration, that is the acquisition, processing, and utilization of knowledge across group boundaries, is a critical source of competitive advantage in modern organizations. Prior research has highlighted the important role of boundary spanning knowledge exchange for intergroup knowledge integration, neglecting, however, the question of what makes individual boundary spanners more effective in fostering intergroup knowledge integration. Integrating boundary spanning literature with theories of group information processing, we hypothesize that the effect of individual boundary spanning ties on intergroup knowledge integration depends on the boundary spanners’ levels of metaknowledge, i.e., knowledge of who knows what in their respective groups, and proactivity. We find general support for our predictions in a study of 457 engineering consultants nested in 22 interdependent business units within an organization. Additional criterion analyses confirm the material importance of intergroup knowledge integration for group performance. Our findings have implications for literatures on intergroup effectiveness, team cognition, and proactivity.</t>
@@ -19364,6 +19406,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their boundaries in ways that complement their preferences.</t>
@@ -19411,6 +19454,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>Background Increasing role complexity has intensiﬁed the boundary spanning functions of managers. Because work demands and scope vary by management position, time in staff contact rather than span may better explain managersÕ capacity to support staff. Methods A descriptive, correlational design was used to collect cross-sectional survey and prospective work log and administrative data from a convenience sample of 558 nurses in 51 clinical areas and 31 front-line nurse managers from four acute care hospitals in 2007–2008. Data were analysed using hierarchical linear modelling. Results Span, but not time in staff contact, interacted with leadership and operational hours to explain supervision satisfaction. Conclusions With compressed operational hours, supervision satisfaction was lower with highly transformational leadership in combination with wider spans. With extended operational hours, supervision satisfaction was higher with highly transformational leadership, and this effect was more pronounced under wider spans. Implications for Nursing Management Operational hours, which inﬂuence the managerÕs daily span (average number of direct report staff working per weekday), should be factored into the design of front-line management positions.</t>
@@ -19557,6 +19601,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>Background: Emotions play a central role in how employees respond to workplace bullying, influencing both their well-being and organizational outcomes. The purpose of the current study was to examine how workplace bullying and turnover intention are related to negative emotions and workplace unfairness. Methods: The research involved collecting data from 269 boundary-spanning bank workers (call center workers, frontline office staff, and customer service representatives) who experienced bullying. A moderated mediation was tested using Model 7 of the Process macro. The relationship between workplace bullying and turnover intention was analyzed, emphasizing the moderating effect of workplace unfairness and the mediating role of negative emotions. Results: The results validated the model, showing that an increase in negative emotions and workplace unfairness promotes the link between workplace bullying and the intention to leave. Increased negative emotions and perceived workplace unfairness amplified the relationship between workplace bullying and turnover intention. Conclusions: The findings underscored the cumulative risk of bullying environments for employee well-being and retention, providing practical recommendations for HRM and leadership strategies to cultivate healthier, more inclusive workplace settings. This study adds to the bullying–turnover literature by examining the joint role of negative emotions and workplace unfairness in a moderated mediation framework. The study connects these findings to sustainable labor management, emphasizing both theoretical and practical implications for organizations.</t>
@@ -19651,6 +19696,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>Abstract             In organizational contexts, professional boundaries serve a dual purpose by distinguishing various professions from one another and regulating access to power, status, and rewards. Individuals operating within professions in which such boundaries are not clearly or explicitly defined face the risk of compromising their status and autonomy. However, they possess the agency to actively define their profession and enhance its standing among both internal and external stakeholders. This study explores how homeroom teachers in the Israeli education system—recognized as a distinct occupation within the broader teaching profession—engage in boundary work to form and define their professional group. Our findings reveal that (1) homeroom teachers employ adaptable boundary work strategies, tailored to their interactions with different key stakeholders. Specifically, they (a) define boundaries to clarify, for themselves, the parameters of their own roles; (b) balance boundaries with partners inside the school (administrators and subject teachers) to facilitate day-to-day collaboration while simultaneously asserting their own roles; and (c) orchestrate boundaries when interacting with external partners (students’ parents), acknowledging the distinction between roles while primarily seeking to foster effective joint work towards the common goal of helping students succeed. (2) Despite the diversity in their approaches, all homeroom teachers exhibit a unique expertise, allowing them to combine boundary-setting with inclusivity, highlighting the dynamic and interactive nature of the boundary work process. This dual nature enhances the effectiveness of communication and collaboration within the educational system, molding the role of homeroom teachers as a distinct professional group.</t>
@@ -19896,6 +19942,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>Urban metabolism approaches are increasingly becoming relevant in providing pathways to sustainable development. The ways through which urban green infrastructures are planned and designed can influence resource flows in cities. Yet, little is known about the agency and contributions of landscape architects and spatial planners as curators of urban greenery, in facilitating circular resource flows, and accelerating the transition to a circular economy. This paper offers an empirical inquiry into the understanding and use of metabolic approaches in spatial planning and design practices. Through a multi-method approach and the use of boundary spanning as an analytical lens, we identify different modes of agency of spatial practitioners in enhancing resource efficiency across the life stages of urban landscape projects. Results show that while the ‘urban metabolism’ concept is not widely used by practitioners, its relevance to planning and designing green infrastructure for sustainable resource flows is well understood. Additionally, we highlight existing barriers including policy constraints in engaging with metabolic approaches and offer recommendations to facilitate a resource-sensitive turn in planning and designing urban landscapes. This study highlights important contributions of design practice to an expanding discourse of urban metabolism, including policy reforms for enabling circular resource flows in cities.</t>
@@ -19943,6 +19990,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -24535,7 +24583,7 @@
       </c>
       <c r="P546" t="inlineStr">
         <is>
-          <t>Excluded due to multiple reasons: [Code 1 &amp; Code 3]. The study uses individuals as proxy informants for firm-level supply chain initiatives, and the individual-level measure is a personality trait/orientation rather than actual boundary-spanning behavior.. Verbatim Evidence: [Theoretical Development] Tangpong, Hung, and Ro (2010) conceptualize this particular disposition in the buyer-supplier setting as “cooperativeness”; an example is the personality trait that entails acting toward others in tolerant, empathetic, supportive, and compassionate ways for mutual benefit. [Appendix] I am willing to share risks and benefits with my partners. [Research Methods] We selected 2,000 SMEs identified from the Korean Chamber of Commerce and Industry Directory, and to ensure that our respondents were in boundary-spanning roles in their companies, included a covering letter asking that the questionnaire be completed by BSIs such as sales managers. [Appendix] My company shares operational information with our partners. [Appendix] My company does strategic supply-chain planning jointly with our partners.</t>
+          <t>Excluded due to multiple reasons: [Code 1 &amp; Code 3]. The study uses individuals as proxy informants for firm-level supply chain initiatives, and the individual-level measure is a personality trait/orientation rather than actual boundary-spanning behavior.. Verbatim Evidence: [Theoretical Development] Tangpong, Hung, and Ro (2010) conceptualize this particular disposition in the buyer-supplier setting as âcooperativenessâ; an example is the personality trait that entails acting toward others in tolerant, empathetic, supportive, and compassionate ways for mutual benefit. [Appendix] I am willing to share risks and benefits with my partners. [Research Methods] We selected 2,000 SMEs identified from the Korean Chamber of Commerce and Industry Directory, and to ensure that our respondents were in boundary-spanning roles in their companies, included a covering letter asking that the questionnaire be completed by BSIs such as sales managers. [Appendix] My company shares operational information with our partners. [Appendix] My company does strategic supply-chain planning jointly with our partners.</t>
         </is>
       </c>
     </row>
@@ -24988,7 +25036,7 @@
       </c>
       <c r="P555" t="inlineStr">
         <is>
-          <t>Qualitative study analyzing interorganizational projects [Code 1 &amp; Code 3]. Verbatim Evidence: [Qualitative study analyzing interorganizational projects lacking effect sizes] [Code 1 &amp; Code 3]. Verbatim Evidence: "[Abstract] The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." "[3. Research setting and methods] We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." "[3. Research setting and methods] Our data analysis followed an “abductive” approach (Alvesson and Sköldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
+          <t>Qualitative study analyzing interorganizational projects [Code 1 &amp; Code 3]. Verbatim Evidence: [Qualitative study analyzing interorganizational projects lacking effect sizes] [Code 1 &amp; Code 3]. Verbatim Evidence: "[Abstract] The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." "[3. Research setting and methods] We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." "[3. Research setting and methods] Our data analysis followed an âabductiveâ approach (Alvesson and SkÃ¶ldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
         </is>
       </c>
     </row>
@@ -27344,6 +27392,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate the individual effects of boundary-spanning search from suppliers (supplier-side search (SS)). It is proposed that SS contributes to innovation ambidexterity (IA) and then business performance (BP). Further, this paper includes buyer–supplier relationships (BSRs) and competitive intensity (CI) as moderators to clarify boundary conditions.</t>
@@ -27391,6 +27440,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -27438,6 +27488,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr">
         <is>
           <t>This study utilizes network exploitation and exploration theory to distinguish the exploitative and exploratory mechanisms (government support and boundary-spanning learning, respectively) that convert political ties into firm innovativeness. It also examines the moderating roles market uncertainty plays in how political ties influence firm innovativeness. An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness. Market uncertainty negatively moderates the impact of political ties on boundary-spanning learning but does not significantly moderate their impact on government support. Moreover, market uncertainty moderates the impact of government support on firm innovativeness negatively but moderates the impacts of boundary-spanning learning on firm innovativeness positively. This study theorizes two mediating factors for how firms exploit and explore their political ties to increase their innovativeness and enriches the knowledge of how market uncertainty affects the relationship between political ties and innovation.</t>
@@ -27626,6 +27677,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -28894,6 +28946,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry. Using a multiyear sample of ﬁrms from the computer industry, we found that intra-industry trade-association ties of top managers led to the adoption of a resource-imitation strategy by late movers while extra-industry importation and professional-association ties led to the adoption of a resource-substitution strategy. We also found that trade association ties had a negative effect on the performance of late movers using resource-substitution, while top managers’ service on other ﬁrms’ boards had a positive inﬂuence on the performance of those ﬁrms. Our ﬁndings not only conﬁrm the importance of the role of ﬁt in strategy and performance, but they also highlight the importance of the management and control of boundary-spanning activities.</t>
@@ -29139,6 +29192,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>This study examines how deans and associate deans of a group from similar universities use networking. Specifically, we consider whether the deans, traditionally considered to perform boundary-spanning functions, make more use of external networking than do the associate deans, who are their subordinates. We examine the relationship between accuracy in perceiving a network and influence in the network. Finally, we consider the relationship between reports of networking outside the sample and influence within the sample. We find support for our first two propositions and raise several issues related to our final one.</t>
@@ -29280,6 +29334,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -29327,6 +29382,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>Local government or better known as the local authority vested with the power to plan, develop, and regulate businesses in the area within its jurisdiction plays a significant role in creating a conducive environment for businesses to grow and flourish. In playing this role, employees in local authority must possess a certain degree of innovative work behavior. This paper reports on a study that investigated innovative work behavior orientation among employees of the local government. A total of 100 employees of a local city council responded to a self-administered questionnaire on innovative work behavior. The results revealed that respondents scored a moderate high orientation on the innovative work behavior scale.</t>
@@ -29700,6 +29756,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -30589,6 +30646,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>Based on organizational learning theory, the influence of the transactive memory system of the top management team on business model innovation is discussed, as is the impact of different dimensions of boundary-spanning search on different business model innovation attributes when attention distribution is taken into account. Meanwhile, the moderating effects of environmental dynamism are considered. Regression and bootstrap analysis are used to test hypotheses. The results based on empirical research show that the transactive memory system has a positive effect on the dual attributes of business model innovation; acute boundary-spanning search and concentrated boundary-spanning search affect novelty-centered business model innovation and efficiencycentered business model innovation, respectively, and play mediating roles. Meanwhile, environmental dynamism positively moderates the relationship between acute boundary-spanning search and novelty-centered business model innovation, but negatively moderates the relationship between concentrated boundaryspanning and business efficiency-centered model innovation efficiency.</t>
@@ -30735,6 +30793,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
         <is>
           <t>This study adopts a temporal perspective to investigate how boundary spanners can increase the inflow of external knowledge by engaging with both external and internal parties. We add to prior work on knowledge transfer by shifting the focus from engagement levels to investigating engagement dynamics, especially the degree of switching between external and internal engagement across consecutive time periods. Drawing from a cognitive perspective, we argue that switching strongly between engagement types is associated with a segmented knowledge structure that enables quick and efficient categorical processing when knowledge can simply be “channeled” from source to recipient units. In contrast, weak or no switching is associated with a blended knowledge structure and more reflective processing, which is particularly helpful when knowledge transfer requires more translation and transformation. Correspondingly, we adopt a contingency perspective and theorize that the cognitive advantages associated with stronger versus weaker switching weigh differently, contingent on the stickiness of knowledge to be transferred and the nature of boundary-spanning activities that vary in importance over time. Fixed effects models of eight waves of original survey data reveal that, in line with our theorizing, the association between switching and knowledge transfer becomes increasingly negative (1) the more boundary spanners access knowledge that is transspecialist in nature, (2) the greater the organizational distance between source and recipient units, and (3) in later phases of the boundary-spanning process.</t>
@@ -30819,6 +30878,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 13
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -2926,7 +2926,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Qualitative/descriptive case study of an open-source software community without a correlation matrix or extractable effect sizes.. Verbatim Evidence: [Abstract] "Focusing on the Python community, our study examines a “pushed-by-users” design proposal through the discussions occurring in two mailing-lists: one, user-oriented and the other, developer-oriented." [Method] "The PEP 327 corpus is composed of 52 discussions in python-list and python-dev from the 17 October 2003 to the 23 May 2006, enriched by these five weblog articles and an interview with the user-champion of this PEP." [Results] "Table 4 sums up the distribution of references in the two lists according to the status of the participants and their cross participation role."</t>
+          <t>Qualitative/descriptive case study of an open-source software community without a correlation matrix or extractable effect sizes.. Verbatim Evidence: [Abstract] "Focusing on the Python community, our study examines a âpushed-by-usersâ design proposal through the discussions occurring in two mailing-lists: one, user-oriented and the other, developer-oriented." [Method] "The PEP 327 corpus is composed of 52 discussions in python-list and python-dev from the 17 October 2003 to the 23 May 2006, enriched by these five weblog articles and an interview with the user-champion of this PEP." [Results] "Table 4 sums up the distribution of references in the two lists according to the status of the participants and their cross participation role."</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Non-individual level (QAP network correlations at the organizational dyad level). Verbatim Evidence: [Method and Data] "The empirical study included three steps: (a) mapping and analyzing the organizational collaboration network, (b) mapping and analyzing the personal networks, and (c) analyzing the correlations between organizational collaborations and personal networks." [Network of Organizational Collaboration] "The network of organizational collaboration between science, education, and business that we examine here includes 25 nodes across the three sectors" [Networks of Personal Ties] "We aggregated the survey data by mapping each unique combination of an organizational entity and a contact’s name as a separate node." [Networks of Personal Ties] "Next, we produced three networks connecting the 25 organizations included in the analysis and representing different aspects of personal ties" [Correlations Between Networks of Personal Ties and Organizational Collaborations] "To check for correlations between organizational and personal networks in the Algarve maritime cluster, we applied the QAP correlation (Hubert &amp; Schultz, 1976) to the pairs of networks."</t>
+          <t>Non-individual level (QAP network correlations at the organizational dyad level). Verbatim Evidence: [Method and Data] "The empirical study included three steps: (a) mapping and analyzing the organizational collaboration network, (b) mapping and analyzing the personal networks, and (c) analyzing the correlations between organizational collaborations and personal networks." [Network of Organizational Collaboration] "The network of organizational collaboration between science, education, and business that we examine here includes 25 nodes across the three sectors" [Networks of Personal Ties] "We aggregated the survey data by mapping each unique combination of an organizational entity and a contactâs name as a separate node." [Networks of Personal Ties] "Next, we produced three networks connecting the 25 organizations included in the analysis and representing different aspects of personal ties" [Correlations Between Networks of Personal Ties and Organizational Collaborations] "To check for correlations between organizational and personal networks in the Algarve maritime cluster, we applied the QAP correlation (Hubert &amp; Schultz, 1976) to the pairs of networks."</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Macro-economic study analyzing aggregate employment data at the regional level (203 administrative areas) rather than individual employees.. Verbatim Evidence: [Abstract] "This paper examines the impact of externalities on employment growth in sub-regions of Great Britain by estimating ordinary least-squares (OLS) and maximum likelihood spatial models at the two-digit level for 23 sectors." [Methodology] "data for sub-regions of Great Britain at the two-digit industry level were obtained from the UK’s National On-line Manpower Information System (NOMIS) utilizing the 1992 Standard Industrial Classi-ﬁcation (SIC) classiﬁcation scheme and covering the period 1995–2002." [Methodology] "Data were collected for 203 areas at the local authority, county, and unitary authority levels. These areas are administrative units and vary from large, densely populated urban regions to smaller, rural sub-regions."</t>
+          <t>Macro-economic study analyzing aggregate employment data at the regional level (203 administrative areas) rather than individual employees.. Verbatim Evidence: [Abstract] "This paper examines the impact of externalities on employment growth in sub-regions of Great Britain by estimating ordinary least-squares (OLS) and maximum likelihood spatial models at the two-digit level for 23 sectors." [Methodology] "data for sub-regions of Great Britain at the two-digit industry level were obtained from the UKâs National On-line Manpower Information System (NOMIS) utilizing the 1992 Standard Industrial Classi-ï¬cation (SIC) classiï¬cation scheme and covering the period 1995â2002." [Methodology] "Data were collected for 203 areas at the local authority, county, and unitary authority levels. These areas are administrative units and vary from large, densely populated urban regions to smaller, rural sub-regions."</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Non-primary study (Editorial for a Special Section). Verbatim Evidence: [Page 1] "EDITORIAL Innovating for impact: Harnessing business model innovation to tackle grand challenges" [Abstract] "Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed “ABC” classification and “BMI-GC” concept." [Introduction] "Our objective with this Special Section is to link our improved conceptual and empirical understanding of business models with the important notion of grand challenges, the urgency of which has become increasingly apparent."</t>
+          <t>Non-primary study (Editorial for a Special Section). Verbatim Evidence: [Page 1] "EDITORIAL Innovating for impact: Harnessing business model innovation to tackle grand challenges" [Abstract] "Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed âABCâ classification and âBMI-GCâ concept." [Introduction] "Our objective with this Special Section is to link our improved conceptual and empirical understanding of business models with the important notion of grand challenges, the urgency of which has become increasingly apparent."</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Multiple reasons [Code 1 &amp; Code 2]: Sample consists of independent entrepreneurs rather than organizational employees, and no zero-order correlation matrix is provided.. Verbatim Evidence: [Methods] "Data were collected among Dutch entrepreneurs owning private companies with fewer than 250 employees (cf. Jayasekara et al., 2020). They were recruited via network organizations (e.g. FNV Zelfstandigen), magazines, LinkedIn Groups, and a database (i.e. Prolific)." [Methods] "We examined cross-sectional data from 2021–2023, with 286 entrepreneurs completing the general survey."</t>
+          <t>Multiple reasons [Code 1 &amp; Code 2]: Sample consists of independent entrepreneurs rather than organizational employees, and no zero-order correlation matrix is provided.. Verbatim Evidence: [Methods] "Data were collected among Dutch entrepreneurs owning private companies with fewer than 250 employees (cf. Jayasekara et al., 2020). They were recruited via network organizations (e.g. FNV Zelfstandigen), magazines, LinkedIn Groups, and a database (i.e. Prolific)." [Methods] "We examined cross-sectional data from 2021â2023, with 286 entrepreneurs completing the general survey."</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>The study focuses on work-nonwork (work-family) boundary management rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: [Abstract] The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. [Introduction] Research devoted to the interplay of work and nonwork (e.g., family and leisure) life continues to flourish, as “balancing” both roles becomes a vital concern to an increasing proportion of employees that engages in multiple roles (Kelly et al., 2008; Allen and Martin, 2017).</t>
+          <t>The study focuses on work-nonwork (work-family) boundary management rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: [Abstract] The present study addresses this gap by developing the construct and measure of work-nonwork boundary management fit, based on the needs-supplies fit framework. [Introduction] Research devoted to the interplay of work and nonwork (e.g., family and leisure) life continues to flourish, as âbalancingâ both roles becomes a vital concern to an increasing proportion of employees that engages in multiple roles (Kelly et al., 2008; Allen and Martin, 2017).</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 4] Practitioner article based on a book; lacks quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [ABOUT THE RESEARCH] "This article is based on the authors’ book, Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations (McGraw-Hill, 2010)." [REFERENCES] "2. This article is primarily based on C. Ernst and D. Chrobot-Mason, “Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations” (New York: McGraw-Hill, 2010)."</t>
+          <t>[Code 1 &amp; Code 4] Practitioner article based on a book; lacks quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [ABOUT THE RESEARCH] "This article is based on the authorsâ book, Boundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizations (McGraw-Hill, 2010)." [REFERENCES] "2. This article is primarily based on C. Ernst and D. Chrobot-Mason, âBoundary Spanning Leadership: Six Practices for Solving Problems, Driving Innovation, and Transforming Organizationsâ (New York: McGraw-Hill, 2010)."</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Measures mere communication frequency rather than purposive boundary spanning behavior.. Verbatim Evidence: [Measures] "Extraunit communication frequency is the frequency of oral, work-related communication with categories of individuals outside the subject’s subunit." [Appendix V: Survey Materials] "How often have you discussed technical issues encountered in your current work over the past month, either face to face or by phone, with each person on the list?" [Appendix V: Survey Materials] "Over the past month how often have you discussed work-related issues with the following in personnel in your company?"</t>
+          <t>Measures mere communication frequency rather than purposive boundary spanning behavior.. Verbatim Evidence: [Measures] "Extraunit communication frequency is the frequency of oral, work-related communication with categories of individuals outside the subjectâs subunit." [Appendix V: Survey Materials] "How often have you discussed technical issues encountered in your current work over the past month, either face to face or by phone, with each person on the list?" [Appendix V: Survey Materials] "Over the past month how often have you discussed work-related issues with the following in personnel in your company?"</t>
         </is>
       </c>
     </row>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Firm-level analysis with manager acting as a proxy informant for the organization. Verbatim Evidence: [Methodology] To select the appropriate samples, we adopted four criteria. Firstly, the firms should be in good operating condition and have innovation output over a period of time. Secondly, considering the innovation cycle, the firms should be established for at least one year. ... And the respondents were firm managers. [Measures] boundary-spanning search was measured by five items: “In our firm, we search for knowledge disclosed from patent gazette”, “In our firm, we search for knowledge from technology licensing”, “In our firm, we search for knowledge from research institutions, universities or colleges”, “In our firm, we search for knowledge from industry exhibitions”, “In our firm, we search for knowledge from technical publications and technical conferences”.</t>
+          <t>Firm-level analysis with manager acting as a proxy informant for the organization. Verbatim Evidence: [Methodology] To select the appropriate samples, we adopted four criteria. Firstly, the firms should be in good operating condition and have innovation output over a period of time. Secondly, considering the innovation cycle, the firms should be established for at least one year. ... And the respondents were firm managers. [Measures] boundary-spanning search was measured by five items: âIn our firm, we search for knowledge disclosed from patent gazetteâ, âIn our firm, we search for knowledge from technology licensingâ, âIn our firm, we search for knowledge from research institutions, universities or collegesâ, âIn our firm, we search for knowledge from industry exhibitionsâ, âIn our firm, we search for knowledge from technical publications and technical conferencesâ.</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5689,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
           <t>While there is a burgeoning trend to recognize leadership as an important enabler of new venture development and growth, scant research has explored the performance mechanisms of shared leadership in the entrepreneurial context. Based on the information processing perspective, we propose a moderated mediation model to examine how shared leadership in entrepreneurial teams advance new venture performance by identifying team reflexivity as a pivotal mediator and team boundary spanning as a crucial contingency. The data set from a cross-industry sample of 94 entrepreneurial teams indicated that shared leadership exerts a positive indirect influence on new venture performance via team reflexivity; and team boundary spanning moderates such indirect influence. Finally, how our findings contribute to the entrepreneurship, leadership, team research, and managerial practice are discussed.</t>
@@ -5717,7 +5721,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 2 &amp; Code 3] Sample consists of entrepreneurs/founders rather than embedded employees. Furthermore, boundary spanning is measured at the team level ('We' referent) rather than the individual level.. Verbatim Evidence: [Method - Sample] "we randomly identified 200 new ventures from three high-tech industrial parks in eastern China. ... Accordingly, we gathered a list of 163 entrepreneurial teams. ... a total of 417 questionnaires from 102 teams were received, among which 376 questionnaires from 94 teams are valid." [Method - Measurement] "Team boundary spanning was rated by a nine-item scale selected from Yan et al. (2020). These items reflect the degree to which the teams search diverse sources of external information. These items include three dimensions: ambassador activities (e.g., 'We acquire resources for the team'); task coordinator activities (e.g., 'We coordinate activities with external groups'); and scout activities (e.g., 'We scan the environment for marketing ideas/expertise')."</t>
         </is>
       </c>
     </row>
@@ -5737,6 +5741,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Getting professionals who have been selected and trained to perform individually to work together is a major challenge. The objective of the article is to identify the mechanisms by which a coordinator can ensure a mediation and boundary spanning role to enable the achievement of a project. Adopting a comprehensive approach, this article is based on the case of an innovative hospital project ‘One-Day Diagnosis’ (1DD) – one day instead of several weeks – of hepatobiliary and pancreatic pathologies, for which the professionals had to change their practices. Based on the results of the study, the ﬁndings show that the mediating role of the coordinator consists in making things happen and guiding health care professionals through the innovative pathway until it becomes a routine process. The study contributes to the literature on collaboration and relational coordination by highlighting that the change of practices for collaboration is compatible with personal excellence, by outlining the active role of the boundary spanner in the change of these practices and by demonstrating that the organizational stability of projects based on disembodied procedures is a necessary illusion that requires complementary interindividual relationships and a living leadership.</t>
@@ -5784,6 +5789,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>The current study examined the relationships among role stress, proactive personality, employee creativity, and customer-oriented boundary spanning behaviors (COBSBs) for frontline service employees (FSEs). This study collected data from 382 FSEs in international hotels in Taiwan to test the research model. The empirical results revealed that employee creativity was positively affected by proactive personality but negatively affected by role conflict and role ambiguity. FSEs’ creativity positively affects COBSBs, including external representation, internal influence, and service delivery. Internal influence also positively affects service delivery and mediates the relationship between FSEs’ creativity and service delivery.</t>
@@ -5831,7 +5837,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>A number of studies have found that the performance of NPD projects greatly depends on the support they get from top management. However, research into why some projects get more support than others has been limited. The present paper takes a political approach to NPD, in which top management support is considered to be a function of a project leader’s ability to influence decision processes through personal relationships. Mobilizing the bridging perspective of social capital, we argue that project leaders need both strong ties to high-ranking others and sparseness in their networks. Vertical strong ties bring direct support and solidarity, resulting in improved access to resources and priority over other projects; sparseness provides exposure to the full range of information and interpretations in the organization, resulting in a more accurate picture of the political landscape and thus enabling the implementation of an appropriate influence strategy. A PLS analysis of a sample of 73 French project leaders involved in NPD projects provided support for our hypotheses. Hence, we contribute to a very recent stream of research showing that the structural and relational dimensions of social capital are complementary.</t>
@@ -5931,6 +5936,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>This dissertation examined the relationships between organizational characteristics and firms' timing of entry into emerging product markets. This study is an extension of a stream of research on endogenous entry models. Research on this area essentially holds that not all firms have the same entry skills and costs. Therefore, a firm's entry timing decision is attributable to factors internal to the organization. In this dissertation, specific attention is directed toward the effects of top management team (TMT) demography, corporate governance, level of diversification, boundary spanning, past performance, capital structure, and firm size on entry timing. These organizational characteristics have been shown to be critical determinants of timing in the strategic management literature, but, remain almost unexplored in the entry timing research. Thus, through including these organizational characteristics, this study extends the current knowledge which is critical for answering the question: Why do some firms enter emerging product markets earlier/later than others?</t>
@@ -5978,6 +5984,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>Organisations experience increased social, political and economic pressure that is evident in the increased pressure that stakeholders place on organisations. Organisations increasingly realise that stakeholders’ values and objectives need to be incorporated into organisational strategy as well as the day-to-day management of the organisation. Organisational success and survival consequently depends on the organisation’s network of relationships, which provide the organisation with otherwise inaccessible resources and a competitive advantage.</t>
@@ -6025,6 +6032,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>In this dissertation, I develop a conceptual model for how managers' roles as boundary spanners within their organizations affect the perceptions, attitudes, relationships, and performance of their subordinate employees. Drawing on literatures in social networks, status characteristics theory, social identity theory, and resource allocation theory, I suggest that managers' external relationships—the connections that managers make to organization members outside of their subordinate work group—have a material impact on their subordinates' perceptions of their work environment and their managers. These perceptions, I argue, serve as four specific mechanisms in an indirect effects model that connect managers' external relationship to their employees' task performance and work attitudes (eg organizational commitment) and the Leader Member Exchange (LMX) relationships between manager and subordinate. I apply the theoretical model to two salient types of managerial relationships: those with their bosses and those with their horizontal peers.</t>
@@ -6072,6 +6080,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -6119,6 +6128,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>The state of software development performance is far from being exemplar, with a success rate well below that of other industries, and understanding how to improve these projects is not only substantive but urgent. Software development is at most times a collaborative effort, yet we do not understand clearly how different collaboration structures associate with development performance metrics. This paper empirically examines the association between collaboration patterns, project productivity and product quality through a field study of working software open source new product development teams, using archival data from electronic sources related to Open Source Software projects. Collaboration structures are measured using Social Network Analysis and in terms of their network density, network centralization and the level of boundary spanning activity of team members. Productivity and quality are measured using "hard", code-based metrics. Results of regression analyses testing relevant hypotheses suggest that project managers need to strongly encourage internal collaboration, but be wary of allowing team members to participate in multiple projects. The breadth of skills within the team is a tactical asset that may increase the efficient frontier in the quality–productivity trade-off. Results also show that centralized structures associate with higher product quality and development productivity.</t>
@@ -6166,6 +6176,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Technology Transfer Centres (TTCs) have been analyzed in the last few years by focusing on the relationship between a TTC, provider of knowledge-intensive services, and a ﬁrm client-receiver. Less attention has been devoted to a more complex relationship which involves in the dyadic provider-receiver tie a third relevant body, University. We provide both a theoretical and an empirical contribution by studying whether TTCs can bond the academic and industrial system and we deﬁne the activities that make-up this role such as: scanning and selection of R&amp;D opportunities, bridge building, semantic translation of domain speciﬁc knowledge, co-production of new knowledge. The boundary spanning role of TTCs is discussed drawing on different and complementary theoretical perspectives. Moreover, we test research hypotheses on the antecedents of boundary spanning activity from a knowledge-based perspective. We argue that TTC boundary spanners need to leverage on both technical skills and networking competences. Empirical investigation has been carried out with a survey of the TTC population of North East Italy. The research ﬁndings highlight the task coordination activities implied by a boundary spanning role in joint R&amp;D projects and show that the endowment of human capital at individual level and a qualiﬁed social capital at individual and organizational level are the main determinants.</t>
@@ -6213,7 +6224,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>This paper contributes to open innovation (OI) and boundary spanning literatures by providing a first understanding of industry‐based boundary spanners in university‐industry (U‐I) collaboration through case studies of Chinese multinational corporations (MNCs) and their international OI platforms. Organisational roles created by these platforms within the MNCs and their activity of bridging between organisations are examined. The analysis of 25 in‐depth interviews in two MNCs located in eight countries, along with internal documents, sheds light on U‐I collaboration practices implemented by Chinese MNCs. Two new boundary spanning roles are identified:               Dual Cultural Bridger               – as these OI platforms bridge organisational and national cultural gaps to prevent and solve problems in the collaborative process; and               International Network Enhancer               – as these OI platforms act as trust building and local knowledge listening posts for the MNC’s global network. Managerial and policy implications are provided.</t>
@@ -6293,7 +6303,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>Non-individual level (team/firm/org analysis). Verbatim Evidence: [Abstract] "The statistical analyses in this dissertation are based on survey data on nearly one thousand manufacturing plants in twenty-one industries where metal machining is a normal part of production processes." [Chapter 3] "The quantitative data I analyze in this research are from a survey conducted in 1991 by Kelley and Watkins on 973 plants that perform a significant amount of metal machining in their production process, what they term the Machined Durable Goods Sector (Kelley, 1991)." [Chapter 3] "The measures of close ties I examine are with the focal plants’ single “most important” machining subcontractor, as selected by the plant manager, and their largest customer. Informants for the focal plants report as to whether they engaged in any of three boundary-spanning activities with their most important machining supplier and their largest customer."</t>
+          <t>Non-individual level (team/firm/org analysis). Verbatim Evidence: [Abstract] "The statistical analyses in this dissertation are based on survey data on nearly one thousand manufacturing plants in twenty-one industries where metal machining is a normal part of production processes." [Chapter 3] "The quantitative data I analyze in this research are from a survey conducted in 1991 by Kelley and Watkins on 973 plants that perform a significant amount of metal machining in their production process, what they term the Machined Durable Goods Sector (Kelley, 1991)." [Chapter 3] "The measures of close ties I examine are with the focal plantsâ single âmost importantâ machining subcontractor, as selected by the plant manager, and their largest customer. Informants for the focal plants report as to whether they engaged in any of three boundary-spanning activities with their most important machining supplier and their largest customer."</t>
         </is>
       </c>
     </row>
@@ -6313,6 +6323,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>This cross-sectional study (conducted in April–May 2011) explored associations between partnership functioning synergy and sustainability of innovative programmes in community care. The study sample consisted of 106 professionals (of 244 individuals contacted) participating in 21 partnerships that implemented different innovative community care programmes in Rotterdam, The Netherlands. Partnership functioning was evaluated by assessing leadership, resources administration and efﬁciency. Synergy was considered the proximal outcome of partnership functioning, which, in turn, inﬂuenced the achievement of programme sustainability. On a 5-point scale of increasing sustainability, mean sustainability scores ranged from 1.9 to 4.9. The results of the regression analysis demonstrated that sustainability was positively inﬂuenced by leadership (standardised regression coefﬁcient b = 0.32; P &lt; 0.001) and non-ﬁnancial resources (b = 0.25; P = 0.008). No signiﬁcant relationship was found between administration or efﬁciency and programme sustainability. Partnership synergy acted as a mediator for partnership functioning and signiﬁcantly affected sustainability (b = 0.39; P &lt; 0.001). These ﬁndings suggest that the sustainability of innovative programmes in community care is achieved more readily when synergy is created between partners. Synergy was more likely to emerge with boundaryspanning leaders, who understood and appreciated partners’ different perspectives, and could bridge their diverse cultures and were comfortable sharing ideas, resources and power. In addition, the acknowledgement of and ability to use members’ resources were found to be valuable in engaging partners’ involvement and achieving synergy in community care partnerships.</t>
@@ -6407,7 +6418,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>In this paper, we highlight the networked context of the professions. In particular, we indicate that neo-classical professionals tend to work across organizational boundaries in project teams, often to meet the needs of clients and the wider society. However, little is known about the resources that professionals draw on to meet immediate, fast paced, client demands in project network organizations (PNOs). We pinpoint how knowledge resources, human, social and organizational capital enable professionals to produce outputs at a fast pace/tempo. Temporality emerged as an unexpected but key issue in our empirical research and we explore this further here. First, we put forward how professional work organization(s) has changed by focusing on the boundaries of organizations, and how this is often temporary and project-driven. Second, we use the speciﬁc lens of knowledge resources which are drawn upon to enable networked working and ask the question: which knowledge resources enable professionals to work at a fast pace within networks? Third, appreciative of the vast literature on temporary and networked organizations in professional work, our focus is beyond a single profession or organization, and hence, we build upon the prior research on PNOs. We do this by drawing on empirical data of a humanitarian aid project networked organization (HN) that upscales across its network at high speed, often within days, to generate funds for humanitarian disasters in order to save lives.</t>
@@ -6455,7 +6465,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>This research examines the mechanisms through which entrepreneurial orientation (EO) aﬀects ﬁrm performance in an emerging market context. We argue that EO drives ﬁrms to develop the dynamic capabilities of absorptive capacity (ACAP) and boundary-spanning (BS), and that these capabilities enhance ﬁrm performance. Moreover, the eﬀectiveness of these knowledge- and network-based dynamic capabilities in mediating the EOperformance relationship is contingent on the institutional conditions ﬁrms are exposed to. We test our hypotheses using multi-sourced data on Chinese high-tech ﬁrms in business-to-business (B2B) markets. Our results show that ACAP and BS mediate the positive eﬀect of EO on ﬁrm performance, and that as the development of market-supporting institutions improves, the mediating eﬀect of ACAP becomes stronger while that of BS weakens.</t>
@@ -6503,7 +6512,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Effective work groups engage in external knowledge sharing—the exchange of information, know-how, and feedback with customers, organizational experts, and others outside of the group. This paper argues that the value of external knowledge sharing increases when work groups are more structurally diverse. A structurally diverse work group is one in which the members, by virtue of their different organizational affiliations, roles, or positions, can expose the group to unique sources of knowledge. It is hypothesized that if members of structurally diverse work groups engage in external knowledge sharing, their performance will improve because of this active exchange of knowledge through unique external sources. A field study of 182 work groups in a Fortune 500 telecommunications firm operationalizes structural diversity as member differences in geographic locations, functional assignments, reporting managers, and business units, as indicated by corporate database records. External knowledge sharing was measured with group member surveys and performance was assessed using senior executive ratings. Ordered logit analyses showed that external knowledge sharing was more strongly associated with performance when work groups were more structurally diverse. Implications for theory and practice around the integration of work groups and social networks are addressed.</t>
@@ -6551,7 +6559,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>Our study responds to a call for research to integrate institutional, organizational and individual levels of analysis in examining the implications for work and employment relations of new organizational forms. We empirically examine the implementation of network forms of genetics healthcare delivery that cross organizational and professional boundaries. We highlight that less powerful professional groups may find difficulty in enacting boundary-spanning roles associated with new organizational forms. This is due, first, to inconsistency of government policy, which fragments organizations. Second, professional institutions sustain professional hierarchy and power differentials.</t>
@@ -6599,7 +6606,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to test the inﬂuence of external information search (EIS) on knowledge elaboration and group cognitive complexity (GCC) under the moderating effect of absorptive capacity (AC is indicated by prior knowledge base and gender diversity).</t>
@@ -6699,6 +6705,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>The perspectives of transaction cost economics and the resource-based view of the firm have been used extensively to understand the implications of outsourcing. However, transaction cost economics does not explain how a firm will evolve as it progressively outsources internal functions, and the resource-based view does not operationalize the unspecified competences that will be required over time. On the other hand, the lens of paradox highlights the increased expediency and complexity that outsourcing firms are expected to encounter. In this paper, paradoxes comparing operational expediency gains to increases in management, learning and strategic complexity are discussed, leading to the proposal that often unintended replacement behaviors manifest as extensive boundary spanning and new firm-level competencies are necessary to manage these paradoxes and maintain competitive advantage. In extremum tests of these propositions are provided to demonstrate that the complexity of outsourcing intangibles is informed by a lens of paradox.</t>
@@ -6746,7 +6753,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>The aim of this research is to empirically investigate the relationships among the three vital knowledge management processes of acquisition, integration and application, and their effects on organisational innovation in the pharmaceutical manufacturing industry in Jordan; a knowledge-intensive business service (KIBS) sector. Structural equation modelling findings show an excellent fit among all these processes and innovation, with positive and significant relationships. Moreover, knowledge integration and knowledge application emerged as having strong and significant mediation effects upon the relationship between knowledge acquisition and innovation. As such, an organisation’s innovation efforts would significantly benefit from the synergistic effects of properly integrating and applying externally acquired knowledge. The findings make a valuable contribution to pharmaceutical knowledge management and innovation literature, especially in an era of open innovation. Pharmaceutical companies are advised to focus on developing proficient assimilation and application capabilities in order for acquired knowledge to have notable effects on their innovation performance.</t>
@@ -6841,7 +6847,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6936,7 +6941,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>This study investigated coordinated action in multiteam systems employing 233 correspondent systems, comprising 3 highly specialized 6-person teams, that were engaged in an exercise that was simultaneously “laboratory-like” and “field-like.” It enriches multiteam system theory through the combination of theoretical perspectives from the team and the large organization literatures, underscores the differential impact of large size and modular organization by specialization, and demonstrates that conventional wisdom regarding effective coordination in traditional teams and large organizations does not always transfer to multiteam systems. We empirically show that coordination enacted across team boundaries at the component team level can be detrimental to performance and that coordinated actions enacted by component team boundary spanners and system leadership positively impact system performance only when these actions are centered around the component team most critical to addressing the demands of the task environment.</t>
@@ -6984,6 +6988,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore how and why employees perceive technology-mediated interruptions differently and the role of sociocultural factors in this process using sociomaterial analysis. Design/methodology/approach – Data were gathered from 34 Sri Lankan knowledge workers using a series of workshop-based activities. The concept of sociomateriality is employed to understand how sociocultural elements are entangled with technology in work-life boundary experiences.</t>
@@ -7031,7 +7036,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>In this article, the authors examine antecedents and consequences of the service climate in boundary-spanning self-managing teams (SMTs) that deliver financial services. Using data from members of 61 SMTs and their customers, the authors show a differential impact of the SMT service climate on various marketing performance measures. Furthermore, they obtain support for independent group-level effects of intrateam support and team member flexibility on employee perceptions of the SMT service climate. Both effects are persistent over time and demonstrate that collective perceptions in the SMT have incremental value in the explanation of the service climate.</t>
@@ -7220,6 +7224,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -7318,7 +7323,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -7366,6 +7370,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -7413,7 +7418,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>This article develops a framework for studying cross-functional teams in organizations that focuses on three domains: organizational context, internal process, and outcome measures. The framework was developed from qualitative data from over 200 individual and group interviews, written descriptions, and team observations. We then operationally defined this model through a set of questionnaire items and validated it through quantitative analysis of data from 565 members of cross-functional teams. The resulting framework provides a base for the future study of cross-functional teams.</t>
@@ -7461,7 +7465,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>When working as a member of a team, individuals must make decisions concerning the allocation of resources (eg, effort) toward individual goals and team goals. As a result, individual and team goals, and feedback related to progress toward these goals, should be potent levers for affecting resource allocation decisions. This research develops a multilevel, multiple-goal model of individual and team regulatory processes that affect the allocation of resources across individual and team goals resulting in individual and team performance. On the basis of this model, predictions concerning the impact of individual and team performance feedback are examined empirically to evaluate the model and to understand the influence of feedback on regulatory processes and resource allocation. Two hundred thirty-seven participants were randomly formed into 79 teams of 3 that performed a simulated radar task that required teamwork. Results support the model and the predicted role of feedback in affecting the allocation of resources when individuals strive to accomplish both individual and team goals.</t>
@@ -7556,6 +7559,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing. Informing teams remain relatively isolated from their environment; parading teams have high levels of passive observation of the environment; and probing teams actively engage outsiders. Probing teams revise their knowledge of the environment through external contact, initiate programs with outsiders, and promote their team's achievements within their organization. In this study, they were rated as the highest performers among the teams, although member satisfaction and cohesiveness suffered in the short run. Results suggested that external activities are better predictors of team performance than internal group processes for teams facing external dependence.</t>
@@ -8112,7 +8116,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 2] Laboratory experiment using a student sample (business school undergraduates) and reporting no zero-order correlation matrix.. Verbatim Evidence: [Manipulations] "The research was conducted using a full-factorial experimental design, resulting in 16 (4 × 2 × 2) treatments." [Manipulations] "Fifteen subjects (upper division business school undergraduates) were in each treatment."</t>
+          <t>[Code 1 &amp; Code 2] Laboratory experiment using a student sample (business school undergraduates) and reporting no zero-order correlation matrix.. Verbatim Evidence: [Manipulations] "The research was conducted using a full-factorial experimental design, resulting in 16 (4 Ã 2 Ã 2) treatments." [Manipulations] "Fifteen subjects (upper division business school undergraduates) were in each treatment."</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8948,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>Non-individual level of analysis (multiteam system).. Verbatim Evidence: [Sample and Task] "A total of 3,486 officers were randomly assigned to one of 249 14-person multiteam systems for the entire five-week course, such that each multiteam system was comparable with respect to members’ ability, gender, experience, age, and vocational specialty." [Measures] "We measured between-team coordination behaviorally as the number of missions sent to targets on the COP with a confidence rating indicated (i.e., missions sent to targets with ratings of “1” through “4”; missions with confidence ratings of “0” were excluded; see Appendix C)." [Table 1] "Notes: n = 249; observations are multiteam systems of 14 members each."</t>
+          <t>Non-individual level of analysis (multiteam system).. Verbatim Evidence: [Sample and Task] "A total of 3,486 officers were randomly assigned to one of 249 14-person multiteam systems for the entire five-week course, such that each multiteam system was comparable with respect to membersâ ability, gender, experience, age, and vocational specialty." [Measures] "We measured between-team coordination behaviorally as the number of missions sent to targets on the COP with a confidence rating indicated (i.e., missions sent to targets with ratings of â1â through â4â; missions with confidence ratings of â0â were excluded; see Appendix C)." [Table 1] "Notes: n = 249; observations are multiteam systems of 14 members each."</t>
         </is>
       </c>
     </row>
@@ -9380,7 +9384,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -9617,7 +9620,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>Firm-level analysis (N=1,088 firms) using top managers as proxy informants for the establishment's knowledge search.. Verbatim Evidence: [Firm-level analysis and proxy informants]. Verbatim Evidence: "[Abstract] Using a sample of 1,088 Chinese firms’ data collected by the World Bank in 2012, this paper employs logistic regression to test the hypotheses." "[Method] Following a two-stage procedure, a screening phase over the phone and a face-to-face interview with the top manager of each establishment, the data is collected between December 2011 and February 2013." "[Measurement] In the questionnaire, the item “in what ways has this establishment introduced new products or services and new or improved process?” is used for identifying knowledge search."</t>
+          <t>Firm-level analysis (N=1,088 firms) using top managers as proxy informants for the establishment's knowledge search.. Verbatim Evidence: [Firm-level analysis and proxy informants]. Verbatim Evidence: "[Abstract] Using a sample of 1,088 Chinese firmsâ data collected by the World Bank in 2012, this paper employs logistic regression to test the hypotheses." "[Method] Following a two-stage procedure, a screening phase over the phone and a face-to-face interview with the top manager of each establishment, the data is collected between December 2011 and February 2013." "[Measurement] In the questionnaire, the item âin what ways has this establishment introduced new products or services and new or improved process?â is used for identifying knowledge search."</t>
         </is>
       </c>
     </row>
@@ -9689,6 +9692,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>The digital era is radically changing our societies and how ﬁrms do business. Innovating the business model has become a fundamental capability to survive competition, particularly for small and mediumsized enterprises (SMEs). This study investigates the digital-era role of boundary management capabilities in the processes of Business Model Innovation (BMI) in SMEs. Structural Equation Modelling is adopted to analyse data from a survey of 250 Italian experts who possess direct research and consulting experience with SMEs. Our ﬁndings reveal that digitalisation and ﬁrms’ boundaries aﬀect BMI in SMEs. Moreover, our results demonstrate how boundary management, speciﬁcally its technological and relational aspects, directly impacts BMI and mediates the relationship between boundary size and BMI. The study also oﬀers important theoretical and practical insights, calling on scholars and managers to give more attention to the boundary management of SMEs in order to support BMI.</t>
@@ -9736,7 +9740,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>This study investigated how a project group deals with the contradiction between distributed knowledge in boundary-spanning collaborative processes and the expectation that software systems will provide unified, codified knowledge. It employed an ethnographic, interpretive approach to examine the ways in which relevant knowledge was presented, recognized, shared or otherwise managed during a project concerned with the joint design of business process and IT systems change. Developing a group understanding of how to manage sensemaking and expertise across salient knowledge boundaries were discovered to be central to perceptions of project completion. Four stages of this development were identified. The contribution of this paper is to propose these stages as the basis for boundary-spanning group management approaches and to suggest ways of progressing the complexities of communication, consensus-building, information exchange, problem-formulation and solution-brokering that are fundamental to collaboration in IS definition. These processes are normally taken for granted, rationalized or ignored by managers of IT-related organizational change. The use of specific types of boundary-object may aid in managing such processes explicitly and ensuring rapid progress. Thus the findings have significant implications for research and practice in other forms of boundary-spanning group collaboration, such as organizational innovation and problem-solving.</t>
@@ -9831,6 +9834,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>In this study we examine the impact of market orientation of leaders on their leader-member exchange (IMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the exist five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.</t>
@@ -9878,6 +9882,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>We examine the extent to which executives' boundary spanning relations inside and outside their industry affect organizational strategy and performance. We posit that the informational and social influences of external ties will be reflected in the degree to which the organization's strategy conforms to or deviates from the central tendencies of its industry and that the alignment of executives' external ties with the firm's strategy will be beneficial to firm performance. Using a multiyear sample of firms in the branded foods and computer industries, we find that executives' intraindustry ties are related to strategic conformity, that extraindustry ties are associated with the adoption of deviant strategies, and that alignment of executives' external ties with the informational requirements of the firm's strategy enhances organizational performance. Our results also show that a unique or differentiated strategy is not universally advantageous and that the benefits accruing from strategic conformity are especially strong in the more uncertain computer industry.</t>
@@ -9925,6 +9930,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>The relationship between external communication and R&amp;D team creativity has received increasing attention in the R&amp;D management literature. However, little is known about the motivational mechanism between the two. We propose a second‐stage moderation model based on social cognitive theory to explain whether, how and when R&amp;D team’s external developmental feedback motivates its creativity. Using the data gathered from 452 R&amp;D team members and 84 supervisors in a time‐lagged field study, we found external developmental feedback had a positive effect on R&amp;D team creativity via increasing team creative efficacy. Further, conditional indirect effect analyses found that a high level of cooperative goal interdependence strengthened the positive effect of team creative efficacy on R&amp;D team creativity and the mediating effect of team creative efficacy between external developmental feedback and R&amp;D team creativity.</t>
@@ -9972,6 +9978,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -10019,7 +10026,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -10067,6 +10073,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Even though, over the last two decades, the boundaryless career concept has stimulated a wide theoretical debate, scholars have recently claimed that research on the competencies that are necessary for managing a cross-boundary career is still incomplete. Similarly, the literature on emotional and social competencies has demonstrated how they predict work performance across industries and jobs but has neglected their inﬂuence in explaining the individual’s mobility across boundaries and their impact on career success. This study aims to ﬁll these gaps by examining the effects of emotional and social competencies on boundaryless career and on objective career success. By analyzing a sample of 142 managers over a period of 8 years, we found evidence that emotional competencies positively inﬂuence the propensity of an individual to undertake physical career mobility and that career advancements are related to the possession of social competencies and depend on the adoption of boundaryless career paths. This study also provides a contribution in terms of the evaluation of the emotional and social competencies demonstrated by an individual and of the operationalization of the measurement of boundaryless career paths, considering three facets of the physical mobility construct (organizational, industrial, and geographical boundaries).</t>
@@ -10161,6 +10168,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>To explain how multistakeholder groups organize democratic deliberations about complex sustainability issues, organizational scholars have focused on the key role of deliberative capacity, which encompasses the dimensions of inclusiveness, authenticity and consequentiality. However, the tensions inherent to the search of these three dimensions have been overlooked. In this paper, we argue that focusing on how spaces for deliberation are designed can help one understand how to manage such tensions. We identified the boundary work practices that shape the design of deliberative spaces and generate deliberative capacity properties in a high-level expert group (HLEG) launched by the European Commission about sustainable finance regulation. Our results show how these boundary work practices help balance deliberative tensions. We advance deliberation studies by conceptualizing deliberative boundary work, explaining how deliberative capacity is spatially generated and showing how deliberative tensions are balanced. We also contribute to boundary work theory by making explicit the deliberative nature of configuring boundary work and showing its relevancy to regulatory settings.</t>
@@ -10208,7 +10216,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>Global offshoring has become a key strategy for international staffing, especially in the software industry. Global software teams engage in boundary spanning activities that may help MNEs achieve international connectivity and cope with external disruptions through their use of virtual work. However, offshoring IT professionals who bridge these boundaries in offshoring MNEs must contend with discontinuities, or perceived disruptions in expected communication flows, which impact their job satisfaction. Drawing on survey data from 193 professional consultants from an IT services offshoring MNE located primarily in Eastern Europe and working for a U.S. client, we test a model grounded in Organizational Discontinuity Theory. We find that potential discontinuities arising from the virtual work environment have no impact on the job satisfaction of offshoring IT professionals, but that those who experience team-level continuities of identification and shared vision are more satisfied with their jobs. Our findings suggest that virtual work may have become normalized such that it is not problematic in and of itself, and that fostering connectivity in boundary spanning global teams may be beneficial for MNEs. Our findings have important implications for MNEs managing disruptions created by global work arrangements as well as exogenous disruptions.</t>
@@ -10256,7 +10263,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>Acknowledgements: This research was funded by NSF grant #0422676 and #0726798 as well as support provided by the University of California, Irvine Center for Research on Information Technology in Organizations. The authors would like to acknowledge the helpful comments provided by Christopher Earley, Mark Griffin, John Mathieu, and Jone Pearce; assistance in data collection provided by Diaky Diaz, Christopher Reisdel and Bettina Wolf; and the generous time invested by all the film makers and film viewers who participated in the study.</t>
@@ -10304,6 +10310,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -10388,7 +10395,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -10801,6 +10807,12 @@
           <t>BSMA0198</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>T h i s position paper distinguishes different types of activities needed in software processes and proposes enaction support for t h e m . An architecture of enaction components providing this support is sketched.</t>
@@ -10824,6 +10836,11 @@
       <c r="K201" t="inlineStr">
         <is>
           <t>1995</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11324,6 +11341,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Innovation is considered the engine for firm growth. Especially innovations, through recombining seemingly unrelated knowledge streams, can have groundbreaking impact and lead to sustained competitive advantage. To generate such innovation, firms often need to go beyond their existing technological or geographical boundaries to identify and integrate novel knowledge elements. This article refers to firms’ knowledge activities of drawing upon distant knowledge (i.e., knowledge from dissimilar technological domains or distant geographical regions) to create novel technological solutions, as innovation through boundary spanning. Aiming to investigate the roles of information technology (IT) in facilitating innovation through boundary spanning, we collected data from the pharmaceutical industry over a six-year period to test the research model. The data analysis results indicate that IT supports boundary-spanning activities in firm innovation and different IT-enabled knowledge capabilities affect boundary-spanning innovation differently.</t>
@@ -11408,6 +11426,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -11968,6 +11987,12 @@
           <t>BSMA0229</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>Scholarship in the field of health communication is broad, with interdisciplinary contributions from researchers trained in a variety of fields including communication, nursing, medicine, pharmacy, public health, and social work. In this paper, we explore the role of “health communication boundary spanners” (HCBS), individuals whose scholarly work and academic appointment reflect dual citizenship in both the communication discipline and the health professions or public health. Using a process of critical reflective inquiry, we elucidate opportunities and challenges associated with HCBS across the spectrum of health communication in order to provide guidance for individuals pursuing boundary spanning roles and those who supervise and mentor them. This dual citizen role suggests that HCBS have unique skills, identities, perspectives, and practices that contribute new ways of being and knowing that transcend traditional disciplinary boundaries. The health communication field is evolving in response to the need to address significant healthcare and policy problems. No one discipline has the ability to single-handedly fix our current healthcare systems. Narrative data from this study illustrate the importance of seeing HCBS work beyond simply being informed by disciplinary knowledge. Rather, we suggest that adapting ways of knowing and definitions of expertise is an integral part of the solution to solving persistent health problems.</t>
@@ -11991,6 +12016,11 @@
       <c r="K232" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12005,6 +12035,16 @@
           <t>BSMA0230</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G233" t="inlineStr">
         <is>
           <t>Some audit researchers suggest that high levels of audit team structure may encumber communication within audit teams by impeding information-gathering activities. Others suggest that structure benefits communication by coordinating and controlling information flows. This study evaluated these arguments by examining the relationship between the structure of audit teams and selected communication variables (information overload, boundary spanning, satisfaction with supervision, and accuracy of information). Questionnaire data were gathered from a national sample of 109 audit teams, with three auditors responding from each team (i.e., n = 327). Information overload, satisfaction with supervision, and accuracy of information were less in audit teams with greater structure. The implication is that the level of structure adopted by teams has both positive and negative effects on communication, with structured teams providing greater control over information overload but impairing satisfaction with supervision and the accuracy of information.</t>
@@ -12028,6 +12068,11 @@
       <c r="K233" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12042,6 +12087,16 @@
           <t>BSMA0231</t>
         </is>
       </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G234" t="inlineStr">
         <is>
           <t>In this study of 338 inpatient psychiatric departments five hypotheses concerning organizational performance and size are tested and supported. It is found that psychiatric inpatient department performance varies with hospital ownership and is inversely related to department size. It is also found that increases in department size are not marked by changes in the relative size of administrative components. With increases in size, however, private hospitals tend to employ nonprofessional or paraprofessional support staff, while public hospitals are marked by a proliferation of professional staff. Furthermore, as inpatient departments increase in size they tend to increase the number of boundary spanning and buffering structures in existence. Discussed is the extent to which size and organizational ownership affect the performance of the psychiatric department.</t>
@@ -12065,6 +12120,11 @@
       <c r="K234" t="inlineStr">
         <is>
           <t>1973</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12079,6 +12139,12 @@
           <t>BSMA0232</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>Following the resource-advantage theory, this study advances the existing research of boundaryspanning search by examining which configuration of a new venture’s boundary-spanning search can obtain successful venture performance and how a founding team’s external relationship and the internal firm competences shape the relationship between the distant search and new venture performance. This paper is based on a questionnaire survey/analysis of a sample of 178 new ventures from China, and it offers insight to entrepreneurs with regard to the importance of building external managerial ties and developing idiosyncratic internal competences on boundary-spanning search. In addition, this study also reveals that the effectiveness of the supply-side, demand-side and spatialside boundary-spanning search on venture performance depends on investing resource at a rational level.</t>
@@ -12102,6 +12168,11 @@
       <c r="K235" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12116,6 +12187,12 @@
           <t>BSMA0233</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>Information system development can be considered a collaboration between users and developers. The inability to leverage the localized knowledge embedded in these two stakeholders hinders software development work to achieve high performance. Exploring the ways to counter this difﬁculty is then critical. This study applies an intellectual capital perspective to address the issues around spanning the knowledge boundary between developers and users. Our ﬁndings highlighted how important effective knowledge boundary spanning is to both product and project quality. Furthermore, three dimensions of intellectual capital increased the degree to which knowledge boundary spanning was effective.</t>
@@ -12139,6 +12216,11 @@
       <c r="K236" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12153,6 +12235,12 @@
           <t>BSMA0234</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>There appears to be a consensus that organizational integration across functional and disciplinary specialties drives superior ﬁrm capabilities. The basic assumption is that new practices and concepts emerge from the interaction of individuals engaged in different functional departments. However, communication across functional boundaries is often difﬁcult. As such, Tushman &amp; Scanlan suggested that functional boundaries can be spanned effectively only by boundary spanners who understand the coding schemes that are attuned to the contextual information on both sides of the boundary. The study of boundary spanners has signiﬁcant performance implications to ﬁrms. Compared to its importance, theoretical development and empirical inquiries into this phenomenon are relatively scant. Thus, this study explores the factors that determine who becomes a boundary spanner and examines boundary spanners’ performance implications. A Taiwanese company provided the context for our study. Partial Least Squares (PLS) was used to test the theoretical model. The results imply that a company needs to have an appropriate mixture of boundary spanners and non-boundary spanners, because boundary spanners have higher innovative performance.</t>
@@ -12176,6 +12264,11 @@
       <c r="K237" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12190,6 +12283,12 @@
           <t>BSMA0235</t>
         </is>
       </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate three issues: how does an innovative search (local search and boundary-spanning search) impact ﬁrm innovation performance of latecomers; how does capability reconﬁguration (capability evolution and capability substitution) mediates the relationship between innovative search and ﬁrm innovation performance; and how does the technological leapfrogging process (initial stage, following stage, synchronization stage and leading stage) moderate the relationship between capability reconﬁguration and ﬁrm innovation performance.</t>
@@ -12213,6 +12312,11 @@
       <c r="K238" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12264,6 +12368,12 @@
           <t>BSMA0237</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Boundary‐spanning personnel such as tax preparers, travel agents and hairdressers interface directly with customers. In their unique position, between the organization and customer, these service providers market the service to consumers while they simultaneously carry out operational functions. Both the customer and the provider bring certain expectations to the service encounter. These expectations then shape the perceptions of the service encounter. The research reported uses script methodology to compare the expectations between boundary‐spanning service providers and consumers of the same service. Draws its theoretical foundation from the expectations and scripts literatures. In Phase One, scripts of the service were elicited in order to test hypotheses based on the discovery and comparison of consumers′ and service providers′ subgoals for a typical service encounter (               H1               ). A hypothesis also tested the point at which providers and consumers enter their respective scripts of a typical service encounter (               H2               ). In Phase Two, the subgoals mentioned most frequently in Phase One were used as stimuli to elicit the specific actions which comprise the complete script. These complete scripts enabled a comparison of the elaborateness of provider and consumer scripts (               H3               ). The results of Phase One revealed that a portion of consumers′ subgoals for a service encounter are shared by providers of the service while other subgoals are unique, supporting               H1               . The point of activation of the script differed dramatically between customers and providers, supporting               H2               . The Phase Two findings provide support for the hypothesis that service providers have more elaborate scripts. Overall, the results support the notion that scripts operationalize expectations. Closes with implications for management and suggestions for future research.</t>
@@ -12287,6 +12397,11 @@
       <c r="K240" t="inlineStr">
         <is>
           <t>1995</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12301,6 +12416,12 @@
           <t>BSMA0238</t>
         </is>
       </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to explore how integration teams can build trusting relationships in component teams to enhance their leadership capability within multiteam systems to achieve common superordinate goals. The study investigates how an integration team diagnoses contextual dynamics to enhance understanding of goals in component teams and spans boundaries to create trusting relationships.</t>
@@ -12324,6 +12445,11 @@
       <c r="K241" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12338,6 +12464,16 @@
           <t>BSMA0239</t>
         </is>
       </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G242" t="inlineStr">
         <is>
           <t>Now more than ever, marketing is assuming a key boundary-spanning role—a role that has also redefined the composition of the marketing organization. In this paper, the marketing organization’s integrative and mutually reinforcing components of marketing activities, customer value–creating processes, networks, and stakeholders are delineated within their boundary-spanning roles as a particular emphasis (labeled MOR theory). Thematic marketing insights from a collection of 31 organization theories are used to advance knowledge on the boundary-spanning marketing organization within four areas—strategic marketing resources, marketing leadership and decision making, network alliances and collaborations, and the domestic and global marketplace.</t>
@@ -12361,6 +12497,11 @@
       <c r="K242" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12375,6 +12516,12 @@
           <t>BSMA0240</t>
         </is>
       </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>While there is a growing interest in the role of market information processing activities (i.e., the acquisition, dissemination, and use of market information) in new product development (NPD), a number of gaps remain in our knowledge on this topic. When investigating the performance impact of market information processing, most studies have treated the three activities as independent. Our research adds to the extant knowledge by exploring not only both direct relationships between each of the market information processing activities and new product performance, but also interaction effects. We, thus, ask the question of whether there may be synergies in obtaining performance increases by jointly improving two processing activities, rather than just considering each activity independently. In addition, we investigate these effects for different levels of information quality; a topic largely neglected in the market information processing literature. Our analysis is based on empirical data from 152 Dutch NPD projects. The results indicate that market information acquisition and use are both directly associated with increased performance. We also ﬁnd signiﬁcant interaction effects for information acquisition and dissemination, and for information dissemination and use. Finally, the importance of information quality is emphasized, with lower quality information producing lower performance and wiping out the effects between various aspects of market information processing and new product performance. We provide several implications of our ﬁndings for managers and academics.</t>
@@ -12398,6 +12545,11 @@
       <c r="K243" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12412,6 +12564,12 @@
           <t>BSMA0241</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>Background: Rehabilitation services depend on competent professionals who collaborate effectively. Wellfunctioning interprofessional teams are expected to positively impact continuity of care. Key factors in continuity of care are communication and collaboration among health care professionals in a team and their patients. This study assessed the associations between team functioning and patient-reported benefits and continuity of care in somatic rehabilitation centres. Methods: This prospective cohort study uses survey data from 984 patients and from health care professionals in 15 teams in seven somatic rehabilitation centres in Western Norway. Linear mixed effect models were used to investigate associations between the interprofessional team communication and relationship scores (measured by the Relational Coordination [RC] Survey and patient-reported benefit and personal-, team- and cross-boundary continuity of care. Patient-reported continuity of care was measured using the Norwegian version of the Nijmegen Continuity Questionnaire. Results: The mean communication score for healthcare teams was 3.9 (standard deviation [SD] = 0.63, 95% confidence interval [CI] = 3.78, 4.00), and the mean relationship score was 4.1 (SD = 0.56, 95% CI = 3.97, 4.18). Communication scores in rehabilitation teams varied from 3.4–4.3 and relationship scores from 3.6–4.5. Patients treated by teams with higher relationship scores experienced better continuity between health care professionals in the team at the rehabilitation centre (b = 0.36, 95% CI = 0.05, 0.68; p = 0.024). There was a positive association between RC communication in the team the patient was treated by and patient-reported activities of daily living benefit score; all other associations between RC scores and rehabilitation benefit scores were not significant. Conclusion: Team function is associated with better patient-reported continuity of care and higher ADL-benefit scores among patients after rehabilitation. These findings indicate that interprofessional teams’ RC scores may predict rehabilitation outcomes, but further studies are needed before RC scores can be used as a quality indicator in somatic rehabilitation.</t>
@@ -12435,6 +12593,11 @@
       <c r="K244" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12449,6 +12612,16 @@
           <t>BSMA0242</t>
         </is>
       </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G245" t="inlineStr">
         <is>
           <t>Purpose The purpose of this study was to investigate how changes in patient-rated health and disability from baseline to after rehabilitation were associated with communication and relationships in rehabilitation teams and patient-rated continuity of care. Methods Linear models were used to assess the associations between relational coordination [RC] and Nijmegen Continuity Questionnaire-Norwegian version [NCQ-N] with changes in the World Health Association Disability Assessment Schedule 2.0 [WHODAS 2.0] and EuroQol EQ-VAS [EQ-VAS]. To express change in WHODAS 2.0 and EQ-VAS, the model was adjusted for WHODAS 2.0 and EQ-VAS baseline scores. Analyses for possible slopes for the various diagnosis groups were performed. Results A sample of 701 patients were included in the patient cohort, followed from before rehabilitation to 1 year after a rehabilitation stay involving treatment by 15 different interprofessional teams. The analyses revealed associations between continuity of care and changes in patient-rated health, measured with EQ-VAS (all p values &lt; 0.01). RC communication was associated with more improvement in functioning in neoplasms patient group, compared to improvement of health among included patient groups. The results revealed no associations between NCQ-N and WHODAS 2.0 global score, or between RC in the rehabilitation teams treating the patients and changes in WHODAS 2.0 global score. Conclusion The current results revealed that better personal, team and cross-boundary continuity of rehabilitation care was associated with better patient health after rehabilitation at 1-year follow-up. Measures of patient experiences with different types of continuity of care may provide a promising indicator of the quality of rehabilitation care.</t>
@@ -12472,6 +12645,11 @@
       <c r="K245" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12486,6 +12664,16 @@
           <t>BSMA0243</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G246" t="inlineStr">
         <is>
           <t>Based on the four principles of self‐organization formulated by Morgan (1986), a four‐stage implementation model for empowering teams was developed. From the first to the last stage, the attention shifts from routine tasks to non‐routine tasks, from the individual to the group, and from inwards oriented to outwards directed activities. This model was used to develop five teams in an industrial glass producing firm. After two years, team progress was measured by means of a questionnaire and the results were discussed with each team. These data were used to evaluate the viability and applicability of the empowerment plan and to find relevant factors which facilitate or hinder the empowerment process. The results indicate that the step‐by‐step plan facilitates the development of empowered teams but that it should not be seen necessarily as the best or the only way of empowering working groups. Moreover, the attitude and style of management, the team cohesion and the nature of the work involved seem to interfere with team empowerment.</t>
@@ -12509,6 +12697,11 @@
       <c r="K246" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12824,6 +13017,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>Marketing boundary spanners—especially customer service representatives—are notably susceptible to burnout. The authors define the burnout construct and develop hypotheses to examine if burnout acts as a partial mediator between role stressors and key behavioral and psychological job outcomes. Responses from 377 customer service representatives reveal that burnout levels are high relative to other burnout-prone occupations (e.g., police, nursing) and that burnout has consistent, significant, and dysfunctional effects on their behavioral and psychological outcomes. Moreover, burnout mediates the negative effects of role stressors on job outcomes, whereas the positive effects of role stressors are unmediated.</t>
@@ -12871,6 +13065,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -12918,6 +13113,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>Because of their boundary-spanning nature, manufacturers’ representatives frequently are involved in team selling. The results from a survey of 362 manufacturers’ representatives indicates that team selling is more likely to be used by manufacturers’ representatives when the customer faces a first-time buy of a complex product, when the information needs of the customer are great, when the account requires special treatment, and when a number of people are involved in the decision to buy. In addition, team selling is more likely when the potential sale is large for the representative firm and when the product is new to the representative’s product line.</t>
@@ -12965,6 +13161,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>With congeneric mergers, which involve firms with interrelated but not identical business lines that develop diverse products and services, a major challenge for organizations is the development of a common platform that fulfills similar business functions across multiple divisions. Through a field study of a postmerger common platform development initiative, we develop a framework that highlights how environmental and organizational contexts shape the process of common platform development (CPD). Our study provides an account of how the focal organization transitioned to a platform-based approach by achieving a balance between stable and flexible aspects of the common platform through negotiations among the divisions acquired through mergers and acquisitions. These negotiations were enabled through various boundary-spanning activities and the guided successive enrichment of boundary objects used in CPD process. European Journal of Information Systems (2015) 24(2), 159–177.</t>
@@ -13012,7 +13209,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>Two main targets of contemporary preferential innovation policy support, especially in Europe, are key enabling technologies (KETs) and innovation ‘missions’ focused on solving societal challenges. Both topics are associated with uniting disparate sets of capabilities, either by driving technology-based innovation into various application domains or by eliciting interdisciplinary and cross-sectoral solutions to urgent societal demands. In this study we assess to what extent pre-commercial R&amp;D collaborations span geographic and cognitive boundaries. We analyze firm-level tie formation in Dutch collaborative R&amp;D projects initiated in the period 2013–2018. Gravity models reveal that, while results for geographic proximity are mixed, some KET types are indeed related to projects in which cognitive proximity is significantly less relevant for tie formation. This contrasts with the findings for projects that retroactively received a mission label. Projects on health and care missions, and especially energy transition and sustainability missions, instead spur collaborations between cognitively proximate firms. The latter suggests that without additional policy intervention, such projects might interconnect similar rather than dissimilar knowledge bases. We conclude by discussing research and policy implications.</t>
@@ -13060,7 +13256,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -13108,6 +13303,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>This study investigated the effects of small business owner decision styles on the search for external assistance information, community information, and competitor information. Results confirmed the existence of decision style differences in selection of boundary spanning activities. A conclusion is drawn that small business owners use preferred sources for gathering information related to business operations, but need to utilize additional sources to ensure a comprehensive boundary spanning role. Ways to enhance boundary spanning activities are provided</t>
@@ -13155,6 +13351,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>The influence of boundary spanning roles on strategic decision-making was explored in a field study in fifteen organizations. Results support the importance of boundary spanning roles in the strategic decision-making process and the relationship of technology to the differential strategic decision-making influence of different boundary spanning roles.</t>
@@ -14497,6 +14694,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -15917,7 +16115,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>Science parks are a type of organizational sponsorship initiative aimed at generating resource-munificent environments through the provision of bridging and buffering services. While extant research has studied the relationship between these services and firm outcomes, it has neglected to provide insights into when tenant firms utilize these services to a greater or lesser extent. Our study evaluates science parks’ buffering mechanism and identifies firm-level characteristics affecting tenants’ use intensity of buffering services. To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries. Taking a resource dependence perspective, our findings indicate that tenants’ managerial resources (particularly top management team size and functional experience) and boundary-spanning capacity jointly determine the extent to which firms rely upon the science park’s buffering mechanism. This study contributes to the organizational sponsorship, resource dependence, and science park literatures, as well as has important practical implications.</t>
@@ -15965,6 +16162,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>Purpose – As teams are built around specialized and different knowledge, they need to regulate their knowledge boundaries to exchange their specialized knowledge with other teams and to protect the value of such specialized knowledge. However, prior studies focus primarily on boundary spanning and imply that boundaries are obstacles to sharing knowledge. To ﬁll this research gap, this study aims to indicate the importance of knowledge protection regulation, an activity that sets an adequate boundary for protecting knowledge, and investigate the factors that facilitate knowledge protection regulation and its consequences.</t>
@@ -16049,7 +16247,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the effects of relationship bonds on the psychological response and behavior of bank employees based on the job demands–resources theory. Specifically, it examines the effects of relationship bonds in terms of person–job (P–J) fit, emotional exhaustion, job satisfaction and boundary-spanning behaviors, all of which comprise the behavioral dimensions of bank employees. In addition, the study examines how the resiliency of bank employees influences their emotional exhaustion and determines whether a moderating effect related to emotional exhaustion exists.</t>
@@ -16097,7 +16294,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -16197,6 +16393,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -16244,6 +16441,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>Improving performance often requires creative ideas in extreme work settings like health care. Frontline workers are promising sources of creative ideas. The authors assert that their job dissatisfaction is positively associated with creativity in health care settings because negative emotion spurs creativity when tied to engaging work and that characteristics such as shorter tenure, greater role centrality, and high boundary spanning can strengthen this relationship. The authors find supporting evidence in data on ideas generated over 18 months by health professionals in 12 clinics.</t>
@@ -16291,7 +16489,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>Innovation is a risky business. Notwithstanding the attention in research on the determinants of innovation success, the estimates of the extremely high failure rates (ranging from 40% to 90%) have not come down. As a result, new approaches have to be found to address the issues that prevent organizations from reaching innovation success over a longer period of time. In this study, Signal Detection Theory (SDT) is introduced to show that it may be less important to improve innovation practices in companies, than it is to change the nature of the projects that enter the corporate innovation funnel. In our empirical study of 44 innovation projects in the pharmaceutical and electronics industry, we show that pursuing more noisy signals (uncertain technological and market opportunities) is currently beneficial for innovation success. In general, companies allocate too few resources to noisy innovation opportunities. Interestingly, we find a positive, and not an inverted U-shaped, relationship between noise/signal ratios and innovation success. This indicates that there are almost no companies that take too much risk in the current competitive environment and that many can gain from increasing their noise tolerance. The implications from this study are quite counter-intuitive in a sense that ‘risk’ is not the cause of the innovation problems, but may be a solution.</t>
@@ -16339,6 +16536,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to provide a novel way of thinking about firm internationalization. We offer a stylized view of family firms as internationalizers who choose to engage in “boundary-spanning” across global product markets while engaging in “boundary-buffering” to insulate themselves from global financial markets.</t>
@@ -16386,6 +16584,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>Multiteam systems (MTSs) have been increasingly adopted as an organizational form to manage large-scale projects. However, new product development (NPD) in the MTSs structure entails challenges with respect to achieving efﬁciency due to interteam coordination challenges. Shared mental models (SMMs) within a single team have been found to facilitate intrateam coordination; however, further exploration is needed as to whether SMMs within MTSs can improve interteam coordination among component teams and, if so, what mechanisms underlie this. The present article examines the theoretical underpinning of the impacts of SMMs among component team leaders on MTSs’ NPD efﬁciency, and further considers the impact of external conditions of requirement uncertainty, the most common external situation during NPD. Using survey data from 110 information technology development MTSs and drawing on boundary management perspective, the results reveal that SMMs among component team leaders positively affect NPD efﬁciency by managing the MTSs boundary, i.e., through boundary entrainment and boundary buffering activities at the system level. In addition, we ﬁnd that requirement uncertainty plays a vital role in determining the nature of this relationship. Taken together, our ﬁndings highlight the importance of the role of SMMs among component team leaders in facilitating NPD efﬁciency in MTSs settings.</t>
@@ -16433,7 +16632,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>Past research on team boundary work has focused on a “cold,” information-exchange perspective to explain why boundary activities affect team innovation. Although the theory is widely accepted, empirical studies on the actual mechanism are scant and produce inconsistent results. Drawing from Interaction Ritual Theory (Collins, 2004), we propose a “warm,” affective perspective that emphasizes team emotional energy - a shared feeling of enthusiasm among team members - as a mechanism linking boundary work and team innovation. Moreover, we examine a theory-driven contextual factor -team role overload - that modifies the hypothesized mediated relationship. Based on field data from four different sources of 89 automotive research and development teams (comprising 724 employees, 89 direct supervisors and 18 managers), we found that both team boundary-spanning and boundary-buffering activities are associated with higher levels of team emotional energy, which, in turn, are related to greater levels of team innovation. Moreover, the mediated relationship of boundary-buffering activities, team emotional energy and team innovation is moderated by team role overload, such that the mediated relationship is stronger when team role overload is higher. Our study contributes to the literature by broadening our understanding of why boundary work is effective and when it matters most.</t>
@@ -16528,7 +16726,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>Boundary spanning activity Is conceived of as an intervening variable between organization structure and perceived environmental uncertainty. This is because boundary spanners operate at the skin of the organization and hence their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relationships between perceived environmental uncertainty, organization structure, and boundary spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relationships were found between all three variables. Partial relationships indicated that PEtJ does not influence the boundary spanning-structure relationship, but structure reduces the PEtJ-boundary spanning relationship to zero, and boundary spanning reduces the structurePEU relationship to zero. Thus, not only is the boundary spanning as an intervening variable supported, but results suggest that causality in the Btructure-PEU relationship may be in the direction of structure to PEU rather than current contingency notions of PEU effecting structure.</t>
@@ -16576,7 +16773,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>Boundary-spanning activity is conceived of as an intervening variable between organization structure and perceived environmental uncertainty (PEU). This is due primarily because, since boundary spanners operate at the skin of the organization, their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relations between PEU, organization structure, and boundary-spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relations were found between all three variables. Partial relations indicated that PEU does not influence the relationship of boundary spanning to structure but structure reduces the relationship of PEU to boundary spanning to zero, and boundary spanning reduces the relationship between structure and PEU to zero. Thus, not only is the notion of boundary spanning as an intervening variable supported, but results suggest that causality in the relationship between structure and PEU may be from structure to PEU rather than current contingency notions of PEU affecting structure.</t>
@@ -16624,7 +16820,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>Building on the theories of knowledge recombination, we argue that the external acquisition of technologies acts as a boundary spanning mechanism that impacts on the recipient firm’ subsequent technology development. The effect is moderated by two additional mechanisms, namely the retention of star scientists and the experience in upstream strategic alliances. We tested our hypotheses on a sample of 6208 USPTO patented technologies acquired by 350 biotechnology firms over the period 1980–2012. Findings reveal an inverted U-shaped effect of the pioneering nature of the acquired technology on firm’s subsequent developments, in terms of (self) citations of firm’s subsequent patents to the acquired one. Moreover, the main relationship is negatively moderated by the retention of star scientists, while the experience in upstream alliances demonstrates to be a positive moderator.</t>
@@ -16672,7 +16867,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>Successful product development requires managing tensions—coping with fluctuating contingencies to foster innovation and efficiency. To investigate this challenge, we explored the nature, dynamics, and impacts of contrasting project management styles. Our conceptual framework details emergent and planned styles. Following 80 projects over two-year periods, we find that these styles offer disparate but interwoven approaches to monitoring, evaluation, and control activities; use of these activities fluctuates over time; a paradoxical blend of styles enhances performance; and uncertainty moderates project management-performance relationships.</t>
@@ -16720,7 +16914,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>Boundary spanning has been proven to have positive implications for innovation performance; yet, some individuals are less boundary-spanning than others. Drawing on the attachment theory and organizational support theory, this study develops a multi-level theoretical model to investigate how individuals’ attachment insecurity influences boundaryspanning behavior through self-efficacy and the moderating role of organizational support climate. To validate the proposed model, we adopted a survey research, and collected data from NPD project teams in China. The results revealed that both insecure attachment styles were associated with lower levels of individual boundary-spanning behavior, and self-efficacy partially mediated these relationships. Moreover, organizational support climate played a moderating role in the relationship between attachment anxiety and boundary-spanning behavior. With a high level of support climate, the negative impact of attachment anxiety on boundary-spanning behavior was weakened. This elucidates the role of individual affective motivation and team shared perceptions in shaping individual externally focused behavior.</t>
@@ -16820,7 +17013,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>From a knowledge-based perspective, this paper highlights the need for a framework linking perceived competition of the industry and ﬁrms’ strategic location choices of external knowledge search and examines whether the perceived competition increases the propensity of cluster ﬁrms to search more widely from extra-cluster knowledge sources than intra-cluster knowledge sources. Furthermore, we emphasise that cluster ﬁrms with varying degrees of tacitness in their knowledge base might respond to such competition diﬀerently when conducting external knowledge search activities. Using a sample of 310 cluster ﬁrms in the Zhejiang Province of China, we ﬁnd that the cluster ﬁrm would increase the propensity for more geographic boundary-spanning search relative to local search while under the pressure of competition. Moreover, the positive relationship between perceived competition and the propensity towards geographic knowledge search is weaker when the tacitness of the cluster ﬁrm’s knowledge base is higher. The ﬁndings contribute to the understanding of the relationship between competition and the choice of location strategies in external knowledge search.</t>
@@ -16868,6 +17060,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -17722,7 +17915,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>Based on the social identity theory, this study investigates whether and how employee perceptions of corporate environmental behavior (CEB) influence the realization of an organization's internal value. Using employees' organizational citizenship behavior (OCB) as a direct agent for corporate internal value, the current study constructs a theoretical model of perceived CEB and OCB, with work meaningfulness and person–organization (P-O) value fit serving as mediator and moderator, respectively. After analyzing 235 questionnaire samples, we discovered that the perceived CEB positively influenced OCB via work meaningfulness and that this positive effect was strengthened by a greater P-O value fit. These findings suggest that in the process of motivating employees to implement OCB, firms should address the significance of internal driving roles of work meaningfulness and boundary-spanning roles of P-O value fit in order to enhance corporate internal value and correct managers' misconceptions about the value of CEB.</t>
@@ -17770,7 +17962,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F378" t="inlineStr"/>
       <c r="G378" t="inlineStr">
         <is>
           <t>A central focus of cross-cultural management research is how individuals and organizations differ across national cultures and how that fundamentally shapes their thoughts and actions and serves as a unit of identification. In this article, we critically reconsider the essential categorical nature of culture, problematizing categorization and questioning national culture as the primary basis of differentiation. We draw on intersectionality, an approach that helps understand how multiple categories are experienced by the individual, and on relationality, an approach that conceptualizes people, organizations, and their actions within dynamic patterns of relations and cultural meanings. Both approaches challenge the primacy, unity, and separateness of any given category, the a priori determination of categories (and associated boundaries) in research, and the nature and stability of boundaries. Based on this we advance notions of boundary work and boundary shifting that help explore how today’s sociocultural groups and categories, and the boundaries that separate them, emerge and change. We conclude that, while the extant crosscultural literature has come far in identifying differences, relationality and intersectionality can enable cross-cultural scholars to engage in research practice that better reflects the complexities of sociocultural life. We contribute to theory by suggesting why and how these two approaches can be used to explore complex cross-cultural management phenomena.</t>
@@ -17818,7 +18009,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F379" t="inlineStr"/>
       <c r="G379" t="inlineStr">
         <is>
           <t>The paper explores how formal leaders make sense of and deal with autonomy of knowledge-workers. Based on interviews, I suggest that leaders make sense of knowledge-workers’ autonomy as ranging from perfectly autonomous to too autonomous to less independent to acting childish. This ambiguity was dealt with by making sense of leading as ranging from facilitative and supportive approaches to more controlling, even reprimanding acts. This empirical investigation of constructions of ‘leader/ship’ and ‘followers’ contributes to leader/ship-follower/ship literature. The paper’s contribution to theory lies in the notion of situated ambiguity; a way to understand the emerging way through which formal leaders navigate and smoothly move between their own diﬀering perspectives, diﬀerent practical situations, various culturally acceptable understandings of leaders and knowledgeworkers.</t>
@@ -17940,7 +18130,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>Building on the “loose coupling” logic, this study examines the importance of boundary spanners' shared perceptions of procedural justice in cross-cultural cooperative alliances. I argue that alliance profitability is higher when both parties perceive high rather than low procedural justice. Profitability is also higher when both parties' perceptions are high than when one party perceives high procedural justice but the other perceives low procedural justice. Shared justice perceptions become even more important for alliance profitability when the cultural distance between partners is high or when the industry of operation is uncertain. Analysis of 124 cross-cultural alliances in China supports these propositions.</t>
@@ -17988,7 +18177,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>This study extends research on strategic alliances by exploring independent and combined effects of distributive, procedural, and interactional justice in these alliances. An integrated framework links cooperation payoffs with organizational justice as perceived by boundary-spanning alliance executives, through whom justice perceptions become parent actions. Analysis of 127 alliances demonstrates that when goal differences between parties are high, the joint effect on alliance performance of procedural and distributive justice is significantly positive. When interactional justice is high, procedural justice exerts a stronger performance effect. This perspective enriches alliance research, especially regarding procedural formalization, incentive structure, and interparty attachment.</t>
@@ -18036,7 +18224,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19216,7 +19403,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>The purpose of this research is to determine the description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, to determine and analyze the influence of Emotional Dissonance on Service Sabotage, to determine and analyze the influence of Emotional Intelligence on Service Sabotage, and to determine and analyze the influence of Emotional Exhaustion on Service Sabotage. The population in this study were all employees of the Grand Mercure Hotel Kemayoran Jakarta. In this research, a quantitative method approach was used with a survey and a sample of 225 people was obtained using a purposive sampling technique. Survey research is carried out by distributing questionnaires. Previously, the questionnaire was tested for validity and reliability first. The data analysis technique in this research uses descriptive analysis and linear regression analysis. Description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, most of whom are male, most employees are under 35 years old, and most employees have worked at the hotel for 0-2 years. The results of this research explain that Emotional Dissonance has a positive and significant effect on Service Sabotage with p-value of 0.012. Emotional Intelligence has a negative and significant effect on Service Sabotage with p-value of 0.023. Emotional Exhaustion has a positive and significant effect on Service Sabotage with p-value of 0.045.</t>
@@ -19264,6 +19450,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -19311,7 +19498,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>Intergroup knowledge integration, that is the acquisition, processing, and utilization of knowledge across group boundaries, is a critical source of competitive advantage in modern organizations. Prior research has highlighted the important role of boundary spanning knowledge exchange for intergroup knowledge integration, neglecting, however, the question of what makes individual boundary spanners more effective in fostering intergroup knowledge integration. Integrating boundary spanning literature with theories of group information processing, we hypothesize that the effect of individual boundary spanning ties on intergroup knowledge integration depends on the boundary spanners’ levels of metaknowledge, i.e., knowledge of who knows what in their respective groups, and proactivity. We find general support for our predictions in a study of 457 engineering consultants nested in 22 interdependent business units within an organization. Additional criterion analyses confirm the material importance of intergroup knowledge integration for group performance. Our findings have implications for literatures on intergroup effectiveness, team cognition, and proactivity.</t>
@@ -19406,7 +19592,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their boundaries in ways that complement their preferences.</t>
@@ -19454,7 +19639,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>Background Increasing role complexity has intensiﬁed the boundary spanning functions of managers. Because work demands and scope vary by management position, time in staff contact rather than span may better explain managersÕ capacity to support staff. Methods A descriptive, correlational design was used to collect cross-sectional survey and prospective work log and administrative data from a convenience sample of 558 nurses in 51 clinical areas and 31 front-line nurse managers from four acute care hospitals in 2007–2008. Data were analysed using hierarchical linear modelling. Results Span, but not time in staff contact, interacted with leadership and operational hours to explain supervision satisfaction. Conclusions With compressed operational hours, supervision satisfaction was lower with highly transformational leadership in combination with wider spans. With extended operational hours, supervision satisfaction was higher with highly transformational leadership, and this effect was more pronounced under wider spans. Implications for Nursing Management Operational hours, which inﬂuence the managerÕs daily span (average number of direct report staff working per weekday), should be factored into the design of front-line management positions.</t>
@@ -19502,6 +19686,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>This dissertation investigates factors that influence efforts by lower-level employees to initiate organizational change and innovation from the bottom up. Specifically, I attempt to reconcile competing theories regarding the effects of structural and social integration on individual innovation efforts. One theoretical view posits that integration provides information, ideas, and motivation necessary for innovation. An alternative view is that integration constrains individuals and routines, and thereby hinders innovation efforts. Drawing on both theoretical perspectives, I predict the effects of distinct types of structural integration (eg, centralization, cross-unit integration, boundary spanning) and social integration determinants (eg, geographic dispersion, decision process involvement, workplace network size) on the likelihood of individual innovation efforts among lower-level employees. I also consider the effects of interactions of social and structural integration with individual characteristics (ie, personality, and experience) on innovation efforts. I test these predictions using survey data collected from interns and supervisors in the context of MBA and undergraduate internships. Analyses demonstrate that several aspects of structural integration do influence the levels of individual innovation efforts. For example, centralization and boundary spanning levels of the work unit have inverse U-shaped relationships with the level of innovation effort. These findings suggest that for certain types of innovation, structural integration can constrain efforts at the extremes (very high or low) and facilitate efforts at modest levels of integration. Predicted social integration effects are largely non-significant, suggesting the need for further consideration and alternative empirical tests of such effects. Nevertheless, the structural integration findings reaffirm the need to bring together both theoretical perspectives (ie, the view that integration fosters innovation efforts, and the alternative view that isolation and independence are necessary for innovation). By empirically demonstrating that distinct types of integration have unique, yet theoretically consistent effects on several different classes of individual innovation efforts (both process and strategy related), this study contributes to efforts to reconcile these competing theories. Additionally, this research enhances our understanding of a class of little-studied behaviors that play a potentially important role in autonomous strategic change and organizational learning.</t>
@@ -19601,7 +19786,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>Background: Emotions play a central role in how employees respond to workplace bullying, influencing both their well-being and organizational outcomes. The purpose of the current study was to examine how workplace bullying and turnover intention are related to negative emotions and workplace unfairness. Methods: The research involved collecting data from 269 boundary-spanning bank workers (call center workers, frontline office staff, and customer service representatives) who experienced bullying. A moderated mediation was tested using Model 7 of the Process macro. The relationship between workplace bullying and turnover intention was analyzed, emphasizing the moderating effect of workplace unfairness and the mediating role of negative emotions. Results: The results validated the model, showing that an increase in negative emotions and workplace unfairness promotes the link between workplace bullying and the intention to leave. Increased negative emotions and perceived workplace unfairness amplified the relationship between workplace bullying and turnover intention. Conclusions: The findings underscored the cumulative risk of bullying environments for employee well-being and retention, providing practical recommendations for HRM and leadership strategies to cultivate healthier, more inclusive workplace settings. This study adds to the bullying–turnover literature by examining the joint role of negative emotions and workplace unfairness in a moderated mediation framework. The study connects these findings to sustainable labor management, emphasizing both theoretical and practical implications for organizations.</t>
@@ -19649,6 +19833,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
           <t>It is widely recognized that new product development (NPD) is a highly interdependent process, yet efforts to empirically model the interdependence and examine its effect on ﬁrm performance are scarce. Our study addresses this research gap. We model ﬁrms’ abilities to collectively collaborate with suppliers, customers, and internal employee teams in NPD as collaborative competence and examine its impact on project and market performance. Using responses collected from 189 NPD managers, we ﬁnd empirical evidence for collaborative competence and its differential impact on project and market performance. Speciﬁcally, we ﬁnd that collaborative competence has a direct impact on project performance, but its impact on market performance is indirect, mediated through project performance. The results have signiﬁcant managerial implications; achieving superior market performance from inter- and intra-organizational involvement is contingent on achieving superior project performance, and companies that fail to achieve desired project performance outcomes will also fail in achieving market performance goals.</t>
@@ -19696,7 +19881,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>Abstract             In organizational contexts, professional boundaries serve a dual purpose by distinguishing various professions from one another and regulating access to power, status, and rewards. Individuals operating within professions in which such boundaries are not clearly or explicitly defined face the risk of compromising their status and autonomy. However, they possess the agency to actively define their profession and enhance its standing among both internal and external stakeholders. This study explores how homeroom teachers in the Israeli education system—recognized as a distinct occupation within the broader teaching profession—engage in boundary work to form and define their professional group. Our findings reveal that (1) homeroom teachers employ adaptable boundary work strategies, tailored to their interactions with different key stakeholders. Specifically, they (a) define boundaries to clarify, for themselves, the parameters of their own roles; (b) balance boundaries with partners inside the school (administrators and subject teachers) to facilitate day-to-day collaboration while simultaneously asserting their own roles; and (c) orchestrate boundaries when interacting with external partners (students’ parents), acknowledging the distinction between roles while primarily seeking to foster effective joint work towards the common goal of helping students succeed. (2) Despite the diversity in their approaches, all homeroom teachers exhibit a unique expertise, allowing them to combine boundary-setting with inclusivity, highlighting the dynamic and interactive nature of the boundary work process. This dual nature enhances the effectiveness of communication and collaboration within the educational system, molding the role of homeroom teachers as a distinct professional group.</t>
@@ -19744,6 +19928,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
           <t>Recent research has emphasized cross functional integration as a key facilitator of success in new product development (NPD) projects. This dissertation developed and tested a model using supply chain integration as a key enabler influencing both planning of the new product and execution of the development process in NPD projects. Supply chain integration was operationalized to include cross functional (for example, between design and manufacturing) and boundary spanning integration mechanisms (such as supplier integration). Product concept effectiveness (a construct capturing the planning of the new product), and development process performance (a construct measuring the execution of new product development process) were theorized to influence overall project success. Hypotheses drawn from this framework were tested on a multi-industry sample (electronics, communications, semiconductors, and computers) of firms. Data analysis was conducted using regression analyses, partial correlations, confirmatory factor analyses and structural equation modeling.</t>
@@ -19843,6 +20028,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
           <t>Mentoring is a valuable resource that enhances outcomes like career success. Applying conservation of resources theory, we examine the interaction effects of workers’ management aspirations and lengthy career interruption(s) on the mentoring-career success relationship. Utilizing 259 older professional workers, we test these relationships with both cross-sectional and time-separated data. Although the pattern of results was similar when comparing the crosssectional data to the time-separated data, we found that relationships were stronger within the cross-sectional data, resulting in the support of two additional hypotheses. With the timeseparated data, we found evidence of a three-way interaction. Speciﬁcally, mentoring is more valuable for the perceived career success of workers with higher management aspirations who had not experienced a lengthy career interruption than it is for workers with higher management aspirations who had experienced a lengthy career interruption or for workers with lower management aspirations regardless of whether they had experienced a career interruption.</t>
@@ -19942,7 +20128,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>Urban metabolism approaches are increasingly becoming relevant in providing pathways to sustainable development. The ways through which urban green infrastructures are planned and designed can influence resource flows in cities. Yet, little is known about the agency and contributions of landscape architects and spatial planners as curators of urban greenery, in facilitating circular resource flows, and accelerating the transition to a circular economy. This paper offers an empirical inquiry into the understanding and use of metabolic approaches in spatial planning and design practices. Through a multi-method approach and the use of boundary spanning as an analytical lens, we identify different modes of agency of spatial practitioners in enhancing resource efficiency across the life stages of urban landscape projects. Results show that while the ‘urban metabolism’ concept is not widely used by practitioners, its relevance to planning and designing green infrastructure for sustainable resource flows is well understood. Additionally, we highlight existing barriers including policy constraints in engaging with metabolic approaches and offer recommendations to facilitate a resource-sensitive turn in planning and designing urban landscapes. This study highlights important contributions of design practice to an expanding discourse of urban metabolism, including policy reforms for enabling circular resource flows in cities.</t>
@@ -19990,7 +20175,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -22439,6 +22623,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>Abstract             In this study, we analyse the discursive strategies of professionalization used by psychology in Spain during its professionalization phase in the health sector in the early twenty-first century. Our primary focus is the conflict with political regulators and other healthcare professions after the Ley de Ordenación de Profesiones Sanitarias (Healthcare Professions Act) came into effect, since this Act calls into question the extent to which psychology can be viewed as health care. We use discourse analysis to determine the discursive structure of the conflict, which has an interprofessional dimension, as well as the professionalization and social closure strategies of psychology within the framework of professional relationships (boundary work). We argue that understanding this conflict requires viewing it as part of the European and international regulation context of healthcare professions. Highlighted in the analysis is the emergence of two psychology discourses divided into four modes of enunciation (professionalizing, cultural, scientific, and political–economic). Among other aspects, the conclusions focus on the dual interprofessional and intraprofessional nature of the conflict and evidence of a dual closure in psychology. The latter’s professionalization strategies in the sector occasionally resemble those employed by nursing, although at other times they are similar to those followed by some paramedical professions.</t>
@@ -22538,6 +22723,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -24115,7 +24301,7 @@
       </c>
       <c r="P537" t="inlineStr">
         <is>
-          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Abstract] "This paper proposes a radical empirical look on the concrete activities of project managers involved in creative projects, with a speciﬁc focus on ‘‘non-administrative’’ issues. Through four case studies in the video-game industry, multimedia, advertising and a circus, we propose an integrated synthesis of what creative project managers actually do." [Research method] "This is a cases study based research which derives from an exploratory ethnographic ﬁeld study on the video-game industry in the tradition of grounded theory [43,44] and qualitative research on emergent phenomena [45–47] ."</t>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Abstract] "This paper proposes a radical empirical look on the concrete activities of project managers involved in creative projects, with a speciï¬c focus on âânon-administrativeââ issues. Through four case studies in the video-game industry, multimedia, advertising and a circus, we propose an integrated synthesis of what creative project managers actually do." [Research method] "This is a cases study based research which derives from an exploratory ethnographic ï¬eld study on the video-game industry in the tradition of grounded theory [43,44] and qualitative research on emergent phenomena [45â47] ."</t>
         </is>
       </c>
     </row>
@@ -24167,7 +24353,7 @@
       </c>
       <c r="P538" t="inlineStr">
         <is>
-          <t>Excluded due to multiple reasons: the unit of analysis is the manufacturer-supplier dyad (Code 3), and the boundary-spanning proxy merely measures communication frequency (Code 1).. Verbatim Evidence: [4.1. Data Collection and Sample Characteristics] "The unit of analysis for this study is a manufacturer (buyer)–supplier dyad." [4.1. Data Collection and Sample Characteristics] "The respondents answered questions regarding the overall relationship between the two firms, including listing all of the buyer plant locations that received products from the supplier." [Appendix A: Survey Questions] "Media-Rich Communication (Source = Buyer) (1 = Never; 2 = Annually; 3 = Semi-annually; 4 = Quarterly; 5 = Monthly; 6 = Weekly; 7 = Daily) How often do personnel from your firm and &lt;&lt;SUPPLIER&gt;&gt; communicate using the following methods. . . PC1 Face-to-face PC3 Telephone"</t>
+          <t>Excluded due to multiple reasons: the unit of analysis is the manufacturer-supplier dyad (Code 3), and the boundary-spanning proxy merely measures communication frequency (Code 1).. Verbatim Evidence: [4.1. Data Collection and Sample Characteristics] "The unit of analysis for this study is a manufacturer (buyer)âsupplier dyad." [4.1. Data Collection and Sample Characteristics] "The respondents answered questions regarding the overall relationship between the two firms, including listing all of the buyer plant locations that received products from the supplier." [Appendix A: Survey Questions] "Media-Rich Communication (Source = Buyer) (1 = Never; 2 = Annually; 3 = Semi-annually; 4 = Quarterly; 5 = Monthly; 6 = Weekly; 7 = Daily) How often do personnel from your firm and &lt;&lt;SUPPLIER&gt;&gt; communicate using the following methods. . . PC1 Face-to-face PC3 Telephone"</t>
         </is>
       </c>
     </row>
@@ -24531,7 +24717,7 @@
       </c>
       <c r="P545" t="inlineStr">
         <is>
-          <t>Team Level Aggregation (N = 60 teams). Verbatim Evidence: [Sample] "Sixty product development teams were recruited from different high-technology companies in Israel, specializing in telecommunications, computer software, computer hardware, and semiconductors." [Level of Analysis] "In the present study, the unit of analysis was the team. All the hypotheses referred to the team and such study variables as boundary activities and inter-team goal interdependence were framed at the team level, and aggregated to team level." [Correlation Matrix] "Table 1. Means, Standard Deviations, and Correlation Matrix of Study’s Variables (N = 60)."</t>
+          <t>Team Level Aggregation (N = 60 teams). Verbatim Evidence: [Sample] "Sixty product development teams were recruited from different high-technology companies in Israel, specializing in telecommunications, computer software, computer hardware, and semiconductors." [Level of Analysis] "In the present study, the unit of analysis was the team. All the hypotheses referred to the team and such study variables as boundary activities and inter-team goal interdependence were framed at the team level, and aggregated to team level." [Correlation Matrix] "Table 1. Means, Standard Deviations, and Correlation Matrix of Studyâs Variables (N = 60)."</t>
         </is>
       </c>
     </row>
@@ -24724,7 +24910,7 @@
       </c>
       <c r="P549" t="inlineStr">
         <is>
-          <t>No correlation matrix or extractable zero-order effect size (reports only GLMs with McFadden's pseudo-R^2). Verbatim Evidence: [Methods] "I then constructed 5 generalized linear models (GLMs) to understand the influence of social network position and personal factors on collaborative behavior." [Results] "I ran five different generalized linear models (GLM) with CS as the dependent variable, using the “quasibinomial” family to account for CS being a proportion." [Results] "Table 4. Results of 5 GLMs predicting influence of variables on Collaborative Score (CS)."</t>
+          <t>No correlation matrix or extractable zero-order effect size (reports only GLMs with McFadden's pseudo-R^2). Verbatim Evidence: [Methods] "I then constructed 5 generalized linear models (GLMs) to understand the influence of social network position and personal factors on collaborative behavior." [Results] "I ran five different generalized linear models (GLM) with CS as the dependent variable, using the âquasibinomialâ family to account for CS being a proportion." [Results] "Table 4. Results of 5 GLMs predicting influence of variables on Collaborative Score (CS)."</t>
         </is>
       </c>
     </row>
@@ -24776,7 +24962,7 @@
       </c>
       <c r="P550" t="inlineStr">
         <is>
-          <t>No effect size of interest. Measures coping strategies rather than boundary spanning behavior.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] The study collected data from multiple sources: survey data from 452 boundary-spanning salespeople and sales commission from a company’s personnel record." "[Methodology] For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)." "[Appendix] Problem-focused coping (CI-P) I try to work more efficiently. I devote more time and energy to my job. I decide what I think should be done and explain this to the people who are affected."</t>
+          <t>No effect size of interest. Measures coping strategies rather than boundary spanning behavior.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] The study collected data from multiple sources: survey data from 452 boundary-spanning salespeople and sales commission from a companyâs personnel record." "[Methodology] For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)." "[Appendix] Problem-focused coping (CI-P) I try to work more efficiently. I devote more time and energy to my job. I decide what I think should be done and explain this to the people who are affected."</t>
         </is>
       </c>
     </row>
@@ -25307,7 +25493,7 @@
       </c>
       <c r="P560" t="inlineStr">
         <is>
-          <t>Qualitative/Q-methodology study lacking extractable zero-order effect sizes and measuring cross-boundary tensions rather than boundary spanning behavior.. Verbatim Evidence: [Abstract] "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions." [Step 1: Interviews and Q Statements] "They were asked to respond to questions related to cross-boundary tensions, for example: “What do you believe are the biggest barriers to interaction between project owners and project managers across organizations and stages in the process of achieving project objectives?”" [Step 2: Q Surveys] "Between July and December 2023, 20 participants were invited to rank-order 20 Q statements, presented on cards, in a quasinormal distribution (see Figure 3)."</t>
+          <t>Qualitative/Q-methodology study lacking extractable zero-order effect sizes and measuring cross-boundary tensions rather than boundary spanning behavior.. Verbatim Evidence: [Abstract] "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions." [Step 1: Interviews and Q Statements] "They were asked to respond to questions related to cross-boundary tensions, for example: âWhat do you believe are the biggest barriers to interaction between project owners and project managers across organizations and stages in the process of achieving project objectives?â" [Step 2: Q Surveys] "Between July and December 2023, 20 participants were invited to rank-order 20 Q statements, presented on cards, in a quasinormal distribution (see Figure 3)."</t>
         </is>
       </c>
     </row>
@@ -27392,7 +27578,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate the individual effects of boundary-spanning search from suppliers (supplier-side search (SS)). It is proposed that SS contributes to innovation ambidexterity (IA) and then business performance (BP). Further, this paper includes buyer–supplier relationships (BSRs) and competitive intensity (CI) as moderators to clarify boundary conditions.</t>
@@ -27440,7 +27625,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -27488,7 +27672,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr">
         <is>
           <t>This study utilizes network exploitation and exploration theory to distinguish the exploitative and exploratory mechanisms (government support and boundary-spanning learning, respectively) that convert political ties into firm innovativeness. It also examines the moderating roles market uncertainty plays in how political ties influence firm innovativeness. An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness. Market uncertainty negatively moderates the impact of political ties on boundary-spanning learning but does not significantly moderate their impact on government support. Moreover, market uncertainty moderates the impact of government support on firm innovativeness negatively but moderates the impacts of boundary-spanning learning on firm innovativeness positively. This study theorizes two mediating factors for how firms exploit and explore their political ties to increase their innovativeness and enriches the knowledge of how market uncertainty affects the relationship between political ties and innovation.</t>
@@ -27536,6 +27719,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F619" t="inlineStr"/>
       <c r="G619" t="inlineStr">
         <is>
           <t>Organizational values and beliefs significantly influence employee decision making and behavior and manifest themselves as multiple climates existing within a single organization. A subset of organizational climate is an ethical climate, embodying normative values and beliefs involving moral issues shared by the employees of the organization. Reseachers have found multiple ethical climates present in an organization.</t>
@@ -27583,6 +27767,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F620" t="inlineStr"/>
       <c r="G620" t="inlineStr">
         <is>
           <t>Boundary‐spanning communication has been found to be important to various types of organizations and groups as a source of new information and awareness of environmental changes. Although the importance of formal, public channels in building the knowledge base of a field has long been recognized, most studies of boundary‐spanning activity have been limited to direct, personal (informal) communication. This study examines both informal and formal communication patterns of three groups in order to determine whether, in fact, a variety of media are used in boundary‐spanning communication. The groups selected were the members of three professions which fill intermediary positions between the creators and consumers of cultural products; one located in academia and two in the private sector. Major findings were that: (1) A boundary‐spanning structure linking 82.2% of the survey respondents was composed of both informal and formal media. (2) The professions differed in which type of channel was most heavily used, but were similar in their perceptions of the importance of the channels. (3) Individuals central to the informal part of the structure were also more likely to use the formal parts of the structure. (4) Boundary‐spanning media were among the five most frequently cited media for all three of the professions.</t>
@@ -27630,6 +27815,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>Research-practice partnerships (RPPs) offer promising approaches to improve educational outcomes. Navigating boundaries between contexts is essential for RPP effectiveness, yet much work remains to establish a conceptual framework of boundary spanning in partnerships. Our longitudinal comparative case study draws from our experiences as graduate student boundary spanners in three long-term partnerships to examine boundary spanning roles in RPPs, with particular attention to the ways in which power permeates partnership work. Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums: institutional focus, task orientation, expertise, partnership disposition, and agency. Our roles were shaped by the organizational, cultural, relational, and historical features of the partnerships and contexts of interaction. We aim to promote the development of effective RPP strategies by leveraging the perspectives and positionality of graduate students in order to advance understanding of boundary spanning roles.</t>
@@ -27677,7 +27863,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -28946,7 +29131,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry. Using a multiyear sample of ﬁrms from the computer industry, we found that intra-industry trade-association ties of top managers led to the adoption of a resource-imitation strategy by late movers while extra-industry importation and professional-association ties led to the adoption of a resource-substitution strategy. We also found that trade association ties had a negative effect on the performance of late movers using resource-substitution, while top managers’ service on other ﬁrms’ boards had a positive inﬂuence on the performance of those ﬁrms. Our ﬁndings not only conﬁrm the importance of the role of ﬁt in strategy and performance, but they also highlight the importance of the management and control of boundary-spanning activities.</t>
@@ -29093,6 +29277,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr">
         <is>
           <t>Individuals in work teams frequently cross boundaries across teams, often by using information and communication technologies (ICTs). The current study investigates the effects of members’ boundary work and the visibility affordance of teams’ ICTs on Transactive Memory Systems (TMS) in teams. Survey data from 212 fulltime employees whose work hours were divided between multiple teams reveals that boundary spanning enhances the focal team’s TMS specialization and credibility and negatively inﬂuences TMS coordination. Additionally, boundary reinforcement positively affects TMS credibility and coordination. The visibility affordance has a direct positive effect on all three dimensions of TMS and a moderating effect for boundary reinforcement such that higher visibility overrides the positive direct effect of boundary reinforcement on TMS. These ﬁndings suggest that different types of boundary work contribute to different dimensions of TMS and that teams might consider prioritizing the use of ICTs with high visibility to enhance their TMS.</t>
@@ -29192,7 +29377,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>This study examines how deans and associate deans of a group from similar universities use networking. Specifically, we consider whether the deans, traditionally considered to perform boundary-spanning functions, make more use of external networking than do the associate deans, who are their subordinates. We examine the relationship between accuracy in perceiving a network and influence in the network. Finally, we consider the relationship between reports of networking outside the sample and influence within the sample. We find support for our first two propositions and raise several issues related to our final one.</t>
@@ -29240,6 +29424,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F662" t="inlineStr"/>
       <c r="G662" t="inlineStr">
         <is>
           <t>This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of noncore firms operating in the context of sustainable development. The dynamic nature of technological innovation, exacerbated by market flattening and the challenges posed by the COVID-19 pandemic, has compelled small and medium-sized enterprises (SMEs) to seek innovative breakthroughs. Cooperative innovation emerges as a strategic avenue for SMEs to mitigate risks and enhance their willingness to innovate. However, non-core firms often encounter technological and market disadvantages, hindering innovation efforts. This study explores how boundary-spanning knowledge search, which bridges the gap between non-core firms and the external environment, influences cooperative innovation. Furthermore, the research delves into the mediating role of both potential and actual absorptive capacity in the relationship between boundaryspanning knowledge search and cooperative innovation performance. Empirical findings indicate that boundary-spanning knowledge searches positively impact cooperative innovation, with technological and market knowledge searches yield significant results. Moreover, absorptive capacity exhibits a dual mechanism, directly influencing cooperative innovation and mediating the relationship between knowledge search and performance. This paper extends existing research by focusing on non-core firms within the sustainable development context, offering valuable insights for SMEs seeking innovative strategies. It also highlights the diverse pathways through which boundary-spanning knowledge search affects cooperative innovation. These findings offer practical implications for enhancing non-core firms’ innovation capabilities, including encouraging proactive knowledge search and developing absorptive capacity-inducing mechanisms through employee training and information platforms.</t>
@@ -29287,6 +29472,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F663" t="inlineStr"/>
       <c r="G663" t="inlineStr">
         <is>
           <t>This paper examines the influence of boundary-spanning knowledge search on cooperative innovation performance and explores the moderating role of innovation passion in Chinese firms. We collected 229 valid responses from Chinese firms participating in collaborative innovation projects and applied confirmatory factor analysis to test the reliability and validity of the constructs, multiple stepwise regressions to verify the direct effect, and the PROCESS macro to test the moderating effect. The results show that all three dimensions of boundary-spanning knowledge search (i.e. network capability, IT capability, and absorptive capacity) positively affect cooperative innovation performance. Harmonious innovation passion positively moderates the relationship between network capability and cooperative innovation performance. In contrast, compulsive innovation passion plays a negative moderating role in the relationship between absorptive capacity and cooperative innovation performance. This study further enriches and extends the theoretical framework of cooperative innovation performance by emphasizing the impact of the three dimensions of boundary-spanning knowledge search.</t>
@@ -29334,7 +29520,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -29382,7 +29567,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>Local government or better known as the local authority vested with the power to plan, develop, and regulate businesses in the area within its jurisdiction plays a significant role in creating a conducive environment for businesses to grow and flourish. In playing this role, employees in local authority must possess a certain degree of innovative work behavior. This paper reports on a study that investigated innovative work behavior orientation among employees of the local government. A total of 100 employees of a local city council responded to a self-administered questionnaire on innovative work behavior. The results revealed that respondents scored a moderate high orientation on the innovative work behavior scale.</t>
@@ -29551,6 +29735,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>Due to their complexity and high social impact, urban infrastructure projects often face challenges in managing the design decision-making processes across disparate disciplinary and knowledge domain boundaries. This paper introduces the notion of design boundary dynamics to describe the various cross-boundary coordination phenomena associated with organising the design of infrastructure projects. Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project. Findings illustrate the entangled processes, through which the disciplinary, knowledge-domain and stage-based design boundaries emerged as a result of unfolding project practices. Paper identifies the key role of resource allocation constraints, path dependency of project decisions, and problem-solving nature of design and concludes with strategic recommendations for upstream operational integration to mitigate the impact of design boundary dynamics on infrastructure projects.</t>
@@ -29672,6 +29857,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -29756,7 +29942,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -30599,6 +30784,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F696" t="inlineStr"/>
       <c r="G696" t="inlineStr">
         <is>
           <t>Purpose – Business model innovation (BMI) is an important channel of enterprise innovation, and BMI’s antecedents have attracted extensive attention. The purpose of this paper is to address a substantial gap in the extant literature by developing a moderate model to explain the effects of boundary-spanning search on BMI as well as whether and how innovative cognitive imprinting (ICI) and environmental dynamics (ED) affect the above relationship.</t>
@@ -30646,7 +30832,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>Based on organizational learning theory, the influence of the transactive memory system of the top management team on business model innovation is discussed, as is the impact of different dimensions of boundary-spanning search on different business model innovation attributes when attention distribution is taken into account. Meanwhile, the moderating effects of environmental dynamism are considered. Regression and bootstrap analysis are used to test hypotheses. The results based on empirical research show that the transactive memory system has a positive effect on the dual attributes of business model innovation; acute boundary-spanning search and concentrated boundary-spanning search affect novelty-centered business model innovation and efficiencycentered business model innovation, respectively, and play mediating roles. Meanwhile, environmental dynamism positively moderates the relationship between acute boundary-spanning search and novelty-centered business model innovation, but negatively moderates the relationship between concentrated boundaryspanning and business efficiency-centered model innovation efficiency.</t>
@@ -30793,7 +30978,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
         <is>
           <t>This study adopts a temporal perspective to investigate how boundary spanners can increase the inflow of external knowledge by engaging with both external and internal parties. We add to prior work on knowledge transfer by shifting the focus from engagement levels to investigating engagement dynamics, especially the degree of switching between external and internal engagement across consecutive time periods. Drawing from a cognitive perspective, we argue that switching strongly between engagement types is associated with a segmented knowledge structure that enables quick and efficient categorical processing when knowledge can simply be “channeled” from source to recipient units. In contrast, weak or no switching is associated with a blended knowledge structure and more reflective processing, which is particularly helpful when knowledge transfer requires more translation and transformation. Correspondingly, we adopt a contingency perspective and theorize that the cognitive advantages associated with stronger versus weaker switching weigh differently, contingent on the stickiness of knowledge to be transferred and the nature of boundary-spanning activities that vary in importance over time. Fixed effects models of eight waves of original survey data reveal that, in line with our theorizing, the association between switching and knowledge transfer becomes increasingly negative (1) the more boundary spanners access knowledge that is transspecialist in nature, (2) the greater the organizational distance between source and recipient units, and (3) in later phases of the boundary-spanning process.</t>
@@ -30878,7 +31062,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>
@@ -30973,6 +31156,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 14
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -5741,7 +5741,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Getting professionals who have been selected and trained to perform individually to work together is a major challenge. The objective of the article is to identify the mechanisms by which a coordinator can ensure a mediation and boundary spanning role to enable the achievement of a project. Adopting a comprehensive approach, this article is based on the case of an innovative hospital project ‘One-Day Diagnosis’ (1DD) – one day instead of several weeks – of hepatobiliary and pancreatic pathologies, for which the professionals had to change their practices. Based on the results of the study, the ﬁndings show that the mediating role of the coordinator consists in making things happen and guiding health care professionals through the innovative pathway until it becomes a routine process. The study contributes to the literature on collaboration and relational coordination by highlighting that the change of practices for collaboration is compatible with personal excellence, by outlining the active role of the boundary spanner in the change of these practices and by demonstrating that the organizational stability of projects based on disembodied procedures is a necessary illusion that requires complementary interindividual relationships and a living leadership.</t>
@@ -5789,7 +5788,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>The current study examined the relationships among role stress, proactive personality, employee creativity, and customer-oriented boundary spanning behaviors (COBSBs) for frontline service employees (FSEs). This study collected data from 382 FSEs in international hotels in Taiwan to test the research model. The empirical results revealed that employee creativity was positively affected by proactive personality but negatively affected by role conflict and role ambiguity. FSEs’ creativity positively affects COBSBs, including external representation, internal influence, and service delivery. Internal influence also positively affects service delivery and mediates the relationship between FSEs’ creativity and service delivery.</t>
@@ -5936,7 +5934,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>This dissertation examined the relationships between organizational characteristics and firms' timing of entry into emerging product markets. This study is an extension of a stream of research on endogenous entry models. Research on this area essentially holds that not all firms have the same entry skills and costs. Therefore, a firm's entry timing decision is attributable to factors internal to the organization. In this dissertation, specific attention is directed toward the effects of top management team (TMT) demography, corporate governance, level of diversification, boundary spanning, past performance, capital structure, and firm size on entry timing. These organizational characteristics have been shown to be critical determinants of timing in the strategic management literature, but, remain almost unexplored in the entry timing research. Thus, through including these organizational characteristics, this study extends the current knowledge which is critical for answering the question: Why do some firms enter emerging product markets earlier/later than others?</t>
@@ -5984,7 +5981,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>Organisations experience increased social, political and economic pressure that is evident in the increased pressure that stakeholders place on organisations. Organisations increasingly realise that stakeholders’ values and objectives need to be incorporated into organisational strategy as well as the day-to-day management of the organisation. Organisational success and survival consequently depends on the organisation’s network of relationships, which provide the organisation with otherwise inaccessible resources and a competitive advantage.</t>
@@ -6032,7 +6028,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>In this dissertation, I develop a conceptual model for how managers' roles as boundary spanners within their organizations affect the perceptions, attitudes, relationships, and performance of their subordinate employees. Drawing on literatures in social networks, status characteristics theory, social identity theory, and resource allocation theory, I suggest that managers' external relationships—the connections that managers make to organization members outside of their subordinate work group—have a material impact on their subordinates' perceptions of their work environment and their managers. These perceptions, I argue, serve as four specific mechanisms in an indirect effects model that connect managers' external relationship to their employees' task performance and work attitudes (eg organizational commitment) and the Leader Member Exchange (LMX) relationships between manager and subordinate. I apply the theoretical model to two salient types of managerial relationships: those with their bosses and those with their horizontal peers.</t>
@@ -6080,7 +6075,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -6128,7 +6122,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>The state of software development performance is far from being exemplar, with a success rate well below that of other industries, and understanding how to improve these projects is not only substantive but urgent. Software development is at most times a collaborative effort, yet we do not understand clearly how different collaboration structures associate with development performance metrics. This paper empirically examines the association between collaboration patterns, project productivity and product quality through a field study of working software open source new product development teams, using archival data from electronic sources related to Open Source Software projects. Collaboration structures are measured using Social Network Analysis and in terms of their network density, network centralization and the level of boundary spanning activity of team members. Productivity and quality are measured using "hard", code-based metrics. Results of regression analyses testing relevant hypotheses suggest that project managers need to strongly encourage internal collaboration, but be wary of allowing team members to participate in multiple projects. The breadth of skills within the team is a tactical asset that may increase the efficient frontier in the quality–productivity trade-off. Results also show that centralized structures associate with higher product quality and development productivity.</t>
@@ -6176,7 +6169,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Technology Transfer Centres (TTCs) have been analyzed in the last few years by focusing on the relationship between a TTC, provider of knowledge-intensive services, and a ﬁrm client-receiver. Less attention has been devoted to a more complex relationship which involves in the dyadic provider-receiver tie a third relevant body, University. We provide both a theoretical and an empirical contribution by studying whether TTCs can bond the academic and industrial system and we deﬁne the activities that make-up this role such as: scanning and selection of R&amp;D opportunities, bridge building, semantic translation of domain speciﬁc knowledge, co-production of new knowledge. The boundary spanning role of TTCs is discussed drawing on different and complementary theoretical perspectives. Moreover, we test research hypotheses on the antecedents of boundary spanning activity from a knowledge-based perspective. We argue that TTC boundary spanners need to leverage on both technical skills and networking competences. Empirical investigation has been carried out with a survey of the TTC population of North East Italy. The research ﬁndings highlight the task coordination activities implied by a boundary spanning role in joint R&amp;D projects and show that the endowment of human capital at individual level and a qualiﬁed social capital at individual and organizational level are the main determinants.</t>
@@ -6323,7 +6315,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>This cross-sectional study (conducted in April–May 2011) explored associations between partnership functioning synergy and sustainability of innovative programmes in community care. The study sample consisted of 106 professionals (of 244 individuals contacted) participating in 21 partnerships that implemented different innovative community care programmes in Rotterdam, The Netherlands. Partnership functioning was evaluated by assessing leadership, resources administration and efﬁciency. Synergy was considered the proximal outcome of partnership functioning, which, in turn, inﬂuenced the achievement of programme sustainability. On a 5-point scale of increasing sustainability, mean sustainability scores ranged from 1.9 to 4.9. The results of the regression analysis demonstrated that sustainability was positively inﬂuenced by leadership (standardised regression coefﬁcient b = 0.32; P &lt; 0.001) and non-ﬁnancial resources (b = 0.25; P = 0.008). No signiﬁcant relationship was found between administration or efﬁciency and programme sustainability. Partnership synergy acted as a mediator for partnership functioning and signiﬁcantly affected sustainability (b = 0.39; P &lt; 0.001). These ﬁndings suggest that the sustainability of innovative programmes in community care is achieved more readily when synergy is created between partners. Synergy was more likely to emerge with boundaryspanning leaders, who understood and appreciated partners’ different perspectives, and could bridge their diverse cultures and were comfortable sharing ideas, resources and power. In addition, the acknowledgement of and ability to use members’ resources were found to be valuable in engaging partners’ involvement and achieving synergy in community care partnerships.</t>
@@ -6705,7 +6696,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>The perspectives of transaction cost economics and the resource-based view of the firm have been used extensively to understand the implications of outsourcing. However, transaction cost economics does not explain how a firm will evolve as it progressively outsources internal functions, and the resource-based view does not operationalize the unspecified competences that will be required over time. On the other hand, the lens of paradox highlights the increased expediency and complexity that outsourcing firms are expected to encounter. In this paper, paradoxes comparing operational expediency gains to increases in management, learning and strategic complexity are discussed, leading to the proposal that often unintended replacement behaviors manifest as extensive boundary spanning and new firm-level competencies are necessary to manage these paradoxes and maintain competitive advantage. In extremum tests of these propositions are provided to demonstrate that the complexity of outsourcing intangibles is informed by a lens of paradox.</t>
@@ -6988,7 +6978,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore how and why employees perceive technology-mediated interruptions differently and the role of sociocultural factors in this process using sociomaterial analysis. Design/methodology/approach – Data were gathered from 34 Sri Lankan knowledge workers using a series of workshop-based activities. The concept of sociomateriality is employed to understand how sociocultural elements are entangled with technology in work-life boundary experiences.</t>
@@ -7224,7 +7213,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -7370,7 +7358,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -7559,7 +7546,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing. Informing teams remain relatively isolated from their environment; parading teams have high levels of passive observation of the environment; and probing teams actively engage outsiders. Probing teams revise their knowledge of the environment through external contact, initiate programs with outsiders, and promote their team's achievements within their organization. In this study, they were rated as the highest performers among the teams, although member satisfaction and cohesiveness suffered in the short run. Results suggested that external activities are better predictors of team performance than internal group processes for teams facing external dependence.</t>
@@ -9692,7 +9678,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>The digital era is radically changing our societies and how ﬁrms do business. Innovating the business model has become a fundamental capability to survive competition, particularly for small and mediumsized enterprises (SMEs). This study investigates the digital-era role of boundary management capabilities in the processes of Business Model Innovation (BMI) in SMEs. Structural Equation Modelling is adopted to analyse data from a survey of 250 Italian experts who possess direct research and consulting experience with SMEs. Our ﬁndings reveal that digitalisation and ﬁrms’ boundaries aﬀect BMI in SMEs. Moreover, our results demonstrate how boundary management, speciﬁcally its technological and relational aspects, directly impacts BMI and mediates the relationship between boundary size and BMI. The study also oﬀers important theoretical and practical insights, calling on scholars and managers to give more attention to the boundary management of SMEs in order to support BMI.</t>
@@ -9834,7 +9819,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>In this study we examine the impact of market orientation of leaders on their leader-member exchange (IMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the exist five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.</t>
@@ -9882,7 +9866,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>We examine the extent to which executives' boundary spanning relations inside and outside their industry affect organizational strategy and performance. We posit that the informational and social influences of external ties will be reflected in the degree to which the organization's strategy conforms to or deviates from the central tendencies of its industry and that the alignment of executives' external ties with the firm's strategy will be beneficial to firm performance. Using a multiyear sample of firms in the branded foods and computer industries, we find that executives' intraindustry ties are related to strategic conformity, that extraindustry ties are associated with the adoption of deviant strategies, and that alignment of executives' external ties with the informational requirements of the firm's strategy enhances organizational performance. Our results also show that a unique or differentiated strategy is not universally advantageous and that the benefits accruing from strategic conformity are especially strong in the more uncertain computer industry.</t>
@@ -9930,7 +9913,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>The relationship between external communication and R&amp;D team creativity has received increasing attention in the R&amp;D management literature. However, little is known about the motivational mechanism between the two. We propose a second‐stage moderation model based on social cognitive theory to explain whether, how and when R&amp;D team’s external developmental feedback motivates its creativity. Using the data gathered from 452 R&amp;D team members and 84 supervisors in a time‐lagged field study, we found external developmental feedback had a positive effect on R&amp;D team creativity via increasing team creative efficacy. Further, conditional indirect effect analyses found that a high level of cooperative goal interdependence strengthened the positive effect of team creative efficacy on R&amp;D team creativity and the mediating effect of team creative efficacy between external developmental feedback and R&amp;D team creativity.</t>
@@ -9978,7 +9960,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -10073,7 +10054,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Even though, over the last two decades, the boundaryless career concept has stimulated a wide theoretical debate, scholars have recently claimed that research on the competencies that are necessary for managing a cross-boundary career is still incomplete. Similarly, the literature on emotional and social competencies has demonstrated how they predict work performance across industries and jobs but has neglected their inﬂuence in explaining the individual’s mobility across boundaries and their impact on career success. This study aims to ﬁll these gaps by examining the effects of emotional and social competencies on boundaryless career and on objective career success. By analyzing a sample of 142 managers over a period of 8 years, we found evidence that emotional competencies positively inﬂuence the propensity of an individual to undertake physical career mobility and that career advancements are related to the possession of social competencies and depend on the adoption of boundaryless career paths. This study also provides a contribution in terms of the evaluation of the emotional and social competencies demonstrated by an individual and of the operationalization of the measurement of boundaryless career paths, considering three facets of the physical mobility construct (organizational, industrial, and geographical boundaries).</t>
@@ -10168,7 +10148,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>To explain how multistakeholder groups organize democratic deliberations about complex sustainability issues, organizational scholars have focused on the key role of deliberative capacity, which encompasses the dimensions of inclusiveness, authenticity and consequentiality. However, the tensions inherent to the search of these three dimensions have been overlooked. In this paper, we argue that focusing on how spaces for deliberation are designed can help one understand how to manage such tensions. We identified the boundary work practices that shape the design of deliberative spaces and generate deliberative capacity properties in a high-level expert group (HLEG) launched by the European Commission about sustainable finance regulation. Our results show how these boundary work practices help balance deliberative tensions. We advance deliberation studies by conceptualizing deliberative boundary work, explaining how deliberative capacity is spatially generated and showing how deliberative tensions are balanced. We also contribute to boundary work theory by making explicit the deliberative nature of configuring boundary work and showing its relevancy to regulatory settings.</t>
@@ -10310,7 +10289,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -10437,6 +10415,12 @@
           <t>BSMA0188</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>This paper investigates boundary-work in management accounting in the context of globalization and hybrid professionalism. The paper demonstrates how permeable symbolic boundaries of the management accounting ﬁeld can be altered by employing expansion boundary-work. Contrasting boundary-work of IMA ofﬁcials and IMA members in Russia, we show that IMA ofﬁcials employ primarily monopolization boundary-work while IMA members employ primarily expansion boundary-work. Our ﬁndings illustrate how boundary-work is employed to exhibit organizational and occupational professionalism in the symbolic realm. The paper provides additional insight into the discursive domain of the accounting profession by linking boundary-work to globalization, two forms of professionalism, legitimacy, status and professional identity. This suggests that the professionalization process is inﬂuenced by the properties of professional boundaries.</t>
@@ -10460,6 +10444,11 @@
       <c r="K191" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10511,6 +10500,12 @@
           <t>BSMA0190</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>Past research has studied how the selection and use of control portfolios in software projects is based on environmental and task characteristics. However, little research has examined the consequences of control mode choices on project performance. This paper reports on a study that addresses this issue in the context of outsourced software projects. In addition, we propose that boundary-spanning activities between the vendor and the client enable knowledge sharing across organizational and knowledge domain boundaries. This is expected to lead to facilitation of control through specific incentives and performance norms that are suited to client needs as well as the vendor context. Therefore, we argue that boundary spanning between the vendor and client moderates the relationship between formal controls instituted by the vendor on the development team and project performance. We also hypothesize the effect of collaboration as a clan control on project performance. We examine project performance in terms of software quality and project efficiency. The research model is empirically tested in the Indian software industry setting on a sample of 96 projects. The results suggest that formal and informal control modes have a significant impact on software project outcomes, but need to be finely tuned and directed toward appropriate objectives. In addition, boundary-spanning activities significantly improve the effectiveness of formal controls. Finally, we find that collaborative culture has provided mixed benefits by enhancing quality but reducing efficiency.</t>
@@ -10534,6 +10529,11 @@
       <c r="K193" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10770,6 +10770,12 @@
           <t>BSMA0197</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>As employees’ personal lives are increasingly splintered by work demands, the boundary between work and nonwork domains is becoming ever more blurred. Grounded within a self-regulatory approach and the executive control function of inhibitory control, we operationalize and examine nonwork role re-engagement (NWRR)—the extent to which individuals can redirect attentional resources back to nonwork tasks following work-related intrusions. In phases 1 and 2, we develop and refine a psychometrically sound unidimensional measure for NWRR aligned with the self-regulatory processes of self-control and interference control underlying inhibitory control. In phase 3, we confirm the factor structure with a new sample. In phase 4 we validate the measure using the samples from phases 2 and 3 to provide evidence of criterion-related, convergent, and discriminant validity. NWRR was related to important well-being and work-related outcomes above and beyond existing self-regulatory and boundary management constructs. We offer theoretical and practical implications and an agenda to guide future research, as attentional agility becomes increasingly relevant in a home life replete with interruptions from work.</t>
@@ -10793,6 +10799,11 @@
       <c r="K200" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10812,7 +10823,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>T h i s position paper distinguishes different types of activities needed in software processes and proposes enaction support for t h e m . An architecture of enaction components providing this support is sketched.</t>
@@ -10855,6 +10865,12 @@
           <t>BSMA0199</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>This article guides the development of creative insights in supply chain management. The authors begin by describing analogies’ role in advancing organization theory with a focus on image transfers between knowledge domains. While much has been said about the merits of conceptual transfers between domains, much equally remains unknown, particularly about how to deliberately develop creative insights that have the potential to challenge or enhance existing supply chain management theory. To address this issue, this research builds on prior work on analogies, creativity, and design thinking to develop a heuristic-analytic model. This model is designed to assist researchers in theorizing by analogy through a controlled dual cognitive process of divergence before convergence combined with a distant boundary-spanning knowledge search. An illustration of the model shows how creative output can provide a fresh perspective that helps render supply chains potentially more resilient.</t>
@@ -10878,6 +10894,11 @@
       <c r="K202" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10892,6 +10913,12 @@
           <t>BSMA0200</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>The period after completing primary and adjuvant cancer treatment until recurrence or death is now recognized as a unique phase in the cancer control continuum. The term “survivorship” has been adopted to connote this phase. Survivorship is a time of transition: Issues related to diagnosis and treatment diminish in importance, and concerns related to long-term follow-up care, management of late effects, rehabilitation, and health promotion predominate. In this article, we explore the unique challenges of care and health service delivery in terms of the interface between primary care and specialist care during the survivorship period. The research literature points to problems of communication between primary and specialist providers, as well as lack of clarity about the respective roles of different members of the health-care team. Survivorship care plans are recommended as an important tool to facilitate communication and allocation of responsibility during the transition from active treatment to survivorship. Research questions that remain to be answered with respect to survivorship care plans and other aspects of survivorship care are discussed.</t>
@@ -10915,6 +10942,11 @@
       <c r="K203" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10929,6 +10961,12 @@
           <t>BSMA0201</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>In multidisciplinary teams in the oil and gas industry, we examined expertise diversity's relationship with team learning and team performance under varying levels of collective team identification. In teams with low collective identification, expertise diversity was negatively related to team learning and performance; where team identification was high, those relationships were positive. Results also supported nonlinear relationships between expertise diversity and both team learning and performance. Finally, team learning partially mediated the linear and nonlinear relationships between diversity and performance. Findings broaden understanding of the process by which and the conditions under which expertise diversity may promote team performance.</t>
@@ -10952,6 +10990,11 @@
       <c r="K204" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11341,7 +11384,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Innovation is considered the engine for firm growth. Especially innovations, through recombining seemingly unrelated knowledge streams, can have groundbreaking impact and lead to sustained competitive advantage. To generate such innovation, firms often need to go beyond their existing technological or geographical boundaries to identify and integrate novel knowledge elements. This article refers to firms’ knowledge activities of drawing upon distant knowledge (i.e., knowledge from dissimilar technological domains or distant geographical regions) to create novel technological solutions, as innovation through boundary spanning. Aiming to investigate the roles of information technology (IT) in facilitating innovation through boundary spanning, we collected data from the pharmaceutical industry over a six-year period to test the research model. The data analysis results indicate that IT supports boundary-spanning activities in firm innovation and different IT-enabled knowledge capabilities affect boundary-spanning innovation differently.</t>
@@ -11384,6 +11426,16 @@
           <t>BSMA0213</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G216" t="inlineStr">
         <is>
           <t>Purpose – The current article investigates the impact of generational diversity on knowledge sharing and group performance. It, further, explores the moderating effects of intergenerational climate, boundaryspanning leadership, and respect in facilitating greater knowledge sharing and enhanced group performance. Design/methodology/approach – The authors applied partial least square structural equation modeling to test the model, using a sample of 635 employees working in the banking industry.</t>
@@ -11407,6 +11459,11 @@
       <c r="K216" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Exclude under Code 5 [Code 1 &amp; Code 3]. The BSL construct measures internal demographic diversity management (inclusive leadership) rather than structural BSB, and the study assigns branch-level constructs (Blau's index) to individual employees, violating statistical independence.. Verbatim Evidence: [Measures] "Boundary-spanning leadership refers to an employee’s perception about whether his leader is engaged in boundary-spanning behaviors or not." [Measures] "Boundary-spanning leadership was measured using a three-item scale adopted from the Intergroup Rhetoric Scale by Rast (2013)." [Literature review] "Leaders who equally interact, spend time, and share their expertise with members of different groups help bridge the divide among groups and enable inter-group collaboration." [Abstract] "The authors applied partial least square structural equation modeling to test the model, using a sample of 635 employees working in the banking industry." [Measures] "Generational diversity was measured using Blau’s (1977) index of heterogeneity (1 Pρi 2), where ρ was the proportion of group members in a category, and i was the number of different categories represented on a group." [Measures] "Branch performance from employees and branch managers was measured using a four-item scale developed by Chow and Chan (2008)."</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11483,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -11469,6 +11525,16 @@
           <t>BSMA0215</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G218" t="inlineStr">
         <is>
           <t>This project provides an interpretation of how one cooperative support organization, the Nebraska Cooperative Council, discursively functions to help its constituent cooperatives consolidate resources in order to better intersect with organizations in a larger bureaucratic system. In analyzing qualitative data collected through in-depth interviews, surveys, and organizational documents, we found the paradox of stability and change a revealing prism through which to make sense of participants’ experiences. We work toward locating and describing how the Council, through its boundary-spanning activities, helps cooperatives manage the paradox of stability and change while protecting their core participatory ideologies. By providing networks of learning, promoting the legitimacy of cooperative forms of organizing, and protecting cooperatives’ interests, the Council is an entity helping cooperatives to reconcile their internal requirements for democracy with the external demands of the marketplace.</t>
@@ -11492,6 +11558,11 @@
       <c r="K218" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Qualitative study without quantitative effect sizes (thematic analysis of discourse).. Verbatim Evidence: [Abstract] In analyzing qualitative data collected through in-depth interviews, surveys, and organizational documents, we found the paradox of stability and change a revealing prism through which to make sense of participants’ experiences. [Procedures] A thematic analysis of the discourse collected through in-depth interviews, survey questionnaires, and organizational documents was conducted using the constant comparative method (Lindlof, 1995).</t>
         </is>
       </c>
     </row>
@@ -11506,6 +11577,16 @@
           <t>BSMA0216</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G219" t="inlineStr">
         <is>
           <t>Work teams must increasingly operate in complex environments characterized by multiple external actors beyond team and organizational boundaries. Although previous research demonstrates the importance of boundary spanning activities to team effectiveness, it reveals relatively little about the process of boundary spanning in these environments. In this article, we investigated the processes of boundary spanning across multiple external actors in 10 cross-organizational teams. We identified three sequences for reaching out to external actors: (a) moving inside-out from vertical actors inside the host organization to horizontal actors outside of the host organization, (b) moving outside-in from horizontal actors to vertical, and (c) staying-inside with vertical actors from the host organization. Our observations suggest that inside-out and outside-in sequences were more successful than simply pleasing the host organization. We build on our empirical findings to develop a process theory of how team boundary spanning activities across multiple external actors influence team effectiveness. Our research underscores the importance of a team’s interactions with actors in its external environment beyond those in an immediate supervisory role and provides insight into the dynamics of boundary spanning in multi-organizational contexts.</t>
@@ -11529,6 +11610,11 @@
       <c r="K219" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Qualitative case study lacking quantitative effect sizes, and the unit of analysis is the team.. Verbatim Evidence: [Qualitative study without effect size and team-level unit of analysis]. Verbatim Evidence: "[Abstract] In this article, we investigated the processes of boundary spanning across multiple external actors in 10 cross-organizational teams." "[Method] Following other researchers who are interested in organizational processes (e.g., Anand, Gardner, &amp; Morris, 2007; Bresman, 2013; Nag &amp; Gioia, 2012), we combined a case study approach with grounded theory methodology (Langley, 1999)." "[Unit of analysis] Our unit of analysis was the COT, and specifically, the initial five non-repeating boundary spanning activities in the sequence of a COT’s boundary spanning process."</t>
         </is>
       </c>
     </row>
@@ -11543,6 +11629,16 @@
           <t>BSMA0217</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G220" t="inlineStr">
         <is>
           <t>The paper explains the effects of internal and external team learning behaviors on the performance of marketing teams. The survey was conducted in the context of a multinational Pharmaceutical Corporation marketing its products in Turkey. Data were collected from members of marketing team which included medical sales representatives, specialized medical sales representatives and districts heads of marketing. The results indicate that both the internal team learning and the external team learning behaviors play significant roles in ensuring the success of marketing teams in continuously identifying, anticipating and satisfying the customer requirements profitably through an efficient deployment of the marketing teams’ resources.</t>
@@ -11566,6 +11662,11 @@
       <c r="K220" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Team-level construct (survey referent is the group/team). Verbatim Evidence: [Participants] "The survey involved all the 90 members of the marketing team. 49 out of 90 members returned the questionnaire yielding a response rate of 54%." [Measures] "1. Group members go out and get all the relevant work information they possibly can from others –such as customers, or other parts of the organization. 2. My group keeps others in the organization informed about what we plan and accomplish. 3. We invite people from outside the group to present information or have discussions with us."</t>
         </is>
       </c>
     </row>
@@ -11992,7 +12093,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>Scholarship in the field of health communication is broad, with interdisciplinary contributions from researchers trained in a variety of fields including communication, nursing, medicine, pharmacy, public health, and social work. In this paper, we explore the role of “health communication boundary spanners” (HCBS), individuals whose scholarly work and academic appointment reflect dual citizenship in both the communication discipline and the health professions or public health. Using a process of critical reflective inquiry, we elucidate opportunities and challenges associated with HCBS across the spectrum of health communication in order to provide guidance for individuals pursuing boundary spanning roles and those who supervise and mentor them. This dual citizen role suggests that HCBS have unique skills, identities, perspectives, and practices that contribute new ways of being and knowing that transcend traditional disciplinary boundaries. The health communication field is evolving in response to the need to address significant healthcare and policy problems. No one discipline has the ability to single-handedly fix our current healthcare systems. Narrative data from this study illustrate the importance of seeing HCBS work beyond simply being informed by disciplinary knowledge. Rather, we suggest that adapting ways of knowing and definitions of expertise is an integral part of the solution to solving persistent health problems.</t>
@@ -12144,7 +12244,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>Following the resource-advantage theory, this study advances the existing research of boundaryspanning search by examining which configuration of a new venture’s boundary-spanning search can obtain successful venture performance and how a founding team’s external relationship and the internal firm competences shape the relationship between the distant search and new venture performance. This paper is based on a questionnaire survey/analysis of a sample of 178 new ventures from China, and it offers insight to entrepreneurs with regard to the importance of building external managerial ties and developing idiosyncratic internal competences on boundary-spanning search. In addition, this study also reveals that the effectiveness of the supply-side, demand-side and spatialside boundary-spanning search on venture performance depends on investing resource at a rational level.</t>
@@ -12192,7 +12291,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>Information system development can be considered a collaboration between users and developers. The inability to leverage the localized knowledge embedded in these two stakeholders hinders software development work to achieve high performance. Exploring the ways to counter this difﬁculty is then critical. This study applies an intellectual capital perspective to address the issues around spanning the knowledge boundary between developers and users. Our ﬁndings highlighted how important effective knowledge boundary spanning is to both product and project quality. Furthermore, three dimensions of intellectual capital increased the degree to which knowledge boundary spanning was effective.</t>
@@ -12240,7 +12338,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>There appears to be a consensus that organizational integration across functional and disciplinary specialties drives superior ﬁrm capabilities. The basic assumption is that new practices and concepts emerge from the interaction of individuals engaged in different functional departments. However, communication across functional boundaries is often difﬁcult. As such, Tushman &amp; Scanlan suggested that functional boundaries can be spanned effectively only by boundary spanners who understand the coding schemes that are attuned to the contextual information on both sides of the boundary. The study of boundary spanners has signiﬁcant performance implications to ﬁrms. Compared to its importance, theoretical development and empirical inquiries into this phenomenon are relatively scant. Thus, this study explores the factors that determine who becomes a boundary spanner and examines boundary spanners’ performance implications. A Taiwanese company provided the context for our study. Partial Least Squares (PLS) was used to test the theoretical model. The results imply that a company needs to have an appropriate mixture of boundary spanners and non-boundary spanners, because boundary spanners have higher innovative performance.</t>
@@ -12288,7 +12385,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate three issues: how does an innovative search (local search and boundary-spanning search) impact ﬁrm innovation performance of latecomers; how does capability reconﬁguration (capability evolution and capability substitution) mediates the relationship between innovative search and ﬁrm innovation performance; and how does the technological leapfrogging process (initial stage, following stage, synchronization stage and leading stage) moderate the relationship between capability reconﬁguration and ﬁrm innovation performance.</t>
@@ -12331,6 +12427,12 @@
           <t>BSMA0236</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>This study examines personal ties between boundary-spanning personnel in interorganizational exchanges in emerging markets. Drawing on social embeddedness theory and boundary spanning theory, we propose that strong ties between boundary spanners may benefit exchange parties in their interorganizational relationships through two heightened boundary-spanning behaviors—information processing and external representation. The results from 225 manufacturer–distributor dyads in China indicate that interpersonal ties at the higher levels (between top executives) and at the lower levels (between salespersons and individual buyers) are both positively associated with relationship quality of the buyer–supplier relationship through dyadic boundary-spanning behaviors. Between two levels of interpersonal ties, ties at the lower levels exhibit a stronger association with relationship quality than do ties at the higher levels. Furthermore, the positive effects of interpersonal ties on conflict resolution and cooperation are amplified when both levels of ties are strong in the focal relationship.</t>
@@ -12354,6 +12456,11 @@
       <c r="K239" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12373,7 +12480,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Boundary‐spanning personnel such as tax preparers, travel agents and hairdressers interface directly with customers. In their unique position, between the organization and customer, these service providers market the service to consumers while they simultaneously carry out operational functions. Both the customer and the provider bring certain expectations to the service encounter. These expectations then shape the perceptions of the service encounter. The research reported uses script methodology to compare the expectations between boundary‐spanning service providers and consumers of the same service. Draws its theoretical foundation from the expectations and scripts literatures. In Phase One, scripts of the service were elicited in order to test hypotheses based on the discovery and comparison of consumers′ and service providers′ subgoals for a typical service encounter (               H1               ). A hypothesis also tested the point at which providers and consumers enter their respective scripts of a typical service encounter (               H2               ). In Phase Two, the subgoals mentioned most frequently in Phase One were used as stimuli to elicit the specific actions which comprise the complete script. These complete scripts enabled a comparison of the elaborateness of provider and consumer scripts (               H3               ). The results of Phase One revealed that a portion of consumers′ subgoals for a service encounter are shared by providers of the service while other subgoals are unique, supporting               H1               . The point of activation of the script differed dramatically between customers and providers, supporting               H2               . The Phase Two findings provide support for the hypothesis that service providers have more elaborate scripts. Overall, the results support the notion that scripts operationalize expectations. Closes with implications for management and suggestions for future research.</t>
@@ -12421,7 +12527,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to explore how integration teams can build trusting relationships in component teams to enhance their leadership capability within multiteam systems to achieve common superordinate goals. The study investigates how an integration team diagnoses contextual dynamics to enhance understanding of goals in component teams and spans boundaries to create trusting relationships.</t>
@@ -12521,7 +12626,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>While there is a growing interest in the role of market information processing activities (i.e., the acquisition, dissemination, and use of market information) in new product development (NPD), a number of gaps remain in our knowledge on this topic. When investigating the performance impact of market information processing, most studies have treated the three activities as independent. Our research adds to the extant knowledge by exploring not only both direct relationships between each of the market information processing activities and new product performance, but also interaction effects. We, thus, ask the question of whether there may be synergies in obtaining performance increases by jointly improving two processing activities, rather than just considering each activity independently. In addition, we investigate these effects for different levels of information quality; a topic largely neglected in the market information processing literature. Our analysis is based on empirical data from 152 Dutch NPD projects. The results indicate that market information acquisition and use are both directly associated with increased performance. We also ﬁnd signiﬁcant interaction effects for information acquisition and dissemination, and for information dissemination and use. Finally, the importance of information quality is emphasized, with lower quality information producing lower performance and wiping out the effects between various aspects of market information processing and new product performance. We provide several implications of our ﬁndings for managers and academics.</t>
@@ -12569,7 +12673,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>Background: Rehabilitation services depend on competent professionals who collaborate effectively. Wellfunctioning interprofessional teams are expected to positively impact continuity of care. Key factors in continuity of care are communication and collaboration among health care professionals in a team and their patients. This study assessed the associations between team functioning and patient-reported benefits and continuity of care in somatic rehabilitation centres. Methods: This prospective cohort study uses survey data from 984 patients and from health care professionals in 15 teams in seven somatic rehabilitation centres in Western Norway. Linear mixed effect models were used to investigate associations between the interprofessional team communication and relationship scores (measured by the Relational Coordination [RC] Survey and patient-reported benefit and personal-, team- and cross-boundary continuity of care. Patient-reported continuity of care was measured using the Norwegian version of the Nijmegen Continuity Questionnaire. Results: The mean communication score for healthcare teams was 3.9 (standard deviation [SD] = 0.63, 95% confidence interval [CI] = 3.78, 4.00), and the mean relationship score was 4.1 (SD = 0.56, 95% CI = 3.97, 4.18). Communication scores in rehabilitation teams varied from 3.4–4.3 and relationship scores from 3.6–4.5. Patients treated by teams with higher relationship scores experienced better continuity between health care professionals in the team at the rehabilitation centre (b = 0.36, 95% CI = 0.05, 0.68; p = 0.024). There was a positive association between RC communication in the team the patient was treated by and patient-reported activities of daily living benefit score; all other associations between RC scores and rehabilitation benefit scores were not significant. Conclusion: Team function is associated with better patient-reported continuity of care and higher ADL-benefit scores among patients after rehabilitation. These findings indicate that interprofessional teams’ RC scores may predict rehabilitation outcomes, but further studies are needed before RC scores can be used as a quality indicator in somatic rehabilitation.</t>
@@ -12716,6 +12819,12 @@
           <t>BSMA0244</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>This three-essay project explores boundary management and work-nonwork enrichment to explain how thriving in the work domain relates to thriving in the nonwork domain. The Cross-Domain Thriving model proposed in Study 1 theorizes that when employees experience growth and energy at work, they create and deplete resources within and across roles and individual boundary management strategies, role congruency, and ease of transition moderate the degree to which thriving translates into enrichment and/or conflict across roles. Study 2 tested aspects of the cross-domain thriving model and found that neither work nor nonwork thriving was related to increased time-based conflict, but both forms of thriving predicted enrichment gains across domains. Moreover, higher levels of work-nonwork role segmentation were associated with a stronger relationship between learning in nonwork roles and affective and efficiency enrichment gains in the nonwork-to-work direction. In the work-to-nonwork direction, role congruency and cycling boundary management behavior were related to greater developmental and affective enrichment, respectively. Cycling also strengthened the positive relationship between vitality at work and work-to-nonwork capital enrichment. Study 3, a qualitative study investigating work and nonwork thriving in employees working from home during a pandemic, suggested the importance of boundary management skills as demands on learning and energy increase. Findings highlight how key employer actions and employee regulatory behavior can leverage the benefits of growth and energy in work and nonwork domains.</t>
@@ -12739,6 +12848,11 @@
       <c r="K247" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12753,6 +12867,12 @@
           <t>BSMA0245</t>
         </is>
       </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>Community-based initiatives (CBIs) are thriving in Western countries. In CBIs, citizens take a leading role in providing public services and goods. CBIs have been acclaimed for their innovativeness, problem-solving capacity, and legitimacy. However, we lack large N studies on performance of CBIs and its antecedents. This article develops and tests a model that identiﬁes relationships between performance and four antecedents by using survey data on CBIs collected in the Netherlands (N = 671). Using structural equation modelling, positive direct and indirect relationships between transformational leadership, boundary spanning leadership, organizational capacity, social capital ties, government support, and performance are found.</t>
@@ -12776,6 +12896,11 @@
       <c r="K248" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12790,6 +12915,12 @@
           <t>BSMA0246</t>
         </is>
       </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>The study examines the effects of the individual characteristics, job type, role stressors, boundary spanning activities, career outcomes, and job characteristics on the turnover propensity of 464 information systems personnel. Results show that age, organizational level, organizational tenure, job tenure, and number of years in the computer field are negatively correlated with the intention to leave the organization. Education was found to be positively correlated with turnover intentions, and while project leaders are more likely to leave the organization, IS managers are less likely. Results also show that both role stressors (role ambiguity and role conflict) and boundary spanning activities are positively correlated with turnover intentions, and that job involvement, career plateau, promotability, salary, organizational commitment, job satisfaction, satisfaction with progress, promotion, pay, status, and projects are negatively correlated while career opportunity is positively correlated with turnover intentions. Finally, all job characteristics are negatively correlated with turnover intentions. Implications of the results for practice and research are offered.</t>
@@ -12813,6 +12944,11 @@
       <c r="K249" t="inlineStr">
         <is>
           <t>1992</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12827,6 +12963,12 @@
           <t>BSMA0247</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>This study examines the relationships between career decisions and directions and a set of independent variables including job title, demographic variables, role stressors, boundary spanning activities, perceived job characteristics, and career outcomes for 348 IS employees. Results show that the majority had already defined specific jobs they would like to hold in the near future. They were also able to define four directions for their future careers: IS technical, IS management, business, and consultant. Results show that career decisions and directions are related to some of the independent variables. IS employees in each of the four career directions could be further categorized into groups on the basis of similar characteristics. Implications of theses findings are discussed.</t>
@@ -12850,6 +12992,11 @@
       <c r="K250" t="inlineStr">
         <is>
           <t>1993</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12864,6 +13011,12 @@
           <t>BSMA0248</t>
         </is>
       </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>This study examined the relative influence of transformational and gatekeeping leadership on team performance in a study of researchers working in industrial R&amp;D teams in Japan. Potential effects of both internal and external communication and group norms for consensus were studied as possible mediating influences on the leadership-performance relationship. Results found that, while both forms of leadership enhanced communication processes within and between groups, only gatekeeping leadership served to reduce group norms for consensus. As a result, team cultures became somewhat more accepting of expressions of divergent opinions and new ideas from various team members, an important factor in R&amp;D innovation and performance. By contrast, transformational leadership served to create team cultures in which divergence from group norms by various members was discouraged, leading to fewer innovative ideas and no performance increment. Results are discussed both in the context of the unique Japanese work environment and in the larger context of leadership processes across regions and cultures.</t>
@@ -12887,6 +13040,11 @@
       <c r="K251" t="inlineStr">
         <is>
           <t>2012</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -12938,6 +13096,12 @@
           <t>BSMA0250</t>
         </is>
       </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>In this article the authors discuss research they conducted that examined the relationship between task difficulty and the extent of boundary-spanning activity within an organization. The authors believed that they greater degree of interunit interdependence that existed in an organization would result in a greater amount of boundary-spanning activity by that organization's members. They also believed that the greater degree of task difficulty in a given situation would also result in a greater amount of boundary-spanning activity by members. The authors hoped to examine the relationships that exist between organizational structure and the amount of intergroup activity fostered by those structures.</t>
@@ -12961,6 +13125,11 @@
       <c r="K253" t="inlineStr">
         <is>
           <t>1986</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13017,7 +13186,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>Marketing boundary spanners—especially customer service representatives—are notably susceptible to burnout. The authors define the burnout construct and develop hypotheses to examine if burnout acts as a partial mediator between role stressors and key behavioral and psychological job outcomes. Responses from 377 customer service representatives reveal that burnout levels are high relative to other burnout-prone occupations (e.g., police, nursing) and that burnout has consistent, significant, and dysfunctional effects on their behavioral and psychological outcomes. Moreover, burnout mediates the negative effects of role stressors on job outcomes, whereas the positive effects of role stressors are unmediated.</t>
@@ -13065,7 +13233,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -13113,7 +13280,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>Because of their boundary-spanning nature, manufacturers’ representatives frequently are involved in team selling. The results from a survey of 362 manufacturers’ representatives indicates that team selling is more likely to be used by manufacturers’ representatives when the customer faces a first-time buy of a complex product, when the information needs of the customer are great, when the account requires special treatment, and when a number of people are involved in the decision to buy. In addition, team selling is more likely when the potential sale is large for the representative firm and when the product is new to the representative’s product line.</t>
@@ -13161,7 +13327,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>With congeneric mergers, which involve firms with interrelated but not identical business lines that develop diverse products and services, a major challenge for organizations is the development of a common platform that fulfills similar business functions across multiple divisions. Through a field study of a postmerger common platform development initiative, we develop a framework that highlights how environmental and organizational contexts shape the process of common platform development (CPD). Our study provides an account of how the focal organization transitioned to a platform-based approach by achieving a balance between stable and flexible aspects of the common platform through negotiations among the divisions acquired through mergers and acquisitions. These negotiations were enabled through various boundary-spanning activities and the guided successive enrichment of boundary objects used in CPD process. European Journal of Information Systems (2015) 24(2), 159–177.</t>
@@ -13303,7 +13468,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>This study investigated the effects of small business owner decision styles on the search for external assistance information, community information, and competitor information. Results confirmed the existence of decision style differences in selection of boundary spanning activities. A conclusion is drawn that small business owners use preferred sources for gathering information related to business operations, but need to utilize additional sources to ensure a comprehensive boundary spanning role. Ways to enhance boundary spanning activities are provided</t>
@@ -13351,7 +13515,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>The influence of boundary spanning roles on strategic decision-making was explored in a field study in fifteen organizations. Results support the importance of boundary spanning roles in the strategic decision-making process and the relationship of technology to the differential strategic decision-making influence of different boundary spanning roles.</t>
@@ -14694,7 +14857,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -16162,7 +16324,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>Purpose – As teams are built around specialized and different knowledge, they need to regulate their knowledge boundaries to exchange their specialized knowledge with other teams and to protect the value of such specialized knowledge. However, prior studies focus primarily on boundary spanning and imply that boundaries are obstacles to sharing knowledge. To ﬁll this research gap, this study aims to indicate the importance of knowledge protection regulation, an activity that sets an adequate boundary for protecting knowledge, and investigate the factors that facilitate knowledge protection regulation and its consequences.</t>
@@ -16393,7 +16554,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -16441,7 +16601,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>Improving performance often requires creative ideas in extreme work settings like health care. Frontline workers are promising sources of creative ideas. The authors assert that their job dissatisfaction is positively associated with creativity in health care settings because negative emotion spurs creativity when tied to engaging work and that characteristics such as shorter tenure, greater role centrality, and high boundary spanning can strengthen this relationship. The authors find supporting evidence in data on ideas generated over 18 months by health professionals in 12 clinics.</t>
@@ -16536,7 +16695,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to provide a novel way of thinking about firm internationalization. We offer a stylized view of family firms as internationalizers who choose to engage in “boundary-spanning” across global product markets while engaging in “boundary-buffering” to insulate themselves from global financial markets.</t>
@@ -16584,7 +16742,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>Multiteam systems (MTSs) have been increasingly adopted as an organizational form to manage large-scale projects. However, new product development (NPD) in the MTSs structure entails challenges with respect to achieving efﬁciency due to interteam coordination challenges. Shared mental models (SMMs) within a single team have been found to facilitate intrateam coordination; however, further exploration is needed as to whether SMMs within MTSs can improve interteam coordination among component teams and, if so, what mechanisms underlie this. The present article examines the theoretical underpinning of the impacts of SMMs among component team leaders on MTSs’ NPD efﬁciency, and further considers the impact of external conditions of requirement uncertainty, the most common external situation during NPD. Using survey data from 110 information technology development MTSs and drawing on boundary management perspective, the results reveal that SMMs among component team leaders positively affect NPD efﬁciency by managing the MTSs boundary, i.e., through boundary entrainment and boundary buffering activities at the system level. In addition, we ﬁnd that requirement uncertainty plays a vital role in determining the nature of this relationship. Taken together, our ﬁndings highlight the importance of the role of SMMs among component team leaders in facilitating NPD efﬁciency in MTSs settings.</t>
@@ -17060,7 +17217,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -18451,6 +18607,12 @@
           <t>BSMA0387</t>
         </is>
       </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr">
         <is>
           <t>Although the use of generative artificial intelligence (AI) within organizations is becoming increasingly common, research on how to enhance employees' competitive advantage through generative AI use within organizations is very limited. Using a resource-based view model, this study investigates the relationship between generative AI use and employees' competitive advantage, as well as the moderating role of perceived organization support. From an analysis of data from 264 employees from 200 organizations, it is found that work-related generative AI use has a positive effect on employee boundary spanning, which contributes to employee competitive advantage. Secondly, work-related generative AI use also has a positive effect on employee agility, including employee resilience and employee adaptability, which further contributes to employee competitive advantage. However, work-related generative AI use has a positive effect on employee proactivity, while the effect of employee proactivity on employee competitive advantage is not significant. Thirdly, perceived organizational support can enhance the effect between employee boundary spanning and employee competitive advantage. However, it is interesting to observe that perceived organizational support enhances the effect between employee adaptability and employee competitive advantage, while weakening the effect between employee proactivity and employee competitive advantage. It does not exert a moderating effect between employee resilience and employee competitive advantage. These findings can help deepen the current understanding of the relationship between generative AI use in the organization and employee competitive advantage, and provide suggestions for business managers on how to use generative AI to improve employee competitive advantage.</t>
@@ -18474,6 +18636,11 @@
       <c r="K390" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18525,6 +18692,12 @@
           <t>BSMA0389</t>
         </is>
       </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr"/>
       <c r="G392" t="inlineStr">
         <is>
           <t>Although difficult, complicated, and sometimes discouraging, collaboration is recognized as a viable approach for addressing uncertain, complex and wicked problems. Collaborations can attract resources and increase efficiency, facilitate visions of mutual benefit that can ignite common desires of partners to work across and within sectors, and create shared feelings of responsibility. Collaboration can also promote conceptualized synergy, the sense that something will “be achieved that could not have been attained by any of the organizations acting alone”(Huxham, 2003). However, previous inquiries into the problems encountered in collaborations have not solved an important question: How to enable successful collaboration? Through exploratory sequential mixed-methods research conducted in three empirical studies, I discover how interorganizational collaborations can overcome barriers to innovate and rejuvenate communities and understand the factors and antecedents that influence successful collaboration.</t>
@@ -18548,6 +18721,11 @@
       <c r="K392" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18562,6 +18740,16 @@
           <t>BSMA0390</t>
         </is>
       </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G393" t="inlineStr">
         <is>
           <t>Boundary spanners play an important role in multinational corporations (MNC), yet it is unclear who these valuable individuals are and why certain individuals, and not others, perform this role. We advance a ‘recognition’ perspective based on whether and how relevant others on both sides on the boundary experience positive impact. A dynamic integrated mixed method analysis of 118 individuals involved in headquarterssubsidiary interactions in four MNCs, shows that only a minority are ‘recognized boundary spanners’, experienced by others to positively impact intergroup relations. We identify diﬀerent categories and mechanisms of recognition, and make a methodological contribution by integrating qualitative and quantitative analysis.</t>
@@ -18585,6 +18773,11 @@
       <c r="K393" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18599,6 +18792,12 @@
           <t>BSMA0391</t>
         </is>
       </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr">
         <is>
           <t>Adaptive supply chain partnerships are a key factor in driving the ability of extended enterprise partners to achieve long-term goals in an environment characterized by disruptive environmental shifts. Adaptive extended enterprise arrangements allow participating enterprises to leverage their combined assets for collective exploration and exploitation. In the context of extended enterprises, where significant investments have been directed toward instituting common interfaces, this study examines the question: How does the use of standard electronic business interfaces (SEBIs) enable supply chain partnerships to become more adaptive?             This study conceptualizes the use of SEBIs as a boundary-spanning mechanism that helps overcome boundaries that impede knowledge transfer between enterprises in supply chains. SEBIs enables partners to gain insight into their broader environments, enriching each partner's perspective (enhanced bridging). SEBIs also help strengthen the cooperative ties between partners, motivating each partner to adapt for collective gain (enhanced bonding).             Our research model is empirically tested using data collected from 41 demand-side supply chain partnerships (between original equipment manufacturers (OEMs), distributors, and retailers) in the information technology (IT) industry. The results show that collaborative information exchange (CIE) between supply chain partners mediates the relationship between use of SEBIs and mutual adaptation (MA) and adaptive knowledge creation between supply chain partners. Interestingly, the use of SEBIs is found to be directly associated with MA but only indirectly associated with adaptive knowledge creation.             The study points out that the strategic impacts of SEBIs go well beyond the exchange of transaction information and process integration. It also shows that multilateral, quasi-open, and information exchange–and process linkage–oriented SEBIs can result in both bonding and bridging across supply chain partners without binding them inflexibly to specific partners. Based on the model and results, the study offers practical implications for how SEBIs should be developed, adopted, and used.</t>
@@ -18622,6 +18821,11 @@
       <c r="K394" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18673,6 +18877,12 @@
           <t>BSMA0393</t>
         </is>
       </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr">
         <is>
           <t>Technology transfer’ is a misnomer; this popular phrase and the studies from which it originates often suggest passivity and inertia on the part of developing country recipient firms. This paper, which uses the technological capability building system (TCB) approach as a conceptual framework, suggests that firms in developing countries exercise constrained agency in technological acquisition processes. The evidence discussed here is taken from a study of technological capability accumulation by twenty-six firms in the telecommunication sector of four developing countries: Uganda, Ghana, Tanzania and South Africa. Important insights into technological acquisition by firms in a service sector in developing countries emerged from that study, such as the existence of specific boundary management capabilities for managing relationships with suppliers; confirmation that firms use different mechanisms for acquiring codified and tacit knowledge; and support for the view that technical change and industry features have significant effects on technology acquisition strategies and their effectiveness.</t>
@@ -18696,6 +18906,11 @@
       <c r="K396" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19450,7 +19665,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -19686,7 +19900,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>This dissertation investigates factors that influence efforts by lower-level employees to initiate organizational change and innovation from the bottom up. Specifically, I attempt to reconcile competing theories regarding the effects of structural and social integration on individual innovation efforts. One theoretical view posits that integration provides information, ideas, and motivation necessary for innovation. An alternative view is that integration constrains individuals and routines, and thereby hinders innovation efforts. Drawing on both theoretical perspectives, I predict the effects of distinct types of structural integration (eg, centralization, cross-unit integration, boundary spanning) and social integration determinants (eg, geographic dispersion, decision process involvement, workplace network size) on the likelihood of individual innovation efforts among lower-level employees. I also consider the effects of interactions of social and structural integration with individual characteristics (ie, personality, and experience) on innovation efforts. I test these predictions using survey data collected from interns and supervisors in the context of MBA and undergraduate internships. Analyses demonstrate that several aspects of structural integration do influence the levels of individual innovation efforts. For example, centralization and boundary spanning levels of the work unit have inverse U-shaped relationships with the level of innovation effort. These findings suggest that for certain types of innovation, structural integration can constrain efforts at the extremes (very high or low) and facilitate efforts at modest levels of integration. Predicted social integration effects are largely non-significant, suggesting the need for further consideration and alternative empirical tests of such effects. Nevertheless, the structural integration findings reaffirm the need to bring together both theoretical perspectives (ie, the view that integration fosters innovation efforts, and the alternative view that isolation and independence are necessary for innovation). By empirically demonstrating that distinct types of integration have unique, yet theoretically consistent effects on several different classes of individual innovation efforts (both process and strategy related), this study contributes to efforts to reconcile these competing theories. Additionally, this research enhances our understanding of a class of little-studied behaviors that play a potentially important role in autonomous strategic change and organizational learning.</t>
@@ -19833,7 +20046,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
           <t>It is widely recognized that new product development (NPD) is a highly interdependent process, yet efforts to empirically model the interdependence and examine its effect on ﬁrm performance are scarce. Our study addresses this research gap. We model ﬁrms’ abilities to collectively collaborate with suppliers, customers, and internal employee teams in NPD as collaborative competence and examine its impact on project and market performance. Using responses collected from 189 NPD managers, we ﬁnd empirical evidence for collaborative competence and its differential impact on project and market performance. Speciﬁcally, we ﬁnd that collaborative competence has a direct impact on project performance, but its impact on market performance is indirect, mediated through project performance. The results have signiﬁcant managerial implications; achieving superior market performance from inter- and intra-organizational involvement is contingent on achieving superior project performance, and companies that fail to achieve desired project performance outcomes will also fail in achieving market performance goals.</t>
@@ -19928,7 +20140,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
           <t>Recent research has emphasized cross functional integration as a key facilitator of success in new product development (NPD) projects. This dissertation developed and tested a model using supply chain integration as a key enabler influencing both planning of the new product and execution of the development process in NPD projects. Supply chain integration was operationalized to include cross functional (for example, between design and manufacturing) and boundary spanning integration mechanisms (such as supplier integration). Product concept effectiveness (a construct capturing the planning of the new product), and development process performance (a construct measuring the execution of new product development process) were theorized to influence overall project success. Hypotheses drawn from this framework were tested on a multi-industry sample (electronics, communications, semiconductors, and computers) of firms. Data analysis was conducted using regression analyses, partial correlations, confirmatory factor analyses and structural equation modeling.</t>
@@ -20028,7 +20239,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
           <t>Mentoring is a valuable resource that enhances outcomes like career success. Applying conservation of resources theory, we examine the interaction effects of workers’ management aspirations and lengthy career interruption(s) on the mentoring-career success relationship. Utilizing 259 older professional workers, we test these relationships with both cross-sectional and time-separated data. Although the pattern of results was similar when comparing the crosssectional data to the time-separated data, we found that relationships were stronger within the cross-sectional data, resulting in the support of two additional hypotheses. With the timeseparated data, we found evidence of a three-way interaction. Speciﬁcally, mentoring is more valuable for the perceived career success of workers with higher management aspirations who had not experienced a lengthy career interruption than it is for workers with higher management aspirations who had experienced a lengthy career interruption or for workers with lower management aspirations regardless of whether they had experienced a career interruption.</t>
@@ -22623,7 +22833,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>Abstract             In this study, we analyse the discursive strategies of professionalization used by psychology in Spain during its professionalization phase in the health sector in the early twenty-first century. Our primary focus is the conflict with political regulators and other healthcare professions after the Ley de Ordenación de Profesiones Sanitarias (Healthcare Professions Act) came into effect, since this Act calls into question the extent to which psychology can be viewed as health care. We use discourse analysis to determine the discursive structure of the conflict, which has an interprofessional dimension, as well as the professionalization and social closure strategies of psychology within the framework of professional relationships (boundary work). We argue that understanding this conflict requires viewing it as part of the European and international regulation context of healthcare professions. Highlighted in the analysis is the emergence of two psychology discourses divided into four modes of enunciation (professionalizing, cultural, scientific, and political–economic). Among other aspects, the conclusions focus on the dual interprofessional and intraprofessional nature of the conflict and evidence of a dual closure in psychology. The latter’s professionalization strategies in the sector occasionally resemble those employed by nursing, although at other times they are similar to those followed by some paramedical professions.</t>
@@ -22723,7 +22932,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -27719,7 +27927,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F619" t="inlineStr"/>
       <c r="G619" t="inlineStr">
         <is>
           <t>Organizational values and beliefs significantly influence employee decision making and behavior and manifest themselves as multiple climates existing within a single organization. A subset of organizational climate is an ethical climate, embodying normative values and beliefs involving moral issues shared by the employees of the organization. Reseachers have found multiple ethical climates present in an organization.</t>
@@ -27767,7 +27974,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F620" t="inlineStr"/>
       <c r="G620" t="inlineStr">
         <is>
           <t>Boundary‐spanning communication has been found to be important to various types of organizations and groups as a source of new information and awareness of environmental changes. Although the importance of formal, public channels in building the knowledge base of a field has long been recognized, most studies of boundary‐spanning activity have been limited to direct, personal (informal) communication. This study examines both informal and formal communication patterns of three groups in order to determine whether, in fact, a variety of media are used in boundary‐spanning communication. The groups selected were the members of three professions which fill intermediary positions between the creators and consumers of cultural products; one located in academia and two in the private sector. Major findings were that: (1) A boundary‐spanning structure linking 82.2% of the survey respondents was composed of both informal and formal media. (2) The professions differed in which type of channel was most heavily used, but were similar in their perceptions of the importance of the channels. (3) Individuals central to the informal part of the structure were also more likely to use the formal parts of the structure. (4) Boundary‐spanning media were among the five most frequently cited media for all three of the professions.</t>
@@ -27815,7 +28021,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>Research-practice partnerships (RPPs) offer promising approaches to improve educational outcomes. Navigating boundaries between contexts is essential for RPP effectiveness, yet much work remains to establish a conceptual framework of boundary spanning in partnerships. Our longitudinal comparative case study draws from our experiences as graduate student boundary spanners in three long-term partnerships to examine boundary spanning roles in RPPs, with particular attention to the ways in which power permeates partnership work. Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums: institutional focus, task orientation, expertise, partnership disposition, and agency. Our roles were shaped by the organizational, cultural, relational, and historical features of the partnerships and contexts of interaction. We aim to promote the development of effective RPP strategies by leveraging the perspectives and positionality of graduate students in order to advance understanding of boundary spanning roles.</t>
@@ -29277,7 +29482,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr">
         <is>
           <t>Individuals in work teams frequently cross boundaries across teams, often by using information and communication technologies (ICTs). The current study investigates the effects of members’ boundary work and the visibility affordance of teams’ ICTs on Transactive Memory Systems (TMS) in teams. Survey data from 212 fulltime employees whose work hours were divided between multiple teams reveals that boundary spanning enhances the focal team’s TMS specialization and credibility and negatively inﬂuences TMS coordination. Additionally, boundary reinforcement positively affects TMS credibility and coordination. The visibility affordance has a direct positive effect on all three dimensions of TMS and a moderating effect for boundary reinforcement such that higher visibility overrides the positive direct effect of boundary reinforcement on TMS. These ﬁndings suggest that different types of boundary work contribute to different dimensions of TMS and that teams might consider prioritizing the use of ICTs with high visibility to enhance their TMS.</t>
@@ -29424,7 +29628,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F662" t="inlineStr"/>
       <c r="G662" t="inlineStr">
         <is>
           <t>This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of noncore firms operating in the context of sustainable development. The dynamic nature of technological innovation, exacerbated by market flattening and the challenges posed by the COVID-19 pandemic, has compelled small and medium-sized enterprises (SMEs) to seek innovative breakthroughs. Cooperative innovation emerges as a strategic avenue for SMEs to mitigate risks and enhance their willingness to innovate. However, non-core firms often encounter technological and market disadvantages, hindering innovation efforts. This study explores how boundary-spanning knowledge search, which bridges the gap between non-core firms and the external environment, influences cooperative innovation. Furthermore, the research delves into the mediating role of both potential and actual absorptive capacity in the relationship between boundaryspanning knowledge search and cooperative innovation performance. Empirical findings indicate that boundary-spanning knowledge searches positively impact cooperative innovation, with technological and market knowledge searches yield significant results. Moreover, absorptive capacity exhibits a dual mechanism, directly influencing cooperative innovation and mediating the relationship between knowledge search and performance. This paper extends existing research by focusing on non-core firms within the sustainable development context, offering valuable insights for SMEs seeking innovative strategies. It also highlights the diverse pathways through which boundary-spanning knowledge search affects cooperative innovation. These findings offer practical implications for enhancing non-core firms’ innovation capabilities, including encouraging proactive knowledge search and developing absorptive capacity-inducing mechanisms through employee training and information platforms.</t>
@@ -29472,7 +29675,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F663" t="inlineStr"/>
       <c r="G663" t="inlineStr">
         <is>
           <t>This paper examines the influence of boundary-spanning knowledge search on cooperative innovation performance and explores the moderating role of innovation passion in Chinese firms. We collected 229 valid responses from Chinese firms participating in collaborative innovation projects and applied confirmatory factor analysis to test the reliability and validity of the constructs, multiple stepwise regressions to verify the direct effect, and the PROCESS macro to test the moderating effect. The results show that all three dimensions of boundary-spanning knowledge search (i.e. network capability, IT capability, and absorptive capacity) positively affect cooperative innovation performance. Harmonious innovation passion positively moderates the relationship between network capability and cooperative innovation performance. In contrast, compulsive innovation passion plays a negative moderating role in the relationship between absorptive capacity and cooperative innovation performance. This study further enriches and extends the theoretical framework of cooperative innovation performance by emphasizing the impact of the three dimensions of boundary-spanning knowledge search.</t>
@@ -29735,7 +29937,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>Due to their complexity and high social impact, urban infrastructure projects often face challenges in managing the design decision-making processes across disparate disciplinary and knowledge domain boundaries. This paper introduces the notion of design boundary dynamics to describe the various cross-boundary coordination phenomena associated with organising the design of infrastructure projects. Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project. Findings illustrate the entangled processes, through which the disciplinary, knowledge-domain and stage-based design boundaries emerged as a result of unfolding project practices. Paper identifies the key role of resource allocation constraints, path dependency of project decisions, and problem-solving nature of design and concludes with strategic recommendations for upstream operational integration to mitigate the impact of design boundary dynamics on infrastructure projects.</t>
@@ -29857,7 +30058,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -30784,7 +30984,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F696" t="inlineStr"/>
       <c r="G696" t="inlineStr">
         <is>
           <t>Purpose – Business model innovation (BMI) is an important channel of enterprise innovation, and BMI’s antecedents have attracted extensive attention. The purpose of this paper is to address a substantial gap in the extant literature by developing a moderate model to explain the effects of boundary-spanning search on BMI as well as whether and how innovative cognitive imprinting (ICI) and environmental dynamics (ED) affect the above relationship.</t>
@@ -31156,7 +31355,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_1
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -10331,6 +10331,12 @@
           <t>BSMA0186</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>Drawing on corporate entrepreneurship (CE) and social network research, this study focuses on strategic renewal as a form of CE and examines the impact of boundary-spanning at top and middle management levels on business units’ exploratory innovation. Analyses of multi-source and multi-level data, collected from 72 top managers (TMs) and 397 middle managers (MMs) operating in 34 units of a multi-national organization, indicate that TMs’ boundary-spanning is positively related to units’ exploratory innovation, but also has a cascading effect on MMs by increasing their perceived role conflict. MMs’ role conflict is negatively related to units’ exploratory innovation and thus offsets some of the benefits gained through TMs’ boundary-spanning activities. Taking a configurational perspective on social exchanges at multiple levels, we show that role conflict is reduced by overlapping boundary-spanning ties among TMs and MMs. Surprisingly, MMs’ boundary-spanning does not relate to exploratory innovation. Our study shows that with regard to boundary-spanning, a top-down approach to CE as strategic renewal may be most effective because TMs play a key role in driving exploratory innovation. However, TMs need to be aware of the cascading social liabilities of their boundary-spanning behavior and ensure MMs develop similar networks. We advance ongoing debates in studies about CE and social networks by providing empirically validated insights into who drives strategic renewal and by uncovering the benefits and costs of social exchanges for strategic renewal. Furthermore, we uncover potential causes of mixed findings in network theory research and highlight a remedy to social liabilities.</t>
@@ -10354,6 +10360,11 @@
       <c r="K189" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10420,7 +10431,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>This paper investigates boundary-work in management accounting in the context of globalization and hybrid professionalism. The paper demonstrates how permeable symbolic boundaries of the management accounting ﬁeld can be altered by employing expansion boundary-work. Contrasting boundary-work of IMA ofﬁcials and IMA members in Russia, we show that IMA ofﬁcials employ primarily monopolization boundary-work while IMA members employ primarily expansion boundary-work. Our ﬁndings illustrate how boundary-work is employed to exhibit organizational and occupational professionalism in the symbolic realm. The paper provides additional insight into the discursive domain of the accounting profession by linking boundary-work to globalization, two forms of professionalism, legitimacy, status and professional identity. This suggests that the professionalization process is inﬂuenced by the properties of professional boundaries.</t>
@@ -10463,6 +10473,12 @@
           <t>BSMA0189</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>This article explores the joint production and consumption of health information and advice in the context of NHS Direct, the new telephone health information and advice service. NHS Direct is an atypical call centre environment in so far as its core staff (nurses) are highly skilled professionals. These nurses are required to collaborate closely with, and are to some extent dependent upon, non-professional lower skilled staff (call handlers) to deﬁne and prioritize their work. This introduces a number of tensions between the two groups. Nurses respond to these tensions by engaging in ‘boundary work’, the micropolitical strategies through which work identities and occupational margins are negotiated, to protect their own status. Call handlers are more subject to the pressures of work ‘speed-up’, highly aware of the risks inherent in their role, but are unable to call upon professional status, either in their resistance to managerial imperatives or in their interactions with health consumers. They are required to manage the tension between offering a safe and high quality service, characterized in their training as ‘professional’, and nurses’ boundary work, which positions them as ‘non-professional’. Here we draw on qualitative research, including call interaction data between call handler and consumer, to show how call handlers’ occupation of the contested territory between professional and non-professional status leaves them wide open to the agency of consumers, as consumers attempt to shape the service in their own interests.</t>
@@ -10486,6 +10502,11 @@
       <c r="K192" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10505,7 +10526,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>Past research has studied how the selection and use of control portfolios in software projects is based on environmental and task characteristics. However, little research has examined the consequences of control mode choices on project performance. This paper reports on a study that addresses this issue in the context of outsourced software projects. In addition, we propose that boundary-spanning activities between the vendor and the client enable knowledge sharing across organizational and knowledge domain boundaries. This is expected to lead to facilitation of control through specific incentives and performance norms that are suited to client needs as well as the vendor context. Therefore, we argue that boundary spanning between the vendor and client moderates the relationship between formal controls instituted by the vendor on the development team and project performance. We also hypothesize the effect of collaboration as a clan control on project performance. We examine project performance in terms of software quality and project efficiency. The research model is empirically tested in the Indian software industry setting on a sample of 96 projects. The results suggest that formal and informal control modes have a significant impact on software project outcomes, but need to be finely tuned and directed toward appropriate objectives. In addition, boundary-spanning activities significantly improve the effectiveness of formal controls. Finally, we find that collaborative culture has provided mixed benefits by enhancing quality but reducing efficiency.</t>
@@ -10548,6 +10568,12 @@
           <t>BSMA0191</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>Recently, discussion has begun to consider serving the base of the economic pyramid for business and societal benefit. Suggestions for so doing have focused on business model innovation, improving internal capabilities, promoting stronger governance, and providing leapfrog technologies (such as ICT) to promote effective change. We consider the questions of what types of innovation are occurring when businesses and other organizations enter the base of the pyramid and what types of social, economic, and consumer benefits they bring to local communities. We base our findings on an analysis of more than 1,000 cases describing base of the pyramid activities.</t>
@@ -10571,6 +10597,11 @@
       <c r="K194" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10775,7 +10806,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>As employees’ personal lives are increasingly splintered by work demands, the boundary between work and nonwork domains is becoming ever more blurred. Grounded within a self-regulatory approach and the executive control function of inhibitory control, we operationalize and examine nonwork role re-engagement (NWRR)—the extent to which individuals can redirect attentional resources back to nonwork tasks following work-related intrusions. In phases 1 and 2, we develop and refine a psychometrically sound unidimensional measure for NWRR aligned with the self-regulatory processes of self-control and interference control underlying inhibitory control. In phase 3, we confirm the factor structure with a new sample. In phase 4 we validate the measure using the samples from phases 2 and 3 to provide evidence of criterion-related, convergent, and discriminant validity. NWRR was related to important well-being and work-related outcomes above and beyond existing self-regulatory and boundary management constructs. We offer theoretical and practical implications and an agenda to guide future research, as attentional agility becomes increasingly relevant in a home life replete with interruptions from work.</t>
@@ -10870,7 +10900,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>This article guides the development of creative insights in supply chain management. The authors begin by describing analogies’ role in advancing organization theory with a focus on image transfers between knowledge domains. While much has been said about the merits of conceptual transfers between domains, much equally remains unknown, particularly about how to deliberately develop creative insights that have the potential to challenge or enhance existing supply chain management theory. To address this issue, this research builds on prior work on analogies, creativity, and design thinking to develop a heuristic-analytic model. This model is designed to assist researchers in theorizing by analogy through a controlled dual cognitive process of divergence before convergence combined with a distant boundary-spanning knowledge search. An illustration of the model shows how creative output can provide a fresh perspective that helps render supply chains potentially more resilient.</t>
@@ -10918,7 +10947,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>The period after completing primary and adjuvant cancer treatment until recurrence or death is now recognized as a unique phase in the cancer control continuum. The term “survivorship” has been adopted to connote this phase. Survivorship is a time of transition: Issues related to diagnosis and treatment diminish in importance, and concerns related to long-term follow-up care, management of late effects, rehabilitation, and health promotion predominate. In this article, we explore the unique challenges of care and health service delivery in terms of the interface between primary care and specialist care during the survivorship period. The research literature points to problems of communication between primary and specialist providers, as well as lack of clarity about the respective roles of different members of the health-care team. Survivorship care plans are recommended as an important tool to facilitate communication and allocation of responsibility during the transition from active treatment to survivorship. Research questions that remain to be answered with respect to survivorship care plans and other aspects of survivorship care are discussed.</t>
@@ -10966,7 +10994,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>In multidisciplinary teams in the oil and gas industry, we examined expertise diversity's relationship with team learning and team performance under varying levels of collective team identification. In teams with low collective identification, expertise diversity was negatively related to team learning and performance; where team identification was high, those relationships were positive. Results also supported nonlinear relationships between expertise diversity and both team learning and performance. Finally, team learning partially mediated the linear and nonlinear relationships between diversity and performance. Findings broaden understanding of the process by which and the conditions under which expertise diversity may promote team performance.</t>
@@ -11681,6 +11708,16 @@
           <t>BSMA0218</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G221" t="inlineStr">
         <is>
           <t>Integration of organisational units has been extensively researched in various streams of management and organization sciences. It is very important whenever knowledge differences have to be overcome due to functional departmentalisation and the ensuing knowledge specialisation. However, extant literature does not yet appreciate the mediating role of absorptive capacity (AC) in this context. We argue that departments use integration mechanisms in order to develop and maintain such an organisational capability to absorb knowledge from other departments, so that integration can succeed to increase innovation performance. Our unique dataset of Italian manufacturing firms from various industries allows us to study this in the context of the integration of research and development (R&amp;D) and marketing and sales (M&amp;S) departments. Thereby, we provide empirical evidence on the mediating role of AC. We find evidence that R&amp;D departments build AC via formal cross-functional integration, while M&amp;S departments do so through informal integration. Moreover, we provide evidence of AC’s mediating role for the relationship between cross-functional integration mechanisms and innovation performance. Our findings also reveal significant differences between R&amp;D and M&amp;S functions in terms of effect sizes and significance levels. AC of R&amp;D departments has a significant and substantial effect on innovation performance and thus effectively acts as a mediating variable, while in case of M&amp;S departments we observe a significant direct effect between formal cross-functional integration and innovation performance without any mediation by AC.</t>
@@ -11704,6 +11741,11 @@
       <c r="K221" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Proxy Informant Trap. Constructs measure department-level integration rather than individual behavior.. Verbatim Evidence: [Data] &lt;The sample in the present study includes responses from 126 professionals in Italian manufacturing firms (31 pairwise, 38 with a response from only one department).&gt; [Appendix] &lt;To what extent does your department use: (1) liaison personnel with ... (2) temporary task forces with ... (3) permanent teams with ...&gt;</t>
         </is>
       </c>
     </row>
@@ -12432,7 +12474,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>This study examines personal ties between boundary-spanning personnel in interorganizational exchanges in emerging markets. Drawing on social embeddedness theory and boundary spanning theory, we propose that strong ties between boundary spanners may benefit exchange parties in their interorganizational relationships through two heightened boundary-spanning behaviors—information processing and external representation. The results from 225 manufacturer–distributor dyads in China indicate that interpersonal ties at the higher levels (between top executives) and at the lower levels (between salespersons and individual buyers) are both positively associated with relationship quality of the buyer–supplier relationship through dyadic boundary-spanning behaviors. Between two levels of interpersonal ties, ties at the lower levels exhibit a stronger association with relationship quality than do ties at the higher levels. Furthermore, the positive effects of interpersonal ties on conflict resolution and cooperation are amplified when both levels of ties are strong in the focal relationship.</t>
@@ -12824,7 +12865,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>This three-essay project explores boundary management and work-nonwork enrichment to explain how thriving in the work domain relates to thriving in the nonwork domain. The Cross-Domain Thriving model proposed in Study 1 theorizes that when employees experience growth and energy at work, they create and deplete resources within and across roles and individual boundary management strategies, role congruency, and ease of transition moderate the degree to which thriving translates into enrichment and/or conflict across roles. Study 2 tested aspects of the cross-domain thriving model and found that neither work nor nonwork thriving was related to increased time-based conflict, but both forms of thriving predicted enrichment gains across domains. Moreover, higher levels of work-nonwork role segmentation were associated with a stronger relationship between learning in nonwork roles and affective and efficiency enrichment gains in the nonwork-to-work direction. In the work-to-nonwork direction, role congruency and cycling boundary management behavior were related to greater developmental and affective enrichment, respectively. Cycling also strengthened the positive relationship between vitality at work and work-to-nonwork capital enrichment. Study 3, a qualitative study investigating work and nonwork thriving in employees working from home during a pandemic, suggested the importance of boundary management skills as demands on learning and energy increase. Findings highlight how key employer actions and employee regulatory behavior can leverage the benefits of growth and energy in work and nonwork domains.</t>
@@ -12872,7 +12912,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>Community-based initiatives (CBIs) are thriving in Western countries. In CBIs, citizens take a leading role in providing public services and goods. CBIs have been acclaimed for their innovativeness, problem-solving capacity, and legitimacy. However, we lack large N studies on performance of CBIs and its antecedents. This article develops and tests a model that identiﬁes relationships between performance and four antecedents by using survey data on CBIs collected in the Netherlands (N = 671). Using structural equation modelling, positive direct and indirect relationships between transformational leadership, boundary spanning leadership, organizational capacity, social capital ties, government support, and performance are found.</t>
@@ -12920,7 +12959,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>The study examines the effects of the individual characteristics, job type, role stressors, boundary spanning activities, career outcomes, and job characteristics on the turnover propensity of 464 information systems personnel. Results show that age, organizational level, organizational tenure, job tenure, and number of years in the computer field are negatively correlated with the intention to leave the organization. Education was found to be positively correlated with turnover intentions, and while project leaders are more likely to leave the organization, IS managers are less likely. Results also show that both role stressors (role ambiguity and role conflict) and boundary spanning activities are positively correlated with turnover intentions, and that job involvement, career plateau, promotability, salary, organizational commitment, job satisfaction, satisfaction with progress, promotion, pay, status, and projects are negatively correlated while career opportunity is positively correlated with turnover intentions. Finally, all job characteristics are negatively correlated with turnover intentions. Implications of the results for practice and research are offered.</t>
@@ -12968,7 +13006,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>This study examines the relationships between career decisions and directions and a set of independent variables including job title, demographic variables, role stressors, boundary spanning activities, perceived job characteristics, and career outcomes for 348 IS employees. Results show that the majority had already defined specific jobs they would like to hold in the near future. They were also able to define four directions for their future careers: IS technical, IS management, business, and consultant. Results show that career decisions and directions are related to some of the independent variables. IS employees in each of the four career directions could be further categorized into groups on the basis of similar characteristics. Implications of theses findings are discussed.</t>
@@ -13016,7 +13053,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>This study examined the relative influence of transformational and gatekeeping leadership on team performance in a study of researchers working in industrial R&amp;D teams in Japan. Potential effects of both internal and external communication and group norms for consensus were studied as possible mediating influences on the leadership-performance relationship. Results found that, while both forms of leadership enhanced communication processes within and between groups, only gatekeeping leadership served to reduce group norms for consensus. As a result, team cultures became somewhat more accepting of expressions of divergent opinions and new ideas from various team members, an important factor in R&amp;D innovation and performance. By contrast, transformational leadership served to create team cultures in which divergence from group norms by various members was discouraged, leading to fewer innovative ideas and no performance increment. Results are discussed both in the context of the unique Japanese work environment and in the larger context of leadership processes across regions and cultures.</t>
@@ -13059,6 +13095,12 @@
           <t>BSMA0249</t>
         </is>
       </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -13082,6 +13124,11 @@
       <c r="K252" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13101,7 +13148,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>In this article the authors discuss research they conducted that examined the relationship between task difficulty and the extent of boundary-spanning activity within an organization. The authors believed that they greater degree of interunit interdependence that existed in an organization would result in a greater amount of boundary-spanning activity by that organization's members. They also believed that the greater degree of task difficulty in a given situation would also result in a greater amount of boundary-spanning activity by members. The authors hoped to examine the relationships that exist between organizational structure and the amount of intergroup activity fostered by those structures.</t>
@@ -13144,6 +13190,12 @@
           <t>BSMA0251</t>
         </is>
       </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>Innovation has an intrinsic relationship with social networks because it provides a mechanism for knowledge and information to travel freely between individuals. Consequently, there is abundant research linking social networks to innovation. However, two critical gaps still exist. First, most research studies use a structural approach, and less attention is paid to the behavioral dimensions in a network. Secondly, the majority of empirical research focuses on egocentric networks or dyadic relationships between two organizations, instead of the network of organizations as a whole.</t>
@@ -13167,6 +13219,11 @@
       <c r="K254" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13604,6 +13661,12 @@
           <t>BSMA0261</t>
         </is>
       </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>Purpose – In today’s digital and post-pandemic era, construction teams can span their boundary to obtain important resources and support in computer-mediated ways. However, the benefits of computer-mediated team boundary spanning (TBS) are mostly assumed. Empirical evidence for these benefits is in lack. Thus, this study attempts to investigate the influence of computer-mediated (instant messaging in this study) TBS on construction project performance and the underlying mechanism.</t>
@@ -13627,6 +13690,11 @@
       <c r="K264" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13641,6 +13709,12 @@
           <t>BSMA0262</t>
         </is>
       </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>International joint ventures (IJVs) have become an important source of critical knowledge for multinational enterprises, but little is known about how knowledge can be effectively transferred to parent ﬁrms when the potential for interpartner opportunism still exists. Drawing on attachment theory, we study how boundary-spanning commitments to IJVs may help mitigate interpartner opportunism and facilitate effective knowledge transfer to parents. Speciﬁcally, we argue that knowledge transfer from IJVs to their parents is positively mediated by both boundary spanners’ organizational commitment to IJVs and parent ﬁrms’ resource commitment to IJVs. We test our arguments using survey data collected from 600 dyadic Chinese–foreign managers of 100 IJVs established in China. The results provide evidence that knowledge sharing between boundary spanners in IJVs positively affects their organizational commitment to these IJVs, which in turn positively affects knowledge transfer to parents. Similarly, knowledge sharing between such boundary spanners positively affects parent ﬁrms’ resource commitment to IJVs, which in turn positively affects knowledge transfer to parents. The mediating role of boundary spanners’ organizational commitment is stronger than that of parent ﬁrms’ resource commitment. Collectively, our ﬁndings suggest that commitment-based relational mechanisms are imperative for safeguarding effective knowledge transfer from IJVs to parent ﬁrms.</t>
@@ -13664,6 +13738,11 @@
       <c r="K265" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13678,6 +13757,12 @@
           <t>BSMA0263</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>This paper collects 103 sample firms' 2015 to 2019 data through data envelopment analysis to measure their technical innovation performance and social network analysis to build joint-patent networks and explore knowledge-creating alliance relationships. The article highlights how tacit knowledge recombination works as a mechanism of boundary spanning. It emphasizes the significance of strategic balancing networks' position to improve technical innovation performance and competitiveness of patent-intensive (PI) firms. This research contributes to shedding additional light on the nature of the boundary-spanning mechanism and PI firms' knowledge exchanges. Specifically, it examines how balancing boundaries spanning through joint-patent networks can influence the processes of tacit knowledge transmission and recombination between knowledge-based actors.</t>
@@ -13701,6 +13786,11 @@
       <c r="K266" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13715,6 +13805,12 @@
           <t>BSMA0264</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>Setting the research background in China, this study draws on absorptive capacity, knowledge inertia and prospect theory to show the relationship between R&amp;D capability and innovation performance which comprises exploitation and exploration. We propose that stronger R&amp;D capability promotes exploitation performance but inhibits exploration performance. As exploitation represents immediate interest and exploration represents long-term interest, we introduce the notion of knowledge boundary spanning of R&amp;D network to balance short-term and long-term benefits. The empirical results show that R&amp;D capability and knowledge boundary spanning of R&amp;D network complement each other for explorative innovation while they present trade-offs for exploitative innovation. This study contributes to existing literature on R&amp;D capability–innovation performance, and it further extends our understanding by investigating the impact of knowledge boundary spanning of R&amp;D network on the R&amp;D capacity–innovation performance relationships. In addition, this study provides references on resources configuration to achieve different innovation strategies.</t>
@@ -13738,6 +13834,11 @@
       <c r="K267" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13752,6 +13853,12 @@
           <t>BSMA0265</t>
         </is>
       </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>Open innovation is crucial for achieving high-quality and sustainable business growth. However, it remains unclear how prospective boundary-spanning search and responsive boundary-spanning search impact organizational resilience and open innovation in the VUCA (Volatility, Uncertainty, Complexity, and Ambiguity) new normal. Based on the resource-based theory and dynamic capabilities theory, this paper classifies boundaryspanning search into prospective boundary-spanning search and responsive boundary-spanning search to investigates the impact on open innovation and organizational resilience, and analyze the moderating role of big data analytics capability. The empirical study of 293 Chinese smart manufacturing firms indicates that both prospective and responsive boundary-spanning search have an inverted U-shaped impact on open innovation and organizational resilience. Organizational resilience partially mediates the relationships between prospective boundary-spanning search, responsive boundary-spanning search, and open innovation. Moreover, big data analytics capability moderates and flattens the inverted U-shaped relationships between prospective and responsive boundary-spanning search, and organizational resilience. This study explores the intrinsic mechanism of prospective and responsive boundary-spanning search on open innovation through organizational resilience. The findings enrich and expand the research on the antecedents of open innovation.</t>
@@ -13775,6 +13882,11 @@
       <c r="K268" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13826,6 +13938,12 @@
           <t>BSMA0267</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>This study examines the antecedents of job satisfaction, commitment and turnover for 229 information systems development personnel (ISDP) employed by nine companies within several industries. The antecedents studied include boundary spanning, role ambiguity and role conflict. A model of these variables is built and tested via path analysis. A secondary analysis is performed to explore the impacts of task and individual differences on the study variables. The task differences include analytic and programming tasks while the individual differences studied are age, tenure, education and years of data processing experience.</t>
@@ -13849,6 +13967,11 @@
       <c r="K270" t="inlineStr">
         <is>
           <t>1984</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13863,6 +13986,12 @@
           <t>BSMA0268</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
           <t>The relationship between boundary-spanning role activities and conflict management styles was examined with data gathered from 189 project managers who belong to a national professional association. Five conflict management styles and six boundary role activities were measured with a survey instrument constructed from previously developed scales. The conflict management styles measured were integrating, avoiding, dominating, obliging, and compromising. The six boundary role activities measured were gathering, filtering, and transmitting information; transacting; proacting; and protecting. Hypotheses proposing specific relationships between each of the five conflict management styles and the six boundary role activities were tested with the data. Results indicated that unique combinations of boundary role activities are associated with each of the conflict management styles. Further, more cooperative conflict management styles are related to a greater number of boundary role activities that emphasize information sharing and managing relationships. Results also indicated that length of a project manager's experience moderates this relationship in that those with greater experience use more cooperative styles. A revision is suggested to the conflict management style construct.</t>
@@ -13886,6 +14015,11 @@
       <c r="K271" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13900,6 +14034,12 @@
           <t>BSMA0269</t>
         </is>
       </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>Owing to their growing numbers and importance, both managers and researchers are increasingly concerned with the work experiences of boundary-spanning employees. Employee perceptions of organizational support *POS) may be particularly relevant to this crucial employee group. Thus reports a study of the relations between two individual-level and two organizationallevel antecedents to boundary-spanner POS. The results indicate that employee gender, amount of formal organizational recognition received, and the quality of task-related training are associated with POS. However, type of employee pay plan is not. Concludes with a discussion of these findings and their implications for effectively managing boundary-spanning employee POS.</t>
@@ -13923,6 +14063,11 @@
       <c r="K272" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13937,6 +14082,12 @@
           <t>BSMA0270</t>
         </is>
       </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate a boundary spanning, interprofessional collaboration between advanced practice nurses (APNs) and junior doctors to support junior doctors’ learning and improve patient management during the overtime shift.</t>
@@ -13960,6 +14111,11 @@
       <c r="K273" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14011,6 +14167,12 @@
           <t>BSMA0272</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>Firms are challenged to achieve organizational goals in an environment of increasingly decentralized information. Cross-functional project teams are employed widely as a strategy to facilitate better coordination, yet projects still fail at a rate of 31% per year. Communication is a leading cause of failure. While inter-team communication has been studied extensively, less is understood about the intra-team communication of a cross-functional project team.</t>
@@ -14034,6 +14196,11 @@
       <c r="K275" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14048,6 +14215,12 @@
           <t>BSMA0273</t>
         </is>
       </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>This paper describes one of the first empirical explorations into organisational knowledge creation theory as first elucidated by Nonaka and Takeuchi [1]. We extend the theory and examine it in the inter-organisational context of University-Industry (U-I) collaborative R&amp;D Projects. More specifically, the relationship between enabling conditions and knowledge conversion processes as well as the effects of these processes on the achievement of technological objectives are studied using a sample of 25 U-I collaborative R&amp;D projects into advanced technology. Quantitative and qualitative evidence supports the theory that some enabling conditions are significant for knowledge conversion processes. Furthermore, the presence of the aggregate knowledge processes is positively associated with the achievement of successful technological objectives. The theoretical and practical implications of these findings are discussed.</t>
@@ -14071,6 +14244,11 @@
       <c r="K276" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14085,6 +14263,12 @@
           <t>BSMA0274</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>BACKGROUND: There is a need for a better understanding of how the use of technology to complete work outside regular ofﬁce hours is related to work-life outcomes. Few studies have also investigated how individual differences in work-nonwork boundary management relate to work-life outcomes. OBJECTIVE: This study was conducted to examine how teleworking outside regular ofﬁce hours and individual boundary management relate to work-family conﬂict. METHODS: A web survey was sent to fulltime employees at the headquarters of a multinational high-tech ﬁrm in Sweden. A total of 71 answers were obtained and analyzed using regression analysis. RESULTS: The extent of teleworking after hours was unrelated to work-family conﬂict. However, as previous research has shown, having more permeable boundaries and allowing work to interrupt nonwork behavior was related to higher levels of conﬂict. CONCLUSIONS: The ﬁndings suggest that teleworking after hours is not as problematic in terms of work-family conﬂict as has been reported in previous studies. Furthermore, in order to prevent high levels of work-family conﬂict, it is seemingly beneﬁcial to avoid work interruptions during nonwork behavior.</t>
@@ -14108,6 +14292,11 @@
       <c r="K277" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14122,6 +14311,12 @@
           <t>BSMA0275</t>
         </is>
       </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>While the introduction of a new product or service carries considerable risk, incorporating customer input into the new product/service development (NPD) process increases the probability of commercial success. In their boundary spanning role, industrial (B-to-B) salespeople are well suited to serve as a conduit between customers and those inside their company who are largely responsible for the NPD process. The current study investigates the perceptions of sales managers and examines the role the sales force may play in the early stages of the NPD process. An empirical analysis is conducted to determine whether differences exist between organizations that employ key account management (KAM) systems and those that do not employ KAM systems. The findings of this study suggest that salespeople from KAM organizations are better suited to provide input into the NPD process than their non-KAM counterparts.</t>
@@ -14145,6 +14340,11 @@
       <c r="K278" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15791,6 +15991,12 @@
           <t>BSMA0319</t>
         </is>
       </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>Purpose – This study investigates the relationship between buyer-supplier top management team (TMT) demographic misalignment (defined as differences in TMT composition based on background, age and gender) and environmental performance (EVP).</t>
@@ -15814,6 +16020,11 @@
       <c r="K322" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15865,6 +16076,12 @@
           <t>BSMA0321</t>
         </is>
       </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>As a core organizational resource, business processes are vital for organizational teams. To deal with today’s volatile business environment, organizations need to be ambidextrous in terms of process capabilities. However, little is known about how process ambidexterity, process standardization, and process agility, are enabled by information technology (IT) and related to team-level activities. To fill this gap in the literature, we conducted a field study based on 160 teams of 1081 individuals from seven companies in South Korea. Our results show that IT enables both process standardization and agility, and that a team’s process ambidexterity has a positive effect on inter-team coordination and team innovation, which in turn have a direct impact on team performance. Our findings highlight the importance of process ambidexterity by investigating the enabling role of IT and its outcomes in a team. Our results offer theoretical and practical implications from the perspective of team process ambidexterity.</t>
@@ -15888,6 +16105,11 @@
       <c r="K324" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15939,6 +16161,16 @@
           <t>BSMA0323</t>
         </is>
       </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G326" t="inlineStr">
         <is>
           <t>abstract                                                         Although firms increasingly invest in systems (e.g. ISO, knowledge centres, IT systems) for utilizing stored knowledge and acquiring market information during new product development, few manage to benefit from these investments. To explore this issue, we suggest that firms rely on two distinct types of               knowledge stocks               – procedural and declarative memory – that affect new product short‐term financial performance and creativity in distinct ways. Additionally, we suggest that internal or external               information flows               can have distinct moderating impact on the memory types–product outcomes relationship. Our empirical study of product development activities indicates that there is an inverted U‐shaped relationship between procedural memory and product outcomes as well as a positive relationship between declarative memory and financial performance. Also procedural and declarative memory may work in a               complementary               fashion enhancing both outcomes. Finally, procedural memory is found to reduce the value of internal or external information flows for product creativity. These findings have important implications for the organizational knowledge, capabilities, and product development literatures as well as for practice and they open ways for future research.</t>
@@ -15962,6 +16194,11 @@
       <c r="K326" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18612,7 +18849,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr">
         <is>
           <t>Although the use of generative artificial intelligence (AI) within organizations is becoming increasingly common, research on how to enhance employees' competitive advantage through generative AI use within organizations is very limited. Using a resource-based view model, this study investigates the relationship between generative AI use and employees' competitive advantage, as well as the moderating role of perceived organization support. From an analysis of data from 264 employees from 200 organizations, it is found that work-related generative AI use has a positive effect on employee boundary spanning, which contributes to employee competitive advantage. Secondly, work-related generative AI use also has a positive effect on employee agility, including employee resilience and employee adaptability, which further contributes to employee competitive advantage. However, work-related generative AI use has a positive effect on employee proactivity, while the effect of employee proactivity on employee competitive advantage is not significant. Thirdly, perceived organizational support can enhance the effect between employee boundary spanning and employee competitive advantage. However, it is interesting to observe that perceived organizational support enhances the effect between employee adaptability and employee competitive advantage, while weakening the effect between employee proactivity and employee competitive advantage. It does not exert a moderating effect between employee resilience and employee competitive advantage. These findings can help deepen the current understanding of the relationship between generative AI use in the organization and employee competitive advantage, and provide suggestions for business managers on how to use generative AI to improve employee competitive advantage.</t>
@@ -18655,6 +18891,12 @@
           <t>BSMA0388</t>
         </is>
       </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
           <t>Chronic excessive turnover among information technology (IT) professionals has been costly to firms for decades with annual turnover rates as high as 24% even among Computerworld’s “100 Best Places to Work in IT.” Prior information systems literature has identified two key factors affecting turnover: boundary-spanning roles and low promotability in one’s current firm. We draw on tournament theory, which is primarily concerned with inducing effort in employees, to decompose promotability into two distinct constructs: the likelihood of promotion and benefit from promotion, and demonstrate that each has a distinct role in affecting turnover rates. Our key result is that a job ladder motivating IT professionals with large, infrequent promotions will lead to higher turnover than a job ladder with smaller, more frequent promotions. We describe the conditions under which rearranging the job ladder creates economic value for the firm. We also offer an explanation for the observation that jobs characterized by boundary-spanning activities have higher turnover, and show that such jobs are more sensitive to the effect of likelihood of promotion on turnover. We test our hypotheses on a detailed data set covering 5,704 IT professionals over a five-year period. We confirm that likelihood of promotion has the predicted effects on turnover of IT professionals. A one standard deviation increase in likelihood of promotion decreases turnover by over 99%, consistent with our prediction. The empirical analysis also confirms the predicted effects of boundary spanning activities.</t>
@@ -18678,6 +18920,11 @@
       <c r="K391" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18697,7 +18944,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F392" t="inlineStr"/>
       <c r="G392" t="inlineStr">
         <is>
           <t>Although difficult, complicated, and sometimes discouraging, collaboration is recognized as a viable approach for addressing uncertain, complex and wicked problems. Collaborations can attract resources and increase efficiency, facilitate visions of mutual benefit that can ignite common desires of partners to work across and within sectors, and create shared feelings of responsibility. Collaboration can also promote conceptualized synergy, the sense that something will “be achieved that could not have been attained by any of the organizations acting alone”(Huxham, 2003). However, previous inquiries into the problems encountered in collaborations have not solved an important question: How to enable successful collaboration? Through exploratory sequential mixed-methods research conducted in three empirical studies, I discover how interorganizational collaborations can overcome barriers to innovate and rejuvenate communities and understand the factors and antecedents that influence successful collaboration.</t>
@@ -18797,7 +19043,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr">
         <is>
           <t>Adaptive supply chain partnerships are a key factor in driving the ability of extended enterprise partners to achieve long-term goals in an environment characterized by disruptive environmental shifts. Adaptive extended enterprise arrangements allow participating enterprises to leverage their combined assets for collective exploration and exploitation. In the context of extended enterprises, where significant investments have been directed toward instituting common interfaces, this study examines the question: How does the use of standard electronic business interfaces (SEBIs) enable supply chain partnerships to become more adaptive?             This study conceptualizes the use of SEBIs as a boundary-spanning mechanism that helps overcome boundaries that impede knowledge transfer between enterprises in supply chains. SEBIs enables partners to gain insight into their broader environments, enriching each partner's perspective (enhanced bridging). SEBIs also help strengthen the cooperative ties between partners, motivating each partner to adapt for collective gain (enhanced bonding).             Our research model is empirically tested using data collected from 41 demand-side supply chain partnerships (between original equipment manufacturers (OEMs), distributors, and retailers) in the information technology (IT) industry. The results show that collaborative information exchange (CIE) between supply chain partners mediates the relationship between use of SEBIs and mutual adaptation (MA) and adaptive knowledge creation between supply chain partners. Interestingly, the use of SEBIs is found to be directly associated with MA but only indirectly associated with adaptive knowledge creation.             The study points out that the strategic impacts of SEBIs go well beyond the exchange of transaction information and process integration. It also shows that multilateral, quasi-open, and information exchange–and process linkage–oriented SEBIs can result in both bonding and bridging across supply chain partners without binding them inflexibly to specific partners. Based on the model and results, the study offers practical implications for how SEBIs should be developed, adopted, and used.</t>
@@ -18840,6 +19085,12 @@
           <t>BSMA0392</t>
         </is>
       </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr">
         <is>
           <t>In this study of the business communication that connects an organization with others in its environment, we link boundary spanning with network theory and propose the concept of an extended network of communication. This extended net work is the structure of business communication which flows in work-related ties that organization members maintain both within the organization and across its boundary. We study the relationship between boundary-spanning communication and individual influence in a network with 108 organizational members. We find that boundary spanning correlates with influence, regardless of hierarchical level. There is also a curvilinear relationship between boundary-spanning communication and individual influence. Thus, managers need to balance their communication within and across the organizational boundary.</t>
@@ -18863,6 +19114,11 @@
       <c r="K395" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18882,7 +19138,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr">
         <is>
           <t>Technology transfer’ is a misnomer; this popular phrase and the studies from which it originates often suggest passivity and inertia on the part of developing country recipient firms. This paper, which uses the technological capability building system (TCB) approach as a conceptual framework, suggests that firms in developing countries exercise constrained agency in technological acquisition processes. The evidence discussed here is taken from a study of technological capability accumulation by twenty-six firms in the telecommunication sector of four developing countries: Uganda, Ghana, Tanzania and South Africa. Important insights into technological acquisition by firms in a service sector in developing countries emerged from that study, such as the existence of specific boundary management capabilities for managing relationships with suppliers; confirmation that firms use different mechanisms for acquiring codified and tacit knowledge; and support for the view that technical change and industry features have significant effects on technology acquisition strategies and their effectiveness.</t>
@@ -18925,6 +19180,12 @@
           <t>BSMA0394</t>
         </is>
       </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -18948,6 +19209,11 @@
       <c r="K397" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18962,6 +19228,12 @@
           <t>BSMA0395</t>
         </is>
       </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr"/>
       <c r="G398" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -18985,6 +19257,11 @@
       <c r="K398" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18999,6 +19276,12 @@
           <t>BSMA0396</t>
         </is>
       </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr"/>
       <c r="G399" t="inlineStr">
         <is>
           <t>The authors examined how networks of teams integrate their efforts to succeed collectively. They proposed that integration processes used to align efforts among multiple teams are important predictors of multiteam performance. The authors used a multiteam system (MTS) simulation to assess how both cross-team and within-team processes relate to MTS performance over multiple performance episodes that differed in terms of required interdependence levels. They found that cross-team processes predicted MTS performance beyond that accounted for by within-team processes. Further, cross-team processes were more important for MTS effectiveness when there were high cross-team interdependence demands as compared with situations in which teams could work more independently. Results are discussed in terms of extending theory and applications from teams to multiteam systems.</t>
@@ -19022,6 +19305,11 @@
       <c r="K399" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19036,6 +19324,12 @@
           <t>BSMA0397</t>
         </is>
       </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
           <t>In response to increased complexity of work tasks, flatter organizational structures, and changing environmental conditions, organizational work teams must increasingly coordinate efforts across their boundaries and actively manage key relationships external to the team itself. Despite evidence of the importance of these processes—referred to as team boundary spanning—for both team and organizational success, significant gaps exist in our understanding of the nature of team boundary spanning, how and when these behaviors are carried out by teams, and the resulting impacts of team boundary spanning beyond that of enhanced team performance. Therefore, this article seeks to advance knowledge in this area by offering a taxonomy of team boundary spanning actions, reviewing the existing stream of team boundary spanning literature across multiple levels of analysis, and integrating this body of work with findings and perspectives from other boundary spanning research areas so as to stimulate fruitful avenues for future research.</t>
@@ -19059,6 +19353,11 @@
       <c r="K400" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19073,6 +19372,12 @@
           <t>BSMA0398</t>
         </is>
       </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr"/>
       <c r="G401" t="inlineStr">
         <is>
           <t>As organizations encounter unpredictable external environments, expectations are changing for managers and team leaders toward providing more facilitative, less directive coaching in order to stimulate more flexibility and adaptability. Prior research has underscored the role of team leader supportive coaching behaviors in reinforcing and growing team member capabilities to work independently from the leader. What is not yet understood, however, is if and how supportive coaching behaviors relate to team member engagement in boundary-spanning behaviors, which are team member efforts to establish and maintain relationships with key parties external to their team. This study examines how team leaders’ supportive coaching of boundary spanning—defined as a set of behaviors that (a) encourages team members to engage in frequent and open collaborations with key parties external to the team and (b) grants team members the latitude to engage external parties in ways the team members deem necessary—relates to team member boundary-spanning behavior and job satisfaction through a motivational pathway. We test a hypothesized indirect-effects model within a field sample of 256 engineering employees working in teams. Results indicate that leaders’ supportive coaching of boundary spanning is positively related to team member boundary-spanning self-efficacy, which in turn is positively related to team member engagement in boundary-spanning behavior for their teams. Also, team members who reported more boundary-spanning behavior experienced greater job satisfaction. The findings have important implications for organizations, team leaders, and team members.</t>
@@ -19096,6 +19401,11 @@
       <c r="K401" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19280,6 +19590,12 @@
           <t>BSMA0403</t>
         </is>
       </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
         <is>
           <t>Abstract                                                                                     According to numerous studies across multiple disciplines in the social sciences, business organizations tend to develop adversarial relationships with representatives of the public interest. A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter‐organizational conflict, organizational communication and stakeholder management. Empirical results support the descriptive power of a two‐dimensional model reflecting four relational styles that participating organizations exhibited: avoidance, compliance, co‐optation and negotiation. The two dimensions that constitute the model are cooperativeness and boundary spanning. More importantly, managers who attributed power and legitimacy to public interest group stakeholders reported that their organizations were more likely to cooperate with these stakeholders. On the other hand, managers who perceived public interest groups' claims having                     urgency                     were more likely to develop communicative, boundary spanning relationships with public interest groups but these relationships were less likely to be cooperative. Because unhealthy relationships with these groups can be detrimental to an organization's long‐term prospects, managers must be careful to recognize public interest organizations as potent and legitimate potential allies.                                                                  Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19303,6 +19619,11 @@
       <c r="K406" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19354,6 +19675,16 @@
           <t>BSMA0405</t>
         </is>
       </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G408" t="inlineStr">
         <is>
           <t>Thanks to the pervasive adoption of digital technologies across different industries, “digital-born companies” nowadays play a pivotal role in the current techno-economic scenario. The concurrent sustainability imperative has generated constraints and entrepreneurial opportunities for new ventures. A narrow part of the entrepreneurship literature has analyzed the relationship between the emerging digital phenomenon and the transformative capacity of ICT start-ups as a potential key driver to tackle grand societal challenges due to their ability to alter business models and/ or optimize existing resources. Following this line of reasoning, we analyze how strategic orientation and boundary-spanning activities of ICT start-ups relate to their socio-environmental sustainability. Poisson family estimations (negative binomial and zero-inflated negative binomial) of 172 innovative ICT start-ups based in Italy reveal different driving factors of their socio-environmental sustainability. Our work provides novel insights into the sustainability drivers of digital start-ups, suggesting differentiated strategies for entrepreneurs aimed at fostering socio-environmental sustainability as one of their primary goals. Market strategic orientation is more associated with social sustainability, while technological strategic orientation is more associated with environmental sustainability. The development of a wide portfolio of partnerships seems beneficial only for social sustainability, with no effect on environmental sustainability.</t>
@@ -19377,6 +19708,11 @@
       <c r="K408" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 15
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -10336,7 +10336,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>Drawing on corporate entrepreneurship (CE) and social network research, this study focuses on strategic renewal as a form of CE and examines the impact of boundary-spanning at top and middle management levels on business units’ exploratory innovation. Analyses of multi-source and multi-level data, collected from 72 top managers (TMs) and 397 middle managers (MMs) operating in 34 units of a multi-national organization, indicate that TMs’ boundary-spanning is positively related to units’ exploratory innovation, but also has a cascading effect on MMs by increasing their perceived role conflict. MMs’ role conflict is negatively related to units’ exploratory innovation and thus offsets some of the benefits gained through TMs’ boundary-spanning activities. Taking a configurational perspective on social exchanges at multiple levels, we show that role conflict is reduced by overlapping boundary-spanning ties among TMs and MMs. Surprisingly, MMs’ boundary-spanning does not relate to exploratory innovation. Our study shows that with regard to boundary-spanning, a top-down approach to CE as strategic renewal may be most effective because TMs play a key role in driving exploratory innovation. However, TMs need to be aware of the cascading social liabilities of their boundary-spanning behavior and ensure MMs develop similar networks. We advance ongoing debates in studies about CE and social networks by providing empirically validated insights into who drives strategic renewal and by uncovering the benefits and costs of social exchanges for strategic renewal. Furthermore, we uncover potential causes of mixed findings in network theory research and highlight a remedy to social liabilities.</t>
@@ -10478,7 +10477,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>This article explores the joint production and consumption of health information and advice in the context of NHS Direct, the new telephone health information and advice service. NHS Direct is an atypical call centre environment in so far as its core staff (nurses) are highly skilled professionals. These nurses are required to collaborate closely with, and are to some extent dependent upon, non-professional lower skilled staff (call handlers) to deﬁne and prioritize their work. This introduces a number of tensions between the two groups. Nurses respond to these tensions by engaging in ‘boundary work’, the micropolitical strategies through which work identities and occupational margins are negotiated, to protect their own status. Call handlers are more subject to the pressures of work ‘speed-up’, highly aware of the risks inherent in their role, but are unable to call upon professional status, either in their resistance to managerial imperatives or in their interactions with health consumers. They are required to manage the tension between offering a safe and high quality service, characterized in their training as ‘professional’, and nurses’ boundary work, which positions them as ‘non-professional’. Here we draw on qualitative research, including call interaction data between call handler and consumer, to show how call handlers’ occupation of the contested territory between professional and non-professional status leaves them wide open to the agency of consumers, as consumers attempt to shape the service in their own interests.</t>
@@ -10573,7 +10571,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>Recently, discussion has begun to consider serving the base of the economic pyramid for business and societal benefit. Suggestions for so doing have focused on business model innovation, improving internal capabilities, promoting stronger governance, and providing leapfrog technologies (such as ICT) to promote effective change. We consider the questions of what types of innovation are occurring when businesses and other organizations enter the base of the pyramid and what types of social, economic, and consumer benefits they bring to local communities. We base our findings on an analysis of more than 1,000 cases describing base of the pyramid activities.</t>
@@ -13100,7 +13097,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -13195,7 +13191,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>Innovation has an intrinsic relationship with social networks because it provides a mechanism for knowledge and information to travel freely between individuals. Consequently, there is abundant research linking social networks to innovation. However, two critical gaps still exist. First, most research studies use a structural approach, and less attention is paid to the behavioral dimensions in a network. Secondly, the majority of empirical research focuses on egocentric networks or dyadic relationships between two organizations, instead of the network of organizations as a whole.</t>
@@ -13666,7 +13661,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>Purpose – In today’s digital and post-pandemic era, construction teams can span their boundary to obtain important resources and support in computer-mediated ways. However, the benefits of computer-mediated team boundary spanning (TBS) are mostly assumed. Empirical evidence for these benefits is in lack. Thus, this study attempts to investigate the influence of computer-mediated (instant messaging in this study) TBS on construction project performance and the underlying mechanism.</t>
@@ -13714,7 +13708,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>International joint ventures (IJVs) have become an important source of critical knowledge for multinational enterprises, but little is known about how knowledge can be effectively transferred to parent ﬁrms when the potential for interpartner opportunism still exists. Drawing on attachment theory, we study how boundary-spanning commitments to IJVs may help mitigate interpartner opportunism and facilitate effective knowledge transfer to parents. Speciﬁcally, we argue that knowledge transfer from IJVs to their parents is positively mediated by both boundary spanners’ organizational commitment to IJVs and parent ﬁrms’ resource commitment to IJVs. We test our arguments using survey data collected from 600 dyadic Chinese–foreign managers of 100 IJVs established in China. The results provide evidence that knowledge sharing between boundary spanners in IJVs positively affects their organizational commitment to these IJVs, which in turn positively affects knowledge transfer to parents. Similarly, knowledge sharing between such boundary spanners positively affects parent ﬁrms’ resource commitment to IJVs, which in turn positively affects knowledge transfer to parents. The mediating role of boundary spanners’ organizational commitment is stronger than that of parent ﬁrms’ resource commitment. Collectively, our ﬁndings suggest that commitment-based relational mechanisms are imperative for safeguarding effective knowledge transfer from IJVs to parent ﬁrms.</t>
@@ -13762,7 +13755,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>This paper collects 103 sample firms' 2015 to 2019 data through data envelopment analysis to measure their technical innovation performance and social network analysis to build joint-patent networks and explore knowledge-creating alliance relationships. The article highlights how tacit knowledge recombination works as a mechanism of boundary spanning. It emphasizes the significance of strategic balancing networks' position to improve technical innovation performance and competitiveness of patent-intensive (PI) firms. This research contributes to shedding additional light on the nature of the boundary-spanning mechanism and PI firms' knowledge exchanges. Specifically, it examines how balancing boundaries spanning through joint-patent networks can influence the processes of tacit knowledge transmission and recombination between knowledge-based actors.</t>
@@ -13810,7 +13802,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>Setting the research background in China, this study draws on absorptive capacity, knowledge inertia and prospect theory to show the relationship between R&amp;D capability and innovation performance which comprises exploitation and exploration. We propose that stronger R&amp;D capability promotes exploitation performance but inhibits exploration performance. As exploitation represents immediate interest and exploration represents long-term interest, we introduce the notion of knowledge boundary spanning of R&amp;D network to balance short-term and long-term benefits. The empirical results show that R&amp;D capability and knowledge boundary spanning of R&amp;D network complement each other for explorative innovation while they present trade-offs for exploitative innovation. This study contributes to existing literature on R&amp;D capability–innovation performance, and it further extends our understanding by investigating the impact of knowledge boundary spanning of R&amp;D network on the R&amp;D capacity–innovation performance relationships. In addition, this study provides references on resources configuration to achieve different innovation strategies.</t>
@@ -13858,7 +13849,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>Open innovation is crucial for achieving high-quality and sustainable business growth. However, it remains unclear how prospective boundary-spanning search and responsive boundary-spanning search impact organizational resilience and open innovation in the VUCA (Volatility, Uncertainty, Complexity, and Ambiguity) new normal. Based on the resource-based theory and dynamic capabilities theory, this paper classifies boundaryspanning search into prospective boundary-spanning search and responsive boundary-spanning search to investigates the impact on open innovation and organizational resilience, and analyze the moderating role of big data analytics capability. The empirical study of 293 Chinese smart manufacturing firms indicates that both prospective and responsive boundary-spanning search have an inverted U-shaped impact on open innovation and organizational resilience. Organizational resilience partially mediates the relationships between prospective boundary-spanning search, responsive boundary-spanning search, and open innovation. Moreover, big data analytics capability moderates and flattens the inverted U-shaped relationships between prospective and responsive boundary-spanning search, and organizational resilience. This study explores the intrinsic mechanism of prospective and responsive boundary-spanning search on open innovation through organizational resilience. The findings enrich and expand the research on the antecedents of open innovation.</t>
@@ -13901,6 +13891,16 @@
           <t>BSMA0266</t>
         </is>
       </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G269" t="inlineStr">
         <is>
           <t>No abstract</t>
@@ -13924,6 +13924,11 @@
       <c r="K269" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team-level aggregation. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -13943,7 +13948,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>This study examines the antecedents of job satisfaction, commitment and turnover for 229 information systems development personnel (ISDP) employed by nine companies within several industries. The antecedents studied include boundary spanning, role ambiguity and role conflict. A model of these variables is built and tested via path analysis. A secondary analysis is performed to explore the impacts of task and individual differences on the study variables. The task differences include analytic and programming tasks while the individual differences studied are age, tenure, education and years of data processing experience.</t>
@@ -13991,7 +13995,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
           <t>The relationship between boundary-spanning role activities and conflict management styles was examined with data gathered from 189 project managers who belong to a national professional association. Five conflict management styles and six boundary role activities were measured with a survey instrument constructed from previously developed scales. The conflict management styles measured were integrating, avoiding, dominating, obliging, and compromising. The six boundary role activities measured were gathering, filtering, and transmitting information; transacting; proacting; and protecting. Hypotheses proposing specific relationships between each of the five conflict management styles and the six boundary role activities were tested with the data. Results indicated that unique combinations of boundary role activities are associated with each of the conflict management styles. Further, more cooperative conflict management styles are related to a greater number of boundary role activities that emphasize information sharing and managing relationships. Results also indicated that length of a project manager's experience moderates this relationship in that those with greater experience use more cooperative styles. A revision is suggested to the conflict management style construct.</t>
@@ -14039,7 +14042,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>Owing to their growing numbers and importance, both managers and researchers are increasingly concerned with the work experiences of boundary-spanning employees. Employee perceptions of organizational support *POS) may be particularly relevant to this crucial employee group. Thus reports a study of the relations between two individual-level and two organizationallevel antecedents to boundary-spanner POS. The results indicate that employee gender, amount of formal organizational recognition received, and the quality of task-related training are associated with POS. However, type of employee pay plan is not. Concludes with a discussion of these findings and their implications for effectively managing boundary-spanning employee POS.</t>
@@ -14087,7 +14089,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate a boundary spanning, interprofessional collaboration between advanced practice nurses (APNs) and junior doctors to support junior doctors’ learning and improve patient management during the overtime shift.</t>
@@ -14130,6 +14131,12 @@
           <t>BSMA0271</t>
         </is>
       </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>National Sun Yat-sen University, Kaohsiung, Taiwan This research report compares three differing explanations of the dynamic interrelationships between internal and external innovation-related communication in a new organizational form. In the functional specialization explanation, individuals are said to focus on the mix of internal and/or external communication dictated by their formal positions. The communication stars explanation suggests that individuals maintain similar levels of communication in both networks. The cyclical model posits a more dynamic pattern that shifts back and forth between internal and external communication, depending on the consequences of their prior communication behavior. The new organizational form examined for three years was the Cancer Information Service, a geographically dispersed federal government health information program. Our results indicated that there was a lagged effect for the communication stars explanation.</t>
@@ -14153,6 +14160,11 @@
       <c r="K274" t="inlineStr">
         <is>
           <t>2000</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14172,7 +14184,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>Firms are challenged to achieve organizational goals in an environment of increasingly decentralized information. Cross-functional project teams are employed widely as a strategy to facilitate better coordination, yet projects still fail at a rate of 31% per year. Communication is a leading cause of failure. While inter-team communication has been studied extensively, less is understood about the intra-team communication of a cross-functional project team.</t>
@@ -14220,7 +14231,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>This paper describes one of the first empirical explorations into organisational knowledge creation theory as first elucidated by Nonaka and Takeuchi [1]. We extend the theory and examine it in the inter-organisational context of University-Industry (U-I) collaborative R&amp;D Projects. More specifically, the relationship between enabling conditions and knowledge conversion processes as well as the effects of these processes on the achievement of technological objectives are studied using a sample of 25 U-I collaborative R&amp;D projects into advanced technology. Quantitative and qualitative evidence supports the theory that some enabling conditions are significant for knowledge conversion processes. Furthermore, the presence of the aggregate knowledge processes is positively associated with the achievement of successful technological objectives. The theoretical and practical implications of these findings are discussed.</t>
@@ -14268,7 +14278,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>BACKGROUND: There is a need for a better understanding of how the use of technology to complete work outside regular ofﬁce hours is related to work-life outcomes. Few studies have also investigated how individual differences in work-nonwork boundary management relate to work-life outcomes. OBJECTIVE: This study was conducted to examine how teleworking outside regular ofﬁce hours and individual boundary management relate to work-family conﬂict. METHODS: A web survey was sent to fulltime employees at the headquarters of a multinational high-tech ﬁrm in Sweden. A total of 71 answers were obtained and analyzed using regression analysis. RESULTS: The extent of teleworking after hours was unrelated to work-family conﬂict. However, as previous research has shown, having more permeable boundaries and allowing work to interrupt nonwork behavior was related to higher levels of conﬂict. CONCLUSIONS: The ﬁndings suggest that teleworking after hours is not as problematic in terms of work-family conﬂict as has been reported in previous studies. Furthermore, in order to prevent high levels of work-family conﬂict, it is seemingly beneﬁcial to avoid work interruptions during nonwork behavior.</t>
@@ -14316,7 +14325,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>While the introduction of a new product or service carries considerable risk, incorporating customer input into the new product/service development (NPD) process increases the probability of commercial success. In their boundary spanning role, industrial (B-to-B) salespeople are well suited to serve as a conduit between customers and those inside their company who are largely responsible for the NPD process. The current study investigates the perceptions of sales managers and examines the role the sales force may play in the early stages of the NPD process. An empirical analysis is conducted to determine whether differences exist between organizations that employ key account management (KAM) systems and those that do not employ KAM systems. The findings of this study suggest that salespeople from KAM organizations are better suited to provide input into the NPD process than their non-KAM counterparts.</t>
@@ -15996,7 +16004,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>Purpose – This study investigates the relationship between buyer-supplier top management team (TMT) demographic misalignment (defined as differences in TMT composition based on background, age and gender) and environmental performance (EVP).</t>
@@ -16081,7 +16088,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>As a core organizational resource, business processes are vital for organizational teams. To deal with today’s volatile business environment, organizations need to be ambidextrous in terms of process capabilities. However, little is known about how process ambidexterity, process standardization, and process agility, are enabled by information technology (IT) and related to team-level activities. To fill this gap in the literature, we conducted a field study based on 160 teams of 1081 individuals from seven companies in South Korea. Our results show that IT enables both process standardization and agility, and that a team’s process ambidexterity has a positive effect on inter-team coordination and team innovation, which in turn have a direct impact on team performance. Our findings highlight the importance of process ambidexterity by investigating the enabling role of IT and its outcomes in a team. Our results offer theoretical and practical implications from the perspective of team process ambidexterity.</t>
@@ -16287,6 +16293,12 @@
           <t>BSMA0326</t>
         </is>
       </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>The literature on small stand-alone teams has suggested that decentralization has predominantly positive features. However, in multiteam systems, the presence of other highly interdependent teams adds a level of complexity that may preclude generalizing from teams to multiteam systems. We studied the effects of decentralized planning in 210 multiteam systems, each composed of three six-person, functionally specialized component teams. As has previous research, we find that decentralized planning has positive effects on multiteam system performance, attributable to enhanced proactivity and aspiration levels. However, we also find that the positive effects associated with decentralized planning are offset by the even stronger negative effects attributable to excessive risk seeking and coordination failures. We discuss the implications for theories of intrateam and interteam dynamics, along with the applied implications for designing empowerment interventions in team and multiteam contexts.</t>
@@ -16310,6 +16322,11 @@
       <c r="K329" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The unit of analysis is the multiteam system (N = 210 multiteam systems), not the individual employee. All variables in the correlation matrix represent system-level aggregated constructs.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18896,7 +18913,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
           <t>Chronic excessive turnover among information technology (IT) professionals has been costly to firms for decades with annual turnover rates as high as 24% even among Computerworld’s “100 Best Places to Work in IT.” Prior information systems literature has identified two key factors affecting turnover: boundary-spanning roles and low promotability in one’s current firm. We draw on tournament theory, which is primarily concerned with inducing effort in employees, to decompose promotability into two distinct constructs: the likelihood of promotion and benefit from promotion, and demonstrate that each has a distinct role in affecting turnover rates. Our key result is that a job ladder motivating IT professionals with large, infrequent promotions will lead to higher turnover than a job ladder with smaller, more frequent promotions. We describe the conditions under which rearranging the job ladder creates economic value for the firm. We also offer an explanation for the observation that jobs characterized by boundary-spanning activities have higher turnover, and show that such jobs are more sensitive to the effect of likelihood of promotion on turnover. We test our hypotheses on a detailed data set covering 5,704 IT professionals over a five-year period. We confirm that likelihood of promotion has the predicted effects on turnover of IT professionals. A one standard deviation increase in likelihood of promotion decreases turnover by over 99%, consistent with our prediction. The empirical analysis also confirms the predicted effects of boundary spanning activities.</t>
@@ -19090,7 +19106,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr">
         <is>
           <t>In this study of the business communication that connects an organization with others in its environment, we link boundary spanning with network theory and propose the concept of an extended network of communication. This extended net work is the structure of business communication which flows in work-related ties that organization members maintain both within the organization and across its boundary. We study the relationship between boundary-spanning communication and individual influence in a network with 108 organizational members. We find that boundary spanning correlates with influence, regardless of hierarchical level. There is also a curvilinear relationship between boundary-spanning communication and individual influence. Thus, managers need to balance their communication within and across the organizational boundary.</t>
@@ -19185,7 +19200,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -19233,7 +19247,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F398" t="inlineStr"/>
       <c r="G398" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -19281,7 +19294,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F399" t="inlineStr"/>
       <c r="G399" t="inlineStr">
         <is>
           <t>The authors examined how networks of teams integrate their efforts to succeed collectively. They proposed that integration processes used to align efforts among multiple teams are important predictors of multiteam performance. The authors used a multiteam system (MTS) simulation to assess how both cross-team and within-team processes relate to MTS performance over multiple performance episodes that differed in terms of required interdependence levels. They found that cross-team processes predicted MTS performance beyond that accounted for by within-team processes. Further, cross-team processes were more important for MTS effectiveness when there were high cross-team interdependence demands as compared with situations in which teams could work more independently. Results are discussed in terms of extending theory and applications from teams to multiteam systems.</t>
@@ -19329,7 +19341,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
           <t>In response to increased complexity of work tasks, flatter organizational structures, and changing environmental conditions, organizational work teams must increasingly coordinate efforts across their boundaries and actively manage key relationships external to the team itself. Despite evidence of the importance of these processes—referred to as team boundary spanning—for both team and organizational success, significant gaps exist in our understanding of the nature of team boundary spanning, how and when these behaviors are carried out by teams, and the resulting impacts of team boundary spanning beyond that of enhanced team performance. Therefore, this article seeks to advance knowledge in this area by offering a taxonomy of team boundary spanning actions, reviewing the existing stream of team boundary spanning literature across multiple levels of analysis, and integrating this body of work with findings and perspectives from other boundary spanning research areas so as to stimulate fruitful avenues for future research.</t>
@@ -19377,7 +19388,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F401" t="inlineStr"/>
       <c r="G401" t="inlineStr">
         <is>
           <t>As organizations encounter unpredictable external environments, expectations are changing for managers and team leaders toward providing more facilitative, less directive coaching in order to stimulate more flexibility and adaptability. Prior research has underscored the role of team leader supportive coaching behaviors in reinforcing and growing team member capabilities to work independently from the leader. What is not yet understood, however, is if and how supportive coaching behaviors relate to team member engagement in boundary-spanning behaviors, which are team member efforts to establish and maintain relationships with key parties external to their team. This study examines how team leaders’ supportive coaching of boundary spanning—defined as a set of behaviors that (a) encourages team members to engage in frequent and open collaborations with key parties external to the team and (b) grants team members the latitude to engage external parties in ways the team members deem necessary—relates to team member boundary-spanning behavior and job satisfaction through a motivational pathway. We test a hypothesized indirect-effects model within a field sample of 256 engineering employees working in teams. Results indicate that leaders’ supportive coaching of boundary spanning is positively related to team member boundary-spanning self-efficacy, which in turn is positively related to team member engagement in boundary-spanning behavior for their teams. Also, team members who reported more boundary-spanning behavior experienced greater job satisfaction. The findings have important implications for organizations, team leaders, and team members.</t>
@@ -19420,6 +19430,12 @@
           <t>BSMA0399</t>
         </is>
       </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr">
         <is>
           <t>We adopt a multilevel approach to a paradox that arises when research findings on the performance benefits of team boundary spanning are juxtaposed with earlier work demonstrating the role overload of individuals who span boundaries. Results revealed that individual and team-level factors predicted member boundary-spanning behavior, which increases individual role overload, which then negatively impacts team viability. However, when we aggregated to the team level of analysis, higher levels of boundary spanning resulted in team members' experiencing significantly less role overload. Implications for addressing the boundary-spanning paradox and developing a multilevel theory of team boundary spanning are discussed.</t>
@@ -19443,6 +19459,11 @@
       <c r="K402" t="inlineStr">
         <is>
           <t>2007</t>
+        </is>
+      </c>
+      <c r="P402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19457,6 +19478,12 @@
           <t>BSMA0400</t>
         </is>
       </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr"/>
       <c r="G403" t="inlineStr">
         <is>
           <t>This study examines strategies employed by university administrators and managers to gain compliance from subordinates even as they attempted to increase their workload. These strategies have received comparatively little attention within organizational studies of compliance. The participants in our study included employees at a public university in the Midwest identifying themselves as either “staff/faculty” or “managers/ administrators.” Our findings indicate that when administrators and managers are unable to use formal rewards and punishments they attempt to gain compliance from subordinates through two main strategies that we identify as overtures and interactional trebuchet. Both strategies represent a sequence of interaction that we refer to more generally as “boundary work”—a set of activities through which boundaries on time, resources, and workload are defended or diminished, and for which we provide a model. We draw upon organizational, symbolic interactionist, and dramaturgical theories in the analysis of our data.</t>
@@ -19480,6 +19507,11 @@
       <c r="K403" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19494,6 +19526,12 @@
           <t>BSMA0401</t>
         </is>
       </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr">
         <is>
           <t>Strategic alignment of project portfolios concerns the match between projects in the portfolio and the organization’s strategy. It is often considered either as a selection criterion when creating the project portfolio or as a performance indicator when assessing success. Organizations pursue optimal strategic alignment while retaining responsiveness to changes in the environment. The problem guiding this study is the need to understand how strategic alignment occurs in practice in the work of project portfolio management in the context of multiple project portfolios. We explore large firms’ practices of strategic alignment and cross-portfolio interplay in the innovation project portfolios of three industrial firms. The findings reveal social, mechanistic, and structural practices of portfolios’ strategic alignment and sharing, synergy creation, and boundary-spanning practices in cross-portfolio interplay. Strategic alignment is reported as a dynamic, continuous activity in the work of managers and personnel, with versatile practices that drive both efficiency and renewal.</t>
@@ -19517,6 +19555,11 @@
       <c r="K404" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19595,7 +19638,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
         <is>
           <t>Abstract                                                                                     According to numerous studies across multiple disciplines in the social sciences, business organizations tend to develop adversarial relationships with representatives of the public interest. A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter‐organizational conflict, organizational communication and stakeholder management. Empirical results support the descriptive power of a two‐dimensional model reflecting four relational styles that participating organizations exhibited: avoidance, compliance, co‐optation and negotiation. The two dimensions that constitute the model are cooperativeness and boundary spanning. More importantly, managers who attributed power and legitimacy to public interest group stakeholders reported that their organizations were more likely to cooperate with these stakeholders. On the other hand, managers who perceived public interest groups' claims having                     urgency                     were more likely to develop communicative, boundary spanning relationships with public interest groups but these relationships were less likely to be cooperative. Because unhealthy relationships with these groups can be detrimental to an organization's long‐term prospects, managers must be careful to recognize public interest organizations as potent and legitimate potential allies.                                                                  Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19727,6 +19769,12 @@
           <t>BSMA0406</t>
         </is>
       </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr"/>
       <c r="G409" t="inlineStr">
         <is>
           <t>Salespersons represent an important and challenging set of employees for organizational management. Given frequently high autonomy levels and varied job roles, boundary spanning agents have ample opportunity and motivation to modify/ignore organizational directives. Based on a multi-theoretical perspective, this research sets forth a three-dimensional conceptualization of directive modification intentions and develops and empirically tests a scale designed to better explain this phenomenon while empirically validating its occurrence. Results indicate that boundary spanners have three distinct and relatively stable motivations for modifying/ignoring organizational directives, including customer-, organization-, and self-focused motivations, and that each motivation may potentially relate differently to important antecedent and outcome variables. Managerial and theoretical implications are discussed.</t>
@@ -19750,6 +19798,11 @@
       <c r="K409" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19764,6 +19817,12 @@
           <t>BSMA0407</t>
         </is>
       </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr"/>
       <c r="G410" t="inlineStr">
         <is>
           <t>Despite emerging evidence of contracting for evidence-based practices (EBP), little research has studied how managers lead contract-based human service delivery. A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination (i.e., structuring cross-sector services, coordinating client referrals and eligibility, overseeing EBP implementation) and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning. In conclusion, we underscore the organizational and managerial dimensions of contract-based service delivery.</t>
@@ -19787,6 +19846,11 @@
       <c r="K410" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19838,6 +19902,12 @@
           <t>BSMA0409</t>
         </is>
       </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
           <t>This study is based on a formative evaluation of a case management service for high-intensity service users in Northern England. The evaluation had three main purposes: (i) to assess the quality of the organisational infrastructure; (ii) to obtain a better understanding of the key inﬂuences that played a role in shaping the development of the service; and (iii) to identify potential changes in practice that may help to improve the quality of service provision. The evaluation was informed by Gittell’s relational co-ordination theory, which focuses upon cross-boundary working practices that facilitate task integration. The Assessment of Chronic Illness Care Survey was used to assess the organisational infrastructure and qualitative interviews with front line staff were conducted to explore the key inﬂuences that shaped the development of the service. A high level of strategic commitment and political support for integrated working was identiﬁed. However, the quality of care coordination was variable. The most prominent operational factor that appeared to inﬂuence the scope and quality of care co-ordination was the pattern of interaction between the case managers and their co-workers. The co-ordination of patient care was much more effective in integrated co-ordination networks. Key features included clearly deﬁned, task focussed, relational workspaces with interactive forums where case managers could engage with co-workers in discussions about the management of interdependent care activities. In dispersed co-ordination networks with fewer relational workspaces, the case managers struggled to work as effectively. The evaluation concluded that the creation of ﬂexible and efﬁcient task focused relational workspaces that are systemically managed and adequately resourced could help to improve the quality of care co-ordination, particularly in dispersed networks.</t>
@@ -19861,6 +19931,11 @@
       <c r="K412" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19875,6 +19950,12 @@
           <t>BSMA0410</t>
         </is>
       </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
           <t>This article explores service learning via the lens of activity theory. Through this lens, it is identified as a form of ‘boundary work’ in higher education, with educators identified as ‘boundary workers’. Drawing on the data from a recent study, this paper analyses service learning as an often contradictory and tension filled practice. The ‘expanded community’ and ‘dual but interrelated object’ in the service learning activity system result in many tensions for students and community members alike. This in turn poses significant challenges for boundary workers, and ultimately for the university. The paper concludes by arguing that in order to encourage and value service learning, we need to acknowledge the (new and different) knowledge, values and skills required for playing the role of boundary worker in (boundary) practices such as this.</t>
@@ -19898,6 +19979,11 @@
       <c r="K413" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_2
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -14136,7 +14136,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>National Sun Yat-sen University, Kaohsiung, Taiwan This research report compares three differing explanations of the dynamic interrelationships between internal and external innovation-related communication in a new organizational form. In the functional specialization explanation, individuals are said to focus on the mix of internal and/or external communication dictated by their formal positions. The communication stars explanation suggests that individuals maintain similar levels of communication in both networks. The cyclical model posits a more dynamic pattern that shifts back and forth between internal and external communication, depending on the consequences of their prior communication behavior. The new organizational form examined for three years was the Cancer Information Service, a geographically dispersed federal government health information program. Our results indicated that there was a lagged effect for the communication stars explanation.</t>
@@ -16298,7 +16297,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>The literature on small stand-alone teams has suggested that decentralization has predominantly positive features. However, in multiteam systems, the presence of other highly interdependent teams adds a level of complexity that may preclude generalizing from teams to multiteam systems. We studied the effects of decentralized planning in 210 multiteam systems, each composed of three six-person, functionally specialized component teams. As has previous research, we find that decentralized planning has positive effects on multiteam system performance, attributable to enhanced proactivity and aspiration levels. However, we also find that the positive effects associated with decentralized planning are offset by the even stronger negative effects attributable to excessive risk seeking and coordination failures. We discuss the implications for theories of intrateam and interteam dynamics, along with the applied implications for designing empowerment interventions in team and multiteam contexts.</t>
@@ -16341,6 +16339,12 @@
           <t>BSMA0327</t>
         </is>
       </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>Abstract                            Research Summary               Organizations often struggle to identify promising innovations that balance novelty and feasibility in multidisciplinary domains, yet how does evaluator expertise heterogeneity shape these assessments? This study examines how evaluator expertise influences innovation evaluation through a field experiment with National Aeronautics and Space Administration's (NASA) Astrobee Robotic Arm Challenge, involving 354 evaluators assessing 101 solutions. Domain‐spanning evaluators assign higher novelty ratings while maintaining similar feasibility ratings compared to domain‐specific evaluators. Domain‐adjacent evaluators show higher ratings on both dimensions. Human‐LLM analysis of 3007 evaluator comments reveals a two‐stage process: feasibility filtering (evaluating minimum viability) followed by integrative assessment (evaluating enhancement potential). Different expertise types serve complementary functions: domain‐spanning evaluators recognize enhancement potential while maintaining rigorous standards; domain‐adjacent evaluators show openness to novel approaches; domain‐specific evaluators ensure technical rigor. These findings suggest effective innovation evaluation depends on strategically combining complementary expertise types rather than identifying optimal individual evaluators.                                         Managerial Summary               Organizations often struggle to identify innovations that are both novel and feasible, risking missed breakthroughs or wasted resources. We study how evaluator expertise shapes innovation assessments in a field experiment with NASA, in which 354 evaluators reviewed 101 robotic arm designs. Evaluators with expertise spanning multiple domains recognize more novel yet feasible ideas. Those with single‐domain expertise provide essential technical gatekeeping but overlook cross‐domain improvements, while adjacent‐field experts are more open but less rigorous. Organizations can strengthen innovation selection by strategically combining these complementary expertise types—using domain‐specific experts for initial feasibility screening and domain‐spanning experts to identify integrative opportunities—rather than seeking one “ideal” evaluator.</t>
@@ -16364,6 +16368,11 @@
       <c r="K330" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19435,7 +19444,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr">
         <is>
           <t>We adopt a multilevel approach to a paradox that arises when research findings on the performance benefits of team boundary spanning are juxtaposed with earlier work demonstrating the role overload of individuals who span boundaries. Results revealed that individual and team-level factors predicted member boundary-spanning behavior, which increases individual role overload, which then negatively impacts team viability. However, when we aggregated to the team level of analysis, higher levels of boundary spanning resulted in team members' experiencing significantly less role overload. Implications for addressing the boundary-spanning paradox and developing a multilevel theory of team boundary spanning are discussed.</t>
@@ -19483,7 +19491,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F403" t="inlineStr"/>
       <c r="G403" t="inlineStr">
         <is>
           <t>This study examines strategies employed by university administrators and managers to gain compliance from subordinates even as they attempted to increase their workload. These strategies have received comparatively little attention within organizational studies of compliance. The participants in our study included employees at a public university in the Midwest identifying themselves as either “staff/faculty” or “managers/ administrators.” Our findings indicate that when administrators and managers are unable to use formal rewards and punishments they attempt to gain compliance from subordinates through two main strategies that we identify as overtures and interactional trebuchet. Both strategies represent a sequence of interaction that we refer to more generally as “boundary work”—a set of activities through which boundaries on time, resources, and workload are defended or diminished, and for which we provide a model. We draw upon organizational, symbolic interactionist, and dramaturgical theories in the analysis of our data.</t>
@@ -19531,7 +19538,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr">
         <is>
           <t>Strategic alignment of project portfolios concerns the match between projects in the portfolio and the organization’s strategy. It is often considered either as a selection criterion when creating the project portfolio or as a performance indicator when assessing success. Organizations pursue optimal strategic alignment while retaining responsiveness to changes in the environment. The problem guiding this study is the need to understand how strategic alignment occurs in practice in the work of project portfolio management in the context of multiple project portfolios. We explore large firms’ practices of strategic alignment and cross-portfolio interplay in the innovation project portfolios of three industrial firms. The findings reveal social, mechanistic, and structural practices of portfolios’ strategic alignment and sharing, synergy creation, and boundary-spanning practices in cross-portfolio interplay. Strategic alignment is reported as a dynamic, continuous activity in the work of managers and personnel, with versatile practices that drive both efficiency and renewal.</t>
@@ -19774,7 +19780,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F409" t="inlineStr"/>
       <c r="G409" t="inlineStr">
         <is>
           <t>Salespersons represent an important and challenging set of employees for organizational management. Given frequently high autonomy levels and varied job roles, boundary spanning agents have ample opportunity and motivation to modify/ignore organizational directives. Based on a multi-theoretical perspective, this research sets forth a three-dimensional conceptualization of directive modification intentions and develops and empirically tests a scale designed to better explain this phenomenon while empirically validating its occurrence. Results indicate that boundary spanners have three distinct and relatively stable motivations for modifying/ignoring organizational directives, including customer-, organization-, and self-focused motivations, and that each motivation may potentially relate differently to important antecedent and outcome variables. Managerial and theoretical implications are discussed.</t>
@@ -19822,7 +19827,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F410" t="inlineStr"/>
       <c r="G410" t="inlineStr">
         <is>
           <t>Despite emerging evidence of contracting for evidence-based practices (EBP), little research has studied how managers lead contract-based human service delivery. A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination (i.e., structuring cross-sector services, coordinating client referrals and eligibility, overseeing EBP implementation) and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning. In conclusion, we underscore the organizational and managerial dimensions of contract-based service delivery.</t>
@@ -19865,6 +19869,12 @@
           <t>BSMA0408</t>
         </is>
       </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
           <t>This study explores how pharmacists legitimise the expansion of their clinical work and considers its impact on pharmacists’ professional identity work. In the context of pharmacy in the English NHS, there has been an ongoing policy shift towards pharmacists moving away from ‘medicines supply’ to patient-facing, clinical work since the 1950s. Pharmacists are continuously engaging in ‘identity work’ and ‘boundary work’ to reflect the expansion of their work, which has led to the argument that pharmacists lack a clear professional identity. Drawing insights from linguistics and specifically Van Leeuwen's ‘grammar of legitimation’, this study explains how the Pharmacy Integration Fund, a nationally funded learning programme, provides the discursive strategies for pharmacists to legitimise their identity work as clinicians.</t>
@@ -19888,6 +19898,11 @@
       <c r="K411" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19907,7 +19922,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
           <t>This study is based on a formative evaluation of a case management service for high-intensity service users in Northern England. The evaluation had three main purposes: (i) to assess the quality of the organisational infrastructure; (ii) to obtain a better understanding of the key inﬂuences that played a role in shaping the development of the service; and (iii) to identify potential changes in practice that may help to improve the quality of service provision. The evaluation was informed by Gittell’s relational co-ordination theory, which focuses upon cross-boundary working practices that facilitate task integration. The Assessment of Chronic Illness Care Survey was used to assess the organisational infrastructure and qualitative interviews with front line staff were conducted to explore the key inﬂuences that shaped the development of the service. A high level of strategic commitment and political support for integrated working was identiﬁed. However, the quality of care coordination was variable. The most prominent operational factor that appeared to inﬂuence the scope and quality of care co-ordination was the pattern of interaction between the case managers and their co-workers. The co-ordination of patient care was much more effective in integrated co-ordination networks. Key features included clearly deﬁned, task focussed, relational workspaces with interactive forums where case managers could engage with co-workers in discussions about the management of interdependent care activities. In dispersed co-ordination networks with fewer relational workspaces, the case managers struggled to work as effectively. The evaluation concluded that the creation of ﬂexible and efﬁcient task focused relational workspaces that are systemically managed and adequately resourced could help to improve the quality of care co-ordination, particularly in dispersed networks.</t>
@@ -19955,7 +19969,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
           <t>This article explores service learning via the lens of activity theory. Through this lens, it is identified as a form of ‘boundary work’ in higher education, with educators identified as ‘boundary workers’. Drawing on the data from a recent study, this paper analyses service learning as an often contradictory and tension filled practice. The ‘expanded community’ and ‘dual but interrelated object’ in the service learning activity system result in many tensions for students and community members alike. This in turn poses significant challenges for boundary workers, and ultimately for the university. The paper concludes by arguing that in order to encourage and value service learning, we need to acknowledge the (new and different) knowledge, values and skills required for playing the role of boundary worker in (boundary) practices such as this.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 16
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11070,6 +11070,12 @@
           <t>BSMA0203</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>Personnel is one of the most important resources for the performance of Information Systems (IS) and Information Center (IC) organizations. The scarcity of new employees, the difficulty of training and a high turnover make personnel management in these areas a difficult problem. For IS employees, the relationships between job satisfaction, organizational commitment and intention to leave the organization have been established. Because the size of the investment and the number of organizations establishing IC organizations are growing dramatically, it has become important to understand the determinants of turnover intentions for IC as well as IS employees. Are IC employees similar to their IS counterparts? Or, is their nature basically different, as some studies have suggested? This study examines the differences between IS and IC employees in terms of demographic characteristics, participation on boundary spanning activities, role stressors, overall job satisfaction, organizational commitment and turnover intentions. The differences are found to be significant and call for special attention from IC managers to manage more properly their personnel resources. IC employees were found to participate more extensively in boundary spanning activities, experienced more role stressors (role ambiguity and role conflict), were less satisfied with their jobs and less committed to their organization. The findings also demonstrate the importance of organizational commitment as an intervening variable in models of turnover. While overall job satisfaction had both direct and indirect effects on turnover intentions among IC employees, for IS personnel it had only indirect effects through organizational commitment. The effects of role stressors and boundary spanning activities were found to be indirect via overall job satisfaction and organizational commitment for both IC and IS employees. The implications of these findings for practicing managers and for future research are discussed.</t>
@@ -11093,6 +11099,11 @@
       <c r="K206" t="inlineStr">
         <is>
           <t>1992</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Included. The study explicitly measures intra-organizational boundary spanning behavior (information systems employees interacting with other internal departments) and provides an extractable zero-order correlation with intention to leave. Verbatim Evidence: [Sample] "A questionnaire was distributed to 2548 members of the Association for Computing Machinery (ACM) in Pennsylvania, Delaware, and Southern New Jersey. The sample was chosen because members of ACM represent a wide variety of jobs and organizational settings. Five hundred and seventeen questionnaires (response rate of 20.3%) were returned to the researchers. This response rate appears to be consistent with other mail surveys Fifty three questionnaires were eliminated due to missing data or subject unsuitability (retired employees and faculty at academic institutions), leaving a final sample of 464 employees (response rate of 18.2%). The participants in this study held a variety of positions within the computer field reflecting considerable heterogeneity within the MIS profession." [Measures] "Boundary spanning activities, defined as those by which employees interact and communicate with others outside their departments, including formal and informal written and oral communications, were measured by modifying the ten-item scale developed by Miles and Perreault [12] and used by Baroudi [2]. Each item (e.g., 'assist other units in determining appropriate uses of information technology'; 'recommend new applications of information technology to top management') was scored on a five-point scale ranging from (1) not part of my job to (5) a very significant part of my job. The internal consistency reliability of the scale was 0.91." [Results] "Boundary spanning activities for IS personnel were found to be negatively correlated with the intention to leave the organization."</t>
         </is>
       </c>
     </row>
@@ -11181,6 +11192,16 @@
           <t>BSMA0206</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G209" t="inlineStr">
         <is>
           <t>Leadership has been suggested to be an important factor affecting innovation. A number of studies have shown that transformational leadership positively influences organizational innovation. However, there is a lack of studies examining the contextual conditions under which this effect occurs or is augmented. Therefore, this study aimed to investigate the impact of transformational leadership on organizational innovation and to determine whether internal and external support for innovation as contextual conditions influence this effect. Organizational innovation was conceptualized as the tendency of the organization to develop new or improved products or services and its success in bringing those products or services to the market. Transformational leadership was hypothesized to have a positive influence on organizational innovation. Furthermore, this effect was proposed to be moderated by internal support for innovation, which refers to an innovation supporting climate and adequate resources allocated to innovation. Support received from external organizations for the purposes of knowledge and resource acquisition was also proposed to moderate the relationship between transformational leadership and organizational innovation. To test these hypotheses, data were collected from 163 research and development (R&amp;D) employees and managers of 43 micro‐ and small‐sized Turkish entrepreneurial software development companies. Two separate questionnaires were used to collect the data. Employees' questionnaires included measures of transformational leadership and internal support for innovation, whereas managers' questionnaires included questions about product innovations of their companies and the degree of support they received from external institutions. Organizational innovation was measured with a market‐oriented criterion developed specifically for developing countries and newly developing industries. Hierarchical regression analysis was used to test the hypothesized effects. The results of the analysis provided support for the positive influence of transformational leadership on organizational innovation. This finding is significant because this positive effect was identified in micro‐ and small‐sized companies, whereas previous research focused mainly on large companies. In addition, external support for innovation was found to significantly moderate this effect. Specifically, the relationship between transformational leadership and organizational innovation was stronger when external support was at high levels than when there was no external support. This study is the first to investigate and empirically show the importance of this contextual condition for organizational innovation. The moderating effect of internal support for innovation, however, was not significant. This study shows that transformational leadership is an important determinant of organizational innovation and encourages managers to engage in transformational leadership behaviors to promote organizational innovation. In line with this, transformational leadership, which is heavily suggested to be a subject of management training and development in developed countries, should also be incorporated into such programs in developing countries. Moreover, this study highlights the importance of external support in the organizational innovation process. The results suggest that technical and financial support received from outside the organization can be a more important contextual influence in boosting up innovation than an innovation‐supporting internal climate. Therefore, managers, particularly of micro‐ and small‐sized companies, should play external roles such as boundary spanning and should build relationships with external institutions that provide technical and financial support. The findings of this study are especially important for managers of companies that plan to or currently operate in countries with developing economies.</t>
@@ -11204,6 +11225,11 @@
       <c r="K209" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11218,6 +11244,12 @@
           <t>BSMA0207</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>Organizations have recognized that effective informal leadership is a source of competitive advantage and invest heavily in leadership development efforts. Moreover, because of historical shifts in the nature of work, this informal leadership often takes the form of inter-unit boundary spanning. Because of these two developments, discretionary boundary spanning (DBS) between units has increasingly become a critical, dynamic, bottom-up activity where individuals lacking formal authority step up and take on informal leadership responsibilities. In this study, we draw upon Simmelian Tie Theory (STT) to examine the relationship between different types of DBS and formal leaders’ perceptions of a subordinate’s informal leadership and performance. We empirically document that a small number of closed task-oriented and closed friendship-oriented DBSs are instrumental in helping individuals demonstrate informal leadership. However, we also show that DBS places constraints on informal leadership when closed ties become too numerous. This results in an inverted-U relationship between the number of closed DBS ties and perceptions of leadership where the apex (i.e., point of overembeddedness) emerges at a smaller number for friendship-oriented DBS relative to the apex for taskoriented DBSs. We discuss the theoretical implications of these results, as well as the practical implications for managers of organizations.</t>
@@ -11241,6 +11273,11 @@
       <c r="K210" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Valid individual-level intra-organizational boundary spanning behavior (DBS) measured via social network task-oriented and friendship ties, with a zero-order correlation matrix provided.. Verbatim Evidence: [Sample] "This resulted in the recruitment of 181 full-time employees from 55 different teams (M = 5.74, SD = 3.69)." [Procedure] "Together, 132 out of the 149 employees who had completed the relational survey also received external ratings of informal leadership. This set of 132 individuals comprised our final sample for data analysis." [Measures] "We tasked respondents to characterize whether the person identified in the first stage of the procedure was (a) someone with whom they exchanged work-related information and/or (b) someone whom they considered a friend (or neither)." [Closed DBS Ties] "Because we are interested in ties that bridged different teams, we defined closed DBS ties as occurring when (a) individual i and individual j are in different teams, (b) they have a reciprocated, confirmed tie, and (c) both have a reciprocated, confirmed tie in common with at least one other individual in a team different from both individual i and individual j." [Results] "Table 1 Descriptive Statistics and Correlations"</t>
         </is>
       </c>
     </row>
@@ -16255,6 +16292,12 @@
           <t>BSMA0325</t>
         </is>
       </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>We examine leadership over-emergence, defined as instances when the level of one’s leadership emergence is higher than the level of one’s leadership effectiveness, in a sample of intact self-managing teams who worked together for a period of seven months. We draw from Gender Role Theory and Expectancy Violation Theory to examine the role of gender in predicting leadership over-emergence. Building on arguments from Gender Role Theory, we find that all else equal, men over-emerge as leaders. However, Expectancy Violation Theory suggests that women are likely to benefit from a countervailing bias. Specifically, women are attributed with higher levels of leadership emergence than men when they engage in agentic leadership behaviors—even if the level of the behaviors exhibited by men is exactly the same. Because the impact of these behaviors on leadership effectiveness is not contingent on gender, however, women who engage in more task behaviors and boundary spanning behaviors in self-managing teams also over-emerge as leaders. We discuss the implications of this study for Gender Role Theory and Expectancy Violation Theory, along with practical implications for managing the problem of leadership over-emergence in work groups.</t>
@@ -16278,6 +16321,11 @@
       <c r="K328" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16344,7 +16392,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>Abstract                            Research Summary               Organizations often struggle to identify promising innovations that balance novelty and feasibility in multidisciplinary domains, yet how does evaluator expertise heterogeneity shape these assessments? This study examines how evaluator expertise influences innovation evaluation through a field experiment with National Aeronautics and Space Administration's (NASA) Astrobee Robotic Arm Challenge, involving 354 evaluators assessing 101 solutions. Domain‐spanning evaluators assign higher novelty ratings while maintaining similar feasibility ratings compared to domain‐specific evaluators. Domain‐adjacent evaluators show higher ratings on both dimensions. Human‐LLM analysis of 3007 evaluator comments reveals a two‐stage process: feasibility filtering (evaluating minimum viability) followed by integrative assessment (evaluating enhancement potential). Different expertise types serve complementary functions: domain‐spanning evaluators recognize enhancement potential while maintaining rigorous standards; domain‐adjacent evaluators show openness to novel approaches; domain‐specific evaluators ensure technical rigor. These findings suggest effective innovation evaluation depends on strategically combining complementary expertise types rather than identifying optimal individual evaluators.                                         Managerial Summary               Organizations often struggle to identify innovations that are both novel and feasible, risking missed breakthroughs or wasted resources. We study how evaluator expertise shapes innovation assessments in a field experiment with NASA, in which 354 evaluators reviewed 101 robotic arm designs. Evaluators with expertise spanning multiple domains recognize more novel yet feasible ideas. Those with single‐domain expertise provide essential technical gatekeeping but overlook cross‐domain improvements, while adjacent‐field experts are more open but less rigorous. Organizations can strengthen innovation selection by strategically combining these complementary expertise types—using domain‐specific experts for initial feasibility screening and domain‐spanning experts to identify integrative opportunities—rather than seeking one “ideal” evaluator.</t>
@@ -16387,6 +16434,12 @@
           <t>BSMA0328</t>
         </is>
       </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
           <t>Nonprofit organizations have historically been seen as a vanguard in U.S. civil society, supplying places and spaces for innovation and change to flourish. According to the Competing Values Culture Framework (CVCF), a developmental organizational culture, characterized by innovation and risk-taking, may help organizations respond to changes in their operating environments and be more effective at boundary-spanning activities, such as fostering external support, acquiring resources, and spurring growth. Despite its importance, the culture–effectiveness relationship has not been studied sufficiently in nonprofit organizations. The exploratory study described in this article examines the links between developmental culture and nonprofit organizational effectiveness. Results suggest that nonprofit executive directors see organizational culture as more than a phenomenon to be experienced. Specifically, findings indicate that executive directors perceive there to be a positive and significant relationship between developmental culture and how effective their organization is at performing boundary-spanning activities. The practical and theoretical implications of this finding are discussed.</t>
@@ -16410,6 +16463,11 @@
       <c r="K331" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P331" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study uses executive directors as key informants to evaluate the organizational-level effectiveness of boundary-spanning activities (e.g., increasing funding, influencing policy), rather than evaluating individual-level boundary spanning behavior.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19686,6 +19744,12 @@
           <t>BSMA0404</t>
         </is>
       </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
           <t>The rapid growth in the use of teams and multiple team membership has led more organizations to structure work around dynamic teams, characterized by short lifespans and fluid membership boundaries. This approach to organizing work makes it difficult for teams to work efficiently or to support the learning and growth of members. Given the importance of productivity and learning, we ask how these processes can be supported in dynamic teams. We do so in a randomized controlled field experiment conducted with 91 teams in a teaching hospital, a context in which physician trainees must learn while providing patient care in dynamic teams of care providers. We randomly assigned physician teams, or “core” teams, to launch their work with an intervention focused either on internal coordination among the core team members or on external coordination with a changing cast of external contributors such as nurses and specialists. We measured resulting levels of internal and external coordination over teams’ week-long lifespans and observed that external coordination was associated with improved team efficiency, whereas internal coordination was associated with improved individual learning. Post hoc exploratory analysis suggested that individual learning was highest when teams achieved high levels of both internal and external coordination, and it was positively correlated with improvement in the team’s patients’ average length of hospital stay. We discuss the implications of the demonstrated causal effects of team launches, along with our exploratory findings, for the management of dynamic teams and the opportunities to mitigate potential trade-offs between learning and productivity.</t>
@@ -19709,6 +19773,11 @@
       <c r="K407" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19874,7 +19943,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
           <t>This study explores how pharmacists legitimise the expansion of their clinical work and considers its impact on pharmacists’ professional identity work. In the context of pharmacy in the English NHS, there has been an ongoing policy shift towards pharmacists moving away from ‘medicines supply’ to patient-facing, clinical work since the 1950s. Pharmacists are continuously engaging in ‘identity work’ and ‘boundary work’ to reflect the expansion of their work, which has led to the argument that pharmacists lack a clear professional identity. Drawing insights from linguistics and specifically Van Leeuwen's ‘grammar of legitimation’, this study explains how the Pharmacy Integration Fund, a nationally funded learning programme, provides the discursive strategies for pharmacists to legitimise their identity work as clinicians.</t>
@@ -20011,6 +20079,16 @@
           <t>BSMA0411</t>
         </is>
       </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G414" t="inlineStr">
         <is>
           <t>The vast majority of research on self‐monitoring in the workplace focuses on the benefits that accrue to chameleon‐like high self‐monitors (relative to true‐to‐themselves low self‐monitors). In this study, we depart from the mainstream by focusing on a potential liability of being a high self‐monitor: high levels of experienced role conflict. We hypothesize that high self‐monitors tend to choose work situations that, although consistent with the expression of their characteristic personality, inherently involve greater role conflict (i.e. competing role expectations from different role senders). Data collected from a 116‐member high‐tech firm showed support for this mediation hypothesis: relative to low self‐monitors, high self‐monitors tended to experience greater role conflict in work organizations because high self‐monitors were more likely to occupy boundary spanning positions. To help draw a more realistic and balanced portrait of self‐monitoring in the workplace, we call for more theoretically grounded research on the price chameleons pay.</t>
@@ -20034,6 +20112,11 @@
       <c r="K414" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -20914,6 +20997,12 @@
           <t>BSMA0430</t>
         </is>
       </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
           <t>The management of quality and development of effective cross-functional cooperation have assumed a new strate gic importance over the past decade. However, many com panies have reported that quality strategies have failed to deliver anticipated performance benefits and that ineffec tive interfunctional relationships may be to blame. This study explores marketing-quality interfunctional relation ships as a potential source of quality strategy implemen tation failure at the strategic business unit (SBU) level. This study focuses on interdepartmental connectedness, communication and conflict between marketing and qual ity, and the antecedents and consequences of these dimen sions of interfunctional interaction. Using data from a pooled response mail survey, the results suggest that mar keting-quality interactions are associated with senior management quality leadership, strategic quality plan ning process, and control system characteristics. Inter-functional interactions between marketing and quality are found to be only weakly related to relative quality, market performance, and financial performance outcomes.</t>
@@ -20937,6 +21026,11 @@
       <c r="K433" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -20951,6 +21045,12 @@
           <t>BSMA0431</t>
         </is>
       </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
           <t>Boundary spanning research is increasing recognition among scholars and policymakers due to its potential in generating novel and breakthrough scientific contributions. However, while previous research mainly investigated its effect for the scientific domain, less is known about how boundary spanning approaches in science are related to technology transfer activities. To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council under the 7th Framework Programme and Horizon 2020 Programme in the period 2008–2016. Our results show that boundary spanning research projects and the probability to generate technological impact through patent citations are linked through an inverted U-shape relation, thus recognizing both benefits and costs to this research approach. Moreover, as research integrates knowledge from more diverse scientific domains, its technological applications expand correspondingly across a broader range of technical fields. Finally, we show that these relations change according to the seniority of the researcher performing the scientific activity.</t>
@@ -20974,6 +21074,11 @@
       <c r="K434" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -20988,6 +21093,16 @@
           <t>BSMA0432</t>
         </is>
       </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G435" t="inlineStr">
         <is>
           <t>The increasing prevalence of team-based organizations places a premium on leadership that will “mind the gap” and enable smooth synchronization of activities across multiple distinct teams. Prior work shows that leaders can be trained to directly facilitate between-team coordination processes. Yet, relatively little is known about the intervening psychological mechanisms that enable between-team coordination. Here, we advance multiteam-interaction mental models—cognitive structures containing knowledge of appropriate between-team activities—as one mechanism that facilitates coordination among multiple teams. We use leader and team cognition data gathered in DeChurch and Marks' (2006) MTS study to test these ideas. Results reveal leaders' multiteam-interaction mental model accuracy “transfers” to teams through strategic communication, and leader strategic communication enables between-team coordination by promoting accuracy in followers' mental models. This study highlights the importance of leadership for developing collective cognition that allows teams to “scale up” from small stand-alone teams to larger and more complex systems.</t>
@@ -21011,6 +21126,11 @@
       <c r="K435" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_3
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11075,7 +11075,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>Personnel is one of the most important resources for the performance of Information Systems (IS) and Information Center (IC) organizations. The scarcity of new employees, the difficulty of training and a high turnover make personnel management in these areas a difficult problem. For IS employees, the relationships between job satisfaction, organizational commitment and intention to leave the organization have been established. Because the size of the investment and the number of organizations establishing IC organizations are growing dramatically, it has become important to understand the determinants of turnover intentions for IC as well as IS employees. Are IC employees similar to their IS counterparts? Or, is their nature basically different, as some studies have suggested? This study examines the differences between IS and IC employees in terms of demographic characteristics, participation on boundary spanning activities, role stressors, overall job satisfaction, organizational commitment and turnover intentions. The differences are found to be significant and call for special attention from IC managers to manage more properly their personnel resources. IC employees were found to participate more extensively in boundary spanning activities, experienced more role stressors (role ambiguity and role conflict), were less satisfied with their jobs and less committed to their organization. The findings also demonstrate the importance of organizational commitment as an intervening variable in models of turnover. While overall job satisfaction had both direct and indirect effects on turnover intentions among IC employees, for IS personnel it had only indirect effects through organizational commitment. The effects of role stressors and boundary spanning activities were found to be indirect via overall job satisfaction and organizational commitment for both IC and IS employees. The implications of these findings for practicing managers and for future research are discussed.</t>
@@ -11249,7 +11248,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>Organizations have recognized that effective informal leadership is a source of competitive advantage and invest heavily in leadership development efforts. Moreover, because of historical shifts in the nature of work, this informal leadership often takes the form of inter-unit boundary spanning. Because of these two developments, discretionary boundary spanning (DBS) between units has increasingly become a critical, dynamic, bottom-up activity where individuals lacking formal authority step up and take on informal leadership responsibilities. In this study, we draw upon Simmelian Tie Theory (STT) to examine the relationship between different types of DBS and formal leaders’ perceptions of a subordinate’s informal leadership and performance. We empirically document that a small number of closed task-oriented and closed friendship-oriented DBSs are instrumental in helping individuals demonstrate informal leadership. However, we also show that DBS places constraints on informal leadership when closed ties become too numerous. This results in an inverted-U relationship between the number of closed DBS ties and perceptions of leadership where the apex (i.e., point of overembeddedness) emerges at a smaller number for friendship-oriented DBS relative to the apex for taskoriented DBSs. We discuss the theoretical implications of these results, as well as the practical implications for managers of organizations.</t>
@@ -11329,6 +11327,16 @@
           <t>BSMA0209</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G212" t="inlineStr">
         <is>
           <t>Knowledge gathering can create problems as well as benefits for project teams in work environments characterized by overload, ambiguity, and politics. This paper proposes that the value of knowledge gathering in such environments is greater under conditions that enhance team processing, sensemaking, and buffering capabilities. The hypotheses were tested using independent quality ratings of 96 projects and survey data from 485 project-team members collected during a multimethod field study. The findings reveal that three capability-enhancing conditions moderated the relationship between knowledge gathering and project quality: slack time, organizational experience, and decision-making autonomy. More knowledge gathering helped teams to perform more effectively under favorable conditions but hurt performance under conditions that limited their capabilities to utilize that knowledge successfully. Implications for theory and research on knowledge and learning in organizations, team effectiveness, and organizational design are discussed.</t>
@@ -11352,6 +11360,11 @@
       <c r="K212" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Team-level analysis. Verbatim Evidence: [Team-level analysis]. Verbatim Evidence: "[Methods] Data from the 485 members of the 96 qualifying teams were used to construct the team-level measures below; both core and noncore member responses were used because the contributions and views of each were important to project quality (Hackman 2002)." [Methods] "The responses to all eight questions were averaged across all the members of each team to create an aggregate measure of the amount of external knowledge gathered with a Cronbach's alpha of 0.85 (knowledge gathering)." [Results] "Table 1 Descriptive Statistics and Bivariate Correlations (n = 96)"</t>
         </is>
       </c>
     </row>
@@ -16255,6 +16268,12 @@
           <t>BSMA0324</t>
         </is>
       </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>This study draws on theories of collective action and organizational ecology to investigate a particular type of voluntary association: mixed-mode groups. Mixed-mode groups are created and organized online to meet physically in geographically deﬁned ways. An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups. Analysis shows that even when a mixed-mode group implements strategies focused on internal group processes, it beneﬁts from tapping into its external networks to obtain resources for group operation. Also, the differential impacts of internal and external strategies indicate that in the case of environment-prone mixed-mode groups, implementation of internal strategies alone, with or without solicited external networking resources, is helpful for generating positive group outcomes. Together, these results establish that boundary spanning represents not only a type of strategic action to obtain resources and produce positive outcomes but also an inherent and deﬁning mechanism of contemporary voluntary groups for engaging in collective action.</t>
@@ -16278,6 +16297,11 @@
       <c r="K327" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16297,7 +16321,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>We examine leadership over-emergence, defined as instances when the level of one’s leadership emergence is higher than the level of one’s leadership effectiveness, in a sample of intact self-managing teams who worked together for a period of seven months. We draw from Gender Role Theory and Expectancy Violation Theory to examine the role of gender in predicting leadership over-emergence. Building on arguments from Gender Role Theory, we find that all else equal, men over-emerge as leaders. However, Expectancy Violation Theory suggests that women are likely to benefit from a countervailing bias. Specifically, women are attributed with higher levels of leadership emergence than men when they engage in agentic leadership behaviors—even if the level of the behaviors exhibited by men is exactly the same. Because the impact of these behaviors on leadership effectiveness is not contingent on gender, however, women who engage in more task behaviors and boundary spanning behaviors in self-managing teams also over-emerge as leaders. We discuss the implications of this study for Gender Role Theory and Expectancy Violation Theory, along with practical implications for managing the problem of leadership over-emergence in work groups.</t>
@@ -16439,7 +16462,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
           <t>Nonprofit organizations have historically been seen as a vanguard in U.S. civil society, supplying places and spaces for innovation and change to flourish. According to the Competing Values Culture Framework (CVCF), a developmental organizational culture, characterized by innovation and risk-taking, may help organizations respond to changes in their operating environments and be more effective at boundary-spanning activities, such as fostering external support, acquiring resources, and spurring growth. Despite its importance, the culture–effectiveness relationship has not been studied sufficiently in nonprofit organizations. The exploratory study described in this article examines the links between developmental culture and nonprofit organizational effectiveness. Results suggest that nonprofit executive directors see organizational culture as more than a phenomenon to be experienced. Specifically, findings indicate that executive directors perceive there to be a positive and significant relationship between developmental culture and how effective their organization is at performing boundary-spanning activities. The practical and theoretical implications of this finding are discussed.</t>
@@ -19638,6 +19660,12 @@
           <t>BSMA0402</t>
         </is>
       </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr">
         <is>
           <t>Software project teams are often faced with the potential for changing
@@ -19685,6 +19713,11 @@
           <t>2006</t>
         </is>
       </c>
+      <c r="P405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -19749,7 +19782,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
           <t>The rapid growth in the use of teams and multiple team membership has led more organizations to structure work around dynamic teams, characterized by short lifespans and fluid membership boundaries. This approach to organizing work makes it difficult for teams to work efficiently or to support the learning and growth of members. Given the importance of productivity and learning, we ask how these processes can be supported in dynamic teams. We do so in a randomized controlled field experiment conducted with 91 teams in a teaching hospital, a context in which physician trainees must learn while providing patient care in dynamic teams of care providers. We randomly assigned physician teams, or “core” teams, to launch their work with an intervention focused either on internal coordination among the core team members or on external coordination with a changing cast of external contributors such as nurses and specialists. We measured resulting levels of internal and external coordination over teams’ week-long lifespans and observed that external coordination was associated with improved team efficiency, whereas internal coordination was associated with improved individual learning. Post hoc exploratory analysis suggested that individual learning was highest when teams achieved high levels of both internal and external coordination, and it was positively correlated with improvement in the team’s patients’ average length of hospital stay. We discuss the implications of the demonstrated causal effects of team launches, along with our exploratory findings, for the management of dynamic teams and the opportunities to mitigate potential trade-offs between learning and productivity.</t>
@@ -21002,7 +21034,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
           <t>The management of quality and development of effective cross-functional cooperation have assumed a new strate gic importance over the past decade. However, many com panies have reported that quality strategies have failed to deliver anticipated performance benefits and that ineffec tive interfunctional relationships may be to blame. This study explores marketing-quality interfunctional relation ships as a potential source of quality strategy implemen tation failure at the strategic business unit (SBU) level. This study focuses on interdepartmental connectedness, communication and conflict between marketing and qual ity, and the antecedents and consequences of these dimen sions of interfunctional interaction. Using data from a pooled response mail survey, the results suggest that mar keting-quality interactions are associated with senior management quality leadership, strategic quality plan ning process, and control system characteristics. Inter-functional interactions between marketing and quality are found to be only weakly related to relative quality, market performance, and financial performance outcomes.</t>
@@ -21050,7 +21081,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
           <t>Boundary spanning research is increasing recognition among scholars and policymakers due to its potential in generating novel and breakthrough scientific contributions. However, while previous research mainly investigated its effect for the scientific domain, less is known about how boundary spanning approaches in science are related to technology transfer activities. To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council under the 7th Framework Programme and Horizon 2020 Programme in the period 2008–2016. Our results show that boundary spanning research projects and the probability to generate technological impact through patent citations are linked through an inverted U-shape relation, thus recognizing both benefits and costs to this research approach. Moreover, as research integrates knowledge from more diverse scientific domains, its technological applications expand correspondingly across a broader range of technical fields. Finally, we show that these relations change according to the seniority of the researcher performing the scientific activity.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 17
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11033,6 +11033,12 @@
           <t>BSMA0202</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
           <t>The definition of innovation varies from individual to individual and between individual and the team or the team and an organization. The perception of innovation and how individuals define innovation can make an organization stay competitive or go out of business. Research had shown that a traditional approach of idea generation as innovation at well intentioned organizations afforded success only 10% of the time after three years. In forming and managing project teams, which are made up of individuals or selling a service or product to a certain demography it is important and beneficial to understand their perception of innovation and if they see innovation as new, change or improvement. This study is built upon the earlier work of Zhuang (1995), Zhuang, Williamson, and Carter (1999), and McLaughlin and (2013). Prior research conducted by Caraballo and McLaughlin (2012) focused on understanding the perception of innovation as defined or understood by a homogeneous demography of Latino American professionals. This dissertation furthers the research conducted by Caraballo and McLaughlin (2012) with a focus on comprehending how a homogenous group Indian American professionals in the United States perceive or define innovation into the three categories of new, improve and change. While innovation may be understood by individuals as a multi-dimensional construct, the research tried to identify the relationship between perceptions, and gender, age and job function for the homogenous group of Indian Americans in the United States. The research followed the approach and methodology used by Caraballo and McLaughlin (2012) and the study is quantitative, exploratory and used web-based surveys to gather responses from respondents.</t>
@@ -11056,6 +11062,11 @@
       <c r="K205" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11290,6 +11301,16 @@
           <t>BSMA0208</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G211" t="inlineStr">
         <is>
           <t>With the emergence of "boundaryless organizations" and the increase in boundary-spanning activities, the sustainable development of organizations has been affected. Effectively promoting employees to engage in boundaryspanning activities has become of great practical significance. Besides, performance pressure has become a prevalent workplace stressor, significantly impacting employees' work behaviors. Therefore, drawing upon the cognitive-affective processing system theory and stressor-strain relationship theory, this study aims to investigate the mechanisms and boundary conditions of performance pressure on employee boundaryspanning behavior. Data collected from 336 questionnaires at two different time points is analyzed using bootstrapping and hierarchical regression to test hypotheses. The results indicate that performance pressure boosts employee boundary-spanning behavior by enhancing cognitive flexibility, while hindering this behavior by producing obsessive work passion. Moreover, achievement orientation plays a key role in moderating the impact of performance pressure on cognitive flexibility and obsessive work passion. Specifically, achievement orientation positively moderates the link between performance pressure and cognitive flexibility, while negatively moderating the relationship between performance pressure and obsessive work passion. Additionally, achievement orientation is found to moderate the indirect influence of performance pressure on employee boundaryspanning behavior through these two mediators. This study reveals that employees with high achievement orientation under performance pressure tend to develop cognitive flexibility, which motivates them to engage in more employee boundary-spanning activities. This paper also provides practical guidance for enterprises to promote employee boundary-spanning behavior. This study not only expands the research on the antecedents of employee boundary-spanning behavior but also confirms the double-edged sword effect of performance pressure on employee boundary-spanning behavior from both cognitive and affective perspectives.</t>
@@ -11313,6 +11334,11 @@
       <c r="K211" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>The study measures individual-level employee boundary-spanning behavior (using the Marrone et al. 2007 scale) and provides a zero-order correlation matrix for a sample of 336 working individuals.. Verbatim Evidence: [Participants] "Questionnaires are distributed via social media and through the help of acquaintances such as colleagues, friends, and MBA classmates to increase the sample size." [Participants] "in terms of the number of years of working experience in the organization, 85 people (25.30%) have worked in the organization for less than one year, 89 people (26.49%) have worked there for 1-3 years, and 69 people (20.54%) have worked there for 4-5 years, and 93 people (27.68%) have worked more than 5 years." [Measures] "Employee boundary-spanning behavior. It is assessed using the six-item scale developed by Marrone et al. (2007). A sample item is “I would Persuade outsiders (e.g., faculty, clients) to support the team decisions.”, with Cronbach’s alpha of 0.885."</t>
         </is>
       </c>
     </row>
@@ -11379,6 +11405,16 @@
           <t>BSMA0210</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G213" t="inlineStr">
         <is>
           <t>Extending the differentiation-integration view of organizational design to teams, I propose that self-managing teams engaged in knowledge-intensive work can perform more effectively by combining autonomy and external knowledge to capture the benefits of each while offsetting their risks. The complementarity between having autonomy and using external knowledge is contingent, however, on characteristics of the knowledge and the task involved. To test the hypotheses, I examined the strategic and operational effectiveness of 96 teams in a large multinational organization. Findings provide support for the theoretical model and offer implications for research on team ambidexterity and multinational management as well as team effectiveness.</t>
@@ -11402,6 +11438,11 @@
       <c r="K213" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=96 teams). Verbatim Evidence: [Participants] "After excluding teams for which fewer than 50 percent of the respondents were core members (Hackman, 2002: 47), 96 teams qualified for the study (80 percent; 50 financial and 46 technical teams, with 485 member respondents)." [Measures] "To construct the external knowledge variable, I averaged the responses to the eight survey items for each team member and then within teams"</t>
         </is>
       </c>
     </row>
@@ -14614,6 +14655,12 @@
           <t>BSMA0281</t>
         </is>
       </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>This study performs an in-depth analysis of the causes and consequences of team boundary-spanning activities in the context of Chinese technology transfer, by addressing three related research questions: what are the drivers of teams’ boundary-spanning activities? How do teams conduct boundary-spanning activities? What is the impact of teams’ boundary-spanning activities? Based on the “input–moderator–output–input” model of team effectiveness theory, this study firstly explores which factors drive technology transfer teams to engage in boundary-spanning activities. Then, it examines the effects that such activities have on technology transfer performance, both directly and indirectly, through a set of mediating factors. Finally, it explores whether external environmental conditions play any moderating role in the relationship between team boundary-spanning activities and team performance. The empirical analysis is based on original primary survey data collected from a representative sample of organizations involved in the Chinese technology transfer system. The study both contributes the team effectiveness theory applied to the specific context of technology transfer and offers practical suggestions to managers of technology transfer intermediaries.</t>
@@ -14637,6 +14684,11 @@
       <c r="K284" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-individual level (team analysis). Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16095,6 +16147,12 @@
           <t>BSMA0320</t>
         </is>
       </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>The importance of emotional labouring and performance of frontline service employees, who in their boundary-spanning positions significantly affect service-rendering organisations’ efficiency by their direct communications with customers, continues to increase. However, it is still important to ascertain an efficient understanding of the comprehensive process including behavioural mechanism and a common perception of the rewards’ impacts on motivation and creativity. Therefore, guided by self-determination theory, this study examined the mechanism and boundary conditions between emotional labour and job performance (creative and task)–specifically, taking charge has been considered as a mediator and performance-based pay as a moderator in between relationships. The authors selected a time-lagged cross-sectional design to investigate interrelations amongst study variables at two different time points and surveyed 417 team members and 186 team leaders in Pakistan’s commercial banks. Findings were consistent with the assumed conceptual framework. For instance, deep-acting affected taking charge positively, surface-acting demonstrated a positive link with task performance and taking charge partially mediated the relationships between deep-acting and performances under boundary conditions of low performance-based pay. By summing up, the study adds to the literature and recommends managerial implications with a more affluent view of nomothetic linkage among frontline employees’ emotional labor, HR practices, and the service sector.</t>
@@ -16118,6 +16176,11 @@
       <c r="K323" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16273,7 +16336,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>This study draws on theories of collective action and organizational ecology to investigate a particular type of voluntary association: mixed-mode groups. Mixed-mode groups are created and organized online to meet physically in geographically deﬁned ways. An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups. Analysis shows that even when a mixed-mode group implements strategies focused on internal group processes, it beneﬁts from tapping into its external networks to obtain resources for group operation. Also, the differential impacts of internal and external strategies indicate that in the case of environment-prone mixed-mode groups, implementation of internal strategies alone, with or without solicited external networking resources, is helpful for generating positive group outcomes. Together, these results establish that boundary spanning represents not only a type of strategic action to obtain resources and produce positive outcomes but also an inherent and deﬁning mechanism of contemporary voluntary groups for engaging in collective action.</t>
@@ -16504,6 +16566,16 @@
           <t>BSMA0329</t>
         </is>
       </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G332" t="inlineStr">
         <is>
           <t>Landscapes are conceptually fuzzy and rich, and subject to plural framings. They are places of inquiry and intervention for scientists and practitioners, but also concepts bound to peoples’ dynamic identities, knowledge systems, inspiration, and well-being. These varying interpretations change the way landscapes function and evolve. Developed in the 1930s, Q-methodology is increasingly recognized for being useful in documenting and interrogating environmental discourses. Yet its application in the context of how integrated landscape approaches better navigate land-use dilemmas is still in its infancy. Based on our experience and emerging literature, such as the papers in this special collection, this article discusses the value of Q-methodology in addressing landscape sustainability issues. Q-methodology helps unravel and communicate common and contradicting landscape imaginaries and narratives in translational and boundary-spanning ways, thus bridging actors’ different understandings of problems and solutions and revealing common or differentiated entry points for negotiating trade-offs between competing land uses. The methodology can be empowering for marginalized people by uncovering their views and aspirational values to decision-makers and policymakers. We argue that this potential can be further strengthened by using Q to identify counter-hegemonic discourses and alliances that combat injustices regarding whose knowledge and visions count. In this way, applying Q-methodology in integrated landscape approaches can become a key tool for transitioning toward just, inclusive, and sustainable landscapes.</t>
@@ -16527,6 +16599,11 @@
       <c r="K332" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19665,7 +19742,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr">
         <is>
           <t>Software project teams are often faced with the potential for changing
@@ -21212,6 +21288,12 @@
           <t>BSMA0434</t>
         </is>
       </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
           <t>Efforts to understand how an organization monitors its environment often focus on boundary spanning individuals or units. The concept of boundary spanning was one introduced by Thompson in 1967 in a book that has since become the classic statement of the open systems model of organizations. This dissertation uses Thompson's model of boundary spanning units to generate hypotheses which are then tested in a sample of personnel/human resource departments. A theory driven argument is presented which suggests that the P/HR function in an organization meets Thompson's criteria for a boundary spanning unit. An historical review of the roots of personnel administration suggests that its emergence as a field fits Thompson's conceptualization of the development of boundary spanning units. This dissertation suggests that from its origin through this most recent period of transition, the development of the personnel function (now generally referred to as human resource management) has been due to a recognition by organizations that an increasing complexity and concomitant uncertainty in the human resource arena caused by such factors as labor unions, the expansion of due process in organizations, and intervention by government agencies, needed to be addressed.</t>
@@ -21235,6 +21317,11 @@
       <c r="K437" t="inlineStr">
         <is>
           <t>1989</t>
+        </is>
+      </c>
+      <c r="P437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21286,6 +21373,12 @@
           <t>BSMA0436</t>
         </is>
       </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
           <t>Purpose – Literature on small and medium enterprises (SMEs) has so far produced limited evidence on how these firms pursue their organizational flexibility with information and communication technology (ICT) and ad hoc work practices. The purpose of this paper is to contribute to the extant literature by focusing on how SMEs use flexible work practices that provide latitude with respect to when employees work, where they work and via which communication medium. Specifically, the authors analyze how such practices are related to the conditions that SMEs face in reference to their competitive environment and their patterns of ICT usage.</t>
@@ -21309,6 +21402,11 @@
       <c r="K439" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_4
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11038,7 +11038,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
           <t>The definition of innovation varies from individual to individual and between individual and the team or the team and an organization. The perception of innovation and how individuals define innovation can make an organization stay competitive or go out of business. Research had shown that a traditional approach of idea generation as innovation at well intentioned organizations afforded success only 10% of the time after three years. In forming and managing project teams, which are made up of individuals or selling a service or product to a certain demography it is important and beneficial to understand their perception of innovation and if they see innovation as new, change or improvement. This study is built upon the earlier work of Zhuang (1995), Zhuang, Williamson, and Carter (1999), and McLaughlin and (2013). Prior research conducted by Caraballo and McLaughlin (2012) focused on understanding the perception of innovation as defined or understood by a homogeneous demography of Latino American professionals. This dissertation furthers the research conducted by Caraballo and McLaughlin (2012) with a focus on comprehending how a homogenous group Indian American professionals in the United States perceive or define innovation into the three categories of new, improve and change. While innovation may be understood by individuals as a multi-dimensional construct, the research tried to identify the relationship between perceptions, and gender, age and job function for the homogenous group of Indian Americans in the United States. The research followed the approach and methodology used by Caraballo and McLaughlin (2012) and the study is quantitative, exploratory and used web-based surveys to gather responses from respondents.</t>
@@ -11165,6 +11164,12 @@
           <t>BSMA0205</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>This study examines the influence of the social network of board interlocks on strategic alliance formation. Our theoretical framework suggests how board interlock ties to other firms can increase or decrease the likelihood of alliance formation, depending on the content of relationships between CEOs (chief executive officers) and outside directors. Results suggest that CEO-board relationships characterized by independent board control reduce the likelihood of alliance formation by prompting distrust between corporate leaders, while CEO-board cooperation in strategic decision making appears to promote alliance formation by enhancing trust. The findings also show how the effects of direct interlock ties are amplified further by third-party network ties.</t>
@@ -11188,6 +11193,11 @@
       <c r="K208" t="inlineStr">
         <is>
           <t>1999</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11457,6 +11467,12 @@
           <t>BSMA0211</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>SUMMARY             Previous research has focused on purchasing managers’ experience with role stressors and the negative effect of stress on job attitudes and performance. The potential benefits of having multiple responsibilities and a diverse role set have been overlooked. This study explored the relationship between purchasing managers’ involvement in multiple boundary spanning roles and their perceptions of positive social outcomes related to work. The relationship of these social benefits to job satisfaction was also evaluated. The relationships were analyzed using structural equation modeling. The results indicated positive relationships between each variable in the model. The implications for recruitment, supervision, and job design are discussed.</t>
@@ -11480,6 +11496,11 @@
       <c r="K214" t="inlineStr">
         <is>
           <t>1999</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Included. The study measures individual-level purposive boundary spanning roles among purchasing managers and provides zero-order correlations with obtained and desired social benefits.. Verbatim Evidence: [Sample Characteristics] "A total of 134 completed questionnaires were returned for a response rate of 25.3 percent. Job title classifications were adapted from a previous study (Carter and Narasimhan 1994). The majority of respondents indicated that they were purchasing managers or senior purchasing officers." [Measures] "Boundary spanning roles. A 23-item scale describing the activities associated with each boundary spanning role was developed. Respondents were asked to indicate on a 5-point scale their involvement in each of the role activities (1 = Almost never; 5 = Almost always)." [Results] "Correlational matrices of the relationships of specific boundary spanning roles to the obtained and desired social benefits are presented in Tables III and IV, respectively."</t>
         </is>
       </c>
     </row>
@@ -14618,6 +14639,12 @@
           <t>BSMA0280</t>
         </is>
       </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries. Not only must this structure be clearly defined, but it also must account for the integration of a broad range of cross-government activities. Like the overarching performance network, the cross-boundary structure has the characteristics of a dynamic system, including flexibility, adaptability, growth, and the continual emergence of new forms and functions. Summer 2000 featured perfect conditions for gridlock in the sky. Flying had become an increasingly popular way to travel, and the airlines had marketed aggressively to vacationing families and business travelers. Airports were already crowded when unusual and frequent patterns of bad weather hit aviation especially hard. Delays and canceled flights became almost daily events. The public complained loudly, congressional hearings were scheduled, and the Federal Aviation Administration was about to experience unfriendly fire from an aroused media.</t>
@@ -14641,6 +14668,11 @@
       <c r="K283" t="inlineStr">
         <is>
           <t>2009</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14660,7 +14692,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>This study performs an in-depth analysis of the causes and consequences of team boundary-spanning activities in the context of Chinese technology transfer, by addressing three related research questions: what are the drivers of teams’ boundary-spanning activities? How do teams conduct boundary-spanning activities? What is the impact of teams’ boundary-spanning activities? Based on the “input–moderator–output–input” model of team effectiveness theory, this study firstly explores which factors drive technology transfer teams to engage in boundary-spanning activities. Then, it examines the effects that such activities have on technology transfer performance, both directly and indirectly, through a set of mediating factors. Finally, it explores whether external environmental conditions play any moderating role in the relationship between team boundary-spanning activities and team performance. The empirical analysis is based on original primary survey data collected from a representative sample of organizations involved in the Chinese technology transfer system. The study both contributes the team effectiveness theory applied to the specific context of technology transfer and offers practical suggestions to managers of technology transfer intermediaries.</t>
@@ -16152,7 +16183,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>The importance of emotional labouring and performance of frontline service employees, who in their boundary-spanning positions significantly affect service-rendering organisations’ efficiency by their direct communications with customers, continues to increase. However, it is still important to ascertain an efficient understanding of the comprehensive process including behavioural mechanism and a common perception of the rewards’ impacts on motivation and creativity. Therefore, guided by self-determination theory, this study examined the mechanism and boundary conditions between emotional labour and job performance (creative and task)–specifically, taking charge has been considered as a mediator and performance-based pay as a moderator in between relationships. The authors selected a time-lagged cross-sectional design to investigate interrelations amongst study variables at two different time points and surveyed 417 team members and 186 team leaders in Pakistan’s commercial banks. Findings were consistent with the assumed conceptual framework. For instance, deep-acting affected taking charge positively, surface-acting demonstrated a positive link with task performance and taking charge partially mediated the relationships between deep-acting and performances under boundary conditions of low performance-based pay. By summing up, the study adds to the literature and recommends managerial implications with a more affluent view of nomothetic linkage among frontline employees’ emotional labor, HR practices, and the service sector.</t>
@@ -16786,6 +16816,12 @@
           <t>BSMA0334</t>
         </is>
       </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
           <t>This study of Korean industrial salespeople (N = 140) examines the relationships among organizational formalization, role stress, organizational commitment, and propensity to leave. Although most of the theoretical and empirical research in this area was done in the United States, this study examines whether the same concepts could be applied to a culturally different salesforce. The results of the structural modeling analysis suggest that overall the model of job variables and propensity to leave developed in the U.S. could be applied to a Korean salesforce. However, some culture-related differences do exist in the nature of specific relationships.</t>
@@ -16809,6 +16845,11 @@
       <c r="K337" t="inlineStr">
         <is>
           <t>1997</t>
+        </is>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21293,7 +21334,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
           <t>Efforts to understand how an organization monitors its environment often focus on boundary spanning individuals or units. The concept of boundary spanning was one introduced by Thompson in 1967 in a book that has since become the classic statement of the open systems model of organizations. This dissertation uses Thompson's model of boundary spanning units to generate hypotheses which are then tested in a sample of personnel/human resource departments. A theory driven argument is presented which suggests that the P/HR function in an organization meets Thompson's criteria for a boundary spanning unit. An historical review of the roots of personnel administration suggests that its emergence as a field fits Thompson's conceptualization of the development of boundary spanning units. This dissertation suggests that from its origin through this most recent period of transition, the development of the personnel function (now generally referred to as human resource management) has been due to a recognition by organizations that an increasing complexity and concomitant uncertainty in the human resource arena caused by such factors as labor unions, the expansion of due process in organizations, and intervention by government agencies, needed to be addressed.</t>
@@ -21336,6 +21376,12 @@
           <t>BSMA0435</t>
         </is>
       </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to know that how group resources (internal and external) and the relationship quality among group members relate to group performance. Design/methodology/approach – Given the normative nature of group performance, the study is carried out in a contrived environment. Participants were 204 master of business administration students who were allocated to 51 study groups. Data were collected in three waves and from two different sources, i.e., students and instructors. Data analysis was carried out by employing regression analysis and the bootstrapping procedure, i.e., PROCESS.</t>
@@ -21359,6 +21405,11 @@
       <c r="K438" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21378,7 +21429,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
           <t>Purpose – Literature on small and medium enterprises (SMEs) has so far produced limited evidence on how these firms pursue their organizational flexibility with information and communication technology (ICT) and ad hoc work practices. The purpose of this paper is to contribute to the extant literature by focusing on how SMEs use flexible work practices that provide latitude with respect to when employees work, where they work and via which communication medium. Specifically, the authors analyze how such practices are related to the conditions that SMEs face in reference to their competitive environment and their patterns of ICT usage.</t>
@@ -21421,6 +21471,12 @@
           <t>BSMA0437</t>
         </is>
       </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr">
         <is>
           <t>Business Process Reengineering (BPR) was developed as a new idea which, it was suggested, could revolutionise the corporation and give it a major competitive advantage by simplifying key business processes and utilising information technology to secure cross-functional communication and focus on customer requirements. Rather than continue the debate about whether BPR is ‘good’ or ‘bad’, ‘old’ or ‘new’ (e.g. Earl, M.J., 1994. The new and the old of business process redesign. Journal of Strategic Information Systems 3 (1), 5–22; Mumford, E., 1994. New treatments or old remedies: is business process reengineering really socio-technical design. Journal of Strategic Information Systems 3 (4), 313–326), the focus here is on understanding how the concept ‘BPR’, however deﬁned, has been diffused across European ﬁrms. The results from a survey of ﬁrms in four countries support previous research on the diffusion process with the rate of adoption of BPR related to microorganisational level variables—characteristics of the ﬁrm and the boundary spanning activities of individual members. In addition there were differences across industry sectors and across countries in the extent of adoption of BPR. It is argued that attention to these meso-industry level and macro-national level factors, as well as the micro-organisational level dynamics, will improve our understanding of the relationship between networking and innovation processes. In particular, the paper focuses on how networking activity can be restrictive and lead to the creation of fashions which limit the extent of organisational learning during BPR adoption. q 1999 Elsevier Science B.V. All rights reserved.</t>
@@ -21444,6 +21500,11 @@
       <c r="K440" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 18
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11127,6 +11127,12 @@
           <t>BSMA0204</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>As software development projects continue to be over budget and behind schedule, researchers continue to look for ways to improve the likelihood of project success. In this research we juxtapose two different views of what influences software development team performance during the requirements development phase. In an examination of 66 teams from 15 companies we found that team skill, managerial involvement, and little variance in team experience enable more effective team processes than do software development tools and methods. Further, we found that development teams exhibit both positive and negative boundary-spanning behaviors. Team members promote and champion their projects to the outside environment, which is considered valuable by project stakeholders. They also, however, guard themselves from their environments; keeping important information a secret from stakeholders negatively predicts performance.</t>
@@ -11150,6 +11156,11 @@
       <c r="K207" t="inlineStr">
         <is>
           <t>1998</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11169,7 +11180,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>This study examines the influence of the social network of board interlocks on strategic alliance formation. Our theoretical framework suggests how board interlock ties to other firms can increase or decrease the likelihood of alliance formation, depending on the content of relationships between CEOs (chief executive officers) and outside directors. Results suggest that CEO-board relationships characterized by independent board control reduce the likelihood of alliance formation by prompting distrust between corporate leaders, while CEO-board cooperation in strategic decision making appears to promote alliance formation by enhancing trust. The findings also show how the effects of direct interlock ties are amplified further by third-party network ties.</t>
@@ -11472,7 +11482,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>SUMMARY             Previous research has focused on purchasing managers’ experience with role stressors and the negative effect of stress on job attitudes and performance. The potential benefits of having multiple responsibilities and a diverse role set have been overlooked. This study explored the relationship between purchasing managers’ involvement in multiple boundary spanning roles and their perceptions of positive social outcomes related to work. The relationship of these social benefits to job satisfaction was also evaluated. The relationships were analyzed using structural equation modeling. The results indicated positive relationships between each variable in the model. The implications for recruitment, supervision, and job design are discussed.</t>
@@ -14589,6 +14598,12 @@
           <t>BSMA0279</t>
         </is>
       </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>Information and communication technologies enable employees to be available anywhere and anytime, raising availability expectations
@@ -14627,6 +14642,11 @@
           <t>2022</t>
         </is>
       </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -14644,7 +14664,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries. Not only must this structure be clearly defined, but it also must account for the integration of a broad range of cross-government activities. Like the overarching performance network, the cross-boundary structure has the characteristics of a dynamic system, including flexibility, adaptability, growth, and the continual emergence of new forms and functions. Summer 2000 featured perfect conditions for gridlock in the sky. Flying had become an increasingly popular way to travel, and the airlines had marketed aggressively to vacationing families and business travelers. Airports were already crowded when unusual and frequent patterns of bad weather hit aviation especially hard. Delays and canceled flights became almost daily events. The public complained loudly, congressional hearings were scheduled, and the Federal Aviation Administration was about to experience unfriendly fire from an aroused media.</t>
@@ -14808,6 +14827,16 @@
           <t>BSMA0284</t>
         </is>
       </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G287" t="inlineStr">
         <is>
           <t>This article proposes to examine the self-concept of members of an occupational category referred to as the “solo self-employed”—women and men who work alone and do not employ other workers. Our findings reveal that although the solo self-employed themselves do not make clear phenomenological use of the solo-self-employed category, they do speak similarly about their occupational independence, albeit without group awareness. The self-concept of the solo self-employed is mainly based on boundary work in relation to two well-known cultural-occupational categories: “employed workers” and “businesspeople.” Solo-employed workers prefer to distance themselves from these two categories and define themselves through negative comparisons between themselves and the two preceding categories. The Discussion section proposes perceiving solo selfemployment as a social category that constructs an alternative self in relation to the selves associated with popular cultural-occupational scenarios.</t>
@@ -14831,6 +14860,11 @@
       <c r="K287" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14845,6 +14879,12 @@
           <t>BSMA0285</t>
         </is>
       </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>The purpose of this paper is to develop the concept of project management system from the perspective of systems science. There is a need to extend the body of knowledge for project management. In particular, the application of systems perspectives and systems theory offers a significant opportunity to advance the current state of project management knowledge. Although there have been suggestions of systems approaches for project management, rigorous systems science has not been used to support these depictions. First, we develop the background and define a perspective of project management systems. Second, assumptions and principles are drawn from systems science to provide a foundation for project management systems. Third, a model for project management systems is developed from systems sciences and management cybernetics. Our initial explorations are promising, demonstrated by a case study application review using a complex system of systems (SoS) project encompassed multiple government agencies, and we offer future directions and implications for further model refinements, applications, and research into project management systems.</t>
@@ -14868,6 +14908,11 @@
       <c r="K288" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16272,6 +16317,12 @@
           <t>BSMA0322</t>
         </is>
       </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>Though improvisation has emerged as a crucial organizational competence, research wrestles with a key question – how can organizations benefit from improvisation? To advance research, I build a richer conceptualization of the role of knowledge resources – market information sources and memory types – in improvisation. I argue that as (a) internal and external sources of market information differ in speed and novelty and (b) procedural and declarative memory differ in articulation and abstractness, they shape the impact of improvisation on new product outcomes in a distinct way. A longitudinal survey of new products in the Dutch food industry uncovers that, contrary to prior thinking, improvisation increases cost efficiency when new product teams rely on internal market information and declarative memory and they minimize external market information. Though both sources of market information and low procedural memory weaken the negative impact of improvisation on market effectiveness, these conditions were not enough to make its impact positive, echoing traditional concerns with improvisation.</t>
@@ -16295,6 +16346,11 @@
       <c r="K325" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P325" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16685,6 +16741,12 @@
           <t>BSMA0331</t>
         </is>
       </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>Prompted by the relationship management literature which has appeared recently in marketing, we posit that the performance of sellers in ongoing buyer-seller relationships is influenced significantly by the manner in which sellers interact with buyers, which we refer to as" boundary behavior." Although a growing literature has drawn attention to the importance of relationship management, no research has investigated the extent to which, if any, relationship management leads to improved performance in terms of" hard" measures, such as sales. We fill this gap by examining how managerially controllable boundary behaviors influence sellers' sales performance. We further examine how situational factors moderate these effects, and consequently illuminate contexts in which the actions of boundary spanning personnel are most critical. The findings are likely to be of interest to managers who operate at the organization boundary, and who are therefore concerned with the effective deployment of these important resources.</t>
@@ -16708,6 +16770,11 @@
       <c r="K334" t="inlineStr">
         <is>
           <t>1991</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16821,7 +16888,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
           <t>This study of Korean industrial salespeople (N = 140) examines the relationships among organizational formalization, role stress, organizational commitment, and propensity to leave. Although most of the theoretical and empirical research in this area was done in the United States, this study examines whether the same concepts could be applied to a culturally different salesforce. The results of the structural modeling analysis suggest that overall the model of job variables and propensity to leave developed in the U.S. could be applied to a Korean salesforce. However, some culture-related differences do exist in the nature of specific relationships.</t>
@@ -21381,7 +21447,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to know that how group resources (internal and external) and the relationship quality among group members relate to group performance. Design/methodology/approach – Given the normative nature of group performance, the study is carried out in a contrived environment. Participants were 204 master of business administration students who were allocated to 51 study groups. Data were collected in three waves and from two different sources, i.e., students and instructors. Data analysis was carried out by employing regression analysis and the bootstrapping procedure, i.e., PROCESS.</t>
@@ -21476,7 +21541,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr">
         <is>
           <t>Business Process Reengineering (BPR) was developed as a new idea which, it was suggested, could revolutionise the corporation and give it a major competitive advantage by simplifying key business processes and utilising information technology to secure cross-functional communication and focus on customer requirements. Rather than continue the debate about whether BPR is ‘good’ or ‘bad’, ‘old’ or ‘new’ (e.g. Earl, M.J., 1994. The new and the old of business process redesign. Journal of Strategic Information Systems 3 (1), 5–22; Mumford, E., 1994. New treatments or old remedies: is business process reengineering really socio-technical design. Journal of Strategic Information Systems 3 (4), 313–326), the focus here is on understanding how the concept ‘BPR’, however deﬁned, has been diffused across European ﬁrms. The results from a survey of ﬁrms in four countries support previous research on the diffusion process with the rate of adoption of BPR related to microorganisational level variables—characteristics of the ﬁrm and the boundary spanning activities of individual members. In addition there were differences across industry sectors and across countries in the extent of adoption of BPR. It is argued that attention to these meso-industry level and macro-national level factors, as well as the micro-organisational level dynamics, will improve our understanding of the relationship between networking and innovation processes. In particular, the paper focuses on how networking activity can be restrictive and lead to the creation of fashions which limit the extent of organisational learning during BPR adoption. q 1999 Elsevier Science B.V. All rights reserved.</t>
@@ -21556,6 +21620,12 @@
           <t>BSMA0439</t>
         </is>
       </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
           <t>This dissertation presents a critical perspective on the development of American journalism education by combining historical methods and a sociological framework. That framework is boundary work, and it serves as the organizing principle of this project. As such, this study privileges boundary work paradigms–participation, practices, and professionalism–over a chronological narrative. It uncovers the interrelationships and power dynamics that structured the development of journalism instruction in higher education. Moreover, it heeds the call for journalism historians to engage with other disciplines and develop more theoretical approaches to understanding the past.</t>
@@ -21579,6 +21649,11 @@
       <c r="K442" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_5
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -11132,7 +11132,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>As software development projects continue to be over budget and behind schedule, researchers continue to look for ways to improve the likelihood of project success. In this research we juxtapose two different views of what influences software development team performance during the requirements development phase. In an examination of 66 teams from 15 companies we found that team skill, managerial involvement, and little variance in team experience enable more effective team processes than do software development tools and methods. Further, we found that development teams exhibit both positive and negative boundary-spanning behaviors. Team members promote and champion their projects to the outside environment, which is considered valuable by project stakeholders. They also, however, guard themselves from their environments; keeping important information a secret from stakeholders negatively predicts performance.</t>
@@ -14603,7 +14602,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>Information and communication technologies enable employees to be available anywhere and anytime, raising availability expectations
@@ -14884,7 +14882,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>The purpose of this paper is to develop the concept of project management system from the perspective of systems science. There is a need to extend the body of knowledge for project management. In particular, the application of systems perspectives and systems theory offers a significant opportunity to advance the current state of project management knowledge. Although there have been suggestions of systems approaches for project management, rigorous systems science has not been used to support these depictions. First, we develop the background and define a perspective of project management systems. Second, assumptions and principles are drawn from systems science to provide a foundation for project management systems. Third, a model for project management systems is developed from systems sciences and management cybernetics. Our initial explorations are promising, demonstrated by a case study application review using a complex system of systems (SoS) project encompassed multiple government agencies, and we offer future directions and implications for further model refinements, applications, and research into project management systems.</t>
@@ -16322,7 +16319,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>Though improvisation has emerged as a crucial organizational competence, research wrestles with a key question – how can organizations benefit from improvisation? To advance research, I build a richer conceptualization of the role of knowledge resources – market information sources and memory types – in improvisation. I argue that as (a) internal and external sources of market information differ in speed and novelty and (b) procedural and declarative memory differ in articulation and abstractness, they shape the impact of improvisation on new product outcomes in a distinct way. A longitudinal survey of new products in the Dutch food industry uncovers that, contrary to prior thinking, improvisation increases cost efficiency when new product teams rely on internal market information and declarative memory and they minimize external market information. Though both sources of market information and low procedural memory weaken the negative impact of improvisation on market effectiveness, these conditions were not enough to make its impact positive, echoing traditional concerns with improvisation.</t>
@@ -16746,7 +16742,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>Prompted by the relationship management literature which has appeared recently in marketing, we posit that the performance of sellers in ongoing buyer-seller relationships is influenced significantly by the manner in which sellers interact with buyers, which we refer to as" boundary behavior." Although a growing literature has drawn attention to the importance of relationship management, no research has investigated the extent to which, if any, relationship management leads to improved performance in terms of" hard" measures, such as sales. We fill this gap by examining how managerially controllable boundary behaviors influence sellers' sales performance. We further examine how situational factors moderate these effects, and consequently illuminate contexts in which the actions of boundary spanning personnel are most critical. The findings are likely to be of interest to managers who operate at the organization boundary, and who are therefore concerned with the effective deployment of these important resources.</t>
@@ -21625,7 +21620,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
           <t>This dissertation presents a critical perspective on the development of American journalism education by combining historical methods and a sociological framework. That framework is boundary work, and it serves as the organizing principle of this project. As such, this study privileges boundary work paradigms–participation, practices, and professionalism–over a chronological narrative. It uncovers the interrelationships and power dynamics that structured the development of journalism instruction in higher education. Moreover, it heeds the call for journalism historians to engage with other disciplines and develop more theoretical approaches to understanding the past.</t>
@@ -21668,6 +21662,12 @@
           <t>BSMA0440</t>
         </is>
       </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
           <t>Research Summary:                              We study antecedents of innovation performance for the subsidiaries of multinational enterprises (MNEs) using the microfoundations approach. Based on the upper echelon perspective, we argue that managers’ characteristics, such as prior MNE work experience and industry experience, affect subsidiary innovation. We tested our hypotheses on a sample of 228 MNE subsidiaries from 11 countries. Results indicate that managers’ industry experience serves as an external boundary‐spanning capability and, therefore, it has a greater effect on autonomous subsidiaries. In contrast, managers’ prior MNE work experience functions as an internal boundary‐spanning capability and, therefore, it has a smaller effect on subsidiaries that are less autonomous or engage in R&amp;D.                                                          Managerial Summary:                              The success of an MNE now increasingly depends on its ability to generate knowledge anywhere in the world. Thus, the ability of foreign subsidiaries to generate innovation plays an increasingly important role in enhancing the performance of MNEs. In this regard, what factors determine the innovativeness of foreign subsidiaries is an important question for managers. Our study suggests that the international experience of the top management team (TMT) of a subsidiary and its CEO’s industry experience positively affect subsidiary innovation. Furthermore, the TMT’s international experience has a greater effect on the innovativeness of subsidiaries that remain dependent on their headquarters for knowledge transfer. In contrast, the CEO’s industry experience has a greater effect on the innovativeness of autonomous subsidiaries.</t>
@@ -21691,6 +21691,11 @@
       <c r="K443" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 19
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -14523,6 +14523,12 @@
           <t>BSMA0277</t>
         </is>
       </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to evaluate the recognition of sexual harassment (SH); to describe the relationships among SH, employees’ burnout, customer-oriented boundary-spanning behaviors (COBSB); and to verify the moderating effect of employees’ psychological safety (PS), all within deluxe hotels in South Korea.</t>
@@ -14546,6 +14552,11 @@
       <c r="K280" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14924,6 +14935,12 @@
           <t>BSMA0286</t>
         </is>
       </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>Smart cities emphasize the use of advanced technology to deliver better services to and improve the well-being of their residents. Since the administrative authorities that manage cities often lack the knowledge and skills needed to transform their operations in this way, smart city initiatives usually involve a complex set of actors, from local urban authorities and their technical departments to small and large IT firms, academics, and civic organizations, as well as individual citizens. Mediating organizations are often set up to coordinate and manage such interactions. However, little is known about the roles and activities of such bodies. Using data from the Dublin smart city projects, this study draws on the concept of boundary spanning to develop a taxonomy of the work of such intermediaries. Divided into technical, political, social, and cultural domains, the study demonstrates the critical role of the work done by such bodies in enhancing collaboration among and the participation of a diverse group of citizens, IT and digital strategy departments of local authorities, universities and local/international IT companies (e.g., Google, Facebook or Airbnb), leading to a bottom-up governance style of leading smart city initiatives and projects.</t>
@@ -14947,6 +14964,11 @@
       <c r="K289" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14961,6 +14983,12 @@
           <t>BSMA0287</t>
         </is>
       </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>Purpose – The recent COVID-19 pandemic has (triggered) lots of interest in work from home (WFH) practices. Many organizations in India are changing their work practices and adopting new models of getting the work done. The purpose of the study to look at the boundary-ﬁt perspective (Ammons (2013) and two factors, namely, individual preferences (boundary control, family identity, work identity and technology stress) and environmental factors (job control, supervisor support and organizational policies). These dimensions are used and considered to create various clusters for employees working from home.</t>
@@ -14984,6 +15012,11 @@
       <c r="K290" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14998,6 +15031,12 @@
           <t>BSMA0288</t>
         </is>
       </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>This study investigates the role of gatekeepers in the transfer of information within a single R &amp; D location by comparing directly t h e performance of project groups with and without gatekeepers. The results show that gatekeepers performed a linking role only for projects performing tasks that were 'locally-oriented' while 'universallyoriented' tasks were most effectively linked to external areas by direct project member communication. Gatekeepers also appear to facilitate external communication by their locallyoriented project colleagues. A follow-up study five years later showed that almost all gatekeeping project leaders had been promoted up the managerial ladder; in contrast, one half of the non-gatekeeping project leaders had ascended the technical ladder. This implies that higher managerial levels demand strong interpersonal a s well a s technical skills.</t>
@@ -15021,6 +15060,11 @@
       <c r="K291" t="inlineStr">
         <is>
           <t>1981</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17781,6 +17825,12 @@
           <t>BSMA0353</t>
         </is>
       </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>This article theoretically and empirically examines the antecedents and consequences of project communication during the new financial service innovation process. The authors analyze project communication comprising both intraproject communication and extraproject communication (i.e., boundary spanners) and adopt the view that project teams within banks are primarily information-processing systems directed toward reducing innovative uncertainty. The research findings indicate that the level of complexity contributes to intraproject communication, whereas centralized project environments appear to be a barrier for communication within the project team. Curvilinear relationships (inverted U) are substantiated between project climate and intraproject communication and between formalization and boundary-spanning communication. The authors’ findings provide support for the fact that effective project communication is contingent upon the level of cross-functional cooperation and that the relationship with project success is an indirect one, mediated by the level of innovative uncertainty reduction.</t>
@@ -17804,6 +17854,11 @@
       <c r="K356" t="inlineStr">
         <is>
           <t>2000</t>
+        </is>
+      </c>
+      <c r="P356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17855,6 +17910,12 @@
           <t>BSMA0355</t>
         </is>
       </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
           <t>This study expands the scope of research on knowledge search and innovation search by investigating the effect of boundary-spanning search behavior on breakthrough innovations of new ventures. Based on an environmental coalignment perspective, we argue that boundary-spanning search is a key activity for new ventures so that they can deal with different market forces to enhance their breakthrough innovations. Most of the hypotheses proposed are supported by the results of a survey of 227 ventures in the high-technology zone of Shenzhen. We found that boundary-spanning search is not only associated positively with breakthrough innovations of new ventures but also plays a signiﬁcant role in inﬂuencing the effect of market forces on both types of innovations. This paper offers insight into the way in which new ventures can achieve both market innovations and technological innovations through different types of boundary-spanning search. Furthermore, this study argues that boundary-spanning search is an important tool that enables new ventures to create more innovative performance under competitive environments.</t>
@@ -17878,6 +17939,11 @@
       <c r="K358" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P358" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21667,7 +21733,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
           <t>Research Summary:                              We study antecedents of innovation performance for the subsidiaries of multinational enterprises (MNEs) using the microfoundations approach. Based on the upper echelon perspective, we argue that managers’ characteristics, such as prior MNE work experience and industry experience, affect subsidiary innovation. We tested our hypotheses on a sample of 228 MNE subsidiaries from 11 countries. Results indicate that managers’ industry experience serves as an external boundary‐spanning capability and, therefore, it has a greater effect on autonomous subsidiaries. In contrast, managers’ prior MNE work experience functions as an internal boundary‐spanning capability and, therefore, it has a smaller effect on subsidiaries that are less autonomous or engage in R&amp;D.                                                          Managerial Summary:                              The success of an MNE now increasingly depends on its ability to generate knowledge anywhere in the world. Thus, the ability of foreign subsidiaries to generate innovation plays an increasingly important role in enhancing the performance of MNEs. In this regard, what factors determine the innovativeness of foreign subsidiaries is an important question for managers. Our study suggests that the international experience of the top management team (TMT) of a subsidiary and its CEO’s industry experience positively affect subsidiary innovation. Furthermore, the TMT’s international experience has a greater effect on the innovativeness of subsidiaries that remain dependent on their headquarters for knowledge transfer. In contrast, the CEO’s industry experience has a greater effect on the innovativeness of autonomous subsidiaries.</t>
@@ -21747,6 +21812,12 @@
           <t>BSMA0442</t>
         </is>
       </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
           <t>In this dissertation I first develop a theoretical framework that explores different
@@ -21791,6 +21862,11 @@
           <t>2013</t>
         </is>
       </c>
+      <c r="P445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -21803,6 +21879,12 @@
           <t>BSMA0443</t>
         </is>
       </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
           <t>Purpose – This study recognizes service as the majority contributor to global and US gross domestic product and the importance of innovation speed to service innovation. Generating innovative products and services at a faster rate generates advantages for business-to-business (B2B) service organizations in keeping up with and moving ahead of rivals. This study aims to introduce the concept of capacity for social exchange (CSE) in buyer–supplier relationships, which reflects the degree to which individuals possess competencies that enable the exchange of information, and this study also explores how CSE affects knowledge sharing and innovation speed within a supply chain organization.</t>
@@ -21826,6 +21908,11 @@
       <c r="K446" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_6
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -14528,7 +14528,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to evaluate the recognition of sexual harassment (SH); to describe the relationships among SH, employees’ burnout, customer-oriented boundary-spanning behaviors (COBSB); and to verify the moderating effect of employees’ psychological safety (PS), all within deluxe hotels in South Korea.</t>
@@ -14571,6 +14570,12 @@
           <t>BSMA0278</t>
         </is>
       </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
           <t>Data from high-technology firms in Hong Kong were used to investigate whether the outcomes of problem-solving processes (solutions found, problem-solving speed, and solution quality) mediated the effects of centrifugal forces (decentralization, free flow of information, and reach) and centripetal forces (connectedness, temporal pacing, project leader expertise, and superordinate goal) on product development performance (development speed and product quality). Centrifugal and centripetal forces were indirectly related to performance through problem-solving outcomes, although some direct effects of these forces were also found. The results suggest a more complex model of product development than previously envisaged.</t>
@@ -14594,6 +14599,11 @@
       <c r="K281" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14762,6 +14772,12 @@
           <t>BSMA0282</t>
         </is>
       </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>One of the main reasons that firms participate in alliances is to learn know‐how and capabilities from their alliance partners. At the same time firms want to protect themselves from the opportunistic behavior of their partner to retain their own core proprietary assets. Most research has generally viewed the achievement of these objectives as mutually exclusive. In contrast, we provide empirical evidence using large‐sample survey data to show that when firms build relational capital in conjunction with an integrative approach to managing conflict, they are able to achieve both objectives simultaneously. Relational capital based on mutual trust and interaction at the individual level between alliance partners creates a basis for learning and know‐how transfer across the exchange interface. At the same time, it curbs opportunistic behavior of alliance partners, thus preventing the leakage of critical know‐how between them.</t>
@@ -14785,6 +14801,11 @@
       <c r="K285" t="inlineStr">
         <is>
           <t>2000</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14940,7 +14961,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>Smart cities emphasize the use of advanced technology to deliver better services to and improve the well-being of their residents. Since the administrative authorities that manage cities often lack the knowledge and skills needed to transform their operations in this way, smart city initiatives usually involve a complex set of actors, from local urban authorities and their technical departments to small and large IT firms, academics, and civic organizations, as well as individual citizens. Mediating organizations are often set up to coordinate and manage such interactions. However, little is known about the roles and activities of such bodies. Using data from the Dublin smart city projects, this study draws on the concept of boundary spanning to develop a taxonomy of the work of such intermediaries. Divided into technical, political, social, and cultural domains, the study demonstrates the critical role of the work done by such bodies in enhancing collaboration among and the participation of a diverse group of citizens, IT and digital strategy departments of local authorities, universities and local/international IT companies (e.g., Google, Facebook or Airbnb), leading to a bottom-up governance style of leading smart city initiatives and projects.</t>
@@ -14988,7 +15008,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>Purpose – The recent COVID-19 pandemic has (triggered) lots of interest in work from home (WFH) practices. Many organizations in India are changing their work practices and adopting new models of getting the work done. The purpose of the study to look at the boundary-ﬁt perspective (Ammons (2013) and two factors, namely, individual preferences (boundary control, family identity, work identity and technology stress) and environmental factors (job control, supervisor support and organizational policies). These dimensions are used and considered to create various clusters for employees working from home.</t>
@@ -15036,7 +15055,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>This study investigates the role of gatekeepers in the transfer of information within a single R &amp; D location by comparing directly t h e performance of project groups with and without gatekeepers. The results show that gatekeepers performed a linking role only for projects performing tasks that were 'locally-oriented' while 'universallyoriented' tasks were most effectively linked to external areas by direct project member communication. Gatekeepers also appear to facilitate external communication by their locallyoriented project colleagues. A follow-up study five years later showed that almost all gatekeeping project leaders had been promoted up the managerial ladder; in contrast, one half of the non-gatekeeping project leaders had ascended the technical ladder. This implies that higher managerial levels demand strong interpersonal a s well a s technical skills.</t>
@@ -15116,6 +15134,16 @@
           <t>BSMA0290</t>
         </is>
       </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G293" t="inlineStr">
         <is>
           <t>An investigation of the influence of boundary spanning project supervisors on the turnover and promotion of engineering professionals found that, in general, boundary spanning supervisors had little direct effect on the careers of all project subordinates. However, project supervisors who also were technical gatekeepers significantly affected the organizational careers of young engineers.</t>
@@ -15139,6 +15167,11 @@
       <c r="K293" t="inlineStr">
         <is>
           <t>1983</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17830,7 +17863,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>This article theoretically and empirically examines the antecedents and consequences of project communication during the new financial service innovation process. The authors analyze project communication comprising both intraproject communication and extraproject communication (i.e., boundary spanners) and adopt the view that project teams within banks are primarily information-processing systems directed toward reducing innovative uncertainty. The research findings indicate that the level of complexity contributes to intraproject communication, whereas centralized project environments appear to be a barrier for communication within the project team. Curvilinear relationships (inverted U) are substantiated between project climate and intraproject communication and between formalization and boundary-spanning communication. The authors’ findings provide support for the fact that effective project communication is contingent upon the level of cross-functional cooperation and that the relationship with project success is an indirect one, mediated by the level of innovative uncertainty reduction.</t>
@@ -17915,7 +17947,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
           <t>This study expands the scope of research on knowledge search and innovation search by investigating the effect of boundary-spanning search behavior on breakthrough innovations of new ventures. Based on an environmental coalignment perspective, we argue that boundary-spanning search is a key activity for new ventures so that they can deal with different market forces to enhance their breakthrough innovations. Most of the hypotheses proposed are supported by the results of a survey of 227 ventures in the high-technology zone of Shenzhen. We found that boundary-spanning search is not only associated positively with breakthrough innovations of new ventures but also plays a signiﬁcant role in inﬂuencing the effect of market forces on both types of innovations. This paper offers insight into the way in which new ventures can achieve both market innovations and technological innovations through different types of boundary-spanning search. Furthermore, this study argues that boundary-spanning search is an important tool that enables new ventures to create more innovative performance under competitive environments.</t>
@@ -21817,7 +21848,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
           <t>In this dissertation I first develop a theoretical framework that explores different
@@ -21884,7 +21914,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
           <t>Purpose – This study recognizes service as the majority contributor to global and US gross domestic product and the importance of innovation speed to service innovation. Generating innovative products and services at a faster rate generates advantages for business-to-business (B2B) service organizations in keeping up with and moving ahead of rivals. This study aims to introduce the concept of capacity for social exchange (CSE) in buyer–supplier relationships, which reflects the degree to which individuals possess competencies that enable the exchange of information, and this study also explores how CSE affects knowledge sharing and innovation speed within a supply chain organization.</t>
@@ -21927,6 +21956,12 @@
           <t>BSMA0444</t>
         </is>
       </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr"/>
       <c r="G447" t="inlineStr">
         <is>
           <t>Purpose – The authors aim to develop and test hypotheses that link outsourcing and subcontracting-in activities of small high-tech ﬁrms to their radical innovativeness. In addition, they seek to investigate how a ﬁrm’s strategy moderates the associations between their outsourcing and subcontracting-in activities and radical innovativeness.</t>
@@ -21950,6 +21985,11 @@
       <c r="K447" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop 20
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -13217,6 +13217,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -14575,7 +14576,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
           <t>Data from high-technology firms in Hong Kong were used to investigate whether the outcomes of problem-solving processes (solutions found, problem-solving speed, and solution quality) mediated the effects of centrifugal forces (decentralization, free flow of information, and reach) and centripetal forces (connectedness, temporal pacing, project leader expertise, and superordinate goal) on product development performance (development speed and product quality). Centrifugal and centripetal forces were indirectly related to performance through problem-solving outcomes, although some direct effects of these forces were also found. The results suggest a more complex model of product development than previously envisaged.</t>
@@ -14777,7 +14777,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>One of the main reasons that firms participate in alliances is to learn know‐how and capabilities from their alliance partners. At the same time firms want to protect themselves from the opportunistic behavior of their partner to retain their own core proprietary assets. Most research has generally viewed the achievement of these objectives as mutually exclusive. In contrast, we provide empirical evidence using large‐sample survey data to show that when firms build relational capital in conjunction with an integrative approach to managing conflict, they are able to achieve both objectives simultaneously. Relational capital based on mutual trust and interaction at the individual level between alliance partners creates a basis for learning and know‐how transfer across the exchange interface. At the same time, it curbs opportunistic behavior of alliance partners, thus preventing the leakage of critical know‐how between them.</t>
@@ -15097,6 +15096,12 @@
           <t>BSMA0289</t>
         </is>
       </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>This study examines the impacts of problem-solving and administrative communication patterns on the technical performance of 61 projects in an industrial R&amp;D laboratory. While there were no differences in the relative patterns of these two types of communication, there were systematic differences in the mechanisms by which project groups transferred administrative and problem-solving information with other areas both within and outside the organization. The overall patterns of communication were influenced by the nature of the projects' work, while the effectiveness of the various interfaces was explored via two contrasting methods: (1) direct contact by all project members and (2) contact mediated through boundary spanning individuals. The effectiveness of each of these linking mechanisms was also contingent upon the projects' tasks. This research reinforces the importance of managing communication patterns in organizations and further supports the importance of boundary spanning individuals.</t>
@@ -15120,6 +15125,11 @@
       <c r="K292" t="inlineStr">
         <is>
           <t>1979</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15358,6 +15368,16 @@
           <t>BSMA0295</t>
         </is>
       </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G298" t="inlineStr">
         <is>
           <t>Multiple project team membership is a prevalent phenomenon in modern organizational life. However, is any leadership behavior in such a setting beneficial to individual team members’ performance? Our study suggests that working in a multiple project team setting requires particular types of leadership. In an experimental design, we manipulated charismatic and boundary-spanning leadership behaviors in single and multiple team project settings and we studied their effects on project members’ performance. When workers are part of a single team, charismatic leadership enhances their performance to a greater extent than a boundary spanning leader. When members are part of two project teams concurrently, boundary-spanning leadership behavior becomes more beneficial for individual performance compared to charismatic leadership. The main theoretical contribution lies in the insight that different organizational project forms ask for different leadership behaviors to nurture individual performance. Practically, (future) project leaders must be prepared for operating in different project settings.</t>
@@ -15381,6 +15401,11 @@
       <c r="K298" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17905,6 +17930,12 @@
           <t>BSMA0354</t>
         </is>
       </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>Using a longitudinal in-depth field study at NASA, I investigate how the open, or peer-production, innovation model affects R&amp;D professionals, their work, and the locus of innovation. R&amp;D professionals are known for keeping their knowledge work within clearly defined boundaries, protecting it from individuals outside those boundaries, and rejecting meritorious innovation that is created outside disciplinary boundaries. The open innovation model challenges these boundaries and opens the knowledge work to be conducted by anyone who chooses to contribute. At NASA, the open model led to a scientific breakthrough at unprecedented speed using unusually limited resources; yet it challenged not only the knowledge-work boundaries but also the professional identity of the R&amp;D professionals. This led to divergent reactions from R&amp;D professionals, as adopting the open model required them to go through a multifaceted transformation. Only R&amp;D professionals who underwent identity refocusing work dismantled their boundaries, truly adopting the knowledge from outside and sharing their internal knowledge. Others who did not go through that identity work failed to incorporate the solutions the open model produced. Adopting open innovation without a change in R&amp;D professionals’ identity resulted in no real change in the R&amp;D process. This paper reveals how such processes unfold and illustrates the critical role of professional identity work in changing knowledge-work boundaries and shifting the locus of innovation.</t>
@@ -17928,6 +17959,11 @@
       <c r="K357" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P357" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17989,6 +18025,12 @@
           <t>BSMA0356</t>
         </is>
       </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>Triggered by the fierce competition and substantial changes in worldwide markets during the past two decades, an increasing number of firms have adopted a logistics outsourcing strategy to maintain core competencies and gain competitive advantages. Accordingly, the relevant research has achieved both practical and academic attention, ranging from the type of logistics activities outsourced, the motivation for such operations, and the positive and/or negative results of the actions. Nevertheless, the relevant supply chain management (SCM) literature is sparse and scattered and thus considerable opportunities remain for further exploration, especially in logistics outsourcing relationship management (LORM). Unfortunately, due to various reasons such as the dominant focus on organisational level issues, the difficulty of evaluating people issues and the lack of a comprehensive theoretical foundation, the literature thus far has not adequately explored this phenomenon.</t>
@@ -18012,6 +18054,11 @@
       <c r="K359" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P359" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18026,6 +18073,12 @@
           <t>BSMA0357</t>
         </is>
       </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>Driven by fierce global competition, flatter organizational structures and the growing complexity of tasks, boundary spanning behavior (BSB) in externally dependent work teams has increasingly been emphasized in both theory and practice. The current study aims to answer the questions of whether, when and how an individual’s BSB impacts his or her task performance within a team. Based on a sample of 272 employees from 57 new product development teams in China, we found that informal leader emergence mediated the relationship between an individual’s BSB and his or her performance within a team. Moreover, group-level power distance positively moderated the association between BSB and informal leader emergence. An overall mediated moderation model of the effect of the interaction between BSB and group power distance (PD) on task performance via informal leadership emergence was also confirmed. In particular, the relationship between BSB and task performance via informal leadership emergence was stronger for teams with less PD than for those with more PD. The implications of the research are discussed.</t>
@@ -18049,6 +18102,11 @@
       <c r="K360" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18063,6 +18121,12 @@
           <t>BSMA0358</t>
         </is>
       </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
           <t>Currently boundary spanning behavior is a hot topic in team research field, which involves phenomena at two levels (team level and individual level). Compared to team level, employee's boundary spanning has not been well discussed yet. In addition, few studies have systematically explored its outcomes and impact mechanism in Chinese context. This study aimed to address the above gaps by examining whether, when and how employee's boundary spanning behavior impacted his or her task performance. Specifically, integrating culture and social network theory into boundary spanning field, this study theorized that boundary spanning behavior led to centrality of the employee's social network, and in turn enhance his or her task behavior. At the same time, team's collectivism climate moderated the above path. The participants were recruited from 17 companies in two high-tech parks located in Beijing and Tianjin, China. We invited 135 team leaders and their subordinates to participate the survey, after collecting 2 wave longitudinal data sets and dropping out invalid questionnaires, responses from 61 team leaders and 292 team members were valid finally. To get enough whole network data, we purposely chose teams with small size. All measurements were (or adapted from) well-established scales. Employee's boundary spanning behavior, centrality, and collectivism were collected at time 1, and after 8 weeks, employees' task performance was collected at time 2. Confirmatory factor analyses showed satisfactory model fit indices. Inter-rated agreement (Rwg) and intra-class correlation (ICC) value justified the aggregation of team collectivism climate. HLM were applied to test our hypotheses since this is a cross-level research. Variables like age, education, gender, tenure and collectivism orientation at individual level, and team size at group level were controlled for. The results showed that centrality of the social network positively mediated the relation between employees' boundary spanning behavior and his or her task performance. The climate of team collectivism positively moderated the relation between employees' boundary spanning behavior and network centrality. In addition, network centrality mediated the interaction between boundary spanning behavior and team collectivism climate on employee's task performance such that the relation between boundary spanning behavior and task performance via network centrality will be stronger for teams higher on collectivism climate than for those lower on collectivism. This study revealed that employee's boundary spanning behavior had positive influence on task performance and confirmed the mechanism between the two constructs. Interestingly, we found collectivism at individual level and at team level had different effects for the effect of boundary spanning behavior, which revealed that in transformational Chinese context, cultural elements at micro levels were worthy of discussing. The finding of mediating mechanism of centrality established a logic chain of" external relationship—internal embeddedness—performance", helping in explaining the formation of performance and social network in teams. Managerial implications, limitations and future directions were discussed at the end.</t>
@@ -18086,6 +18150,11 @@
       <c r="K361" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21961,7 +22030,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F447" t="inlineStr"/>
       <c r="G447" t="inlineStr">
         <is>
           <t>Purpose – The authors aim to develop and test hypotheses that link outsourcing and subcontracting-in activities of small high-tech ﬁrms to their radical innovativeness. In addition, they seek to investigate how a ﬁrm’s strategy moderates the associations between their outsourcing and subcontracting-in activities and radical innovativeness.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_7
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -13217,7 +13217,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -15101,7 +15100,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>This study examines the impacts of problem-solving and administrative communication patterns on the technical performance of 61 projects in an industrial R&amp;D laboratory. While there were no differences in the relative patterns of these two types of communication, there were systematic differences in the mechanisms by which project groups transferred administrative and problem-solving information with other areas both within and outside the organization. The overall patterns of communication were influenced by the nature of the projects' work, while the effectiveness of the various interfaces was explored via two contrasting methods: (1) direct contact by all project members and (2) contact mediated through boundary spanning individuals. The effectiveness of each of these linking mechanisms was also contingent upon the projects' tasks. This research reinforces the importance of managing communication patterns in organizations and further supports the importance of boundary spanning individuals.</t>
@@ -18030,7 +18028,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>Triggered by the fierce competition and substantial changes in worldwide markets during the past two decades, an increasing number of firms have adopted a logistics outsourcing strategy to maintain core competencies and gain competitive advantages. Accordingly, the relevant research has achieved both practical and academic attention, ranging from the type of logistics activities outsourced, the motivation for such operations, and the positive and/or negative results of the actions. Nevertheless, the relevant supply chain management (SCM) literature is sparse and scattered and thus considerable opportunities remain for further exploration, especially in logistics outsourcing relationship management (LORM). Unfortunately, due to various reasons such as the dominant focus on organisational level issues, the difficulty of evaluating people issues and the lack of a comprehensive theoretical foundation, the literature thus far has not adequately explored this phenomenon.</t>
@@ -18078,7 +18075,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>Driven by fierce global competition, flatter organizational structures and the growing complexity of tasks, boundary spanning behavior (BSB) in externally dependent work teams has increasingly been emphasized in both theory and practice. The current study aims to answer the questions of whether, when and how an individual’s BSB impacts his or her task performance within a team. Based on a sample of 272 employees from 57 new product development teams in China, we found that informal leader emergence mediated the relationship between an individual’s BSB and his or her performance within a team. Moreover, group-level power distance positively moderated the association between BSB and informal leader emergence. An overall mediated moderation model of the effect of the interaction between BSB and group power distance (PD) on task performance via informal leadership emergence was also confirmed. In particular, the relationship between BSB and task performance via informal leadership emergence was stronger for teams with less PD than for those with more PD. The implications of the research are discussed.</t>
@@ -18126,7 +18122,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
           <t>Currently boundary spanning behavior is a hot topic in team research field, which involves phenomena at two levels (team level and individual level). Compared to team level, employee's boundary spanning has not been well discussed yet. In addition, few studies have systematically explored its outcomes and impact mechanism in Chinese context. This study aimed to address the above gaps by examining whether, when and how employee's boundary spanning behavior impacted his or her task performance. Specifically, integrating culture and social network theory into boundary spanning field, this study theorized that boundary spanning behavior led to centrality of the employee's social network, and in turn enhance his or her task behavior. At the same time, team's collectivism climate moderated the above path. The participants were recruited from 17 companies in two high-tech parks located in Beijing and Tianjin, China. We invited 135 team leaders and their subordinates to participate the survey, after collecting 2 wave longitudinal data sets and dropping out invalid questionnaires, responses from 61 team leaders and 292 team members were valid finally. To get enough whole network data, we purposely chose teams with small size. All measurements were (or adapted from) well-established scales. Employee's boundary spanning behavior, centrality, and collectivism were collected at time 1, and after 8 weeks, employees' task performance was collected at time 2. Confirmatory factor analyses showed satisfactory model fit indices. Inter-rated agreement (Rwg) and intra-class correlation (ICC) value justified the aggregation of team collectivism climate. HLM were applied to test our hypotheses since this is a cross-level research. Variables like age, education, gender, tenure and collectivism orientation at individual level, and team size at group level were controlled for. The results showed that centrality of the social network positively mediated the relation between employees' boundary spanning behavior and his or her task performance. The climate of team collectivism positively moderated the relation between employees' boundary spanning behavior and network centrality. In addition, network centrality mediated the interaction between boundary spanning behavior and team collectivism climate on employee's task performance such that the relation between boundary spanning behavior and task performance via network centrality will be stronger for teams higher on collectivism climate than for those lower on collectivism. This study revealed that employee's boundary spanning behavior had positive influence on task performance and confirmed the mechanism between the two constructs. Interestingly, we found collectivism at individual level and at team level had different effects for the effect of boundary spanning behavior, which revealed that in transformational Chinese context, cultural elements at micro levels were worthy of discussing. The finding of mediating mechanism of centrality established a logic chain of" external relationship—internal embeddedness—performance", helping in explaining the formation of performance and social network in teams. Managerial implications, limitations and future directions were discussed at the end.</t>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_8
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -1727,7 +1727,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Qualitative study (autoethnography) lacking extractable quantitative effect sizes.. Verbatim Evidence: [Abstract] "The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegroâs anti-doping policy with WADA." [3.2. Collaborative Autoethnography] "Qualitative in nature, autoethnography is a method that shifts the attention from the perceived reality of research participants to the researcher him/herself (as a subject), thereby giving them a voice towards explaining the phenomenon under study in a self-reflective and often critical, fashion (Ellis &amp; Bochner, 2000)."</t>
+          <t>Qualitative study (autoethnography) lacking extractable quantitative effect sizes.. Verbatim Evidence: [Abstract] "The study employs a collaborative analytical autoethnography where, through memo-writings, emails, and reflective notes by the second author, it micro-theorizes the political, technical, and cultural activities that the institutional entrepreneur carried in order to harmonize Montenegro’s anti-doping policy with WADA." [3.2. Collaborative Autoethnography] "Qualitative in nature, autoethnography is a method that shifts the attention from the perceived reality of research participants to the researcher him/herself (as a subject), thereby giving them a voice towards explaining the phenomenon under study in a self-reflective and often critical, fashion (Ellis &amp; Bochner, 2000)."</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>[Code 4 &amp; Code 3 &amp; Code 1] Conceptual paper on macro-level supply chain network design.. Verbatim Evidence: [Conceptual study on supply chain network design]. Verbatim Evidence: "[Abstract] Designing a supply chain network provides the basic structure for supply chain operations, where the network is a ma-jor element in a ï¬rmâs competitiveness and a signiï¬cant area ofcapital investment." "[1. Introduction] In this article, the impact of the supply chain move-ment on facility location analysis will be examined tosee the challenges posed to traditional location method-ology."</t>
+          <t>[Code 4 &amp; Code 3 &amp; Code 1] Conceptual paper on macro-level supply chain network design.. Verbatim Evidence: [Conceptual study on supply chain network design]. Verbatim Evidence: "[Abstract] Designing a supply chain network provides the basic structure for supply chain operations, where the network is a ma-jor element in a ﬁrm’s competitiveness and a signiﬁcant area ofcapital investment." "[1. Introduction] In this article, the impact of the supply chain move-ment on facility location analysis will be examined tosee the challenges posed to traditional location method-ology."</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix.. Verbatim Evidence: [Reason summary] The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix. Verbatim Evidence: "[Sampling and data collection procedure] The research team received approval from 14 hotelsâ Management to collect data from their FLEs." "[Sampling and data collection procedure] At time II 309 questionnaires were redistributed, and 250 responses were used after deletion of unusable and incomplete questionnaires." "[Measures] Staffsâ COBSBs were assessed with the scale developed by Bettencourt et al. (2005) that measures service delivery with 5 items, internal influence and external representation with both 4 items." "[Results] Table 2. Intercorrelations and discriminant validity criterion."</t>
+          <t>The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix.. Verbatim Evidence: [Reason summary] The study uses a quantitative design with an employee sample, measures customer-oriented boundary spanning behaviors, and includes a zero-order correlation matrix. Verbatim Evidence: "[Sampling and data collection procedure] The research team received approval from 14 hotels’ Management to collect data from their FLEs." "[Sampling and data collection procedure] At time II 309 questionnaires were redistributed, and 250 responses were used after deletion of unusable and incomplete questionnaires." "[Measures] Staffs’ COBSBs were assessed with the scale developed by Bettencourt et al. (2005) that measures service delivery with 5 items, internal influence and external representation with both 4 items." "[Results] Table 2. Intercorrelations and discriminant validity criterion."</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Valid measurement of Leader Boundary Spanning Behavior (scouting, persuading) with real employee sample and extractable correlation matrix.. Verbatim Evidence: [Sample] "Data were collected from 92 management teams from 92 public educational organizations in Israel." [Sample] "School administrators, usually the principal, typically serve as the leaders of these teams." [Measures] "external scouting (six items, for example, âHow often does the leader seek information and advice from peers for the teamâs benefit,â Î± = .89); external persuading (seven items, for example, âHow often does the leader act as a representative of the team with parts of the school environmentâ [parents, educational ministry, district], Î± = .92)" [Correlation Matrix] "Table 1. Descriptive Statistics and Intercorrelation Matrix for Study Variables, N = 92."</t>
+          <t>Valid measurement of Leader Boundary Spanning Behavior (scouting, persuading) with real employee sample and extractable correlation matrix.. Verbatim Evidence: [Sample] "Data were collected from 92 management teams from 92 public educational organizations in Israel." [Sample] "School administrators, usually the principal, typically serve as the leaders of these teams." [Measures] "external scouting (six items, for example, “How often does the leader seek information and advice from peers for the team’s benefit,” α = .89); external persuading (seven items, for example, “How often does the leader act as a representative of the team with parts of the school environment” [parents, educational ministry, district], α = .92)" [Correlation Matrix] "Table 1. Descriptive Statistics and Intercorrelation Matrix for Study Variables, N = 92."</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Sample and data collection] "Overall, we received usable data from 244 respondents in 122 units, yielding a response rate of 76.7 percent." [Measures] "In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit." [Level of analysis] "We performed three tests to determine whether the data should be aggregated to the unit level (see Table 1)." [RESULTS] "Table 2. Means, standard deviations, and Pearsonâs correlations between research variables... N = 122"</t>
+          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Sample and data collection] "Overall, we received usable data from 244 respondents in 122 units, yielding a response rate of 76.7 percent." [Measures] "In this study, the unit was considered to be the level of analysis. Hence, all measures were specified at the unit level. Respondents were asked to evaluate the relational capital, knowledge combination capabilities, and performance of the unit." [Level of analysis] "We performed three tests to determine whether the data should be aggregated to the unit level (see Table 1)." [RESULTS] "Table 2. Means, standard deviations, and Pearson’s correlations between research variables... N = 122"</t>
         </is>
       </c>
     </row>
@@ -5835,6 +5835,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>A number of studies have found that the performance of NPD projects greatly depends on the support they get from top management. However, research into why some projects get more support than others has been limited. The present paper takes a political approach to NPD, in which top management support is considered to be a function of a project leader’s ability to influence decision processes through personal relationships. Mobilizing the bridging perspective of social capital, we argue that project leaders need both strong ties to high-ranking others and sparseness in their networks. Vertical strong ties bring direct support and solidarity, resulting in improved access to resources and priority over other projects; sparseness provides exposure to the full range of information and interpretations in the organization, resulting in a more accurate picture of the political landscape and thus enabling the implementation of an appropriate influence strategy. A PLS analysis of a sample of 73 French project leaders involved in NPD projects provided support for our hypotheses. Hence, we contribute to a very recent stream of research showing that the structural and relational dimensions of social capital are complementary.</t>
@@ -6216,6 +6217,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>This paper contributes to open innovation (OI) and boundary spanning literatures by providing a first understanding of industry‐based boundary spanners in university‐industry (U‐I) collaboration through case studies of Chinese multinational corporations (MNCs) and their international OI platforms. Organisational roles created by these platforms within the MNCs and their activity of bridging between organisations are examined. The analysis of 25 in‐depth interviews in two MNCs located in eight countries, along with internal documents, sheds light on U‐I collaboration practices implemented by Chinese MNCs. Two new boundary spanning roles are identified:               Dual Cultural Bridger               – as these OI platforms bridge organisational and national cultural gaps to prevent and solve problems in the collaborative process; and               International Network Enhancer               – as these OI platforms act as trust building and local knowledge listening posts for the MNC’s global network. Managerial and policy implications are provided.</t>
@@ -6409,6 +6411,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>In this paper, we highlight the networked context of the professions. In particular, we indicate that neo-classical professionals tend to work across organizational boundaries in project teams, often to meet the needs of clients and the wider society. However, little is known about the resources that professionals draw on to meet immediate, fast paced, client demands in project network organizations (PNOs). We pinpoint how knowledge resources, human, social and organizational capital enable professionals to produce outputs at a fast pace/tempo. Temporality emerged as an unexpected but key issue in our empirical research and we explore this further here. First, we put forward how professional work organization(s) has changed by focusing on the boundaries of organizations, and how this is often temporary and project-driven. Second, we use the speciﬁc lens of knowledge resources which are drawn upon to enable networked working and ask the question: which knowledge resources enable professionals to work at a fast pace within networks? Third, appreciative of the vast literature on temporary and networked organizations in professional work, our focus is beyond a single profession or organization, and hence, we build upon the prior research on PNOs. We do this by drawing on empirical data of a humanitarian aid project networked organization (HN) that upscales across its network at high speed, often within days, to generate funds for humanitarian disasters in order to save lives.</t>
@@ -6456,6 +6459,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>This research examines the mechanisms through which entrepreneurial orientation (EO) aﬀects ﬁrm performance in an emerging market context. We argue that EO drives ﬁrms to develop the dynamic capabilities of absorptive capacity (ACAP) and boundary-spanning (BS), and that these capabilities enhance ﬁrm performance. Moreover, the eﬀectiveness of these knowledge- and network-based dynamic capabilities in mediating the EOperformance relationship is contingent on the institutional conditions ﬁrms are exposed to. We test our hypotheses using multi-sourced data on Chinese high-tech ﬁrms in business-to-business (B2B) markets. Our results show that ACAP and BS mediate the positive eﬀect of EO on ﬁrm performance, and that as the development of market-supporting institutions improves, the mediating eﬀect of ACAP becomes stronger while that of BS weakens.</t>
@@ -6550,6 +6554,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>Our study responds to a call for research to integrate institutional, organizational and individual levels of analysis in examining the implications for work and employment relations of new organizational forms. We empirically examine the implementation of network forms of genetics healthcare delivery that cross organizational and professional boundaries. We highlight that less powerful professional groups may find difficulty in enacting boundary-spanning roles associated with new organizational forms. This is due, first, to inconsistency of government policy, which fragments organizations. Second, professional institutions sustain professional hierarchy and power differentials.</t>
@@ -6597,6 +6602,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to test the inﬂuence of external information search (EIS) on knowledge elaboration and group cognitive complexity (GCC) under the moderating effect of absorptive capacity (AC is indicated by prior knowledge base and gender diversity).</t>
@@ -6931,6 +6937,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>This study investigated coordinated action in multiteam systems employing 233 correspondent systems, comprising 3 highly specialized 6-person teams, that were engaged in an exercise that was simultaneously “laboratory-like” and “field-like.” It enriches multiteam system theory through the combination of theoretical perspectives from the team and the large organization literatures, underscores the differential impact of large size and modular organization by specialization, and demonstrates that conventional wisdom regarding effective coordination in traditional teams and large organizations does not always transfer to multiteam systems. We empirically show that coordination enacted across team boundaries at the component team level can be detrimental to performance and that coordinated actions enacted by component team boundary spanners and system leadership positively impact system performance only when these actions are centered around the component team most critical to addressing the demands of the task environment.</t>
@@ -7025,6 +7032,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>In this article, the authors examine antecedents and consequences of the service climate in boundary-spanning self-managing teams (SMTs) that deliver financial services. Using data from members of 61 SMTs and their customers, the authors show a differential impact of the SMT service climate on various marketing performance measures. Furthermore, they obtain support for independent group-level effects of intrateam support and team member flexibility on employee perceptions of the SMT service climate. Both effects are persistent over time and demonstrate that collective perceptions in the SMT have incremental value in the explanation of the service climate.</t>
@@ -7166,6 +7174,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>This manuscript investigates the role of individual team members' breadth of functional experience for their interteam coordination behavior. Integrating personal construct and social identity theories, we examine interpersonal cognitive complexity as a mediating variable and organizational identification as a moderator. We test our hypotheses across two independent field studies, comprising an international peace support training mission (Study 1) and a municipality administration (Study 2). Corroborating our predictions, interpersonal cognitive complexity appeared as a conditional mediating variable that can translate an individual's breadth of functional experience into interteam coordination. The strength and direction of this indirect relationship, however, depended on the individual's identification with the organization as a whole. Moreover, on the team level of analysis, we found members' overall interteam coordination to positively relate with team performance in Study 2. All in all, this paper advances new knowledge on the antecedents, mechanisms, contingency factors, and team-level consequences of members' boundary spanning.</t>
@@ -7405,6 +7414,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>This article develops a framework for studying cross-functional teams in organizations that focuses on three domains: organizational context, internal process, and outcome measures. The framework was developed from qualitative data from over 200 individual and group interviews, written descriptions, and team observations. We then operationally defined this model through a set of questionnaire items and validated it through quantitative analysis of data from 565 members of cross-functional teams. The resulting framework provides a base for the future study of cross-functional teams.</t>
@@ -7452,6 +7462,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>When working as a member of a team, individuals must make decisions concerning the allocation of resources (eg, effort) toward individual goals and team goals. As a result, individual and team goals, and feedback related to progress toward these goals, should be potent levers for affecting resource allocation decisions. This research develops a multilevel, multiple-goal model of individual and team regulatory processes that affect the allocation of resources across individual and team goals resulting in individual and team performance. On the basis of this model, predictions concerning the impact of individual and team performance feedback are examined empirically to evaluate the model and to understand the influence of feedback on regulatory processes and resource allocation. Two hundred thirty-seven participants were randomly formed into 79 teams of 3 that performed a simulated radar task that required teamwork. Results support the model and the predicted role of feedback in affecting the allocation of resources when individuals strive to accomplish both individual and team goals.</t>
@@ -8050,7 +8061,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>Construct Homonymy (Boundaryless Career). The study measures cross-boundary mobility preferences (career mobility / turnover intention) across jobs, organizations, and industries, not interpersonal Boundary Spanning Behavior.. Verbatim Evidence: [Introduction] "First, we take into account the multiplicity of career boundaries (job, organisation and industry), refining the understanding of âboundaryâ in boundaryless careers (Inkson et al. 2012)." [Measures] "For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference." [Measures] "We created the mobility preference variables using individualsâ responses to this question: âIn regard to your job, where do you want to be in 12 monthsâ time?â"</t>
+          <t>Construct Homonymy (Boundaryless Career). The study measures cross-boundary mobility preferences (career mobility / turnover intention) across jobs, organizations, and industries, not interpersonal Boundary Spanning Behavior.. Verbatim Evidence: [Introduction] "First, we take into account the multiplicity of career boundaries (job, organisation and industry), refining the understanding of ‘boundary’ in boundaryless careers (Inkson et al. 2012)." [Measures] "For dependent variables, we created three binary variables using the individual survey in the AWRS data: cross-job mobility preference, cross-organisation mobility preference and cross-industry mobility preference." [Measures] "We created the mobility preference variables using individuals’ responses to this question: ‘In regard to your job, where do you want to be in 12 months’ time?’"</t>
         </is>
       </c>
     </row>
@@ -9194,7 +9205,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 3] Qualitative field study conducted at the organizational level without extractable effect sizes.. Verbatim Evidence: [Abstract] "This investigation explores the external motivators of self-assessment through a field study of 14 organizations." [Research method] "The research was carried out in 14 organizations." [Research method] "While Glaser and Straussâs (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion."</t>
+          <t>[Code 1 &amp; Code 3] Qualitative field study conducted at the organizational level without extractable effect sizes.. Verbatim Evidence: [Abstract] "This investigation explores the external motivators of self-assessment through a field study of 14 organizations." [Research method] "The research was carried out in 14 organizations." [Research method] "While Glaser and Strauss’s (1967) grounded theory notion provided a useful methodological framework, we found the techniques of Strauss and Corbin (1990) and Miles and Huberman (1994) effective for operationalizing the theoretical insights from our qualitative data in a systematic fashion."</t>
         </is>
       </c>
     </row>
@@ -9725,6 +9736,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>This study investigated how a project group deals with the contradiction between distributed knowledge in boundary-spanning collaborative processes and the expectation that software systems will provide unified, codified knowledge. It employed an ethnographic, interpretive approach to examine the ways in which relevant knowledge was presented, recognized, shared or otherwise managed during a project concerned with the joint design of business process and IT systems change. Developing a group understanding of how to manage sensemaking and expertise across salient knowledge boundaries were discovered to be central to perceptions of project completion. Four stages of this development were identified. The contribution of this paper is to propose these stages as the basis for boundary-spanning group management approaches and to suggest ways of progressing the complexities of communication, consensus-building, information exchange, problem-formulation and solution-brokering that are fundamental to collaboration in IS definition. These processes are normally taken for granted, rationalized or ignored by managers of IT-related organizational change. The use of specific types of boundary-object may aid in managing such processes explicitly and ensuring rapid progress. Thus the findings have significant implications for research and practice in other forms of boundary-spanning group collaboration, such as organizational innovation and problem-solving.</t>
@@ -9772,6 +9784,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>Research Summary: This paper builds theoretical arguments and shows empirical evidence of the direct benefits and indirect costs of corporate volunteering in developing countries. Spanning corporate and humanitarian sectors to work in challenging environments should activate motivational and learning benefits for participating employees. However, results from a field study of a 10-year partnership between logistics provider TNT and the United Nations World Food Program show that such boundary-spanning corporate social responsibility (CSR) can be a double-edged sword. Task interdependence with nonprofit peers while volunteering strengthens employees' partnership identification and institutional learning. However, institutional learning triggers identity strain (associated with attrition) when they return, unless firms foster a sense that they recognize CSR experiences as valuable. The findings inform the behavioral and microfoundations of the potential consequences of CSR.</t>
@@ -10101,6 +10114,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>Aim: To identify learning from a clinical microsystems (CMS) quality improvement initiative to develop a more integrated service across a falls care pathway spanning community and hospital services. Background: Falls present a major challenge to healthcare providers internationally as populations age. A review of the falls care pathway in Sheffield, United Kingdom, identified that pathway implementation was constrained by inconsistent coordination and integration at the hospital–community interface. Approach: The initiative utilised the CMS quality improvement approach and comprised three phases. Phase 1 focussed on developing a climate for change through engaging stakeholders across the existing pathway and coaching frontline teams operating as microsystems in quality improvement. Phase 2 involved initiating change by working at the mesosystem level to identify priorities for improvement and undertake tests of change. Phase 3 engaged decision makers at the macrosystem level from across the wider pathway in achieving change identified in earlier phases of the initiative. Findings: The initiative was successful in delivering change in relation to key aspects of the pathway, engaging frontline staff and decision makers from different services within the pathway, and in building quality improvement capability within the workforce. Viewing the pathway as a series of interrelated CMS enabled stakeholders to understand the complex nature of the pathway and to target key areas for change. Particular challenges encountered arose from organisational reconfiguration and cross-boundary working. Conclusion: CMS quality improvement methodology may be a useful approach to promoting integration across a care pathway. Using a CMS approach contributed towards clinical and professional integration of some aspects of the service. Recognition of the pathway operating at meso- and macrosystem levels fostered wider stakeholder engagement with the potential of improving integration of care across a range of health and care providers involved in the pathway.</t>
@@ -10195,6 +10209,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>Global offshoring has become a key strategy for international staffing, especially in the software industry. Global software teams engage in boundary spanning activities that may help MNEs achieve international connectivity and cope with external disruptions through their use of virtual work. However, offshoring IT professionals who bridge these boundaries in offshoring MNEs must contend with discontinuities, or perceived disruptions in expected communication flows, which impact their job satisfaction. Drawing on survey data from 193 professional consultants from an IT services offshoring MNE located primarily in Eastern Europe and working for a U.S. client, we test a model grounded in Organizational Discontinuity Theory. We find that potential discontinuities arising from the virtual work environment have no impact on the job satisfaction of offshoring IT professionals, but that those who experience team-level continuities of identification and shared vision are more satisfied with their jobs. Our findings suggest that virtual work may have become normalized such that it is not problematic in and of itself, and that fostering connectivity in boundary spanning global teams may be beneficial for MNEs. Our findings have important implications for MNEs managing disruptions created by global work arrangements as well as exogenous disruptions.</t>
@@ -10242,6 +10257,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>Acknowledgements: This research was funded by NSF grant #0422676 and #0726798 as well as support provided by the University of California, Irvine Center for Research on Information Technology in Organizations. The authors would like to acknowledge the helpful comments provided by Christopher Earley, Mark Griffin, John Mathieu, and Jone Pearce; assistance in data collection provided by Diaky Diaz, Christopher Reisdel and Bettina Wolf; and the generous time invested by all the film makers and film viewers who participated in the study.</t>
@@ -10383,6 +10399,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>Compared to job-specific conditions, the interpersonal context of work has received less attention from work–family scholars. Using data from a 2007 U.S. survey of workers (N = 1,286), we examine the impact of workplace social support and interpersonal conflict on work–family conflict and exposure to boundary-spanning demands—as indexed by the frequency that workers receive work-related contact outside of normal work hours. Findings indicate that workplace social support is associated negatively with work-to-family conflict, while interpersonal conflict at work is associated with higher levels of work-to-family conflict. Results also indicate that both supportive and conflictive work contexts are associated with more frequent exposure to boundary-spanning demands. However, workers in supportive contexts are more likely to appraise these demands as beneficial for accomplishing work tasks, and are less likely to appraise them as disruptive to family roles. By contrast, workers in conflictive contexts are more likely to appraise demands as disruptive to family roles, and are less likely to appraise them as beneficial for paid work. Consequently, our findings underscore the resource and demands aspects of interpersonal work contexts and their implications for the work–family interface.</t>
@@ -10850,6 +10867,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>T h i s position paper distinguishes different types of activities needed in software processes and proposes enaction support for t h e m . An architecture of enaction components providing this support is sketched.</t>
@@ -12497,6 +12515,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>There appears to be a consensus that organizational integration across functional and disciplinary specialties drives superior ﬁrm capabilities. The basic assumption is that new practices and concepts emerge from the interaction of individuals engaged in different functional departments. However, communication across functional boundaries is often difﬁcult. As such, Tushman &amp; Scanlan suggested that functional boundaries can be spanned effectively only by boundary spanners who understand the coding schemes that are attuned to the contextual information on both sides of the boundary. The study of boundary spanners has signiﬁcant performance implications to ﬁrms. Compared to its importance, theoretical development and empirical inquiries into this phenomenon are relatively scant. Thus, this study explores the factors that determine who becomes a boundary spanner and examines boundary spanners’ performance implications. A Taiwanese company provided the context for our study. Partial Least Squares (PLS) was used to test the theoretical model. The results imply that a company needs to have an appropriate mixture of boundary spanners and non-boundary spanners, because boundary spanners have higher innovative performance.</t>
@@ -13123,6 +13142,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>This study examines the relationships between career decisions and directions and a set of independent variables including job title, demographic variables, role stressors, boundary spanning activities, perceived job characteristics, and career outcomes for 348 IS employees. Results show that the majority had already defined specific jobs they would like to hold in the near future. They were also able to define four directions for their future careers: IS technical, IS management, business, and consultant. Results show that career decisions and directions are related to some of the independent variables. IS employees in each of the four career directions could be further categorized into groups on the basis of similar characteristics. Implications of theses findings are discussed.</t>
@@ -13546,6 +13566,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>Two main targets of contemporary preferential innovation policy support, especially in Europe, are key enabling technologies (KETs) and innovation ‘missions’ focused on solving societal challenges. Both topics are associated with uniting disparate sets of capabilities, either by driving technology-based innovation into various application domains or by eliciting interdisciplinary and cross-sectoral solutions to urgent societal demands. In this study we assess to what extent pre-commercial R&amp;D collaborations span geographic and cognitive boundaries. We analyze firm-level tie formation in Dutch collaborative R&amp;D projects initiated in the period 2013–2018. Gravity models reveal that, while results for geographic proximity are mixed, some KET types are indeed related to projects in which cognitive proximity is significantly less relevant for tie formation. This contrasts with the findings for projects that retroactively received a mission label. Projects on health and care missions, and especially energy transition and sustainability missions, instead spur collaborations between cognitively proximate firms. The latter suggests that without additional policy intervention, such projects might interconnect similar rather than dissimilar knowledge bases. We conclude by discussing research and policy implications.</t>
@@ -13734,6 +13755,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>The impact of perceived environmental demands on the roles and job satisfaction of the school psychologist in rural school systems was explored. Superintendents rated their perceptions of the community context and the psychologist’s involvement in interagency linking functions. School psychologists rated their performance of boundary-spanning functions and their job perceptions. Results indicated that certain perceived environmental pressures are related to the performance of boundaryspanning activities. Those who performed boundary-spanning functions are more satisfied with their jobs and more influential in determining their roles.</t>
@@ -13781,6 +13803,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>Purpose – In today’s digital and post-pandemic era, construction teams can span their boundary to obtain important resources and support in computer-mediated ways. However, the benefits of computer-mediated team boundary spanning (TBS) are mostly assumed. Empirical evidence for these benefits is in lack. Thus, this study attempts to investigate the influence of computer-mediated (instant messaging in this study) TBS on construction project performance and the underlying mechanism.</t>
@@ -14303,6 +14326,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>Firms are challenged to achieve organizational goals in an environment of increasingly decentralized information. Cross-functional project teams are employed widely as a strategy to facilitate better coordination, yet projects still fail at a rate of 31% per year. Communication is a leading cause of failure. While inter-team communication has been studied extensively, less is understood about the intra-team communication of a cross-functional project team.</t>
@@ -14776,6 +14800,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>One of the main reasons that firms participate in alliances is to learn know‐how and capabilities from their alliance partners. At the same time firms want to protect themselves from the opportunistic behavior of their partner to retain their own core proprietary assets. Most research has generally viewed the achievement of these objectives as mutually exclusive. In contrast, we provide empirical evidence using large‐sample survey data to show that when firms build relational capital in conjunction with an integrative approach to managing conflict, they are able to achieve both objectives simultaneously. Relational capital based on mutual trust and interaction at the individual level between alliance partners creates a basis for learning and know‐how transfer across the exchange interface. At the same time, it curbs opportunistic behavior of alliance partners, thus preventing the leakage of critical know‐how between them.</t>
@@ -14892,7 +14917,7 @@
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 2] Qualitative study measuring identity boundary-work among solo self-employed individuals (non-employees).. Verbatim Evidence: [Study design] "This article is based on in-depth interviews with 30 subjects—15 men and 15 women." [Abstract] "This article proposes to examine the self-concept of members of an occupational category referred to as the 'solo self-employed'—women and men who work alone and do not employ other workers." [Solo self-employed criteria] "Self-employed business owners, registered as such with the authorities for one year or more."</t>
         </is>
       </c>
     </row>
@@ -15192,6 +15217,16 @@
       <c r="B294" t="inlineStr">
         <is>
           <t>BSMA0291</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -15233,6 +15268,11 @@
           <t>2009</t>
         </is>
       </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -15245,6 +15285,12 @@
           <t>BSMA0292</t>
         </is>
       </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>Boundary -spanning activity (BSA) was studied in two departments of a large governmental research and develop ment organization. BSA was found to be higher and to have significant effects for employees when departmental goals were unclear and technology was non-routine. Under these conditions, BSA was negatively related to role ambiguity and positively related to job satisfaction. Contrary to prior re search, this study found roles with high levels of BSA to have favorable aspects for their incumbents depending upon gorl clarity and type of technology of the parent organization. Implications for the management of research and development organizations are discussed.</t>
@@ -15268,6 +15314,11 @@
       <c r="K295" t="inlineStr">
         <is>
           <t>1975</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15282,6 +15333,16 @@
           <t>BSMA0293</t>
         </is>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G296" t="inlineStr">
         <is>
           <t>The article reports on the importance of boundary-spanning roles (BSA), which serve to link organizations confirmed by research. They are vital to the effective monitoring of the environment as well as the transfer of technology and information across boundaries. Research has shown boundary-spanning activity (BSA) to have negative effects for their incumbents, such as higher rates of marginality. Marginality is defined as one's self-orientation when presented with two or more groups with conflicting value systems. Boundary spanning activity could be positively related to levels of role conflict and ambiguity or negatively related to levels of job satisfaction. Research is conducted to test to the theory of role dynamics in BSA.</t>
@@ -15305,6 +15366,11 @@
       <c r="K296" t="inlineStr">
         <is>
           <t>1975</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>Valid individual-level quantitative study measuring Boundary-Spanning Activity of professional employees with an extractable correlation matrix.. Verbatim Evidence: [Method] "The sample of 51 professional employees (a 58 percent response rate) was similar to its population in age, work experience, and education." [Method] "To measure the level of BSA, a four item scale was constructed based on items successfully used in prior research (1, 2, 4)." [Method] "(c) During the last month, indicate the frequency with which you have sought information/advice from members of other organizations outside (name of organization)."</t>
         </is>
       </c>
     </row>
@@ -15373,7 +15439,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
+          <t>2 = Non-employee samples</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -15403,7 +15469,7 @@
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Excluded because the study relies on a student sample (undergraduate students participating in an experimental simulation) rather than organizational employees.. Verbatim Evidence: [3.4. Participants] "Participants of the study were 118 undergraduate students (age MEAN = 21.55, with 91 females, 77 % of the sample) enrolled at a Dutch university, who were randomly assigned to project teams, as part of a course." [3.4. Participants] "In the simulation, participants experienced project work in a virtual MTM setting and were invited to write a reflection assignment based on it." [3.4. Participants] "We chose a student sample for two main reasons."</t>
         </is>
       </c>
     </row>
@@ -15455,6 +15521,16 @@
           <t>BSMA0297</t>
         </is>
       </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="G300" t="inlineStr">
         <is>
           <t>Purpose – Our paper examines how entrepreneurial leadership (EL) impacts firm export innovativeness via digital transformation and supply chain agility. Using the dynamic capability view theory, our paper also explores the moderating impact of leaders’ boundary-spanning behavior on the connection between EL and export innovativeness.</t>
@@ -15478,6 +15554,11 @@
       <c r="K300" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15492,6 +15573,16 @@
           <t>BSMA0298</t>
         </is>
       </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G301" t="inlineStr">
         <is>
           <t>Given the growing importance of B2B digital platform capabilities for competitive advantage, research on its antecedents and outcomes in the business-to-business context remains scarce. To address this gap, we built on dynamic capability theory to examine how B2B organizations’ digital platform capabilities contribute to sustainable positioning. Specifically, we examined the direct and indirect associations (via organizational knowledge depth, breadth, and agility) between digital platform capabilities and sustainable positioning. Additionally, we explored the moderating role of leader boundary-spanning behaviors in the relationship between digital platform capabilities and organizational knowledge depth and breadth. Our study based on two-source survey data from top management in Chinese manufacturing firms. The findings fully support all our proposed hypotheses. Digital platform capabilities significantly enhance sustainable positioning, both directly and through improved organizational knowledge depth, breadth, and agility. Furthermore, leader boundary-spanning behaviors strengthen the impact of digital platform capabilities on both knowledge depth and breadth. These insights offer practical implications for B2B firms seeking to leverage digital platform capabilities to enhance knowledge depth, breadth, agility, and sustainable market positioning.</t>
@@ -15515,6 +15606,11 @@
       <c r="K301" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>Valid individual-level Leader Boundary Spanning Behavior self-rated by top managers.. Verbatim Evidence: [3.1. Sample and procedure] "Through the alumni, we were able to approach the top managers of 600 organizations (CEOs, general managers, and managing directors) to invite them to participate in our study." [3.2. Measures and variables] "We assessed leader boundary-spanning behavior by adapting six items (α = 0.96) from Ancona and Caldwell (1992). Sample item: “I reach out to individuals outside of our organization who can offer expertise or ideas.”" [Appendix A. Scale Items] "A.6. Leader boundary-spanning behavior LBBs1: I absorb outside pressures so that organizational members can work free of interference. LBBs2: I persuade outsiders (e.g., clients, stakeholders) to support organizational decisions."</t>
         </is>
       </c>
     </row>
@@ -15566,6 +15662,16 @@
           <t>BSMA0300</t>
         </is>
       </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G303" t="inlineStr">
         <is>
           <t>Innovation and knowledge creation are processes, which require intensive collaboration of several people. Nevertheless, the constituents of successful collaboration in innovation activities are not well-known, and the understanding of the inherently social processes by which new intangibles are created is still in its infancy. This paper examines the key facilitators of innovation in knowledge-intensive group-level collaboration based on empirical evidence. The results demonstrate that social factors are highly influential for knowledge worker teams’ ability to produce innovations. Teams whose internal processes were characterised by trust, vision, aim for excellence, participative safety and support for innovation were likely to attain high levels of innovation. Team diversity based on highly visible attributes was found to be negatively related with team innovation. Surprisingly, also external collaboration seemed to affect team innovation outcomes negatively, except for when it was aimed at general scanning for ideas and information. In addition, the differences between the more and the less innovative teams arose mainly from differences in their internal interaction processes, rather than patterns of collaboration with people outside the team.</t>
@@ -15589,6 +15695,11 @@
       <c r="K303" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15714,6 +15825,16 @@
           <t>BSMA0304</t>
         </is>
       </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G307" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this research is to examine the positive relationship between leader’s boundaryspanning behavior and employee creative behavior. Moreover, the research investigates a three-way effect by exploring leader’s boundary-spanning behavior, need for status and creative self-efficacy on employee creative behavior.</t>
@@ -15737,6 +15858,11 @@
       <c r="K307" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>Valid individual-level Leader Boundary Spanning Behavior (rated by subordinates), providing an extractable correlation matrix.. Verbatim Evidence: [Sample] "We distributed pairs of survey packages to students enrolled in an executive MBA program at a university in South Korea. We collected data from various companies mainly manufacturing, finance and IT services." [Level of Analysis] "a total of 260 pairs were used for final analyses representing a subordinate-supervisor ratio of 1.37:1." [Measures] "Leader boundary-spanning behavior. We assessed leader’s boundary-spanning behavior using 6 items of Marrone et al.’s (2007). A sample item is, “My team leader reaches out to individuals outside of our team that can provide project-related expertise or ideas”." [Cross-Entity Rating] "employee creative behavior was rated by the employees’ direct supervisor while other variables (i.e. leader’s boundary-spanning behavior, need for status, creative self-efficacy and control variables) were rated by the employees."</t>
         </is>
       </c>
     </row>
@@ -15829,6 +15955,16 @@
           <t>BSMA0307</t>
         </is>
       </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G310" t="inlineStr">
         <is>
           <t>The article examines the process of innovation and knowledge sharing from a perspective that focuses on the inﬂuence that local circumstances can have. In particular, it looks at the problems of knowledge sharing between groups of professionals. It presents a comparative analysis of two studies, one involving two groups of IT professionals; the other a network of healthcare professionals. The data was collected in two sets. The ﬁrst set consisted of the results from two earlier, independent studies; the second was collected speciﬁcally for this article. We investigate the role played by boundary objects and brokers. Through an analysis of the interplay between boundary object and broker, we uncover the dynamics of the innovation process and show that the role played by the broker can be political. We identify two strategies that are used by brokers in the selection of a boundary object. The ﬁrst is directed towards achieving a balance between the actors involved and the second is directed towards controlling their activities. We conclude by suggesting that other researchers should also consider the interplay between broker and boundary object when examining cross-boundary knowledge sharing.</t>
@@ -15852,6 +15988,11 @@
       <c r="K310" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>Qualitative case study based on interviews, lacking any quantitative effect sizes or correlation matrix.. Verbatim Evidence: [Abstract] "The article examines the process of innovation and knowledge sharing from a perspective that focuses on the influence that local circumstances can have. In particular, it looks at the problems of knowledge sharing between groups of professionals. It presents a comparative analysis of two studies, one involving two groups of IT professionals; the other a network of healthcare professionals." [3.1. Methodology] "All of the actors involved were interviewed several times at different points in the process; the interviews lasted from 30 to 90 min." [3.1. Methodology] "The analysis followed what Denzin and Lincoln (2000) describe as a moderate inductive approach." [3.1. Methodology] "Throughout the analysis, we followed the general principles outlined in Miles and Huberman’s (1994) methodological framework: data reduction, coding and analysis based on codes created from a review of the literature and emergent codes created during analysis."</t>
         </is>
       </c>
     </row>
@@ -16199,6 +16340,16 @@
           <t>BSMA0317</t>
         </is>
       </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G320" t="inlineStr">
         <is>
           <t>Creativity is essential for research and development efforts. Unfortunately, little is known about how the role of team leaders determines the team’s creativity. Based on a sample of 39 engineering design teams in the space industry, this study examines the effects of leader position within different ﬂows of communication on team creativity. The results indicate that the balance between holding a central or a peripheral position indeed determines the creativity of such teams. Speciﬁcally, very central and very peripheral positions of team leaders within the work-ﬂow and awareness network hamper team creativity, whereas peripheral situated team leaders within the information network propel the creativity. In addition, team leaders stimulate creativity when they stay central in the external information network. In managerial terms, the analyses implicate that stimulating engineering design team creativity requires team leaders to smartly limit their involvement in communication and mainly act as gatekeepers to external sources of information.</t>
@@ -16222,6 +16373,11 @@
       <c r="K320" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=39 teams). Verbatim Evidence: [Participants] "To explore the social structure of leadership and creativity in engineering design teams, we collected data on 39 engineering design teams with 321 team members engaged in the space industry around the globe in 17 countries." [Aggregation] "We therefore will limit ourselves to incorporating team-level aggregates into our analysis." [Correlation matrix] "Table 2 Descriptives and correlations: main variables (n = 39)."</t>
         </is>
       </c>
     </row>
@@ -16372,6 +16528,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G324" t="inlineStr">
         <is>
           <t>As a core organizational resource, business processes are vital for organizational teams. To deal with today’s volatile business environment, organizations need to be ambidextrous in terms of process capabilities. However, little is known about how process ambidexterity, process standardization, and process agility, are enabled by information technology (IT) and related to team-level activities. To fill this gap in the literature, we conducted a field study based on 160 teams of 1081 individuals from seven companies in South Korea. Our results show that IT enables both process standardization and agility, and that a team’s process ambidexterity has a positive effect on inter-team coordination and team innovation, which in turn have a direct impact on team performance. Our findings highlight the importance of process ambidexterity by investigating the enabling role of IT and its outcomes in a team. Our results offer theoretical and practical implications from the perspective of team process ambidexterity.</t>
@@ -16399,7 +16560,7 @@
       </c>
       <c r="P324" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level analysis (N = 160 teams) using aggregated responses and proxy informants rating team-level behavior.. Verbatim Evidence: [3.1. Data and sample] The final data set for further analysis included 160 teams with 1081 individuals. [4. Results] To use the individuals’ responses for further analysis, the responses were aggregated by extracting the mean scores. To test our hypotheses, we used the partial least squares (PLS) method because of its minimal restrictions on the distribution of residuals and advantage in testing a small sample size (n = 160) [Appendix A] IC2 We had no problems in coordinating with other teams. ... IC5 Our team is able to adjust processes with respect to coordination with other teams.</t>
         </is>
       </c>
     </row>
@@ -16518,6 +16679,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>This study draws on theories of collective action and organizational ecology to investigate a particular type of voluntary association: mixed-mode groups. Mixed-mode groups are created and organized online to meet physically in geographically deﬁned ways. An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups. Analysis shows that even when a mixed-mode group implements strategies focused on internal group processes, it beneﬁts from tapping into its external networks to obtain resources for group operation. Also, the differential impacts of internal and external strategies indicate that in the case of environment-prone mixed-mode groups, implementation of internal strategies alone, with or without solicited external networking resources, is helpful for generating positive group outcomes. Together, these results establish that boundary spanning represents not only a type of strategic action to obtain resources and produce positive outcomes but also an inherent and deﬁning mechanism of contemporary voluntary groups for engaging in collective action.</t>
@@ -16659,6 +16821,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>Abstract                            Research Summary               Organizations often struggle to identify promising innovations that balance novelty and feasibility in multidisciplinary domains, yet how does evaluator expertise heterogeneity shape these assessments? This study examines how evaluator expertise influences innovation evaluation through a field experiment with National Aeronautics and Space Administration's (NASA) Astrobee Robotic Arm Challenge, involving 354 evaluators assessing 101 solutions. Domain‐spanning evaluators assign higher novelty ratings while maintaining similar feasibility ratings compared to domain‐specific evaluators. Domain‐adjacent evaluators show higher ratings on both dimensions. Human‐LLM analysis of 3007 evaluator comments reveals a two‐stage process: feasibility filtering (evaluating minimum viability) followed by integrative assessment (evaluating enhancement potential). Different expertise types serve complementary functions: domain‐spanning evaluators recognize enhancement potential while maintaining rigorous standards; domain‐adjacent evaluators show openness to novel approaches; domain‐specific evaluators ensure technical rigor. These findings suggest effective innovation evaluation depends on strategically combining complementary expertise types rather than identifying optimal individual evaluators.                                         Managerial Summary               Organizations often struggle to identify innovations that are both novel and feasible, risking missed breakthroughs or wasted resources. We study how evaluator expertise shapes innovation assessments in a field experiment with NASA, in which 354 evaluators reviewed 101 robotic arm designs. Evaluators with expertise spanning multiple domains recognize more novel yet feasible ideas. Those with single‐domain expertise provide essential technical gatekeeping but overlook cross‐domain improvements, while adjacent‐field experts are more open but less rigorous. Organizations can strengthen innovation selection by strategically combining these complementary expertise types—using domain‐specific experts for initial feasibility screening and domain‐spanning experts to identify integrative opportunities—rather than seeking one “ideal” evaluator.</t>
@@ -16800,6 +16963,12 @@
           <t>BSMA0330</t>
         </is>
       </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
           <t>The purpose of the study was to explore the relationships among environmental characteristics, uncertainty, boundary spanning activities, managerial discretion, and power of the department store apparel buyer who assumes combination or independent buyer responsibilities. Almubarek’s Model of Organizational Boundary Spanning and Duncan’s (1972) Model of Environmental Uncertainty were used as conceptualframeworks. A questionnaire was mailed to buyers who purchased merchandise in the moderate-to-better sportswear areas in the top 10 department store groups in the United States.</t>
@@ -16823,6 +16992,11 @@
       <c r="K333" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -16842,6 +17016,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>Prompted by the relationship management literature which has appeared recently in marketing, we posit that the performance of sellers in ongoing buyer-seller relationships is influenced significantly by the manner in which sellers interact with buyers, which we refer to as" boundary behavior." Although a growing literature has drawn attention to the importance of relationship management, no research has investigated the extent to which, if any, relationship management leads to improved performance in terms of" hard" measures, such as sales. We fill this gap by examining how managerially controllable boundary behaviors influence sellers' sales performance. We further examine how situational factors moderate these effects, and consequently illuminate contexts in which the actions of boundary spanning personnel are most critical. The findings are likely to be of interest to managers who operate at the organization boundary, and who are therefore concerned with the effective deployment of these important resources.</t>
@@ -16889,6 +17064,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G335" t="inlineStr">
         <is>
           <t>Science parks are a type of organizational sponsorship initiative aimed at generating resource-munificent environments through the provision of bridging and buffering services. While extant research has studied the relationship between these services and firm outcomes, it has neglected to provide insights into when tenant firms utilize these services to a greater or lesser extent. Our study evaluates science parks’ buffering mechanism and identifies firm-level characteristics affecting tenants’ use intensity of buffering services. To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries. Taking a resource dependence perspective, our findings indicate that tenants’ managerial resources (particularly top management team size and functional experience) and boundary-spanning capacity jointly determine the extent to which firms rely upon the science park’s buffering mechanism. This study contributes to the organizational sponsorship, resource dependence, and science park literatures, as well as has important practical implications.</t>
@@ -16916,7 +17096,7 @@
       </c>
       <c r="P335" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Firm-level analysis (N=201 firms) where the manager acts as a key informant reporting on the firm's boundary-spanning capacity.. Verbatim Evidence: [Plain English Summary] "Which firm-level factors determine the use intensity of science parks’ buffering services? We study our research question in a sample of 201 firms located in 35 science parks in Denmark, Spain, and Belgium." [3.1 Data and sample] "In the spring of 2018, we sent out an online survey to these tenants, specifically addressed to the manager in charge of the firm on the SP." [3.1 Data and sample] "As such, our final sample consists of 201 responses from tenants in 35 different SPs." [Appendix 1, Table 5] "Boundary-spanning capacity To which extent does … BS1 … The firm encourages its members to solicit information and resources from elsewhere?"</t>
         </is>
       </c>
     </row>
@@ -17458,6 +17638,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G347" t="inlineStr">
         <is>
           <t>Drawing from team-level job demands-resources theory, we hypothesize that team workload demands moderate the positive link between team boundary work (i.e., boundary spanning and boundary buffering) and team effectiveness (i.e., team innovation and team performance), such that boundary work is more beneficial for team effectiveness when teams face higher team workload demands. Furthermore, we predict that this interaction occurs through increased team vigor, where team vigor is defined as an affective emergent state characterized by positive valences and high activation levels experienced by team members. We largely find support for our model across two field studies: a cross-sectional survey using three independent data sources (89 automotive research and development teams, including 724 team members, 89 team leaders and 18 managers) and a time-lagged survey using two independent data sources (139 teams working in a Chinese utility company, including 640 team members and 139 team leaders). Our article contributes to team research by broadening our understanding of when and how team boundary work is associated with greater team effectiveness.</t>
@@ -17485,7 +17670,7 @@
       </c>
       <c r="P347" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Non-individual level (team analysis). Verbatim Evidence: [Sample] "Our final sample consisted of 89 teams with matched responses between team leaders and team members (724 team members, 89 team leaders, and 18 managers), resulting in a response rate of 87% of the teams (65% for team members, 87% for team leaders, and 82% for managers)." [Aggregation] "To justify the aggregation of boundary spanning, boundary buffering, and team workload demand ratings to the team level, we computed within-group interrater agreement (rwg; James et al., 1993) and intraclass correlation (ICC) values. Boundary spanning had a median rwg value of 0.74 with ICC [1, 2] values of 0.10 and 0.47, respectively. Boundary buffering had a median rwg value of 0.77 with ICC [1, 2] values of 0.18 and 0.63, respectively. Team workload demands had a median rwg value of 0.76 with ICC [1, 2] values of 0.25 and 0.72, respectively. These values provide adequate support for aggregation to the team level (James et al., 1984)." [Correlation Table 1] "Note: N = 89 teams." [Correlation Table 3] "Note: N = 139 teams."</t>
         </is>
       </c>
     </row>
@@ -17505,6 +17690,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G348" t="inlineStr">
         <is>
           <t>Boundary spanning activity Is conceived of as an intervening variable between organization structure and perceived environmental uncertainty. This is because boundary spanners operate at the skin of the organization and hence their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relationships between perceived environmental uncertainty, organization structure, and boundary spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relationships were found between all three variables. Partial relationships indicated that PEtJ does not influence the boundary spanning-structure relationship, but structure reduces the PEtJ-boundary spanning relationship to zero, and boundary spanning reduces the structurePEU relationship to zero. Thus, not only is the boundary spanning as an intervening variable supported, but results suggest that causality in the Btructure-PEU relationship may be in the direction of structure to PEU rather than current contingency notions of PEU effecting structure.</t>
@@ -17532,7 +17722,7 @@
       </c>
       <c r="P348" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Construct is mere communication frequency (hours/times communicating) without purposive boundary spanning action, and study only reports Goodman-Kruskal Gamma (ordinal association) rather than Pearson correlations.. Verbatim Evidence: [Measures of the Variables] "Eight questions concerning the subject's frequency of boundary spanning activity were asked (see Appendix)..." [Appendix] "1a. how many hours do you attend formal meetings, (committees, planning, etc.) ... 1b. how many hours do you confer about your work in informal face-to-face conversation or telephone conversation with people of other organizations. ... 1c. how many times do you send or receive formal, written, but work related communications in the form of reports or data from people in other organizations. ... 1d. how many times do you send or receive informal, written communications in the form of reports, memos or the like from people in other organizations in regard to your work." [Data Analysis] "The 182 scores were organized in three contingency tables ... The data were first analyzed using the Goodman-Kruskal Gamma (Y), a nonparametric measure of association... We felt that interval scale interpretation of these perceptual measures was not appropriate and hence the non-parametric statistic."</t>
         </is>
       </c>
     </row>
@@ -17599,6 +17789,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>Building on the theories of knowledge recombination, we argue that the external acquisition of technologies acts as a boundary spanning mechanism that impacts on the recipient firm’ subsequent technology development. The effect is moderated by two additional mechanisms, namely the retention of star scientists and the experience in upstream strategic alliances. We tested our hypotheses on a sample of 6208 USPTO patented technologies acquired by 350 biotechnology firms over the period 1980–2012. Findings reveal an inverted U-shaped effect of the pioneering nature of the acquired technology on firm’s subsequent developments, in terms of (self) citations of firm’s subsequent patents to the acquired one. Moreover, the main relationship is negatively moderated by the retention of star scientists, while the experience in upstream alliances demonstrates to be a positive moderator.</t>
@@ -17646,6 +17837,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>Successful product development requires managing tensions—coping with fluctuating contingencies to foster innovation and efficiency. To investigate this challenge, we explored the nature, dynamics, and impacts of contrasting project management styles. Our conceptual framework details emergent and planned styles. Following 80 projects over two-year periods, we find that these styles offer disparate but interwoven approaches to monitoring, evaluation, and control activities; use of these activities fluctuates over time; a paradoxical blend of styles enhances performance; and uncertainty moderates project management-performance relationships.</t>
@@ -18075,6 +18267,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>Driven by fierce global competition, flatter organizational structures and the growing complexity of tasks, boundary spanning behavior (BSB) in externally dependent work teams has increasingly been emphasized in both theory and practice. The current study aims to answer the questions of whether, when and how an individual’s BSB impacts his or her task performance within a team. Based on a sample of 272 employees from 57 new product development teams in China, we found that informal leader emergence mediated the relationship between an individual’s BSB and his or her performance within a team. Moreover, group-level power distance positively moderated the association between BSB and informal leader emergence. An overall mediated moderation model of the effect of the interaction between BSB and group power distance (PD) on task performance via informal leadership emergence was also confirmed. In particular, the relationship between BSB and task performance via informal leadership emergence was stronger for teams with less PD than for those with more PD. The implications of the research are discussed.</t>
@@ -18164,6 +18357,12 @@
           <t>BSMA0359</t>
         </is>
       </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine team external learning, particularly focusing on: how leader external learning behavior affects team external learning; how team external learning inﬂuences employee creativity; and whether team internal learning is a moderator between the cross-level relationship of external learning and employee creativity in Chinese R&amp;D teams.</t>
@@ -18187,6 +18386,11 @@
       <c r="K362" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18201,6 +18405,12 @@
           <t>BSMA0360</t>
         </is>
       </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
           <t>Expatriates typically perform boundary-spanning to address challenges related to functional, linguistic, and cultural variations within multinational enterprises (MNEs), which in turn influences their relationships with host-country employees. Integrating social capital and role theory perspectives, this study explores the relational dynamics between expatriates and host-country employees by developing a novel theoretical framework that examines the double-edged effects of expatriates’ boundary-spanning. We propose that expatriates’ boundary-spanning nurtures mutual trust between expatriates and hostcountry employees, further facilitating expatriates’ identification with subsidiaries and host-country employees’ identification with MNEs. On the other hand, we propose that boundary-spanning increases expatriates’ role stressors, causing expatriates’ emotional exhaustion and outgroup categorization by host-country employees. We further categorize expatriates’ boundaryspanning into three types (functional, linguistic, and cultural) and theorize about their varying effects on the cognitive and affective bases of mutual trust and on role stressors. With data from 177 expatriate–host-country coworker dyads in Chinese MNEs, our double-edged framework is generally supported. Our findings suggest that cultural boundary-spanning exhibits the strongest double-edged effect, while functional boundary-spanning shows asymmetric effects, with negative outcomes surpassing positive ones, and linguistic boundary-spanning demonstrates the weakest effect. This study offers realistic and comprehensive insights into expatriates’ boundary-spanning, particularly in expatriate–host-country employee relationships.</t>
@@ -18224,6 +18434,11 @@
       <c r="K363" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18275,6 +18490,12 @@
           <t>BSMA0362</t>
         </is>
       </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>In an increasingly global research landscape, it is important to identify the most prolific researchers in various institutions and their influence on the diffusion of knowledge. Knowledge diffusion within institutions is influenced by not just the status of individual researchers but also the collaborative culture that determines status. There are various methods to measure individual status, but few studies have compared them or explored the possible effects of different cultures on the status measures. In this article, we examine knowledge diffusion within science and technology‐oriented research organizations. Using social network analysis metrics to measure individual status in large‐scale coauthorship networks, we studied an individual's impact on the recombination of knowledge to produce innovation in nanotechnology. Data from the most productive and high‐impact institutions in China (Chinese Academy of Sciences), Russia (Russian Academy of Sciences), and India (Indian Institutes of Technology) were used. We found that boundary‐spanning individuals influenced knowledge diffusion in all countries. However, our results also indicate that cultural and institutional differences may influence knowledge diffusion.</t>
@@ -18298,6 +18519,11 @@
       <c r="K365" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18754,6 +18980,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>Based on the social identity theory, this study investigates whether and how employee perceptions of corporate environmental behavior (CEB) influence the realization of an organization's internal value. Using employees' organizational citizenship behavior (OCB) as a direct agent for corporate internal value, the current study constructs a theoretical model of perceived CEB and OCB, with work meaningfulness and person–organization (P-O) value fit serving as mediator and moderator, respectively. After analyzing 235 questionnaire samples, we discovered that the perceived CEB positively influenced OCB via work meaningfulness and that this positive effect was strengthened by a greater P-O value fit. These findings suggest that in the process of motivating employees to implement OCB, firms should address the significance of internal driving roles of work meaningfulness and boundary-spanning roles of P-O value fit in order to enhance corporate internal value and correct managers' misconceptions about the value of CEB.</t>
@@ -18801,6 +19028,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F378" t="inlineStr"/>
       <c r="G378" t="inlineStr">
         <is>
           <t>A central focus of cross-cultural management research is how individuals and organizations differ across national cultures and how that fundamentally shapes their thoughts and actions and serves as a unit of identification. In this article, we critically reconsider the essential categorical nature of culture, problematizing categorization and questioning national culture as the primary basis of differentiation. We draw on intersectionality, an approach that helps understand how multiple categories are experienced by the individual, and on relationality, an approach that conceptualizes people, organizations, and their actions within dynamic patterns of relations and cultural meanings. Both approaches challenge the primacy, unity, and separateness of any given category, the a priori determination of categories (and associated boundaries) in research, and the nature and stability of boundaries. Based on this we advance notions of boundary work and boundary shifting that help explore how today’s sociocultural groups and categories, and the boundaries that separate them, emerge and change. We conclude that, while the extant crosscultural literature has come far in identifying differences, relationality and intersectionality can enable cross-cultural scholars to engage in research practice that better reflects the complexities of sociocultural life. We contribute to theory by suggesting why and how these two approaches can be used to explore complex cross-cultural management phenomena.</t>
@@ -19016,6 +19244,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>This study extends research on strategic alliances by exploring independent and combined effects of distributive, procedural, and interactional justice in these alliances. An integrated framework links cooperation payoffs with organizational justice as perceived by boundary-spanning alliance executives, through whom justice perceptions become parent actions. Analysis of 127 alliances demonstrates that when goal differences between parties are high, the joint effect on alliance performance of procedural and distributive justice is significantly positive. When interactional justice is high, procedural justice exerts a stronger performance effect. This perspective enriches alliance research, especially regarding procedural formalization, incentive structure, and interparty attachment.</t>
@@ -19063,6 +19292,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19090,7 +19324,7 @@
       </c>
       <c r="P384" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Alliance-level analysis (N=168 alliances) measuring procedural justice, not individual Boundary Spanning Behavior.. Verbatim Evidence: [Reason summary] Verbatim Evidence: "[Introduction] This study deﬁnes procedural justice in the alliance context as the extent to which an alliance’s strategic decision-making process and procedures are impartial and fair as perceived by this alliance’s boundary spanners." "[Methods] We limited the sample to those alliances with two partners since the multiparty case (three or more) complicates the measurement of most constructs used and differs in cooperation logic and behavior from the two-party case." "[Methods] We measured justice based on the convergent score from the matched 168 sample alliances"</t>
         </is>
       </c>
     </row>
@@ -19342,6 +19576,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G391" t="inlineStr">
         <is>
           <t>Chronic excessive turnover among information technology (IT) professionals has been costly to firms for decades with annual turnover rates as high as 24% even among Computerworld’s “100 Best Places to Work in IT.” Prior information systems literature has identified two key factors affecting turnover: boundary-spanning roles and low promotability in one’s current firm. We draw on tournament theory, which is primarily concerned with inducing effort in employees, to decompose promotability into two distinct constructs: the likelihood of promotion and benefit from promotion, and demonstrate that each has a distinct role in affecting turnover rates. Our key result is that a job ladder motivating IT professionals with large, infrequent promotions will lead to higher turnover than a job ladder with smaller, more frequent promotions. We describe the conditions under which rearranging the job ladder creates economic value for the firm. We also offer an explanation for the observation that jobs characterized by boundary-spanning activities have higher turnover, and show that such jobs are more sensitive to the effect of likelihood of promotion on turnover. We test our hypotheses on a detailed data set covering 5,704 IT professionals over a five-year period. We confirm that likelihood of promotion has the predicted effects on turnover of IT professionals. A one standard deviation increase in likelihood of promotion decreases turnover by over 99%, consistent with our prediction. The empirical analysis also confirms the predicted effects of boundary spanning activities.</t>
@@ -19369,7 +19608,7 @@
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>No correlation matrix provided, and BSB is measured as a job type dummy variable (occupational characteristic) rather than individual behavior.. Verbatim Evidence: [Measures] "Our primary data source is the firm’s human resources records, which includes demographic information and date of hire for each employee. We also observe time-varying job titles, base salaries, and scheduled hours for each employee." [Measures] "We also coded the job titles in Table 2 according to the relative level of boundary-spanning activities in each job. Note that the suffixes in Table 3 do not indicate within-level steps on the job ladder, so each category in Table 3 represents a number of distinct jobs."</t>
         </is>
       </c>
     </row>
@@ -19535,6 +19774,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr">
         <is>
           <t>In this study of the business communication that connects an organization with others in its environment, we link boundary spanning with network theory and propose the concept of an extended network of communication. This extended net work is the structure of business communication which flows in work-related ties that organization members maintain both within the organization and across its boundary. We study the relationship between boundary-spanning communication and individual influence in a network with 108 organizational members. We find that boundary spanning correlates with influence, regardless of hierarchical level. There is also a curvilinear relationship between boundary-spanning communication and individual influence. Thus, managers need to balance their communication within and across the organizational boundary.</t>
@@ -19676,6 +19916,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F398" t="inlineStr"/>
       <c r="G398" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -19770,6 +20011,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G400" t="inlineStr">
         <is>
           <t>In response to increased complexity of work tasks, flatter organizational structures, and changing environmental conditions, organizational work teams must increasingly coordinate efforts across their boundaries and actively manage key relationships external to the team itself. Despite evidence of the importance of these processes—referred to as team boundary spanning—for both team and organizational success, significant gaps exist in our understanding of the nature of team boundary spanning, how and when these behaviors are carried out by teams, and the resulting impacts of team boundary spanning beyond that of enhanced team performance. Therefore, this article seeks to advance knowledge in this area by offering a taxonomy of team boundary spanning actions, reviewing the existing stream of team boundary spanning literature across multiple levels of analysis, and integrating this body of work with findings and perspectives from other boundary spanning research areas so as to stimulate fruitful avenues for future research.</t>
@@ -19797,7 +20043,7 @@
       </c>
       <c r="P400" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Review article (Non-primary study). Verbatim Evidence: [Abstract] "Therefore, this article seeks to advance knowledge in this area by offering a taxonomy of team boundary spanning actions, reviewing the existing stream of team boundary spanning literature across multiple levels of analysis, and integrating this body of work with findings and perspectives from other boundary spanning research areas so as to stimulate fruitful avenues for future research."</t>
         </is>
       </c>
     </row>
@@ -20121,6 +20367,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G407" t="inlineStr">
         <is>
           <t>The rapid growth in the use of teams and multiple team membership has led more organizations to structure work around dynamic teams, characterized by short lifespans and fluid membership boundaries. This approach to organizing work makes it difficult for teams to work efficiently or to support the learning and growth of members. Given the importance of productivity and learning, we ask how these processes can be supported in dynamic teams. We do so in a randomized controlled field experiment conducted with 91 teams in a teaching hospital, a context in which physician trainees must learn while providing patient care in dynamic teams of care providers. We randomly assigned physician teams, or “core” teams, to launch their work with an intervention focused either on internal coordination among the core team members or on external coordination with a changing cast of external contributors such as nurses and specialists. We measured resulting levels of internal and external coordination over teams’ week-long lifespans and observed that external coordination was associated with improved team efficiency, whereas internal coordination was associated with improved individual learning. Post hoc exploratory analysis suggested that individual learning was highest when teams achieved high levels of both internal and external coordination, and it was positively correlated with improvement in the team’s patients’ average length of hospital stay. We discuss the implications of the demonstrated causal effects of team launches, along with our exploratory findings, for the management of dynamic teams and the opportunities to mitigate potential trade-offs between learning and productivity.</t>
@@ -20148,7 +20399,7 @@
       </c>
       <c r="P407" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level analysis (N = 91 teams) rather than individual-level.. Verbatim Evidence: [Sample and Design] "Because of the reconstitution of each core team each week, we treated the core teams from week to week as separate entities such that the unit of analysis was a core team in a given week, along with the periphery members associated with each patient case." [Results] "Table 2. Descriptive Statistics and Correlations" "Notes. Values in bold are significant at p &lt; 0.05. N = 91."</t>
         </is>
       </c>
     </row>
@@ -20361,6 +20612,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G412" t="inlineStr">
         <is>
           <t>This study is based on a formative evaluation of a case management service for high-intensity service users in Northern England. The evaluation had three main purposes: (i) to assess the quality of the organisational infrastructure; (ii) to obtain a better understanding of the key inﬂuences that played a role in shaping the development of the service; and (iii) to identify potential changes in practice that may help to improve the quality of service provision. The evaluation was informed by Gittell’s relational co-ordination theory, which focuses upon cross-boundary working practices that facilitate task integration. The Assessment of Chronic Illness Care Survey was used to assess the organisational infrastructure and qualitative interviews with front line staff were conducted to explore the key inﬂuences that shaped the development of the service. A high level of strategic commitment and political support for integrated working was identiﬁed. However, the quality of care coordination was variable. The most prominent operational factor that appeared to inﬂuence the scope and quality of care co-ordination was the pattern of interaction between the case managers and their co-workers. The co-ordination of patient care was much more effective in integrated co-ordination networks. Key features included clearly deﬁned, task focussed, relational workspaces with interactive forums where case managers could engage with co-workers in discussions about the management of interdependent care activities. In dispersed co-ordination networks with fewer relational workspaces, the case managers struggled to work as effectively. The evaluation concluded that the creation of ﬂexible and efﬁcient task focused relational workspaces that are systemically managed and adequately resourced could help to improve the quality of care co-ordination, particularly in dispersed networks.</t>
@@ -20388,7 +20644,7 @@
       </c>
       <c r="P412" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Qualitative evaluation study lacking a formal correlation matrix or extractable quantitative effect sizes (r).. Verbatim Evidence: [Abstract] "This study is based on a formative evaluation of a case management service for high-intensity service users in Northern England." [Abstract] "The Assessment of Chronic Illness Care Survey was used to assess the organisational infrastructure and qualitative interviews with front line staff were conducted to explore the key inﬂuences that shaped the development of the service." [Methods] "The ACIC questionnaires were posted to 23 of the team members and managerial staff who had been employed or involved in the development of the case management service. Ten questionnaires were completed and returned (response rate 44%)." [Methods] "A total of 19 individual and four group interviews were conducted." [Methods] "The interview data were analysed using a combination of elements from framework analysis (Ritchie &amp; Spencer 1994) and the realistic evaluation approach developed by Pawson &amp; Tilley (1997). The interviews were independently analysed by two of the authors (PM and DE) who then worked together to code the transcripts and construct a thematic matrix."</t>
         </is>
       </c>
     </row>
@@ -20695,6 +20951,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their boundaries in ways that complement their preferences.</t>
@@ -20833,12 +21090,12 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>1 = Include</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
@@ -20868,7 +21125,7 @@
       </c>
       <c r="P422" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Study measures individual-level boundary spanning behavior among purchasing agents and provides a zero-order correlation matrix.. Verbatim Evidence: [RESEARCH METHODS] "The sample consisted of 133 (41% usable response rate) purchasing agents from electronics firms in the southwest United States." [INTRODUCTION] "Boundary spanning is conceptualized using Jemison’s (1979) list of 25 Boundary-Spanning Activities (BSA)." [Table II] "N = 133."</t>
         </is>
       </c>
     </row>
@@ -21274,6 +21531,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -21301,7 +21563,7 @@
       </c>
       <c r="P431" t="inlineStr">
         <is>
-          <t xml:space="preserve">The study analyzes data at the firm level, using CEOs as key informants to evaluate firm-level functional capabilities (logistics, production, marketing) and business performance, rather than measuring individual-level interpersonal boundary spanning behavior.. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 3] Firm-level analysis of organizational logistics and functional capabilities rather than individual-level boundary spanning behavior.. Verbatim Evidence: [Methodology] "The present research is concerned with interfunctional process relationships, specific boundary-spanning interface relationships, and overall business performance relationships." [Subjects and sample] "The subjects consisted of the CEOs from 65 furniture manufacturing firms." [Business performance indicator variables] "To measure overall business performance, data were collected on subject firms for five business performance indicators. The five financial performance ratios consisted of return on assets (ROA), return on investment (ROI), return on sales (ROS), and the two growth ratios of ROI growth and ROS growth."</t>
         </is>
       </c>
     </row>
@@ -21373,6 +21635,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
           <t>The management of quality and development of effective cross-functional cooperation have assumed a new strate gic importance over the past decade. However, many com panies have reported that quality strategies have failed to deliver anticipated performance benefits and that ineffec tive interfunctional relationships may be to blame. This study explores marketing-quality interfunctional relation ships as a potential source of quality strategy implemen tation failure at the strategic business unit (SBU) level. This study focuses on interdepartmental connectedness, communication and conflict between marketing and qual ity, and the antecedents and consequences of these dimen sions of interfunctional interaction. Using data from a pooled response mail survey, the results suggest that mar keting-quality interactions are associated with senior management quality leadership, strategic quality plan ning process, and control system characteristics. Inter-functional interactions between marketing and quality are found to be only weakly related to relative quality, market performance, and financial performance outcomes.</t>
@@ -21514,6 +21777,16 @@
           <t>BSMA0433</t>
         </is>
       </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G436" t="inlineStr">
         <is>
           <t>Although social interactions and exchanges between partners are emphasized as imperative for alliance success, comprehensive examination of how social exchanges facilitate learning and knowledge transfer in strategic alliances is lacking. Drawing on social exchange theory, we examined the effects of social exchange processes between alliance partners on the extent of learning and knowledge transfer in a strategic alliance. An empirical examination of data collected from alliance managers of 144 strategic alliances revealed that social exchanges such as reciprocal commitment, trust, and mutual inﬂuence between partners are positively related to learning and knowledge transfer in strategic alliances.</t>
@@ -21537,6 +21810,11 @@
       <c r="K436" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21556,6 +21834,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G437" t="inlineStr">
         <is>
           <t>Efforts to understand how an organization monitors its environment often focus on boundary spanning individuals or units. The concept of boundary spanning was one introduced by Thompson in 1967 in a book that has since become the classic statement of the open systems model of organizations. This dissertation uses Thompson's model of boundary spanning units to generate hypotheses which are then tested in a sample of personnel/human resource departments. A theory driven argument is presented which suggests that the P/HR function in an organization meets Thompson's criteria for a boundary spanning unit. An historical review of the roots of personnel administration suggests that its emergence as a field fits Thompson's conceptualization of the development of boundary spanning units. This dissertation suggests that from its origin through this most recent period of transition, the development of the personnel function (now generally referred to as human resource management) has been due to a recognition by organizations that an increasing complexity and concomitant uncertainty in the human resource arena caused by such factors as labor unions, the expansion of due process in organizations, and intervention by government agencies, needed to be addressed.</t>
@@ -21583,7 +21866,7 @@
       </c>
       <c r="P437" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>The unit of analysis is the organizational department/firm (N=119 worksites), not individual employee boundary spanning behavior.. Verbatim Evidence: [Summary] "This dissertation uses Thompson's model of boundary spanning units to generate hypotheses which are then tested in a sample of personnel/human resource departments." [Summary] "The dissertation tests hypotheses generated from Thompson's theory of boundary spanning units using a sample of personnel/human resource departments (N = 124) in the eighteen county Atlanta Standard Metropolitan Statistical Area. The data analyzed are from face to face interviews and mailback questionnaires completed by the highest level personnel/human resource person at each site." [Chapter II] "The important difference between a focus on boundary spanning units and jobs is a level of analysis issue and has bearing on the choice of dependent variables. For example, research on boundary spanning jobs (or roles), explicitly involves an individual level analysis and would be appropriately focused on outcomes the individual faces, such as role conflict or ambiguity. This set of questions has been partially addressed by research on boundary spanning activity. On the other hand, research on boundary spanning units requires an organizational level of analysis, and would more appropriately examine the relationship between boundary spanning and perceptions of environmental uncertainty held by both top management and boundary spanners, and ultimately organizational performance in light of its understanding of the environment." [Method] "The data for this analysis were collected from a sample of Atlanta area worksites with at least 250 employees."</t>
         </is>
       </c>
     </row>
@@ -21870,6 +22153,12 @@
           <t>BSMA0441</t>
         </is>
       </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr"/>
       <c r="G444" t="inlineStr">
         <is>
           <t>Horizontal arrangements are increasingly deployed in organizational networks, yet research has rarely examined the effectiveness of these alliances. The coalition of disparate corporate cultures yields appreciable levels of role stress for people in boundary-spanning positions. Dedicated assets and communication modality are factors that influence the level of role ambiguity and conflict. The authors implicate these facets of role stress as antecedents to four forms of effectiveness drawn from the competing values framework. The authors present alternative perspectives that examine the relationship between stress and performance. The received view frames role stressors as linear, negative antecedents to organizational outcomes. The authors contrast this perspective with theories that espouse triphasic, parabolic, and interactive influences of stressors on organizational outcomes. Data gathered with 218 managers of dual-branded retail oil outlets indicate that the relevance of these alternative perspectives is mitigated by the form of effectiveness pursued by the organization. The results support a linear relationship between role conflict and bargaining efforts, yet they also offer evidence of nonlinear influences of role ambiguity on contributions to sales, customer satisfaction, and competence. The study concludes with a discussion of relevance of the findings to the management of horizontal alliances and to interorganizational theory.</t>
@@ -21893,6 +22182,11 @@
       <c r="K444" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21978,6 +22272,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G446" t="inlineStr">
         <is>
           <t>Purpose – This study recognizes service as the majority contributor to global and US gross domestic product and the importance of innovation speed to service innovation. Generating innovative products and services at a faster rate generates advantages for business-to-business (B2B) service organizations in keeping up with and moving ahead of rivals. This study aims to introduce the concept of capacity for social exchange (CSE) in buyer–supplier relationships, which reflects the degree to which individuals possess competencies that enable the exchange of information, and this study also explores how CSE affects knowledge sharing and innovation speed within a supply chain organization.</t>
@@ -22005,7 +22304,7 @@
       </c>
       <c r="P446" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Firm-level analysis via key informant (survey referent is 'We' and 'Our employees'). Verbatim Evidence: [Abstract] "The data was collected from 264 B2B service sector executives." [Measures] "The knowledge channel items were adapted from Rosenzweig and Roth (2007) and captured the boundary-spanning activities used in the supply chain to create, recombine and transfer knowledge." [Appendix] "Please respond to Items 14–16 related to knowledge management practices of your business unit." [Appendix] "14. Our employees regularly visit supply chain partners to enable two-way sharing of expertise." [Appendix] "15. We are able to capture best practices via an information source that spans company boundaries."</t>
         </is>
       </c>
     </row>
@@ -22104,6 +22403,16 @@
           <t>BSMA0446</t>
         </is>
       </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G449" t="inlineStr">
         <is>
           <t>Background The health-care environment requires hospital units to coordinate efforts autonomously across their boundaries and to manage relationships with other professionals, units and departments. Boundary spanning has become increasingly important for ﬁrst-line nurse managers as unit gatekeepers; however, the available measures are limited. Method The 30-item instrument was developed from a literature review. Survey participants were 4918 nurses at 231 hospital units. Statistical analyses of construct validity and internal consistency were performed. Furthermore, the correlation between nurses’ scores on the Nurse Managers Boundary Spanning Scale and nurses’ evaluations of their managers were examined. Results Three factors and 26 items were derived from factor analyses: connecting and mediating, informing and feedback utilisation, and resource acquisition. Cronbach’s subscales’ alpha coefﬁcients were above 0.9. Correlation analysis indicated that the Nurse Managers Boundary Spanning Scale score correlated with nurses’ positive perceptions of their managers. Conclusion This study demonstrates tentative support for the validity and reliability of the Nurse Managers Boundary Spanning Scale. Although further study is needed, the Nurse Managers Boundary Spanning Scale shows possibilities as a new measurement of nursing leadership. Implications This study underscores measures to build on nurse managers’ roles by building on the limited research available.</t>
@@ -22127,6 +22436,11 @@
       <c r="K449" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P449" t="inlineStr">
+        <is>
+          <t>The study develops and tests a measure of nurse managers' boundary spanning behavior rated by subordinate nurses (Leader BSB). It provides individual-level zero-order correlations (N=166) with nurses' evaluation of their manager.. Verbatim Evidence: [Methodology] "In addition, to examine whether the NMBS is a useful indicator of nursing management, we recruited 166 nurses at an acute-care hospital as another sample. They were asked to respond to the NMBS and an additional item evaluating their nurse manager as a unit leader: ‘The nurse manager is a good leader for nurses in this unit’." [Results] "Correlation coefficients between the NMBS subscales and nurses’ evaluations for nurse managers are presented in Table 3. All three subscales demonstrated significant positive correlation coefficients."</t>
         </is>
       </c>
     </row>
@@ -22176,6 +22490,16 @@
       <c r="B451" t="inlineStr">
         <is>
           <t>BSMA0448</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -22237,6 +22561,11 @@
           <t>2013</t>
         </is>
       </c>
+      <c r="P451" t="inlineStr">
+        <is>
+          <t>Measures Work-Nonwork boundary management rather than inter/intra-organizational boundary spanning.. Verbatim Evidence: [Title] "Testing the role of boundary management tactics within the work-nonwork interface" [Abstract] "In an effort to balance competing work and personal demands, recent research suggests that individuals put forth effort to control the implicit or explicit boundaries around their work and nonwork domains by either segmenting domains from one another or integrating them."</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -22693,6 +23022,16 @@
           <t>BSMA0461</t>
         </is>
       </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G464" t="inlineStr">
         <is>
           <t>We argue in this paper that when the knowledge base of an industry is both complex and expanding and the sources of expertise are widely dispersed, the locus of innovation will be found in networks of learning, rather than in individual firms. The large-scale reliance on interorganizational collaborations in the biotechnology industry reflects a fundamental and pervasive concern with access to knowledge. We develop a network approach to organizational learning and derive firm-level, longitudinal hypotheses that link research and development alliances, experience with managing interfirm relationships, network position, rates of growth, and portfolios of collaborative activities. We test these hypotheses on a sample of dedicated biotechnology firms in the years 1990-1994. Results from pooled, within-firm, time series analyses support a learning view and have broad implications for future theoretical and empirical research on organizational networks and strategic alliances.</t>
@@ -22716,6 +23055,11 @@
       <c r="K464" t="inlineStr">
         <is>
           <t>1996</t>
+        </is>
+      </c>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>The study uses an archival database (Bioscan) to analyze firm-level interorganizational alliances among biotechnology companies, lacking both individual-level analysis and a human employee sample.. Verbatim Evidence: [Code 2 &amp; Code 3] Firm-level archival analysis of strategic alliances without a human employee sample. Verbatim Evidence: "[Method] We built a relational database that contains separate files for (1) DBFs in human therapeutics and diagnostics, (2) the formal contractual, interorganizational agreements involving DBFs, and (3) the partners to these agreements." "[Method] We began assembling the database in 1990, using Bioscan, an independent industry directory published six times a year that lists a great range of organizations (domestic and foreign, commercial, nonprofit, or government-owned, biotech, and diversified health care corporations)." "[Method] Our focus on research-driven DBFs in human therapeutics resulted in a sample of approximately 225 independently owned companies."</t>
         </is>
       </c>
     </row>
@@ -23063,6 +23407,16 @@
           <t>BSMA0471</t>
         </is>
       </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G474" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this research is to explore how ﬁrm market orientation, as a culture, affects the service climate that develops in the ﬁrm. Design/methodology/approach – Empirical testing is performed at the managerial level and boundary-spanning employee level as part of this multilevel study. The sample includes participants from a US-based ﬁrm operating in the hospitality industry.</t>
@@ -23086,6 +23440,11 @@
       <c r="K474" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P474" t="inlineStr">
+        <is>
+          <t>The paper measures boundary-spanner flexibility using the Spiro &amp; Weitz (1990) ADAPTS scale (adaptive selling), which is explicitly excluded under Code 1 as it represents a sales tactic rather than purposive boundary spanning behavior. The other constructs (market orientation, service climate, boundary-spanner control) are also not BSB.. Verbatim Evidence: [Purpose and gap] "This research investigates how one of these boundary-spanning employee attributes, flexible disposition, facilitates the service climate. Research widely recognizes that personal flexibility reflects the degree to which a person will engage in adaptive selling techniques (Spiro and Weitz, 1990)." [Measures] "Boundary-spanning employee flexibility was assessed using four items based on Spiro and Weitz’s (1990) ADAPTS scale."</t>
         </is>
       </c>
     </row>
@@ -23100,6 +23459,16 @@
           <t>BSMA0472</t>
         </is>
       </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G475" t="inlineStr">
         <is>
           <t>Software professionals perform boundary-spanning activities, and thus need strong interpersonal, technical, and organizational knowledge to be professionally competent. They have to perform in a demanding work environment characterized by strict deadlines, differing time zones, interdependency in teams, increased interaction with clients, and extended work hours. These characteristics lead to occupational stress and work exhaustion. Yet, the impact of stress is felt in different ways by different people, even if they perform the same functions. These differences in the perception of stress can be caused by varying confidence in their technical capabilities. People possess varying technical capabilities, based on their acquisition of technical skills, comfort level in using the technology, and intrinsic motivation. These attributes represent the human-computer interaction (HCI) personality of software professionals. This article examines whether these HCI factors moderate the relationship between occupational stress and work exhaustion. Data were collected from software professionals located in Chennai and Bangalore in India. The data revealed that HCI factors had a main effect but no significant moderating effects on work exhaustion. The control over the technology variable emerged as the key variable among the HCI factors that affected software professionals' ability to cope with stress and work exhaustion.</t>
@@ -23123,6 +23492,11 @@
       <c r="K475" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t>No boundary spanning behavior construct measured. BSB is only mentioned as a contextual job characteristic.. Verbatim Evidence: [Abstract] "Software professionals perform boundary-spanning activities, and thus need strong interpersonal, technical, and organizational knowledge to be professionally competent." [Introduction] "The focus of this study, therefore, is to inquire whether HCI factors play a moderating role in the relationship between occupational stress and work exhaustion." [Results] "Table 3: Relationship Between Occupational Stress, Work Exhaustion, and Human-Computer Interaction Variables"</t>
         </is>
       </c>
     </row>
@@ -23137,6 +23511,16 @@
           <t>BSMA0473</t>
         </is>
       </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G476" t="inlineStr">
         <is>
           <t>Contrary to much boundary spanning research, we examined the negative consequences of boundary spanning contact in multi-organizational contexts. Results from a sample of 833 Dutch peacekeepers show that employees’ boundary spanning contact with members of other organizations was associated with reports of negative relationships with external parties (e.g., work-speciﬁc problems, culture-speciﬁc problems). These negative relationships also had a spillover effect such that they mediated the effect of boundary spanning contact on boundary spanners’ negative attitudes toward their own jobs and organization (e.g., job attractiveness and conﬁdence in the organization). Copyright # 2010 John Wiley &amp; Sons, Ltd.</t>
@@ -23160,6 +23544,11 @@
       <c r="K476" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P476" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct merely measures communication frequency rather than purposive boundary-spanning behaviors.. Verbatim Evidence: [Sample] "The participants were a sample of Dutch military peacekeepers stationed in one region who had participated in peacekeeping missions between 1995 and 1999 (N = 833)." [Measures] "Since we were interested in all instances of employees’ inter-organizational contact, we operationalized this variable as frequency of boundary-spanning contact between peacekeepers and members of other organizations such as NGOs, inter-governmental organizations, and local authorities." [Measures] "Participants responded to the question, 'What parties did you have contact with? Please indicate the frequency of these contacts for your job.'" [Measures] "Frequency of contact was measured on a five-point Likert scale (1 = hardly ever; 5 = daily) for each item, and the items were averaged to create the scale for contact (Cronbach’s alpha = 0.73)."</t>
         </is>
       </c>
     </row>
@@ -23174,6 +23563,16 @@
           <t>BSMA0474</t>
         </is>
       </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G477" t="inlineStr">
         <is>
           <t>Boundary-spanning activities were studied in 15 organizations engaged in basic and applied research. Included in the study were 281 scientists and engineers. Contrary to prior theory and research, this study found bound-ary-spanning activities to be unrelated to job satisfaction. It was strongly related to perceptions of research and development team collaboration, job motivation, task uncertainty, locus of control, team cohesiveness, and individualproductivity. The research reported here makes a strong case for including group processes and characteristics in future studies involving boundary-spanning activities. The results also give increased impetus to re-search which examines the relationships between boundary-spanning activi-ties and individual productivity.</t>
@@ -23197,6 +23596,11 @@
       <c r="K477" t="inlineStr">
         <is>
           <t>1979</t>
+        </is>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>Study measures individual-level boundary-spanning activities of R&amp;D scientists/engineers and provides zero-order Pearson correlations.. Verbatim Evidence: [Sample] "The study was conducted in 15 R&amp;D organizations located in the Rocky Mountain west. R&amp;D activities in these organizations ranged from environmental research to defense contracting and space exploration. The subjects were 281 scientists and engineers who were organized into 45 project groups ranging in size from 2 to 19 members." [Measures] "Boundary-Spanning Activities (BSA). A four-item BSA scale based on the work of Keller et al. (1976) was used to assess boundary spanning in this study." [Results] "The correlational analysis performed on the sample (N = 281) is reported in Table I."</t>
         </is>
       </c>
     </row>
@@ -23211,6 +23615,16 @@
           <t>BSMA0475</t>
         </is>
       </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G478" t="inlineStr">
         <is>
           <t>A review of previous studies on the relationship between boundary spanning activity and environment indicates that the full effects of environment have not been investigated due to the restricted representation of environmental effects. In addition, we argue that the boundary spanning-environment relationship may be moderated by function, hierarchical level, perceived influence, size, and industry. Accordingly, an enlarged model of the boundary spanning-environment relationship is tested in both the high-technology electronics industry and the wood products industry. Results indicate that boundary spanning activity is related to environment, but this relationship appears to vary along dimensions of environment as well as by industry. In addition, size, perceived influence, and function are found to moderate the boundary spanning-environment relationship. Implications for further studies include a reconceptualization of the boundary spanning-environment relationship based on the findings.</t>
@@ -23234,6 +23648,11 @@
       <c r="K478" t="inlineStr">
         <is>
           <t>1985</t>
+        </is>
+      </c>
+      <c r="P478" t="inlineStr">
+        <is>
+          <t>Study measures individual-level boundary spanning behavior in a real employee sample and provides zero-order correlations.. Verbatim Evidence: [Sample] "Questionnaires were sent to the chief executive officer or his designated representative for distribution to employees believed to have primary responsibility for dealing with the external environment. Three hundred seventy-nine individuals from 36 companies participated in the study, for a 57% response rate (287 individuals from 24 high-technology electronics companies, for a 54% response rate; 92 individuals from 12 wood products firms, for a 68% response rate)." [Measures] "Boundary spanning was measured using Miles’ (1980) set of eight boundary spanning activities, slightly modified by splitting his “transacting” activity into two parts: acquiring and distributing." [Matrix] "Table 2 Zero-Order Correlations Among Study Variables"</t>
         </is>
       </c>
     </row>
@@ -23322,6 +23741,16 @@
           <t>BSMA0478</t>
         </is>
       </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G481" t="inlineStr">
         <is>
           <t>We examined the relationship between group boundary spanners' work group identification and effective (i. E., harmonious and productive) intergroup relations in 53 work groups in five health care organizations. The data suggest this relationship was moderated by boundary spanners' levels of organizational identification, thus supporting a dual identity model. Limited support was found for the moderating effect of intergroup contact. Finally, if boundary spanners displayed frequent intergroup contact and identified highly with their organization, group identification was most strongly related to effective intergroup relations.</t>
@@ -23345,6 +23774,11 @@
       <c r="K481" t="inlineStr">
         <is>
           <t>2006</t>
+        </is>
+      </c>
+      <c r="P481" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Measures mere contact frequency rather than purposive BSB, and conducts analysis at the group/team level (N=53 groups).. Verbatim Evidence: [Measure of Intergroup Contact] "The amount of such contact was determined from responses to a question adapted from van de Ven and Ferry (1980): 'How frequently do you interact on work-related matters with members of [out-group's name]?' (1, 'not at all'; 7, 'daily')." [Mere Exposure] "First and foremost, we used a single-item measure of intergroup contact, which raises concerns about uncertain reliability. Testing the predictions derived from the 'mere exposure' perspective on intergroup contact theory may not require a contact measure that embraces multiple facets of contact, and researchers have frequently used single-item measures to test predictions derived from intergroup contact theory (see Pettigrew &amp; Tropp, 2006)." [Level of Analysis] "We examined the relationship between group boundary spanners' work group identification and effective (i.e., harmonious and productive) intergroup relations in 53 work groups in five health care organizations." [Aggregation] "Aggregation of data at the group level requires both a theoretical basis and empirical justification (Kozlowski &amp; Klein, 2000). Even though intergroup conflict may be the result of interaction between group representatives, these individuals represent their groups' interests, and not their own, on interface issues that exist at the group rather than the individual level (Brett &amp; Rognes, 1986). Therefore, both intergroup conflict scales were aggregated by groups."</t>
         </is>
       </c>
     </row>
@@ -23507,6 +23941,16 @@
           <t>BSMA0483</t>
         </is>
       </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G486" t="inlineStr">
         <is>
           <t>As firms experience relentless pressure to innovate and improve, many are responding by creating organizational structures that promote cross‐functional and cross‐boundary communication, coordination, and collaboration. Because most firms studied expect to use teams to support future procurement and sourcing decision making, it is important to understand how to best manage the cross‐functional sourcing team process. Unfortunately, researchers who study teams rarely reach the same conclusions about the factors affecting team success. There is one variable, however, that most researchers agree consistently affects team success — the effectiveness of the formal team leader.
@@ -23533,6 +23977,11 @@
           <t>1996</t>
         </is>
       </c>
+      <c r="P486" t="inlineStr">
+        <is>
+          <t>No correlation matrix and measures LBDQ instead of BSB. Verbatim Evidence: [Introduction] "The purpose of this article is to examine the critical role that team leaders play and the challenges they face in a cross-functional sourcing team environment. The final section details three assessment scales used to help identify a sourcing team leader’s behavioral style and ability to satisfy critical leadership requirements." [Assessing Cross-Functional Sourcing Team Leadership] "Two of the scales, those presented in Figures 2 and 3, are factor-analyzed versions of the Leader-ship Behavior Description Questionnaire (LBDQ) originally developed at Ohio State University almost 40 years ago." [Assessing Cross-Functional Sourcing Team Leadership] "The statistical revision and development of these scales used responses from over 620 team members and team leaders working at 18 firms based in the United States."</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -23619,6 +24068,16 @@
           <t>BSMA0486</t>
         </is>
       </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G489" t="inlineStr">
         <is>
           <t>Employee contextual performance is a crucial determinant of organizational effectiveness, growth, and performance. Therefore, this research focuses on employees’ contextual performance issues seen from the perspective of boundary-spanning leaders (BSL), creativity, and proactive work behavior (PWB). The aim is to reveal the effect of BSL, creativity, and PWB on employees’ contextual performance and find new models of the role of creativity and PWB in mediating the effect of BSL on employees’ contextual performance. The research involved 420 employees from companies in the finance, trade, services, and investment industry sectors in Indonesia. A Likert scale questionnaire designed in Google Forms was used to conduct a survey via the WhatsApp application. Data analysis using structural equation modelling (SEM) shows that BSL, creativity, and PWB significantly direct affect employees' contextual performance; BSL and creativity significantly direct affect employees' PWB; and BSL significantly indirectly affect employees' contextual performance mediated by creativity and PWB. Accordingly, this study proves a new empirical model regarding the effect of BSL on employee contextual performance mediated by creativity and PWB. Based on these findings, this study suggests that researchers and practitioners utilize the empirical model from this study as a strategy to improve employee contextual performance through BSL with a mediation mechanism of creativity and PWB in the future.</t>
@@ -23642,6 +24101,11 @@
       <c r="K489" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P489" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning leadership (BSL) as rated by individual employees. A correlation matrix reporting zero-order correlations among the dimensions of BSL and other variables is provided.. Verbatim Evidence: [Abstract] "The research involved 420 employees from companies in the finance, trade, services, and investment industry sectors in Indonesia." [Sample and Sampling Technique] "This research sample is 420 participants. They are companies’ employees of finance, trade, services, and investment industry across six provinces in Java Island as Indonesian industry and business centers..." [Instrument] "For BSL, indicators were collaboration across functions (CAF), empowering employees at all levels (EEAL), and developing cross-organizational learning capabilities (DCLC) (Yip et al., 2016)."</t>
         </is>
       </c>
     </row>
@@ -23693,6 +24157,16 @@
           <t>BSMA0488</t>
         </is>
       </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G491" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the impact of product management as a set of organizational capabilities. It aims to investigate product management as a set of boundary spanning capabilities, by empirically relating these to ﬁrm performance.</t>
@@ -23716,6 +24190,11 @@
       <c r="K491" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P491" t="inlineStr">
+        <is>
+          <t>Firm-level unit of analysis with key informant. Verbatim Evidence: [Abstract] "A model is proposed and tested using a heterogeneous sample of 316 Canadian small and medium-sized enterprises, where PM mediates the relationship between MOand ﬁrm performance." [Sample and data collection] "The method of data collection was a self-reported on-line survey answered by senior managers of SMEs in May 2009." [Appendix] "PM01 We have strong systems for deciding which products and/or service opportunities to pursue or which to phase-out." [Appendix] "PM07 We foster communication about our products and/or services within our ﬁrm in order to generate product improvement ideas."</t>
         </is>
       </c>
     </row>
@@ -23730,6 +24209,16 @@
           <t>BSMA0489</t>
         </is>
       </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G492" t="inlineStr">
         <is>
           <t>No Abstract</t>
@@ -23756,6 +24245,11 @@
           <t>1984</t>
         </is>
       </c>
+      <c r="P492" t="inlineStr">
+        <is>
+          <t>Multiple flaws: [Code 1 &amp; Code 3] The study analyzes structural interorganizational linkages (shared board members) rather than individual interpersonal boundary spanning behavior. The unit of analysis is project funding requests (N=398), not individual employees.. Verbatim Evidence: [Level of Analysis] "The unit of analysis for this study was a request for project funding approval submitted by a health industry activity. There were 398 projects reviewed and acted upon by the three Indiana HSAs during 1980, the sample year." [Construct Validity] "Boundary spanning for purposes of this dissertation is the exchange or sharing of members between two organizations." [Construct Validity] "The three dimensions of the interorganizational linking mechanism of boundary spanning which were analyzed in this study were directionality, directness and intensity."</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -23768,6 +24262,16 @@
           <t>BSMA0490</t>
         </is>
       </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G493" t="inlineStr">
         <is>
           <t>In this paper, we present an empirical study of 1,156 open source virtual reality (VR) projects from Unity List. Our study shows that the number of open source VR software projects are steadily growing, and some large projects attracting many developers are emerging. The most popular topic of VR software is still games. We also found that VR developers often face misscommit of automatically generated ﬁles.</t>
@@ -23791,6 +24295,11 @@
       <c r="K493" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P493" t="inlineStr">
+        <is>
+          <t>Multiple flaws [Code 1, Code 2, &amp; Code 3]. Verbatim Evidence: [Abstract] "In this paper, we present an empirical study of 1,156 open source virtual reality (VR) projects from Unity List." [Introduction] "we present an empirical study on all 1,156 open source virtual-reality software projects collected from Unity List 3 on Apr. 1st, 2017, an on-line VR software repository holding open source software projects based on Unity 3D framework." [The Study] "RQ1: How fast does the number of open-source VR software projects grows?"</t>
         </is>
       </c>
     </row>
@@ -23946,6 +24455,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -23973,7 +24487,7 @@
       </c>
       <c r="P497" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 4] Conceptual paper lacking empirical data and effect sizes.. Verbatim Evidence: [Abstract] "This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team." [7. FUTURE RESEARCH] "Quantitative and case research is needed to determine if the time, effort, and cost of caring for and investing in the individuals on the project team generate a positive value for the business."</t>
         </is>
       </c>
     </row>
@@ -24109,6 +24623,16 @@
           <t>BSMA0498</t>
         </is>
       </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G501" t="inlineStr">
         <is>
           <t>A model of cross-functional project groups was developed and hypotheses were tested in a study of 93 research and new product development groups from four companies. The results showed that functional diversity had indirect effects through external communication on one-year-later measures. Technical quality and schedule and budget performance improved, but group cohesiveness diminished. Functional diversity also had an indirect effect through job stress on group cohesiveness, which was again reduced. Implications for the development of conceptual models of cross-functional groups and their effective management are discussed.</t>
@@ -24132,6 +24656,11 @@
       <c r="K501" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P501" t="inlineStr">
+        <is>
+          <t>Team Level Aggregation (N = 93 groups). Verbatim Evidence: [Abstract] "a study of 93 research and new product development groups from four companies;"</t>
         </is>
       </c>
     </row>
@@ -24146,6 +24675,16 @@
           <t>BSMA0499</t>
         </is>
       </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G502" t="inlineStr">
         <is>
           <t>Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors. Contrary to prior theory and research, this study found boundary-spanning activity unrelated to role conflict or ambiguity and positively related to job satisfac-tion for the total sample. Boundary-spanning activity was also positively related to a number of job characteristics for the total sample. Marked dif-ferences in boundary-spanning activity and its relationships with other variables, however, were found across occupational levels. While managers and engineers generally had boundary-spanning activity related to high levels of job satisfaction and job characteristics, first-level supervisors had boundary-spanning activity related to higher role conflict and lower job satisfaction with opportunities for promotion.</t>
@@ -24169,6 +24708,11 @@
       <c r="K502" t="inlineStr">
         <is>
           <t>1976</t>
+        </is>
+      </c>
+      <c r="P502" t="inlineStr">
+        <is>
+          <t>Valid individual-level BSB study with a real employee sample and zero-order correlations.. Verbatim Evidence: [Abstract] "Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors." [Sample] "The subjects were 192 managerial, engineering, and supervisory personnel (64% response rate) located at the company headquarters and main manufacturing plant." [Appendix] "3. During the last month, indicate with a check the frequency with which you have sought information/advice from members of other organizations outside (name of company)." [Results] "Table I. Zero-Order Correlations between Boundary-Spanning Activity and Role, Satisfaction, and Job Characteristic Variables (Total Sample, N=192)"</t>
         </is>
       </c>
     </row>
@@ -24444,6 +24988,16 @@
           <t>BSMA0507</t>
         </is>
       </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G510" t="inlineStr">
         <is>
           <t>Manufacturing ﬁrms are increasingly seeking cost and other competitive advantages by tightly coupling and managing their relationship with suppliers. Among other mechanisms, interorganizational systems (IOS) that facilitate boundary-spanning activities of a ﬁrm enable them to effectively manage different types of buyer–supplier relationships. This study integrates literature from the operations and information systems ﬁelds to create a joint perspective in understanding the linkages between the nature of the IOS, buyer–supplier relationships, and manufacturing performance at the dyadic level. External integration, breadth, and initiation are used to capture IOS functionality, and their effect on process efﬁciency and sourcing leverage is examined. The study also explores the differences in how manufacturing ﬁrms use IOS when operating under varying levels of competitive intensity and product standardization. In order to test the research models and related hypothesis, empirical data on buyer–supplier dyads is collected from manufacturing ﬁrms. The results show that only higher levels of external integration that go beyond simple procurement systems, as well as who initiates the IOS, allow manufacturing ﬁrms to enhance process efﬁciency. In contrast, IOS breadth and IOS initiation enable manufacturing ﬁrms to enhance sourcing leverage over their suppliers. In addition, ﬁrms making standardized products in highly competitive environments tend to achieve higher process efﬁciencies and have higher levels of external integration. The study shows how speciﬁc IOS decisions allow manufacturing ﬁrms to better manage their dependence on the supplier for resources and thereby select system functionalities that are consistent with their own operating environments and the desired supply chain design.</t>
@@ -24467,6 +25021,11 @@
       <c r="K510" t="inlineStr">
         <is>
           <t>2005</t>
+        </is>
+      </c>
+      <c r="P510" t="inlineStr">
+        <is>
+          <t>The study measures firm-level interorganizational system (IOS) electronic linkages rather than individual-level interpersonal boundary spanning behavior (Code 1), and data is analyzed at the firm level with N=38 companies (Code 3).. Verbatim Evidence: [Introduction] "This study addresses these questions at the dyadic level in an attempt to enhance our understanding of choices a firm makes regarding these systems, their alignment with desired performance outcomes, and their contingent context." [Data Sources and Method] "Standard and Poor’s Corporation Description (Standard and Poor’s Corporation, 1999) was used to select vice presidents of manufacturing or operations as key target respondents for the study." [Data Sources and Method] "Data from the 38 companies that had established electronic linkages were used for testing the research framework." [Table 1: Construct operationalization and measurement] "Process Efficiency (PE) • Electronic linkages with vendors reduce transaction costs for our firm."</t>
         </is>
       </c>
     </row>
@@ -24518,6 +25077,16 @@
           <t>BSMA0509</t>
         </is>
       </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G512" t="inlineStr">
         <is>
           <t>Many humanitarian aid workers receive training prior to being dispatched into the field, but they often encounter challenges that require additional learning and creativity. Consequently, aid organizations formally support collaboration among the expatriate and local workers in a field office. At best, those aid workers would not only exploit their joint knowledge but also explore novel ways of managing the challenges at hand. Yet differences between expatriate and local groups (e.g., in ethnicity, religion, education, and salary) often thwart intergroup collaboration in field offices and, by extension, any joint learning or creativity. In response to this issue, we study the role of field office leaders—specifically, how their boundary‐spanning behavior may inspire collaboration between the two groups and therefore facilitate joint learning and creativity. We propose that a leader's in‐group prototypicality additionally catalyzes this process—that is, a leader's behavior has more impact if s/he is seen as representing his/her group. We tested and found support for our hypothesized moderated mediation model in a field sample of 137 aid workers from 59 humanitarian organizations. Thus, our study generally highlights the pivotal role that field office leaders play for crucial outcomes in humanitarian aid operations. Furthermore, we offer concrete steps for field office leaders who want to inspire better collaboration between the expatriate and local aid workers they lead.</t>
@@ -24541,6 +25110,11 @@
       <c r="K512" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P512" t="inlineStr">
+        <is>
+          <t>Study measures Boundary Spanning Leadership (Leader BSB) where aid workers rate their field office manager's boundary spanning between local and expatriate groups. Includes a valid correlation matrix for N=137 individuals.. Verbatim Evidence: [Sample] "Our sample consisted of 137 humanitarian aid workers who voluntarily participated in an anonymous online survey." [Level of Analysis] "In the final sample, 36% of participants were local humanitarian aid workers, whereas 64% belonged to the expatriate group." "Table 1 shows the means, standard deviations, intercorrelations of variables, and Cronbach's α-value." [Measures] "We measured boundary-spanning leadership using a three-item scale adopted from the Intergroup Rhetoric Scale by Rast (2013). We separately asked expatriate and local respondents to describe whether their field office manager (1) “interacts frequently with both local and expatriate employees”, (2) “is equally available for the local and expatriate employees during office hours”, and (3) “puts a lot of effort in strengthening the relationship between the local and expatriate group”."</t>
         </is>
       </c>
     </row>
@@ -24629,6 +25203,16 @@
           <t>BSMA0512</t>
         </is>
       </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G515" t="inlineStr">
         <is>
           <t>The public sector is increasingly collaborating with the private sector in the development of large-scale public infrastructure projects. However, the difficulties arising due to working across organizational boundaries are often detrimental to project performance. This article argues that boundary-spanning activities can enhance the quality of collaboration and subsequently the performance of projects. Boundary spanners utilize relational governance mechanisms and undertake conscious endeavors for building interorganizational relationships by engaging in activities, such as coordination and communication with the stakeholders. The data for this study are composed of 158 survey responses from lead public managers involved in Dutch national public infrastructure projects. The data are analyzed using structural equation modeling. The study demonstrates that the quality of collaboration has a significant impact on the performance of the project during the implementation phase. Further, we find that the different boundary-spanning activities are interconnected and that they have a significant positive relationship on project performance, with a mediating effect of collaboration. The study concludes that, and shows how boundary spanners are vital to the collaborative processes through which public infrastructure projects are implemented.</t>
@@ -24652,6 +25236,11 @@
       <c r="K515" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P515" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning behaviors of 158 public managers working on inter-organizational infrastructure projects, providing a zero-order latent correlation matrix.. Verbatim Evidence: [Sample] "The data were collected through a survey sent to public managers from Rijkswaterstaat, the executive agency of the Ministry of Infrastructure and Water Management in the Netherlands." [Sample Size] "This brings the number of observations in the dataset to a total of 158(from 58 projects)." [Level of Analysis] "The assumption of independence of observations and errors could be compromised as the data are clustered by projects. This has been accounted for, however, in the analysis by using clustered robust standard errors, which relaxes the assumption of independence of errors to the assumption of independence of clusters." [Measures] "Boundary spanning activities (BS, Cronbach ’s alpha ¼0.97, composite reliability ¼0.97) “To what extent were you involved in …”" [Measures] "RA1: Building and maintaining lasting relationships with the partner organization."</t>
         </is>
       </c>
     </row>
@@ -24666,6 +25255,16 @@
           <t>BSMA0513</t>
         </is>
       </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G516" t="inlineStr">
         <is>
           <t>We report results from a longitudinal study of information systems development (ISD) teams. We use data drawn from 60 ISD teams at 22 sites of 15 Fortune 500 organizations to explore variations in performance relative to these teams’ social interactions. To do this, we characterize ISD as a form of new product development and focus on team-level social interactions with external stakeholders. Drawing on cluster analysis, we identify ﬁve patterns of team-level social interactions and the relationships of these patterns to a suite of objective and subjective measures of ISD performance. Analysis leads us to report three ﬁndings. First, data indicate that no one of the ﬁve identiﬁed patterns maximizes all performance measures. Second, data make clear that the most common approach to ISD is the least effective relative to our suite of performance measures. Third, data from this study show that early indications of ISD project success do not predict actual outcomes. These ﬁndings suggest two issues for research and practice. First, these ﬁndings indicate that varying patterns of social interactions lead to differences in ISD team performance. Second, the ﬁndings illustrate that singular measures of ISD performance are an oversimpliﬁcation and that multiple measures of ISD performance are unlikely to agree.</t>
@@ -24689,6 +25288,11 @@
       <c r="K516" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P516" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=60 teams). Verbatim Evidence: [Abstract] "We use data drawn from 60 ISD teams at 22 sites of 15 Fortune 500 organizations to explore variations in performance relative to these teams’ social interactions." [ANALYSIS AND FINDINGS] "Data collection instruments were specifically designed to be collected at the individual level and then aggregated (by averaging responses of the team’s members) to the team level for analysis (Jones &amp; James, 1979; James, 1982; Klein et al., 1994; Klein &amp; Kozlowski, 2000)."</t>
         </is>
       </c>
     </row>
@@ -25471,7 +26075,7 @@
       </c>
       <c r="P536" t="inlineStr">
         <is>
-          <t>Firm-level analysis of scientific publications using accounting and patent databases lacking individual employee samples [Code 2 &amp; Code 3].. Verbatim Evidence: [Abstract] "Thispaper investigatesthe impactofscientific activities onthefirm'smarket value, using accountingdataforU.S.firms andmatched patentandscientific publication data." [Introduction] "Ourempirical analysisusesfirm-level information fromtheCompustat database andmatched scientificpublication andpatentdataforarepresentativesampleof1,739stockmarketlistedfirms(9,920 firm-year observations) fromallhigh-technologysectors,coveringtheperiod1996-2006."</t>
+          <t>[Code 2 &amp; Code 3] The study analyzes firm-level financial valuation and patent/publication data (N = 1,739 firms) without an individual employee sample.. Verbatim Evidence: [Code 2 &amp; Code 3] The study analyzes firm-level financial valuation and patent/publication data (N = 1,739 firms) without an individual employee sample. Verbatim Evidence: "[Abstract] This paper investigates the impact of scientific activities on the firm's market value, using accounting data for U.S. firms and matched patent and scientific publication data." "[Data and Methodology] Our analysis was based on a sample of U.S. public companies from high-technology industries, as defined by the Organisation for Economic Co-operation and Development (2011), including pharmaceuticals and biotechnology, telecommunication equipment and semiconductors, aircraft, as well as scientific and medical instruments." "[Data and Methodology] Firm-level data came from Standard and Poor's Compustat, patent data came from the Worldwide Patent Statistical Database (Patstat, version April 2014) provided by the European Patent office, and publication data came from Elsevier's Scopus database." "[Data and Methodology] The final sample size contained 9,920 firm-year observations, composed as shown in Table 1."</t>
         </is>
       </c>
     </row>
@@ -25575,7 +26179,7 @@
       </c>
       <c r="P538" t="inlineStr">
         <is>
-          <t>Excluded due to multiple reasons: the unit of analysis is the manufacturer-supplier dyad (Code 3), and the boundary-spanning proxy merely measures communication frequency (Code 1).. Verbatim Evidence: [4.1. Data Collection and Sample Characteristics] "The unit of analysis for this study is a manufacturer (buyer)âsupplier dyad." [4.1. Data Collection and Sample Characteristics] "The respondents answered questions regarding the overall relationship between the two firms, including listing all of the buyer plant locations that received products from the supplier." [Appendix A: Survey Questions] "Media-Rich Communication (Source = Buyer) (1 = Never; 2 = Annually; 3 = Semi-annually; 4 = Quarterly; 5 = Monthly; 6 = Weekly; 7 = Daily) How often do personnel from your firm and &lt;&lt;SUPPLIER&gt;&gt; communicate using the following methods. . . PC1 Face-to-face PC3 Telephone"</t>
+          <t>[Code 1 &amp; Code 3] Measures mere communication frequency between firms, and uses proxy informants to evaluate firm-level manufacturer-supplier dyads.. Verbatim Evidence: [Appendix A: Survey Questions] "Media-Rich Communication (Source = Buyer) (1 = Never; 2 = Annually; 3 = Semi-annually; 4 = Quarterly; 5 = Monthly; 6 = Weekly; 7 = Daily) How often do personnel from your firm and &lt;&lt;SUPPLIER&gt;&gt; communicate using the following methods... PC1 Face-to-face PC2 Video conferencing** PC3 Telephone" [4.1. Data Collection and Sample Characteristics] "The unit of analysis for this study is a manufacturer (buyer)–supplier dyad. To obtain dyadic responses, we contacted manufacturers and asked participants to respond about a specific supplier to whom the manufacturer had outsourced the manufacturing of products. The respondents answered questions regarding the overall relationship between the two firms, including listing all of the buyer plant locations that received products from the supplier."</t>
         </is>
       </c>
     </row>
@@ -25835,7 +26439,7 @@
       </c>
       <c r="P543" t="inlineStr">
         <is>
-          <t>Multiple reasons [Code 1 &amp; Code 3]: Team-level analysis of time pressure and creativity, with no measure of individual boundary spanning behavior.. Verbatim Evidence: [Abstract] Focusing on team creativity as the outcome of interest, we explore how teams with varying time pressures function alongside the distinct time pressures experienced by their supervisors. [Method] Our analysis is based on a multi-source, time-lagged sample of 377 salespeople in 51 teams. [Method] we aggregated our data from individuals to teams.</t>
+          <t>[Code 1 &amp; Code 3] No boundary spanning behavior measured and team-level analysis.. Verbatim Evidence: [Table 1] &lt;Table 1. Descriptive Statistics and Correlations. Variables M SD 1 2 3 4 5 6 1. Supervisor age 2. Supervisor gender 3. Team size 4. Supervisor time pressure 5. Team time pressure 6. Team creativity&gt; [Data and Research Sample] &lt;To explore our research question, we conducted a time-lagged study in which we collected data from teams and their direct-level supervisors in a large financial service firm in Canada.&gt; [Validity and Data Aggregation] &lt;Considering the results obtained from the tests, their satisfactory values, and the small team sizes within our sample (LeBreton &amp; Senter, 2008; Shieh, 2016), we aggregated our data from individuals to teams.&gt; [Table 1] &lt;Note. n=51 teams.&gt;</t>
         </is>
       </c>
     </row>
@@ -26444,7 +27048,7 @@
       </c>
       <c r="P555" t="inlineStr">
         <is>
-          <t>Qualitative study analyzing interorganizational projects [Code 1 &amp; Code 3]. Verbatim Evidence: [Qualitative study analyzing interorganizational projects lacking effect sizes] [Code 1 &amp; Code 3]. Verbatim Evidence: "[Abstract] The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." "[3. Research setting and methods] We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." "[3. Research setting and methods] Our data analysis followed an âabductiveâ approach (Alvesson and SkÃ¶ldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
+          <t>Qualitative study with no extractable quantitative effect sizes [Code 1], analyzing interorganizational projects at the firm/project level [Code 3].. Verbatim Evidence: [Abstract] "The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." [3. Research setting and methods] "We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." [3. Research setting and methods] "Our data analysis followed an “abductive” approach (Alvesson and Sköldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
         </is>
       </c>
     </row>
@@ -26730,6 +27334,16 @@
           <t>BSMA0558</t>
         </is>
       </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G561" t="inlineStr">
         <is>
           <t>In multinational corporations (MNCs), cross-cultural interactions and collaboration are unavoidable. Cultural boundary spanning (CBS) is a behavior that has been shown to reduce conflict and ensure project success. It is a behavior that bridges internal and external organizational boundaries. This study examined if and how CBS functions (behaviors) change across national and cultural boundaries in MNCs. These boundaries were characterized by four demographic groups of people found within MNCs:(a) parent country nationals,(b) host country nationals,(c) third country nationals, and (d) parent country national expats. The findings of this research suggest that any of these demographic groups can perform CBS. Variances in the use of CBS functions between the groups were also identified. These variances seem to be influenced by the strength of the individual’s social networks and the interdependent leadership culture within the MNC.</t>
@@ -26753,6 +27367,11 @@
       <c r="K561" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P561" t="inlineStr">
+        <is>
+          <t>Qualitative/descriptive mixed-methods study lacking a correlation matrix or extractable zero-order effect sizes.. Verbatim Evidence: [Research Design] This study utilized an explanatory sequential mixed-methods research approach whereby an initial quantitative survey was utilized to set the stage for further exploration of the proposed theory through a set of qualitative semi-structured interviews (Creswell &amp; Creswell, 2018). To derive basic means and standard deviations of the variable of CBS functions across the groups of national and cultural staffing combinations in MNCs, a quantitative survey was employed. [Participants] The study participants comprised of 17 working professionals, 19 years of age and older, who acted as cultural boundary spanners working for an MNC across national and cultural boundaries. [Quantitative Survey Results] Note. 1 = Never; 5 = Always N=20; (PCN – N=6, HCN – N=5, TCN – N=5, XPT N=4)</t>
         </is>
       </c>
     </row>
@@ -26989,6 +27608,16 @@
           <t>BSMA0565</t>
         </is>
       </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G568" t="inlineStr">
         <is>
           <t>Purpose – The aim of this paper is to investigate the link between store managers’ evaluation of how customers assess a shopping centre and their own evaluation of the centre and, based on that, the relevance of store managers in reflecting on and informing the management and marketing practices of the local shopping centre management.</t>
@@ -27012,6 +27641,11 @@
       <c r="K568" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P568" t="inlineStr">
+        <is>
+          <t>No effect size of interest. Boundary spanning is used as a theoretical lens, but the study measures shopping center attributes and satisfaction, not Boundary Spanning Behavior.. Verbatim Evidence: [Abstract] The model is tested using a Web-based survey of 217 managers,representing stores located in shopping malls, and by applying covariance-based structural equationmodelling. [Abstract] The study reveals store managers to be engaging in a significant information-processing pathway,from customers’ evaluation of the shopping centre (as perceived by the store manager) to their own evaluation of the centre in terms of managerial satisfaction and loyalty. [Table I] Tenant mix (/H92641) Atmosphere (/H92642) Orientation (/H92643) Infrastructural services (/H92644) (Evaluated) customer satisfaction with the shopping centre (/H926451) (Evaluated) customer loyalty towards the shopping centre (/H926452) (Evaluated) customer retention proneness in the shopping centre (/H926453) Managerial satisfaction with (overall evaluation of) the shopping centre (/H92571) Managerial loyalty (in terms of future suitability) to the shopping centre as a store location (/H92572)</t>
         </is>
       </c>
     </row>
@@ -27130,6 +27764,16 @@
           <t>BSMA0568</t>
         </is>
       </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G571" t="inlineStr">
         <is>
           <t>Flexible work arrangements (FWAs) are widely implemented for organizational purposes including recruitment. Theoretically, these arrangements alter temporal and physical boundaries around work. However, the time and place dimensions are frequently confounded in research, making the separate and joint effect of each on various outcomes unclear. To determine the relative importance of                 FWA                 dimensions as anticipated resources, this study experimentally manipulates discretion over when (flextime) and where (flexplace) one is expected to work on anticipated organizational support (                 AOS                 ) and organization attraction. Prospective employees (                 N                  = 130) participated in a 3 × 3 within‐subject experiment in which they rated nine hypothetical organizations that varied in flextime and flexplace. Results indicated main effects for both flextime and flexplace on both                 AOS                 and organization attraction with flextime having the stronger impact. Although the combination of a high level of both flextime and flexplace yielded the highest ratings of                 AOS                 and organization attraction, the interaction between flextime and flexplace was not statistically significant, suggesting flextime and flexplace have independent effects on recruitment outcomes. Relationships between flextime and flexplace and organizational attraction were slightly stronger for individuals who prefer to integrate their work and non‐work roles. Managerial implications and directions for future research are discussed.                                                        Practitioner points                                                                        Potential applicants rate flextime without a required core time as significantly more supportive and attractive than flextime with core time.                                                           Potential applicants rate flextime with a required core time as significantly more supportive and attractive than no flextime.                                                           Potential applicants rate working from home 2 to 3 days a week as significantly more supportive and attractive than not being able to work from home at all.                                                           The supportiveness and attractiveness of flextime does not depend on the supportiveness or attractiveness of flexplace or vice versa.</t>
@@ -27153,6 +27797,11 @@
       <c r="K571" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P571" t="inlineStr">
+        <is>
+          <t>Multiple flaws: Student sample and no measure of boundary spanning behavior [Code 1 &amp; Code 2].. Verbatim Evidence: [Participants] "Study participants consisted of primarily upper-level undergraduate students from a large university in the south-west United States." [Measures] "Participants rated AOS and organization attraction on a 5-point scale (1 = not at all, 5 = extremely) for each organization description; thus, these variables were assessed nine times by each respondent."</t>
         </is>
       </c>
     </row>
@@ -27278,6 +27927,16 @@
           <t>BSMA0572</t>
         </is>
       </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G575" t="inlineStr">
         <is>
           <t>Efforts to initiate new startups rely heavily on teams and networks. Research demonstrates that 95 percent of the individuals trying to start a business involved others in helping build the new business. This article provides an overview of the team performance literature that can be used when making managerial decisions about building and managing successful entrepreneurial teams. I integrate and review prior research in three areas that have been disconnected previously: 1) innovation networks and teams; 2) team boundary spanning and internal processes; and 3) shared ownership and team motivation. The integration and review in this article provide new insights towards an evidence-based approach on managing entrepreneurial teams.</t>
@@ -27301,6 +27960,11 @@
       <c r="K575" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P575" t="inlineStr">
+        <is>
+          <t>Non-primary study (review article). Verbatim Evidence: [Abstract] "This article provides an overview of the team performance literature that can be used when making managerial decisions about building and managing successful entrepreneurial teams. I integrate and review prior research in three areas that have been disconnected previously" [Introduction] "The goal of this article is to provide an overview of the team performance literature that can be used when making managerial decisions about building and managing successful entrepreneurial teams."</t>
         </is>
       </c>
     </row>
@@ -27648,6 +28312,16 @@
           <t>BSMA0582</t>
         </is>
       </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G585" t="inlineStr">
         <is>
           <t>The literature recognizes that the sales profession is an inherently competitive and self-interested occupation that can be negatively impacted by deviant behavior and rationalizations of unethical conduct. The unique boundary-spanning nature and autonomy of such work means that there is often little management oversight of sales professionals' behavior, which may lead to misbehavior and poor work attitudes. Yet, evidence suggests that the development of corporate ethical values (CEVs) can mitigate concerns about unethical conduct, suggesting that these principles might be used to reduce workplace bullying and enhance job satisfaction. Using a self-report questionnaire, information was collected from national and regional samples of selling professionals employed in different organizations located in the USA (N = 356). While controlling for the effects of sampling and social desirability, results indicated that increased communication of an ethics code was associated with stronger perceptions of CEVs, while ethical values were negatively related to perceptions of workplace bullying and positively related to job satisfaction. Workplace bullying was also negatively related to job satisfaction. The findings suggest that an ethical work environment should be instituted in sales organizations to reduce misconduct and enhance work attitudes.</t>
@@ -27671,6 +28345,11 @@
       <c r="K585" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P585" t="inlineStr">
+        <is>
+          <t>No boundary spanning behavior construct measured. The study uses the boundary-spanning nature of sales as context but empirically measures corporate ethical values, workplace bullying, and job satisfaction.. Verbatim Evidence: [Abstract] "The unique boundary-spanning nature and autonomy of such work means that there is often little management oversight of sales professionals’ behavior, which may lead to misbehavior and poor work attitudes. Yet, evidence suggests that the development of corporate ethical values (CEVs) can mitigate concerns about unethical conduct, suggesting that these principles might be used to reduce workplace bullying and enhance job satisfaction." [Table 5] "Table 5. Variable descriptive statistics, correlations, and reliability statistics. Variable M SD N α 1 2 3 4 5 6 7 1. Availability of ethics code 1.71 .45 347 – – 2. Communication of ethics code 2.35 .68 273 – .58*** – 3. Corporate ethical values 5.04 1.65 351 .82 .22*** .36*** – 4. Workplace bullying 2.83 1.88 345 .89 −.08 −.05 −.13* – 5. Job satisfaction 5.29 1.57 351 .86 .10 .12* .47*** −.23*** – 6. National vs. Regional samples 1.63 .48 356 – .14** .06 −.19*** .10* −.21*** – 7. Social desirability 5.60 1.40 354 .75 .03 .04 .32*** .12 .30*** −.21*** –"</t>
         </is>
       </c>
     </row>
@@ -27833,6 +28512,16 @@
           <t>BSMA0587</t>
         </is>
       </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G590" t="inlineStr">
         <is>
           <t>Previous research has extensively analyzed the role, and indicated the importance, of network management for the functioning and performance of public or governance networks. In this article, we focus on the inﬂuence of boundary spanning actors in such networks—an aspect less examined in the governance network literature. Boundary spanners are considered to be important for governance network performance. Building on the literature, we expect a mediating role of trust in this relationship. To empirically test these relationships, we conducted survey research (N = 141) among project managers involved in urban governance networks: networks around complex urban projects that include the organizations involved in the governance process (the formulation of policies, decision making, and implementation) in these complex projects. We found a strong positive relationship between the presence of boundary spanners and trust and governance network performance. The results indicate a partially mediating role of trust in this relationship. Furthermore, we found that these boundary spanners originated mainly from private and societal organizations, and less from governmental organizations.</t>
@@ -27856,6 +28545,11 @@
       <c r="K590" t="inlineStr">
         <is>
           <t>2014</t>
+        </is>
+      </c>
+      <c r="P590" t="inlineStr">
+        <is>
+          <t>Network/Project-level analysis. Respondents act as key informants evaluating the presence of boundary spanners within a governance network, not their own individual behavior.. Verbatim Evidence: [Unit of analysis] "Our unit of analysis is on the level of the governance network. We study the presence of boundary spanners in the network, which do not necessarily be the official project manager but also can turn out to be other persons (resident, private project developer, etc.). We therefore asked the leading project manager of each network to what extent they witnessed boundary spanners in the network." [Measurement items and constructs’ reliability] "Presence of boundary spanners in the governance network ... 1. In this project, there are many persons active who are able to build and maintain sustainable relationships with different organizations in the network"</t>
         </is>
       </c>
     </row>
@@ -28499,6 +29193,16 @@
           <t>BSMA0605</t>
         </is>
       </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G608" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate the antecedents of frontline employees’ boundary-spanning behaviors in the hospitality industry. Anchored in transactional stress theory, affective events theory and motivation theories, a conceptual model was built to explore the impacts of hindrance stressors on boundary-spanning behavior.</t>
@@ -28522,6 +29226,11 @@
       <c r="K608" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P608" t="inlineStr">
+        <is>
+          <t>This study measures the boundary-spanning behaviors of individual frontline hospitality employees using a valid BSB scale and provides an extractable matrix of (squared) zero-order correlations.. Verbatim Evidence: [Abstract] "Data were collected from frontline employees in the hospitality industry in the USA." [3. Methodology] "Two screening questions were implemented at the beginning of the questionnaire: “Do you work in the hospitality industry (hotels, restaurants, resorts) in the USA?” and “At work, do you directly interact with guests daily?”" [4.1 Sample profile] "unusable questionnaires, 557 responses were included for data analysis" [3.1 Questionnaire design] "Finally, based on the conceptual definitions developed by Bettencourt et al. (2005), the boundary-spanning behavioral items were classified into three dimensions: evaluate external representation (four items), internal influence (four items) and service delivery (five items)." [4.2 Measurement model] "Furthermore, by comparing AVEs and correlation coefficients’ squares, discriminant validity of the scales was confirmed. As shown in Table 3, AVE scores for all dimensions, presented in the diagonal of the matrix, exceeded the squares of paired correlation coefficients, shown in the off-diagonal of the matrix, satisfying discriminant validity"</t>
         </is>
       </c>
     </row>
@@ -28536,6 +29245,16 @@
           <t>BSMA0606</t>
         </is>
       </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G609" t="inlineStr">
         <is>
           <t>The present study explores the antecedents of frontline employees’ boundary-spanning behaviors in the hospitality industry. Based on social exchange theory and role theory, a conceptual model was built to explore how three dimensions of perceived organizational support (perceived supervisory support, internal communication, and training) cultivate frontline employees’ boundary-spanning behaviors through job satisfaction and organizational commitment. Based on the analysis of 597 hospitality frontline employees in the United States, which were recruited through Amazon Mechanical Turk, this study shows the differential impacts of organizational support types on driving boundary spanning staff to effectively operate on the boundary. Theoretical and practical implications of the findings are articulated.</t>
@@ -28559,6 +29278,11 @@
       <c r="K609" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P609" t="inlineStr">
+        <is>
+          <t>Valid BSB construct (External Representation and Internal Influence) measured at the individual level using a sample of 597 hospitality frontline employees.. Verbatim Evidence: [Abstract] "Based on the analysis of 597 hospitality frontline employees in the United States, which were recruited through Amazon Mechanical Turk, this study shows the differential impacts of organizational support types on driving boundary spanning staff to effectively operate on the boundary." [Methodology] "The measurement of boundary-spanning behaviors in this study is based on the conceptual definitions by Bettencourt et al. (2005). Particularly, external representation was assessed by four items, internal influence was measured via four items, and service delivery was tested through five items." [Findings] "The sample contains 325 males and 270 females."</t>
         </is>
       </c>
     </row>
@@ -28573,6 +29297,12 @@
           <t>BSMA0607</t>
         </is>
       </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr"/>
       <c r="G610" t="inlineStr">
         <is>
           <t>Building on resource‐based theory and resource orchestration theory, we investigate the impact of two characteristics of boundary‐spanning search, search breadth and search depth, on firms' exploitative and exploratory green innovations. We also examine the moderating role of resource orchestration capability. The results of data analysis from 186 manufacturing firms in China show that both search breadth and search depth have inverted U‐shaped relationships with exploitative and exploratory green innovations. Furthermore, resource orchestration capability is found to moderate the inverted U‐shaped relationship between boundary‐spanning search and green innovation. Specifically, with high resource orchestration capability, the inverted U‐shaped relationships of search breadth with exploitative and exploratory green innovations are flattened, whereas the relationships of search depth with exploitative and exploratory green innovations are almost linear. Our research contributes to the literature on green innovation by uncovering the complex effects of boundary‐spanning search on exploitative and exploratory green innovations.</t>
@@ -28596,6 +29326,11 @@
       <c r="K610" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P610" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28721,6 +29456,16 @@
           <t>BSMA0611</t>
         </is>
       </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G614" t="inlineStr">
         <is>
           <t>Based on social information processing theory, we provide a novel theoretical account of how and when leader humor influences subordinate boundary-spanning behavior. We develop a moderated mediation model explicating the mechanism of psychological safety and the boundary condition of subordinate interpersonal influence. Using multiwave data, we tested our research hypotheses with a sample of 452 members from 140 teams in a Chinese information technology (IT) company. Results showed that leader humor positively affects subordinate boundary-spanning behavior               via               increased psychological safety. Moreover, this mediated effect is stronger when subordinates have high interpersonal influence. These findings offer theoretical and practical insights into boundary-spanning activities and leader humor, which we discuss.</t>
@@ -28744,6 +29489,11 @@
       <c r="K614" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P614" t="inlineStr">
+        <is>
+          <t>Valid individual-level BSB with N=452 subordinates providing a correlation matrix.. Verbatim Evidence: [Sample] "we had final responses from 452 subordinates in 140 teams, constituting a final effective response rate of 78%." [Measures] "We measured boundary-spanning behavior with a six-item scale developed by Marrone et al. (2007). Subordinates were asked to evaluate the extent to which they engage in boundary-spanning behavior. A sample item is “I can persuade outsiders (e.g., faculty, clients) to support our team decisions.”" [Matrix N] "TABLE 1 Descriptive statistics and correlations... N = 452 subordinates."</t>
         </is>
       </c>
     </row>
@@ -28847,6 +29597,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -29082,6 +29833,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -29124,6 +29876,16 @@
           <t>BSMA0620</t>
         </is>
       </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G623" t="inlineStr">
         <is>
           <t>Teams have a high potential for innovation development by carrying out innovative work behaviour (IWB), but research remains limited on how engagement in team learning behaviours (TLBs) can foster IWB among team members. Especially longitudinal studies investigating the dynamic character of both constructs are missing. To clarify the relationship between TLBs and IWB over time, we conducted a threewave longitudinal survey among interdisciplinary work teams in German vocational education. Based on a sample of 66 work teams with 275 team members consisting of vocational educators, such as teachers, school principals and social workers, a manifest cross-lagged panel model was estimated to capture the dynamic relationship between TLBs and IWB. The hierarchical structure was taken into account and missing data were imputed. The results indicate that knowledge sharing and team reﬂexivity at the beginning of the teamwork predict future engagement in dimensions of IWB. In the further course of the teamwork boundary spanning becomes an important TLB for IWB. The TLBs that are relevant for IWB are inﬂuenced by task interdependence and team structure. The results provide insight into how IWB can be fostered through TLBs over time. At the beginning of a work task, knowledge sharing and team reﬂexivity should be fostered by encouraging discussion and enriching diﬀerent perspectives to reach high engagement in IWB. In the further course of teamwork information should be gathered from outside the team, for instance by inviting experts.</t>
@@ -29147,6 +29909,11 @@
       <c r="K623" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P623" t="inlineStr">
+        <is>
+          <t>Team-level referent. The boundary spanning items ask respondents to rate the behavior of 'team members' collectively rather than their own individual behavior, making them proxy informants for team-level boundary spanning.. Verbatim Evidence: [Measures] Boundary spanning was assessed using Hirst and Mann’s(2004) four-item scale, including such items as (a) ‘When necessary, team members consult with individuals who possess knowledge relevant to the project’; (b) ‘Team members seek relevant information from across the college’.</t>
         </is>
       </c>
     </row>
@@ -29198,6 +29965,16 @@
           <t>BSMA0622</t>
         </is>
       </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G625" t="inlineStr">
         <is>
           <t>Inter‐organizational frameworks of intervention dominate the resolution of complex societal problems facing the UK and many other countries. Strategic alliances, joint working arrangements, networks, partnerships and many other forms of collaboration across sectoral and organizational boundaries currently proliferate across the policy landscape. However, the discourse is positioned at an institutional and organizational level, and comparatively little attention is accorded to the pivotal role of individual actors in the management of inter‐organizational relationships. This paper attempts to redress this balance by focusing on the skills, competencies and behaviour of boundary spanners. A critical review of the relevant literature, both from an institutional and relational perspective, is undertaken. This is complemented by some new empirical research that involves an engagement with groups of particular types of boundary spanner using a combination of surveys and in‐depth interviews. Finally, a discussion makes connections between the existing literature and the research findings and offers suggestions for future areas of enquiry.</t>
@@ -29221,6 +29998,11 @@
       <c r="K625" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P625" t="inlineStr">
+        <is>
+          <t>Qualitative/descriptive study lacking quantitative effect sizes (r) or a correlation matrix.. Verbatim Evidence: [Abstract] "This is complemented by some new empirical research that involves an engagement with groups of particular types of boundary spanner using a combination of surveys and in-depth interviews." [RESEARCH METHODOLOGY] "Phase 1 is directed to an initial identification and categorization of boundary spanning competencies together with a short attitudinal investigation." [RESEARCH METHODOLOGY] "Phase 2 sharpened the focus of the research with a more intensive exploration and understanding of the potential determinants of effective boundary spanning framed within a particular geographical area." [RESEARCH METHODOLOGY] "The findings from Phase 1 were used to inform the topic guide for a series of in-depth and semi-structured interviews."</t>
         </is>
       </c>
     </row>
@@ -29346,6 +30128,16 @@
           <t>BSMA0626</t>
         </is>
       </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G629" t="inlineStr">
         <is>
           <t>Drawing from the structural perspective of social capital theory, this research investigates how internal and external advice network structures inﬂuence knowledge overlap and variety and, how these knowledge dimensions in turn inﬂuence group effectiveness. Findings from two studies on knowledge-intensive groups indicate that different advice network structures are associated with knowledge overlap and knowledge variety, and only knowledge variety was signiﬁcantly associated with group effectiveness. In addition, despite implicit understanding that advice networks aid performance through enhancing knowledge outcomes, only knowledge variety was found to mediate the relationship between external network and group effectiveness. Implications for theory and practice are discussed. Copyright # 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -29369,6 +30161,11 @@
       <c r="K629" t="inlineStr">
         <is>
           <t>2008</t>
+        </is>
+      </c>
+      <c r="P629" t="inlineStr">
+        <is>
+          <t>Team Level Aggregation (N = teams) based on the focus on Team Boundary-Spanning.. Verbatim Evidence: [Title] "Does Team Boundary-Spanning Enhance the Quality of Megaprojects The Underlying"</t>
         </is>
       </c>
     </row>
@@ -29494,6 +30291,16 @@
           <t>BSMA0630</t>
         </is>
       </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G633" t="inlineStr">
         <is>
           <t>Motivated by the inconsistent findings of the linkage between early supplier involvement practice and new product development success, this study adopts both the resource-based perspective and agency theory to investigate dynamic relationships between the manufacturer and supplier during the collaboration process. Survey data were used to empirically examine the impact of the resource factor (i.e. collaboration effect) and agency factors (i.e. interaction effect) on project team effectiveness. The results showed that selecting suppliers with appropriate knowledge and resources is necessary yet insufficient to improve project team effectiveness. The agency problem plays a dominant role in determining the quality of collaboration. In particular, the study identified information sharing and task programmability as two key governance mechanisms to curb suppliers’ opportunistic behaviour. The study provides insightful managerial and policy implications for firms considering early supplier involvement practice in their innovation process.</t>
@@ -29517,6 +30324,11 @@
       <c r="K633" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P633" t="inlineStr">
+        <is>
+          <t>Non-individual level (project/buyer-supplier relationship analysis) and proxy informant. Verbatim Evidence: [4 Research methodology] "The unit of analysis in this study is a specific case of supplier involvement in the NPD process. Respondents were asked to select a completed case of supplier involvement with which they were familiar and answer the questions based on the experience in that particular project." [4.2 Measures] "IS1 Sharing of cost information between my business unit and the supplier. IS2 Sharing of technology information between my business unit and the supplier"</t>
         </is>
       </c>
     </row>
@@ -29605,6 +30417,16 @@
           <t>BSMA0633</t>
         </is>
       </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G636" t="inlineStr">
         <is>
           <t>Transnational knowledge networks provide organizations with information useful in addressing shared problems. Social media may enable the formation of those networks, yet their role in the process has received little attention. This article examines the structure and antecedents of two networks facilitated by the microblogging platform Twitter operating in the policy domain of emergency management. One network includes national-level government agencies responsible for disaster response and recovery operations; the other includes nongovernmental organizations in the form of Red Cross and Red Crescent national societies. We use a logistic regression quadratic assignment procedure to test hypotheses derived from related literature. While findings indicate that shared language and geographic proximity shaped network formation, both networks exhibit boundary spanning behavior in which organizations sought out information from high-profile, resource-rich organizations. Those organizations helped to connect otherwise regionally bound clusters and demonstrate the nascent potential of social media to create global transnational knowledge networks.</t>
@@ -29628,6 +30450,11 @@
       <c r="K636" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P636" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3]. Verbatim Evidence: [Data Collection] "Our dependent variable is whether an organization seeks out information from another via social media, and we operationalize it as whether an emergency management organization follows the Twitter account of another emergency management organization in a foreign country. Thus, our unit of analysis is the directional dyad." [Data Collection] "First, we identified government emergency management organizations... We also identified Red Cross and Red Crescent national societies" [Results] "Table 5 QAP Logistic Regression Results... Num. obs. 3540... 9312"</t>
         </is>
       </c>
     </row>
@@ -29938,6 +30765,12 @@
           <t>BSMA0642</t>
         </is>
       </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr"/>
       <c r="G645" t="inlineStr">
         <is>
           <t>Purpose – In today’s complex and rapidly changing business environment, cross-boundary growth is increasingly critical to the survival or even success of organizations. The purpose of this study is to examine the forming mechanism of ﬁrm’s cross-boundary growth by integrating the two important antecedent factors of performance pressure and managerial discretion into a united framework and theoretically analyze the direct role of performance pressure on ﬁrm’s cross-boundary growth as well as reveal the moderating role of managerial discretion. Also, the authors select listed manufacturing companies in China as samples to empirically test the research hypotheses.</t>
@@ -29961,6 +30794,11 @@
       <c r="K645" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P645" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The study conducts a firm-level analysis using panel data of 1,334 listed manufacturing companies from a financial database. The dependent variable is firm-level cross-boundary growth (measured by the Herfindahl Index of cross-regional and cross-industry revenue), and it does not measure interpersonal boundary-spanning behavior by individual employees.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -30049,6 +30887,12 @@
           <t>BSMA0645</t>
         </is>
       </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr"/>
       <c r="G648" t="inlineStr">
         <is>
           <t>Summary                            Team creativity, as one of the most important sources of organizational competitiveness and continuous innovation, requires rich and non‐redundant information from both internal and external sources. Although an emerging line of research has shed light on the role of team boundary‐spanning activity in promoting creativity, it has solely focused on the mean level of team boundary‐spanning activity and rarely addressed the fact that not all team members engage in boundary‐spanning behaviors to the same extent. In this study, we broaden the existing knowledge by examining               when               and               how               the pattern of team boundary spanning, particularly the differentiation in team member boundary‐spanning activities, promotes team creativity. Based on the categorization‐elaboration model, we propose a curvilinear relationship between team member boundary‐spanning differentiation and creativity that is mediated through information sharing. Further, we add an important layer of understanding to the nature of this curvilinear relationship by identifying team goal interdependence as an important moderator. Using multisource data collected from two time points in 70 teams, we have received general support for our hypotheses. As such, we enrich the conversation about the importance of team boundary spanning by answering “               Whether               team boundary‐spanning differentiation fosters creativity, and               when               and               how               ?”</t>
@@ -30072,6 +30916,11 @@
       <c r="K648" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P648" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -30350,6 +31199,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry. Using a multiyear sample of ﬁrms from the computer industry, we found that intra-industry trade-association ties of top managers led to the adoption of a resource-imitation strategy by late movers while extra-industry importation and professional-association ties led to the adoption of a resource-substitution strategy. We also found that trade association ties had a negative effect on the performance of late movers using resource-substitution, while top managers’ service on other ﬁrms’ boards had a positive inﬂuence on the performance of those ﬁrms. Our ﬁndings not only conﬁrm the importance of the role of ﬁt in strategy and performance, but they also highlight the importance of the management and control of boundary-spanning activities.</t>
@@ -30496,6 +31346,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G659" t="inlineStr">
         <is>
           <t>Individuals in work teams frequently cross boundaries across teams, often by using information and communication technologies (ICTs). The current study investigates the effects of members’ boundary work and the visibility affordance of teams’ ICTs on Transactive Memory Systems (TMS) in teams. Survey data from 212 fulltime employees whose work hours were divided between multiple teams reveals that boundary spanning enhances the focal team’s TMS specialization and credibility and negatively inﬂuences TMS coordination. Additionally, boundary reinforcement positively affects TMS credibility and coordination. The visibility affordance has a direct positive effect on all three dimensions of TMS and a moderating effect for boundary reinforcement such that higher visibility overrides the positive direct effect of boundary reinforcement on TMS. These ﬁndings suggest that different types of boundary work contribute to different dimensions of TMS and that teams might consider prioritizing the use of ICTs with high visibility to enhance their TMS.</t>
@@ -30523,7 +31378,7 @@
       </c>
       <c r="P659" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Non-individual level (proxy informant for team-level boundary spanning). Verbatim Evidence: [Measures] "Boundary spanning was measured using items including “Does the team value team members for making use of their relationships with others on behalf of the team?, ”and“Does your primary team encourage its members to solicit information and resources from elsewhere inand/or beyond the team? ”" [Participants] "The ﬁnal sample included 212 participants."</t>
         </is>
       </c>
     </row>
@@ -30595,6 +31450,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>This study examines how deans and associate deans of a group from similar universities use networking. Specifically, we consider whether the deans, traditionally considered to perform boundary-spanning functions, make more use of external networking than do the associate deans, who are their subordinates. We examine the relationship between accuracy in perceiving a network and influence in the network. Finally, we consider the relationship between reports of networking outside the sample and influence within the sample. We find support for our first two propositions and raise several issues related to our final one.</t>
@@ -30736,6 +31592,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -30993,6 +31850,16 @@
           <t>BSMA0667</t>
         </is>
       </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G670" t="inlineStr">
         <is>
           <t>Innovations transform our research traditions and become the driving force to advance individual, group, and social creativity. Meanwhile, interdisciplinary research is increasingly being promoted as a route to advance the complex challenges we face as a society. In this paper, we use Latent Dirichlet Allocation (LDA) citation as a proxy context for the diffusion of an innovation. With an analysis of topic evolution, we divide the diffusion process into five stages: testing and evaluation, implementation, improvement, extending, and fading. Through a correlation analysis of topic and subject, we show the application of LDA in different subjects. We also reveal the cross‐boundary diffusion between different subjects based on the analysis of the interdisciplinary studies. The results show that as LDA is transferred into different areas, the adoption of each subject is relatively adjacent to those with similar research interests. Our findings further support researchers' understanding of the impact formation of innovation.</t>
@@ -31016,6 +31883,11 @@
       <c r="K670" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P670" t="inlineStr">
+        <is>
+          <t>Bibliometric analysis of citations rather than a measure of individual Boundary Spanning Behavior [Code 1 &amp; Code 2].. Verbatim Evidence: [Abstract] "In this paper, we use Latent Dirichlet Allocation (LDA) citation as a proxy context for the diffusion of an innovation." [Methodology] "The search result of citation numbers of LDA is 6,822 in Scopus and only 3,797 in Web of Science between 2003 and 2015. So in this study, we used LDA citation extracted from Scopus."</t>
         </is>
       </c>
     </row>
@@ -31156,6 +32028,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -31198,6 +32071,16 @@
           <t>BSMA0672</t>
         </is>
       </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G675" t="inlineStr">
         <is>
           <t>Purpose – In the field of innovation, there is growing interest in exploring the factors that determine the extent to which firms can learn from external sources. However, most previous studies neglect the role of human factors. Little is known about which employee behaviors are desirable for boundary-spanning learning activities and which human resource management (HRM) practices are appropriate to respond to external knowledge transfer across boundaries. To fill this gap, the authors investigate the role of empowermentfocused HRM in interfirm learning and explore the integration of external inputs from the perspective of employees.</t>
@@ -31221,6 +32104,11 @@
       <c r="K675" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P675" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] The study analyzes plant-level learning rather than individual boundary spanning behavior (N=288 plants). The construct is firm-level relationship learning rather than interpersonal boundary spanning.. Verbatim Evidence: [Methodology] "The data were collected from 288 manufacturing plants located in 13 different countries and three different industrial sectors (electronics, machinery and transportation equipment)." [Methodology] "To avoid common method bias, each questionnaire had two informants. We ultimately collected 288 useable questionnaires with a response rate of 65%." [Measurements] "Information sharing was assessed by a four-item scale, involving whether the plant exchanges information related to changes in demand, sensitive content, organizational strategies and policies and key product technologies with their partners."</t>
         </is>
       </c>
     </row>
@@ -31235,6 +32123,16 @@
           <t>BSMA0673</t>
         </is>
       </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G676" t="inlineStr">
         <is>
           <t>Enterprise social media (ESM) provides convenient channels for employees to access enterprise-wide work resources but also exposes employees to potential distractions. Prior studies have confirmed this “two-sided” role of ESM usage on employee work performance. Ongoing studies are exploring possible methods to alleviate side effects of ESM usage. Drawing on boundary management literature and information processing theory, we propose the concept of individual boundary spanning to capture employees’ information-obtaining behaviors via ESM and identify two mediating mechanisms—mindfulness and information overload—through which an individual’s boundary spanning affects work performance. We also propose the concept of individual boundary buffering to capture protective actions by individuals that prevent them from becoming disturbed or overloaded with ESM requests. We further investigate the interaction effects of these two boundary activities in the ESM context. We conducted a survey and collected data from 202 ESM users from a research and development enterprise in China. The results suggest that individual boundary spanning triggers mindfulness in individuals that benefits their work performance but also increases information overload, harming work performance. Individual boundary buffering can enhance the positive relationship between individual boundary spanning and mindfulness, and mitigate the positive relationship between spanning activity and information overload.</t>
@@ -31258,6 +32156,11 @@
       <c r="K676" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P676" t="inlineStr">
+        <is>
+          <t>Valid individual-level intra-organizational boundary spanning behavior with an employee sample and extractable correlations.. Verbatim Evidence: [Sample] &lt;We collected data from a large Chinese telecommunications and information technology corporation with over 10,000 employees in Xi’an, China.&gt; [Sample] &lt;After deleting responses with missing data, we analyzed 202 usable responses to test the proposed model.&gt; [Measures] &lt;We specified the 'external' (the connotation of boundary) of the respondents as the demarcation formed by the accessibility officially provided by the project team that they are in.&gt; [Measures] &lt;BS1. I use ESM to solicit information and resources from external channels.&gt; [Data] &lt;Table 5 The correlation matrix of constructs.&gt;</t>
         </is>
       </c>
     </row>
@@ -31272,6 +32175,16 @@
           <t>BSMA0674</t>
         </is>
       </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G677" t="inlineStr">
         <is>
           <t>Research Summary: This study elucidates the previously underexplored structural heterogeneity inherent in multinational corporations' (MNCs) internal linkages by examining the concentration of cross-border collaborations among inventors within host countries. Building on the boundary spanning literature, we develop a two-stage framework identifying the knowledge distortion mechanism arising from this concentration: information overload in the cross-country knowledge absorption stage and long transmission paths and knowledge hoarding in the within-country diffusion stage. Both hinder local knowledge creation. We further propose that cross-country and withincountry network structures serve as contingencies moderating this relationship. The negative effects of collaboration concentration are exacerbated by structural holes in cross-country networks but attenuated by the reach and density of within-country networks. Empirical results based on American pharmaceutical MNCs from 1980 to 2008 support our hypotheses.</t>
@@ -31295,6 +32208,11 @@
       <c r="K677" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P677" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] The study uses archival patent data at the MNC-country-year level of analysis, not individual employee survey data.. Verbatim Evidence: [Code 2 &amp; Code 3] The study uses archival patent data and analyzes data at the MNC-country-year level rather than the individual employee level. Verbatim Evidence: "[3.1 | Sample and data collection] We investigated the concentration of cross-border collaborations in MNCs using data on listed pharmaceutical MNCs headquartered in the United States from 1980 to 2008." "[3.1 | Sample and data collection] We eventually obtained 97 MNCs involving 60,185 patents, whose overseas research operations are located across 24 host countries, comprising an unbalanced panel of 1954 MNC-country-year observations."</t>
         </is>
       </c>
     </row>
@@ -31586,6 +32504,16 @@
           <t>BSMA0682</t>
         </is>
       </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G685" t="inlineStr">
         <is>
           <t>This article draws on status characteristics theory to explore the mechanisms of individual-level boundaryspanning behavior on employee creative performance, as well as the mediating role of informal status and the moderating role of Zhongyong thinking. The results of a two-wave questionnaire survey of 202 employees show that boundary-spanning behavior has a significant positive relationship with employees’ creative performance, informal status mediates the link between boundary-spanning behavior and creative performance of this employee, Zhongyong thinking plays a moderating role between employees’ boundary-spanning behavior and their informal status, and Zhongyong thinking also moderates the mediating role of informal status between boundary-spanning behavior and employee creative performance. In this paper, a moderated mediation model is established to enhance the understanding of the effects and mechanisms of individual boundary-spanning behavior, as well as to provide some constructive insight into how boundary-spanning behavior can be effectively employed in management practice within the Chinese context.</t>
@@ -31609,6 +32537,11 @@
       <c r="K685" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P685" t="inlineStr">
+        <is>
+          <t>Measures individual-level boundary spanning behavior (focal employee) with extractable zero-order correlations in a sample of real employees.. Verbatim Evidence: [Procedure and samples] "The research data of the field survey were collected from 6 companies located in Taiyuan, China. These companies involve the internet, landscape architecture, and consulting industries." [Procedure and samples] "In the questionnaire, BSB, meaning of work, team Chaxu climate, and demographic variables were reported by team members, and team leaders evaluated the creative performance of team members. 211 valid samples from 46 teams were finally obtained after deleting invalid questionnaires" [Measures] "Boundary spanning behavior was measured by a 6-item scale adopted by Marrone et al. (2007). A sample item was 'persuade outsiders (e.g., faculty, clients) to support team decisions'." [Results] "Table 2 Means, Standard deviations and Correlation among variables ... n=221 at the individual level, N=46 at the team level"</t>
         </is>
       </c>
     </row>
@@ -32094,7 +33027,7 @@
       </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
+          <t>5 = Multiple reasons (specify in Notes)</t>
         </is>
       </c>
       <c r="G698" t="inlineStr">
@@ -32124,7 +33057,7 @@
       </c>
       <c r="P698" t="inlineStr">
         <is>
-          <t>Team and system-level analysis (N=268 teams, N=44 systems). Verbatim Evidence: [Abstract] The findings of a multimethod study of 44 MTSs composed of 295 teams and 930 members show that as interteam interactions exceed intrateam interactions, team conflict arises and detracts from component team performance. At the system level, a balance between intrateam and interteam interactions enhances system success. [Results] Tables 1 and 2 provide descriptive statistics for and intercorrelations among study variables at the team level and the system level, respectively. [Table 1] Notes: Entries are bivariate correlations. n=268 teams nested within 44 systems.</t>
+          <t>[Code 2 &amp; Code 3]. Verbatim Evidence: Student sample and team-level aggregation. Verbatim Evidence: "[Research Setting] We tested our hypotheses in a multisource and multimethod study of MTSs that were formed as part of the laboratory component of a required undergraduate engineering course at a university on the East Coast of the United States." "[Analyses] Our hypotheses consider relationships at two levels of analysis—the team level and the system level." "[TABLE 1] Notes: Entries are bivariate correlations. n = 268 teams nested within 44 systems."</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_9
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -4075,7 +4075,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Non-primary study (Editorial for a Special Section). Verbatim Evidence: [Page 1] "EDITORIAL Innovating for impact: Harnessing business model innovation to tackle grand challenges" [Abstract] "Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed âABCâ classification and âBMI-GCâ concept." [Introduction] "Our objective with this Special Section is to link our improved conceptual and empirical understanding of business models with the important notion of grand challenges, the urgency of which has become increasingly apparent."</t>
+          <t>Non-primary study (Editorial for a Special Section). Verbatim Evidence: [Page 1] "EDITORIAL Innovating for impact: Harnessing business model innovation to tackle grand challenges" [Abstract] "Research Summary: This Special Section of the Strategic Entrepreneurship Journal explores how business model innovation (BMI) can address grand challenges (GCs), including artificial intelligence (AI), business and global unrest, and climate change through a proposed “ABC” classification and “BMI-GC” concept." [Introduction] "Our objective with this Special Section is to link our improved conceptual and empirical understanding of business models with the important notion of grand challenges, the urgency of which has become increasingly apparent."</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Methodology] "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000)." [Methodology] "More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sourcesâdocumentary data, in-depth interviews, and digital dataâto obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit."</t>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Methodology] "Given that the objective of this study is to develop our understanding of how and why offshoring emerged as an organizational matter, changing the way audit work is organized and perceived in a Big 4 firm, a qualitative research methodology was deemed most appropriate (Cooper and Morgan 2008; Denzin and Lincoln 2003; Flick 2006; Given 2008; Silverman 2000)." [Methodology] "More specifically, we used a case study approach (Cooper and Morgan 2008) drawing upon multiple data sources—documentary data, in-depth interviews, and digital data—to obtain detailed information about the complexities underpinning the real-life phenomenon (Miles and Huberman 1994; Patton 2002) of offshoring in audit."</t>
         </is>
       </c>
     </row>
@@ -5689,11 +5689,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
-        </is>
-      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>While there is a burgeoning trend to recognize leadership as an important enabler of new venture development and growth, scant research has explored the performance mechanisms of shared leadership in the entrepreneurial context. Based on the information processing perspective, we propose a moderated mediation model to examine how shared leadership in entrepreneurial teams advance new venture performance by identifying team reflexivity as a pivotal mediator and team boundary spanning as a crucial contingency. The data set from a cross-industry sample of 94 entrepreneurial teams indicated that shared leadership exerts a positive indirect influence on new venture performance via team reflexivity; and team boundary spanning moderates such indirect influence. Finally, how our findings contribute to the entrepreneurship, leadership, team research, and managerial practice are discussed.</t>
@@ -5721,7 +5717,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>[Code 2 &amp; Code 3] Sample consists of entrepreneurs/founders rather than embedded employees. Furthermore, boundary spanning is measured at the team level ('We' referent) rather than the individual level.. Verbatim Evidence: [Method - Sample] "we randomly identified 200 new ventures from three high-tech industrial parks in eastern China. ... Accordingly, we gathered a list of 163 entrepreneurial teams. ... a total of 417 questionnaires from 102 teams were received, among which 376 questionnaires from 94 teams are valid." [Method - Measurement] "Team boundary spanning was rated by a nine-item scale selected from Yan et al. (2020). These items reflect the degree to which the teams search diverse sources of external information. These items include three dimensions: ambassador activities (e.g., 'We acquire resources for the team'); task coordinator activities (e.g., 'We coordinate activities with external groups'); and scout activities (e.g., 'We scan the environment for marketing ideas/expertise')."</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -6076,6 +6072,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -6507,6 +6504,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Effective work groups engage in external knowledge sharing—the exchange of information, know-how, and feedback with customers, organizational experts, and others outside of the group. This paper argues that the value of external knowledge sharing increases when work groups are more structurally diverse. A structurally diverse work group is one in which the members, by virtue of their different organizational affiliations, roles, or positions, can expose the group to unique sources of knowledge. It is hypothesized that if members of structurally diverse work groups engage in external knowledge sharing, their performance will improve because of this active exchange of knowledge through unique external sources. A field study of 182 work groups in a Fortune 500 telecommunications firm operationalizes structural diversity as member differences in geographic locations, functional assignments, reporting managers, and business units, as indicated by corporate database records. External knowledge sharing was measured with group member surveys and performance was assessed using senior executive ratings. Ordered logit analyses showed that external knowledge sharing was more strongly associated with performance when work groups were more structurally diverse. Implications for theory and practice around the integration of work groups and social networks are addressed.</t>
@@ -6749,6 +6747,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>The aim of this research is to empirically investigate the relationships among the three vital knowledge management processes of acquisition, integration and application, and their effects on organisational innovation in the pharmaceutical manufacturing industry in Jordan; a knowledge-intensive business service (KIBS) sector. Structural equation modelling findings show an excellent fit among all these processes and innovation, with positive and significant relationships. Moreover, knowledge integration and knowledge application emerged as having strong and significant mediation effects upon the relationship between knowledge acquisition and innovation. As such, an organisation’s innovation efforts would significantly benefit from the synergistic effects of properly integrating and applying externally acquired knowledge. The findings make a valuable contribution to pharmaceutical knowledge management and innovation literature, especially in an era of open innovation. Pharmaceutical companies are advised to focus on developing proficient assimilation and application capabilities in order for acquired knowledge to have notable effects on their innovation performance.</t>
@@ -6796,6 +6795,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>The “variance hypothesis” predicts that external search breadth leads to innovation outcomes, but people have limited attention for search and cultivating breadth consumes attention. How does individuals' search breadth affect innovation outcomes? How does individuals' allocation of attention affect the efficacy of search breadth? We matched survey data with complete patent records, to examine the search behaviors of elite boundary spanners at                 IBM                 . Surprisingly, individuals who allocated attention to people inside the firm were more innovative. Individuals with high external search breadth were more innovative only when they allocated more attention to those sources. Our research identifies limits to the “variance hypothesis” and reveals two successful approaches to innovation search: “cosmopolitans” who cultivate and attend to external people and “locals” who draw upon internal people                              . © 2014 The Authors.               Strategic Management Journal               published by John Wiley &amp; Sons Ltd.</t>
@@ -6843,6 +6843,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -7320,6 +7321,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -8113,7 +8115,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 2] Laboratory experiment using a student sample (business school undergraduates) and reporting no zero-order correlation matrix.. Verbatim Evidence: [Manipulations] "The research was conducted using a full-factorial experimental design, resulting in 16 (4 Ã 2 Ã 2) treatments." [Manipulations] "Fifteen subjects (upper division business school undergraduates) were in each treatment."</t>
+          <t>[Code 1 &amp; Code 2] Laboratory experiment using a student sample (business school undergraduates) and reporting no zero-order correlation matrix.. Verbatim Evidence: [Manipulations] "The research was conducted using a full-factorial experimental design, resulting in 16 (4 × 2 × 2) treatments." [Manipulations] "Fifteen subjects (upper division business school undergraduates) were in each treatment."</t>
         </is>
       </c>
     </row>
@@ -8477,7 +8479,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>Firm-level analysis / Proxy informants rating firm inter-organizational partnerships and intra-firm project integration. Verbatim Evidence: [Methodology] "The ï¬nal sampling frame of the study consisted of 731 ï¬rms." [Methodology] "The study targeted two key informants for each ï¬rm to reduce the threat of common method variance" [Methodology] "The overall number of usable responses was 202 complete cases or approximately 27% response rate." [Measures] "âWhat is the approximate working hour overlap between your company and the foreign company?" [Measures] "âJointly discuss customer's requirements at the beginning of the project."</t>
+          <t>Firm-level analysis / Proxy informants rating firm inter-organizational partnerships and intra-firm project integration. Verbatim Evidence: [Methodology] "The ﬁnal sampling frame of the study consisted of 731 ﬁrms." [Methodology] "The study targeted two key informants for each ﬁrm to reduce the threat of common method variance" [Methodology] "The overall number of usable responses was 202 complete cases or approximately 27% response rate." [Measures] "–What is the approximate working hour overlap between your company and the foreign company?" [Measures] "–Jointly discuss customer's requirements at the beginning of the project."</t>
         </is>
       </c>
     </row>
@@ -8633,7 +8635,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>Systematic literature review, no primary effect sizes.. Verbatim Evidence: [Abstract] This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in businessâtoâbusiness (B2B) interorganizational relationships, pointing out directions for future research. [Methodology] A systematic literature review allows the synthesizing of results and evidence from existing studies and producing new knowledge.</t>
+          <t>Systematic literature review, no primary effect sizes.. Verbatim Evidence: [Abstract] This paper consists of a literature review analyzing, consolidating, and synthesizing studies on boundary spanners in business–to–business (B2B) interorganizational relationships, pointing out directions for future research. [Methodology] A systematic literature review allows the synthesizing of results and evidence from existing studies and producing new knowledge.</t>
         </is>
       </c>
     </row>
@@ -9101,7 +9103,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>Qualitative ethnographic case study lacking an extractable quantitative effect size or correlation matrix.. Verbatim Evidence: [Abstract] "Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the companyâs transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities." [Methodological aspects: Embedded in a utility] "To flesh out the reorganisation of a municipal utility and better capture the âsocio-technical geometry of powers in townâ (Graham and Marvin, 2001), I decided to immerse myself directly in this technical world by being embedded within the teams of infrastructure management of a German multi-utility."</t>
+          <t>Qualitative ethnographic case study lacking an extractable quantitative effect size or correlation matrix.. Verbatim Evidence: [Abstract] "Based on a detailed analysis of a traditional German local multi-utility and informed by a six-month internship within the company, the article deciphers the rationale of multi-sectoral practices, in particular the company’s transformation into a cross-utility that devised a common strategy for all its infrastructure networks and its ambiguities." [Methodological aspects: Embedded in a utility] "To flesh out the reorganisation of a municipal utility and better capture the ‘socio-technical geometry of powers in town’ (Graham and Marvin, 2001), I decided to immerse myself directly in this technical world by being embedded within the teams of infrastructure management of a German multi-utility."</t>
         </is>
       </c>
     </row>
@@ -9381,6 +9383,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Self-initiated expatriates (SIEs) who work for a subsidiary of a multinational enterprise from their country of origin and hence are familiar with both countries’ language and culture can be expected to act as boundary-spanners between the assigned expatriates sent from the parent country and host country nationals, and between the headquarters and the subsidiary. We develop a new model of boundary-spanning that encompasses both individual and organizational antecedents and validate the model using survey data from Japanese-affiliated companies in China. We find that familiarity with Chinese language and culture and the potential dual allegiance of SIEs contribute to enhancing their boundary-spanning behavior. We also find that relationships of trust among the parties concerned (social capital) and global career opportunities for such self-initiated expatriates (geocentric staffing) have positive influences on their dual allegiance. Finally, normative and systems integration of human resource management are associated with increasing levels of social capital and geocentric staffing.</t>
@@ -9973,6 +9976,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -10020,6 +10024,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -10494,6 +10499,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>This article explores the joint production and consumption of health information and advice in the context of NHS Direct, the new telephone health information and advice service. NHS Direct is an atypical call centre environment in so far as its core staff (nurses) are highly skilled professionals. These nurses are required to collaborate closely with, and are to some extent dependent upon, non-professional lower skilled staff (call handlers) to deﬁne and prioritize their work. This introduces a number of tensions between the two groups. Nurses respond to these tensions by engaging in ‘boundary work’, the micropolitical strategies through which work identities and occupational margins are negotiated, to protect their own status. Call handlers are more subject to the pressures of work ‘speed-up’, highly aware of the risks inherent in their role, but are unable to call upon professional status, either in their resistance to managerial imperatives or in their interactions with health consumers. They are required to manage the tension between offering a safe and high quality service, characterized in their training as ‘professional’, and nurses’ boundary work, which positions them as ‘non-professional’. Here we draw on qualitative research, including call interaction data between call handler and consumer, to show how call handlers’ occupation of the contested territory between professional and non-professional status leaves them wide open to the agency of consumers, as consumers attempt to shape the service in their own interests.</t>
@@ -10704,6 +10710,12 @@
           <t>BSMA0194</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
           <t>Firms recognize that working together through collaborative relationships offers potential benefits such as improving cooperation, information sharing, and overall performance. An additional and extremely valuable benefit of working together is the potential for creating innovative business approaches and solutions. Thus, developing external linkages has become a higher priority within many organizations. Boundary spanning employees offer one means of achieving closer cross‐firm relationships. We investigate the roles of boundary spanners by examining service providers and their relationships with customers. More specifically, we examine boundary spanning employees that are physically on‐site at customer facilities. Results provide strong support that boundary spanners perceiving higher levels of external organizational support from a client subsequently develop affective commitment to the customer. This, in turn, drives knowledge exchange and logistics innovation. A relationship between logistics innovation and performance (of service providers and of customers) was also found. Managerial implications of the research findings are discussed and suggestions presented covering future research.</t>
@@ -10727,6 +10739,11 @@
       <c r="K197" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -11150,6 +11167,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>As software development projects continue to be over budget and behind schedule, researchers continue to look for ways to improve the likelihood of project success. In this research we juxtapose two different views of what influences software development team performance during the requirements development phase. In an examination of 66 teams from 15 companies we found that team skill, managerial involvement, and little variance in team experience enable more effective team processes than do software development tools and methods. Further, we found that development teams exhibit both positive and negative boundary-spanning behaviors. Team members promote and champion their projects to the outside environment, which is considered valuable by project stakeholders. They also, however, guard themselves from their environments; keeping important information a secret from stakeholders negatively predicts performance.</t>
@@ -11197,6 +11215,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>This study examines the influence of the social network of board interlocks on strategic alliance formation. Our theoretical framework suggests how board interlock ties to other firms can increase or decrease the likelihood of alliance formation, depending on the content of relationships between CEOs (chief executive officers) and outside directors. Results suggest that CEO-board relationships characterized by independent board control reduce the likelihood of alliance formation by prompting distrust between corporate leaders, while CEO-board cooperation in strategic decision making appears to promote alliance formation by enhancing trust. The findings also show how the effects of direct interlock ties are amplified further by third-party network ties.</t>
@@ -11499,6 +11518,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>SUMMARY             Previous research has focused on purchasing managers’ experience with role stressors and the negative effect of stress on job attitudes and performance. The potential benefits of having multiple responsibilities and a diverse role set have been overlooked. This study explored the relationship between purchasing managers’ involvement in multiple boundary spanning roles and their perceptions of positive social outcomes related to work. The relationship of these social benefits to job satisfaction was also evaluated. The relationships were analyzed using structural equation modeling. The results indicated positive relationships between each variable in the model. The implications for recruitment, supervision, and job design are discussed.</t>
@@ -12803,6 +12823,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>While there is a growing interest in the role of market information processing activities (i.e., the acquisition, dissemination, and use of market information) in new product development (NPD), a number of gaps remain in our knowledge on this topic. When investigating the performance impact of market information processing, most studies have treated the three activities as independent. Our research adds to the extant knowledge by exploring not only both direct relationships between each of the market information processing activities and new product performance, but also interaction effects. We, thus, ask the question of whether there may be synergies in obtaining performance increases by jointly improving two processing activities, rather than just considering each activity independently. In addition, we investigate these effects for different levels of information quality; a topic largely neglected in the market information processing literature. Our analysis is based on empirical data from 152 Dutch NPD projects. The results indicate that market information acquisition and use are both directly associated with increased performance. We also ﬁnd signiﬁcant interaction effects for information acquisition and dissemination, and for information dissemination and use. Finally, the importance of information quality is emphasized, with lower quality information producing lower performance and wiping out the effects between various aspects of market information processing and new product performance. We provide several implications of our ﬁndings for managers and academics.</t>
@@ -12850,6 +12871,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>Background: Rehabilitation services depend on competent professionals who collaborate effectively. Wellfunctioning interprofessional teams are expected to positively impact continuity of care. Key factors in continuity of care are communication and collaboration among health care professionals in a team and their patients. This study assessed the associations between team functioning and patient-reported benefits and continuity of care in somatic rehabilitation centres. Methods: This prospective cohort study uses survey data from 984 patients and from health care professionals in 15 teams in seven somatic rehabilitation centres in Western Norway. Linear mixed effect models were used to investigate associations between the interprofessional team communication and relationship scores (measured by the Relational Coordination [RC] Survey and patient-reported benefit and personal-, team- and cross-boundary continuity of care. Patient-reported continuity of care was measured using the Norwegian version of the Nijmegen Continuity Questionnaire. Results: The mean communication score for healthcare teams was 3.9 (standard deviation [SD] = 0.63, 95% confidence interval [CI] = 3.78, 4.00), and the mean relationship score was 4.1 (SD = 0.56, 95% CI = 3.97, 4.18). Communication scores in rehabilitation teams varied from 3.4–4.3 and relationship scores from 3.6–4.5. Patients treated by teams with higher relationship scores experienced better continuity between health care professionals in the team at the rehabilitation centre (b = 0.36, 95% CI = 0.05, 0.68; p = 0.024). There was a positive association between RC communication in the team the patient was treated by and patient-reported activities of daily living benefit score; all other associations between RC scores and rehabilitation benefit scores were not significant. Conclusion: Team function is associated with better patient-reported continuity of care and higher ADL-benefit scores among patients after rehabilitation. These findings indicate that interprofessional teams’ RC scores may predict rehabilitation outcomes, but further studies are needed before RC scores can be used as a quality indicator in somatic rehabilitation.</t>
@@ -13095,6 +13117,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>The study examines the effects of the individual characteristics, job type, role stressors, boundary spanning activities, career outcomes, and job characteristics on the turnover propensity of 464 information systems personnel. Results show that age, organizational level, organizational tenure, job tenure, and number of years in the computer field are negatively correlated with the intention to leave the organization. Education was found to be positively correlated with turnover intentions, and while project leaders are more likely to leave the organization, IS managers are less likely. Results also show that both role stressors (role ambiguity and role conflict) and boundary spanning activities are positively correlated with turnover intentions, and that job involvement, career plateau, promotability, salary, organizational commitment, job satisfaction, satisfaction with progress, promotion, pay, status, and projects are negatively correlated while career opportunity is positively correlated with turnover intentions. Finally, all job characteristics are negatively correlated with turnover intentions. Implications of the results for practice and research are offered.</t>
@@ -13284,6 +13307,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>In this article the authors discuss research they conducted that examined the relationship between task difficulty and the extent of boundary-spanning activity within an organization. The authors believed that they greater degree of interunit interdependence that existed in an organization would result in a greater amount of boundary-spanning activity by that organization's members. They also believed that the greater degree of task difficulty in a given situation would also result in a greater amount of boundary-spanning activity by members. The authors hoped to examine the relationships that exist between organizational structure and the amount of intergroup activity fostered by those structures.</t>
@@ -13378,6 +13402,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>Marketing boundary spanners—especially customer service representatives—are notably susceptible to burnout. The authors define the burnout construct and develop hypotheses to examine if burnout acts as a partial mediator between role stressors and key behavioral and psychological job outcomes. Responses from 377 customer service representatives reveal that burnout levels are high relative to other burnout-prone occupations (e.g., police, nursing) and that burnout has consistent, significant, and dysfunctional effects on their behavioral and psychological outcomes. Moreover, burnout mediates the negative effects of role stressors on job outcomes, whereas the positive effects of role stressors are unmediated.</t>
@@ -13614,6 +13639,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -13851,6 +13877,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>International joint ventures (IJVs) have become an important source of critical knowledge for multinational enterprises, but little is known about how knowledge can be effectively transferred to parent ﬁrms when the potential for interpartner opportunism still exists. Drawing on attachment theory, we study how boundary-spanning commitments to IJVs may help mitigate interpartner opportunism and facilitate effective knowledge transfer to parents. Speciﬁcally, we argue that knowledge transfer from IJVs to their parents is positively mediated by both boundary spanners’ organizational commitment to IJVs and parent ﬁrms’ resource commitment to IJVs. We test our arguments using survey data collected from 600 dyadic Chinese–foreign managers of 100 IJVs established in China. The results provide evidence that knowledge sharing between boundary spanners in IJVs positively affects their organizational commitment to these IJVs, which in turn positively affects knowledge transfer to parents. Similarly, knowledge sharing between such boundary spanners positively affects parent ﬁrms’ resource commitment to IJVs, which in turn positively affects knowledge transfer to parents. The mediating role of boundary spanners’ organizational commitment is stronger than that of parent ﬁrms’ resource commitment. Collectively, our ﬁndings suggest that commitment-based relational mechanisms are imperative for safeguarding effective knowledge transfer from IJVs to parent ﬁrms.</t>
@@ -14091,6 +14118,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>This study examines the antecedents of job satisfaction, commitment and turnover for 229 information systems development personnel (ISDP) employed by nine companies within several industries. The antecedents studied include boundary spanning, role ambiguity and role conflict. A model of these variables is built and tested via path analysis. A secondary analysis is performed to explore the impacts of task and individual differences on the study variables. The task differences include analytic and programming tasks while the individual differences studied are age, tenure, education and years of data processing experience.</t>
@@ -14232,6 +14260,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate a boundary spanning, interprofessional collaboration between advanced practice nurses (APNs) and junior doctors to support junior doctors’ learning and improve patient management during the overtime shift.</t>
@@ -14468,6 +14497,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>While the introduction of a new product or service carries considerable risk, incorporating customer input into the new product/service development (NPD) process increases the probability of commercial success. In their boundary spanning role, industrial (B-to-B) salespeople are well suited to serve as a conduit between customers and those inside their company who are largely responsible for the NPD process. The current study investigates the perceptions of sales managers and examines the role the sales force may play in the early stages of the NPD process. An empirical analysis is conducted to determine whether differences exist between organizations that employ key account management (KAM) systems and those that do not employ KAM systems. The findings of this study suggest that salespeople from KAM organizations are better suited to provide input into the NPD process than their non-KAM counterparts.</t>
@@ -14510,6 +14540,12 @@
           <t>BSMA0276</t>
         </is>
       </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
           <t>We examine how two highly successful new biotechnology firms (NBFs) source their most critical input—scientific knowledge. We find that scientists at the two NBFs enter into large numbers of collaborative research efforts with scientists at other organizations, especially universities. Formal market contracts are rarely used to govern these exchanges of scientific knowledge. Our findings suggest that the use of boundary-spanning social networks by the two NBFs increases both their learning and their flexibility in ways that would not be possible within a self-contained hierarchical organization.</t>
@@ -14533,6 +14569,11 @@
       <c r="K279" t="inlineStr">
         <is>
           <t>1996</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -14552,6 +14593,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to evaluate the recognition of sexual harassment (SH); to describe the relationships among SH, employees’ burnout, customer-oriented boundary-spanning behaviors (COBSB); and to verify the moderating effect of employees’ psychological safety (PS), all within deluxe hotels in South Korea.</t>
@@ -14706,6 +14748,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries. Not only must this structure be clearly defined, but it also must account for the integration of a broad range of cross-government activities. Like the overarching performance network, the cross-boundary structure has the characteristics of a dynamic system, including flexibility, adaptability, growth, and the continual emergence of new forms and functions. Summer 2000 featured perfect conditions for gridlock in the sky. Flying had become an increasingly popular way to travel, and the airlines had marketed aggressively to vacationing families and business travelers. Airports were already crowded when unusual and frequent patterns of bad weather hit aviation especially hard. Delays and canceled flights became almost daily events. The public complained loudly, congressional hearings were scheduled, and the Federal Aviation Administration was about to experience unfriendly fire from an aroused media.</t>
@@ -14843,6 +14886,16 @@
           <t>BSMA0283</t>
         </is>
       </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G286" t="inlineStr">
         <is>
           <t>Purpose – Despite the increasing importance of boundary-spanning behaviors in construction projects, the research on how leader anger expressions impact employees’ boundary-spanning behaviors remains unclear. This study aims to investigate the impact of leader anger expressions on employees’ boundaryspanning behaviors in construction projects while exploring the mediating effect of work hope and the moderating effect of power distance orientation through the lens of social information processing theory. Design/methodology/approach – The empirical data were collected from a questionnaire survey of 235 employees in construction projects, and the hypotheses were tested using the PROCESS program developed by Hayes.</t>
@@ -14866,6 +14919,11 @@
       <c r="K286" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>Study measures individual employee boundary-spanning behavior in a sample of 235 construction project employees and provides a zero-order correlation matrix.. Verbatim Evidence: [Abstract] "The empirical data were collected from a questionnaire survey of 235 employees in construction projects, and the hypotheses were tested using the PROCESS program developed by Hayes." [Sampling and data collection] "The sample involved employees working on construction projects in China, selected from the author’s extensive alumni network in the construction industry." [Measurement] "Boundary-spanning behaviors were assessed using a six-item scale developed by Marrone et al. (2007). One sample item is 'I will endeavor to convince external stakeholders, such as faculty and clients, to support project decisions'." [Results] "Table 2 shows a descriptive analysis of all variables and their bivariate correlations."</t>
         </is>
       </c>
     </row>
@@ -14937,6 +14995,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>The purpose of this paper is to develop the concept of project management system from the perspective of systems science. There is a need to extend the body of knowledge for project management. In particular, the application of systems perspectives and systems theory offers a significant opportunity to advance the current state of project management knowledge. Although there have been suggestions of systems approaches for project management, rigorous systems science has not been used to support these depictions. First, we develop the background and define a perspective of project management systems. Second, assumptions and principles are drawn from systems science to provide a foundation for project management systems. Third, a model for project management systems is developed from systems sciences and management cybernetics. Our initial explorations are promising, demonstrated by a case study application review using a complex system of systems (SoS) project encompassed multiple government agencies, and we offer future directions and implications for further model refinements, applications, and research into project management systems.</t>
@@ -14984,6 +15043,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G289" t="inlineStr">
         <is>
           <t>Smart cities emphasize the use of advanced technology to deliver better services to and improve the well-being of their residents. Since the administrative authorities that manage cities often lack the knowledge and skills needed to transform their operations in this way, smart city initiatives usually involve a complex set of actors, from local urban authorities and their technical departments to small and large IT firms, academics, and civic organizations, as well as individual citizens. Mediating organizations are often set up to coordinate and manage such interactions. However, little is known about the roles and activities of such bodies. Using data from the Dublin smart city projects, this study draws on the concept of boundary spanning to develop a taxonomy of the work of such intermediaries. Divided into technical, political, social, and cultural domains, the study demonstrates the critical role of the work done by such bodies in enhancing collaboration among and the participation of a diverse group of citizens, IT and digital strategy departments of local authorities, universities and local/international IT companies (e.g., Google, Facebook or Airbnb), leading to a bottom-up governance style of leading smart city initiatives and projects.</t>
@@ -15011,7 +15075,7 @@
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Qualitative single-case study with no quantitative effect sizes, analyzing a boundary-spanning organization rather than individual employees.. Verbatim Evidence: [Methodology] "A single-case design for this study offers a unique opportunity to produce concrete, context-dependent knowledge in depth and in its particular type of setting (e.g., process, mechanism, or practice) (Flyvbjerg, 2006; Small, 2009; Yin, 2013)." [Data collection] "Semi-structured interviews were identified as the primary data collection method for this study and twenty-five interviews were conducted." [Conclusions, limitations, and future research] "This study examined the experiences of a boundary-spanning organization set up as part of a city's drive to offer smart services to its residents."</t>
         </is>
       </c>
     </row>
@@ -15078,6 +15142,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G291" t="inlineStr">
         <is>
           <t>This study investigates the role of gatekeepers in the transfer of information within a single R &amp; D location by comparing directly t h e performance of project groups with and without gatekeepers. The results show that gatekeepers performed a linking role only for projects performing tasks that were 'locally-oriented' while 'universallyoriented' tasks were most effectively linked to external areas by direct project member communication. Gatekeepers also appear to facilitate external communication by their locallyoriented project colleagues. A follow-up study five years later showed that almost all gatekeeping project leaders had been promoted up the managerial ladder; in contrast, one half of the non-gatekeeping project leaders had ascended the technical ladder. This implies that higher managerial levels demand strong interpersonal a s well a s technical skills.</t>
@@ -15105,7 +15174,7 @@
       </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level analysis (N = projects). Individual communication scores were aggregated to the project level.. Verbatim Evidence: [Non-individual level (team/project analysis)]. Verbatim Evidence: "[Communication] As discussed by Katz &amp; Tushman (1979), these individual scores were also aggregated to obtain project measures of internal and external communication." "[Table 2] Table 2. Correlations between project performance and external communication by project type and gatekeeper presence"</t>
         </is>
       </c>
     </row>
@@ -15125,6 +15194,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>This study examines the impacts of problem-solving and administrative communication patterns on the technical performance of 61 projects in an industrial R&amp;D laboratory. While there were no differences in the relative patterns of these two types of communication, there were systematic differences in the mechanisms by which project groups transferred administrative and problem-solving information with other areas both within and outside the organization. The overall patterns of communication were influenced by the nature of the projects' work, while the effectiveness of the various interfaces was explored via two contrasting methods: (1) direct contact by all project members and (2) contact mediated through boundary spanning individuals. The effectiveness of each of these linking mechanisms was also contingent upon the projects' tasks. This research reinforces the importance of managing communication patterns in organizations and further supports the importance of boundary spanning individuals.</t>
@@ -15290,7 +15360,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>Boundary -spanning activity (BSA) was studied in two departments of a large governmental research and develop ment organization. BSA was found to be higher and to have significant effects for employees when departmental goals were unclear and technology was non-routine. Under these conditions, BSA was negatively related to role ambiguity and positively related to job satisfaction. Contrary to prior re search, this study found roles with high levels of BSA to have favorable aspects for their incumbents depending upon gorl clarity and type of technology of the parent organization. Implications for the management of research and development organizations are discussed.</t>
@@ -15390,6 +15459,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -15417,7 +15491,7 @@
       </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Qualitative field study without quantitative effect sizes (r) or a correlation matrix.. Verbatim Evidence: [Research Methods] "Our field study focused on the everyday project-based practices of members in one of Adweb’s larger offices (110 employees), and was conducted over five months in 2001. Our data collection was exploratory in nature and included interviewing, observation, and review of documents and websites." [Research Methods] "We used inductive, qualitative techniques to analyze the data (Agar 1980, Eisenhardt 1989, Glaser and Strauss 1967, Strauss and Corbin 1990), informed by our focus on practices, technology use, and consequences, while remaining alert to emerging ideas."</t>
         </is>
       </c>
     </row>
@@ -15523,12 +15597,12 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -15558,7 +15632,7 @@
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Valid self-rated individual-level BSB by middle/senior managers representing their firms (matches the CEO vs Firm Exception) with zero-order correlations provided.. Verbatim Evidence: [Sample and procedure] Participants were drawn from the alumni network of a major public university in China. These individuals, occupying middle and senior management roles, were considered well-positioned to provide informed insights into their firms’ leadership behaviors, digital practices, and export strategies. [Measures] LBSB was gauged by adapting a 6-item scale (α = 0.88) from Marrone et al. (2007). An example item is 'I reach out to individuals outside of our organization who can offer expertise or ideas about the task at hand.' [Measures] We measured EL with 8 items (α = 0.92) (Renko et al., 2015). An example item is 'I often come up with radical improvement ideas for the products/services we are selling.'</t>
         </is>
       </c>
     </row>
@@ -15625,6 +15699,12 @@
           <t>BSMA0299</t>
         </is>
       </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts [1]. Thus, OB spans para-organizational concerns such as interorganizational networks and delivery systems. It deals with macro-organizational phenomena-organizational goals, strategies, climates, cultures, structure, management styles, and performances-and how they are shaped by one another and by such contextual factors as operating environments, societal values and institutions, technology, size, dependence, and other</t>
@@ -15648,6 +15728,11 @@
       <c r="K302" t="inlineStr">
         <is>
           <t>1988</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15699,7 +15784,7 @@
       </c>
       <c r="P303" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level analysis where individual responses were aggregated to N=20 teams.. Verbatim Evidence: [Participants and procedure] "Respondents belonged to 20 teams." [Independent measures] "Team level scores for the external activities were acquired by averaging individual members' sum-scores for each team and dividing the score by number of items." [Results] "As the sample size was small (N = 20), it was necessary to combine independent variables into composites to avoid the risk of an overfit model."</t>
         </is>
       </c>
     </row>
@@ -15714,6 +15799,12 @@
           <t>BSMA0301</t>
         </is>
       </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate how frontline service employees’ (FSEs) perceptions of corporate social responsibility (CSR) can enhance meaningful work perceptions as well as help alleviate FSEs’ perceptions of verbal dysfunctional customer behavior.</t>
@@ -15737,6 +15828,11 @@
       <c r="K304" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15751,6 +15847,16 @@
           <t>BSMA0302</t>
         </is>
       </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G305" t="inlineStr">
         <is>
           <t>Leaders' positions as external brokers in organizational networks—those acting as a bridge between individuals outside the boundaries of their team—can enhance or constrain their effectiveness. Yet, whereas extant research on network brokerage views it as a private good whose benefits accrue directly to the broker, recent research suggests brokering between external communities can serve as both a public good as well as a public liability that can spillover to team members. We integrate network leadership theory with the externalities of network brokerage perspective to examine the countervailing effects of leaders' external brokerage in an information network with peer leaders and executives on team performance. In a sample of 465 team members in 80 teams distributed across 10 sister companies within one conglomerate, we used multilevel structural equation modeling to test our hypotheses. On one hand, we found that leader external brokerage was positively associated with team performance through team members' perceptions of organizational support; on the other hand, we found that leader brokerage is detrimental to team performance by compromising leaders' commitment to their teams. Our results suggest that, while leaders are encouraged to forge connections outside their team to harvest social capital benefits, there are both public benefits and liabilities of team leaders' external networks that can impact team performance.</t>
@@ -15774,6 +15880,11 @@
       <c r="K305" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>Included. The study uses a real employee sample and measures individual-level leader boundary spanning behavior via intra-organizational network brokerage. Zero-order correlations are provided.. Verbatim Evidence: [Participants and procedure] "We collected data from a small-sized industrial conglomerate in South Korea comprising 10 sister companies in a variety of industries, including chemistry, construction, IT, investment, and biotechnology." [Participants and procedure] "Thus, there were 44 executives, 80 teams (ranging from 2 to 10 members), and 465 members in the final sample, and all constructs in our hypothesized framework were modeled at the team level of analysis." [Leader brokerage in external information network] "Specifically, team leaders and executives were first asked to list peer leaders and executives (within their organizational subunit and in the larger conglomerate) from whom they “seek work-related advice and information.”" [Leader brokerage in external information network] "To assess leader brokerage, we computed Gould and Fernandez's (1989) total brokerage metric in UCINET 6 (Borgatti et al., 2002)." [Leader brokerage in external information network] "The total brokerage routine generated brokerage scores for each of the 124 leaders and executives in the information network; we then extracted the scores for the 80 team leaders in our core sample, which we modeled as our independent variable."</t>
         </is>
       </c>
     </row>
@@ -15788,6 +15899,12 @@
           <t>BSMA0303</t>
         </is>
       </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
           <t>Purpose – The research aims to examine the impacts of two different types of goal orientation, i.e. leaning goal orientation (LGO) and performance-prove goal orientation (PPGO), on employee knowledge sharing, and whether these relationships are altered by leaders’ boundary spanning behavior (BSB).</t>
@@ -15811,6 +15928,11 @@
       <c r="K306" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -15877,6 +15999,16 @@
           <t>BSMA0305</t>
         </is>
       </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G308" t="inlineStr">
         <is>
           <t>Purpose – Drawing on conservation of resources (COR) theory, this research aims to advance the current understanding of leader boundary spanning by examining its effect on task performance, psychological mechanism and boundary conditions.</t>
@@ -15900,6 +16032,11 @@
       <c r="K308" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>Included. The study examines Leader Boundary Spanning measured by subordinates using a standard purposive BSB scale (Marrone et al., 2007). Zero-order correlations are provided for an individual-level employee sample (N=155 dyads). This triggers the mandatory inclusion override for Leader BSB (Rule 16).. Verbatim Evidence: [Sample and procedure] "We collected survey data in South Korea. To secure field data, one author reached out to both leaders and employees through professional networks available to us. We explained the nature of the study, which required leaders and employees to participate together with their respective subordinates or supervisors, and provided them with a survey packet containing detailed information." [Measures] "Leader boundary spanning. Leader boundary spanning was evaluated using the 6-item measure developed by Marrone et al. (2007). The sample item is 'My supervisor acquires resources and access (e.g. access to information) for the team' (α = 0.94)."</t>
         </is>
       </c>
     </row>
@@ -16155,6 +16292,16 @@
           <t>BSMA0312</t>
         </is>
       </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G315" t="inlineStr">
         <is>
           <t>As much as prior research has shed light on the boundary-spanning processes of global organizations and their (positive) impact on an MNC’s performance, whether, when and how past performance ultimately shapes an MNC’s boundary-spanning activities remains an open question in management research. To tackle these questions, we examine the behaviour of technology scouts in global organizations who span organizational and national boundaries to tap into novel knowledge and span internal boundaries to present this knowledge to constituents inside the MNC. Drawing on the behavioural theory of the ﬁrm, we propose that the intensity of organizational boundary spanning, the likelihood of spanning national boundaries and the way technology scouts span internal boundaries to engage with members inside the organization are sensitive to how the MNC has performed relative to its aspirations. We support our theoretical expositions with insights gained from interviewing senior industry professionals with direct experience in technology scouting in MNCs.</t>
@@ -16178,6 +16325,11 @@
       <c r="K315" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>Qualitative and theoretical study lacking quantitative effect sizes or a correlation matrix.. Verbatim Evidence: [ABSTRACT] &lt;We support our theoretical expositions with insights gained from interviewing senior industry professionals with direct experience in technology scouting in MNCs.&gt; [THEORY] &lt;Specifically, between 2011–15, we conducted 15 in-depth interviews with managers in European and North American MNCs (including Bayer, Johnson &amp; Johnson, Merck &amp; Co, and Novo Nordisk) on the MNCs’ sites, at technology conferences such as the Wharton Mack Institute’s Technology Conference or via phone.&gt;</t>
         </is>
       </c>
     </row>
@@ -16229,6 +16381,16 @@
           <t>BSMA0314</t>
         </is>
       </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G317" t="inlineStr">
         <is>
           <t>Entrepreneurial teams often struggle with simultaneous task and team challenges at an early stage of new venture creation. The way in which teams shape their teamwork is key in leveraging performance in the pre‐founding phase. Learning should help the team in establishing good teamwork and in expanding its members’ entrepreneurial capabilities. Leadership is needed to facilitate and guide this learning. Accordingly, we investigated learning and leadership as facilitators of performance in the pre‐founding phase. Specifically, we examined team reflexivity as a collective internal learning process and boundary spanning behaviour as an externally directed individual activity, operating at different levels in fostering team and individual performance. Charismatic team leadership was examined as a catalyst of learning, shaping team and individual performance ultimately. The multilevel mediation model was tested based on data from 196 members of 58 teams of a venture creation programme. Team reflexivity predicted team and individual performance. Boundary spanning behaviour was not related to performance. As hypothesised, charismatic team leadership predicted team and individual performance, both mediated by team reflexivity. This research highlights the relevance of team learning in pre‐founding teams and emphasises leadership in shaping learning and moving new ventures forward.</t>
@@ -16252,6 +16414,11 @@
       <c r="K317" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>[Code 2 &amp; Code 3] Excluded because it uses a non-employee sample of nascent entrepreneurs (pre-founding teams in an education program) and the correlation matrix is aggregated to the team level (N=58).. Verbatim Evidence: [Sample and Procedure] "We studied teams who participated in a venture creation programme that combines education and incubation (Lackéus &amp; Williams Middleton, 2015), which often results in nascent behaviour (Bae, Qian, Miao, &amp; Fiet, 2014; Martin, McNally, &amp; Kay, 2013)." [Sample and Procedure] "The final sample included 196 participants in 58 teams of three to five members (41.4% with three and 53.4% with four members)." [Table 1] "TABLE 1 Descriptives and Intercorrelations of Study Variables on the Team Level" [Table 1] "Note: N = 58 teams. Age of the team leader was available for N = 55 teams only. Gender: 0 = male, 1 = female. Correlations are given using pairwise exclusion. Individual-level variables were aggregated to the team level."</t>
         </is>
       </c>
     </row>
@@ -16266,6 +16433,16 @@
           <t>BSMA0315</t>
         </is>
       </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G318" t="inlineStr">
         <is>
           <t>The omnichannel varies across countries due to different retail environments and retailers’ growth strategies. The Japanese big retailers’ omnichannel can be characterized by having multiple retail formats, such as department stores, general merchandise stores, convenience stores, specialty stores, Internet stores, and so on. They have grown by multiplying retail formats to appeal to different customer segments, and they have unique challenges in managing an omnichannel with many retail formats. These are (1) extremely wide variety of merchandise, (2) enormous quantity of data from transaction, inventory, logistics, and customers, (3) different organization structures and management, and (4) unique organizational capabilities in each retail format. From these challenges, we could propose further research issues as follows: (1) theoretical consideration of boundary-spanning functions among retail formats, (2) international comparative analysis reflecting the different conditions in each country, and (3) clarifying the characteristics of the omnichannel shopper in the Japanese omnichannel environment.</t>
@@ -16289,6 +16466,11 @@
       <c r="K318" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>This is a conceptual research note proposing future theoretical research directions for omnichannel management in Japan. It does not contain primary empirical data or report quantitative effect sizes.. Verbatim Evidence: [Abstract] "From these challenges, we could propose further research issues as follows: (1) theoretical consideration of boundary-spanning functions among retail formats, (2) international comparative analysis reflecting the different conditions in each country, and (3) clarifying the characteristics of the omnichannel shopper in the Japanese omnichannel environment." [Further research] "We propose several further research issues from the discussion so far." [Further research] "What is critical is boundary spanning across the retail formats to smoothly implement its omnichannel strategy. So, it is important to theoretically consider boundary spanning functions in Japanese omnichannel retailing."</t>
         </is>
       </c>
     </row>
@@ -16303,6 +16485,16 @@
           <t>BSMA0316</t>
         </is>
       </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G319" t="inlineStr">
         <is>
           <t>This article makes a further contribution to opening the ‘black box’ of micropractices in ministry–agency relationships. We argue that the mechanisms that come into play in the course of institutionalizing agencification reforms – such as renegotiating mutual roles and rules in ministry–agency interactions – are only poorly covered in the existing literature. To adequately address the negotiated and contingent nature of de facto agency autonomy and political control, we develop an interpretive approach based on the concept of ‘boundary work’. The empirical focus is on ministry–agency interactions at the science–policy nexus in the contested policy field of food safety. By studying actors' stories about the institutionalization processes following the fundamental reorganization of the German food safety administration in the wake of the               BSE               crisis from a longitudinal perspective, we show how actors manage boundary conflicts via increasingly differentiated backstage coordination.</t>
@@ -16326,6 +16518,11 @@
       <c r="K319" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Qualitative study lacking extractable quantitative effect sizes.. Verbatim Evidence: [Introduction] "Methodically, we draw on narrative data from semi-structured, personal expert interviews conducted with various members of the organizations involved." [Abstract] "By studying actors' stories about the institutionalization processes following the fundamental reorganization of the German food safety administration in the wake of the BSE crisis from a longitudinal perspective, we show how actors manage boundary conflicts via increasingly differentiated backstage coordination."</t>
         </is>
       </c>
     </row>
@@ -16434,6 +16631,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G322" t="inlineStr">
         <is>
           <t>Purpose – This study investigates the relationship between buyer-supplier top management team (TMT) demographic misalignment (defined as differences in TMT composition based on background, age and gender) and environmental performance (EVP).</t>
@@ -16461,7 +16663,7 @@
       </c>
       <c r="P322" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1, Code 2 &amp; Code 3] The study uses secondary firm-level databases (Compustat, Bloomberg, KLD) to analyze buyer-supplier dyads (N=7,493 dyad-year observations), measuring TMT demographic misalignment rather than individual boundary spanning behavior.. Verbatim Evidence: [Abstract] "The study employs panel data regression methods on an unbalanced panel dataset of 7,493 dyad-year observations comprising 427 unique firms." [Methods] "The empirical setting is publicly held U.S. manufacturing firms that are present in KLD’s annual EVP ratings, the WRDS Compustat database and Bloomberg’s SPLC database." [Methods] "The analysis is performed at the level of the buyer-supplier dyad, meaning that each observation is a buyer-supplier pair." [Methods] "In total there are 7,493 dyad-year observations for a seven-year period, 2009 through 2015." [Methods] "The misalignment variables are scores of three different dissimilarity variables based on backgrounds of the TMT of the buyer firm and its suppliers."</t>
         </is>
       </c>
     </row>
@@ -16481,6 +16683,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G323" t="inlineStr">
         <is>
           <t>The importance of emotional labouring and performance of frontline service employees, who in their boundary-spanning positions significantly affect service-rendering organisations’ efficiency by their direct communications with customers, continues to increase. However, it is still important to ascertain an efficient understanding of the comprehensive process including behavioural mechanism and a common perception of the rewards’ impacts on motivation and creativity. Therefore, guided by self-determination theory, this study examined the mechanism and boundary conditions between emotional labour and job performance (creative and task)–specifically, taking charge has been considered as a mediator and performance-based pay as a moderator in between relationships. The authors selected a time-lagged cross-sectional design to investigate interrelations amongst study variables at two different time points and surveyed 417 team members and 186 team leaders in Pakistan’s commercial banks. Findings were consistent with the assumed conceptual framework. For instance, deep-acting affected taking charge positively, surface-acting demonstrated a positive link with task performance and taking charge partially mediated the relationships between deep-acting and performances under boundary conditions of low performance-based pay. By summing up, the study adds to the literature and recommends managerial implications with a more affluent view of nomothetic linkage among frontline employees’ emotional labor, HR practices, and the service sector.</t>
@@ -16508,7 +16715,7 @@
       </c>
       <c r="P323" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>No effect size of interest. The study mentions boundary-spanning positions but measures emotional labor (surface/deep acting) and taking charge, not boundary spanning behavior.. Verbatim Evidence: [Abstract] "The importance of emotional labouring and performance of frontline service employees, who in their boundary-spanning positions significantly affect service-rendering organisations’ efficiency by their direct communications with customers, continues to increase." [Measures] "Emotional labor. We used six items from Emotional Labor scale developed by [54] to measure surface acting (3 items; e.g., “I pretend to have emotions that I do not really have”) and deep acting (3 items; e.g., “I make an effort to actually feel the emotions that I need to display to others”)." [Measures] "Taking charge. We used [30] ten-item scale to measure taking charge. [...] The sample item is, “I try to institute new work methods that are more effective for the company.”"</t>
         </is>
       </c>
     </row>
@@ -16580,6 +16787,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G325" t="inlineStr">
         <is>
           <t>Though improvisation has emerged as a crucial organizational competence, research wrestles with a key question – how can organizations benefit from improvisation? To advance research, I build a richer conceptualization of the role of knowledge resources – market information sources and memory types – in improvisation. I argue that as (a) internal and external sources of market information differ in speed and novelty and (b) procedural and declarative memory differ in articulation and abstractness, they shape the impact of improvisation on new product outcomes in a distinct way. A longitudinal survey of new products in the Dutch food industry uncovers that, contrary to prior thinking, improvisation increases cost efficiency when new product teams rely on internal market information and declarative memory and they minimize external market information. Though both sources of market information and low procedural memory weaken the negative impact of improvisation on market effectiveness, these conditions were not enough to make its impact positive, echoing traditional concerns with improvisation.</t>
@@ -16607,7 +16819,7 @@
       </c>
       <c r="P325" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level unit of analysis with key informant reporting on team behavior.. Verbatim Evidence: [Research Setting] "The questionnaire asked informants to focus on a NPD project (our unit of analysis) completed in the past 12 months." [Measures] "I used the scale of Moorman and Miner (1998b) to measure team-level improvisation, which captures the degree of simultaneity of planning and execution without being confounded with correlates of improvisation such as innovation or bricolage." [Appendix] "Internal market information flows (Kyriakopoulos &amp; de Ruyter, 2004) During this project, we: regularly received market information, i.e., customer needs, competitive action, from other teams"</t>
         </is>
       </c>
     </row>
@@ -16659,7 +16871,7 @@
       </c>
       <c r="P326" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team/project level analysis with key informant rating team behavior. Verbatim Evidence: [Research Setting] The questionnaire asked participants to focus on a product development project for which their business unit was responsible over the last twelve months. [APPENDIX] For this project, my team relied on: [APPENDIX] During this project, we: regularly received market information, i.e. customer needs, competitive action changes from other teams</t>
         </is>
       </c>
     </row>
@@ -16679,7 +16891,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G327" t="inlineStr">
         <is>
           <t>This study draws on theories of collective action and organizational ecology to investigate a particular type of voluntary association: mixed-mode groups. Mixed-mode groups are created and organized online to meet physically in geographically deﬁned ways. An online survey was conducted with 171 randomly sampled groups on Meetup.com—a website that facilitates the creation and coordination of mixed-mode groups. Analysis shows that even when a mixed-mode group implements strategies focused on internal group processes, it beneﬁts from tapping into its external networks to obtain resources for group operation. Also, the differential impacts of internal and external strategies indicate that in the case of environment-prone mixed-mode groups, implementation of internal strategies alone, with or without solicited external networking resources, is helpful for generating positive group outcomes. Together, these results establish that boundary spanning represents not only a type of strategic action to obtain resources and produce positive outcomes but also an inherent and deﬁning mechanism of contemporary voluntary groups for engaging in collective action.</t>
@@ -16707,7 +16923,7 @@
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 2 &amp; Code 3]. Verbatim Evidence: [Code 2 &amp; Code 3]. Verbatim Evidence: "[Methods] The data were collected from Meetup.com, a website specifically designed to facilitate the creation of online groups based on shared interests and physical locations and to coordinate offline group meetings." "[Methods] Those 1,237 selected organizers were asked individually through the contact function on Meetup.com to participate in the online survey, and 171 responded" "[Limitations and conclusion] Third, due to resource and time constraints, this study could only collect data at the group level, so group organizers were the ones providing responses to the survey questions."</t>
         </is>
       </c>
     </row>
@@ -16774,6 +16990,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>The literature on small stand-alone teams has suggested that decentralization has predominantly positive features. However, in multiteam systems, the presence of other highly interdependent teams adds a level of complexity that may preclude generalizing from teams to multiteam systems. We studied the effects of decentralized planning in 210 multiteam systems, each composed of three six-person, functionally specialized component teams. As has previous research, we find that decentralized planning has positive effects on multiteam system performance, attributable to enhanced proactivity and aspiration levels. However, we also find that the positive effects associated with decentralized planning are offset by the even stronger negative effects attributable to excessive risk seeking and coordination failures. We discuss the implications for theories of intrateam and interteam dynamics, along with the applied implications for designing empowerment interventions in team and multiteam contexts.</t>
@@ -16869,6 +17086,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
           <t>Nonprofit organizations have historically been seen as a vanguard in U.S. civil society, supplying places and spaces for innovation and change to flourish. According to the Competing Values Culture Framework (CVCF), a developmental organizational culture, characterized by innovation and risk-taking, may help organizations respond to changes in their operating environments and be more effective at boundary-spanning activities, such as fostering external support, acquiring resources, and spurring growth. Despite its importance, the culture–effectiveness relationship has not been studied sufficiently in nonprofit organizations. The exploratory study described in this article examines the links between developmental culture and nonprofit organizational effectiveness. Results suggest that nonprofit executive directors see organizational culture as more than a phenomenon to be experienced. Specifically, findings indicate that executive directors perceive there to be a positive and significant relationship between developmental culture and how effective their organization is at performing boundary-spanning activities. The practical and theoretical implications of this finding are discussed.</t>
@@ -17064,11 +17282,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
-        </is>
-      </c>
+      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>Science parks are a type of organizational sponsorship initiative aimed at generating resource-munificent environments through the provision of bridging and buffering services. While extant research has studied the relationship between these services and firm outcomes, it has neglected to provide insights into when tenant firms utilize these services to a greater or lesser extent. Our study evaluates science parks’ buffering mechanism and identifies firm-level characteristics affecting tenants’ use intensity of buffering services. To do so, we build upon survey data collected from 201 tenant firms located in science parks in three European countries. Taking a resource dependence perspective, our findings indicate that tenants’ managerial resources (particularly top management team size and functional experience) and boundary-spanning capacity jointly determine the extent to which firms rely upon the science park’s buffering mechanism. This study contributes to the organizational sponsorship, resource dependence, and science park literatures, as well as has important practical implications.</t>
@@ -17096,7 +17310,7 @@
       </c>
       <c r="P335" t="inlineStr">
         <is>
-          <t>Firm-level analysis (N=201 firms) where the manager acts as a key informant reporting on the firm's boundary-spanning capacity.. Verbatim Evidence: [Plain English Summary] "Which firm-level factors determine the use intensity of science parks’ buffering services? We study our research question in a sample of 201 firms located in 35 science parks in Denmark, Spain, and Belgium." [3.1 Data and sample] "In the spring of 2018, we sent out an online survey to these tenants, specifically addressed to the manager in charge of the firm on the SP." [3.1 Data and sample] "As such, our final sample consists of 201 responses from tenants in 35 different SPs." [Appendix 1, Table 5] "Boundary-spanning capacity To which extent does … BS1 … The firm encourages its members to solicit information and resources from elsewhere?"</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -17116,6 +17330,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G336" t="inlineStr">
         <is>
           <t>Purpose – As teams are built around specialized and different knowledge, they need to regulate their knowledge boundaries to exchange their specialized knowledge with other teams and to protect the value of such specialized knowledge. However, prior studies focus primarily on boundary spanning and imply that boundaries are obstacles to sharing knowledge. To ﬁll this research gap, this study aims to indicate the importance of knowledge protection regulation, an activity that sets an adequate boundary for protecting knowledge, and investigate the factors that facilitate knowledge protection regulation and its consequences.</t>
@@ -17143,7 +17362,7 @@
       </c>
       <c r="P336" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 3] Exclude because the unit of analysis is the team (N=138 teams) and the survey items ask about 'Our team', and the study measures knowledge protection regulation rather than individual boundary spanning behavior.. Verbatim Evidence: [Data collection] "Within these seven companies, the survey was distributed to 3,546 individuals working in 198 teams; 2,326 individuals from 196 teams responded to the questionnaires, for a response rate of 65.6 per cent." [Data collection] "A team as the unit of analysis in this study is the smallest formal structure of each company and differs by well-defined tasks, such as inspection, technology planning, database management and customer support." [Data collection] "The individual responses were aggregated into team-level variables with validity." [Table III] "Notes: n = 138; The numbers in the diagonal are the square roots of the variance shared between the constructs and their measures." [Appendix 1] "Our team has processes to protect knowledge from inappropriate use outside the team" [Appendix 1] "Our team has technology that restricts access to some sources of knowledge"</t>
         </is>
       </c>
     </row>
@@ -17163,6 +17382,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G337" t="inlineStr">
         <is>
           <t>This study of Korean industrial salespeople (N = 140) examines the relationships among organizational formalization, role stress, organizational commitment, and propensity to leave. Although most of the theoretical and empirical research in this area was done in the United States, this study examines whether the same concepts could be applied to a culturally different salesforce. The results of the structural modeling analysis suggest that overall the model of job variables and propensity to leave developed in the U.S. could be applied to a Korean salesforce. However, some culture-related differences do exist in the nature of specific relationships.</t>
@@ -17190,7 +17414,7 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>No boundary spanning behavior measured. The study examines role stressors (role conflict, role ambiguity), formalization, commitment, and propensity to leave among salespeople, but lacks a measure of boundary spanning behavior itself.. Verbatim Evidence: [Abstract] "This study of Korean industrial salespeople (N = 140) examines the relationships among organizational formalization, role stress, organizational commitment, and propensity to leave." [Measurement] "Formalization was measured on a 4-item scale adapted from a scale developed by Aiken and Hage (1966)." [Measurement] "Role ambiguity and role conflict were measured using Rizzo, House, and Lirtzman's (1970) six and eight items, respectively." [Measurement] "Organizational commitment of Korean salespersons was measured on the 15-item Organizational Commitment Questionnaire (OCQ)."</t>
         </is>
       </c>
     </row>
@@ -17210,6 +17434,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the effects of relationship bonds on the psychological response and behavior of bank employees based on the job demands–resources theory. Specifically, it examines the effects of relationship bonds in terms of person–job (P–J) fit, emotional exhaustion, job satisfaction and boundary-spanning behaviors, all of which comprise the behavioral dimensions of bank employees. In addition, the study examines how the resiliency of bank employees influences their emotional exhaustion and determines whether a moderating effect related to emotional exhaustion exists.</t>
@@ -17257,6 +17482,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -17356,6 +17582,11 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G341" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -17383,7 +17614,7 @@
       </c>
       <c r="P341" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Included. The study measures individual-level boundary-spanning behavior among full-time project members and reports correlations.. Verbatim Evidence: [Sample] "We recruited full-time project members in construction and engineering industries through online panelists in Australia and the USA" [Measures] "Boundary-spanning behavior. We adapted nine items to measure boundary-related activities (Ancona and Caldwell, 1992). Respondents were asked to indicate the extent to which they felt several listed behaviors were part of their responsibility in dealing with non-team members." "Example items are: 'I keep other teams in the company informed of my team’s activities', 'I collect technical information or ideas from individuals outside of my team', and 'I scan the environment inside or outside the organization for technical ideas or expertise'" [Results] "Table 1 shows the bivariate correlation coefficients and descriptive statistics for key variables."</t>
         </is>
       </c>
     </row>
@@ -17450,6 +17681,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>Innovation is a risky business. Notwithstanding the attention in research on the determinants of innovation success, the estimates of the extremely high failure rates (ranging from 40% to 90%) have not come down. As a result, new approaches have to be found to address the issues that prevent organizations from reaching innovation success over a longer period of time. In this study, Signal Detection Theory (SDT) is introduced to show that it may be less important to improve innovation practices in companies, than it is to change the nature of the projects that enter the corporate innovation funnel. In our empirical study of 44 innovation projects in the pharmaceutical and electronics industry, we show that pursuing more noisy signals (uncertain technological and market opportunities) is currently beneficial for innovation success. In general, companies allocate too few resources to noisy innovation opportunities. Interestingly, we find a positive, and not an inverted U-shaped, relationship between noise/signal ratios and innovation success. This indicates that there are almost no companies that take too much risk in the current competitive environment and that many can gain from increasing their noise tolerance. The implications from this study are quite counter-intuitive in a sense that ‘risk’ is not the cause of the innovation problems, but may be a solution.</t>
@@ -17591,6 +17823,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>Past research on team boundary work has focused on a “cold,” information-exchange perspective to explain why boundary activities affect team innovation. Although the theory is widely accepted, empirical studies on the actual mechanism are scant and produce inconsistent results. Drawing from Interaction Ritual Theory (Collins, 2004), we propose a “warm,” affective perspective that emphasizes team emotional energy - a shared feeling of enthusiasm among team members - as a mechanism linking boundary work and team innovation. Moreover, we examine a theory-driven contextual factor -team role overload - that modifies the hypothesized mediated relationship. Based on field data from four different sources of 89 automotive research and development teams (comprising 724 employees, 89 direct supervisors and 18 managers), we found that both team boundary-spanning and boundary-buffering activities are associated with higher levels of team emotional energy, which, in turn, are related to greater levels of team innovation. Moreover, the mediated relationship of boundary-buffering activities, team emotional energy and team innovation is moderated by team role overload, such that the mediated relationship is stronger when team role overload is higher. Our study contributes to the literature by broadening our understanding of why boundary work is effective and when it matters most.</t>
@@ -17742,6 +17975,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G349" t="inlineStr">
         <is>
           <t>Boundary-spanning activity is conceived of as an intervening variable between organization structure and perceived environmental uncertainty (PEU). This is due primarily because, since boundary spanners operate at the skin of the organization, their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relations between PEU, organization structure, and boundary-spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relations were found between all three variables. Partial relations indicated that PEU does not influence the relationship of boundary spanning to structure but structure reduces the relationship of PEU to boundary spanning to zero, and boundary spanning reduces the relationship between structure and PEU to zero. Thus, not only is the notion of boundary spanning as an intervening variable supported, but results suggest that causality in the relationship between structure and PEU may be from structure to PEU rather than current contingency notions of PEU affecting structure.</t>
@@ -17769,7 +18007,7 @@
       </c>
       <c r="P349" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>The study measures mere communication frequency rather than purposive boundary-spanning behavior, and lacks a zero-order Pearson correlation matrix (reporting only Goodman-Kruskal's Gamma).. Verbatim Evidence: [Measures of the Variables] "In this study, boundary-spanning activity is defined by the total verbal and written interactions with extra work units." [Table 4] "2. How many hours do you confer about your work in informal face-to-face conversation or telephone conversation with people of other organizations."</t>
         </is>
       </c>
     </row>
@@ -17885,6 +18123,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>Boundary spanning has been proven to have positive implications for innovation performance; yet, some individuals are less boundary-spanning than others. Drawing on the attachment theory and organizational support theory, this study develops a multi-level theoretical model to investigate how individuals’ attachment insecurity influences boundaryspanning behavior through self-efficacy and the moderating role of organizational support climate. To validate the proposed model, we adopted a survey research, and collected data from NPD project teams in China. The results revealed that both insecure attachment styles were associated with lower levels of individual boundary-spanning behavior, and self-efficacy partially mediated these relationships. Moreover, organizational support climate played a moderating role in the relationship between attachment anxiety and boundary-spanning behavior. With a high level of support climate, the negative impact of attachment anxiety on boundary-spanning behavior was weakened. This elucidates the role of individual affective motivation and team shared perceptions in shaping individual externally focused behavior.</t>
@@ -17984,6 +18223,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>From a knowledge-based perspective, this paper highlights the need for a framework linking perceived competition of the industry and ﬁrms’ strategic location choices of external knowledge search and examines whether the perceived competition increases the propensity of cluster ﬁrms to search more widely from extra-cluster knowledge sources than intra-cluster knowledge sources. Furthermore, we emphasise that cluster ﬁrms with varying degrees of tacitness in their knowledge base might respond to such competition diﬀerently when conducting external knowledge search activities. Using a sample of 310 cluster ﬁrms in the Zhejiang Province of China, we ﬁnd that the cluster ﬁrm would increase the propensity for more geographic boundary-spanning search relative to local search while under the pressure of competition. Moreover, the positive relationship between perceived competition and the propensity towards geographic knowledge search is weaker when the tacitness of the cluster ﬁrm’s knowledge base is higher. The ﬁndings contribute to the understanding of the relationship between competition and the choice of location strategies in external knowledge search.</t>
@@ -18031,6 +18271,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -18058,7 +18303,7 @@
       </c>
       <c r="P355" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Firm-level analysis of boundary-spanning search (managers acting as key informants for the firm). Verbatim Evidence: [3.1 Questionnaire design and data collection] "The research questions of this study revolve around innovative behaviors, so firms with independent innovation capabilities were specifically selected as the research subjects." [3.1 Questionnaire design and data collection] "Middle and senior managers who had worked for the firm for at least two years and possessed a good understanding of R&amp;D activities were included." [Appendix] "1a. We closely monitors the dynamics of companies with whom we have established cooperative relationships" [Appendix] "1b. We proactively seeks to understand changes in customer preferences for products or services"</t>
         </is>
       </c>
     </row>
@@ -18125,7 +18370,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>Using a longitudinal in-depth field study at NASA, I investigate how the open, or peer-production, innovation model affects R&amp;D professionals, their work, and the locus of innovation. R&amp;D professionals are known for keeping their knowledge work within clearly defined boundaries, protecting it from individuals outside those boundaries, and rejecting meritorious innovation that is created outside disciplinary boundaries. The open innovation model challenges these boundaries and opens the knowledge work to be conducted by anyone who chooses to contribute. At NASA, the open model led to a scientific breakthrough at unprecedented speed using unusually limited resources; yet it challenged not only the knowledge-work boundaries but also the professional identity of the R&amp;D professionals. This led to divergent reactions from R&amp;D professionals, as adopting the open model required them to go through a multifaceted transformation. Only R&amp;D professionals who underwent identity refocusing work dismantled their boundaries, truly adopting the knowledge from outside and sharing their internal knowledge. Others who did not go through that identity work failed to incorporate the solutions the open model produced. Adopting open innovation without a change in R&amp;D professionals’ identity resulted in no real change in the R&amp;D process. This paper reveals how such processes unfold and illustrates the critical role of professional identity work in changing knowledge-work boundaries and shifting the locus of innovation.</t>
@@ -18220,6 +18464,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>Triggered by the fierce competition and substantial changes in worldwide markets during the past two decades, an increasing number of firms have adopted a logistics outsourcing strategy to maintain core competencies and gain competitive advantages. Accordingly, the relevant research has achieved both practical and academic attention, ranging from the type of logistics activities outsourced, the motivation for such operations, and the positive and/or negative results of the actions. Nevertheless, the relevant supply chain management (SCM) literature is sparse and scattered and thus considerable opportunities remain for further exploration, especially in logistics outsourcing relationship management (LORM). Unfortunately, due to various reasons such as the dominant focus on organisational level issues, the difficulty of evaluating people issues and the lack of a comprehensive theoretical foundation, the literature thus far has not adequately explored this phenomenon.</t>
@@ -18315,6 +18560,7 @@
           <t>1 = Include</t>
         </is>
       </c>
+      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
           <t>Currently boundary spanning behavior is a hot topic in team research field, which involves phenomena at two levels (team level and individual level). Compared to team level, employee's boundary spanning has not been well discussed yet. In addition, few studies have systematically explored its outcomes and impact mechanism in Chinese context. This study aimed to address the above gaps by examining whether, when and how employee's boundary spanning behavior impacted his or her task performance. Specifically, integrating culture and social network theory into boundary spanning field, this study theorized that boundary spanning behavior led to centrality of the employee's social network, and in turn enhance his or her task behavior. At the same time, team's collectivism climate moderated the above path. The participants were recruited from 17 companies in two high-tech parks located in Beijing and Tianjin, China. We invited 135 team leaders and their subordinates to participate the survey, after collecting 2 wave longitudinal data sets and dropping out invalid questionnaires, responses from 61 team leaders and 292 team members were valid finally. To get enough whole network data, we purposely chose teams with small size. All measurements were (or adapted from) well-established scales. Employee's boundary spanning behavior, centrality, and collectivism were collected at time 1, and after 8 weeks, employees' task performance was collected at time 2. Confirmatory factor analyses showed satisfactory model fit indices. Inter-rated agreement (Rwg) and intra-class correlation (ICC) value justified the aggregation of team collectivism climate. HLM were applied to test our hypotheses since this is a cross-level research. Variables like age, education, gender, tenure and collectivism orientation at individual level, and team size at group level were controlled for. The results showed that centrality of the social network positively mediated the relation between employees' boundary spanning behavior and his or her task performance. The climate of team collectivism positively moderated the relation between employees' boundary spanning behavior and network centrality. In addition, network centrality mediated the interaction between boundary spanning behavior and team collectivism climate on employee's task performance such that the relation between boundary spanning behavior and task performance via network centrality will be stronger for teams higher on collectivism climate than for those lower on collectivism. This study revealed that employee's boundary spanning behavior had positive influence on task performance and confirmed the mechanism between the two constructs. Interestingly, we found collectivism at individual level and at team level had different effects for the effect of boundary spanning behavior, which revealed that in transformational Chinese context, cultural elements at micro levels were worthy of discussing. The finding of mediating mechanism of centrality established a logic chain of" external relationship—internal embeddedness—performance", helping in explaining the formation of performance and social network in teams. Managerial implications, limitations and future directions were discussed at the end.</t>
@@ -18362,7 +18608,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine team external learning, particularly focusing on: how leader external learning behavior affects team external learning; how team external learning inﬂuences employee creativity; and whether team internal learning is a moderator between the cross-level relationship of external learning and employee creativity in Chinese R&amp;D teams.</t>
@@ -18410,7 +18655,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
           <t>Expatriates typically perform boundary-spanning to address challenges related to functional, linguistic, and cultural variations within multinational enterprises (MNEs), which in turn influences their relationships with host-country employees. Integrating social capital and role theory perspectives, this study explores the relational dynamics between expatriates and host-country employees by developing a novel theoretical framework that examines the double-edged effects of expatriates’ boundary-spanning. We propose that expatriates’ boundary-spanning nurtures mutual trust between expatriates and hostcountry employees, further facilitating expatriates’ identification with subsidiaries and host-country employees’ identification with MNEs. On the other hand, we propose that boundary-spanning increases expatriates’ role stressors, causing expatriates’ emotional exhaustion and outgroup categorization by host-country employees. We further categorize expatriates’ boundaryspanning into three types (functional, linguistic, and cultural) and theorize about their varying effects on the cognitive and affective bases of mutual trust and on role stressors. With data from 177 expatriate–host-country coworker dyads in Chinese MNEs, our double-edged framework is generally supported. Our findings suggest that cultural boundary-spanning exhibits the strongest double-edged effect, while functional boundary-spanning shows asymmetric effects, with negative outcomes surpassing positive ones, and linguistic boundary-spanning demonstrates the weakest effect. This study offers realistic and comprehensive insights into expatriates’ boundary-spanning, particularly in expatriate–host-country employee relationships.</t>
@@ -18495,7 +18739,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>In an increasingly global research landscape, it is important to identify the most prolific researchers in various institutions and their influence on the diffusion of knowledge. Knowledge diffusion within institutions is influenced by not just the status of individual researchers but also the collaborative culture that determines status. There are various methods to measure individual status, but few studies have compared them or explored the possible effects of different cultures on the status measures. In this article, we examine knowledge diffusion within science and technology‐oriented research organizations. Using social network analysis metrics to measure individual status in large‐scale coauthorship networks, we studied an individual's impact on the recombination of knowledge to produce innovation in nanotechnology. Data from the most productive and high‐impact institutions in China (Chinese Academy of Sciences), Russia (Russian Academy of Sciences), and India (Indian Institutes of Technology) were used. We found that boundary‐spanning individuals influenced knowledge diffusion in all countries. However, our results also indicate that cultural and institutional differences may influence knowledge diffusion.</t>
@@ -18538,6 +18781,12 @@
           <t>BSMA0363</t>
         </is>
       </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr"/>
       <c r="G366" t="inlineStr">
         <is>
           <t>Individual innovation involves many contradicted behavioral options such as creative vs. habitual actions and explorative vs. exploitative activities. However, the agentic nature of innovative behaviors has been widely ignored, and we know less about what factors lead individuals to approach and balance the contradictions caused by competing demands and intentionally engage in innovative behaviors. Integrating social cognitive theory and innovation paradox, we propose a chain-mediating model to explain how employees with a paradox mindset realize the creative benefits through their innovative endeavors, considering role breadth self-efficacy (RBSE) and individual ambidexterity as two mediators. Using data collected from 480 employees paired with 100 supervisors at 3-time points, the results show that RBSE and individual ambidexterity play a mediating role, respectively, even though they sequentially play a chain-mediating role between employees’ paradox mindset and innovative performance. Individuals who hold a paradox mindset are more likely to perceive high capability beliefs in successfully undertaking expanded roles, promoting behavioral tendencies to switch between exploration and exploitation, and in turn encouraging employees to undertake more innovative behaviors. Finally, we discuss the theoretical and practical implications for promoting employees’ innovative performance from an agentic perspective. Employees with a paradox mindset can make creative things happen by managing the tensions between exploration and exploitation proactively. Thus, organizations may try to enhance employees’ proactive motivation states and behavioral capability to encourage individual innovation.</t>
@@ -18561,6 +18810,11 @@
       <c r="K366" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18612,6 +18866,12 @@
           <t>BSMA0365</t>
         </is>
       </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr"/>
       <c r="G368" t="inlineStr">
         <is>
           <t>Research Summary: Chief executive officer (CEO) entrepreneurial orientation (EO) is an emerging topic within entrepreneurship research. This research offers the attention-based view (ABV), and its principles of attentional focus, situated attention, and structural distribution of attention to explain how CEO EO fosters an innovative organizational workforce. We theorize that CEO EO predicts lower-level employee innovative behavior when their top managerial attentional focus on entrepreneurship is translated into highperformance work practices, which structurally distribute their strategic attention throughout the organization and promotes a situated attentional condition for employees emphasizing innovation. Moreover, we consider (a) humanresource management (HRM) perceived importance and (b) departmental functional foci as boundary conditions. Using a multi-level and multi-source sample from 152 Chinese firms, results support our arguments.</t>
@@ -18635,6 +18895,11 @@
       <c r="K368" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P368" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -18686,6 +18951,16 @@
           <t>BSMA0367</t>
         </is>
       </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G370" t="inlineStr">
         <is>
           <t>This study examined Hosmer's (1994) proposition that an ethical approach to management engenders stakeholder trust, which, in turn, brings about commitment and innovation from the perspectives of traditionally out-group suppliers and in-group employees, respectively. Boundary-spanning employees of the Internet-enhanced manufacturing companies participated in the study in their roles as either suppliers or employees. A sample of 54 buyer-supplier inter-organizational relationships and 54 employer-employee intra-organizational relationships were used to test the proposition.</t>
@@ -18709,6 +18984,11 @@
       <c r="K370" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P370" t="inlineStr">
+        <is>
+          <t>No effect size of interest (Boundary spanning is a characteristic of the sample, not a measured variable). Verbatim Evidence: [Domain of the Study] "This study focuses on examining whether suppliers’ and employees’ perceptions about Internet-based company’s ethical climate influence their respective trust in the company. It also looks at whether such trust influences their respective perceptions of commitment and innovation." [Sample and Setting] "Boundary-spanning employees, who use the Internet in their job performances, are the focus of this study because e-collaboration of internal and external stakeholders is essential to innovations that are critical for success in an Internet based world." [Analysis] "Table 11 Pearson Correlation Coefficient 1. Caring/ Benevolence 2. Law and Code/Principle -Cosmopolitan 3. Rules/ Principle-Local 4. Instrumental/ Egoism 5. Independence/ Principle-Individual 6. Trust 7. Commitment and Innovation"</t>
         </is>
       </c>
     </row>
@@ -18760,6 +19040,16 @@
           <t>BSMA0369</t>
         </is>
       </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G372" t="inlineStr">
         <is>
           <t>Abstract             This research provides an improved understanding of how ventures successfully organize via resource allocations. Conceptually, we apply elements of action theory to account for resource trade-offs that occur as entrepreneurs make decisions about adding staff members to boundary spanning, technical core, and management functions. We then model how these allocation decisions differentially impact nascent venture performance. Empirically, we test our model with a sample of 2484 entrepreneurs captured in the Kauffman Firm Survey, a longitudinal dataset that tracks a random sample of US startups over an 8-year period. Results from dynamic panel estimation reveal evidence of both performance penalties and performance boosts as the result of entrepreneurs adding staff to specific areas, revealing optimality in specific configurations of entrepreneurial organizing elements.</t>
@@ -18783,6 +19073,11 @@
       <c r="K372" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P372" t="inlineStr">
+        <is>
+          <t>Firm-level analysis of nascent ventures, entrepreneur sample, and boundary spanning measured as the number of sales employees.. Verbatim Evidence: [Sample and Level of Analysis] "We use the KFS, a longitudinal dataset that tracks a random sample of 4928 US nascent ventures over an 8-year period." [Sample and Level of Analysis] "Due to missing data, our final sample consists of an unbalanced panel of 2484 nascent ventures and 11,802 firm-year observations." [Measures] "In testing H1, we use the number of sales employees as a proxy for the boundary span capacity."</t>
         </is>
       </c>
     </row>
@@ -19028,7 +19323,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F378" t="inlineStr"/>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G378" t="inlineStr">
         <is>
           <t>A central focus of cross-cultural management research is how individuals and organizations differ across national cultures and how that fundamentally shapes their thoughts and actions and serves as a unit of identification. In this article, we critically reconsider the essential categorical nature of culture, problematizing categorization and questioning national culture as the primary basis of differentiation. We draw on intersectionality, an approach that helps understand how multiple categories are experienced by the individual, and on relationality, an approach that conceptualizes people, organizations, and their actions within dynamic patterns of relations and cultural meanings. Both approaches challenge the primacy, unity, and separateness of any given category, the a priori determination of categories (and associated boundaries) in research, and the nature and stability of boundaries. Based on this we advance notions of boundary work and boundary shifting that help explore how today’s sociocultural groups and categories, and the boundaries that separate them, emerge and change. We conclude that, while the extant crosscultural literature has come far in identifying differences, relationality and intersectionality can enable cross-cultural scholars to engage in research practice that better reflects the complexities of sociocultural life. We contribute to theory by suggesting why and how these two approaches can be used to explore complex cross-cultural management phenomena.</t>
@@ -19056,7 +19355,7 @@
       </c>
       <c r="P378" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Conceptual paper without empirical data [Code 1 &amp; Code 4]. Verbatim Evidence: [Abstract] "Our objective in this paper is to advance the field of cross-cultural management by suggesting different ways of theorizing and empirically addressing categories and boundaries." [Conclusion] "We encourage researchers to challenge cross-cultural management phenomena, specifically to reconsider these in terms of fluid social processes rather than isolated individuals or rigid (external) influences. This does not of course deny the existence of a certain order, which remains at the core of any cultural phenomenon. In this article, we propose focusing on relations and the emergence, changing, and reconceiving of categorical boundaries and/or intersecting multiple categories as a way forward."</t>
         </is>
       </c>
     </row>
@@ -19076,6 +19375,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F379" t="inlineStr"/>
       <c r="G379" t="inlineStr">
         <is>
           <t>The paper explores how formal leaders make sense of and deal with autonomy of knowledge-workers. Based on interviews, I suggest that leaders make sense of knowledge-workers’ autonomy as ranging from perfectly autonomous to too autonomous to less independent to acting childish. This ambiguity was dealt with by making sense of leading as ranging from facilitative and supportive approaches to more controlling, even reprimanding acts. This empirical investigation of constructions of ‘leader/ship’ and ‘followers’ contributes to leader/ship-follower/ship literature. The paper’s contribution to theory lies in the notion of situated ambiguity; a way to understand the emerging way through which formal leaders navigate and smoothly move between their own diﬀering perspectives, diﬀerent practical situations, various culturally acceptable understandings of leaders and knowledgeworkers.</t>
@@ -19118,6 +19418,16 @@
           <t>BSMA0377</t>
         </is>
       </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G380" t="inlineStr">
         <is>
           <t>Prior research on professional boundary work emphasises the importance of subtle interactions among affected individuals when a new role is inserted into an established professional setting, which inevitably changes the prevalent division of labour. Thus, managers may set reflective spaces for professionals to collaboratively arrange their boundaries and make room for the new professional. This ethnomethodologically oriented study examines boundary arrangements in work development meetings in a university hospital, while professionals made room for a new role, a hospitalist. Examining professionals’ naturally occurring interactions in reflective spaces, the findings depict seven categorisations for the hospitalist. Elaborating on the dynamics of these categorisations, we propose that technically based categorisations sustain stability, and context-bound categorisations allow change in work practices, whereas their combination enables transformation within the institutional context. Accordingly, the study adds to the literature on the transformative potential of reflective spaces by illuminating the intertwining of engaged professionals’ boundary talk in interaction with the consequences of configurational boundary work in relation to a new professional role.</t>
@@ -19141,6 +19451,11 @@
       <c r="K380" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>Qualitative study lacking quantitative effect sizes (no correlation matrix). Verbatim Evidence: [Abstract] "This ethnomethodologically oriented study examines boundary arrangements in work development meetings in a university hospital, while professionals made room for a new role, a hospitalist." [Data] "The primary data applied in this study were acquired by video-recording and transcribing interactions during eight work development meetings using the transcription system introduced by Jefferson (1984) (see Table 1) to illustrate the manifested accounts in detail." [Analytical process] "In the analytical process, we drew on membership categorisation analysis (Housley and Fitzgerald, 2002; Stokoe, 2012)."</t>
         </is>
       </c>
     </row>
@@ -19155,6 +19470,16 @@
           <t>BSMA0378</t>
         </is>
       </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G381" t="inlineStr">
         <is>
           <t>This study examines how personal attachments between boundary spanners within cross-cultural international cooperative ventures (ICVs) are established and their association with venture performance. Results of analysis of 282 ICVs in an emerging market (People's Republic of China) show that the development of personal attachment depends on factors at three levels. At the individual level, attachment is an increasing function of overlap in tenure between boundary spanners. At the organizational level, attachment is heightened by goal congruity between the parent firms but is impeded by cultural distance. At the environmental level, market disturbance and regulatory deterrence lead to strong attachments. Such attachments stimulate an ICV's process performance and increase financial returns.</t>
@@ -19178,6 +19503,11 @@
       <c r="K381" t="inlineStr">
         <is>
           <t>2001</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr">
+        <is>
+          <t>Firm-level analysis of international cooperative ventures (ICVs) where managers act as key informants.. Verbatim Evidence: [Sample and unit of analysis] "The respondents were the ICVs' general managers (or, in 10 cases, deputy general managers) whose names were given in the above List and Directory." [Sample and unit of analysis] "After several rounds of follow-up reminders, 282 useful questionnaires were received, representing a 35.25 percent response rate." [Key Informant] "Each respondent was asked to represent the venture in answering the above questions in his or her capacity as an ICV's leading manager." [Construct Items] "Personal attachment was measured by the average of the responses, on a 7-point Likert scale, to the following items: (1) the extent to which interpersonal relations have been developed to date between each party's boundary spanners since the ICV was formed; (2) the extent to which interpersonal relations had been developed between these boundary spanners through previous trade, investments, or negotiations before the ICV was formed; (3) the extent to which foreign boundary spanners have provided Chinese boundary spanners with needed personal skills and knowledge; and (4) the extent to which Chinese boundary spanners have provided foreign boundary spanners with needed personal skills and knowledge."</t>
         </is>
       </c>
     </row>
@@ -19197,6 +19527,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>Building on the “loose coupling” logic, this study examines the importance of boundary spanners' shared perceptions of procedural justice in cross-cultural cooperative alliances. I argue that alliance profitability is higher when both parties perceive high rather than low procedural justice. Profitability is also higher when both parties' perceptions are high than when one party perceives high procedural justice but the other perceives low procedural justice. Shared justice perceptions become even more important for alliance profitability when the cultural distance between partners is high or when the industry of operation is uncertain. Analysis of 124 cross-cultural alliances in China supports these propositions.</t>
@@ -19292,11 +19623,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr">
-        <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
-        </is>
-      </c>
+      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>Abstract             This study applies the justice theory to address interpartner cooperation in strategic alliances. It emphasizes how procedural fairness as perceived by boundary spanners in these alliances influences cooperation outcomes. We theorize that procedural fairness improves cooperation results through enhancing relational value and curtailing relational risk in an environment characterized by both economic and social exchange. Our path analysis suggests that procedural fairness has a direct effect on operational outcome, but an indirect effect on financial outcome via increased trust driven by fairness. Procedural fairness contributes more to performance outcomes when strategic alliances are equity joint ventures than if they are contractual agreements. Theoretical and managerial implications arising from the findings are highlighted. Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -19324,7 +19651,7 @@
       </c>
       <c r="P384" t="inlineStr">
         <is>
-          <t>Alliance-level analysis (N=168 alliances) measuring procedural justice, not individual Boundary Spanning Behavior.. Verbatim Evidence: [Reason summary] Verbatim Evidence: "[Introduction] This study deﬁnes procedural justice in the alliance context as the extent to which an alliance’s strategic decision-making process and procedures are impartial and fair as perceived by this alliance’s boundary spanners." "[Methods] We limited the sample to those alliances with two partners since the multiparty case (three or more) complicates the measurement of most constructs used and differs in cooperation logic and behavior from the two-party case." "[Methods] We measured justice based on the convergent score from the matched 168 sample alliances"</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19339,6 +19666,16 @@
           <t>BSMA0382</t>
         </is>
       </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G385" t="inlineStr">
         <is>
           <t>Purpose – Public sector employees’ contributions play a crucial role in improving public service quality and promoting the image of public organizations. The aim of this research is to unravel how and when human resource (HR) flexibility activates citizen-oriented boundary-spanning behaviors among public sector employees.</t>
@@ -19362,6 +19699,11 @@
       <c r="K385" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P385" t="inlineStr">
+        <is>
+          <t>Included. The study measures citizen-oriented boundary-spanning behaviors of individual public sector employees using the canonical Bettencourt et al. (2005) scale and provides a valid zero-order correlation matrix.. Verbatim Evidence: [Sample] "The data were garnered from employees who belonged to governmental agencies in a major city in Vietnam." [Sample Size] "At T2, 427 complete responses (response rate: 58.8%) were obtained from employees who partook in T1. At T3, among 144 survey links that had been distributed to supervisors, 102 complete responses (response rate: 70.8%) were obtained from supervisors." [Measures] "Citizen-oriented boundary-spanning behaviors were examined through items adapted from Bettencourt et al. (2005), comprising four items for internal influence (e.g. “Contributes many ideas for citizen promotions and communication”), four items for external representation (e.g. “Says good things about the organization to others”) and five items for service delivery (e.g.“Regardless of circumstances, exceptionally courteous and respectful to citizens”)."</t>
         </is>
       </c>
     </row>
@@ -19413,6 +19755,16 @@
           <t>BSMA0384</t>
         </is>
       </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G387" t="inlineStr">
         <is>
           <t>Evidence suggests that product managers' need to communicate across organizational and environmental boundaries under conditions of uncertainty can give rise to powerful role pressures of conflict and ambiguity. These pressures are generally associated with negative or dysfunctional personal outcomes such as job‐related tension, dissatisfaction, and poorer performance. Moreover, in situations where role conflict is particularly high, experienced product managers are susceptible to “burnout.” Some practical approaches to overcoming these difficulties are discussed.</t>
@@ -19436,6 +19788,11 @@
       <c r="K387" t="inlineStr">
         <is>
           <t>1988</t>
+        </is>
+      </c>
+      <c r="P387" t="inlineStr">
+        <is>
+          <t>Construct invalid (Mere communication frequency). Verbatim Evidence: [Boundary Spanning Activity] "Eleven items were used to measure the extent of boundary spanning by the product managers. Total boundary spanning activity was separated into formal versus informal and internal versus external communications (excluding strictly social contacts). Separate items were used for verbal and written communications. A typical item was: 'How many times a week do you send or receive formal written communication, in the form of reports or data from people (a) outside the marketing department but within your company? (b) outside your company?'"</t>
         </is>
       </c>
     </row>
@@ -19529,6 +19886,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr">
         <is>
           <t>Although the use of generative artificial intelligence (AI) within organizations is becoming increasingly common, research on how to enhance employees' competitive advantage through generative AI use within organizations is very limited. Using a resource-based view model, this study investigates the relationship between generative AI use and employees' competitive advantage, as well as the moderating role of perceived organization support. From an analysis of data from 264 employees from 200 organizations, it is found that work-related generative AI use has a positive effect on employee boundary spanning, which contributes to employee competitive advantage. Secondly, work-related generative AI use also has a positive effect on employee agility, including employee resilience and employee adaptability, which further contributes to employee competitive advantage. However, work-related generative AI use has a positive effect on employee proactivity, while the effect of employee proactivity on employee competitive advantage is not significant. Thirdly, perceived organizational support can enhance the effect between employee boundary spanning and employee competitive advantage. However, it is interesting to observe that perceived organizational support enhances the effect between employee adaptability and employee competitive advantage, while weakening the effect between employee proactivity and employee competitive advantage. It does not exert a moderating effect between employee resilience and employee competitive advantage. These findings can help deepen the current understanding of the relationship between generative AI use in the organization and employee competitive advantage, and provide suggestions for business managers on how to use generative AI to improve employee competitive advantage.</t>
@@ -19628,6 +19986,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G392" t="inlineStr">
         <is>
           <t>Although difficult, complicated, and sometimes discouraging, collaboration is recognized as a viable approach for addressing uncertain, complex and wicked problems. Collaborations can attract resources and increase efficiency, facilitate visions of mutual benefit that can ignite common desires of partners to work across and within sectors, and create shared feelings of responsibility. Collaboration can also promote conceptualized synergy, the sense that something will “be achieved that could not have been attained by any of the organizations acting alone”(Huxham, 2003). However, previous inquiries into the problems encountered in collaborations have not solved an important question: How to enable successful collaboration? Through exploratory sequential mixed-methods research conducted in three empirical studies, I discover how interorganizational collaborations can overcome barriers to innovate and rejuvenate communities and understand the factors and antecedents that influence successful collaboration.</t>
@@ -19655,7 +20018,7 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Respondent acts as a key informant rating team-level boundary spanning rather than individual behavior.. Verbatim Evidence: [Sample] "A total of 452 qualified respondents (i.e., they participated in a late-stage or completed project involving a collaboration with another organization and held an appropriate management category position) contributed to the data analysis." [Measures] "1. The team encourage its members to solicit information and/or resources from beyond the organization. 2. The team encourage its members to try to influence important stakeholders on behalf of the team and its work."</t>
         </is>
       </c>
     </row>
@@ -19771,10 +20134,14 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
-        </is>
-      </c>
-      <c r="F395" t="inlineStr"/>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G395" t="inlineStr">
         <is>
           <t>In this study of the business communication that connects an organization with others in its environment, we link boundary spanning with network theory and propose the concept of an extended network of communication. This extended net work is the structure of business communication which flows in work-related ties that organization members maintain both within the organization and across its boundary. We study the relationship between boundary-spanning communication and individual influence in a network with 108 organizational members. We find that boundary spanning correlates with influence, regardless of hierarchical level. There is also a curvilinear relationship between boundary-spanning communication and individual influence. Thus, managers need to balance their communication within and across the organizational boundary.</t>
@@ -19802,7 +20169,7 @@
       </c>
       <c r="P395" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Included. The study measures boundary spanning behavior via network degree centrality of external contacts at the individual level (managers in a transit authority) and provides a zero-order correlation matrix.. Verbatim Evidence: [Sample] "These hypotheses were tested using data gathered from 108 managers in an urban transit authority in the western United States." [Measures] "Boundary spanning communication: Do you interact with people in other organizations (such as vendors, contractors, government agencies, other transit agencies, etc.) to get your job done?" [Matrix] "Table 1 Descriptive Statistics and Correlations (N = 108)"</t>
         </is>
       </c>
     </row>
@@ -19869,6 +20236,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr">
         <is>
           <t>Co‐development with customers attracts considerable interest as a means to improve companies’ product innovativeness and performance. Forward‐thinking companies integrate co‐development within their business models, but many remain uncertain about which levers best foster its implementation. This study therefore takes a top‐down perspective on ways to stimulate co‐development with customers. Relying on boundary theory and its wider contextualization in relation to resource dependence theory, the authors argue that an innovation‐oriented strategy, combined with transformational and transactional leadership, represents senior management levers for driving general openness and providing strategic directions for innovation, which then helps bridge the boundary with customers and facilitate the co‐development of new products. Data from 135 managers and 415 subordinates reveal that some senior management levers can foster co‐development. Specifically, the results of the hierarchical regression analyses confirm the hypothesized positive interaction effect of innovation‐oriented strategy and transformational leadership, whereas the combination of innovation‐oriented strategy and transactional leadership is not beneficial. The strength of innovation‐oriented strategy as an important senior management lever differs for goods and services, which is not the case for the other two levers. Finally, this study provides a more fine‐grained perspective on the new product frequency outcomes of co‐development, by relying on organizational learning theory. Most research is restricted to linear relationships, but the current investigation unveils an inverted U‐shaped relationship between co‐development and companies’ new product frequency. Hence, companies can profit from co‐development at lower and medium levels, but the common notion of “the more, the better” does not apply to an unlimited degree for co‐development.                                         Practitioner Points                                                                        Senior managers should implement an innovation‐oriented strategy to provide guidance regarding the company's innovation generation goals in co‐development projects.                                                           Companies need to support organizational members with adequate freedom and flexibility in terms of co‐development projects, instead of focusing on fixed goals, expectations, or rewards.                                                           If they offer services in particular, companies should initiate appropriate training and coaching for senior managers, to help them better motivate and lead organizational members with a transformational leadership style.                                                           Co‐development can be fostered by senior managers from the top but also should be tracked, using management tools and key performance indicators, to recognize negative efficiency trends as early as possible.</t>
@@ -19964,6 +20332,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G399" t="inlineStr">
         <is>
           <t>The authors examined how networks of teams integrate their efforts to succeed collectively. They proposed that integration processes used to align efforts among multiple teams are important predictors of multiteam performance. The authors used a multiteam system (MTS) simulation to assess how both cross-team and within-team processes relate to MTS performance over multiple performance episodes that differed in terms of required interdependence levels. They found that cross-team processes predicted MTS performance beyond that accounted for by within-team processes. Further, cross-team processes were more important for MTS effectiveness when there were high cross-team interdependence demands as compared with situations in which teams could work more independently. Results are discussed in terms of extending theory and applications from teams to multiteam systems.</t>
@@ -19991,7 +20364,7 @@
       </c>
       <c r="P399" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 2 &amp; Code 3] Student sample in a simulated environment and team-level (MTS) analysis.. Verbatim Evidence: [Method - Participants] "We recruited 184 students from psychology courses at a southeastern university to participate in the study in exchange for course credit." [Method - Participants] "Participants were assigned to 46 four-member MTSs." [Table 1] "Note. N = 46."</t>
         </is>
       </c>
     </row>
@@ -20249,6 +20622,11 @@
       <c r="E405" t="inlineStr">
         <is>
           <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -20300,7 +20678,7 @@
       </c>
       <c r="P405" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Team-level analysis and survey referent (N=56 teams). Verbatim Evidence: [Page 68] &lt;Table 2.9: Correlations, Means, and Standard Deviations. ... Notes: ... 2. n = 56.&gt; [Page 58] &lt;Of the 79 teams that were involved in software projects, 73 agreed to participate. Of these 73 teams, 56 provided usable responses at all three points of measurement in the study for an effective response rate of 77%.&gt; [Page 46] &lt;The focus (or referent) of the scale items shifts from the individual (who is providing scale ratings) to the team, because the individual is providing responses about the team, not about himself or herself. This referent shift consensus addresses concerns about using individual-level responses to measure unit-level (in this case, team-level) variables (Chan 1998).&gt; [Page 126] &lt;Customer Feedback 1. When design problems arise, we resolve them with the customer 2. We coordinate our activities with our client 3. Our team negotiates delivery deadlines and schedules with the customer 4. We review the project design with the customer&gt;</t>
         </is>
       </c>
     </row>
@@ -20320,6 +20698,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
         <is>
           <t>Abstract                                                                                     According to numerous studies across multiple disciplines in the social sciences, business organizations tend to develop adversarial relationships with representatives of the public interest. A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter‐organizational conflict, organizational communication and stakeholder management. Empirical results support the descriptive power of a two‐dimensional model reflecting four relational styles that participating organizations exhibited: avoidance, compliance, co‐optation and negotiation. The two dimensions that constitute the model are cooperativeness and boundary spanning. More importantly, managers who attributed power and legitimacy to public interest group stakeholders reported that their organizations were more likely to cooperate with these stakeholders. On the other hand, managers who perceived public interest groups' claims having                     urgency                     were more likely to develop communicative, boundary spanning relationships with public interest groups but these relationships were less likely to be cooperative. Because unhealthy relationships with these groups can be detrimental to an organization's long‐term prospects, managers must be careful to recognize public interest organizations as potent and legitimate potential allies.                                                                  Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -20518,6 +20897,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F410" t="inlineStr"/>
       <c r="G410" t="inlineStr">
         <is>
           <t>Despite emerging evidence of contracting for evidence-based practices (EBP), little research has studied how managers lead contract-based human service delivery. A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination (i.e., structuring cross-sector services, coordinating client referrals and eligibility, overseeing EBP implementation) and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning. In conclusion, we underscore the organizational and managerial dimensions of contract-based service delivery.</t>
@@ -20664,6 +21044,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G413" t="inlineStr">
         <is>
           <t>This article explores service learning via the lens of activity theory. Through this lens, it is identified as a form of ‘boundary work’ in higher education, with educators identified as ‘boundary workers’. Drawing on the data from a recent study, this paper analyses service learning as an often contradictory and tension filled practice. The ‘expanded community’ and ‘dual but interrelated object’ in the service learning activity system result in many tensions for students and community members alike. This in turn poses significant challenges for boundary workers, and ultimately for the university. The paper concludes by arguing that in order to encourage and value service learning, we need to acknowledge the (new and different) knowledge, values and skills required for playing the role of boundary worker in (boundary) practices such as this.</t>
@@ -20691,7 +21076,7 @@
       </c>
       <c r="P413" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Qualitative study exploring service learning without any effect sizes, using a non-employee (student and community member) sample [Code 1 &amp; Code 2].. Verbatim Evidence: [Abstract] "This article explores service learning via the lens of activity theory. Through this lens, it is identified as a form of ‘boundary work’ in higher education, with educators identified as ‘boundary workers’." [Methodology] "By the nature of the questions and issues that guided my thinking, I was drawn to undertaking a qualitative study." [Methodology] "interviews with academics and educators involved in the two courses; interviews with community members (more informally); and student reflective journals."</t>
         </is>
       </c>
     </row>
@@ -20763,6 +21148,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>The purpose of this research is to determine the description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, to determine and analyze the influence of Emotional Dissonance on Service Sabotage, to determine and analyze the influence of Emotional Intelligence on Service Sabotage, and to determine and analyze the influence of Emotional Exhaustion on Service Sabotage. The population in this study were all employees of the Grand Mercure Hotel Kemayoran Jakarta. In this research, a quantitative method approach was used with a survey and a sample of 225 people was obtained using a purposive sampling technique. Survey research is carried out by distributing questionnaires. Previously, the questionnaire was tested for validity and reliability first. The data analysis technique in this research uses descriptive analysis and linear regression analysis. Description of the employees of the Grand Mercure Hotel Kemayoran Jakarta, most of whom are male, most employees are under 35 years old, and most employees have worked at the hotel for 0-2 years. The results of this research explain that Emotional Dissonance has a positive and significant effect on Service Sabotage with p-value of 0.012. Emotional Intelligence has a negative and significant effect on Service Sabotage with p-value of 0.023. Emotional Exhaustion has a positive and significant effect on Service Sabotage with p-value of 0.045.</t>
@@ -20810,6 +21196,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -20837,7 +21228,7 @@
       </c>
       <c r="P416" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Non-individual level analysis (data aggregated to directed unit dyads). Verbatim Evidence: [Aggregation to dyad level] "To model boundary spanners’ impact on intergroup knowledge integration, we aggregated boundary spanners’ metaknowledge and proactivity to the inter-unit level (Chan, 1998; Klein and Kozlowski, 2000)." [Correlation matrix N] "Note: N = 462 directed unit dyads."</t>
         </is>
       </c>
     </row>
@@ -20857,6 +21248,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>Intergroup knowledge integration, that is the acquisition, processing, and utilization of knowledge across group boundaries, is a critical source of competitive advantage in modern organizations. Prior research has highlighted the important role of boundary spanning knowledge exchange for intergroup knowledge integration, neglecting, however, the question of what makes individual boundary spanners more effective in fostering intergroup knowledge integration. Integrating boundary spanning literature with theories of group information processing, we hypothesize that the effect of individual boundary spanning ties on intergroup knowledge integration depends on the boundary spanners’ levels of metaknowledge, i.e., knowledge of who knows what in their respective groups, and proactivity. We find general support for our predictions in a study of 457 engineering consultants nested in 22 interdependent business units within an organization. Additional criterion analyses confirm the material importance of intergroup knowledge integration for group performance. Our findings have implications for literatures on intergroup effectiveness, team cognition, and proactivity.</t>
@@ -20951,7 +21343,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr"/>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G419" t="inlineStr">
         <is>
           <t>Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their boundaries in ways that complement their preferences.</t>
@@ -20979,7 +21375,7 @@
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t xml:space="preserve">The study focuses on work-family/work-life role segmentation preferences and boundary management between work and home domains, rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: </t>
+          <t>Multiple reasons [Code 1 &amp; Code 2]: The paper measures Work-Family boundary management rather than inter- or intra-organizational boundary spanning behavior. Additionally, Study 2 utilizes an undergraduate student sample.. Verbatim Evidence: [Abstract] "Purpose We examine the bi-directional nature of role segmentation preferences—preferences to protect the home domain from work intrusions, and to protect the work domain from home intrusions—and hypothesize that the dimensions independently prompt individuals to manage their bound aries in ways that complement their preferences." [Study 2 Method Overview] "Respondents included 1253 undergraduate students from two sections of a management course at a university in the Southeastern United States."</t>
         </is>
       </c>
     </row>
@@ -20999,6 +21395,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>Background Increasing role complexity has intensiﬁed the boundary spanning functions of managers. Because work demands and scope vary by management position, time in staff contact rather than span may better explain managersÕ capacity to support staff. Methods A descriptive, correlational design was used to collect cross-sectional survey and prospective work log and administrative data from a convenience sample of 558 nurses in 51 clinical areas and 31 front-line nurse managers from four acute care hospitals in 2007–2008. Data were analysed using hierarchical linear modelling. Results Span, but not time in staff contact, interacted with leadership and operational hours to explain supervision satisfaction. Conclusions With compressed operational hours, supervision satisfaction was lower with highly transformational leadership in combination with wider spans. With extended operational hours, supervision satisfaction was higher with highly transformational leadership, and this effect was more pronounced under wider spans. Implications for Nursing Management Operational hours, which inﬂuence the managerÕs daily span (average number of direct report staff working per weekday), should be factored into the design of front-line management positions.</t>
@@ -21145,6 +21542,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>Background: Emotions play a central role in how employees respond to workplace bullying, influencing both their well-being and organizational outcomes. The purpose of the current study was to examine how workplace bullying and turnover intention are related to negative emotions and workplace unfairness. Methods: The research involved collecting data from 269 boundary-spanning bank workers (call center workers, frontline office staff, and customer service representatives) who experienced bullying. A moderated mediation was tested using Model 7 of the Process macro. The relationship between workplace bullying and turnover intention was analyzed, emphasizing the moderating effect of workplace unfairness and the mediating role of negative emotions. Results: The results validated the model, showing that an increase in negative emotions and workplace unfairness promotes the link between workplace bullying and the intention to leave. Increased negative emotions and perceived workplace unfairness amplified the relationship between workplace bullying and turnover intention. Conclusions: The findings underscored the cumulative risk of bullying environments for employee well-being and retention, providing practical recommendations for HRM and leadership strategies to cultivate healthier, more inclusive workplace settings. This study adds to the bullying–turnover literature by examining the joint role of negative emotions and workplace unfairness in a moderated mediation framework. The study connects these findings to sustainable labor management, emphasizing both theoretical and practical implications for organizations.</t>
@@ -21239,6 +21637,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>Abstract             In organizational contexts, professional boundaries serve a dual purpose by distinguishing various professions from one another and regulating access to power, status, and rewards. Individuals operating within professions in which such boundaries are not clearly or explicitly defined face the risk of compromising their status and autonomy. However, they possess the agency to actively define their profession and enhance its standing among both internal and external stakeholders. This study explores how homeroom teachers in the Israeli education system—recognized as a distinct occupation within the broader teaching profession—engage in boundary work to form and define their professional group. Our findings reveal that (1) homeroom teachers employ adaptable boundary work strategies, tailored to their interactions with different key stakeholders. Specifically, they (a) define boundaries to clarify, for themselves, the parameters of their own roles; (b) balance boundaries with partners inside the school (administrators and subject teachers) to facilitate day-to-day collaboration while simultaneously asserting their own roles; and (c) orchestrate boundaries when interacting with external partners (students’ parents), acknowledging the distinction between roles while primarily seeking to foster effective joint work towards the common goal of helping students succeed. (2) Despite the diversity in their approaches, all homeroom teachers exhibit a unique expertise, allowing them to combine boundary-setting with inclusivity, highlighting the dynamic and interactive nature of the boundary work process. This dual nature enhances the effectiveness of communication and collaboration within the educational system, molding the role of homeroom teachers as a distinct professional group.</t>
@@ -21286,6 +21685,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G426" t="inlineStr">
         <is>
           <t>Recent research has emphasized cross functional integration as a key facilitator of success in new product development (NPD) projects. This dissertation developed and tested a model using supply chain integration as a key enabler influencing both planning of the new product and execution of the development process in NPD projects. Supply chain integration was operationalized to include cross functional (for example, between design and manufacturing) and boundary spanning integration mechanisms (such as supplier integration). Product concept effectiveness (a construct capturing the planning of the new product), and development process performance (a construct measuring the execution of new product development process) were theorized to influence overall project success. Hypotheses drawn from this framework were tested on a multi-industry sample (electronics, communications, semiconductors, and computers) of firms. Data analysis was conducted using regression analyses, partial correlations, confirmatory factor analyses and structural equation modeling.</t>
@@ -21313,7 +21717,7 @@
       </c>
       <c r="P426" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Project-level analysis measuring team/firm-level integration practices via a key informant, not individual-level boundary spanning behavior.. Verbatim Evidence: [Research Methods] "The unit of analysis for this research was a new product development project. Firms from a variety of industries were selected in order to test for contingency relationships across different settings. Data collection was conducted using a survey instrument. The ideal respondent for the survey was specified to be “the person with overall responsibility for overseeing product development projects”." [Appendix A: Survey Instrument] "The following questions ask about the different practices used by your company in supplier integration, design-manufacturing integration, customer integration, and concurrent process management."</t>
         </is>
       </c>
     </row>
@@ -21365,7 +21769,7 @@
       </c>
       <c r="P427" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 3] No extractable correlation matrix and project-level unit of analysis.. Verbatim Evidence: [Unit of Analysis] "Since the unit of analysis in Hypothesis 4 is the project, individual responses must be pooled to get project scores." [Project Performance] "Each was asked to evaluate the overall technical performance of all projects with which he was technically familiar." [RESULTS] "To test for the existence of gatekeepers (Hypothesis 1), organizational liaisons (Hypothesis 2), and laboratory liaisons (Hypothesis 3), the amount of external communication of stars and nonstars must be compared."</t>
         </is>
       </c>
     </row>
@@ -21464,7 +21868,7 @@
       </c>
       <c r="P429" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Project-level analysis (N = innovation projects) rather than individual-level.. Verbatim Evidence: [Organization Sample] "Forty Belgian companies cooperated in this study." [Organization Sample] "Within each field site, we studied the most recent failure and the most recent success." [Organization Sample] "We examined seventy-eight innovation projects in forty companies: forty successes and thirty-eight failures." [Construct Validity] "The results in Table 1 justify the use of the pooled perceptions by R&amp;D and marketing regarding project centralization and formalization, interfunctional climate, and commercial project success." [External Validity] "The unit of analysis here is the project." [Table 2 Note] "The number of observations varies between 62 and 69."</t>
         </is>
       </c>
     </row>
@@ -21484,6 +21888,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
           <t>Urban metabolism approaches are increasingly becoming relevant in providing pathways to sustainable development. The ways through which urban green infrastructures are planned and designed can influence resource flows in cities. Yet, little is known about the agency and contributions of landscape architects and spatial planners as curators of urban greenery, in facilitating circular resource flows, and accelerating the transition to a circular economy. This paper offers an empirical inquiry into the understanding and use of metabolic approaches in spatial planning and design practices. Through a multi-method approach and the use of boundary spanning as an analytical lens, we identify different modes of agency of spatial practitioners in enhancing resource efficiency across the life stages of urban landscape projects. Results show that while the ‘urban metabolism’ concept is not widely used by practitioners, its relevance to planning and designing green infrastructure for sustainable resource flows is well understood. Additionally, we highlight existing barriers including policy constraints in engaging with metabolic approaches and offer recommendations to facilitate a resource-sensitive turn in planning and designing urban landscapes. This study highlights important contributions of design practice to an expanding discourse of urban metabolism, including policy reforms for enabling circular resource flows in cities.</t>
@@ -21531,11 +21936,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr">
-        <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
-        </is>
-      </c>
+      <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
           <t>Investigates performance relationships for interfunctional process integration and specific logistics interface capabilities. The results indicate that competitive advantage is more likely to emanate from interfunctional process integration rather than individual function (sub) optimization. Logistics’ unique role as a boundary spanning interface between marketing, production, and new product development, is also identified as a potential source of competitive advantage. In terms of overall business performance, logistics followed by new product development are shown to have the greatest impact on profitability and growth. Further, logistics interface capabilities of customer service and logistics quality have the greatest independent impacts on business performance. In total, these results imply that logistics, new product development, and demand‐management capabilities may provide firms with that extra competitive edge which shows up in “bottom‐line” performance. States that the relatively neglected areas of logistics boundary spanning and production customer service also deserve attention.</t>
@@ -21563,7 +21964,7 @@
       </c>
       <c r="P431" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 3] Firm-level analysis of organizational logistics and functional capabilities rather than individual-level boundary spanning behavior.. Verbatim Evidence: [Methodology] "The present research is concerned with interfunctional process relationships, specific boundary-spanning interface relationships, and overall business performance relationships." [Subjects and sample] "The subjects consisted of the CEOs from 65 furniture manufacturing firms." [Business performance indicator variables] "To measure overall business performance, data were collected on subject firms for five business performance indicators. The five financial performance ratios consisted of return on assets (ROA), return on investment (ROI), return on sales (ROS), and the two growth ratios of ROI growth and ROS growth."</t>
+          <t xml:space="preserve">The study analyzes data at the firm level, using CEOs as key informants to evaluate firm-level functional capabilities (logistics, production, marketing) and business performance, rather than measuring individual-level interpersonal boundary spanning behavior.. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -21615,7 +22016,7 @@
       </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 2] The study measures emotional labor (surface vs. deep acting) rather than boundary spanning behavior, and uses a sample of general consumers rather than organizational employees.. Verbatim Evidence: [Code 1 &amp; Code 2]. Verbatim Evidence: "[Abstract] Success in the restaurant industry is, in part, determined by boundary spanning service providers’ ability to manage their emotions with the goal of providing excellent service while simultaneously authentically displaying the proper emotions to connect with the guest." "[Design] Three dichotomous variables (gender, emotional labor and service quality) were the independent variables in this between-subjects quasi-experimental design." "[Data collection] For the full study, a market research firm (Qualtrics) was enlisted to recruit, disseminate, and collect the results of the electronic survey. There were only two requirements for participation: prospective samples must have been at least 18 years of age as well as having dined in a full-service restaurant in the previous 1 year."</t>
         </is>
       </c>
     </row>
@@ -21635,7 +22036,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F433" t="inlineStr"/>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G433" t="inlineStr">
         <is>
           <t>The management of quality and development of effective cross-functional cooperation have assumed a new strate gic importance over the past decade. However, many com panies have reported that quality strategies have failed to deliver anticipated performance benefits and that ineffec tive interfunctional relationships may be to blame. This study explores marketing-quality interfunctional relation ships as a potential source of quality strategy implemen tation failure at the strategic business unit (SBU) level. This study focuses on interdepartmental connectedness, communication and conflict between marketing and qual ity, and the antecedents and consequences of these dimen sions of interfunctional interaction. Using data from a pooled response mail survey, the results suggest that mar keting-quality interactions are associated with senior management quality leadership, strategic quality plan ning process, and control system characteristics. Inter-functional interactions between marketing and quality are found to be only weakly related to relative quality, market performance, and financial performance outcomes.</t>
@@ -21663,7 +22068,7 @@
       </c>
       <c r="P433" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Multiple flaws [Code 1 &amp; Code 3]: SBU-level analysis (N=SBUs) measuring mere communication frequency.. Verbatim Evidence: [Measurement] "Subsequently, the data from each of the respondents in an SBU were averaged to form a single unit of data for each construct." [Measurement] "Interdepartmental communication frequency is conceptualized in terms of information flows through different communication media (Moenaert and Souder 1990; Van de Ven and Ferry 1980)." [Appendix] "Interdepartmental Communication Frequency (7-point scale with never/very frequently anchors) Individual face-to-face contact Meetings between teams Telephone calls Written memos and reports Electronic maila"</t>
         </is>
       </c>
     </row>
@@ -21683,6 +22088,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G434" t="inlineStr">
         <is>
           <t>Boundary spanning research is increasing recognition among scholars and policymakers due to its potential in generating novel and breakthrough scientific contributions. However, while previous research mainly investigated its effect for the scientific domain, less is known about how boundary spanning approaches in science are related to technology transfer activities. To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council under the 7th Framework Programme and Horizon 2020 Programme in the period 2008–2016. Our results show that boundary spanning research projects and the probability to generate technological impact through patent citations are linked through an inverted U-shape relation, thus recognizing both benefits and costs to this research approach. Moreover, as research integrates knowledge from more diverse scientific domains, its technological applications expand correspondingly across a broader range of technical fields. Finally, we show that these relations change according to the seniority of the researcher performing the scientific activity.</t>
@@ -21710,7 +22120,7 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Bibliometric and project-level analysis [Code 2 &amp; Code 3]. Verbatim Evidence: [Bibliometric and project-level analysis]. Verbatim Evidence: "[Abstract] To investigate this issue, we examine 6081 research projects in the Life Sciences, Physical &amp; Engineering, and Social Sciences &amp; Humanities sectors funded by the European Research Council under the 7th Framework Programme and Horizon 2020 Programme in the period 2008–2016." "[5.2. Measures] We calculated this variable as the total number of unique subject areas of all the backward citations reported in the publications of each project."</t>
         </is>
       </c>
     </row>
@@ -21762,7 +22172,7 @@
       </c>
       <c r="P435" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Excluded due to multiple flaws: the study uses an undergraduate student sample (Code 2) and the unit of analysis is the multiteam system (MTS) level, with n=64 (Code 3).. Verbatim Evidence: [Code 2 &amp; Code 3]. Verbatim Evidence: "[Participants] Undergraduate psychology and business students (N = 384) from a large Southeastern United States university participated in the current study." "[Participants] A total of 64, identically-structured MTSs participated in a laboratory simulation designed to model an MTS situation requiring high levels of interdependence and between-team coordination." "[Results] Note. LT = Leadership Team; CT = Component Team; n varies from 57 to 64."</t>
         </is>
       </c>
     </row>
@@ -21933,6 +22343,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
           <t>Purpose – Literature on small and medium enterprises (SMEs) has so far produced limited evidence on how these firms pursue their organizational flexibility with information and communication technology (ICT) and ad hoc work practices. The purpose of this paper is to contribute to the extant literature by focusing on how SMEs use flexible work practices that provide latitude with respect to when employees work, where they work and via which communication medium. Specifically, the authors analyze how such practices are related to the conditions that SMEs face in reference to their competitive environment and their patterns of ICT usage.</t>
@@ -21980,6 +22391,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G440" t="inlineStr">
         <is>
           <t>Business Process Reengineering (BPR) was developed as a new idea which, it was suggested, could revolutionise the corporation and give it a major competitive advantage by simplifying key business processes and utilising information technology to secure cross-functional communication and focus on customer requirements. Rather than continue the debate about whether BPR is ‘good’ or ‘bad’, ‘old’ or ‘new’ (e.g. Earl, M.J., 1994. The new and the old of business process redesign. Journal of Strategic Information Systems 3 (1), 5–22; Mumford, E., 1994. New treatments or old remedies: is business process reengineering really socio-technical design. Journal of Strategic Information Systems 3 (4), 313–326), the focus here is on understanding how the concept ‘BPR’, however deﬁned, has been diffused across European ﬁrms. The results from a survey of ﬁrms in four countries support previous research on the diffusion process with the rate of adoption of BPR related to microorganisational level variables—characteristics of the ﬁrm and the boundary spanning activities of individual members. In addition there were differences across industry sectors and across countries in the extent of adoption of BPR. It is argued that attention to these meso-industry level and macro-national level factors, as well as the micro-organisational level dynamics, will improve our understanding of the relationship between networking and innovation processes. In particular, the paper focuses on how networking activity can be restrictive and lead to the creation of fashions which limit the extent of organisational learning during BPR adoption. q 1999 Elsevier Science B.V. All rights reserved.</t>
@@ -22007,7 +22423,7 @@
       </c>
       <c r="P440" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 3] No correlation matrix reported (unextractable effect sizes) and firm-level unit of analysis.. Verbatim Evidence: [2. Method] "The survey asked respondents to indicate from a list of technologies those that had been adopted in their own organisation (e.g. TQM, MRP2, JIT)." [2. Method] "This methodology provides information about a firm from the perspective of one organisational employee only." [3. Results] "In the analyses below, independent sample t-tests and chi-squares analyses are used as appropriate to compare firms where BPR had been adopted, with firms where it had not been adopted." [Table 1] "Professional networks 2.27 2.18 NS" [Table 1] "Supply chain networks 3.39 3.39 NS"</t>
         </is>
       </c>
     </row>
@@ -22022,6 +22438,16 @@
           <t>BSMA0438</t>
         </is>
       </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G441" t="inlineStr">
         <is>
           <t>This exploratory study examined the practice of public relations in Zimbabwe by surveying and understanding public relations roles typically practiced by Zimbabwean PR practitioners. Through the lens of systems theory, the research investigated whether the practiced public relations roles allow organizations to perform all three boundary spanning functions such as output, throughput, and input. The results confirmed prior theoretically and empirically derived typology of roles (technician, manager, strategist) from the African continent. However, the observed structures of public relations roles deviate from previous findings, indicating that Zimbabwean PR practitioners’ professional roles may differ from those in neighboring countries.</t>
@@ -22045,6 +22471,11 @@
       <c r="K441" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -22158,7 +22589,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F444" t="inlineStr"/>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G444" t="inlineStr">
         <is>
           <t>Horizontal arrangements are increasingly deployed in organizational networks, yet research has rarely examined the effectiveness of these alliances. The coalition of disparate corporate cultures yields appreciable levels of role stress for people in boundary-spanning positions. Dedicated assets and communication modality are factors that influence the level of role ambiguity and conflict. The authors implicate these facets of role stress as antecedents to four forms of effectiveness drawn from the competing values framework. The authors present alternative perspectives that examine the relationship between stress and performance. The received view frames role stressors as linear, negative antecedents to organizational outcomes. The authors contrast this perspective with theories that espouse triphasic, parabolic, and interactive influences of stressors on organizational outcomes. Data gathered with 218 managers of dual-branded retail oil outlets indicate that the relevance of these alternative perspectives is mitigated by the form of effectiveness pursued by the organization. The results support a linear relationship between role conflict and bargaining efforts, yet they also offer evidence of nonlinear influences of role ambiguity on contributions to sales, customer satisfaction, and competence. The study concludes with a discussion of relevance of the findings to the management of horizontal alliances and to interorganizational theory.</t>
@@ -22186,7 +22621,7 @@
       </c>
       <c r="P444" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>The study measures the role stress (role ambiguity and role conflict) of personnel in boundary-spanning positions and its effects on performance outcomes, but it does not quantitatively measure Boundary Spanning Behavior (BSB) itself.. Verbatim Evidence: [Abstract] "The coalition of disparate corporate cultures yields appreciable levels of role stress for people in boundary-spanning positions. Dedicated assets and communication modality are factors that influence the level of role ambiguity and conflict. The authors implicate these facets of role stress as antecedents to four forms of effectiveness drawn from the competing values framework." [Measures] "Role stress . The role stress scales were based on the seven-point measures developed by Rizzo, House, and Lirtzmann (1970). The conflict and ambiguity measures consisted of six and seven items, respectively."</t>
         </is>
       </c>
     </row>
@@ -22455,6 +22890,16 @@
           <t>BSMA0447</t>
         </is>
       </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G450" t="inlineStr">
         <is>
           <t>This study examines how cultural performance orientation moderates the influence of human resource management (HRM) controls on boundary-spanning employees' behavioural strategies and satisfaction. Based on primary data obtained from 1049 salespeople in six countries (France, Ireland, Italy, Spain, United Kingdom, and the United States of America) and secondary data on cultural performance orientation, multilevel regression analyses show that national culture has a strong effect on the way boundary-spanning employees allocate their effort in response to HRM control. In particular, our results suggest that the more behaviour controls are used with boundary-spanning employees, the less attention they pay to customers and the more emphasis they place on their supervisors and non-selling tasks. Specifically, cultural performance orientation is shown to moderate significantly those relationships. Furthermore, results indicate that cultural performance orientation heightens boundary-spanning employees' job satisfaction resulting from behaviour control. Preliminary explanations for the differing impact of HRM control efficiency across cultures can be proposed.</t>
@@ -22478,6 +22923,11 @@
       <c r="K450" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P450" t="inlineStr">
+        <is>
+          <t>Measures percentage of time allocated to customers/supervisors rather than purposive boundary spanning behavior.. Verbatim Evidence: [Measures and psychometric properties] "The three facets of behavioural strategies (i.e., focus on the supervisor, the customer and the administrative aspects of the job) were each measured by the percentage of time the salesperson devotes to supervisors, customers and administrative tasks respectively." [Data collection and sample] "Our primary data came from salespeople working in six countries (France, Ireland, Italy, Spain, United Kingdom and the United States of America) and four industrial sectors (healthcare and pharmaceutical, information systems and technology, fast moving consumer goods, and industrial goods)."</t>
         </is>
       </c>
     </row>
@@ -22652,6 +23102,16 @@
           <t>BSMA0451</t>
         </is>
       </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G454" t="inlineStr">
         <is>
           <t>Committed customers are proﬁtable to an organization for the long term. Customer commitment forms when a customer’s expectation is satisﬁed and the customer realizes fair value from his/her relationship with the organization. From an organization’s perspective, this value reﬂects customer equity, but from a customer’s perspective, it represents the customer’s perceived value of the relationship. In order to manage such a relationship successfully, it is necessary to support diverse customer information – such as of-the-customer, for-the-customer, and by-the-customer information. A customer information system (CIS) plays the role of boundary spanning that manages and distributes customer information. But the gap between marketing and IT strategy is a barrier in implementing a successful CIS. The CIS, which includes the database, communication channel, and decision model for relationship management, should be designed to facilitate the two-way customer relationship exchanges. This paper develops a framework of dynamic customer relationship management, suggests the information technology strategy to support the framework, and illustrates the applicability of such framework and strategy through a real business case.</t>
@@ -22675,6 +23135,11 @@
       <c r="K454" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P454" t="inlineStr">
+        <is>
+          <t>Qualitative case study without effect sizes. The study develops a conceptual framework for CRM and uses qualitative interviews. The 'boundary-spanning' role refers to a Customer Information System (CIS), not individual employee behavior.. Verbatim Evidence: [Abstract] "A customer information system (CIS) plays the role of boundary spanning that manages and distributes customer information." [Study approach] "In this case study, data was collected by the following steps, First, to understand the entire corporate information system environment, we referred to the enterprise information system planning reports that include overall specifications of hardware, software, human resources, and business processes, and gathered information on how the case firm started and managed their customer relationship management activities." [Study approach] "Then we conducted several in-depth interviews with senior managers of the marketing, customer service, and information system divisions."</t>
         </is>
       </c>
     </row>
@@ -22689,6 +23154,16 @@
           <t>BSMA0452</t>
         </is>
       </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G455" t="inlineStr">
         <is>
           <t>Abstract             How do boundary spanners, through processes of temporal sensemaking, use established and newly forming relationships to create value in science‐based SMEs? In addressing this question, we examine the creation of social capital arising from the activities that boundary spanners use in establishing ‘ties that bind’ people together. We show how effective boundary‐spanning activities are able to promote collaborations across scientific and related disciplines, supporting knowledge generation and innovation. Sensemaking is central to this process. We illustrate how retrospective sensemaking draws on knowledge, skills and experiences, often triggered through historical connections and personal contacts, whilst prospective sensemaking often arose in the search for new customers and in the ongoing assessment of future potential markets. We reveal how combining individual and collective boundary spanning with a continual movement between the backward glance (retrospective) and more future‐oriented (prospective) sensemaking was particularly effective in generating new understandings and opportunities. We use our findings to present an inductive model of value creation that frames the dynamic interplay between individual and collective boundary‐spanning activities and temporal sensemaking in the generation of social capital that acts as a knowledge resource for identifying and evaluating ideas for innovation and future pathways to value creation.</t>
@@ -22712,6 +23187,11 @@
       <c r="K455" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P455" t="inlineStr">
+        <is>
+          <t>Qualitative study with no extractable quantitative effect sizes (no correlation matrix).. Verbatim Evidence: [Methodology] "This study draws on data from qualitative fieldwork, allowing an in-depth exploration of the phenomenon of interest. Semi-structured interviews provided the flexibility to gather rich data essential to answering our research question." [Methodology] "Data analysis utilizes a grounded theory approach using first and second-order coding to present our findings (Strauss and Corbin, 1990)." [Methodology] "We conducted 23 in-depth interviews with a range of individuals in the seven companies (Table 3)."</t>
         </is>
       </c>
     </row>
@@ -22726,6 +23206,16 @@
           <t>BSMA0453</t>
         </is>
       </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G456" t="inlineStr">
         <is>
           <t>In this editorial for our special issue on interorganizational collaboration (IOC), we position collaborative action in the context of the concurrent global crises that necessitate the bridging of interests, positions, competencies, and resources. We unpack the notion of IOC in terms of its conditions, phases, practices, and dynamics, and provide an overview of how the contributing authors support such understanding of cross-boundary collaboration. Through their action-oriented approaches to research and learning, they show a promising interplay of insight and impact. We underline their search for impact and aim to reinforce the potential of IOC not just to be successful, but also highly meaningful to address grand challenges. We therefore take a normative stance and describe how the intertwined notions of justice, resilience, and thriving can serve as a compass to legitimize, organize, facilitate, assess, and study IOC as an important pathway for the co-creation of a better world.</t>
@@ -22749,6 +23239,11 @@
       <c r="K456" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P456" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] Non-primary study (editorial) lacking empirical data and effect sizes.. Verbatim Evidence: [Introduction] "In this editorial for our special issue on interorganizational collaboration (IOC), we position collaborative action in the context of the concurrent global crises that necessitate the bridging of interests, positions, competencies, and resources." [Introduction] "To place the papers included in this special issue in context, we ﬁrst describe the basic concepts and approaches that constitute IOC as a ﬁeld of study."</t>
         </is>
       </c>
     </row>
@@ -22837,6 +23332,16 @@
           <t>BSMA0456</t>
         </is>
       </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G459" t="inlineStr">
         <is>
           <t>We present a view of trust in boundary spanners as explained by the extent of role autonomy, a multidimensional concept that reflects the discretion that agents have in interpreting and enacting their roles. We argue that, in a buyer-supplier context, purchasing managers will be trusted to a greater extent by supplier representatives when they are free from constraints that limit their ability to interpret their boundary-spanning roles. We conceptualize and measure three key components of role autonomy: Functional influence, tenure, and clan culture. Taken together, these components of role autonomy shape and define the purchasing manager's willingness and capacity to make and uphold commitments to supplier representatives. Role autonomy permits purchasing managers to engage in discretionary behaviors that allow supplier representatives to leam about their underlying motives and intentions. We test hypotheses linking the components of role autonomy to trust on a sample of 119 buyer-supplier relationships. We use a dyadic research design that combines data from purchasing managers and supplier representatives. The results suggest that granting purchasing managers greater autonomy enhances supplier representative trust in purchasing managers. By drawing attention to role autonomy as a feature of organizations that influences trust we highlight the importance of organizational context in contributing to a deeper understanding of trust.</t>
@@ -22860,6 +23365,11 @@
       <c r="K459" t="inlineStr">
         <is>
           <t>2003</t>
+        </is>
+      </c>
+      <c r="P459" t="inlineStr">
+        <is>
+          <t>Does not measure Boundary Spanning Behavior (measures trust, role autonomy, and mere communication frequency).. Verbatim Evidence: [Abstract] "We test hypotheses linking the components of role autonomy to trust on a sample of 119 buyer-supplier relationships." [Measures] "Trust in the Purchasing Manager. We developed a measure of the supplier representative's trust in the purchasing manager based on a measurement instrument of trust in close, interpersonal relations, created and validated by Rempel et al. (1985)." [Table 1] "Frequency of communication / On average, about how often did you use the following to communicate with your contact person during the past year? / 1. Telephone / 2. Fax / 3. Scheduled meetings / 4. Unscheduled meetings / 5. E-mail"</t>
         </is>
       </c>
     </row>
@@ -22874,6 +23384,16 @@
           <t>BSMA0457</t>
         </is>
       </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G460" t="inlineStr">
         <is>
           <t>Opportunism is a common issue in inter – firm relationships, which increases transaction costs, impairs firm performance and supply chain efficiency, and deteriorates relationship quality. Previous studies have intensively investigated factors influencing opportunism but overfocusing on the organisational level. Recently, supply chain researchers have called for identifying factors influencing opportunism at the individual level to gain a more comprehensive understanding of opportunism. Based on transaction cost theory, resource dependence theory, and boundary spanning theory, this study seeks to advance the emerging research stream on opportunism at the individual level by investigating how buyer agents’ boundary spanning capabilities and firms’ long – term relationship orientation can help manage supplier agents’ opportunism. Using a cross – sectional data set of 406 buyer agents from manufacturing companies collected from February to April 2021 in Japan, we tested a set of hypotheses through regression and conditional process analyses. Our findings suggest that buyer agents’ strategic communication and firms’ long – term relationship orientation are critical factors that reduce supplier agents’ opportunism.</t>
@@ -22897,6 +23417,11 @@
       <c r="K460" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P460" t="inlineStr">
+        <is>
+          <t>The study provides a valid employee sample (N=406 purchasing staff) and measures individual-level boundary spanning behaviors (strategic communication and compromise capability) with zero-order correlations reported.. Verbatim Evidence: [Abstract] "Using a cross-sectional data set of 406 buyer agents from manufacturing companies collected from February to April 2021 in Japan, we tested a set of hypotheses through regression and conditional process analyses." [Methodology] "The target participants in the survey were purchasing staff in the sales and planning sections of manufacturing companies in Japan responsible for business activities with suppliers." [Measures] "Buyer agents' BSC measures were adapted from Zhang et al. (2011)." "The three items of strategic communication capability measured a buyer agent's effectiveness in conveying their firm's purchasing plans and strategies to the supplier firm"</t>
         </is>
       </c>
     </row>
@@ -23259,6 +23784,16 @@
           <t>BSMA0467</t>
         </is>
       </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G470" t="inlineStr">
         <is>
           <t>This study constructs a theoretical model to test and prove that organizational forgetting influences cross-boundary innovation and testifies to the moderating role of Institutionalized organizational mission in the said relationship. Data was collected through a convenient sampling technique from 353 middle and senior managers of entrepreneurial enterprises in China through online and offline modes. Additionally, we used confirmatory factor analysis, multiple regression, and bootstrap analysis to verify hypotheses using Analysis of a moment structures and Statistical Package for the Social Sciences latest versions. The results show that organizational forgetting has a significantly positive impact on cross-boundary innovation and binary knowledge sharing plays a mediating role in the relationship between organizational forgetting and cross-boundary innovation. Moreover, the mediating effect of exploitative knowledge sharing on the relationship between organizational forgetting and cross-boundary innovation is more substantial than exploratory knowledge sharing. This study separates the impact mechanism of exploitative and exploratory knowledge sharing as a mediator unanimously and proves that Institutionalized organizational mission has a significant moderating role in the relationship between organizational forgetting and cross-boundary innovation. This research offers significant implications for Chinese enterprises to bolster cross-boundary innovation to achieve growth.</t>
@@ -23282,6 +23817,11 @@
       <c r="K470" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P470" t="inlineStr">
+        <is>
+          <t>Firm-level analysis using key informants (Code 3) and lacks individual Boundary Spanning Behavior construct (Code 1).. Verbatim Evidence: [Research samples] "This research is about learning and innovation at the enterprise level. Therefore, middle and senior managers and members of the innovation team who are familiar with the overall situation of the enterprise are selected as respondents." [Appendix 1] "CBI1. The firm often introduces elements from different fields to improve the operating conditions of related businesses"</t>
         </is>
       </c>
     </row>
@@ -23333,6 +23873,16 @@
           <t>BSMA0469</t>
         </is>
       </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G472" t="inlineStr">
         <is>
           <t>How do leaders of established organizations effectively manage intrafirm entrepreneurial groups so that they can be successful? Focusing on drivers of breakthrough groups’ performance and radical innovation, this research identifies drivers and proposes a multifaceted model providing a pathway for breakthrough business growth in an organically driven mode. The corporate entrepreneurship (CE) and innovation management literature, while helpful in describing the difficulty associated with leading CE and ambidextrous organizations, are focused on wider structural or behavioral solutions to address ambidexterity challenges and product innovation, omitting the unit of analysis—the group/team—and the drivers that influence groups’ breakthrough innovation and performance aims in a contemporary context in which organizations’ business models can change in the blink of an eye. Using a QUAN→ qual design, the research follows aninside-out logic’to account for the position of each introduced construct in the nomological network, which include (1) intragroup mechanisms;(2) team boundary mechanisms (boundary buffering and spanning);(3) environmental mechanisms including senior management communication, incentives, proactive IT stance; and,(4) contextual influences. The prevalence of a mismatch between conventional incentives vis-a-vis team members’ breakthrough pursuits is also investigated. Findings reveal a paradox around top management communication, as well as the mediating roles of team buffering and spanning on the relationship between relational climate and outcome variables, radical innovation, and team performance. Overall, results suggest that that just having a top team (ie, good relational climate) is not enough for breakthrough performance, and could be for naught should the team’s boundaries not be managed by leaders as to create buffering (from extra-team interference) and spanning (or access to resources) beyond the team. Environmental mechanisms, and particularly proactive IT capabilities and nuanced senior management communication, also matter when it comes to teams’ success. It is hoped that this work, comprising novel constructs and a unique team focus in the context of breakthrough innovation and corporate entrepreneurship, will help drive the two streams of research into new directions.</t>
@@ -23356,6 +23906,11 @@
       <c r="K472" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>Non-individual level (team level analysis). Verbatim Evidence: [Unit of Analysis] &lt;My unit of analysis is the entrepreneurial group pursuing radical innovation initiatives, as previously discussed. More specifically, it includes cross-functional groups participating in non-incremental initiatives within an established company or organization.&gt; [Examples of Groups] &lt;The 252 respondents surveyed serve on 184 groups within 181 mid- to large-size organizations.&gt; [SEM Aggregated] &lt;Of the 252 respondents, 81 cases belonging to 13 groups were aggregated for structural equation modeling (SEM). The 13 aggregated cases were added to the data set, while 81 individuals belonging to the groups were deleted from the data set for SEM Analysis, for a sample of n=184.&gt;</t>
         </is>
       </c>
     </row>
@@ -23704,6 +24259,16 @@
           <t>BSMA0477</t>
         </is>
       </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G480" t="inlineStr">
         <is>
           <t>Examined relationships between major role requirements and experienced role stress, using data from 202 research and development professionals. Measures (including those of JR Rizzo et al, 1970) of role stress included various types of role conflict and ambiguity. Role requirements included integration and boundary-spanning activities, personnel supervision, and scientific research. Role conflict was more sensitive than role ambiguity to differences in research and development role requirements; and integration and boundary-spanning activities were the best predictors of experienced role conflict, especially of the intersender variety.</t>
@@ -23727,6 +24292,11 @@
       <c r="K480" t="inlineStr">
         <is>
           <t>1976</t>
+        </is>
+      </c>
+      <c r="P480" t="inlineStr">
+        <is>
+          <t>Valid individual-level quantitative study measuring Boundary Spanning Behavior and providing zero-order correlations with role stress.. Verbatim Evidence: [Sample] "Relationships between major role requirements and experienced role stress were examined on the basis of data drawn from 202 research and development professionals." [Measures] "Factor II: Integration and boundary-spanning activities 1. Represent your directorate/laboratory to outsiders. 2. Review plans with agencies outside the laboratory... 11. Act as liaison with other units of the organization." [Effect Size] "TABLE 4 CORRELATIONS BETWEEN IMPORTANCE OF ROLE REQUIREMENTS AND VARIOUS TYPES OF ROLE CONFLICT AND AMBIGUITY EXPERIENCED BY ROLE INCUMBENTS"</t>
         </is>
       </c>
     </row>
@@ -23904,6 +24474,16 @@
           <t>BSMA0482</t>
         </is>
       </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G485" t="inlineStr">
         <is>
           <t>Previous research demonstrates the destructive consequences of role stress for the work outcomes of employees occupying boundary-spanning positions. Most studies examine the behavior and performance of industrial salespeople. In contrast, limited evidence exists regarding the antecedents and consequences of role stress in service organizations. This article helps fill this notable gap by investigating the correlates of role ambiguity in the context of frontline managers in banking institutions. The article offers a conceptual model and an empirical test using data gathered from 316 bank branch managers. The study findings reveal that information control is an effective mechanism for reducing role ambiguity. The results also indicate that role ambiguity negatively affects job performance and job satisfaction, intrinsic motivation positively relates to job satisfaction, and bank managers' job performance enhances branch effectiveness. The article concludes with a discussion of study implications and suggestions for future research in the field.</t>
@@ -23927,6 +24507,11 @@
       <c r="K485" t="inlineStr">
         <is>
           <t>2012</t>
+        </is>
+      </c>
+      <c r="P485" t="inlineStr">
+        <is>
+          <t>The study surveys employees occupying boundary-spanning positions (branch managers) but does not measure Boundary Spanning Behavior (BSB), focusing instead on role ambiguity, management control, intrinsic motivation, and job performance.. Verbatim Evidence: [Abstract] "The article offers a conceptual model and an empirical test using data gathered from 316 bank branch managers. The study findings reveal that information control is an effective mechanism for reducing role ambiguity." [1. Introduction] "Branch managers represent a typical example of a boundary spanner." [Table 1] "Constructs and measurement items ... Information control ... Supervisor-related role ambiguity ... Job-related role ambiguity ... Intrinsic motivation ... Job satisfaction ... Job performance"</t>
         </is>
       </c>
     </row>
@@ -23994,6 +24579,16 @@
           <t>BSMA0484</t>
         </is>
       </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G487" t="inlineStr">
         <is>
           <t>For years many researchers and practitioners have been calling for a more boundary-spanning or cross-functional view of the management of businesses. As any student of optimization will note, the combination of several optimized sub-systems will rarely, if ever, result in a globally optimized system. It is much the same with a business. Decisions that may appear extremely good within the confines of a single organizational area are often clearly dysfunctional when viewed from other areas of the organization. To effectively compete in today's marketplace, firms need to effectively link their diverse functional areas. This article provides an example of how the marketing, operations, and purchasing areas can be effectively linked to accomplish the common goal of effectively competing in the value market segment of consumer goods and services.</t>
@@ -24017,6 +24612,11 @@
       <c r="K487" t="inlineStr">
         <is>
           <t>1995</t>
+        </is>
+      </c>
+      <c r="P487" t="inlineStr">
+        <is>
+          <t>[Code 1, Code 2, Code 4] Conceptual and mathematical modeling paper without primary survey data, employee sample, or extractable effect sizes.. Verbatim Evidence: [Abstract] "This article provides an example of how the marketing, operations, and purchasing areas can be effectively linked to accomplish the common goal of effectively competing in the value market segment of consumer goods and services." [AN EXAMPLE OF THE BENEFITS OF INTEGRATION] "Although this example is loosely based on experience with an east coast US grocery firm with approx. 200 retail outlets, the actual values and outcomes reported here are for demonstration purposes only." [APPENDIX III] "A simulation analysis measuring the absolute percent error between projected and actual values for float and the contribution from sales (profits from sales would behave similarly to contribution) supports this conclusion."</t>
         </is>
       </c>
     </row>
@@ -24031,6 +24631,16 @@
           <t>BSMA0485</t>
         </is>
       </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G488" t="inlineStr">
         <is>
           <t>In spite of increasing research attention given to individual creativity and organizational innovation, there are comparatively few studies investigating innovation in work groups. This is unfortunate given the increased use of groups to perform work in organizations. This dissertation addresses some of the inadequacies in the current literature by developing and testing a model of innovation in ongoing, task-performing work groups. The theoretical model uses an input-process-output framework common to group research. The input portion of the model is individual innovativeness. The group process portion of the model is group support for innovation. The output portion of the model is group innovation. Group support for innovation was expected to mediate the influence of individual innovativeness on group innovation. Expectancy theory is used to explain the hypothesized relationships of group support for innovation with group innovative potency, group scouting, group psychological safety, and group innovation encouragement norms. This dissertation used a cross-sectional design in a field setting. Surveys were given to group members and their supervisors in two organizations. Thirty-three work groups were used in the study. Hierarchical regression was used to test the hypotheses. Among the main findings was that group support for innovation was positively associated with group innovation quantity and quality. Group innovative potency and supervisor support were both positively associated with group support for innovation. Constructive controversy moderated the relationship between group support for innovation and group innovation quantity. Contrary to expectations, the relationship between group support for innovation and innovation was stronger when constructive controversy was low than when it was high. The findings, directions for future research, and implications for managers are discussed.</t>
@@ -24054,6 +24664,11 @@
       <c r="K488" t="inlineStr">
         <is>
           <t>2002</t>
+        </is>
+      </c>
+      <c r="P488" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N = 33 work groups).. Verbatim Evidence: [Abstract] Thirty-three work groups were used in the study. Hierarchical regression was used to test the hypotheses. [Aggregation of Group Data] To aggregate individual data to the group level, I averaged the responses from the individual team members for each variable of interest. [DESCRIPTIVE STATISTICS AND CORRELATIONS] Table 2 shows the means, standard deviations, and zero-order correlations for each of the measures of interest at the group level. [Table 2] Note: N = 33</t>
         </is>
       </c>
     </row>
@@ -24120,6 +24735,12 @@
           <t>BSMA0487</t>
         </is>
       </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr">
         <is>
           <t>Purpose – This study seeks to address a gap in the literature by investigating product management (PM) as a set of ﬁrm-level activities, distinct from the behaviours embedded within the market orientation (MO) construct. This research establishes PM as a set of organizational activities, which lie at the boundary between the traditional functions of the ﬁrm.</t>
@@ -24143,6 +24764,11 @@
       <c r="K490" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P490" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -24162,11 +24788,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
-        </is>
-      </c>
+      <c r="F491" t="inlineStr"/>
       <c r="G491" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the impact of product management as a set of organizational capabilities. It aims to investigate product management as a set of boundary spanning capabilities, by empirically relating these to ﬁrm performance.</t>
@@ -24194,7 +24816,7 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>Firm-level unit of analysis with key informant. Verbatim Evidence: [Abstract] "A model is proposed and tested using a heterogeneous sample of 316 Canadian small and medium-sized enterprises, where PM mediates the relationship between MOand ﬁrm performance." [Sample and data collection] "The method of data collection was a self-reported on-line survey answered by senior managers of SMEs in May 2009." [Appendix] "PM01 We have strong systems for deciding which products and/or service opportunities to pursue or which to phase-out." [Appendix] "PM07 We foster communication about our products and/or services within our ﬁrm in order to generate product improvement ideas."</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -24586,6 +25208,16 @@
           <t>BSMA0497</t>
         </is>
       </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G500" t="inlineStr">
         <is>
           <t>We propose and test a relational boundary-blurring framework, examining how employees’ evaluations of colleagues’ characteristics drive their decisions to connect with colleagues as friends online. We use a multi-method approach across four studies to investigate how self-disclosure of personal information, gender, and rank shape warmth evaluations of colleagues and subsequent boundary blurring decisions on online social networks such as Facebook. Study 1, a large archival study using a nationally representative sample, finds that connecting as friends with colleagues online is prevalent. Study 2, examining employees across several industries, shows that people experience connecting as friends with colleagues online as boundary blurring. Two experimental studies (Studies 3 and 4) ascertain that employees are more likely to connect as friends online with colleagues who engage in more (vs. less) self-disclosure and are less likely to connect with bosses (vs. peers). Further, self-disclosure, gender, and rank interact, such that employees are more likely to connect with female bosses who disclose more, compared to those who disclose less, and compared to male bosses, regardless of self-disclosure. Our work contributes to boundary management research by demonstrating that employees’ decisions to blur the personal/professional boundary online crucially depends on whom they are blurring the boundary with.</t>
@@ -24609,6 +25241,11 @@
       <c r="K500" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P500" t="inlineStr">
+        <is>
+          <t>Construct Homonymy: Studies work-life/personal-professional boundary blurring (social media connection) rather than inter- or intra-organizational boundary spanning behavior.. Verbatim Evidence: [Method] "Study 1 uses publicly available data from a nationally representative sample to understand the extent to which people connect as friends with colleagues online. Study 2 uses a panel of employees across several of the largest industries in the United States to understand whether people experience connecting as friends with colleagues online as boundary blurring." [Theoretical Background] "'Boundary management' is the process by which individuals make decisions and act to separate (i.e., segment) or blur (i.e., integrate) the boundaries between multiple life domains"</t>
         </is>
       </c>
     </row>
@@ -24764,6 +25401,12 @@
           <t>BSMA0501</t>
         </is>
       </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr">
         <is>
           <t>The purpose of this research is to explore a novel model whereby boundary-spanning leadership (BSL) enhances nurses’ absorptive capacity (ACAP), ultimately leading to increased job embeddedness (JE) during the COVID-19 pandemic. An autoregressive cross-lagged model was employed to examine the causal relationships among BSL, ACAP, and JE. Data were collected through three waves of surveys conducted at three-month intervals, with a final sample of 297 nurses in Chinese hospitals. This longitudinal design enabled the investigation of both the direct and indirect effects of BSL on JE, mediated by ACAP, as well as the bidirectional influence between BSL and ACAP over time. First, the autoregressive effects confirmed the temporal stability of BSL, ACAP, and JE, indicating that these constructs remained consistently valid in real-world settings over time. Second, the cross-lagged analysis validated that BSL, by fostering ACAP, indirectly enhanced JE, while BSL had no direct effect on JE. Finally, the bidirectional relationship between BSL and ACAP revealed a reciprocal dynamic between these two constructs. This research introduces a unique model that integrates BSL, ACAP, and JE, addressing gaps in prior literature and providing meaningful insights through rigorous analysis using longitudinal data and an autoregressive cross-lagged model. We suggested that hospital administrators and HR leaders foster ACAP through regular feedback sessions and workshops that promote knowledge sharing and the exploration of new ideas, and further emphasized the role of BSL within tailored training programs.</t>
@@ -24791,6 +25434,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="P504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -24877,6 +25525,16 @@
           <t>BSMA0504</t>
         </is>
       </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G507" t="inlineStr">
         <is>
           <t>This paper considers the mutual value co-creation that can occur when both parties in a cross sector partnership learn to innovate within the relationship. Despite suggestions that there are often asymmetrical returns to the business partner, nonproﬁt partners also accrue beneﬁts (Austin &amp; Seitanidi, 2012). In particular we consider how the relationship is inﬂuenced by the actors’ abilities to accommodate, adapt, learn and co-create solutions as they learn how to do things differently or better in response to the challenges they face. This is achieved using data from a longitudinal analysis of a crosssector partnership between a business and an arts organisation in Ireland. This offers a unique opportunity to trace the emergence of the partnership over time, and, speciﬁcally, to consider the impact of innovations co-created by the actors involved. Our analysis will demonstrate that innovation at the level of the relationship emerged from the incremental problem solving processes of the individuals involved. This foregrounds the impact of individual boundary spanners and the import of social capital in realising the potential of this partnership. In this regard we put forward three key boundary spanning roles, boundary spanner as network builder, as entrepreneur, as facilitator/mediator. The paper concludes with suggestions for further research and consideration of managerial implications arising from this study.</t>
@@ -24900,6 +25558,11 @@
       <c r="K507" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P507" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative effect sizes. Verbatim Evidence: [Method] "The evidence presented here is based upon a high level of access to the data, which provides opportunities for historical and real-time analysis (Halinen &amp; Törnroos, 1995). Real time data, in the form of in-depth interviews (9 in total), was collected between 2001 and 2005, and included key boundary spanners from both organisations."</t>
         </is>
       </c>
     </row>
@@ -24914,6 +25577,16 @@
           <t>BSMA0505</t>
         </is>
       </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G508" t="inlineStr">
         <is>
           <t>Retaining information technology (IT) professionals is important for organizations, given the challenges in sourcing for IT talent. Prior research has largely focused on understanding employee turnover from an intra-individual perspective. In this study we examine employee turnover from a structural perspective. We investigate the impact on IT turnover of organizations' Internal Labor Market (ILM) strategies. ILM strategies include human resource rules, practices, and policies including hiring and promotion criteria, job ladders, wage systems and training procedures. We collect data on ILM strategies and turnover rates for eight major IT jobs across forty-one organizations and analyze the data using confirmatory agglomerative hierarchical clustering techniques. Our results show that organizations adopt distinct ILM strategies for different IT jobs, and that these strategies relate to differential turnover rates. Specifically, technically-oriented IT jobs cluster in craft ILM strategies that are associated with higher turnover, whereas managerially-oriented IT jobs cluster in industrial ILM strategies that are associated with lower turnover. Further, depending on their contingencies of goal orientation (not-for-profit versus for-profit), IT focus (IT producer versus user), and information intensity (IT critical versus support), organizations adopt an industrial ILM strategy for their technically-oriented IT jobs to dampen turnover. Not-for-profit and IT user organizations where IT is critical adopt industrial ILM strategies for their technically-oriented IT jobs to attenuate turnover and improve the predictability of their IT workforce. IT producers and IT users where IT plays a supporting role adopt craft ILM strategies that engender higher turnover to remain timely and flexible in IT skills acquisition.</t>
@@ -24937,6 +25610,11 @@
       <c r="K508" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P508" t="inlineStr">
+        <is>
+          <t>The study does not measure boundary spanning behavior (Code 1) and the unit of analysis is at the job/organization level using key informants rather than individual employees (Code 3).. Verbatim Evidence: [Abstract] "We collect data on ILM strategies and turnover rates for eight major IT jobs across forty-one organizations and analyze the data using confirmatory agglomerative hierarchical clustering techniques." [Methodology] "Our subjects were key informants in each organization (including the Chief Information Officer, other IT managers, and HR managers) who were responsible for hiring and firing IT professionals and for establishing human resource policies in their organizations." [Methodology] "To elicit the ILM strategies for IT jobs in each organization, we identified eight major jobs in the IT profession: Chief Information Officer (CIO), Divisional Manager (Applications), Project Leader, Analyst/ Programmer, Divisional Manager (Infrastructure), Database Administrator, Network Specialist and Systems Programmer."</t>
         </is>
       </c>
     </row>
@@ -24951,6 +25629,12 @@
           <t>BSMA0506</t>
         </is>
       </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr"/>
       <c r="G509" t="inlineStr">
         <is>
           <t>While researchers have probed predictors of product managers' performance in consumer goods firms, few have looked at the performance of the industrial product manager. In this article, Steven Lysonski and Arch Woodside use path analysis to examine causal models of industrial product managers' performance during periods of rapid technological change. Key variables are analyzed, including the effects of environmental uncertainty, boundary spanning behavior, role pressures, role outcomes and two performance measures. A total of 69 industrial product managers from New Zealand Telecom completed a questionnaire that included both operational measures of the key variables and their overall job performance. The results suggest that most of the hypothesized relationships are supportable empirically. Performance was hindered by environmental uncertainty, role conflict, role ambiguity, tension and dissatisfaction. The authors discuss their study's implications for improving the effectiveness of product management practices.</t>
@@ -24974,6 +25658,11 @@
       <c r="K509" t="inlineStr">
         <is>
           <t>1989</t>
+        </is>
+      </c>
+      <c r="P509" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -25040,6 +25729,16 @@
           <t>BSMA0508</t>
         </is>
       </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G511" t="inlineStr">
         <is>
           <t>Purpose – Drawing on the conservation of resources theory, this research examines the relationship between managers’ servant leadership and frontline employees’ customer-oriented boundary-spanning behaviors by considering career meaningfulness as an underlying mechanism. Furthermore, this study investigates a moderated mediation model by proposing work centrality as a boundary condition in the relationship between career meaningfulness and customer-oriented boundary-spanning behaviors.</t>
@@ -25063,6 +25762,11 @@
       <c r="K511" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P511" t="inlineStr">
+        <is>
+          <t>Valid employee-level study providing a correlation matrix with a valid boundary-spanning behavior construct.. Verbatim Evidence: [Methodology] "Two-source (manager-frontline employee dyad) data were collected through a survey questionnaire from hospitality organizations" [Methodology] "We got 257 managers' responses about their frontline employees' customer-oriented boundary-spanning behaviors. After aligning the data through distinctive codes and thorough assessment, only 245 responses were kept and used for further analysis." [Measures] "Customer-oriented boundary-spanning behaviors were evaluated using a thirteen-item scale developed by Bettencourt et al. (2005)." [Results] "Table 2. Descriptive statistics and correlations"</t>
         </is>
       </c>
     </row>
@@ -25129,6 +25833,16 @@
           <t>BSMA0510</t>
         </is>
       </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G513" t="inlineStr">
         <is>
           <t>Organisations are increasingly investing in complex technological innovations, such as enterprise information systems, with the aim of improving the operation of the business, and in this way gaining competitive advantage. However, the implementation of technological innovations tends to have an excessive focus on either technological innovation effectiveness, or the resulting operational effectiveness. Focusing on either one of them is detrimental to long-term performance. Cross-functional teams have been used by many organisations as a way of involving expertise from different functional areas in the implementation of technologies. The role of boundary spanning actors is discussed as they bring a common language to the crossfunctional teams. Multiple regression analysis has been used to identify the structural relationships and provide an explanation for the influence of cross-functional teams, technological innovation effectiveness and operational effectiveness in the continuous improvement of operational performance. The findings indicate that cross functional teams have an indirect influence on continuous improvement of operational performance through the alignment between technological innovation effectiveness and operational effectiveness.</t>
@@ -25152,6 +25866,11 @@
       <c r="K513" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P513" t="inlineStr">
+        <is>
+          <t>No effect size of interest. The study does not measure boundary spanning behavior as a quantitative variable; it measures 'Cross-functional Teams' and boundary spanning is only discussed conceptually. Additionally, no correlation matrix is provided.. Verbatim Evidence: [Sample] "The questionnaires were emailed to employees in managerial or executive role, information technology / information systems or engineering role and operators or general staff in the selected service organisations. Of the 450 surveys distributed, 144 were returned (32% response)." [Variables] "The results from the multiple regression analysis (table 1) show that cross-functional teams is a significant predictor of the two dimensions stemming from technological innovation effectiveness and the two performance objectives stemming from operational effectiveness" [Construct Invalid] "The main purpose of this research is to build on and extend the existing literature and to put forward a theoretical framework that examines the following three propositions: ... 2. That, cross-functional project teams influence the alignment between technological innovation effectiveness and operational effectiveness."</t>
         </is>
       </c>
     </row>
@@ -25166,6 +25885,12 @@
           <t>BSMA0511</t>
         </is>
       </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr"/>
       <c r="G514" t="inlineStr">
         <is>
           <t>Boundary spanners are pivotal in developing effective public–private collaboration in public infrastructure projects. As boundary spanners have to account for different interests, perspectives, and ways of working in public–private collaborations, engaging in boundary-spanning activities often comes with role stress, which can negatively impact their job performance. However, despite the significant levels of role stress associated with boundary spanning, there is a dearth of empirical studies on the role stress of boundary spanning public managers and how it can be reduced. In this study, we empirically investigate the reciprocal relationship between role stressors and boundary spanning and test if supporting organizational conditions can alleviate role stressors. The findings show that especially role conflict is detrimental for boundary-spanning activities. We further find that top-management support can diminish both role conflict and role ambiguity and that co-worker support can help in reducing the role ambiguity of boundary spanning public managers.</t>
@@ -25189,6 +25914,11 @@
       <c r="K514" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P514" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -25344,6 +26074,16 @@
           <t>BSMA0515</t>
         </is>
       </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G518" t="inlineStr">
         <is>
           <t>The focus of this dissertation is the role of strategic flexibility and its effect on economic performance of firms in a cyclical industry. The performance consequences of the decision-making processes and CEO boundary-spanning activity are also examined.</t>
@@ -25367,6 +26107,11 @@
       <c r="K518" t="inlineStr">
         <is>
           <t>1986</t>
+        </is>
+      </c>
+      <c r="P518" t="inlineStr">
+        <is>
+          <t>Invalid construct (measures only percentage of time and number of contacts without purposive action). Verbatim Evidence: [Measures] "Please estimate the percentage of your total working hours that you typically spend with each of the groups listed below." [Measures] "Please estimate the approximate number of contacts that you would have with each of the following groups during a normal work week." [Definition] "Dollinger (1984) measured two dimensions of boundary-spanning activity: intensity, which was the number of hours the CEO spent in boundary spanning activity divided by the number of hours worked per week; and extensiveness, the total of the number of contacts that the CEO had each week."</t>
         </is>
       </c>
     </row>
@@ -25492,6 +26237,16 @@
           <t>BSMA0519</t>
         </is>
       </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G522" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to analyze the effects of inpatriates’ abilities, motivation and opportunities on knowledge sharing and the moderating role of boundary spanning in this context. Design/methodology/approach – By integrating the ability–motivation–opportunity framework with the concept of boundary spanning four hypotheses are developed, which are tested against the data of 187 inpatriates working in Germany.</t>
@@ -25515,6 +26270,11 @@
       <c r="K522" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P522" t="inlineStr">
+        <is>
+          <t>Valid individual-level intra-organizational boundary spanning behavior with extractable zero-order correlations.. Verbatim Evidence: [Sample and procedure] "Our hypotheses and overall model proposed above was tested through unique data set obtained from a survey among international assignees working in the HQ of German MNCs." [Measures] "Inpatriate boundary spanning was measured by using a five-item scale (1 = strongly disagree – 7 = strongly agree) developed by Reiche (2011). The measure builds on existing research on boundary spanning and was particularly developed to reflect the brokering function of inpatriates." [Results] "Table I. Descriptive statistics and correlations" "Notes: n = 187."</t>
         </is>
       </c>
     </row>
@@ -25527,6 +26287,16 @@
       <c r="B523" t="inlineStr">
         <is>
           <t>BSMA0520</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G523" t="inlineStr">
@@ -25565,6 +26335,11 @@
           <t>2012</t>
         </is>
       </c>
+      <c r="P523" t="inlineStr">
+        <is>
+          <t>The study does not measure Boundary Spanning Behavior (BSB) as a construct; it surveys employees on the perceived importance of general leadership attributes (e.g., charisma, vision, integrity). Additionally, the paper lacks a zero-order correlation matrix and provides no quantitative effect sizes.. Verbatim Evidence: [Sample and Measures] "Our research was designed to uncover the dimensions of marketing leadership that lead to perceptions of high performance." [Sample and Measures] "We collected data from two large multinational companies across various business functions." [Sample and Measures] "Over 1,000 employees responded to an online survey and 825 responses from six functional departments (engineering, information technology, manufacturing, marketing, sales, and research) were used in the initial analysis." [Sample and Measures] "The employees were asked to rate the importance of 45 leadership attributes to high-performing leadership in their particular business function." [Findings] "Table I shows the top ten leadership ratings as determined by marketing in the first column with the corresponding ratings given by five other business functions (engineering, information technology, manufacturing, research &amp; development, and sales) in the remaining columns."</t>
+        </is>
+      </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -25688,6 +26463,16 @@
           <t>BSMA0524</t>
         </is>
       </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G527" t="inlineStr">
         <is>
           <t>This study explores patterns of individual boundary-spanning communication in a government-managed research and development setting. Individual position in the organization hierarchy and preference for risk, change, and new experiences are the most significant antecedents of general levels of boundary-spanning communication.</t>
@@ -25711,6 +26496,11 @@
       <c r="K527" t="inlineStr">
         <is>
           <t>1989</t>
+        </is>
+      </c>
+      <c r="P527" t="inlineStr">
+        <is>
+          <t>Excluded because the boundary-spanning measure solely assesses mere communication frequency (hours and number of times communicating) without specifying purposive boundary-spanning actions.. Verbatim Evidence: [Measures] "Individual boundary-spanning activity is defined as the weekly frequency or extent of communication, formal and informal, written and spoken, across organizational boundaries between tasks within project organizations and between research centers." [APPENDIX A] "(1) How many hours do you attend formal meetings? (Committees, planning, etc.)" [APPENDIX A] "(2) How many hours do you confer about your work in informal face-to-face conversation or telephone conversation with people outside your immediate department?"</t>
         </is>
       </c>
     </row>
@@ -25799,6 +26589,16 @@
           <t>BSMA0527</t>
         </is>
       </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G530" t="inlineStr">
         <is>
           <t>Over the last decade, there has been a tremendous growth and exploitation of open source geospatial software and technologies. A combination of factors is driving this momentum including the contributions made by hundreds of OSGeo developers and the leading role played by the Open Source Geospatial Foundation (OSGeo), aiming primarily to support and promote the collaborative development of open source geospatial technologies and data. This paper seeks to map out the social history of collaborative activities within the OSGeo ecosystem. We used the archival logs of developers’ contributions, specifically looking for boundary spanning activities where contributions crossed multiple projects. The analysis and visualization of these activities allow us to have a better understanding of the role of boundary spanning in the resourcing of each project, the incubation mechanism advocated by OSGeo, and the significance of the social interrelatedness among projects. The data consisted of the subversion (SVN) commit history made by individual developers in the programming code repository. We applied several network analytical and visualization techniques to explore the data. Our findings indicate that more than one in seven developers spanned multiple projects which potentially had the effects of shaping the projects’ directions, and increased knowledge flow and innovation. Also the OSGeo’s incubation mechanism provided an important encouragement for boundary spanning and increased knowledge sharing. By studying the social history of contributions, further tools can be developed in future to assist tracking of the social history, and make developers mindful of the significance of the interdependence among projects and hence continuously contribute to the healthiness of the OSGeo ecosystem.</t>
@@ -25822,6 +26622,11 @@
       <c r="K530" t="inlineStr">
         <is>
           <t>2012</t>
+        </is>
+      </c>
+      <c r="P530" t="inlineStr">
+        <is>
+          <t>Multiple flaws: No extractable effect size or correlation matrix (descriptive network analysis) [Code 1] and non-employee sample of open source volunteers [Code 2].. Verbatim Evidence: [Abstract] "This paper seeks to map out the social history of collaborative activities within the OSGeo ecosystem. We used the archival logs of developers’ contributions, specifically looking for boundary spanning activities where contributions crossed multiple projects." [1 Introduction] "Open source development attracts a great number of participants from various backgrounds." [2 Data collection] "Three publicly available data sources were identified for deriving contribution metrics: Subversion (SVN) code repository commits; mailing lists; and issue trackers (Gutwin, Penner et al. 2004). SVN commits are used to track individual and aggregate contributions of source code and are taken directly from a project's source code repository."</t>
         </is>
       </c>
     </row>
@@ -26251,11 +27056,7 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F540" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="F540" t="inlineStr"/>
       <c r="G540" t="inlineStr">
         <is>
           <t>This dissertation investigated the effects of intrinsic and extrinsic motivational orientations in a boundary spanning model of retail buyers. Contributions of the dissertation to the field of marketing include the following: First, a boundary spanning/role stress model was tested in the context of retail buyers. No previous work has empirically or conceptually investigated the ability of a boundary spanning/role stress model to explain retail buyers' work-related attitudes. Second, the boundary spanning/role stress model was extended with the inclusion of accumulated role benefits. Previous role stress studies consider only negative role perceptions; accumulated role benefits examines positive role perceptions. Third, the boundary spanning/role stress model considers only external influences of role set members on a role incumbent. In doing so, the model neglects the influence of the individual who is perceiving and interpreting these stimuli. To capture individual differences, effects of intrinsic and extrinsic motivational orientations of the buyers were tested in the model. Finally, scales were developed to measure intrinsic motivational orientations, extrinsic motivational orientations, boundary spanning beliefs, and accumulated role benefits.</t>
@@ -26283,7 +27084,7 @@
       </c>
       <c r="P540" t="inlineStr">
         <is>
-          <t>Included. The study examines individual-level boundary spanning behaviors (beliefs) of retail buyers and provides a zero-order correlation matrix.. Verbatim Evidence: [Sample] "The sample frame was Sheldon's Retail Directory (1986), which lists buyer names, store affiliations with addresses, and type of merchandise bought for department stores, chain stores, and specialty stores." [Methodology] "305 of the original 700 buyers sampled responded to the survey, for a response rate of 43.6%." [Measures] "Three positively worded items address beliefs about external boundary spanning: item Q51 states, "I spend at least half my time dealing with people who work for other companies"; item Q34 states, "Getting my job done often depends on the activities of people who don't even work for my company"; and item Q7 states, "I regularly communicate with employees of other companies in order to get my job done."" [Data] "Table 4-17 Descriptive Statistics for Summated Scales: Matrix of Correlations, 1-Tailed Sig, N of cases"</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -26335,7 +27136,7 @@
       </c>
       <c r="P541" t="inlineStr">
         <is>
-          <t>Work-Family construct homonymy.. Verbatim Evidence: [Abstract] "we observed that work-to-family cognitive role transitioning was negatively related to job performance" [Method] "We used data from the Sloan 500 Family Study (Schneider and Waite, 2008) to test our hypotheses." "The 500 Family Study targeted middle-class, dual-earner families, including mothers, fathers and children sampled from communities dispersed across the United States." [Measures] "Work-to-family cognitive role transition episodes were measured dichotomously where participants were assigned a 0 if no role transition occurred or a 1 if a role transition episode was present." "Cognitive role transition episodes were coded as 1 if a participant was thinking about family-related content."</t>
+          <t>The study examines work-family cognitive role transitions (work-life boundary management), not inter-organizational or intra-organizational boundary spanning behavior.. Verbatim Evidence: [Abstract] "In a multilevel study of 619 employees providing 4371 episodes, we observed that work-to-family cognitive role transitioning was negatively related to job performance, and this effect was mediated by self-regulatory depletion." [The role of cognitive role transitions in boundary theory] "We define cognitive role transitions here as discrete episodes in which an individual is currently engaged in one role (i.e. work), and experiences off-topic thoughts regarding a different role (i.e. family)."</t>
         </is>
       </c>
     </row>
@@ -26439,7 +27240,7 @@
       </c>
       <c r="P543" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 3] No boundary spanning behavior measured and team-level analysis.. Verbatim Evidence: [Table 1] &lt;Table 1. Descriptive Statistics and Correlations. Variables M SD 1 2 3 4 5 6 1. Supervisor age 2. Supervisor gender 3. Team size 4. Supervisor time pressure 5. Team time pressure 6. Team creativity&gt; [Data and Research Sample] &lt;To explore our research question, we conducted a time-lagged study in which we collected data from teams and their direct-level supervisors in a large financial service firm in Canada.&gt; [Validity and Data Aggregation] &lt;Considering the results obtained from the tests, their satisfactory values, and the small team sizes within our sample (LeBreton &amp; Senter, 2008; Shieh, 2016), we aggregated our data from individuals to teams.&gt; [Table 1] &lt;Note. n=51 teams.&gt;</t>
+          <t>Multiple reasons [Code 1 &amp; Code 3]: Team-level analysis of time pressure and creativity, with no measure of individual boundary spanning behavior.. Verbatim Evidence: [Abstract] Focusing on team creativity as the outcome of interest, we explore how teams with varying time pressures function alongside the distinct time pressures experienced by their supervisors. [Method] Our analysis is based on a multi-source, time-lagged sample of 377 salespeople in 51 teams. [Method] we aggregated our data from individuals to teams.</t>
         </is>
       </c>
     </row>
@@ -26491,7 +27292,7 @@
       </c>
       <c r="P544" t="inlineStr">
         <is>
-          <t>The study does not measure boundary spanning behavior (BSB). It focuses on job characteristics and organizational climate.. Verbatim Evidence: [Measures] "Two questionnaires were used for the collection of the data for this research, one addressing job characteristics, the other organizational climate." [Measures] "The job characteristics questionnaire consisted of 20 items." [Measures] "These included job reward policies, interpersonal job aspects, and training opportunities." [Measures] "The Organizational Climate Questionnaire consisted of 19 items." [Measures] "These pertained to policies of improvement of methods and efficiency, participation, reward structure, consideration, and decision making practices"</t>
+          <t>No measure of Boundary Spanning Behavior; the study examines job characteristics and organizational climate.. Verbatim Evidence: [Sample] "Two hundred and forty top managers from a broad range of Israeli work organizations participated in the study. Half the sample consisted of managers from the private sector, the other half of managers from the public sector." [Measures] "The job characteristics questionnaire consisted of 20 items. These included job reward policies, interpersonal job aspects, and training opportunities. Other dimensions such as task autonomy, significance, variety, and feedback corresponded to Hackman and Lawler's (1971) and Hackman and Oldham's (1976) core job dimensions and, finally, a group of items referred to role clarity-ambiguity studied in the literature on role stress" [Measures] "The Organizational Climate Questionnaire consisted of 19 items. These pertained to policies of improvement of methods and efficiency, participation, reward structure, consideration, and decision making practices (Campbell et al., 1970; Likert, 1967; Payne &amp; Pugh, 1976)."</t>
         </is>
       </c>
     </row>
@@ -26595,7 +27396,7 @@
       </c>
       <c r="P546" t="inlineStr">
         <is>
-          <t>Excluded due to multiple reasons: [Code 1 &amp; Code 3]. The study uses individuals as proxy informants for firm-level supply chain initiatives, and the individual-level measure is a personality trait/orientation rather than actual boundary-spanning behavior.. Verbatim Evidence: [Theoretical Development] Tangpong, Hung, and Ro (2010) conceptualize this particular disposition in the buyer-supplier setting as âcooperativenessâ; an example is the personality trait that entails acting toward others in tolerant, empathetic, supportive, and compassionate ways for mutual benefit. [Appendix] I am willing to share risks and benefits with my partners. [Research Methods] We selected 2,000 SMEs identified from the Korean Chamber of Commerce and Industry Directory, and to ensure that our respondents were in boundary-spanning roles in their companies, included a covering letter asking that the questionnaire be completed by BSIs such as sales managers. [Appendix] My company shares operational information with our partners. [Appendix] My company does strategic supply-chain planning jointly with our partners.</t>
+          <t>Excluded due to multiple reasons: [Code 1 &amp; Code 3]. The study uses individuals as proxy informants for firm-level supply chain initiatives, and the individual-level measure is a personality trait/orientation rather than actual boundary-spanning behavior.. Verbatim Evidence: [Theoretical Development] Tangpong, Hung, and Ro (2010) conceptualize this particular disposition in the buyer-supplier setting as “cooperativeness”; an example is the personality trait that entails acting toward others in tolerant, empathetic, supportive, and compassionate ways for mutual benefit. [Appendix] I am willing to share risks and benefits with my partners. [Research Methods] We selected 2,000 SMEs identified from the Korean Chamber of Commerce and Industry Directory, and to ensure that our respondents were in boundary-spanning roles in their companies, included a covering letter asking that the questionnaire be completed by BSIs such as sales managers. [Appendix] My company shares operational information with our partners. [Appendix] My company does strategic supply-chain planning jointly with our partners.</t>
         </is>
       </c>
     </row>
@@ -26617,7 +27418,7 @@
       </c>
       <c r="F547" t="inlineStr">
         <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G547" t="inlineStr">
@@ -26647,7 +27448,7 @@
       </c>
       <c r="P547" t="inlineStr">
         <is>
-          <t>The study analyzes boundary-spanning network variables (degree centrality and structural holes) at the work unit level (N=20), which violates the individual-level requirement [Code 3]. Additionally, the individual-level analysis (N=84) focuses on general knowledge management strategies (personalization and codification) which do not measure purposive boundary spanning behavior [Code 1].. Verbatim Evidence: [3.4 Levels of analysis] "The unit of analysis is individual for intra-unit analysis (H3-H6). All task-related and KM-related measures were measured at the individual level. For inter-unit analysis (H1 and H2), the unit of analysis is at the work unit level." [3. Research methodology] "As a result, 20 leader responses and 84 member responses were used in the data analysis." [Appendix 1. Instruments] "Personalization strategy TO1 Making face-to-face social interactions to exchange knowledge."</t>
+          <t>Non-individual level (Team level analysis). Verbatim Evidence: [Section 3. Research methodology] "As a result, 20 leader responses and 84 member responses were used in the data analysis." [Section 3.4 Levels of analysis] "The unit of analysis is individual for intra-unit analysis ( H3-H6). All task-related and KM- related measures were measured at the individual level. For inter-unit analysis ( H1andH2), the unit of analysis is at the work unit level. Network structure, as described earlier, was measured at the work unit level by collecting responses from unit leaders." [Table II] "Table II Descriptive and correlations of research variables: inter-units ( N= 20)"</t>
         </is>
       </c>
     </row>
@@ -26788,7 +27589,7 @@
       </c>
       <c r="P550" t="inlineStr">
         <is>
-          <t>No effect size of interest. Measures coping strategies rather than boundary spanning behavior.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] The study collected data from multiple sources: survey data from 452 boundary-spanning salespeople and sales commission from a companyâs personnel record." "[Methodology] For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)." "[Appendix] Problem-focused coping (CI-P) I try to work more efficiently. I devote more time and energy to my job. I decide what I think should be done and explain this to the people who are affected."</t>
+          <t>No effect size of interest. Measures coping strategies rather than boundary spanning behavior.. Verbatim Evidence: [No effect size of interest]. Verbatim Evidence: "[Abstract] The study collected data from multiple sources: survey data from 452 boundary-spanning salespeople and sales commission from a company’s personnel record." "[Methodology] For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)." "[Appendix] Problem-focused coping (CI-P) I try to work more efficiently. I devote more time and energy to my job. I decide what I think should be done and explain this to the people who are affected."</t>
         </is>
       </c>
     </row>
@@ -27048,7 +27849,7 @@
       </c>
       <c r="P555" t="inlineStr">
         <is>
-          <t>Qualitative study with no extractable quantitative effect sizes [Code 1], analyzing interorganizational projects at the firm/project level [Code 3].. Verbatim Evidence: [Abstract] "The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." [3. Research setting and methods] "We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." [3. Research setting and methods] "Our data analysis followed an “abductive” approach (Alvesson and Sköldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
+          <t>Qualitative study analyzing interorganizational projects [Code 1 &amp; Code 3]. Verbatim Evidence: [Qualitative study analyzing interorganizational projects lacking effect sizes] [Code 1 &amp; Code 3]. Verbatim Evidence: "[Abstract] The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs." "[3. Research setting and methods] We conducted 51 in-depth, semi-structured interviews with key informants involved in the projects (see Appendix A)." "[3. Research setting and methods] Our data analysis followed an “abductive” approach (Alvesson and Sköldberg, 2011), as it involved an iterative process of moving between the empirical data and the theoretical framework."</t>
         </is>
       </c>
     </row>
@@ -27319,7 +28120,7 @@
       </c>
       <c r="P560" t="inlineStr">
         <is>
-          <t>Qualitative/Q-methodology study lacking extractable zero-order effect sizes and measuring cross-boundary tensions rather than boundary spanning behavior.. Verbatim Evidence: [Abstract] "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions." [Step 1: Interviews and Q Statements] "They were asked to respond to questions related to cross-boundary tensions, for example: âWhat do you believe are the biggest barriers to interaction between project owners and project managers across organizations and stages in the process of achieving project objectives?â" [Step 2: Q Surveys] "Between July and December 2023, 20 participants were invited to rank-order 20 Q statements, presented on cards, in a quasinormal distribution (see Figure 3)."</t>
+          <t>Qualitative/Q-methodology study lacking extractable quantitative effect sizes (r) and a correlation matrix.. Verbatim Evidence: [Abstract] "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions." [Step 2: Q Surveys] "In total, 20 participants were selected, consistent with the suggestion of Brown (1980) that a sample of 20 to 40 individuals provides a solid basis for factor analysis in Q methodology." [Step 2: Q Surveys] "Between July and December 2023, 20 participants were invited to rank-order 20 Q statements, presented on cards, in a quasinormal distribution (see Figure 3)."</t>
         </is>
       </c>
     </row>
@@ -27423,6 +28224,16 @@
           <t>BSMA0560</t>
         </is>
       </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G563" t="inlineStr">
         <is>
           <t>Even as knowledge-intensive firms adopt modes of work design that distribute authority across the workforce, the distribution of ownership and governance, termed “structural power”, continues to vary in these companies. Extant research suggests competing views that, in a knowledge-intensive industry, structural power is (a) irrelevant,(b) less consequential than work design, or (c) reinforces work design. Given these competing views, this project seeks to explore the consequences of variation in the distribution of structural power for knowledge-intensive work. Data comes from a multi-method comparison of knowledge-intensive work practices at two competing automated manufacturing equipment firms with contrasting distributions of structural power.</t>
@@ -27446,6 +28257,11 @@
       <c r="K563" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P563" t="inlineStr">
+        <is>
+          <t>Multiple reasons [Code 1 &amp; Code 3]: The chapter on inter-organizational boundary spanning is purely qualitative, lacking extractable effect sizes (Code 1). The quantitative chapter on cross-functional interaction uses the project/team as the unit of analysis and lacks a correlation matrix (Code 3 &amp; Code 1).. Verbatim Evidence: [Chapter Three] &lt;In the first stage of analysis, to test the relationship between the macro-level distribution of structural power, team-based cross-functional interactions, and team performance, I analyze data from the two companies’ administrative and human resource archives.&gt; [Chapter Three] &lt;This leaves a total of 223 unique projects, which constitutes 15% of total projects.&gt; [Chapter Four] &lt;The analysis that follows draws on qualitative material, collected over eight months at each company, from company documents, emails with participants, field notes, interviews, and meeting transcripts.&gt;</t>
         </is>
       </c>
     </row>
@@ -27571,6 +28387,16 @@
           <t>BSMA0564</t>
         </is>
       </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G567" t="inlineStr">
         <is>
           <t>The mechanisms by which social networks and organizational vocabularies combine jointly to affect communication patterns across organizational boundaries remain largely unexplored. In this paper, we examine the mutually constitutive relation between the network ties through which organizational members communicate with each other and the vocabularies that they use to describe their organization. We suggest that the dynamic structure of social networks and organizational vocabularies is contingent on the formal design of organizational subunits. Within subunit boundaries, members who interact with each other are more likely to develop similar vocabularies over time. Interestingly, between subunits, the more two members share similar organizational vocabularies, the more likely they are to form a tie over time. We ﬁnd empirical evidence for these arguments in a longitudinal study conducted among the managers of a multiunit organization. Organizational vocabularies, we suggest, may sustain communication patterns across organizational boundaries, thus bridging cultural holes within organizations.</t>
@@ -27594,6 +28420,11 @@
       <c r="K567" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P567" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] The study analyzes the existence of interpersonal network ties at the dyadic level (N = dyads), not individual-level boundary spanning behavior.. Verbatim Evidence: [Data and Methods] "Overall, the data set consists of 4,680 dyads involving the 40 managers across the three periods." [Data and Methods] "The dyadic data set includes 4,485 observations; 195 observations were dropped because of missing values in the identity-related variables." [Data and Methods] "Interpersonal tie was measured as a dichotomous variable capturing the existence of a tie between pairs of managers and presented an average value of 0.16"</t>
         </is>
       </c>
     </row>
@@ -27658,6 +28489,16 @@
       <c r="B569" t="inlineStr">
         <is>
           <t>BSMA0566</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
         </is>
       </c>
       <c r="G569" t="inlineStr">
@@ -27715,6 +28556,11 @@
           <t>2004</t>
         </is>
       </c>
+      <c r="P569" t="inlineStr">
+        <is>
+          <t>The study's unit of analysis is the project team (N=132 projects). The respondent serves as a key informant for the team's boundary spanning activities, violating the individual-level analysis requirement.. Verbatim Evidence: [5.4.1 Level of Analysis] "This dissertation explores the development of core competence in emerging technology innovation projects, and the level of analysis is at the project level." [5.4.1 Level of Analysis] "The use of surveys on a project participant as the source of data determines in large part the remaining research design." [5.4.4 Quantitative Sample] "Each survey represents a project with no more than 2 projects from a single firm." [Part II. Innovation Activities] "The purpose of this section is to identify the kinds of activities performed by the organization or group developing the MEMS project. Please indicate how often you or someone in the organization undertook the below activities in the development."</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -27727,6 +28573,16 @@
           <t>BSMA0567</t>
         </is>
       </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G570" t="inlineStr">
         <is>
           <t>A major US workforce trend of the new Millennium has been the decline in membership in private-sector unions. From a 1954 peak of 35% of the workforce, membership now sets at 11% of the workforce. To increase union membership, industry labor leaders are reviving the notion of dual commitment-that a worker can be loyal to both employer and union (Rose, 1952). Earlier attempts at using a unitary dual measure encountered methodological problems, so we explored the commitment attitudes individually. In a Qualtrics-based field study of a Midwest Teamsters local, we look at the degree to which various workplace factors are indicators of organizational and union commitment attitudes. Using hierarchical regression analysis to test hypotheses, we found a positive relationship between union commitment and union participation, and a lesser level of organizational commitment among the boundary-spanning union shop stewards than among rank-and-file employees. Other post-hoc patterns also emerged. Implications for labor officials and managers are discussed, as are ideas for future research. The study offers both practical information for the union leadership, and theoretical testing of the dual commitment phenomenon.</t>
@@ -27750,6 +28606,11 @@
       <c r="K570" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P570" t="inlineStr">
+        <is>
+          <t>The study does not measure Boundary Spanning Behavior; it merely uses the term 'boundary spanners' to describe the role of shop stewards and includes a dummy variable for having served as a shop steward.. Verbatim Evidence: [Chapter 2] "Research by Friedman and Podolny (1992) labels these people as boundary spanners, and explains how they play a central role in intergroup relations." [Chapter 3] "Shop Steward. This is a categorical, dichotomous variable to be used in a logistics regression equation. Whether a person has experience as a shop steward will be used to assess level of organizational commitment." [Appendix E] "Q9 In the last five years have you served as a shop steward? Yes (1) No (2)"</t>
         </is>
       </c>
     </row>
@@ -27816,6 +28677,16 @@
           <t>BSMA0569</t>
         </is>
       </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G572" t="inlineStr">
         <is>
           <t>Twenty years ago, most companies developed their own products in a single location and brought them to market themselves. Today, original equipment manufacturers (OEMs) are enlisting partners on a global scale as subsystem designers and producers in order to create and deliver new products into the market more rapidly and more frequently. This is especially true for large, complex products from the aerospace, telecommunications, electronics, and software industries. To assure the delivery of information across organizational boundaries, new coordination mechanisms need to be adopted (boundary management). In this article, best practices are described on how OEMs and partners self-organize and use agile, cooperative techniques to maintain daily communication among numerous internal and partner engineers to better coordinate product design and system integration. This article focuses on examples from the aerospace industry; however; these tactics can be applied in any organization to innovate at faster rates, to make delivery times more predictable, and to realize shorter product development timelines.</t>
@@ -27839,6 +28710,11 @@
       <c r="K572" t="inlineStr">
         <is>
           <t>2013</t>
+        </is>
+      </c>
+      <c r="P572" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 4] This is a conceptual and best-practices article rather than a primary empirical study. It contains no quantitative data, participant sample, or correlation matrix.. Verbatim Evidence: [Introduction] &lt;In this article, best practices are described on how OEMs and partners self-organize and use agile, cooperative techniques to maintain daily communication among numerous internal and partner engineers to better coordinate product design and system integration.&gt; [Introduction] &lt;Our information and examples are drawn from the field of aircraft development due to our experience in this area; however, the concepts can be generalized to any industry that features technology innovation and product development.&gt;</t>
         </is>
       </c>
     </row>
@@ -27979,6 +28855,12 @@
           <t>BSMA0573</t>
         </is>
       </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr"/>
       <c r="G576" t="inlineStr">
         <is>
           <t>In this article, we study the conditions under which having ties that span organizational boundaries (bridging ties) are conducive to the generation of innovations. Whereas previous research has shown that bridging ties have a positive impact on innovative performance, our analysis of 276 R&amp;D scientists and engineers reveals that there are no advantages associated with bridging per se. In contrast, our findings suggest that the advantages traditionally associated with bridging ties are contingent upon the nature of the ties forming the bridge—specifically, whether these bridging ties are Simmelian.</t>
@@ -28002,6 +28884,11 @@
       <c r="K576" t="inlineStr">
         <is>
           <t>2010</t>
+        </is>
+      </c>
+      <c r="P576" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28053,6 +28940,16 @@
           <t>BSMA0575</t>
         </is>
       </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G578" t="inlineStr">
         <is>
           <t>This study investigates the impact of environmental variability on communications within and outside a large R&amp;D laboratory. For high performing subunits, intra-project communication was found to be contingent on the nature of the unit’s task; extra-unit communication was inversely related to perceived environmental variability, suggesting that communication with external areas may be mediated by special boundary roles.</t>
@@ -28076,6 +28973,11 @@
       <c r="K578" t="inlineStr">
         <is>
           <t>1979</t>
+        </is>
+      </c>
+      <c r="P578" t="inlineStr">
+        <is>
+          <t>Team-level analysis (N=55 projects) and invalid construct (mere communication amount rather than purposive boundary-spanning behavior). [Code 1 &amp; Code 3]. Verbatim Evidence: Excluded due to team-level analysis and measuring mere communication volume. Verbatim Evidence: "[SETTING AND METHODS] Projects within the laboratory were the basic units of analysis. The study focused on all professionals in the facility (N=345)." "[Unit of Analysis] Because projects were the unit of analysis, individual responses were pooled." "[TABLE 2] Correlations Between Task Environment and Work Related Communication^a Total Sample (N=55)" "[Work Related Communication] The professionals were asked to report their actual, work related, verbal communications for a number of selected days (respondents were asked not to report strictly social communications, nor did they report written communications)." "[Work Related Communication] Project communication is a measure of the average absolute amount of work related communication per person per project over the 15 weeks."</t>
         </is>
       </c>
     </row>
@@ -28238,6 +29140,12 @@
           <t>BSMA0580</t>
         </is>
       </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr"/>
       <c r="G583" t="inlineStr">
         <is>
           <t>Abstract             Although recent years have seen a proliferation of research on organizational ambidexterity, important questions remain about the role that leaders play in leveraging learning ambidexterity for organizational benefits. Drawing on the conservation of resources theory, we investigate the indirect links between servant leadership and middle managers’ learning ambidexterity, with structural empowerment and role breadth self‐efficacy (RBSE) as serial mediators. We also examine the importance of leader boundary‐spanning behaviour as a moderating factor for these relationships. Using time‐lagged and multi‐source data from 344 middle managers and their supervisors, we show that servant leadership has a positive indirect influence on two forms of learning ambidexterity: exploitative and explorative learning. In particular, servant leadership promotes structural empowerment (as a contextual resource), which in turn influences RBSE (as a personal resource) and encourages learning ambidexterity. In addition, we show that when leaders engage in boundary‐spanning behaviour, these indirect relationships become more prominent. This research offers new theoretical and practical insights to assist organizations in improving learning ambidexterity and achieving higher levels of performance.</t>
@@ -28261,6 +29169,11 @@
       <c r="K583" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P583" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -28564,6 +29477,16 @@
           <t>BSMA0588</t>
         </is>
       </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G591" t="inlineStr">
         <is>
           <t>Recent team boundary spanning literature has recommended a shift toward assessing the role of virtual tools – such as social media. Simultaneously the proliferation of Enterprise Social Media (ESM) points to the need to theorize and investigate the supra-individual usage of these tools, such as their usefulness for organizational groups. This paper responds to both mandates through a theoretical integration of the team boundary spanning and existing ESM literature. Using data from two studies – one qualitative and one quantitative – this papers addresses two important research questions regarding the empirical relationship between team boundary spanning and ESM for understanding (i) the types of team boundary-spanning activities that group members enact through ESM and (ii) the effects of ESM on extra-team stakeholders’ perceptions and reciprocating actions vis-à-vis the team boundary-spanning activities of these group members. The results of this study show that ESM, largely as a function of their visibility affordance, supports a narrow set of representational activities, but offers only limited support for information search and coordination. Furthermore, the ﬁndings reveal that ESM activity has a positive effect on extra-team stakeholders’ recognition and ﬁnancial support of the representational ESM posts emanating from the boundary-spanning group. Important implications for theory, strategy, and design are discussed.</t>
@@ -28587,6 +29510,11 @@
       <c r="K591" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P591" t="inlineStr">
+        <is>
+          <t>The study does not report a zero-order correlation matrix, and its quantitative survey measures extra-team stakeholders' reciprocating actions rather than individual boundary spanning behavior.. Verbatim Evidence: [The quantitative study focuses on external stakeholders' reciprocating actions, not individual boundary spanning behavior, and does not provide a zero-order correlation matrix]. Verbatim Evidence: "[Data collection] For Study 2, aimed at characterizing the role of ESM in the formation of perceptions and reciprocating actions by extra-team stakeholders to the AR and FR blogs, we collected data from a variety of qualitative and quantitative data sources." [Data collection] "Rather than measure team boundary spanning per se, instead the scale measures an extra-team stakeholder’s possible recognition of and/or response to a team’s boundary-spanning efforts." [Results] "Given the exploratory nature of this study, we conducted basic regression analyses to assess the effect of ESM usage (recency and activity-level) as well as hierarchical level (position) on perceptions and reciprocations of team boundary-spanning activities to investigate Propositions 2 and 3b–5b."</t>
         </is>
       </c>
     </row>
@@ -28675,6 +29603,16 @@
           <t>BSMA0591</t>
         </is>
       </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G594" t="inlineStr">
         <is>
           <t>Widespread use of social media across work and non-work boundaries has heightened concerns about employee engagement in the contemporary workforce. This study examines how employees’ boundary management preferences inﬂuence their work communication on social media, and how these factors impact their engagement. Results from three waves of survey data (N = 361) demonstrate that work communication mediates the relationship between employee boundary preferences and engagement, supporting the hypothesized causal structure over alternative models. Overall, the ﬁndings contribute a novel perspective on employee engagement by showing that mediated work communication plays a central role in constructing engagement, rather than merely demonstrating it. We discuss how organizations can leverage this knowledge to address critical concerns about workplace (dis)engagement in the digital age.</t>
@@ -28698,6 +29636,11 @@
       <c r="K594" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P594" t="inlineStr">
+        <is>
+          <t>Construct Homonymy Trap: Measures work/non-work (work-family) boundary management preferences rather than inter/intra-organizational boundary spanning behavior.. Verbatim Evidence: [Theoretical background and hypotheses] "This research is informed by work/non-work boundary theory (Ashforth, Kreiner, &amp; Fugate, 2000; Nippert-Eng, 1996) and recent theorizing linking social media use to various forms of engagement." [Measures] "First we measured boundary preferences along a continuum based on existing measures by Kreiner, Hollensbe, and Sheep (2006) and Ilies, Wilson, and Wagner (2009). Participants rated their agreement with six statements relating to integration and segmentation preferences on a 5-point scale ranging from: 1 = not at all to 5 = very much."</t>
         </is>
       </c>
     </row>
@@ -28897,6 +29840,16 @@
           <t>BSMA0597</t>
         </is>
       </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G600" t="inlineStr">
         <is>
           <t>In this study, I assess the causal impact of boundary spanning on team innovation. I explore conditions and processes in 144 engagement teams in an enterprise software company driving innovation with customers in North America across industries. In this context, innovation is defined as the development and implementation of technology-based ideas in organizations. Using an integrated conditional process analysis, I find that boundary-spanning team practices combined with a shared vision and functional background diversity lead to a significant team innovation increase. I further assess the team process of information elaboration through which functional diversity and boundary spanning foster solution use. In particular, I argue that boundary spanning amplifies the effects of shared vision and information elaboration, leading to significantly increased team innovation. Consistent with this argument, I find that functional diversity's positive impact on team innovation through information elaboration is conditional on a shared vision, whereas the impact is more significant when team members share a commitment to common goals for their work. Therefore, my findings contribute actionable insight into how to enable cross-functional engagement teams to successfully drive customer innovation with enterprise software in the technology industry.</t>
@@ -28920,6 +29873,11 @@
       <c r="K600" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P600" t="inlineStr">
+        <is>
+          <t>Non-individual level (team-level analysis with N=144 teams). Verbatim Evidence: [Data and Sample] &lt;The unit of analysis is the customer engagement team with team sizes ranging from 3 to 27 and a median of 9 members, including but not limited to sales reps, industry and value advisors, solution and support engineers, enterprise architects, engagement managers, as well as product and adoption experts.&gt; [Descriptive Statistics] &lt;Individual team member responses were aggregated to the team level by computing the means resulting in 162 team cases.&gt; [Descriptive Statistics] &lt;The remaining 144 teams are the basis for the analysis, of which 77 received the treatment, and 67 constituted the control group.&gt; [Descriptive Statistics] &lt;Notes. N=144. * p &lt; .05. ** p &lt; .01&gt;</t>
         </is>
       </c>
     </row>
@@ -29082,6 +30040,16 @@
           <t>BSMA0602</t>
         </is>
       </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G605" t="inlineStr">
         <is>
           <t>Building upon the ambidexterity perspective, this study conceptualizes boundary-spanning activities as both transactional and learning to illuminate their different effects on IT employees’ job satisfaction. Specifically, we offer an overarching theoretical framework rooted in ambidexterity by connecting the role theory and knowledge acquisition perspective to reconcile the inconsistency of extant findings. Role overload has a mediating effect on the relationship between boundary-spanning activities (both transactional and learning) and job satisfaction, whereas knowledge acquisition mediates the relationship between learning boundary-spanning activities and job satisfaction. Furthermore, high achievement motivation and learning goal orientation moderate the positive effect of learning boundary-spanning activities on job satisfaction. The quantitative analysis of IT employees in Chinese state-owned enterprises largely supports our hypotheses. We conclude this paper by discussing theoretical and managerial implications for ambidexterity, boundary spanning, and job satisfaction.</t>
@@ -29105,6 +30073,11 @@
       <c r="K605" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P605" t="inlineStr">
+        <is>
+          <t>Valid quantitative study measuring intra-organizational boundary-spanning activities among IT employees with a correlation matrix provided.. Verbatim Evidence: [Sample] "To control the influence from the difference in industrial and organizational levels on the research results, this research conducted data collection among all employees in one state-owned enterprise in Chongqing, China." [Sample Size] "After matching the information, the researchers formed the data from 112 samples... 110 valid questionnaires remained." [Construct] "Learning boundary-spanning activities (4 items)... I often investigate the status quo of business segments. I often analyse and explore the system requirements for business segments. I often communicate with the business staff to attain their feedback on me or my department."</t>
         </is>
       </c>
     </row>
@@ -29345,6 +30318,16 @@
           <t>BSMA0608</t>
         </is>
       </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G611" t="inlineStr">
         <is>
           <t>Green innovation is critical for firms' sustainable development, and its antecedents have attracted extensive attention. However, how proactive boundary-spanning search enhances firms' green innovation remains unclear. Building on the resourcebased view and dynamic capabilities theory, we explore the impact of proactive boundary-spanning search on firms' green innovation and investigate the mediating role of two types of organizational resilience. Survey data are collected from 218 manufacturing firms in China, and hierarchical regression and bootstrap analysis are used to test hypotheses. The results demonstrate that proactive boundaryspanning search not only has an inverted U-shaped relationship with radical green innovation and incremental green innovation, but also has an inverted U-shaped relationship with precursor resilience and improvisation resilience. Moreover, the results show that precursor resilience and improvisation resilience partially mediate the inverted U-shaped relationship between proactive boundary-spanning search and the two types of green innovation. This research reveals the nonlinear relationship between proactive boundary-spanning search and green innovation, which enriches the research of green innovation by considering organizational resilience.</t>
@@ -29368,6 +30351,11 @@
       <c r="K611" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P611" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N=218 manufacturing firms) using key informants.. Verbatim Evidence: [Abstract] "Survey data are collected from 218 manufacturing firms in China, and hierarchical regression and bootstrap analysis are used to test hypotheses." [Method] "The respondents are middle and senior managers of manufacturing firms as they are familiar with the firms' development status and future strategy." [Measurement] "Proactive boundary-spanning search was adapted from Katila and Ahuja (2002) and Wang et al. (2020), including four items: “Our firm has many channels to search new domain knowledge ahead of competitors,” “Our firm can search new domain knowledge about R&amp;D, production, and marketing ahead of competitors,” “Our firm can search new domain knowledge about technology and management ahead of competitors,” and “Our firm can search more new knowledge ahead of competitors.”"</t>
         </is>
       </c>
     </row>
@@ -29382,6 +30370,16 @@
           <t>BSMA0609</t>
         </is>
       </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G612" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to analyze the mechanism underlying the impact of boundary-spanning search (BS) on the sustainable development ability (SDA) of service-oriented manufacturing enterprises and to emphasize the intermediary role of knowledge integration (KI). The moderating role of knowledge inertia on the link between BS and KI is also investigated.</t>
@@ -29405,6 +30403,11 @@
       <c r="K612" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P612" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N = 110 enterprises). Verbatim Evidence: [Abstract] "This study constructs direct, mediating and moderating effects, selects 110 service-oriented manufacturing enterprises as research samples and obtains empirical data from questionnaires and annual reports." [3.1 Data collection and processing] "Service-oriented manufacturing enterprises are taken as the research object of this paper." [3.1 Data collection and processing] "This paper selects a total of 110 according to the sample demand, which conforms to the criteria for determining the sample size. 110 service-oriented manufacturing enterprises were selected." [3.1 Data collection and processing] "Second, to obtain comprehensive and objective data, three experts from each enterprise completed the questionnaire. Then, dividing the answers of three interviewees of an enterprise into a group helped form a triangular verification to determine whether the data corroborate each other." [Table 3] "Table 3. Descriptive statistics and correlations (N = 110)"</t>
         </is>
       </c>
     </row>
@@ -29419,6 +30422,12 @@
           <t>BSMA0610</t>
         </is>
       </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr"/>
       <c r="G613" t="inlineStr">
         <is>
           <t>Previous studies on IT alignment have attempted to address if, and how, the presence of IT outsourcing can help attain IT alignment. In this study, we advance the literature by investigating how organizations appropriate IT outsourcing for achieving IT alignment. Specifically, drawing on the adaptive structuration theory (AST), we construct a model examining factors associated with outsourcing appropriation, including consensus of appropriation (COA) and faithfulness of appropriation (FOA), and how the latter are associated with IT alignment. To test our proposed model, we use a questionnaire survey of 170 IT executives working in Chinese firms. Our results indicate that both shared IT affordance for knowledge acquisition and boundary spanning positively affect COA and FOA. Boundary buffering positively affects the FOA, but not the COA. Further, our results also show the positive effects on IT alignment from COA and FOA, and the significant moderating effects of adoption of cloud computing and the non-significant moderating effects of degree of outsourcing in the relationships. Interestingly, the moderating effects of three cloud computing adoption modes (SaaS, PaaS, and IaaS) on the impact of outsourcing appropriation on IT alignment vary significantly. These findings enrich our understanding towards how to appropriate IT outsourcing for IT alignment and contribute to the literature on IT alignment in IT outsourcing.</t>
@@ -29442,6 +30451,11 @@
       <c r="K613" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P613" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29508,6 +30522,12 @@
           <t>BSMA0612</t>
         </is>
       </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr"/>
       <c r="G615" t="inlineStr">
         <is>
           <t>The turnover of IT professionals is a perpetual challenge for non-IT organizations. Based on selfcategorization theory, this study proposes that IT employees’ turnover may be mitigated by fostering their identification with non-IT organizations, which can be done by meeting various facilitative conditions. Guided by intergroup contact theory, we identify IT employees’ perceived alignment between IT and the core business of an organization (business-IT alignment), the extent of boundaryspanning activities that IT employees engage in, and the closeness of the relationships between IT and non-IT employees as the drivers of their organizational identification. Using survey data collected from organizations in different industries, we obtained empirical evidence supporting the positive effects of the perceived business-IT alignment, the extent of boundary-spanning activities, and the relationship closeness between IT and non-IT employees on IT employees’ organizational identification. Additionally, there was a three-way interaction effect among the three drivers such that the relationship closeness between IT and non-IT employees reduced the positive effect of the extent of boundary-spanning activities on IT employees’ organizational identification when business-IT alignment was low. However, this negative moderating effect diminished when business-IT alignment increased. The findings of this research advance the literature and offer practical guidelines for non-IT organizations on how to enhance their IT employees’ organizational identification and how to mitigate their turnover intentions.</t>
@@ -29531,6 +30551,11 @@
       <c r="K615" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P615" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -29550,6 +30575,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate the individual effects of boundary-spanning search from suppliers (supplier-side search (SS)). It is proposed that SS contributes to innovation ambidexterity (IA) and then business performance (BP). Further, this paper includes buyer–supplier relationships (BSRs) and competitive intensity (CI) as moderators to clarify boundary conditions.</t>
@@ -29645,6 +30671,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr">
         <is>
           <t>This study utilizes network exploitation and exploration theory to distinguish the exploitative and exploratory mechanisms (government support and boundary-spanning learning, respectively) that convert political ties into firm innovativeness. It also examines the moderating roles market uncertainty plays in how political ties influence firm innovativeness. An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness. Market uncertainty negatively moderates the impact of political ties on boundary-spanning learning but does not significantly moderate their impact on government support. Moreover, market uncertainty moderates the impact of government support on firm innovativeness negatively but moderates the impacts of boundary-spanning learning on firm innovativeness positively. This study theorizes two mediating factors for how firms exploit and explore their political ties to increase their innovativeness and enriches the knowledge of how market uncertainty affects the relationship between political ties and innovation.</t>
@@ -29692,6 +30719,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G619" t="inlineStr">
         <is>
           <t>Organizational values and beliefs significantly influence employee decision making and behavior and manifest themselves as multiple climates existing within a single organization. A subset of organizational climate is an ethical climate, embodying normative values and beliefs involving moral issues shared by the employees of the organization. Reseachers have found multiple ethical climates present in an organization.</t>
@@ -29719,7 +30751,7 @@
       </c>
       <c r="P619" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>No effect size of interest; boundary spanning is not measured as an individual behavior but used as a categorical department classification, and no correlation matrix is provided.. Verbatim Evidence: [Construct Validity] "Finally, three boundary-spanning departments were selected (n = 56, response rate = 90%.) Customer service is the task of these departments: commercial lending, branch banking, and business services. Each department's primary objective is the service of a stakeholder external to the firm." [Data Availability] "Consistent with Victor and Cullen's original statistical analysis of their data investigating the relationship between firms and ethical climate types, a multivariate analysis of variance (MANOVA) was conducted to test the hypotheses depicting relationships between department types and ethical decision components and climate types."</t>
         </is>
       </c>
     </row>
@@ -29739,6 +30771,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G620" t="inlineStr">
         <is>
           <t>Boundary‐spanning communication has been found to be important to various types of organizations and groups as a source of new information and awareness of environmental changes. Although the importance of formal, public channels in building the knowledge base of a field has long been recognized, most studies of boundary‐spanning activity have been limited to direct, personal (informal) communication. This study examines both informal and formal communication patterns of three groups in order to determine whether, in fact, a variety of media are used in boundary‐spanning communication. The groups selected were the members of three professions which fill intermediary positions between the creators and consumers of cultural products; one located in academia and two in the private sector. Major findings were that: (1) A boundary‐spanning structure linking 82.2% of the survey respondents was composed of both informal and formal media. (2) The professions differed in which type of channel was most heavily used, but were similar in their perceptions of the importance of the channels. (3) Individuals central to the informal part of the structure were also more likely to use the formal parts of the structure. (4) Boundary‐spanning media were among the five most frequently cited media for all three of the professions.</t>
@@ -29766,7 +30803,7 @@
       </c>
       <c r="P620" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>The study evaluates communication channel usage (e.g., journals, conferences, personal discussion) rather than purposive boundary-spanning behavior. It only provides descriptive statistics and chi-square tests, completely lacking a zero-order correlation matrix with extractable effect sizes.. Verbatim Evidence: [Methodology] "Questions in the survey instrument were designed to identify informal and formal communication channels used by respondents. Respondents were asked to list journals read most often, associations and organizations in which they held memberships, and conferences and book fairs which they found most interesting or useful to attend." [Methodology] "The importance of the informal and formal channels was assessed through two partial measures. First, the questions described above permit a tally of the total number of respondents using and, therefore, linked by each channel. Second, a bank of questions in the instrument asked respondents to rate the importance of personal discussion, reading of professional and scholarly journals, and attendance of conferences and book fairs."</t>
         </is>
       </c>
     </row>
@@ -29928,6 +30965,12 @@
           <t>BSMA0621</t>
         </is>
       </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr"/>
       <c r="G624" t="inlineStr">
         <is>
           <t>Summary             We examine how demographic context influences the trust that boundary spanners experience in their dyadic relationships with clients. Because of the salience of age as a demographic characteristic as well as the increasing prevalence of age diversity and intergenerational conflict in the workplace, we focus on team age diversity as a demographic social context that affects trust between boundary spanners and their clients. Using social categorization theory and theories of social capital, we develop and test our contextual argument that a boundary spanner's experience of being trusted is influenced by the social categorization processes that occur in dyadic interactions with a specific client and, simultaneously, by similar social categorization processes that influence the degree to which the client team as a whole serves as a cooperative resource for demographically similar versus dissimilar boundary spanner–client dyads. Using a sample of 168 senior boundary spanners from the consulting industry, we find that generational diversity among client team members from a client organization undermines the perception of being trusted within homogeneous boundary spanner–client dyads while it enhances the perception of being trusted within heterogeneous dyads. The perception of being trusted is an important aspect of cross‐boundary relationships because it influences coordination and the costs associated with coordination. © 2015 The Author Journal of Organizational Behavior Published by John Wiley &amp; Sons Ltd</t>
@@ -29951,6 +30994,11 @@
       <c r="K624" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P624" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -30017,6 +31065,16 @@
           <t>BSMA0623</t>
         </is>
       </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G626" t="inlineStr">
         <is>
           <t>This study examines the concept of intra-organizational links as a way for boundary spanners to bring into the project group the information needed to deal with task uncertainty. Several studies have shown that heterogeneous groups are superior to homogeneous groups when novel or creative solutions need to be developed to deal with tasks characterized by high task uncertainty. For boundary spanners in engineering project groups, it is proposed that cross-departmental technical advice links are another source of the information needed to deal with task uncertainty. An empirical test supports the proposition that for high-performing project groups, boundary-spanning technical advice links may compensate for a lack of internal group heterogeneity and vice versa. This is not the case for low-performing project groups. Implications of these finding are presented, including the direction that the open innovation research stream might take to address the findings of this study.</t>
@@ -30040,6 +31098,11 @@
       <c r="K626" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P626" t="inlineStr">
+        <is>
+          <t>Non-individual level (team-level analysis). Verbatim Evidence: [Measures and procedures] "Since the project group is the unit of analysis in the present study, all variables were aggregated to group means." [Measures and procedures] "Using the guidelines found in Kenny and La Voie [1985], it was determined that aggregation to the group level was justified." [Group performance] "Based on these top-management ratings, the 49 project groups were divided into two categories, low performers (n = 24) and high performers (n = 25), by splitting the performance ratings as near as possible at the median."</t>
         </is>
       </c>
     </row>
@@ -30217,6 +31280,16 @@
           <t>BSMA0628</t>
         </is>
       </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G631" t="inlineStr">
         <is>
           <t>Productive relationships between a company and its customers are often the result of positive relationships between the company and its boundary spanning employees. The career entry transition marks the beginning of these interpersonal relationships, which have a significant impact on marketing performance. Using a sample of newly hired boundary spanning employees, we examine the influence of individual difference factors on boundary spanners’ appraisals of the career entry transition. Significant relationships are found between boundary spanners’ positive and negative appraisals of the transition and personal and non-organizational factors: perceived centrality of the work role, availability of resources (finances, social support, personal hope), and sense of coherence.</t>
@@ -30240,6 +31313,11 @@
       <c r="K631" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P631" t="inlineStr">
+        <is>
+          <t>The study samples employees in boundary spanning roles but measures their cognitive/affective appraisals of the career entry transition rather than boundary spanning behavior (BSB) itself.. Verbatim Evidence: [Sample] "Boundary spanners (N = 104) from a variety of industries were included in the study subject to two constraints: (1) they were ages 20-26, and (2) they had been working full-time nine months or less since graduation from a four-year college." [Measures] "Appraisal was conceptualized as two unipolar constructs rather than as a single bipolar construct in order to assess the nature of positive and negative appraisals." [Measures] "To determine each respondent’s perceptions of the centrality of both their college role and their career role, a scale was developed from existing measures of attitude toward objects and attitude toward acts (Batra &amp; Ray 1986; Maheswaren &amp; Meyers-Levy 1990)."</t>
         </is>
       </c>
     </row>
@@ -30254,6 +31332,16 @@
           <t>BSMA0629</t>
         </is>
       </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>4 = Non-primary study</t>
+        </is>
+      </c>
       <c r="G632" t="inlineStr">
         <is>
           <t>Over the last five years, the once vaulted system known as product management has been under attack. Challenged by a variety of mega‐trends, including rising consumer expectations and expertise, revolutionary changes in technology, and shifting power in channels of distribution, product managers now face an environment much more demanding than that of the past. Examines the role of product managers of consumer goods in this new environment, within the context of a conceptual model developed to understand better the dynamics underlying their job performance and satisfaction. The model highlights the interactions among boundary spanning, information power and interfunctional coordination, and incorporates the concepts of strategic orientation, role conflict and role ambiguity. In all, 17 propositions are advanced for future empirical testing.</t>
@@ -30277,6 +31365,11 @@
       <c r="K632" t="inlineStr">
         <is>
           <t>1994</t>
+        </is>
+      </c>
+      <c r="P632" t="inlineStr">
+        <is>
+          <t>Conceptual paper proposing a theoretical model of product managers' boundary spanning, with no empirical data.. Verbatim Evidence: [Introduction] "Drawing on boundary spanning theory, role dynamics theory and strategic contingency theory, this work offers a new conceptualization of the product manager's role and postulates a series of relationships to explain product managers' job performance and satisfaction." [Conclusion] "While theoretically compelling, empirical verification of the proposed linkages in the model is required."</t>
         </is>
       </c>
     </row>
@@ -30343,6 +31436,16 @@
           <t>BSMA0631</t>
         </is>
       </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G634" t="inlineStr">
         <is>
           <t>This study is the first to examine the mediating role of boundary-spanning search and the moderating role of partner similarity in horizontal coopetition for sustainable product innovation. Analyzing empirical data from 236 Chinese firms, we found that horizontal coopetition positively impacts both proactive search (aimed at surpassing competitors) and responsive search (aimed at following competitors), with a stronger influence on proactive search. Both search types mediate the relationship between horizontal coopetition and sustainable product innovation. Furthermore, greater competing similarity (e.g., market coverage) between firms and their partners increases firms' inclination toward proactive search under the influence of horizontal coopetition but weakens their tendency for responsive search. Conversely, greater cooperating similarity (e.g., corporate culture) increases firms' inclination toward responsive search under the influence of horizontal coopetition but weakens their tendency for proactive search.</t>
@@ -30366,6 +31469,11 @@
       <c r="K634" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P634" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N=236 firms) where senior managers act as key informants rating their company's boundary-spanning search.. Verbatim Evidence: [Firm-level analysis and Key Informant] Verbatim Evidence: "[3.1 | Samples and Data Collection] To avoid potential common method bias, we employed a multiple-informant approach to collect our data (Podsakoff et al. 2012). First, we selected two senior managers from each company to serve as our key informants. These senior managers possess extensive knowledge about their firms' interfirm cooperative activities and innovation performance." "[3.1 | Samples and Data Collection] In total, 321 questionnaires were returned, and after rigorous screening, 85 invalid questionnaires were excluded, resulting in a total of 236 responses received." "[3.1 | Samples and Data Collection] The final sample included companies from 18 cities in China, primarily concentrated in provinces and cities such as Shaanxi, Jiangsu, Henan, and Guangzhou." "[TABLE 1 | Measures and validation.] Our company prefers to collect information with no identifiable strategic market needs to ensure experimentation in the project, aiming to surpass competitors."</t>
         </is>
       </c>
     </row>
@@ -30380,6 +31488,16 @@
           <t>BSMA0632</t>
         </is>
       </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G635" t="inlineStr">
         <is>
           <t>Purpose – Two challenges faced by automotive component design projects within contracted design agencies are (1) specification changes requested by the manufacturers and (2) product information or core technology knowledge leakage to external actors. We examine the effects of targeted boundary activities that address these challenges under the contingencies of environmental uncertainty and project complexity.</t>
@@ -30403,6 +31521,11 @@
       <c r="K635" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P635" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Project-level analysis (N=234 projects) and measures boundary buffering rather than spanning; actual BSB variable is omitted from the correlation matrix.. Verbatim Evidence: [2.2 External uncertainty and internal complexity] "The unit of analysis is the new product design team considered at the project level." [3.1 Sample and data collection] "For testing the hypotheses, a survey method was employed, which collected quantitative data from 234 auto-component design projects in 124 automobile design organizations in China." [3.1 Sample and data collection] "In the 124 participating design agencies, 245 projects were identified by this process. After deleting 11 unreturned or incomplete responses, 234 usable observations are used for further data analysis." [Table IV] "Note(s): *p &lt; 0.01, sample size = 234" [3. Research methodology] "Project team boundary spanning has a potential interaction with buffering work on the project performance (Dey and Ganesh, 2017)." [Table III] "The project manager conducts the following activities ... Deflect outside pressures on the team ... Shield the team from outside interference ... Prevent overloading the team with external information and requests ... Withhold news about the team until an appropriate time ... Avoid releasing product information to others in the company ... Release only information that presents the desired profile"</t>
         </is>
       </c>
     </row>
@@ -30617,6 +31740,16 @@
           <t>BSMA0638</t>
         </is>
       </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G641" t="inlineStr">
         <is>
           <t>Purpose – The consulting team intervenes in the integrated construction consulting (ICC) network structure centered on “client-contractor-consultant.” Team boundary-spanning behavior (TBB) driven by the network structure is crucial to project performance. This article investigated how to stimulate the consulting project performance (CPP) improvement by considering the interactive effect of network structure and TBB. To be specific, this paper explored the configuration between structural characteristics of project networks, the dimension of TBB, and project performance in ICC projects.</t>
@@ -30640,6 +31773,11 @@
       <c r="K641" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P641" t="inlineStr">
+        <is>
+          <t>Non-individual level (team/project analysis via key informant). Verbatim Evidence: [Abstract] "This study collected 216 valid responses from construction professionals (including project managers, department managers, and project engineers) via a questionnaire survey and analyzed the data using fsQCA." [Table 1] "AB1 The ICC team frequently convinces the client of the feasibility of supporting the team’s activities or decisions" [Table 1] "CPP1 The project meets project management performance objectives and provides better cost or schedule control or quality control than would otherwise in a traditional model"</t>
         </is>
       </c>
     </row>
@@ -30691,6 +31829,16 @@
           <t>BSMA0640</t>
         </is>
       </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G643" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate how market orientation (MO) motivates ﬁrms to develop business model innovation and how such effects are moderated by strategic ﬂexibility. Design/methodology/approach – In this study, a questionnaire-based survey was undertaken to test the proposed hypotheses. The empirical study was conducted on a sample of 204 ﬁrms using two key informants (408 respondents) in China. The regression model is used to test the proposed model.</t>
@@ -30714,6 +31862,11 @@
       <c r="K643" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P643" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Firm-level analysis using key informants to measure Market Orientation, not individual Boundary Spanning Behavior.. Verbatim Evidence: [Abstract] "The empirical study was conducted on a sample of 204 firms using two key informants (408 respondents) in China." [Methodology] "Because of missing data, our final sample includes 204 firms, which represented a response rate of 35.2 per cent." [Measures] "Following the work of Yannopoulos et al. (2012) and Lamore et al. (2013), we asked senior managers to indicate, on a 1-5 Likert scale, the extent to which nine different statements were true regarding MO in their firms over the past three years." [Measures] "Six of the statements pertain to RMO: 1 We constantly monitor our level of commitment and orientation to serving customers’ needs." [Measures] "2 Our strategy for competitive advantage is based on our understanding of needs."</t>
         </is>
       </c>
     </row>
@@ -30770,7 +31923,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F645" t="inlineStr"/>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G645" t="inlineStr">
         <is>
           <t>Purpose – In today’s complex and rapidly changing business environment, cross-boundary growth is increasingly critical to the survival or even success of organizations. The purpose of this study is to examine the forming mechanism of ﬁrm’s cross-boundary growth by integrating the two important antecedent factors of performance pressure and managerial discretion into a united framework and theoretically analyze the direct role of performance pressure on ﬁrm’s cross-boundary growth as well as reveal the moderating role of managerial discretion. Also, the authors select listed manufacturing companies in China as samples to empirically test the research hypotheses.</t>
@@ -30798,7 +31955,7 @@
       </c>
       <c r="P645" t="inlineStr">
         <is>
-          <t xml:space="preserve">The study conducts a firm-level analysis using panel data of 1,334 listed manufacturing companies from a financial database. The dependent variable is firm-level cross-boundary growth (measured by the Herfindahl Index of cross-regional and cross-industry revenue), and it does not measure interpersonal boundary-spanning behavior by individual employees.. Verbatim Evidence: </t>
+          <t>[Code 1 &amp; Code 2 &amp; Code 3] The study analyzes firm-level cross-boundary growth (measured via Herfindahl index on sales revenue) using archival data from listed companies, not individual-level interpersonal BSB.. Verbatim Evidence: [Participants] "This study adopts the A-stock manufacturing listed companies on the main boards of Shenzhen and Shanghai in China from 2013 to 2016 as the sample." [Participants] "The sample data sources mainly come from the Wind Database, which is mainland China’s leading financial database and software services provider and has built up a huge, complete and accurate data warehouse focused on the financial securities data, covering stocks, funds, bonds, foreign exchange, insurance, futures, financial derivatives, spot trade, macroeconomics, financial news and other fields." [Participants] "Thus, the final sample is 1,334 firms with 3-year observation period from 2013 to 2016, and the number of firm-year observations is 4,002." [Measures] "This paper adopts the Herfindahl Index developed by Berry (2014) to measure firm cross-regional growth." [Measures] "Similarly, the paper uses the Herfindahl index to measure firm cross-industry growth."</t>
         </is>
       </c>
     </row>
@@ -30813,6 +31970,16 @@
           <t>BSMA0643</t>
         </is>
       </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G646" t="inlineStr">
         <is>
           <t>Purpose – The rapid advancement of digital transformation requires a shift in firms’ focus from past met needs to both latent future and unmet past needs. However, how boundary-spanning search with future orientation and past orientation affects breakthrough innovation remains unclear. This study thus aims to investigate the relationship between boundary-spanning search and breakthrough innovation from the perspective of search orientation.</t>
@@ -30836,6 +32003,11 @@
       <c r="K646" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P646" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N=314 firms) using key informants to rate organizational boundary-spanning search.. Verbatim Evidence: [Research design] "This study selected China’s advanced manufacturing firms as the research sample" [Research design] "Given that the directors of R&amp;D department have a broad view on firms’ innovation activities (Atuahene-Gima K, 2005), we issued the final questionnaire to them. After several reminders, we received 352 responses and finally got 314 usable responses by excluding invalid ones, generating an effective response rate of 34.9%." [Variables and measurement] "Forward-looking search (FLS) ... FLS1. Our company continuously scans for external knowledge to capture key trends and potential opportunities for new products"</t>
         </is>
       </c>
     </row>
@@ -30850,6 +32022,12 @@
           <t>BSMA0644</t>
         </is>
       </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr"/>
       <c r="G647" t="inlineStr">
         <is>
           <t>Although the critical role of boundary-spanning search in facilitating sustainable competitive advantage (SCA) has been recognized, how boundary-spanning search affects SCA under the conditions that competitors also search remains unclear. By considering competition, this study divides boundary-spanning search into proactive and responsive searches, and develops a theoretical model, in which proactive and responsive searches respectively influence exploratory and exploitative innovations, and subsequently enhance SCA. Empirical results from Chinese advanced manufacturing firms show that proactive and responsive searches have inverted Ushaped effects on SCA. Additionally, when the levels of proactive and responsive searches are low and moderate, exploratory innovation plays a complementary mediating role between proactive search and SCA, whereas exploitative innovation plays a complementary mediating role between responsive search and SCA. When considering competition, this study offers a crucial condition under which exploratory and exploitative innovations can transform the efforts of boundary-spanning search to SCA.</t>
@@ -30873,6 +32051,11 @@
       <c r="K647" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P647" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -30892,7 +32075,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F648" t="inlineStr"/>
       <c r="G648" t="inlineStr">
         <is>
           <t>Summary                            Team creativity, as one of the most important sources of organizational competitiveness and continuous innovation, requires rich and non‐redundant information from both internal and external sources. Although an emerging line of research has shed light on the role of team boundary‐spanning activity in promoting creativity, it has solely focused on the mean level of team boundary‐spanning activity and rarely addressed the fact that not all team members engage in boundary‐spanning behaviors to the same extent. In this study, we broaden the existing knowledge by examining               when               and               how               the pattern of team boundary spanning, particularly the differentiation in team member boundary‐spanning activities, promotes team creativity. Based on the categorization‐elaboration model, we propose a curvilinear relationship between team member boundary‐spanning differentiation and creativity that is mediated through information sharing. Further, we add an important layer of understanding to the nature of this curvilinear relationship by identifying team goal interdependence as an important moderator. Using multisource data collected from two time points in 70 teams, we have received general support for our hypotheses. As such, we enrich the conversation about the importance of team boundary spanning by answering “               Whether               team boundary‐spanning differentiation fosters creativity, and               when               and               how               ?”</t>
@@ -30972,6 +32154,16 @@
           <t>BSMA0647</t>
         </is>
       </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G650" t="inlineStr">
         <is>
           <t>Innovation often involves high uncertainty, making it difficult for a single entrepreneurial decision-making logic to navigate effectively. Grounded in resource orchestration theory, we advance the discussion on entrepreneurial decision-making logics by examining the interplay between causation and effectuation, and their interactive impacts on innovation within new ventures. Using a multi-wave survey of 404 founding team members from 91 new ventures, we find that new venture innovation is enhanced by the synergy of causation and effectuation. Furthermore, the boundary-spanning behavior of founding teams mediates the relationship between the synergy and new venture innovation, and founding team trust positively moderates this mediated relationship. These insights contribute to understanding the entrepreneurial decision-making logics and strategic behaviors of founding teams as they pursue innovation.</t>
@@ -30995,6 +32187,11 @@
       <c r="K650" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P650" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -31046,6 +32243,12 @@
           <t>BSMA0649</t>
         </is>
       </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr"/>
       <c r="G652" t="inlineStr">
         <is>
           <t>Despite the general agreement of the importance of resources and capabilities to strategic change, the broader question of how resources and capabilities affect strategic change itself remains unresolved. This research focuses on one characteristic of the process of strategic change, i.e., its speed. This study investigates the relationship between dynamic capabilities, the speed of strategic change, and performance. We propose that technological capabilities, marketing capabilities, and market-linking capabilities, due to their absorptive capacity and boundary spanning attributes, will facilitate the speed of strategic change. Furthermore, the risk orientation of managers will moderate this effect such that it would be strengthened for relatively risk-taking managers. Finally, we argue that the speed of strategic change will have an inverted-U relationship with organizational performance. We test these hypotheses on a sample of 213 Chinese ﬁrms and ﬁnd that while dynamic capabilities facilitate rapid strategic change, the risk orientation of decision makers moderates this relationship, but not all as hypothesized. While faster implementation of strategic change has a positive effect on performance, strategic change carried out too quickly has negative performance repercussions. Our ﬁndings suggest that ﬁrms not only need to adjust strategies to complement the changing environment, but also have corresponding capabilities to enable rapid strategic change.</t>
@@ -31069,6 +32272,11 @@
       <c r="K652" t="inlineStr">
         <is>
           <t>2015</t>
+        </is>
+      </c>
+      <c r="P652" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -31083,6 +32291,16 @@
           <t>BSMA0650</t>
         </is>
       </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G653" t="inlineStr">
         <is>
           <t>With the development of economy, the innovation of enterprises can not meet the needs of enterprises. Knowledge transfer in industry-university-research alliance is the process of knowledge creation from universities and scientific research institutes, transfer to the enterprise and use the knowledge to create value. The establishment of industry-university-research alliance is conducive to the realization of knowledge transfer in universities and scientific research institutions to enterprises, expanding the knowledge stock of enterprises, and improving the ability of independent innovation. This paper summarizes the research results of domestic and foreign scholars, defines the connotation of industry-university-research alliance and alliance knowledge transfer, discussed the influence factors of alliance knowledge transfer, and makes research on knowledge transfer promotion measures. It can be used for reference to improve the knowledge transfer effect.</t>
@@ -31106,6 +32324,11 @@
       <c r="K653" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P653" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] Conceptual review paper with no empirical quantitative data and no effect size, focusing on firm/university level macro alliances.. Verbatim Evidence: [Abstract] "This paper summarizes the research results of domestic and foreign scholars, defines the connotation of industry-university-research alliance and alliance knowledge transfer, discussed the influence factors of alliance knowledge transfer, and makes research on knowledge transfer promotion measures." [The Connotation and Characteristics of Industry-University-Research Alliance] "From an economic point of view, the industry university research alliance is an economic activity mode that the participants have the resources to optimize the allocation of two times to get the best benefits [4]."</t>
         </is>
       </c>
     </row>
@@ -31120,6 +32343,12 @@
           <t>BSMA0651</t>
         </is>
       </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr"/>
       <c r="G654" t="inlineStr">
         <is>
           <t>In a recent study by CCL, 86 percent of senior executives said it is "extremely important" to work across boundaries in their current leadership roles. Yet, only 7 percent of these executives believe they are currently "very effective" at doing so. Closing this gap is both a critical challenge and a transformative opportunity for leaders and organizations in today's business environment. This white paper explores why boundary spanning leadership matters and how to make it happen.</t>
@@ -31143,6 +32372,11 @@
       <c r="K654" t="inlineStr">
         <is>
           <t>2016</t>
+        </is>
+      </c>
+      <c r="P654" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -31157,6 +32391,16 @@
           <t>BSMA0652</t>
         </is>
       </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G655" t="inlineStr">
         <is>
           <t>Purpose – The role of management control is frequently emphasized in connection with inter-organizational relationships and value networks. For example, boundary-spanning cost and accounting control techniques have been studied in multifaceted empirical settings. The prevalence of such techniques is, however, currently unknown in conjunction with companies’ interests to increase inter-organizational integration in general. Additionally, also the nexus between the internal state of cost management and the company’s willingness to develop inter-organizational relationships requires further investigation. The paper aims to discuss these issues. Design/methodology/approach – The study is based on an extensive survey that was responded to by more than 1,500 CEOs and CFOs from large, medium-sized and small Finnish enterprises in a variety of industries. As the authors chose the mixed-methods approach, both quantitative and qualitative data were collected for the study.</t>
@@ -31180,6 +32424,11 @@
       <c r="K655" t="inlineStr">
         <is>
           <t>2018</t>
+        </is>
+      </c>
+      <c r="P655" t="inlineStr">
+        <is>
+          <t>[Code 1 &amp; Code 3] The study measures firm-level boundary-spanning cost management techniques, not individual-level interpersonal BSB. The unit of analysis is companies, and CEOs/CFOs act as key informants for the organization.. Verbatim Evidence: [Participants] "The data were collected by conducting structured interviews over the phone with the respondents, who were senior managers, mainly either CEOs (1,103 respondents) or CFOs (403 respondents), in their respective organizations." [Participants] "An individual respondent (i.e. company) has been associated with a cluster with an icon and a matching color." [Measures] "Based on the responses to Q27 ("Does your company have any network-level cost accounting tools, methods or even systems in place?"), it seemed that around 7 percent of the companies were employing boundary-spanning control techniques."</t>
         </is>
       </c>
     </row>
@@ -31498,6 +32747,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G662" t="inlineStr">
         <is>
           <t>This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of noncore firms operating in the context of sustainable development. The dynamic nature of technological innovation, exacerbated by market flattening and the challenges posed by the COVID-19 pandemic, has compelled small and medium-sized enterprises (SMEs) to seek innovative breakthroughs. Cooperative innovation emerges as a strategic avenue for SMEs to mitigate risks and enhance their willingness to innovate. However, non-core firms often encounter technological and market disadvantages, hindering innovation efforts. This study explores how boundary-spanning knowledge search, which bridges the gap between non-core firms and the external environment, influences cooperative innovation. Furthermore, the research delves into the mediating role of both potential and actual absorptive capacity in the relationship between boundaryspanning knowledge search and cooperative innovation performance. Empirical findings indicate that boundary-spanning knowledge searches positively impact cooperative innovation, with technological and market knowledge searches yield significant results. Moreover, absorptive capacity exhibits a dual mechanism, directly influencing cooperative innovation and mediating the relationship between knowledge search and performance. This paper extends existing research by focusing on non-core firms within the sustainable development context, offering valuable insights for SMEs seeking innovative strategies. It also highlights the diverse pathways through which boundary-spanning knowledge search affects cooperative innovation. These findings offer practical implications for enhancing non-core firms’ innovation capabilities, including encouraging proactive knowledge search and developing absorptive capacity-inducing mechanisms through employee training and information platforms.</t>
@@ -31525,7 +32779,7 @@
       </c>
       <c r="P662" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>[Code 3 &amp; Code 99] Firm-level analysis (N = 182 non-core firms) and Retracted Article.. Verbatim Evidence: [Sample] "A total of 270 non-core firms whose senior managers agreed to take part in the survey were finally identified as the sample firms, and a roster was made." "After eliminating invalid questionnaires with blank or missing options, a total of 182 valid questionnaires were returned, with an effective rate of 67.4%." [Measures] "The scale used for boundary-spanning technological knowledge search (denoted as Tkb) is based primarily on the research findings of Sidhu et al. (2007) and Xiong et al. (2020) and is measured by setting six questions, such as “emphasis on the development of industries related to the company’s technology,” etc." "Following the studies of Lichtenthaler and Lichtenthaler (2009), the potential absorptive capacity (denoted as Pac) is measured by developing six questions, such as “Your company is able to recognize changes in the market,” and the actual absorptive capacity (denoted as Aac) is measured by setting up six questions, such as “Your company is able to recognize changes in the market Table 2.”"</t>
         </is>
       </c>
     </row>
@@ -31640,6 +32894,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>Local government or better known as the local authority vested with the power to plan, develop, and regulate businesses in the area within its jurisdiction plays a significant role in creating a conducive environment for businesses to grow and flourish. In playing this role, employees in local authority must possess a certain degree of innovative work behavior. This paper reports on a study that investigated innovative work behavior orientation among employees of the local government. A total of 100 employees of a local city council responded to a self-administered questionnaire on innovative work behavior. The results revealed that respondents scored a moderate high orientation on the innovative work behavior scale.</t>
@@ -31902,6 +33157,16 @@
           <t>BSMA0668</t>
         </is>
       </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G671" t="inlineStr">
         <is>
           <t>This study examines how individual purchasing agents function as boundary spanners with suppliers to inﬂuence trust development in themselves and the buying ﬁrms that employ them. Building upon boundary theory and supply chain cooperation research, we identify three boundary spanning capabilities of purchasing agents and empirically test how these capabilities shape buyer–supplier trust development. Using two samples of data collected from suppliers in the automotive industry and food industry, we found that a purchasing agent’s effectiveness in strategic communication with suppliers affects a supplier’s trust in the buying ﬁrm, while an agent’s professional knowledge and ability to reach compromises with suppliers affect a supplier’s trust in the purchasing agent representing the ﬁrm. Trust in the purchasing agent in turn affects trust in the buying ﬁrm. Theoretical and managerial implications are discussed.</t>
@@ -31925,6 +33190,11 @@
       <c r="K671" t="inlineStr">
         <is>
           <t>2011</t>
+        </is>
+      </c>
+      <c r="P671" t="inlineStr">
+        <is>
+          <t>Non-individual level of analysis (buying situations evaluated via team consensus). Verbatim Evidence: [4.1. Research setting and data collection] &lt;The buying situation was adopted as the unit of analysis since buyer–supplier relationship management practices in manufacturing industries vary significantly across buying situations (Laseter and Ramdas, 2002; Takeishi, 2001; Dyer and Hatch, 2006).&gt; [4.1. Research setting and data collection] &lt;We encouraged the salesperson to whom the survey questionnaire was directed to involve other supplier personnel who worked with the assembler to assist them in answering the questions, if they were uncertain of the appropriate response.&gt; [4.1. Research setting and data collection] &lt;By including an item in the survey asking how the survey was completed, we found that 55.5% of the completed questionnaires for the automotive assembler and 50.2% of the completed questionnaires for the food processor were completed by consensus reached among multiple supplier personnel who were familiar with their firm’s working relations with the manufacturer.&gt;</t>
         </is>
       </c>
     </row>
@@ -31944,6 +33214,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -31971,7 +33246,7 @@
       </c>
       <c r="P672" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Non-individual level (buying situation/relationship analysis). Verbatim Evidence: [4.1. Research setting and data collection] "We focus on the customer–supplier relationship at the buying situation level, which refers to a particular component type delivered to the customer firm by a supplier. Each buying situation represents a unique case, as relationship management practices can differ significantly among business units" [4.1. Research setting and data collection] "Usable data on all focal constructs was received on 198 buying situations for the U.S. sample and 181 buying situations for the European sample." [4.1. Research setting and data collection] "50.3% of the surveys in the European sample and 36.4% of the surveys in the United States were completed by consensus among multiple personnel working for the supplier"</t>
         </is>
       </c>
     </row>
@@ -31986,6 +33261,16 @@
           <t>BSMA0670</t>
         </is>
       </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G673" t="inlineStr">
         <is>
           <t>Purpose – This study extends the concept of managerial efficacy to include managerial means efficacy (MME) attributed to the utility and quality of means external to managers for performing a task. Focusing on its antecedents, the authors theorize and empirically test MME sourced from the organization (MMEO) and situate the examination under extreme events.</t>
@@ -32009,6 +33294,11 @@
       <c r="K673" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+      <c r="P673" t="inlineStr">
+        <is>
+          <t>Multiple reasons: [Code 1 &amp; Code 3] DV is an efficacy belief (not BSB), and the inter-organizational relationship construct is measured at the agency level via a proxy informant.. Verbatim Evidence: [Measurement] "We measure an agency's effectiveness in managing relationships with jurisdictional stakeholders with two variables: Horizontal Relationship Management with local stakeholders and Vertical Relationship Management with state or federal stakeholders. The two measures were based on a survey question asking respondents: 'How effective is your agency in managing its relationship with each of the following groups?' (1) mayor; (2) mayor's council or other elected officials; (3) city departments and agencies; (4) state governor; (5) state legislature; (6) state agencies; (7) federal government"</t>
         </is>
       </c>
     </row>
@@ -32212,7 +33502,8 @@
       </c>
       <c r="P677" t="inlineStr">
         <is>
-          <t>[Code 2 &amp; Code 3] The study uses archival patent data at the MNC-country-year level of analysis, not individual employee survey data.. Verbatim Evidence: [Code 2 &amp; Code 3] The study uses archival patent data and analyzes data at the MNC-country-year level rather than the individual employee level. Verbatim Evidence: "[3.1 | Sample and data collection] We investigated the concentration of cross-border collaborations in MNCs using data on listed pharmaceutical MNCs headquartered in the United States from 1980 to 2008." "[3.1 | Sample and data collection] We eventually obtained 97 MNCs involving 60,185 patents, whose overseas research operations are located across 24 host countries, comprising an unbalanced panel of 1954 MNC-country-year observations."</t>
+          <t>Excluded due to multiple flaws [Code 2 &amp; Code 3]. The study uses patent database records instead of surveying organizational employees (Code 2) and conducts its analysis at the MNC-host country and patent co-inventor network level (Code 3).. Verbatim Evidence: [Methodology] "We investigated the concentration of cross-border collaborations in MNCs using data on listed phar-
+maceutical MNCs headquartered in the United Stat es from 1980 to 2008." [Measures] "The data describing the granted patents allowed us to identify co-inventing collaborationsamong inventors within the same MNC and then build inventor networks."</t>
         </is>
       </c>
     </row>
@@ -32262,6 +33553,16 @@
       <c r="B679" t="inlineStr">
         <is>
           <t>BSMA0676</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
         </is>
       </c>
       <c r="G679" t="inlineStr">
@@ -32307,6 +33608,11 @@
           <t>2019</t>
         </is>
       </c>
+      <c r="P679" t="inlineStr">
+        <is>
+          <t>Firm-level patent and alliance analysis lacking individual BSB measures [Code 1 &amp; Code 2 &amp; Code 3].. Verbatim Evidence: [Abstract] "In my first essay, I propose that the information intermediated by the acquisition target privately and directly reduces information asymmetry between the acquiring firm and its inherited alliance network. I demonstrate that the acquiring firm is more likely to direct its knowledge search towards the inherited alliance partners of the acquired firm as the acquirer can gain more information about them through the acquisition." [Data and Method] "We constructed a dataset containing acquisitions and the acquired firms’ networks of alliances in the biotechnology industry." [Sample and Data] "We then aggregated all individual inventor-year level data up to the firm-year level. In the context of new ventures, initial public offers (IPOs) and mergers and acquisitions (M&amp;As) are strong signals of the firm’s quality or result in the firm no longer operating as an independent organization. In order to isolate the effect of VC prominence and alliance formation, we run the analyses using the years previous to a new venture’s IPO or to the acquisition of the new venture. Therefore, our final sample consists of a panel dataset of 1709 firm-year observations, and we engage in firm fixed effects negative binomial models to test our hypotheses."</t>
+        </is>
+      </c>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr">
@@ -32319,6 +33625,16 @@
           <t>BSMA0677</t>
         </is>
       </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G680" t="inlineStr">
         <is>
           <t>Purpose – The complex and changeable working environment makes individual cross-boundary activities inevitable. Yet, how employee’s boundary-spanning behavior (BSB) stimulates innovation performance remains to be further explored. This study aims to analyze the intermediary mechanism and boundary conditions between employee’s BSB and innovation performance based on knowledge integration theory.</t>
@@ -32342,6 +33658,11 @@
       <c r="K680" t="inlineStr">
         <is>
           <t>2021</t>
+        </is>
+      </c>
+      <c r="P680" t="inlineStr">
+        <is>
+          <t>Valid individual-level study with N=286 employees, measuring employee BSB using Ancona &amp; Caldwell (1992) scale and providing a zero-order correlation matrix.. Verbatim Evidence: [Sample] "We collected data in two waves (July and August 2017) and from two hierarchical levels (from the final sample of 286 employees and their 29 direct supervisors) within ten manufacturing firms located in Nanjing and Anhui, China." [Measures] "Following the existing research study, we used the three-item scale of the information collection dimension developed by Ancona and Caldwell (1992) to measure employee’s BSBs. A sample item was “Collect technical information/ideas from individuals outside of the team.”" [Correlation Matrix] "Table 1. Means, standard deviations and correlations at the individual level"</t>
         </is>
       </c>
     </row>
@@ -32356,6 +33677,16 @@
           <t>BSMA0678</t>
         </is>
       </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G681" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to explore how boundary-spanning demand-side search (BSDSS) fuels radical technological innovations as well as how innovation appropriability moderates this relationship. In particular, based on Teece’s (1986) argument regarding the appropriability of innovation, the authors divide factors to influence innovation appropriability into two types: external institution related and internal capability related.</t>
@@ -32379,6 +33710,11 @@
       <c r="K681" t="inlineStr">
         <is>
           <t>2017</t>
+        </is>
+      </c>
+      <c r="P681" t="inlineStr">
+        <is>
+          <t>Firm-level analysis (N=150 firms) using key informants.. Verbatim Evidence: [Firm-level analysis (N=150 firms) using key informants]. Verbatim Evidence: "[Abstract] &lt;Specifically, the authors collected a sample composed of 150 high-tech manufacturing Chinese firms.&gt;" "[Sampling and data] &lt;Then, they required two top managers who are familiar with the firm’s strategies and innovation activities to finish the Part I and Part II of one questionnaire independently.&gt;" "[Sampling and data] &lt;Finally, we obtained 150 usable questionnaires, with a valid response rate of 30 percent.&gt;"</t>
         </is>
       </c>
     </row>
@@ -32393,6 +33729,16 @@
           <t>BSMA0679</t>
         </is>
       </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G682" t="inlineStr">
         <is>
           <t>Virtual teamwork has become a prevalent mode of collaboration. However, scant empirical attention has been given to the impact of virtual teamwork on individual members’ performance beyond the team setting. In this paper, we fill this gap by studying virtual teams in the context of online medical consultation (OMC) platforms. Specifically, we collect data from two OMC platforms during a time period when both platforms offered individual consultations (i.e., one patient connected with one physician) but only one offered team consultations (i.e., one patient connected with a team of physicians). Using a difference-in-difference-in-differences approach, we find that team participation has a robust, positive effect on physicians’ performance in individual consultations. We further explore the potential mechanisms through which team participation improves physicians’ performance. The empirical results indicate that the observed performance improvement is likely driven by peer effects in team settings. In particular, we find that physicians exert more effort in individual consultations after joining a team, and that performance improvement is stronger when (1) a physician can easily observe the performance of his teammates (peers), (2) a physician has teammates (peers) who performs well in individual consultations, (3) a physician has teammates (peers) from the same hospital or the same city, or (4) a physician has a lower performance prior to joining in a team. Our findings shed new light on the boundary-spanning roles of virtual teams and provide timely insights into the ongoing development of OMC platforms.</t>
@@ -32416,6 +33762,11 @@
       <c r="K682" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P682" t="inlineStr">
+        <is>
+          <t>The study does not measure boundary spanning behavior as an interpersonal construct; it merely uses a binary indicator for virtual team membership on a digital platform and lacks a zero-order correlation matrix.. Verbatim Evidence: [Abstract] "Specifically, we collect data from two OMC platforms during a time period when both platforms offered individual consultations (i.e., one patient connected with one physician) but only one offered team consultations (i.e., one patient connected with a team of physicians). Using a difference-in-difference-in-differences approach, we find that team participation has a robust, positive effect on physicians’ performance in individual consultations." [4.1. Identification Strategy] "where Y_it^W denotes the number of satisfied reviews physician i received on day t on WeDoctor (i.e., SatiNum_it^W). After_it^W is a binary variable, which indicates whether physician i was part of a consultation team on WeDoctor on day t."</t>
         </is>
       </c>
     </row>
@@ -32430,6 +33781,16 @@
           <t>BSMA0680</t>
         </is>
       </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G683" t="inlineStr">
         <is>
           <t>Purpose – Although enterprise social media (ESM) offers new opportunities for developing radical creativity, limited research has been conducted on how to foster such creativity in ESM contexts. Based on the approachinhibition theory of power (AITP), this study examines how supervisor-subordinate instrumental and expressive ties on ESM promote radical creativity through sense of power. Furthermore, it further investigates how boundary buffering moderates the influence of these supervisor-subordinate ties on sense of power.</t>
@@ -32453,6 +33814,11 @@
       <c r="K683" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="P683" t="inlineStr">
+        <is>
+          <t>Valid individual-level quantitative study measuring ESM-enabled boundary spanning behavior among employees.. Verbatim Evidence: [Participants] "The data collection period lasted for one week, during which 378 responses were received. After excluding cases based on trap questions and answering time, 352 valid responses were retained for subsequent data analysis." [Measures] "ESM-enabled Boundary Spanning (BS) (Mell et al., 2022) BS1: I use ESM to solicit information and resources from external channels BS2: I make use of my relationships with external colleagues through ESM to support my work BS3: I actively use ESM to solicit external work resources BS4: My work depends upon information and resources actively solicited through ESM, that is, information and resources beyond what comes through official channels" [Correlation Matrix] "Table 3. Descriptive statistics and inter-construct correlations"</t>
         </is>
       </c>
     </row>
@@ -32467,6 +33833,16 @@
           <t>BSMA0681</t>
         </is>
       </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>5 = Multiple reasons (specify in Notes)</t>
+        </is>
+      </c>
       <c r="G684" t="inlineStr">
         <is>
           <t>Conﬂict among teams is inevitable in a multiteam system. Drawing on the theory of co-operation and competition, we proposed and tested a model linking the approaches teams adopt to conﬂict, inter-team co-ordination, and multiteam system performance. Data collected from 123 operation teams in 44 subway stations in Shanghai revealed that co-operative conﬂict management positively related to inter-team co-ordination, which in turn positively related to performance of the multiteam system. The relationship between competitive conﬂict management and inter-team co-ordination was insigniﬁcant and was moderated by co-operative conﬂict management. When co-operative conﬂict management was at a low level, competitive conﬂict management negatively related to inter-team co-ordination.</t>
@@ -32490,6 +33866,11 @@
       <c r="K684" t="inlineStr">
         <is>
           <t>2019</t>
+        </is>
+      </c>
+      <c r="P684" t="inlineStr">
+        <is>
+          <t>Excluded [Code 1 &amp; Code 3] because it uses station-level aggregated data (N=44 stations) and does not measure Boundary Spanning Behavior (focuses on conflict management and coordination measured via satisfaction).. Verbatim Evidence: [Participants and procedures] "Because the level of analysis was at the station level, we retained a station in the sample only when it had responses from no fewer than two team leaders as well as no fewer than two shift teams." [Participants and procedures] "With these criteria, the final sample consisted of 44 stations with 120 team leaders (mean = 2.7, SD = 0.8), 123 teams (mean = 2.8, SD = 0.8) and 492 members (mean = 11.2, SD = 4.1)." [Table 2] "N = 44." [Appendix 1] "Inter-team co-ordination (adapted from Hoegl, Weinkauf and Gemuenden 2004) 1 Generally speaking, employees from the various shifts are very satisfied with their work with each other. 2 Shift members feel a strong commitment to their joint work for the station."</t>
         </is>
       </c>
     </row>
@@ -32556,6 +33937,16 @@
           <t>BSMA0683</t>
         </is>
       </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G686" t="inlineStr">
         <is>
           <t>With the increasing uncertainty of the environment and the complexity of team tasks, it’s now common practice to encourage employees to implement boundary spanning behaviors. In spite of the fact that a few studies have explored the relationship between boundary spanning behavior and employee creative performance, little is known about the mechanism behind this association. Drawing on the conservation of resource theory (COR), this paper examines the mediating role of meaning of work and the moderating role of team Chaxu climate to reveal the internal process and boundary condition regarding the effect of boundary spanning behavior on employee creative performance. A sample of 211 supervisorsubordinate dyads from six companies located in China is collected in this study, and a hierarchical linear model is used to test the hypotheses. The results show that boundary spanning behavior has a positive effect on employee creative performance, meaning of work mediates the link between them, and team Chaxu climate negatively moderates the relationship between boundary spanning behavior and meaning of work. This research provides a new insight into the linkage between boundary spanning behavior and employee creative performance, as well as further answers the question “how and when boundary spanning behavior influences employee creative performance”.</t>
@@ -32579,6 +33970,11 @@
       <c r="K686" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P686" t="inlineStr">
+        <is>
+          <t>Valid individual-level quantitative study of employee boundary-spanning behavior.. Verbatim Evidence: [Methods] At Time 1, the research team invited 328 employees of the target companies to participate in a questionnaire, and data regarding boundary-spanning behavior, informal status, and Zhongyong thinking were collected. [Methods] There were 202 valid responses after removing responses that could not be correctly matched and those that presented regular answers. [Measures] The scale was developed by Marrone et al. (2007) and consisted of six items. Typical items include ‘persuade outsiders (e.g., faculty and clients) to support team decisions’ and ‘reach out to individuals outside of your team that can provide project-related expertise or ideas’. [Results] Table 1. Mean value, standard deviation, and correlation coefficient of each variable</t>
         </is>
       </c>
     </row>
@@ -32593,6 +33989,16 @@
           <t>BSMA0684</t>
         </is>
       </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G687" t="inlineStr">
         <is>
           <t>In the context of encouraging collaborative innovation, employee boundary spanning has become a source of organizational innovation. However, existing research has mainly explored the impact of employee boundary spanning on themselves from an actor-centered perspective, little is known about whether employee boundary spanning can influence supervisor support. Drawing on the perspective of positive interpersonal interaction, the current study employed a scenario experiment (Study 1) and a multi-wave and multi-source questionnaire survey (Study 2) to explore when and how employee boundary spanning affects supervisor support. Results from Study 1 (N= 220) indicated that when upward advice seeking is high, supervisors develop stronger cognitive trust and affective trust towards boundary spanning employees, leading to higher levels of supervisor support. Study 2 (N= 406) further confirmed that upward advice seeking positively moderates the direct effect of employee boundary spanning on supervisor affective trust as well as the indirect effect of employee boundary spanning on supervisor support via affective trust. However, it did not support the moderating effect of upward advice seeking on the supervisor cognitive trust path. These findings contribute to a comprehensive understanding of the impact of employee boundary spanning on supervisor support, providing decision-making references for organizations to manage employee boundary spanning to maintain harmonious supervisor-subordinate relationships.</t>
@@ -32616,6 +34022,11 @@
       <c r="K687" t="inlineStr">
         <is>
           <t>2024</t>
+        </is>
+      </c>
+      <c r="P687" t="inlineStr">
+        <is>
+          <t>Valid individual-level field study (Study 2) measuring employee boundary spanning behavior with a zero-order correlation matrix.. Verbatim Evidence: [Abstract] "For the field study, we conducted a three-wave questionnaire survey and collected data from 406 supervisor-employee dyads in knowledge-intensive firms in Hubei, Zhejiang, Shanghai, and Beijing provinces." [Measures] "员工跨界。借鉴Ancona 和Caldwell (1992)编制的团队跨界行为量表，结合具体研究情境，通过专家意见和员工反馈，从使节行为、任务协调行为和侦测行为选取13 题项以全面反映员工跨界行为，由员工自评。"</t>
         </is>
       </c>
     </row>
@@ -32630,6 +34041,12 @@
           <t>BSMA0685</t>
         </is>
       </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr"/>
       <c r="G688" t="inlineStr">
         <is>
           <t>To comprehend the mechanism of decent work’s impact on employee boundaryspanning behaviour, this paper constructs a research framework that includes promotion focus and a supportive organizational climate as a mediating factor and moderating variable. A two-stage survey is used to examine these assumptions with data collected from 346 frontline employees. The ﬁndings reveal that decent work has a signiﬁcant positive impact on employee boundary-spanning behaviour and promotion focus has a partial mediating eﬀect on this relationship. A supportive organizational climate plays a positive moderating role in the relationship between decent work and promotion focus.</t>
@@ -32653,6 +34070,11 @@
       <c r="K688" t="inlineStr">
         <is>
           <t>2023</t>
+        </is>
+      </c>
+      <c r="P688" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -32889,6 +34311,16 @@
           <t>BSMA0692</t>
         </is>
       </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G695" t="inlineStr">
         <is>
           <t>Boundary-spanning behavior has attracted considerable interest in recent years. Studies on this type of behavior have focused on its positive outcomes from the perspective of social networks. For decades, research has consistently demonstrated that the boundary-spanning behavior produces a wide array of positive results for teams and organizations. However, scholars have found that such behavior has negative outcomes for individuals. Using the conservation of resources theory (COR), we examined the double-edged-sword effect of boundary- spanning behavior on creativity at different levels, as well as its mediating mechanism and boundary conditions.</t>
@@ -32912,6 +34344,11 @@
       <c r="K695" t="inlineStr">
         <is>
           <t>2020</t>
+        </is>
+      </c>
+      <c r="P695" t="inlineStr">
+        <is>
+          <t>Valid individual-level quantitative study measuring boundary-spanning behavior with an extractable correlation matrix.. Verbatim Evidence: [Sample] "The sample of this study comes from several enterprises in Beijing, Shenzhen and Shanghai, mainly involving in finance, consulting, Internet and other industries." [Method] "We asked subordinates to rate their boundary-spanning behavior, role-breadth self-efficacy, role stress and subordinates' basic personal information." [Measures] "Boundary-spanning behavior. Using a scale developed by Faraj and Yan (2009), employees were asked to rate the extent to which they had received information and resources from outside the team." [Results] "Table 2 Mean, standard deviation and correlation coefficient of variables"</t>
         </is>
       </c>
     </row>
@@ -32978,6 +34415,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>Based on organizational learning theory, the influence of the transactive memory system of the top management team on business model innovation is discussed, as is the impact of different dimensions of boundary-spanning search on different business model innovation attributes when attention distribution is taken into account. Meanwhile, the moderating effects of environmental dynamism are considered. Regression and bootstrap analysis are used to test hypotheses. The results based on empirical research show that the transactive memory system has a positive effect on the dual attributes of business model innovation; acute boundary-spanning search and concentrated boundary-spanning search affect novelty-centered business model innovation and efficiencycentered business model innovation, respectively, and play mediating roles. Meanwhile, environmental dynamism positively moderates the relationship between acute boundary-spanning search and novelty-centered business model innovation, but negatively moderates the relationship between concentrated boundaryspanning and business efficiency-centered model innovation efficiency.</t>
@@ -33074,7 +34512,12 @@
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="G699" t="inlineStr">
@@ -33104,7 +34547,7 @@
       </c>
       <c r="P699" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Study uses a valid employee sample (working MBAs) reporting on their own intra- and inter-organizational information boundary spanning, with an extractable latent correlation matrix.. Verbatim Evidence: [Data Collection] "Data were collected from MBA students at two large Southeastern universities in the United States. Only respondents who were currently working in information intensive occupations were allowed to participate. The use of part-time evening students also provides a sample from an array of organizations that makes it reasonable to generalize the findings more broadly to a working professional." [Appendix B] "Boundary spanning taken from Keller and Holland (1975). Anchors: strongly disagree–strongly agree. 1. Fellow employees frequently seek job related information from me. 2. Individuals who are not part of my organization frequently seek job related information from me." [Results and Analysis] "TABLE 3. Reliabilities and correlations of study constructs."</t>
         </is>
       </c>
     </row>
@@ -33124,6 +34567,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
         <is>
           <t>This study adopts a temporal perspective to investigate how boundary spanners can increase the inflow of external knowledge by engaging with both external and internal parties. We add to prior work on knowledge transfer by shifting the focus from engagement levels to investigating engagement dynamics, especially the degree of switching between external and internal engagement across consecutive time periods. Drawing from a cognitive perspective, we argue that switching strongly between engagement types is associated with a segmented knowledge structure that enables quick and efficient categorical processing when knowledge can simply be “channeled” from source to recipient units. In contrast, weak or no switching is associated with a blended knowledge structure and more reflective processing, which is particularly helpful when knowledge transfer requires more translation and transformation. Correspondingly, we adopt a contingency perspective and theorize that the cognitive advantages associated with stronger versus weaker switching weigh differently, contingent on the stickiness of knowledge to be transferred and the nature of boundary-spanning activities that vary in importance over time. Fixed effects models of eight waves of original survey data reveal that, in line with our theorizing, the association between switching and knowledge transfer becomes increasingly negative (1) the more boundary spanners access knowledge that is transspecialist in nature, (2) the greater the organizational distance between source and recipient units, and (3) in later phases of the boundary-spanning process.</t>
@@ -33166,6 +34610,16 @@
           <t>BSMA0698</t>
         </is>
       </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G701" t="inlineStr">
         <is>
           <t>While digital product innovation offers unprecedented opportunities for incumbent firms to create competitive advantages, its fluid and iterative nature presents distinctive cognitive challenges. There is limited empirical literature explaining the role of constructive cognitive characteristics of executives in differentiating the successful pursuit of digital product innovation. Drawing on upper echelons theory and the attention-based view, we examine how chief executive officer (CEO) cognitive flexibility enables incumbent firms to pursue digital product innovation. Through a mixed-methods approach combining a field survey of 178 machine-building firms and a scenario-based experiment with 134 participants, we demonstrate that CEOs with higher cognitive flexibility achieve superior digital product innovation outcomes by facilitating insightful information acquisition and processing. This relationship is strengthened when CEOs engage in more boundary spanning activities and when firms possess greater social capital. Our study contributes to strategic leadership research by demonstrating how CEO cognitive flexibility enables incumbent firms to navigate the cognitive demands of digital product innovation, while enriching our understanding of how adaptive attention patterns shape strategic adaptation in increasingly digitized environments.</t>
@@ -33189,6 +34643,11 @@
       <c r="K701" t="inlineStr">
         <is>
           <t>2026</t>
+        </is>
+      </c>
+      <c r="P701" t="inlineStr">
+        <is>
+          <t>Valid individual-level BSB (CEO boundary spanning) with an extractable zero-order correlation matrix in Study 1.. Verbatim Evidence: [Measures] &lt;Specifically, we conducted interviews with ten CEOs participating in the survey on the theme of boundary spanning activities to refine the wording of the measurement items and ensure that they are consistent with the CEO’s actual activity scenario.&gt; [Table 2] &lt;1. I solicit information and resources from external channels. 2. I try to influence important external actors.&gt; [Sample and Data Collection] &lt;Our final sample of 178 firms comprises 124 responses collected through online surveys (69.7%) and 54 responses from onsite interviews (30.3%).&gt; [Table 3] &lt;Table 3. Descriptive statistics and correlation matrix&gt; &lt;11. CEO boundary spanning&gt; &lt;Notes: N = 178.&gt;</t>
         </is>
       </c>
     </row>
@@ -33208,6 +34667,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>
@@ -33252,7 +34712,12 @@
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>0 = Exclude</t>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="G703" t="inlineStr">
@@ -33282,7 +34747,7 @@
       </c>
       <c r="P703" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Includes valid employee sample (managers) and reports zero-order correlations for network degree centrality mapping contacts outside the organization, which is a valid BSB measure per Rule 18.. Verbatim Evidence: [Participants and procedure] "We collected the data from managers attending an Executive-MBA program at a business school in a large city in the United States." [Participants and procedure] "The students were managers who continued fulltime work while they studied. A total of 335 managers participated in this study, and 318 of them finished all the surveys." [Network measures] "The network survey allowed each participant (ego) to list up to 24 contacts (alters) whom they deemed most important in their professional network. They were instructed to list contacts who were significant in their professional networks in one or more of the following roles: providing economic resources, task information, career advice, and social support. Furthermore, alters could come from any context and were not restricted to the workplace."</t>
         </is>
       </c>
     </row>
@@ -33302,6 +34767,11 @@
           <t>0 = Exclude</t>
         </is>
       </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>
@@ -33329,7 +34799,7 @@
       </c>
       <c r="P704" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Macro-level analysis (organizational PR communication) in a qualitative dissertation.. Verbatim Evidence: [Abstract] The locus of analysis permits an analysis of an organization's communicative role and corresponding public participation status. The communicative role is the means and product of the organization's public relations communication.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: injected validation 2 intermediate results loop_2_13
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_Validation2.xlsx
+++ b/BSMA_AI_Run_Validation2.xlsx
@@ -5741,7 +5741,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Getting professionals who have been selected and trained to perform individually to work together is a major challenge. The objective of the article is to identify the mechanisms by which a coordinator can ensure a mediation and boundary spanning role to enable the achievement of a project. Adopting a comprehensive approach, this article is based on the case of an innovative hospital project ‘One-Day Diagnosis’ (1DD) – one day instead of several weeks – of hepatobiliary and pancreatic pathologies, for which the professionals had to change their practices. Based on the results of the study, the ﬁndings show that the mediating role of the coordinator consists in making things happen and guiding health care professionals through the innovative pathway until it becomes a routine process. The study contributes to the literature on collaboration and relational coordination by highlighting that the change of practices for collaboration is compatible with personal excellence, by outlining the active role of the boundary spanner in the change of these practices and by demonstrating that the organizational stability of projects based on disembodied procedures is a necessary illusion that requires complementary interindividual relationships and a living leadership.</t>
@@ -5789,7 +5788,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>The current study examined the relationships among role stress, proactive personality, employee creativity, and customer-oriented boundary spanning behaviors (COBSBs) for frontline service employees (FSEs). This study collected data from 382 FSEs in international hotels in Taiwan to test the research model. The empirical results revealed that employee creativity was positively affected by proactive personality but negatively affected by role conflict and role ambiguity. FSEs’ creativity positively affects COBSBs, including external representation, internal influence, and service delivery. Internal influence also positively affects service delivery and mediates the relationship between FSEs’ creativity and service delivery.</t>
@@ -5936,7 +5934,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>This dissertation examined the relationships between organizational characteristics and firms' timing of entry into emerging product markets. This study is an extension of a stream of research on endogenous entry models. Research on this area essentially holds that not all firms have the same entry skills and costs. Therefore, a firm's entry timing decision is attributable to factors internal to the organization. In this dissertation, specific attention is directed toward the effects of top management team (TMT) demography, corporate governance, level of diversification, boundary spanning, past performance, capital structure, and firm size on entry timing. These organizational characteristics have been shown to be critical determinants of timing in the strategic management literature, but, remain almost unexplored in the entry timing research. Thus, through including these organizational characteristics, this study extends the current knowledge which is critical for answering the question: Why do some firms enter emerging product markets earlier/later than others?</t>
@@ -5984,7 +5981,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>Organisations experience increased social, political and economic pressure that is evident in the increased pressure that stakeholders place on organisations. Organisations increasingly realise that stakeholders’ values and objectives need to be incorporated into organisational strategy as well as the day-to-day management of the organisation. Organisational success and survival consequently depends on the organisation’s network of relationships, which provide the organisation with otherwise inaccessible resources and a competitive advantage.</t>
@@ -6032,7 +6028,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>In this dissertation, I develop a conceptual model for how managers' roles as boundary spanners within their organizations affect the perceptions, attitudes, relationships, and performance of their subordinate employees. Drawing on literatures in social networks, status characteristics theory, social identity theory, and resource allocation theory, I suggest that managers' external relationships—the connections that managers make to organization members outside of their subordinate work group—have a material impact on their subordinates' perceptions of their work environment and their managers. These perceptions, I argue, serve as four specific mechanisms in an indirect effects model that connect managers' external relationship to their employees' task performance and work attitudes (eg organizational commitment) and the Leader Member Exchange (LMX) relationships between manager and subordinate. I apply the theoretical model to two salient types of managerial relationships: those with their bosses and those with their horizontal peers.</t>
@@ -6080,7 +6075,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>This study explores whether characteristics of the collaboration structure in software development teams affect development learning rates, with a secondary goal of testing product complexity as a moderator. We develop suitable hypotheses under the theoretical lens of cognitive load theory. The empirical study uses archival data on an ordinary least squares model to find significant associations between collaboration structure, product complexity and the learning rates exhibited by 230 development teams producing open source software. Results show two distinct subgroups of projects: The first subgroup exhibits an average 78% learning rate, and the other subgroup “unlearned”, i.e., productivity deteriorated over time instead of improved. In the learning subgroup, collaboration network density negatively impacted learning, while product complexity interacted with collaboration network centralisation and boundary spanning activity. In the unlearning subgroup, only network density impacted learning rates and no moderating effects were found. Practical implications and future opportunities for research are discussed.</t>
@@ -6128,7 +6122,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>The state of software development performance is far from being exemplar, with a success rate well below that of other industries, and understanding how to improve these projects is not only substantive but urgent. Software development is at most times a collaborative effort, yet we do not understand clearly how different collaboration structures associate with development performance metrics. This paper empirically examines the association between collaboration patterns, project productivity and product quality through a field study of working software open source new product development teams, using archival data from electronic sources related to Open Source Software projects. Collaboration structures are measured using Social Network Analysis and in terms of their network density, network centralization and the level of boundary spanning activity of team members. Productivity and quality are measured using "hard", code-based metrics. Results of regression analyses testing relevant hypotheses suggest that project managers need to strongly encourage internal collaboration, but be wary of allowing team members to participate in multiple projects. The breadth of skills within the team is a tactical asset that may increase the efficient frontier in the quality–productivity trade-off. Results also show that centralized structures associate with higher product quality and development productivity.</t>
@@ -6176,7 +6169,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Technology Transfer Centres (TTCs) have been analyzed in the last few years by focusing on the relationship between a TTC, provider of knowledge-intensive services, and a ﬁrm client-receiver. Less attention has been devoted to a more complex relationship which involves in the dyadic provider-receiver tie a third relevant body, University. We provide both a theoretical and an empirical contribution by studying whether TTCs can bond the academic and industrial system and we deﬁne the activities that make-up this role such as: scanning and selection of R&amp;D opportunities, bridge building, semantic translation of domain speciﬁc knowledge, co-production of new knowledge. The boundary spanning role of TTCs is discussed drawing on different and complementary theoretical perspectives. Moreover, we test research hypotheses on the antecedents of boundary spanning activity from a knowledge-based perspective. We argue that TTC boundary spanners need to leverage on both technical skills and networking competences. Empirical investigation has been carried out with a survey of the TTC population of North East Italy. The research ﬁndings highlight the task coordination activities implied by a boundary spanning role in joint R&amp;D projects and show that the endowment of human capital at individual level and a qualiﬁed social capital at individual and organizational level are the main determinants.</t>
@@ -6323,7 +6315,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>This cross-sectional study (conducted in April–May 2011) explored associations between partnership functioning synergy and sustainability of innovative programmes in community care. The study sample consisted of 106 professionals (of 244 individuals contacted) participating in 21 partnerships that implemented different innovative community care programmes in Rotterdam, The Netherlands. Partnership functioning was evaluated by assessing leadership, resources administration and efﬁciency. Synergy was considered the proximal outcome of partnership functioning, which, in turn, inﬂuenced the achievement of programme sustainability. On a 5-point scale of increasing sustainability, mean sustainability scores ranged from 1.9 to 4.9. The results of the regression analysis demonstrated that sustainability was positively inﬂuenced by leadership (standardised regression coefﬁcient b = 0.32; P &lt; 0.001) and non-ﬁnancial resources (b = 0.25; P = 0.008). No signiﬁcant relationship was found between administration or efﬁciency and programme sustainability. Partnership synergy acted as a mediator for partnership functioning and signiﬁcantly affected sustainability (b = 0.39; P &lt; 0.001). These ﬁndings suggest that the sustainability of innovative programmes in community care is achieved more readily when synergy is created between partners. Synergy was more likely to emerge with boundaryspanning leaders, who understood and appreciated partners’ different perspectives, and could bridge their diverse cultures and were comfortable sharing ideas, resources and power. In addition, the acknowledgement of and ability to use members’ resources were found to be valuable in engaging partners’ involvement and achieving synergy in community care partnerships.</t>
@@ -6705,7 +6696,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>The perspectives of transaction cost economics and the resource-based view of the firm have been used extensively to understand the implications of outsourcing. However, transaction cost economics does not explain how a firm will evolve as it progressively outsources internal functions, and the resource-based view does not operationalize the unspecified competences that will be required over time. On the other hand, the lens of paradox highlights the increased expediency and complexity that outsourcing firms are expected to encounter. In this paper, paradoxes comparing operational expediency gains to increases in management, learning and strategic complexity are discussed, leading to the proposal that often unintended replacement behaviors manifest as extensive boundary spanning and new firm-level competencies are necessary to manage these paradoxes and maintain competitive advantage. In extremum tests of these propositions are provided to demonstrate that the complexity of outsourcing intangibles is informed by a lens of paradox.</t>
@@ -6753,7 +6743,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>The aim of this research is to empirically investigate the relationships among the three vital knowledge management processes of acquisition, integration and application, and their effects on organisational innovation in the pharmaceutical manufacturing industry in Jordan; a knowledge-intensive business service (KIBS) sector. Structural equation modelling findings show an excellent fit among all these processes and innovation, with positive and significant relationships. Moreover, knowledge integration and knowledge application emerged as having strong and significant mediation effects upon the relationship between knowledge acquisition and innovation. As such, an organisation’s innovation efforts would significantly benefit from the synergistic effects of properly integrating and applying externally acquired knowledge. The findings make a valuable contribution to pharmaceutical knowledge management and innovation literature, especially in an era of open innovation. Pharmaceutical companies are advised to focus on developing proficient assimilation and application capabilities in order for acquired knowledge to have notable effects on their innovation performance.</t>
@@ -6801,7 +6790,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>The “variance hypothesis” predicts that external search breadth leads to innovation outcomes, but people have limited attention for search and cultivating breadth consumes attention. How does individuals' search breadth affect innovation outcomes? How does individuals' allocation of attention affect the efficacy of search breadth? We matched survey data with complete patent records, to examine the search behaviors of elite boundary spanners at                 IBM                 . Surprisingly, individuals who allocated attention to people inside the firm were more innovative. Individuals with high external search breadth were more innovative only when they allocated more attention to those sources. Our research identifies limits to the “variance hypothesis” and reveals two successful approaches to innovation search: “cosmopolitans” who cultivate and attend to external people and “locals” who draw upon internal people                              . © 2014 The Authors.               Strategic Management Journal               published by John Wiley &amp; Sons Ltd.</t>
@@ -6849,7 +6837,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>THErelationships between age, aspects of tenure, locus of control, job involvement, and boundary spanning behaviour (B.S.B.) were examined using path analysis for 281 scientists and engineers. It was found that locus of control and age were significant determinants of job involvement. It was also shown that locus of control and job involvement were significant determinants of B.S.B. These findings are discussed relative to previous research on locus of control, job involvement, and B.S.B. Finally, new research designs are advocated which incorporate task characteristics, role dynamics constructs, and environmental uncertainty as determinants of B.S.B.</t>
@@ -6991,7 +6978,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore how and why employees perceive technology-mediated interruptions differently and the role of sociocultural factors in this process using sociomaterial analysis. Design/methodology/approach – Data were gathered from 34 Sri Lankan knowledge workers using a series of workshop-based activities. The concept of sociomateriality is employed to understand how sociocultural elements are entangled with technology in work-life boundary experiences.</t>
@@ -7227,7 +7213,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Data from 409 members of 45 new product teams in five high-technology conpanies indicate the existence of four sets of boundary management activities which can be labeled Ambassador, Task Coordinator,Scout, and Guard. These activities are related to the frequency, type, and destination of communications between team members and others. This paper describes these activities and examines the irrpact of individual and environmental variables on the frequency in vAiich individual team members engage in them.</t>
@@ -7326,7 +7311,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>Leader-Member Exchange theory proposes both the salesperson and manager make contributions to their working relationship. Effective leadership is dependent upon developing a high quality relationship. This study tests the proposals of Leader-Member Exchange by examining the exchange of manager contributions (allowing the salesperson more operating freedom or latitude) and those of the salesperson. While the receipt of managerial latitude has a direct effect on the salesperson's evaluation of the working relationship, the salesperson's contributions also play a part. The manager allows more latitude to salespeople who are seen as more competent and loyal. These exchanges latitude for competency and loyalty) and the quality of the salesperson-manager relationship may be especially important when the sales task requires adaptive selling behaviors.</t>
@@ -7374,7 +7358,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>An information systems (IS) support community represents a knowledge-intensive network where IS professionals interact with end-users to resolve system use problems during the IS post-implementation stage. For IS professionals in the support function, providing support for multiple information systems to multiple business units requires knowledge about different domains (business units or technical systems). In this paper, we take a network perspective to empirically evaluate the effects of an IS worker's network position and knowledge boundary spanning on productivity. Drawing upon theories of experiential learning and knowledge boundary, we perform social network analysis and linear mixed effects modeling to analyze archival data comprising 36 IS workers and 23,450 support requests made by 4568 end-users during the first 13 months post SAP/R3 implementation in a large U.S. organization. Our findings reveal that IS workers' network centrality and boundary spanning positively influence productivity. Surprisingly, their boundary-spanning experience plays a substantially more important role than network centrality. This study makes important contributions to theory and practice in individual experiential learning in knowledge-intensive networks.</t>
@@ -7563,7 +7546,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>Using an external perspective as a research lens, this study examined team-context interaction in five consulting teams. The data revealed three strategies toward the teams' environment: informing, parading, and probing. Informing teams remain relatively isolated from their environment; parading teams have high levels of passive observation of the environment; and probing teams actively engage outsiders. Probing teams revise their knowledge of the environment through external contact, initiate programs with outsiders, and promote their team's achievements within their organization. In this study, they were rated as the highest performers among the teams, although member satisfaction and cohesiveness suffered in the short run. Results suggested that external activities are better predictors of team performance than internal group processes for teams facing external dependence.</t>
@@ -9696,7 +9678,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>The digital era is radically changing our societies and how ﬁrms do business. Innovating the business model has become a fundamental capability to survive competition, particularly for small and mediumsized enterprises (SMEs). This study investigates the digital-era role of boundary management capabilities in the processes of Business Model Innovation (BMI) in SMEs. Structural Equation Modelling is adopted to analyse data from a survey of 250 Italian experts who possess direct research and consulting experience with SMEs. Our ﬁndings reveal that digitalisation and ﬁrms’ boundaries aﬀect BMI in SMEs. Moreover, our results demonstrate how boundary management, speciﬁcally its technological and relational aspects, directly impacts BMI and mediates the relationship between boundary size and BMI. The study also oﬀers important theoretical and practical insights, calling on scholars and managers to give more attention to the boundary management of SMEs in order to support BMI.</t>
@@ -9838,7 +9819,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>In this study we examine the impact of market orientation of leaders on their leader-member exchange (IMX) with their followers. We review the evolution of leader-member exchange (LMX) theory over the exist five decades, and relate the strategic influence of increasing turbulence in the market environment on multiple generations of leadership styles during that period. Whereas vertical dyadic exchanges between hierarchical leaders and their followers may produce satisfactory performance of followers in equilibrium markets with predictable growth, these dyadic exchanges fail to do so in turbulent markets. Disequilibrium markets with disruptive turbulence demand introduction of discontinuous innovation from a new generation of market-oriented lateral leaders working closely with their boundary-spanning followers. We propose a number of hypotheses relating the market environment, leader-member exchange, and performance. Implications for managers and future researchers are discussed.</t>
@@ -9886,7 +9866,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>We examine the extent to which executives' boundary spanning relations inside and outside their industry affect organizational strategy and performance. We posit that the informational and social influences of external ties will be reflected in the degree to which the organization's strategy conforms to or deviates from the central tendencies of its industry and that the alignment of executives' external ties with the firm's strategy will be beneficial to firm performance. Using a multiyear sample of firms in the branded foods and computer industries, we find that executives' intraindustry ties are related to strategic conformity, that extraindustry ties are associated with the adoption of deviant strategies, and that alignment of executives' external ties with the informational requirements of the firm's strategy enhances organizational performance. Our results also show that a unique or differentiated strategy is not universally advantageous and that the benefits accruing from strategic conformity are especially strong in the more uncertain computer industry.</t>
@@ -9934,7 +9913,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>The relationship between external communication and R&amp;D team creativity has received increasing attention in the R&amp;D management literature. However, little is known about the motivational mechanism between the two. We propose a second‐stage moderation model based on social cognitive theory to explain whether, how and when R&amp;D team’s external developmental feedback motivates its creativity. Using the data gathered from 452 R&amp;D team members and 84 supervisors in a time‐lagged field study, we found external developmental feedback had a positive effect on R&amp;D team creativity via increasing team creative efficacy. Further, conditional indirect effect analyses found that a high level of cooperative goal interdependence strengthened the positive effect of team creative efficacy on R&amp;D team creativity and the mediating effect of team creative efficacy between external developmental feedback and R&amp;D team creativity.</t>
@@ -9982,7 +9960,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>This article explores the following hypothesis: There is a statistically significant relationship between a project manager’s leadership competencies and project success. Two proven questionnaires, the leadership dimensions questionnaire (LDQ) and the project success questionnaire (PSQ), were used to gather data from 52 project managers and project sponsors from a financial services company in the United Kingdom. The results from the LDQ and PSQ are presented in this article. A factor analysis of PSQ revealed three independent factors: usability, project delivery, and value of output to clients. The last factor is not related to project leadership or management, so the article concentrates on correlations between the other two factors and project leadership. Eight separate leadership dimensions were found to be statistically significantly related to performance, so the hypothesis was largely supported. Identifying such relationships provides managers with guidance on possible selection and project improvement models, whereby increased capability in leadership dimensions can lead to increased success in project management.</t>
@@ -10030,7 +10007,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Leader-member exchange (LMX) is a multidimensional construct seeking to identify the quality of the relationship between the leader and immediate subordinate. An instrument developed by Schrie-sheim, Neider, Scandura, and Tepper (1992) was utilized to determine the LMX score of 798 non-managerial employees in a casual restaurant chain. The dimensions of perceived contribution, affect, and loyalty were examined. Results demonstrate that LMX quality was high among the surveyed employees of a restaurant chain. The scores of LMX on age, gender and job tenure differed among employees while LMX scores on job status, education, and job type did not differ significantly.</t>
@@ -10078,7 +10054,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Even though, over the last two decades, the boundaryless career concept has stimulated a wide theoretical debate, scholars have recently claimed that research on the competencies that are necessary for managing a cross-boundary career is still incomplete. Similarly, the literature on emotional and social competencies has demonstrated how they predict work performance across industries and jobs but has neglected their inﬂuence in explaining the individual’s mobility across boundaries and their impact on career success. This study aims to ﬁll these gaps by examining the effects of emotional and social competencies on boundaryless career and on objective career success. By analyzing a sample of 142 managers over a period of 8 years, we found evidence that emotional competencies positively inﬂuence the propensity of an individual to undertake physical career mobility and that career advancements are related to the possession of social competencies and depend on the adoption of boundaryless career paths. This study also provides a contribution in terms of the evaluation of the emotional and social competencies demonstrated by an individual and of the operationalization of the measurement of boundaryless career paths, considering three facets of the physical mobility construct (organizational, industrial, and geographical boundaries).</t>
@@ -10173,7 +10148,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>To explain how multistakeholder groups organize democratic deliberations about complex sustainability issues, organizational scholars have focused on the key role of deliberative capacity, which encompasses the dimensions of inclusiveness, authenticity and consequentiality. However, the tensions inherent to the search of these three dimensions have been overlooked. In this paper, we argue that focusing on how spaces for deliberation are designed can help one understand how to manage such tensions. We identified the boundary work practices that shape the design of deliberative spaces and generate deliberative capacity properties in a high-level expert group (HLEG) launched by the European Commission about sustainable finance regulation. Our results show how these boundary work practices help balance deliberative tensions. We advance deliberation studies by conceptualizing deliberative boundary work, explaining how deliberative capacity is spatially generated and showing how deliberative tensions are balanced. We also contribute to boundary work theory by making explicit the deliberative nature of configuring boundary work and showing its relevancy to regulatory settings.</t>
@@ -10315,7 +10289,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to argue that the structure of the response to the World Trade Center (WTC) crisis can be characterized as an inter-organizational network and the majority of the activities can be identified as network management.</t>
@@ -10363,7 +10336,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>Drawing on corporate entrepreneurship (CE) and social network research, this study focuses on strategic renewal as a form of CE and examines the impact of boundary-spanning at top and middle management levels on business units’ exploratory innovation. Analyses of multi-source and multi-level data, collected from 72 top managers (TMs) and 397 middle managers (MMs) operating in 34 units of a multi-national organization, indicate that TMs’ boundary-spanning is positively related to units’ exploratory innovation, but also has a cascading effect on MMs by increasing their perceived role conflict. MMs’ role conflict is negatively related to units’ exploratory innovation and thus offsets some of the benefits gained through TMs’ boundary-spanning activities. Taking a configurational perspective on social exchanges at multiple levels, we show that role conflict is reduced by overlapping boundary-spanning ties among TMs and MMs. Surprisingly, MMs’ boundary-spanning does not relate to exploratory innovation. Our study shows that with regard to boundary-spanning, a top-down approach to CE as strategic renewal may be most effective because TMs play a key role in driving exploratory innovation. However, TMs need to be aware of the cascading social liabilities of their boundary-spanning behavior and ensure MMs develop similar networks. We advance ongoing debates in studies about CE and social networks by providing empirically validated insights into who drives strategic renewal and by uncovering the benefits and costs of social exchanges for strategic renewal. Furthermore, we uncover potential causes of mixed findings in network theory research and highlight a remedy to social liabilities.</t>
@@ -10458,7 +10430,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>This paper investigates boundary-work in management accounting in the context of globalization and hybrid professionalism. The paper demonstrates how permeable symbolic boundaries of the management accounting ﬁeld can be altered by employing expansion boundary-work. Contrasting boundary-work of IMA ofﬁcials and IMA members in Russia, we show that IMA ofﬁcials employ primarily monopolization boundary-work while IMA members employ primarily expansion boundary-work. Our ﬁndings illustrate how boundary-work is employed to exhibit organizational and occupational professionalism in the symbolic realm. The paper provides additional insight into the discursive domain of the accounting profession by linking boundary-work to globalization, two forms of professionalism, legitimacy, status and professional identity. This suggests that the professionalization process is inﬂuenced by the properties of professional boundaries.</t>
@@ -10506,7 +10477,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>This article explores the joint production and consumption of health information and advice in the context of NHS Direct, the new telephone health information and advice service. NHS Direct is an atypical call centre environment in so far as its core staff (nurses) are highly skilled professionals. These nurses are required to collaborate closely with, and are to some extent dependent upon, non-professional lower skilled staff (call handlers) to deﬁne and prioritize their work. This introduces a number of tensions between the two groups. Nurses respond to these tensions by engaging in ‘boundary work’, the micropolitical strategies through which work identities and occupational margins are negotiated, to protect their own status. Call handlers are more subject to the pressures of work ‘speed-up’, highly aware of the risks inherent in their role, but are unable to call upon professional status, either in their resistance to managerial imperatives or in their interactions with health consumers. They are required to manage the tension between offering a safe and high quality service, characterized in their training as ‘professional’, and nurses’ boundary work, which positions them as ‘non-professional’. Here we draw on qualitative research, including call interaction data between call handler and consumer, to show how call handlers’ occupation of the contested territory between professional and non-professional status leaves them wide open to the agency of consumers, as consumers attempt to shape the service in their own interests.</t>
@@ -10554,7 +10524,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>Past research has studied how the selection and use of control portfolios in software projects is based on environmental and task characteristics. However, little research has examined the consequences of control mode choices on project performance. This paper reports on a study that addresses this issue in the context of outsourced software projects. In addition, we propose that boundary-spanning activities between the vendor and the client enable knowledge sharing across organizational and knowledge domain boundaries. This is expected to lead to facilitation of control through specific incentives and performance norms that are suited to client needs as well as the vendor context. Therefore, we argue that boundary spanning between the vendor and client moderates the relationship between formal controls instituted by the vendor on the development team and project performance. We also hypothesize the effect of collaboration as a clan control on project performance. We examine project performance in terms of software quality and project efficiency. The research model is empirically tested in the Indian software industry setting on a sample of 96 projects. The results suggest that formal and informal control modes have a significant impact on software project outcomes, but need to be finely tuned and directed toward appropriate objectives. In addition, boundary-spanning activities significantly improve the effectiveness of formal controls. Finally, we find that collaborative culture has provided mixed benefits by enhancing quality but reducing efficiency.</t>
@@ -10602,7 +10571,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>Recently, discussion has begun to consider serving the base of the economic pyramid for business and societal benefit. Suggestions for so doing have focused on business model innovation, improving internal capabilities, promoting stronger governance, and providing leapfrog technologies (such as ICT) to promote effective change. We consider the questions of what types of innovation are occurring when businesses and other organizations enter the base of the pyramid and what types of social, economic, and consumer benefits they bring to local communities. We base our findings on an analysis of more than 1,000 cases describing base of the pyramid activities.</t>
@@ -10702,7 +10670,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
           <t>The majority of team leadership studies have ignored the specific context in which that leadership takes place and the cyclical correlation of inputs and processes on ongoing performance. It is our contention that leadership is a mediator of team processes and team effectiveness on ongoing functioning of multidisciplinary teams (MDT). The members of 126 multidisciplinary teams responded to a survey on several aspects related to the functioning and leadership of their teams. The results support the hypothesis that leadership does mediate the relationship between reflexivity and effectiveness (i.e. team management performance, boundary spanning and satisfaction) within the team. Theoretically, these findings challenge those of linear models that typically analyse the impact of leadership as something that happens in isolation. Future research should describe and consider not just the team type and tasks but also investigate the roles that context and time play in team leadership.</t>
@@ -10778,7 +10745,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t xml:space="preserve">. Verbatim Evidence: </t>
+          <t>Valid individual-level BSB. The study examines implanted boundary spanners (LSP representatives physically located at customer facilities). The construct 'knowledge exchange' between these implants and the host firm qualifies as valid boundary spanning behavior (Rule 8). The study uses 1:1 matched pairs (N=81 dyads), preserving statistical independence (Rule 4).. Verbatim Evidence: [INTRODUCTION] Our research explores the idea of attaining advantage and enhanced performance through a certain type of collaborative arrangement—closer, more integrated relationships with customers through the placement of boundary spanning employees at customer facilities. Such employees are often referred to as implants or on-sites. [Data collection] The final data for analysis included 81 dyads. [Measurement development] Knowledge exchange and innovation performance were assessed with measurement items from the perspectives of both the LSP representative and the customer representative.</t>
         </is>
       </c>
     </row>
@@ -10793,6 +10760,12 @@
           <t>BSMA0195</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
           <t>Using resource dependency and institutional theories, we create and test a model examining the relationships among senior management commitment, resource allocations, and the structure of public affairs departments. Using a large sample of U.S.-based firms, we find a positive relationship between senior management commitment to the public affairs function and the level of human and monetary resources allocated to the public affairs department. Furthermore, firms structure their public affairs responsibilities into three common activity sets: communications, collaborations, and local activities. These common activities are, in turn, positively associated with senior management commitment and resources allocated to the public affairs department.</t>
@@ -10816,6 +10789,11 @@
       <c r="K198" t="inlineStr">
         <is>
           <t>2004</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -10872,7 +10850,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>As employees’ personal lives are increasingly splintered by work demands, the boundary between work and nonwork domains is becoming ever more blurred. Grounded within a self-regulatory approach and the executive control function of inhibitory control, we operationalize and examine nonwork role re-engagement (NWRR)—the extent to which individuals can redirect attentional resources back to nonwork tasks following work-related intrusions. In phases 1 and 2, we develop and refine a psychometrically sound unidimensional measure for NWRR aligned with the self-regulatory processes of self-control and interference control underlying inhibitory control. In phase 3, we confirm the factor structure with a new sample. In phase 4 we validate the measure using the samples from phases 2 and 3 to provide evidence of criterion-related, convergent, and discriminant validity. NWRR was related to important well-being and work-related outcomes above and beyond existing self-regulatory and boundary management constructs. We offer theoretical and practical implications and an agenda to guide future research, as attentional agility becomes increasingly relevant in a home life replete with interruptions from work.</t>
@@ -10967,7 +10944,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>This article guides the development of creative insights in supply chain management. The authors begin by describing analogies’ role in advancing organization theory with a focus on image transfers between knowledge domains. While much has been said about the merits of conceptual transfers between domains, much equally remains unknown, particularly about how to deliberately develop creative insights that have the potential to challenge or enhance existing supply chain management theory. To address this issue, this research builds on prior work on analogies, creativity, and design thinking to develop a heuristic-analytic model. This model is designed to assist researchers in theorizing by analogy through a controlled dual cognitive process of divergence before convergence combined with a distant boundary-spanning knowledge search. An illustration of the model shows how creative output can provide a fresh perspective that helps render supply chains potentially more resilient.</t>
@@ -11015,7 +10991,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>The period after completing primary and adjuvant cancer treatment until recurrence or death is now recognized as a unique phase in the cancer control continuum. The term “survivorship” has been adopted to connote this phase. Survivorship is a time of transition: Issues related to diagnosis and treatment diminish in importance, and concerns related to long-term follow-up care, management of late effects, rehabilitation, and health promotion predominate. In this article, we explore the unique challenges of care and health service delivery in terms of the interface between primary care and specialist care during the survivorship period. The research literature points to problems of communication between primary and specialist providers, as well as lack of clarity about the respective roles of different members of the health-care team. Survivorship care plans are recommended as an important tool to facilitate communication and allocation of responsibility during the transition from active treatment to survivorship. Research questions that remain to be answered with respect to survivorship care plans and other aspects of survivorship care are discussed.</t>
@@ -11063,7 +11038,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>In multidisciplinary teams in the oil and gas industry, we examined expertise diversity's relationship with team learning and team performance under varying levels of collective team identification. In teams with low collective identification, expertise diversity was negatively related to team learning and performance; where team identification was high, those relationships were positive. Results also supported nonlinear relationships between expertise diversity and both team learning and performance. Finally, team learning partially mediated the linear and nonlinear relationships between diversity and performance. Findings broaden understanding of the process by which and the conditions under which expertise diversity may promote team performance.</t>
@@ -11158,7 +11132,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>Personnel is one of the most important resources for the performance of Information Systems (IS) and Information Center (IC) organizations. The scarcity of new employees, the difficulty of training and a high turnover make personnel management in these areas a difficult problem. For IS employees, the relationships between job satisfaction, organizational commitment and intention to leave the organization have been established. Because the size of the investment and the number of organizations establishing IC organizations are growing dramatically, it has become important to understand the determinants of turnover intentions for IC as well as IS employees. Are IC employees similar to their IS counterparts? Or, is their nature basically different, as some studies have suggested? This study examines the differences between IS and IC employees in terms of demographic characteristics, participation on boundary spanning activities, role stressors, overall job satisfaction, organizational commitment and turnover intentions. The differences are found to be significant and call for special attention from IC managers to manage more properly their personnel resources. IC employees were found to participate more extensively in boundary spanning activities, experienced more role stressors (role ambiguity and role conflict), were less satisfied with their jobs and less committed to their organization. The findings also demonstrate the importance of organizational commitment as an intervening variable in models of turnover. While overall job satisfaction had both direct and indirect effects on turnover intentions among IC employees, for IS personnel it had only indirect effects through organizational commitment. The effects of role stressors and boundary spanning activities were found to be indirect via overall job satisfaction and organizational commitment for both IC and IS employees. The implications of these findings for practicing managers and for future research are discussed.</t>
@@ -11206,7 +11179,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>As software development projects continue to be over budget and behind schedule, researchers continue to look for ways to improve the likelihood of project success. In this research we juxtapose two different views of what influences software development team performance during the requirements development phase. In an examination of 66 teams from 15 companies we found that team skill, managerial involvement, and little variance in team experience enable more effective team processes than do software development tools and methods. Further, we found that development teams exhibit both positive and negative boundary-spanning behaviors. Team members promote and champion their projects to the outside environment, which is considered valuable by project stakeholders. They also, however, guard themselves from their environments; keeping important information a secret from stakeholders negatively predicts performance.</t>
@@ -11353,7 +11325,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>Organizations have recognized that effective informal leadership is a source of competitive advantage and invest heavily in leadership development efforts. Moreover, because of historical shifts in the nature of work, this informal leadership often takes the form of inter-unit boundary spanning. Because of these two developments, discretionary boundary spanning (DBS) between units has increasingly become a critical, dynamic, bottom-up activity where individuals lacking formal authority step up and take on informal leadership responsibilities. In this study, we draw upon Simmelian Tie Theory (STT) to examine the relationship between different types of DBS and formal leaders’ perceptions of a subordinate’s informal leadership and performance. We empirically document that a small number of closed task-oriented and closed friendship-oriented DBSs are instrumental in helping individuals demonstrate informal leadership. However, we also show that DBS places constraints on informal leadership when closed ties become too numerous. This results in an inverted-U relationship between the number of closed DBS ties and perceptions of leadership where the apex (i.e., point of overembeddedness) emerges at a smaller number for friendship-oriented DBS relative to the apex for taskoriented DBSs. We discuss the theoretical implications of these results, as well as the practical implications for managers of organizations.</t>
@@ -11604,7 +11575,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Innovation is considered the engine for firm growth. Especially innovations, through recombining seemingly unrelated knowledge streams, can have groundbreaking impact and lead to sustained competitive advantage. To generate such innovation, firms often need to go beyond their existing technological or geographical boundaries to identify and integrate novel knowledge elements. This article refers to firms’ knowledge activities of drawing upon distant knowledge (i.e., knowledge from dissimilar technological domains or distant geographical regions) to create novel technological solutions, as innovation through boundary spanning. Aiming to investigate the roles of information technology (IT) in facilitating innovation through boundary spanning, we collected data from the pharmaceutical industry over a six-year period to test the research model. The data analysis results indicate that IT supports boundary-spanning activities in firm innovation and different IT-enabled knowledge capabilities affect boundary-spanning innovation differently.</t>
@@ -11704,7 +11674,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>This paper combines the concept of weak ties from social network research and the notion of complex knowledge to explain the role of weak ties in sharing knowledge across organization subunits in a multiunit organization. I use a network study of 120 new-product development projects undertaken by 41 divisions in a large electronics company to examine the task of developing new products in the least amount of time. Findings show that weak interunit ties help a project team search for useful knowledge in other subunits but impede the transfer of complex knowledge, which tends to require a strong tie between the two parties to a transfer. Having weak interunit ties speeds up projects when knowledge is not complex but slows them down when the knowledge to be transferred is highly complex. I discuss the implications of these findings for research on social networks and product innovation.</t>
@@ -12330,7 +12299,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>Scholarship in the field of health communication is broad, with interdisciplinary contributions from researchers trained in a variety of fields including communication, nursing, medicine, pharmacy, public health, and social work. In this paper, we explore the role of “health communication boundary spanners” (HCBS), individuals whose scholarly work and academic appointment reflect dual citizenship in both the communication discipline and the health professions or public health. Using a process of critical reflective inquiry, we elucidate opportunities and challenges associated with HCBS across the spectrum of health communication in order to provide guidance for individuals pursuing boundary spanning roles and those who supervise and mentor them. This dual citizen role suggests that HCBS have unique skills, identities, perspectives, and practices that contribute new ways of being and knowing that transcend traditional disciplinary boundaries. The health communication field is evolving in response to the need to address significant healthcare and policy problems. No one discipline has the ability to single-handedly fix our current healthcare systems. Narrative data from this study illustrate the importance of seeing HCBS work beyond simply being informed by disciplinary knowledge. Rather, we suggest that adapting ways of knowing and definitions of expertise is an integral part of the solution to solving persistent health problems.</t>
@@ -12482,7 +12450,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>Following the resource-advantage theory, this study advances the existing research of boundaryspanning search by examining which configuration of a new venture’s boundary-spanning search can obtain successful venture performance and how a founding team’s external relationship and the internal firm competences shape the relationship between the distant search and new venture performance. This paper is based on a questionnaire survey/analysis of a sample of 178 new ventures from China, and it offers insight to entrepreneurs with regard to the importance of building external managerial ties and developing idiosyncratic internal competences on boundary-spanning search. In addition, this study also reveals that the effectiveness of the supply-side, demand-side and spatialside boundary-spanning search on venture performance depends on investing resource at a rational level.</t>
@@ -12530,7 +12497,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>Information system development can be considered a collaboration between users and developers. The inability to leverage the localized knowledge embedded in these two stakeholders hinders software development work to achieve high performance. Exploring the ways to counter this difﬁculty is then critical. This study applies an intellectual capital perspective to address the issues around spanning the knowledge boundary between developers and users. Our ﬁndings highlighted how important effective knowledge boundary spanning is to both product and project quality. Furthermore, three dimensions of intellectual capital increased the degree to which knowledge boundary spanning was effective.</t>
@@ -12625,7 +12591,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate three issues: how does an innovative search (local search and boundary-spanning search) impact ﬁrm innovation performance of latecomers; how does capability reconﬁguration (capability evolution and capability substitution) mediates the relationship between innovative search and ﬁrm innovation performance; and how does the technological leapfrogging process (initial stage, following stage, synchronization stage and leading stage) moderate the relationship between capability reconﬁguration and ﬁrm innovation performance.</t>
@@ -12673,7 +12638,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>This study examines personal ties between boundary-spanning personnel in interorganizational exchanges in emerging markets. Drawing on social embeddedness theory and boundary spanning theory, we propose that strong ties between boundary spanners may benefit exchange parties in their interorganizational relationships through two heightened boundary-spanning behaviors—information processing and external representation. The results from 225 manufacturer–distributor dyads in China indicate that interpersonal ties at the higher levels (between top executives) and at the lower levels (between salespersons and individual buyers) are both positively associated with relationship quality of the buyer–supplier relationship through dyadic boundary-spanning behaviors. Between two levels of interpersonal ties, ties at the lower levels exhibit a stronger association with relationship quality than do ties at the higher levels. Furthermore, the positive effects of interpersonal ties on conflict resolution and cooperation are amplified when both levels of ties are strong in the focal relationship.</t>
@@ -12721,7 +12685,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Boundary‐spanning personnel such as tax preparers, travel agents and hairdressers interface directly with customers. In their unique position, between the organization and customer, these service providers market the service to consumers while they simultaneously carry out operational functions. Both the customer and the provider bring certain expectations to the service encounter. These expectations then shape the perceptions of the service encounter. The research reported uses script methodology to compare the expectations between boundary‐spanning service providers and consumers of the same service. Draws its theoretical foundation from the expectations and scripts literatures. In Phase One, scripts of the service were elicited in order to test hypotheses based on the discovery and comparison of consumers′ and service providers′ subgoals for a typical service encounter (               H1               ). A hypothesis also tested the point at which providers and consumers enter their respective scripts of a typical service encounter (               H2               ). In Phase Two, the subgoals mentioned most frequently in Phase One were used as stimuli to elicit the specific actions which comprise the complete script. These complete scripts enabled a comparison of the elaborateness of provider and consumer scripts (               H3               ). The results of Phase One revealed that a portion of consumers′ subgoals for a service encounter are shared by providers of the service while other subgoals are unique, supporting               H1               . The point of activation of the script differed dramatically between customers and providers, supporting               H2               . The Phase Two findings provide support for the hypothesis that service providers have more elaborate scripts. Overall, the results support the notion that scripts operationalize expectations. Closes with implications for management and suggestions for future research.</t>
@@ -12769,7 +12732,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to explore how integration teams can build trusting relationships in component teams to enhance their leadership capability within multiteam systems to achieve common superordinate goals. The study investigates how an integration team diagnoses contextual dynamics to enhance understanding of goals in component teams and spans boundaries to create trusting relationships.</t>
@@ -12869,7 +12831,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>While there is a growing interest in the role of market information processing activities (i.e., the acquisition, dissemination, and use of market information) in new product development (NPD), a number of gaps remain in our knowledge on this topic. When investigating the performance impact of market information processing, most studies have treated the three activities as independent. Our research adds to the extant knowledge by exploring not only both direct relationships between each of the market information processing activities and new product performance, but also interaction effects. We, thus, ask the question of whether there may be synergies in obtaining performance increases by jointly improving two processing activities, rather than just considering each activity independently. In addition, we investigate these effects for different levels of information quality; a topic largely neglected in the market information processing literature. Our analysis is based on empirical data from 152 Dutch NPD projects. The results indicate that market information acquisition and use are both directly associated with increased performance. We also ﬁnd signiﬁcant interaction effects for information acquisition and dissemination, and for information dissemination and use. Finally, the importance of information quality is emphasized, with lower quality information producing lower performance and wiping out the effects between various aspects of market information processing and new product performance. We provide several implications of our ﬁndings for managers and academics.</t>
@@ -12917,7 +12878,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>Background: Rehabilitation services depend on competent professionals who collaborate effectively. Wellfunctioning interprofessional teams are expected to positively impact continuity of care. Key factors in continuity of care are communication and collaboration among health care professionals in a team and their patients. This study assessed the associations between team functioning and patient-reported benefits and continuity of care in somatic rehabilitation centres. Methods: This prospective cohort study uses survey data from 984 patients and from health care professionals in 15 teams in seven somatic rehabilitation centres in Western Norway. Linear mixed effect models were used to investigate associations between the interprofessional team communication and relationship scores (measured by the Relational Coordination [RC] Survey and patient-reported benefit and personal-, team- and cross-boundary continuity of care. Patient-reported continuity of care was measured using the Norwegian version of the Nijmegen Continuity Questionnaire. Results: The mean communication score for healthcare teams was 3.9 (standard deviation [SD] = 0.63, 95% confidence interval [CI] = 3.78, 4.00), and the mean relationship score was 4.1 (SD = 0.56, 95% CI = 3.97, 4.18). Communication scores in rehabilitation teams varied from 3.4–4.3 and relationship scores from 3.6–4.5. Patients treated by teams with higher relationship scores experienced better continuity between health care professionals in the team at the rehabilitation centre (b = 0.36, 95% CI = 0.05, 0.68; p = 0.024). There was a positive association between RC communication in the team the patient was treated by and patient-reported activities of daily living benefit score; all other associations between RC scores and rehabilitation benefit scores were not significant. Conclusion: Team function is associated with better patient-reported continuity of care and higher ADL-benefit scores among patients after rehabilitation. These findings indicate that interprofessional teams’ RC scores may predict rehabilitation outcomes, but further studies are needed before RC scores can be used as a quality indicator in somatic rehabilitation.</t>
@@ -13069,7 +13029,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>This three-essay project explores boundary management and work-nonwork enrichment to explain how thriving in the work domain relates to thriving in the nonwork domain. The Cross-Domain Thriving model proposed in Study 1 theorizes that when employees experience growth and energy at work, they create and deplete resources within and across roles and individual boundary management strategies, role congruency, and ease of transition moderate the degree to which thriving translates into enrichment and/or conflict across roles. Study 2 tested aspects of the cross-domain thriving model and found that neither work nor nonwork thriving was related to increased time-based conflict, but both forms of thriving predicted enrichment gains across domains. Moreover, higher levels of work-nonwork role segmentation were associated with a stronger relationship between learning in nonwork roles and affective and efficiency enrichment gains in the nonwork-to-work direction. In the work-to-nonwork direction, role congruency and cycling boundary management behavior were related to greater developmental and affective enrichment, respectively. Cycling also strengthened the positive relationship between vitality at work and work-to-nonwork capital enrichment. Study 3, a qualitative study investigating work and nonwork thriving in employees working from home during a pandemic, suggested the importance of boundary management skills as demands on learning and energy increase. Findings highlight how key employer actions and employee regulatory behavior can leverage the benefits of growth and energy in work and nonwork domains.</t>
@@ -13117,7 +13076,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>Community-based initiatives (CBIs) are thriving in Western countries. In CBIs, citizens take a leading role in providing public services and goods. CBIs have been acclaimed for their innovativeness, problem-solving capacity, and legitimacy. However, we lack large N studies on performance of CBIs and its antecedents. This article develops and tests a model that identiﬁes relationships between performance and four antecedents by using survey data on CBIs collected in the Netherlands (N = 671). Using structural equation modelling, positive direct and indirect relationships between transformational leadership, boundary spanning leadership, organizational capacity, social capital ties, government support, and performance are found.</t>
@@ -13259,7 +13217,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>This study examined the relative influence of transformational and gatekeeping leadership on team performance in a study of researchers working in industrial R&amp;D teams in Japan. Potential effects of both internal and external communication and group norms for consensus were studied as possible mediating influences on the leadership-performance relationship. Results found that, while both forms of leadership enhanced communication processes within and between groups, only gatekeeping leadership served to reduce group norms for consensus. As a result, team cultures became somewhat more accepting of expressions of divergent opinions and new ideas from various team members, an important factor in R&amp;D innovation and performance. By contrast, transformational leadership served to create team cultures in which divergence from group norms by various members was discouraged, leading to fewer innovative ideas and no performance increment. Results are discussed both in the context of the unique Japanese work environment and in the larger context of leadership processes across regions and cultures.</t>
@@ -13307,7 +13264,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>Due to the increasing array of sales technology, salespeople must understand how each application assists them. This study examines how business-to-business salespeople use different forms of sales technology to meet their boundary-spanning roles. Our research draws from social exchange theory and task-technology fit theory to test a model that examines how salespeople use CRM and social media technologies differentially to support competitive information collection, product information communication, and buyer information sharing. Dyadic data from industrial buyers and sellers is used to analyze the technology-behavior relationships. Our study's results reveal social media use and CRM technology both positively influence buyer-seller information exchanges; however, each technology takes a distinct route to enable the information exchange between the buyer and the seller. The results also suggest that managers need to champion the use of both technology applications to their salesforce.</t>
@@ -13355,7 +13311,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>In this article the authors discuss research they conducted that examined the relationship between task difficulty and the extent of boundary-spanning activity within an organization. The authors believed that they greater degree of interunit interdependence that existed in an organization would result in a greater amount of boundary-spanning activity by that organization's members. They also believed that the greater degree of task difficulty in a given situation would also result in a greater amount of boundary-spanning activity by members. The authors hoped to examine the relationships that exist between organizational structure and the amount of intergroup activity fostered by those structures.</t>
@@ -13403,7 +13358,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>Innovation has an intrinsic relationship with social networks because it provides a mechanism for knowledge and information to travel freely between individuals. Consequently, there is abundant research linking social networks to innovation. However, two critical gaps still exist. First, most research studies use a structural approach, and less attention is paid to the behavioral dimensions in a network. Secondly, the majority of empirical research focuses on egocentric networks or dyadic relationships between two organizations, instead of the network of organizations as a whole.</t>
@@ -13451,7 +13405,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>Marketing boundary spanners—especially customer service representatives—are notably susceptible to burnout. The authors define the burnout construct and develop hypotheses to examine if burnout acts as a partial mediator between role stressors and key behavioral and psychological job outcomes. Responses from 377 customer service representatives reveal that burnout levels are high relative to other burnout-prone occupations (e.g., police, nursing) and that burnout has consistent, significant, and dysfunctional effects on their behavioral and psychological outcomes. Moreover, burnout mediates the negative effects of role stressors on job outcomes, whereas the positive effects of role stressors are unmediated.</t>
@@ -13551,7 +13504,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>Because of their boundary-spanning nature, manufacturers’ representatives frequently are involved in team selling. The results from a survey of 362 manufacturers’ representatives indicates that team selling is more likely to be used by manufacturers’ representatives when the customer faces a first-time buy of a complex product, when the information needs of the customer are great, when the account requires special treatment, and when a number of people are involved in the decision to buy. In addition, team selling is more likely when the potential sale is large for the representative firm and when the product is new to the representative’s product line.</t>
@@ -13599,7 +13551,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>With congeneric mergers, which involve firms with interrelated but not identical business lines that develop diverse products and services, a major challenge for organizations is the development of a common platform that fulfills similar business functions across multiple divisions. Through a field study of a postmerger common platform development initiative, we develop a framework that highlights how environmental and organizational contexts shape the process of common platform development (CPD). Our study provides an account of how the focal organization transitioned to a platform-based approach by achieving a balance between stable and flexible aspects of the common platform through negotiations among the divisions acquired through mergers and acquisitions. These negotiations were enabled through various boundary-spanning activities and the guided successive enrichment of boundary objects used in CPD process. European Journal of Information Systems (2015) 24(2), 159–177.</t>
@@ -13694,7 +13645,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>Purpose – To obtain optimal deliverables, more and more crowdsourcing platforms allow contest teams to submit tentative solutions and update scores/rankings on public leaderboards. Such feedback-seeking behavior for progress benchmarking pertains to the team representation activity of boundary spanning. The literature on virtual team performance primarily focuses on team characteristics, among which network closure is generally considered a positive factor. This study further examines how boundary spanning helps mitigate the negative impact of network closure.</t>
@@ -13742,7 +13692,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>This study investigated the effects of small business owner decision styles on the search for external assistance information, community information, and competitor information. Results confirmed the existence of decision style differences in selection of boundary spanning activities. A conclusion is drawn that small business owners use preferred sources for gathering information related to business operations, but need to utilize additional sources to ensure a comprehensive boundary spanning role. Ways to enhance boundary spanning activities are provided</t>
@@ -13790,7 +13739,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>The influence of boundary spanning roles on strategic decision-making was explored in a field study in fifteen organizations. Results support the importance of boundary spanning roles in the strategic decision-making process and the relationship of technology to the differential strategic decision-making influence of different boundary spanning roles.</t>
@@ -13979,7 +13927,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>This paper collects 103 sample firms' 2015 to 2019 data through data envelopment analysis to measure their technical innovation performance and social network analysis to build joint-patent networks and explore knowledge-creating alliance relationships. The article highlights how tacit knowledge recombination works as a mechanism of boundary spanning. It emphasizes the significance of strategic balancing networks' position to improve technical innovation performance and competitiveness of patent-intensive (PI) firms. This research contributes to shedding additional light on the nature of the boundary-spanning mechanism and PI firms' knowledge exchanges. Specifically, it examines how balancing boundaries spanning through joint-patent networks can influence the processes of tacit knowledge transmission and recombination between knowledge-based actors.</t>
@@ -14027,7 +13974,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>Setting the research background in China, this study draws on absorptive capacity, knowledge inertia and prospect theory to show the relationship between R&amp;D capability and innovation performance which comprises exploitation and exploration. We propose that stronger R&amp;D capability promotes exploitation performance but inhibits exploration performance. As exploitation represents immediate interest and exploration represents long-term interest, we introduce the notion of knowledge boundary spanning of R&amp;D network to balance short-term and long-term benefits. The empirical results show that R&amp;D capability and knowledge boundary spanning of R&amp;D network complement each other for explorative innovation while they present trade-offs for exploitative innovation. This study contributes to existing literature on R&amp;D capability–innovation performance, and it further extends our understanding by investigating the impact of knowledge boundary spanning of R&amp;D network on the R&amp;D capacity–innovation performance relationships. In addition, this study provides references on resources configuration to achieve different innovation strategies.</t>
@@ -14075,7 +14021,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>Open innovation is crucial for achieving high-quality and sustainable business growth. However, it remains unclear how prospective boundary-spanning search and responsive boundary-spanning search impact organizational resilience and open innovation in the VUCA (Volatility, Uncertainty, Complexity, and Ambiguity) new normal. Based on the resource-based theory and dynamic capabilities theory, this paper classifies boundaryspanning search into prospective boundary-spanning search and responsive boundary-spanning search to investigates the impact on open innovation and organizational resilience, and analyze the moderating role of big data analytics capability. The empirical study of 293 Chinese smart manufacturing firms indicates that both prospective and responsive boundary-spanning search have an inverted U-shaped impact on open innovation and organizational resilience. Organizational resilience partially mediates the relationships between prospective boundary-spanning search, responsive boundary-spanning search, and open innovation. Moreover, big data analytics capability moderates and flattens the inverted U-shaped relationships between prospective and responsive boundary-spanning search, and organizational resilience. This study explores the intrinsic mechanism of prospective and responsive boundary-spanning search on open innovation through organizational resilience. The findings enrich and expand the research on the antecedents of open innovation.</t>
@@ -14222,7 +14167,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
           <t>The relationship between boundary-spanning role activities and conflict management styles was examined with data gathered from 189 project managers who belong to a national professional association. Five conflict management styles and six boundary role activities were measured with a survey instrument constructed from previously developed scales. The conflict management styles measured were integrating, avoiding, dominating, obliging, and compromising. The six boundary role activities measured were gathering, filtering, and transmitting information; transacting; proacting; and protecting. Hypotheses proposing specific relationships between each of the five conflict management styles and the six boundary role activities were tested with the data. Results indicated that unique combinations of boundary role activities are associated with each of the conflict management styles. Further, more cooperative conflict management styles are related to a greater number of boundary role activities that emphasize information sharing and managing relationships. Results also indicated that length of a project manager's experience moderates this relationship in that those with greater experience use more cooperative styles. A revision is suggested to the conflict management style construct.</t>
@@ -14270,7 +14214,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>Owing to their growing numbers and importance, both managers and researchers are increasingly concerned with the work experiences of boundary-spanning employees. Employee perceptions of organizational support *POS) may be particularly relevant to this crucial employee group. Thus reports a study of the relations between two individual-level and two organizationallevel antecedents to boundary-spanner POS. The results indicate that employee gender, amount of formal organizational recognition received, and the quality of task-related training are associated with POS. However, type of employee pay plan is not. Concludes with a discussion of these findings and their implications for effectively managing boundary-spanning employee POS.</t>
@@ -14318,7 +14261,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate a boundary spanning, interprofessional collaboration between advanced practice nurses (APNs) and junior doctors to support junior doctors’ learning and improve patient management during the overtime shift.</t>
@@ -14366,7 +14308,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>National Sun Yat-sen University, Kaohsiung, Taiwan This research report compares three differing explanations of the dynamic interrelationships between internal and external innovation-related communication in a new organizational form. In the functional specialization explanation, individuals are said to focus on the mix of internal and/or external communication dictated by their formal positions. The communication stars explanation suggests that individuals maintain similar levels of communication in both networks. The cyclical model posits a more dynamic pattern that shifts back and forth between internal and external communication, depending on the consequences of their prior communication behavior. The new organizational form examined for three years was the Cancer Information Service, a geographically dispersed federal government health information program. Our results indicated that there was a lagged effect for the communication stars explanation.</t>
@@ -14461,7 +14402,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>This paper describes one of the first empirical explorations into organisational knowledge creation theory as first elucidated by Nonaka and Takeuchi [1]. We extend the theory and examine it in the inter-organisational context of University-Industry (U-I) collaborative R&amp;D Projects. More specifically, the relationship between enabling conditions and knowledge conversion processes as well as the effects of these processes on the achievement of technological objectives are studied using a sample of 25 U-I collaborative R&amp;D projects into advanced technology. Quantitative and qualitative evidence supports the theory that some enabling conditions are significant for knowledge conversion processes. Furthermore, the presence of the aggregate knowledge processes is positively associated with the achievement of successful technological objectives. The theoretical and practical implications of these findings are discussed.</t>
@@ -14509,7 +14449,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>BACKGROUND: There is a need for a better understanding of how the use of technology to complete work outside regular ofﬁce hours is related to work-life outcomes. Few studies have also investigated how individual differences in work-nonwork boundary management relate to work-life outcomes. OBJECTIVE: This study was conducted to examine how teleworking outside regular ofﬁce hours and individual boundary management relate to work-family conﬂict. METHODS: A web survey was sent to fulltime employees at the headquarters of a multinational high-tech ﬁrm in Sweden. A total of 71 answers were obtained and analyzed using regression analysis. RESULTS: The extent of teleworking after hours was unrelated to work-family conﬂict. However, as previous research has shown, having more permeable boundaries and allowing work to interrupt nonwork behavior was related to higher levels of conﬂict. CONCLUSIONS: The ﬁndings suggest that teleworking after hours is not as problematic in terms of work-family conﬂict as has been reported in previous studies. Furthermore, in order to prevent high levels of work-family conﬂict, it is seemingly beneﬁcial to avoid work interruptions during nonwork behavior.</t>
@@ -14557,7 +14496,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>While the introduction of a new product or service carries considerable risk, incorporating customer input into the new product/service development (NPD) process increases the probability of commercial success. In their boundary spanning role, industrial (B-to-B) salespeople are well suited to serve as a conduit between customers and those inside their company who are largely responsible for the NPD process. The current study investigates the perceptions of sales managers and examines the role the sales force may play in the early stages of the NPD process. An empirical analysis is conducted to determine whether differences exist between organizations that employ key account management (KAM) systems and those that do not employ KAM systems. The findings of this study suggest that salespeople from KAM organizations are better suited to provide input into the NPD process than their non-KAM counterparts.</t>
@@ -14652,7 +14590,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to evaluate the recognition of sexual harassment (SH); to describe the relationships among SH, employees’ burnout, customer-oriented boundary-spanning behaviors (COBSB); and to verify the moderating effect of employees’ psychological safety (PS), all within deluxe hotels in South Korea.</t>
@@ -14747,7 +14684,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>Information and communication technologies enable employees to be available anywhere and anytime, raising availability expectations
@@ -14808,7 +14744,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Problems cross boundaries and so must solutions. The most important challenge for performance networks that aim to deliver better results is designing the structure that coordinates across traditional agency boundaries. Not only must this structure be clearly defined, but it also must account for the integration of a broad range of cross-government activities. Like the overarching performance network, the cross-boundary structure has the characteristics of a dynamic system, including flexibility, adaptability, growth, and the continual emergence of new forms and functions. Summer 2000 featured perfect conditions for gridlock in the sky. Flying had become an increasingly popular way to travel, and the airlines had marketed aggressively to vacationing families and business travelers. Airports were already crowded when unusual and frequent patterns of bad weather hit aviation especially hard. Delays and canceled flights became almost daily events. The public complained loudly, congressional hearings were scheduled, and the Federal Aviation Administration was about to experience unfriendly fire from an aroused media.</t>
@@ -15220,7 +15155,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>This study investigates the role of gatekeepers in the transfer of information within a single R &amp; D location by comparing directly t h e performance of project groups with and without gatekeepers. The results show that gatekeepers performed a linking role only for projects performing tasks that were 'locally-oriented' while 'universallyoriented' tasks were most effectively linked to external areas by direct project member communication. Gatekeepers also appear to facilitate external communication by their locallyoriented project colleagues. A follow-up study five years later showed that almost all gatekeeping project leaders had been promoted up the managerial ladder; in contrast, one half of the non-gatekeeping project leaders had ascended the technical ladder. This implies that higher managerial levels demand strong interpersonal a s well a s technical skills.</t>
@@ -15532,7 +15466,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>In our study of an interactive marketing organization, we examine how members of different communities perform boundary-spanning coordination work in conditions of high speed, uncertainty, and rapid change. We find that members engage in a number of cross-boundary coordination practices that make their work visible and legible to each other, and that enable ongoing revision and alignment. Drawing on the notion of a “trading zone,” we suggest that by engaging in these practices, members enact a coordination structure that affords cross-boundary coordination while facilitating adaptability, speed, and learning. We also find that these coordination practices do not eliminate jurisdictional conflicts, and often generate problematic consequences such as the privileging of speed over quality, suppression of difference, loss of comprehension, misinterpretation and ambiguity, rework, and temporal pressure. After discussing our empirical findings, we explore their implications for organizations attempting to operate in the uncertain and rapidly changing contexts of postbureaucratic work.</t>
@@ -15736,7 +15669,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
           <t>Given the growing importance of B2B digital platform capabilities for competitive advantage, research on its antecedents and outcomes in the business-to-business context remains scarce. To address this gap, we built on dynamic capability theory to examine how B2B organizations’ digital platform capabilities contribute to sustainable positioning. Specifically, we examined the direct and indirect associations (via organizational knowledge depth, breadth, and agility) between digital platform capabilities and sustainable positioning. Additionally, we explored the moderating role of leader boundary-spanning behaviors in the relationship between digital platform capabilities and organizational knowledge depth and breadth. Our study based on two-source survey data from top management in Chinese manufacturing firms. The findings fully support all our proposed hypotheses. Digital platform capabilities significantly enhance sustainable positioning, both directly and through improved organizational knowledge depth, breadth, and agility. Furthermore, leader boundary-spanning behaviors strengthen the impact of digital platform capabilities on both knowledge depth and breadth. These insights offer practical implications for B2B firms seeking to leverage digital platform capabilities to enhance knowledge depth, breadth, agility, and sustainable market positioning.</t>
@@ -15784,7 +15716,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>Organizational behavior (OB) is an area of knowledge rather than a unified theory. It consists of a growing clutch of concepts, approaches, models, and tools pertinent to the structure and functioning of organizations within their socioeconomic contexts and of the study of individuals and groups within their organizational contexts [1]. Thus, OB spans para-organizational concerns such as interorganizational networks and delivery systems. It deals with macro-organizational phenomena-organizational goals, strategies, climates, cultures, structure, management styles, and performances-and how they are shaped by one another and by such contextual factors as operating environments, societal values and institutions, technology, size, dependence, and other</t>
@@ -15936,7 +15867,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
           <t>Leaders' positions as external brokers in organizational networks—those acting as a bridge between individuals outside the boundaries of their team—can enhance or constrain their effectiveness. Yet, whereas extant research on network brokerage views it as a private good whose benefits accrue directly to the broker, recent research suggests brokering between external communities can serve as both a public good as well as a public liability that can spillover to team members. We integrate network leadership theory with the externalities of network brokerage perspective to examine the countervailing effects of leaders' external brokerage in an information network with peer leaders and executives on team performance. In a sample of 465 team members in 80 teams distributed across 10 sister companies within one conglomerate, we used multilevel structural equation modeling to test our hypotheses. On one hand, we found that leader external brokerage was positively associated with team performance through team members' perceptions of organizational support; on the other hand, we found that leader brokerage is detrimental to team performance by compromising leaders' commitment to their teams. Our results suggest that, while leaders are encouraged to forge connections outside their team to harvest social capital benefits, there are both public benefits and liabilities of team leaders' external networks that can impact team performance.</t>
@@ -16196,7 +16126,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F310" t="inlineStr"/>
       <c r="G310" t="inlineStr">
         <is>
           <t>The article examines the process of innovation and knowledge sharing from a perspective that focuses on the inﬂuence that local circumstances can have. In particular, it looks at the problems of knowledge sharing between groups of professionals. It presents a comparative analysis of two studies, one involving two groups of IT professionals; the other a network of healthcare professionals. The data was collected in two sets. The ﬁrst set consisted of the results from two earlier, independent studies; the second was collected speciﬁcally for this article. We investigate the role played by boundary objects and brokers. Through an analysis of the interplay between boundary object and broker, we uncover the dynamics of the innovation process and show that the role played by the broker can be political. We identify two strategies that are used by brokers in the selection of a boundary object. The ﬁrst is directed towards achieving a balance between the actors involved and the second is directed towards controlling their activities. We conclude by suggesting that other researchers should also consider the interplay between broker and boundary object when examining cross-boundary knowledge sharing.</t>
@@ -16296,7 +16225,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr">
         <is>
           <t>The aim of the present study conducted among 1,106 Finnish employees was to identify boundary management profiles based on cross-role interruption behaviors from work to nonwork and from nonwork to work. Adopting a person-oriented approach through latent profile analysis, five profiles were identified: Work Guardians (21% of the employees), Nonwork Guardians (14%), Integrators (25%), Separators (18%) and an Intermediate Group (22%). We then examined differences between these profiles with respect to recovery experiences (psychological detachment from work, relaxation, mastery experiences, and control during off-job time) and recovery outcomes (vigor and exhaustion). Work Guardians had the poorest situation in terms of recovery experiences and outcomes. Integrators came close to Work Guardians in their responses, but they showed better relaxation and control during off-job time. Nonwork Guardians and Separators had the most beneficial recovery experiences. The Intermediate Group scored near the average in all evaluations. Altogether the findings suggest that boundary management profiles play a significant role, especially regarding recovery experiences.</t>
@@ -16344,7 +16272,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr"/>
       <c r="G313" t="inlineStr">
         <is>
           <t>The school safety and security planning process is important because it directs the educational organization's ability to maintain a stable safe learning environment. For this study, continuous comparison of data and theory, and a cross-case analysis generated a grounded theory. This theory stated that: When the educational leader's perception of risk was malleable and well developed, the school safety and security planning process was more comprehensive. Enhancement occurred with the establishment of a systemic approach, and through inter-organizational collaboration with community stakeholders. These stakeholders included, but were not limited to, the departments of public health, mental health, medical care, emergency management, law enforcement, fire, homeland security, and transportation</t>
@@ -16548,7 +16475,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr"/>
       <c r="G317" t="inlineStr">
         <is>
           <t>Entrepreneurial teams often struggle with simultaneous task and team challenges at an early stage of new venture creation. The way in which teams shape their teamwork is key in leveraging performance in the pre‐founding phase. Learning should help the team in establishing good teamwork and in expanding its members’ entrepreneurial capabilities. Leadership is needed to facilitate and guide this learning. Accordingly, we investigated learning and leadership as facilitators of performance in the pre‐founding phase. Specifically, we examined team reflexivity as a collective internal learning process and boundary spanning behaviour as an externally directed individual activity, operating at different levels in fostering team and individual performance. Charismatic team leadership was examined as a catalyst of learning, shaping team and individual performance ultimately. The multilevel mediation model was tested based on data from 196 members of 58 teams of a venture creation programme. Team reflexivity predicted team and individual performance. Boundary spanning behaviour was not related to performance. As hypothesised, charismatic team leadership predicted team and individual performance, both mediated by team reflexivity. This research highlights the relevance of team learning in pre‐founding teams and emphasises leadership in shaping learning and moving new ventures forward.</t>
@@ -16648,7 +16574,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F319" t="inlineStr"/>
       <c r="G319" t="inlineStr">
         <is>
           <t>This article makes a further contribution to opening the ‘black box’ of micropractices in ministry–agency relationships. We argue that the mechanisms that come into play in the course of institutionalizing agencification reforms – such as renegotiating mutual roles and rules in ministry–agency interactions – are only poorly covered in the existing literature. To adequately address the negotiated and contingent nature of de facto agency autonomy and political control, we develop an interpretive approach based on the concept of ‘boundary work’. The empirical focus is on ministry–agency interactions at the science–policy nexus in the contested policy field of food safety. By studying actors' stories about the institutionalization processes following the fundamental reorganization of the German food safety administration in the wake of the               BSE               crisis from a longitudinal perspective, we show how actors manage boundary conflicts via increasingly differentiated backstage coordination.</t>
@@ -16800,7 +16725,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>Purpose – This study investigates the relationship between buyer-supplier top management team (TMT) demographic misalignment (defined as differences in TMT composition based on background, age and gender) and environmental performance (EVP).</t>
@@ -16848,7 +16772,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>The importance of emotional labouring and performance of frontline service employees, who in their boundary-spanning positions significantly affect service-rendering organisations’ efficiency by their direct communications with customers, continues to increase. However, it is still important to ascertain an efficient understanding of the comprehensive process including behavioural mechanism and a common perception of the rewards’ impacts on motivation and creativity. Therefore, guided by self-determination theory, this study examined the mechanism and boundary conditions between emotional labour and job performance (creative and task)–specifically, taking charge has been considered as a mediator and performance-based pay as a moderator in between relationships. The authors selected a time-lagged cross-sectional design to investigate interrelations amongst study variables at two different time points and surveyed 417 team members and 186 team leaders in Pakistan’s commercial banks. Findings were consistent with the assumed conceptual framework. For instance, deep-acting affected taking charge positively, surface-acting demonstrated a positive link with task performance and taking charge partially mediated the relationships between deep-acting and performances under boundary conditions of low performance-based pay. By summing up, the study adds to the literature and recommends managerial implications with a more affluent view of nomothetic linkage among frontline employees’ emotional labor, HR practices, and the service sector.</t>
@@ -16896,7 +16819,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>As a core organizational resource, business processes are vital for organizational teams. To deal with today’s volatile business environment, organizations need to be ambidextrous in terms of process capabilities. However, little is known about how process ambidexterity, process standardization, and process agility, are enabled by information technology (IT) and related to team-level activities. To fill this gap in the literature, we conducted a field study based on 160 teams of 1081 individuals from seven companies in South Korea. Our results show that IT enables both process standardization and agility, and that a team’s process ambidexterity has a positive effect on inter-team coordination and team innovation, which in turn have a direct impact on team performance. Our findings highlight the importance of process ambidexterity by investigating the enabling role of IT and its outcomes in a team. Our results offer theoretical and practical implications from the perspective of team process ambidexterity.</t>
@@ -16944,7 +16866,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>Though improvisation has emerged as a crucial organizational competence, research wrestles with a key question – how can organizations benefit from improvisation? To advance research, I build a richer conceptualization of the role of knowledge resources – market information sources and memory types – in improvisation. I argue that as (a) internal and external sources of market information differ in speed and novelty and (b) procedural and declarative memory differ in articulation and abstractness, they shape the impact of improvisation on new product outcomes in a distinct way. A longitudinal survey of new products in the Dutch food industry uncovers that, contrary to prior thinking, improvisation increases cost efficiency when new product teams rely on internal market information and declarative memory and they minimize external market information. Though both sources of market information and low procedural memory weaken the negative impact of improvisation on market effectiveness, these conditions were not enough to make its impact positive, echoing traditional concerns with improvisation.</t>
@@ -17096,7 +17017,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>We examine leadership over-emergence, defined as instances when the level of one’s leadership emergence is higher than the level of one’s leadership effectiveness, in a sample of intact self-managing teams who worked together for a period of seven months. We draw from Gender Role Theory and Expectancy Violation Theory to examine the role of gender in predicting leadership over-emergence. Building on arguments from Gender Role Theory, we find that all else equal, men over-emerge as leaders. However, Expectancy Violation Theory suggests that women are likely to benefit from a countervailing bias. Specifically, women are attributed with higher levels of leadership emergence than men when they engage in agentic leadership behaviors—even if the level of the behaviors exhibited by men is exactly the same. Because the impact of these behaviors on leadership effectiveness is not contingent on gender, however, women who engage in more task behaviors and boundary spanning behaviors in self-managing teams also over-emerge as leaders. We discuss the implications of this study for Gender Role Theory and Expectancy Violation Theory, along with practical implications for managing the problem of leadership over-emergence in work groups.</t>
@@ -17498,7 +17418,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>Purpose – As teams are built around specialized and different knowledge, they need to regulate their knowledge boundaries to exchange their specialized knowledge with other teams and to protect the value of such specialized knowledge. However, prior studies focus primarily on boundary spanning and imply that boundaries are obstacles to sharing knowledge. To ﬁll this research gap, this study aims to indicate the importance of knowledge protection regulation, an activity that sets an adequate boundary for protecting knowledge, and investigate the factors that facilitate knowledge protection regulation and its consequences.</t>
@@ -17650,7 +17569,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>Purpose – This study investigated the influence of ambiguous customer expectations and customer demandingness, which reflect hindrance and challenge demands, on the boundary spanning behaviors (BSBs) of frontline bank employees (FBEs) through person-job fit and work engagement. It also examined the moderating effect of customer stewardship between job demands and work engagement.</t>
@@ -17750,7 +17668,6 @@
           <t>1 = Include</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>As business environments become even more competitive, project teams are required to make an effort to operate external linkages from within an organization or across organizational boundaries. Nevertheless, some members boundary-span less extensively, isolating themselves and their project teams from external environments. Our study examines why some members boundary-span more or less through the framework of group attachment theory. Data from 521 project-team members in construction and engineering industries revealed that the more individuals worry about their project team’s acceptance (group attachment anxiety), the more likely they are to perceive intergroup competition, and thus put more efforts into operating external linkages and resources to help their own teams outperform competitors. In contrast, a tendency to distrust their project teams (group attachment avoidance) generates members’ negative construal of their team’s external image, and thus fewer efforts are made at operating external linkages. Thus, project leaders and members with high group-attachment-anxiety may be best qualified for external tasks.</t>
@@ -17798,7 +17715,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>Improving performance often requires creative ideas in extreme work settings like health care. Frontline workers are promising sources of creative ideas. The authors assert that their job dissatisfaction is positively associated with creativity in health care settings because negative emotion spurs creativity when tied to engaging work and that characteristics such as shorter tenure, greater role centrality, and high boundary spanning can strengthen this relationship. The authors find supporting evidence in data on ideas generated over 18 months by health professionals in 12 clinics.</t>
@@ -18101,7 +18017,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>Boundary spanning activity Is conceived of as an intervening variable between organization structure and perceived environmental uncertainty. This is because boundary spanners operate at the skin of the organization and hence their functions are to interpret environmental conditions and relay that information to organization decision makers. Three hypotheses examining relationships between perceived environmental uncertainty, organization structure, and boundary spanning activity were investigated. In a field study comprising 12 work units (182 people) working in a health and welfare organization, positive relationships were found between all three variables. Partial relationships indicated that PEtJ does not influence the boundary spanning-structure relationship, but structure reduces the PEtJ-boundary spanning relationship to zero, and boundary spanning reduces the structurePEU relationship to zero. Thus, not only is the boundary spanning as an intervening variable supported, but results suggest that causality in the Btructure-PEU relationship may be in the direction of structure to PEU rather than current contingency notions of PEU effecting structure.</t>
@@ -18456,7 +18371,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>Purpose – This study aims to explore the mechanism of boundary-spanning search on firm’s innovation performance under environmental dynamics from the perspective of strategic knowledge integration. Design/methodology/approach – A survey was conducted among Chinese firm managers and R&amp;D personnel, resulting in the collection of 315 valid samples. Hierarchical regression analysis was mainly adopted to demonstrate the hypothesized relationships, while the Sobel test and bootstrap method were used to further validate the mediating effects.</t>
@@ -18504,7 +18418,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>This article theoretically and empirically examines the antecedents and consequences of project communication during the new financial service innovation process. The authors analyze project communication comprising both intraproject communication and extraproject communication (i.e., boundary spanners) and adopt the view that project teams within banks are primarily information-processing systems directed toward reducing innovative uncertainty. The research findings indicate that the level of complexity contributes to intraproject communication, whereas centralized project environments appear to be a barrier for communication within the project team. Curvilinear relationships (inverted U) are substantiated between project climate and intraproject communication and between formalization and boundary-spanning communication. The authors’ findings provide support for the fact that effective project communication is contingent upon the level of cross-functional cooperation and that the relationship with project success is an indirect one, mediated by the level of innovative uncertainty reduction.</t>
@@ -18552,7 +18465,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>Using a longitudinal in-depth field study at NASA, I investigate how the open, or peer-production, innovation model affects R&amp;D professionals, their work, and the locus of innovation. R&amp;D professionals are known for keeping their knowledge work within clearly defined boundaries, protecting it from individuals outside those boundaries, and rejecting meritorious innovation that is created outside disciplinary boundaries. The open innovation model challenges these boundaries and opens the knowledge work to be conducted by anyone who chooses to contribute. At NASA, the open model led to a scientific breakthrough at unprecedented speed using unusually limited resources; yet it challenged not only the knowledge-work boundaries but also the professional identity of the R&amp;D professionals. This led to divergent reactions from R&amp;D professionals, as adopting the open model required them to go through a multifaceted transformation. Only R&amp;D professionals who underwent identity refocusing work dismantled their boundaries, truly adopting the knowledge from outside and sharing their internal knowledge. Others who did not go through that identity work failed to incorporate the solutions the open model produced. Adopting open innovation without a change in R&amp;D professionals’ identity resulted in no real change in the R&amp;D process. This paper reveals how such processes unfold and illustrates the critical role of professional identity work in changing knowledge-work boundaries and shifting the locus of innovation.</t>
@@ -18803,7 +18715,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine team external learning, particularly focusing on: how leader external learning behavior affects team external learning; how team external learning inﬂuences employee creativity; and whether team internal learning is a moderator between the cross-level relationship of external learning and employee creativity in Chinese R&amp;D teams.</t>
@@ -18851,7 +18762,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
           <t>Expatriates typically perform boundary-spanning to address challenges related to functional, linguistic, and cultural variations within multinational enterprises (MNEs), which in turn influences their relationships with host-country employees. Integrating social capital and role theory perspectives, this study explores the relational dynamics between expatriates and host-country employees by developing a novel theoretical framework that examines the double-edged effects of expatriates’ boundary-spanning. We propose that expatriates’ boundary-spanning nurtures mutual trust between expatriates and hostcountry employees, further facilitating expatriates’ identification with subsidiaries and host-country employees’ identification with MNEs. On the other hand, we propose that boundary-spanning increases expatriates’ role stressors, causing expatriates’ emotional exhaustion and outgroup categorization by host-country employees. We further categorize expatriates’ boundaryspanning into three types (functional, linguistic, and cultural) and theorize about their varying effects on the cognitive and affective bases of mutual trust and on role stressors. With data from 177 expatriate–host-country coworker dyads in Chinese MNEs, our double-edged framework is generally supported. Our findings suggest that cultural boundary-spanning exhibits the strongest double-edged effect, while functional boundary-spanning shows asymmetric effects, with negative outcomes surpassing positive ones, and linguistic boundary-spanning demonstrates the weakest effect. This study offers realistic and comprehensive insights into expatriates’ boundary-spanning, particularly in expatriate–host-country employee relationships.</t>
@@ -18899,7 +18809,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr">
         <is>
           <t>Purpose – Social networking services (SNS) empower users with a robust capability to connect with others and manage their social relationships. However, as the size of users’ social networks increases, coupled with the inherent boundary-spanning technical features of SNS, users are faced with unprecedented role stresses. This, in turn, leads to maladaptive lurking decisions. This study delves into the mechanism of this technologyinduced decision-making process among SNS users.</t>
@@ -18947,7 +18856,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>In an increasingly global research landscape, it is important to identify the most prolific researchers in various institutions and their influence on the diffusion of knowledge. Knowledge diffusion within institutions is influenced by not just the status of individual researchers but also the collaborative culture that determines status. There are various methods to measure individual status, but few studies have compared them or explored the possible effects of different cultures on the status measures. In this article, we examine knowledge diffusion within science and technology‐oriented research organizations. Using social network analysis metrics to measure individual status in large‐scale coauthorship networks, we studied an individual's impact on the recombination of knowledge to produce innovation in nanotechnology. Data from the most productive and high‐impact institutions in China (Chinese Academy of Sciences), Russia (Russian Academy of Sciences), and India (Indian Institutes of Technology) were used. We found that boundary‐spanning individuals influenced knowledge diffusion in all countries. However, our results also indicate that cultural and institutional differences may influence knowledge diffusion.</t>
@@ -19099,7 +19007,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F368" t="inlineStr"/>
       <c r="G368" t="inlineStr">
         <is>
           <t>Research Summary: Chief executive officer (CEO) entrepreneurial orientation (EO) is an emerging topic within entrepreneurship research. This research offers the attention-based view (ABV), and its principles of attentional focus, situated attention, and structural distribution of attention to explain how CEO EO fosters an innovative organizational workforce. We theorize that CEO EO predicts lower-level employee innovative behavior when their top managerial attentional focus on entrepreneurship is translated into highperformance work practices, which structurally distribute their strategic attention throughout the organization and promotes a situated attentional condition for employees emphasizing innovation. Moreover, we consider (a) humanresource management (HRM) perceived importance and (b) departmental functional foci as boundary conditions. Using a multi-level and multi-source sample from 152 Chinese firms, results support our arguments.</t>
@@ -19199,7 +19106,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr">
         <is>
           <t>This study examined Hosmer's (1994) proposition that an ethical approach to management engenders stakeholder trust, which, in turn, brings about commitment and innovation from the perspectives of traditionally out-group suppliers and in-group employees, respectively. Boundary-spanning employees of the Internet-enhanced manufacturing companies participated in the study in their roles as either suppliers or employees. A sample of 54 buyer-supplier inter-organizational relationships and 54 employer-employee intra-organizational relationships were used to test the proposition.</t>
@@ -19247,11 +19153,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F371" t="inlineStr">
-        <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
-        </is>
-      </c>
+      <c r="F371" t="inlineStr"/>
       <c r="G371" t="inlineStr">
         <is>
           <t>Organizations contain multiple social foci—settings for interaction providing members with occasions for structuring their social relations. In this paper we examine how identification with particular social foci within organizations influences the propensity of advice-seeking ties to crosscut the boundaries of organizational subunits. We propose and test a theory of relationship formation based on the strength of organizational members’ identification with social foci. We expect that advice relations of organizational members identifying more strongly with local foci (organizational subunits) will be more likely to be contained within their boundaries. By contrast, we expect that advice relations of organizational members identifying more strongly with a global focus (the organization as a whole) will be more likely to crosscut the boundaries defined around local foci. We test these hypotheses on data we collected on advice-seeking relations among members of the top management team in an industrial multiunit group that comprises five distinct subsidiary companies. Results show that identification with social foci affects the formation of crosscutting network ties over and above the effect of the formal organizational boundaries that encircle the foci. More specifically, we find that organizational members who identify strongly with local foci (subsidiaries, in our case) tend to seek advice within such local foci, whereas organizational members who identify strongly with a global focus (corporate, in our case) tend to be sources of advice across the boundaries of the local foci in which they participate. Cross-boundary advice ties are less likely to occur among managers who identify strongly with their subsidiaries but weakly with the corporate group. As a consequence, identification with local foci constrains knowledge transfer relations within the boundaries of such foci. On the contrary, cross-boundary advice ties are more likely to occur among managers who identify strongly with the corporate group but weakly with their subsidiary. As a consequence, identification with a global focus activates knowledge transfer across the boundaries of local foci.</t>
@@ -19279,7 +19181,7 @@
       </c>
       <c r="P371" t="inlineStr">
         <is>
-          <t>[Code 1 &amp; Code 3] Dyadic data analysis (ERGMs on N=1,722 ties) and no individual-level correlation matrix provided.. Verbatim Evidence: [3.2. Fieldwork and Data] The results we report are based on the analysis of a network with 42 nodes. [3.2. Fieldwork and Data] We collected relational and demographic information by means of a questionnaire administered personally and individually to all the remaining 42 top managers in the group. [3.5. Empirical Model Specification and Estimation] Because ERGMs are based on dyadic observation schemes, the effective number of (nonindependent) observations is N x (N - 1), where N is the number of nodes in the network. In our case the number of observations is 1,722.</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19351,11 +19253,7 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F373" t="inlineStr">
-        <is>
-          <t>5 = Multiple reasons (specify in Notes)</t>
-        </is>
-      </c>
+      <c r="F373" t="inlineStr"/>
       <c r="G373" t="inlineStr">
         <is>
           <t>Guided by feminist politics of reinscription and intersectionality theory, this study theorized how women entrepreneurs from China, Denmark, and the United States depicted their situated struggles to resist simultaneous interlocking oppressions in everyday entrepreneuring based on 40 in-depth interviews. Participants described that they experienced               inscription               whereby multiple power asymmetries of gender, age, culture, race/ethnicity, and so on emerged and entangled to prescribe social scripts that constrained their entrepreneurial agencies. Simultaneously, participants engaged in               reinscription               to deconstruct intersectional controls and rework hegemonic scripts in situated entrepreneurial activities. They deployed three resistance strategies:               recontextualizing               their intersectionalities in different discursive contexts to legitimize and elevate their entrepreneur identities;               reformulating               their intersectionalities by invoking privileged positions to counterbalance marginalization; and               re-envisioning               by transcending their intersectional subordination to create opportunities for change. Instead of focusing on pre-existing and fixed power structures and identities in intersectional resistance-control processes, we demonstrate how intersectionalities are (re)constituted in situ through complex and fluid inscription-reinscription dynamics in women’s entrepreneurship.</t>
@@ -19383,7 +19281,7 @@
       </c>
       <c r="P373" t="inlineStr">
         <is>
-          <t>Qualitative interview study without quantitative effect sizes, investigating women entrepreneurs' resistance practices rather than boundary spanning behavior, and using a non-employee sample of independent business owners [Code 1 &amp; Code 2].. Verbatim Evidence: [Abstract] "Guided by feminist politics of reinscription and intersectionality theory, this study theorized how women entrepreneurs from China, Denmark, and the United States depicted their situated struggles to resist simultaneous interlocking oppressions in everyday entrepreneuring based on 40 in-depth interviews." [Participants] "Women from China, Denmark, and the United States were recruited if they were actively involved in setting up businesses, owned or co-owned, or currently owned-managed new businesses." [Data Collection] "Upon obtaining IRB approval and participants’ consent, in-depth semi-structured interviews ranging from 40 to 110 minutes (average=60) were conducted."</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -19507,7 +19405,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr">
         <is>
           <t>Research on the district’s role in fostering improvements affecting student learning is still in its infancy. Since the early 1990s, when school districts were often viewed as a waste of time and money (Chubb and Moe 1990), the winds have shifted, with states and districts expected to promote coherence and accountability in the loosely coupled US school system (Boyd and Crowson 1981). The articles in this issue not only expand middle-level theories concerning how these enlarged responsibilities and roles may develop but also add empirical meat to expectations in state and federal accountability policies. As advertised, the articles represent a “first installment” on a needed scholarly dialogue. Let me further the dialogue by suggesting topics for additional investigation arising from their work.</t>
@@ -19743,7 +19640,7 @@
       </c>
       <c r="P380" t="inlineStr">
         <is>
-          <t>Qualitative study lacking quantitative effect sizes (no correlation matrix). Verbatim Evidence: [Abstract] "This ethnomethodologically oriented study examines boundary arrangements in work development meetings in a university hospital, while professionals made room for a new role, a hospitalist." [Data] "The primary data applied in this study were acquired by video-recording and transcribing interactions during eight work development meetings using the transcription system introduced by Jefferson (1984) (see Table 1) to illustrate the manifested accounts in detail." [Analytical process] "In the analytical process, we drew on membership categorisation analysis (Housley and Fitzgerald, 2002; Stokoe, 2012)."</t>
+          <t xml:space="preserve">. Verbatim Evidence: </t>
         </is>
       </c>
     </row>
@@ -20226,7 +20123,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr">
         <is>
           <t>Although the use of generative artificial intelligence (AI) within organizations is becoming increasingly common, research on how to enhance employees' competitive advantage through generative AI use within organizations is very limited. Using a resource-based view model, this study investigates the relationship between generative AI use and employees' competitive advantage, as well as the moderating role of perceived organization support. From an analysis of data from 264 employees from 200 organizations, it is found that work-related generative AI use has a positive effect on employee boundary spanning, which contributes to employee competitive advantage. Secondly, work-related generative AI use also has a positive effect on employee agility, including employee resilience and employee adaptability, which further contributes to employee competitive advantage. However, work-related generative AI use has a positive effect on employee proactivity, while the effect of employee proactivity on employee competitive advantage is not significant. Thirdly, perceived organizational support can enhance the effect between employee boundary spanning and employee competitive advantage. However, it is interesting to observe that perceived organizational support enhances the effect between employee adaptability and employee competitive advantage, while weakening the effect between employee proactivity and employee competitive advantage. It does not exert a moderating effect between employee resilience and employee competitive advantage. These findings can help deepen the current understanding of the relationship between generative AI use in the organization and employee competitive advantage, and provide suggestions for business managers on how to use generative AI to improve employee competitive advantage.</t>
@@ -20274,7 +20170,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
           <t>Chronic excessive turnover among information technology (IT) professionals has been costly to firms for decades with annual turnover rates as high as 24% even among Computerworld’s “100 Best Places to Work in IT.” Prior information systems literature has identified two key factors affecting turnover: boundary-spanning roles and low promotability in one’s current firm. We draw on tournament theory, which is primarily concerned with inducing effort in employees, to decompose promotability into two distinct constructs: the likelihood of promotion and benefit from promotion, and demonstrate that each has a distinct role in affecting turnover rates. Our key result is that a job ladder motivating IT professionals with large, infrequent promotions will lead to higher turnover than a job ladder with smaller, more frequent promotions. We describe the conditions under which rearranging the job ladder creates economic value for the firm. We also offer an explanation for the observation that jobs characterized by boundary-spanning activities have higher turnover, and show that such jobs are more sensitive to the effect of likelihood of promotion on turnover. We test our hypotheses on a detailed data set covering 5,704 IT professionals over a five-year period. We confirm that likelihood of promotion has the predicted effects on turnover of IT professionals. A one standard deviation increase in likelihood of promotion decreases turnover by over 99%, consistent with our prediction. The empirical analysis also confirms the predicted effects of boundary spanning activities.</t>
@@ -20530,7 +20425,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr">
         <is>
           <t>Technology transfer’ is a misnomer; this popular phrase and the studies from which it originates often suggest passivity and inertia on the part of developing country recipient firms. This paper, which uses the technological capability building system (TCB) approach as a conceptual framework, suggests that firms in developing countries exercise constrained agency in technological acquisition processes. The evidence discussed here is taken from a study of technological capability accumulation by twenty-six firms in the telecommunication sector of four developing countries: Uganda, Ghana, Tanzania and South Africa. Important insights into technological acquisition by firms in a service sector in developing countries emerged from that study, such as the existence of specific boundary management capabilities for managing relationships with suppliers; confirmation that firms use different mechanisms for acquiring codified and tacit knowledge; and support for the view that technical change and industry features have significant effects on technology acquisition strategies and their effectiveness.</t>
@@ -20677,7 +20571,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F399" t="inlineStr"/>
       <c r="G399" t="inlineStr">
         <is>
           <t>The authors examined how networks of teams integrate their efforts to succeed collectively. They proposed that integration processes used to align efforts among multiple teams are important predictors of multiteam performance. The authors used a multiteam system (MTS) simulation to assess how both cross-team and within-team processes relate to MTS performance over multiple performance episodes that differed in terms of required interdependence levels. They found that cross-team processes predicted MTS performance beyond that accounted for by within-team processes. Further, cross-team processes were more important for MTS effectiveness when there were high cross-team interdependence demands as compared with situations in which teams could work more independently. Results are discussed in terms of extending theory and applications from teams to multiteam systems.</t>
@@ -20933,7 +20826,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr">
         <is>
           <t>Strategic alignment of project portfolios concerns the match between projects in the portfolio and the organization’s strategy. It is often considered either as a selection criterion when creating the project portfolio or as a performance indicator when assessing success. Organizations pursue optimal strategic alignment while retaining responsiveness to changes in the environment. The problem guiding this study is the need to understand how strategic alignment occurs in practice in the work of project portfolio management in the context of multiple project portfolios. We explore large firms’ practices of strategic alignment and cross-portfolio interplay in the innovation project portfolios of three industrial firms. The findings reveal social, mechanistic, and structural practices of portfolios’ strategic alignment and sharing, synergy creation, and boundary-spanning practices in cross-portfolio interplay. Strategic alignment is reported as a dynamic, continuous activity in the work of managers and personnel, with versatile practices that drive both efficiency and renewal.</t>
@@ -21055,7 +20947,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr">
         <is>
           <t>Abstract                                                                                     According to numerous studies across multiple disciplines in the social sciences, business organizations tend to develop adversarial relationships with representatives of the public interest. A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter‐organizational conflict, organizational communication and stakeholder management. Empirical results support the descriptive power of a two‐dimensional model reflecting four relational styles that participating organizations exhibited: avoidance, compliance, co‐optation and negotiation. The two dimensions that constitute the model are cooperativeness and boundary spanning. More importantly, managers who attributed power and legitimacy to public interest group stakeholders reported that their organizations were more likely to cooperate with these stakeholders. On the other hand, managers who perceived public interest groups' claims having                     urgency                     were more likely to develop communicative, boundary spanning relationships with public interest groups but these relationships were less likely to be cooperative. Because unhealthy relationships with these groups can be detrimental to an organization's long‐term prospects, managers must be careful to recognize public interest organizations as potent and legitimate potential allies.                                                                  Copyright © 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -21103,7 +20994,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
           <t>The rapid growth in the use of teams and multiple team membership has led more organizations to structure work around dynamic teams, characterized by short lifespans and fluid membership boundaries. This approach to organizing work makes it difficult for teams to work efficiently or to support the learning and growth of members. Given the importance of productivity and learning, we ask how these processes can be supported in dynamic teams. We do so in a randomized controlled field experiment conducted with 91 teams in a teaching hospital, a context in which physician trainees must learn while providing patient care in dynamic teams of care providers. We randomly assigned physician teams, or “core” teams, to launch their work with an intervention focused either on internal coordination among the core team members or on external coordination with a changing cast of external contributors such as nurses and specialists. We measured resulting levels of internal and external coordination over teams’ week-long lifespans and observed that external coordination was associated with improved team efficiency, whereas internal coordination was associated with improved individual learning. Post hoc exploratory analysis suggested that individual learning was highest when teams achieved high levels of both internal and external coordination, and it was positively correlated with improvement in the team’s patients’ average length of hospital stay. We discuss the implications of the demonstrated causal effects of team launches, along with our exploratory findings, for the management of dynamic teams and the opportunities to mitigate potential trade-offs between learning and productivity.</t>
@@ -21302,7 +21192,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
           <t>This study explores how pharmacists legitimise the expansion of their clinical work and considers its impact on pharmacists’ professional identity work. In the context of pharmacy in the English NHS, there has been an ongoing policy shift towards pharmacists moving away from ‘medicines supply’ to patient-facing, clinical work since the 1950s. Pharmacists are continuously engaging in ‘identity work’ and ‘boundary work’ to reflect the expansion of their work, which has led to the argument that pharmacists lack a clear professional identity. Drawing insights from linguistics and specifically Van Leeuwen's ‘grammar of legitimation’, this study explains how the Pharmacy Integration Fund, a nationally funded learning programme, provides the discursive strategies for pharmacists to legitimise their identity work as clinicians.</t>
@@ -21402,7 +21291,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
           <t>This article explores service learning via the lens of activity theory. Through this lens, it is identified as a form of ‘boundary work’ in higher education, with educators identified as ‘boundary workers’. Drawing on the data from a recent study, this paper analyses service learning as an often contradictory and tension filled practice. The ‘expanded community’ and ‘dual but interrelated object’ in the service learning activity system result in many tensions for students and community members alike. This in turn poses significant challenges for boundary workers, and ultimately for the university. The paper concludes by arguing that in order to encourage and value service learning, we need to acknowledge the (new and different) knowledge, values and skills required for playing the role of boundary worker in (boundary) practices such as this.</t>
@@ -21554,7 +21442,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>The beneﬁts boundary spanners offer organizations by bridging information silos are well documented. However, informational boundary spanning also implies crossing organizational territories, as employees seek advice from others outside their supervisors’ control. Applying a territoriality theory lens, we develop new insights about when and why supervisors may view their subordinates’ informational boundaryspanning activities unfavorably and attempt to undermine boundary spanners. We argue that undermining results from supervisors perceiving the boundary spanning of their employees as weakening their control over their organizational territory. We further argue that subordinates who seek advice across organizational boundaries without also seeking advice from their supervisor are more likely to be seen by their supervisors as having negative intentions when engaging in boundary spanning, which increases their risk of being undermined. We ﬁnd support for our arguments in a ﬁeld study and in a scenario experiment. Our results provide new insights into the potentially negative reactions from supervisors toward employees who engage in boundary spanning. We discuss how these insights contribute to the boundary spanning literature, to territoriality theory, and to the leadership literature.</t>
@@ -21602,7 +21489,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>Intergroup knowledge integration, that is the acquisition, processing, and utilization of knowledge across group boundaries, is a critical source of competitive advantage in modern organizations. Prior research has highlighted the important role of boundary spanning knowledge exchange for intergroup knowledge integration, neglecting, however, the question of what makes individual boundary spanners more effective in fostering intergroup knowledge integration. Integrating boundary spanning literature with theories of group information processing, we hypothesize that the effect of individual boundary spanning ties on intergroup knowledge integration depends on the boundary spanners’ levels of metaknowledge, i.e., knowledge of who knows what in their respective groups, and proactivity. We find general support for our predictions in a study of 457 engineering consultants nested in 22 interdependent business units within an organization. Additional criterion analyses confirm the material importance of intergroup knowledge integration for group performance. Our findings have implications for literatures on intergroup effectiveness, team cognition, and proactivity.</t>
@@ -21806,7 +21692,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>This dissertation investigates factors that influence efforts by lower-level employees to initiate organizational change and innovation from the bottom up. Specifically, I attempt to reconcile competing theories regarding the effects of structural and social integration on individual innovation efforts. One theoretical view posits that integration provides information, ideas, and motivation necessary for innovation. An alternative view is that integration constrains individuals and routines, and thereby hinders innovation efforts. Drawing on both theoretical perspectives, I predict the effects of distinct types of structural integration (eg, centralization, cross-unit integration, boundary spanning) and social integration determinants (eg, geographic dispersion, decision process involvement, workplace network size) on the likelihood of individual innovation efforts among lower-level employees. I also consider the effects of interactions of social and structural integration with individual characteristics (ie, personality, and experience) on innovation efforts. I test these predictions using survey data collected from interns and supervisors in the context of MBA and undergraduate internships. Analyses demonstrate that several aspects of structural integration do influence the levels of individual innovation efforts. For example, centralization and boundary spanning levels of the work unit have inverse U-shaped relationships with the level of innovation effort. These findings suggest that for certain types of innovation, structural integration can constrain efforts at the extremes (very high or low) and facilitate efforts at modest levels of integration. Predicted social integration effects are largely non-significant, suggesting the need for further consideration and alternative empirical tests of such effects. Nevertheless, the structural integration findings reaffirm the need to bring together both theoretical perspectives (ie, the view that integration fosters innovation efforts, and the alternative view that isolation and independence are necessary for innovation). By empirically demonstrating that distinct types of integration have unique, yet theoretically consistent effects on several different classes of individual innovation efforts (both process and strategy related), this study contributes to efforts to reconcile these competing theories. Additionally, this research enhances our understanding of a class of little-studied behaviors that play a potentially important role in autonomous strategic change and organizational learning.</t>
@@ -22625,7 +22510,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
           <t>Efforts to understand how an organization monitors its environment often focus on boundary spanning individuals or units. The concept of boundary spanning was one introduced by Thompson in 1967 in a book that has since become the classic statement of the open systems model of organizations. This dissertation uses Thompson's model of boundary spanning units to generate hypotheses which are then tested in a sample of personnel/human resource departments. A theory driven argument is presented which suggests that the P/HR function in an organization meets Thompson's criteria for a boundary spanning unit. An historical review of the roots of personnel administration suggests that its emergence as a field fits Thompson's conceptualization of the development of boundary spanning units. This dissertation suggests that from its origin through this most recent period of transition, the development of the personnel function (now generally referred to as human resource management) has been due to a recognition by organizations that an increasing complexity and concomitant uncertainty in the human resource arena caused by such factors as labor unions, the expansion of due process in organizations, and intervention by government agencies, needed to be addressed.</t>
@@ -22673,7 +22557,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to know that how group resources (internal and external) and the relationship quality among group members relate to group performance. Design/methodology/approach – Given the normative nature of group performance, the study is carried out in a contrived environment. Participants were 204 master of business administration students who were allocated to 51 study groups. Data were collected in three waves and from two different sources, i.e., students and instructors. Data analysis was carried out by employing regression analysis and the bootstrapping procedure, i.e., PROCESS.</t>
@@ -22721,7 +22604,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
           <t>Purpose – Literature on small and medium enterprises (SMEs) has so far produced limited evidence on how these firms pursue their organizational flexibility with information and communication technology (ICT) and ad hoc work practices. The purpose of this paper is to contribute to the extant literature by focusing on how SMEs use flexible work practices that provide latitude with respect to when employees work, where they work and via which communication medium. Specifically, the authors analyze how such practices are related to the conditions that SMEs face in reference to their competitive environment and their patterns of ICT usage.</t>
@@ -22873,7 +22755,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
           <t>This dissertation presents a critical perspective on the development of American journalism education by combining historical methods and a sociological framework. That framework is boundary work, and it serves as the organizing principle of this project. As such, this study privileges boundary work paradigms–participation, practices, and professionalism–over a chronological narrative. It uncovers the interrelationships and power dynamics that structured the development of journalism instruction in higher education. Moreover, it heeds the call for journalism historians to engage with other disciplines and develop more theoretical approaches to understanding the past.</t>
@@ -22921,7 +22802,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
           <t>Research Summary:                              We study antecedents of innovation performance for the subsidiaries of multinational enterprises (MNEs) using the microfoundations approach. Based on the upper echelon perspective, we argue that managers’ characteristics, such as prior MNE work experience and industry experience, affect subsidiary innovation. We tested our hypotheses on a sample of 228 MNE subsidiaries from 11 countries. Results indicate that managers’ industry experience serves as an external boundary‐spanning capability and, therefore, it has a greater effect on autonomous subsidiaries. In contrast, managers’ prior MNE work experience functions as an internal boundary‐spanning capability and, therefore, it has a smaller effect on subsidiaries that are less autonomous or engage in R&amp;D.                                                          Managerial Summary:                              The success of an MNE now increasingly depends on its ability to generate knowledge anywhere in the world. Thus, the ability of foreign subsidiaries to generate innovation plays an increasingly important role in enhancing the performance of MNEs. In this regard, what factors determine the innovativeness of foreign subsidiaries is an important question for managers. Our study suggests that the international experience of the top management team (TMT) of a subsidiary and its CEO’s industry experience positively affect subsidiary innovation. Furthermore, the TMT’s international experience has a greater effect on the innovativeness of subsidiaries that remain dependent on their headquarters for knowledge transfer. In contrast, the CEO’s industry experience has a greater effect on the innovativeness of autonomous subsidiaries.</t>
@@ -23021,7 +22901,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
           <t>In this dissertation I first develop a theoretical framework that explores different
@@ -23088,7 +22967,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
           <t>Purpose – This study recognizes service as the majority contributor to global and US gross domestic product and the importance of innovation speed to service innovation. Generating innovative products and services at a faster rate generates advantages for business-to-business (B2B) service organizations in keeping up with and moving ahead of rivals. This study aims to introduce the concept of capacity for social exchange (CSE) in buyer–supplier relationships, which reflects the degree to which individuals possess competencies that enable the exchange of information, and this study also explores how CSE affects knowledge sharing and innovation speed within a supply chain organization.</t>
@@ -23240,7 +23118,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F449" t="inlineStr"/>
       <c r="G449" t="inlineStr">
         <is>
           <t>Background The health-care environment requires hospital units to coordinate efforts autonomously across their boundaries and to manage relationships with other professionals, units and departments. Boundary spanning has become increasingly important for ﬁrst-line nurse managers as unit gatekeepers; however, the available measures are limited. Method The 30-item instrument was developed from a literature review. Survey participants were 4918 nurses at 231 hospital units. Statistical analyses of construct validity and internal consistency were performed. Furthermore, the correlation between nurses’ scores on the Nurse Managers Boundary Spanning Scale and nurses’ evaluations of their managers were examined. Results Three factors and 26 items were derived from factor analyses: connecting and mediating, informing and feedback utilisation, and resource acquisition. Cronbach’s subscales’ alpha coefﬁcients were above 0.9. Correlation analysis indicated that the Nurse Managers Boundary Spanning Scale score correlated with nurses’ positive perceptions of their managers. Conclusion This study demonstrates tentative support for the validity and reliability of the Nurse Managers Boundary Spanning Scale. Although further study is needed, the Nurse Managers Boundary Spanning Scale shows possibilities as a new measurement of nursing leadership. Implications This study underscores measures to build on nurse managers’ roles by building on the limited research available.</t>
@@ -23288,7 +23165,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F450" t="inlineStr"/>
       <c r="G450" t="inlineStr">
         <is>
           <t>This study examines how cultural performance orientation moderates the influence of human resource management (HRM) controls on boundary-spanning employees' behavioural strategies and satisfaction. Based on primary data obtained from 1049 salespeople in six countries (France, Ireland, Italy, Spain, United Kingdom, and the United States of America) and secondary data on cultural performance orientation, multilevel regression analyses show that national culture has a strong effect on the way boundary-spanning employees allocate their effort in response to HRM control. In particular, our results suggest that the more behaviour controls are used with boundary-spanning employees, the less attention they pay to customers and the more emphasis they place on their supervisors and non-selling tasks. Specifically, cultural performance orientation is shown to moderate significantly those relationships. Furthermore, results indicate that cultural performance orientation heightens boundary-spanning employees' job satisfaction resulting from behaviour control. Preliminary explanations for the differing impact of HRM control efficiency across cultures can be proposed.</t>
@@ -23526,7 +23402,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F454" t="inlineStr"/>
       <c r="G454" t="inlineStr">
         <is>
           <t>Committed customers are proﬁtable to an organization for the long term. Customer commitment forms when a customer’s expectation is satisﬁed and the customer realizes fair value from his/her relationship with the organization. From an organization’s perspective, this value reﬂects customer equity, but from a customer’s perspective, it represents the customer’s perceived value of the relationship. In order to manage such a relationship successfully, it is necessary to support diverse customer information – such as of-the-customer, for-the-customer, and by-the-customer information. A customer information system (CIS) plays the role of boundary spanning that manages and distributes customer information. But the gap between marketing and IT strategy is a barrier in implementing a successful CIS. The CIS, which includes the database, communication channel, and decision model for relationship management, should be designed to facilitate the two-way customer relationship exchanges. This paper develops a framework of dynamic customer relationship management, suggests the information technology strategy to support the framework, and illustrates the applicability of such framework and strategy through a real business case.</t>
@@ -23574,7 +23449,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F455" t="inlineStr"/>
       <c r="G455" t="inlineStr">
         <is>
           <t>Abstract             How do boundary spanners, through processes of temporal sensemaking, use established and newly forming relationships to create value in science‐based SMEs? In addressing this question, we examine the creation of social capital arising from the activities that boundary spanners use in establishing ‘ties that bind’ people together. We show how effective boundary‐spanning activities are able to promote collaborations across scientific and related disciplines, supporting knowledge generation and innovation. Sensemaking is central to this process. We illustrate how retrospective sensemaking draws on knowledge, skills and experiences, often triggered through historical connections and personal contacts, whilst prospective sensemaking often arose in the search for new customers and in the ongoing assessment of future potential markets. We reveal how combining individual and collective boundary spanning with a continual movement between the backward glance (retrospective) and more future‐oriented (prospective) sensemaking was particularly effective in generating new understandings and opportunities. We use our findings to present an inductive model of value creation that frames the dynamic interplay between individual and collective boundary‐spanning activities and temporal sensemaking in the generation of social capital that acts as a knowledge resource for identifying and evaluating ideas for innovation and future pathways to value creation.</t>
@@ -23622,7 +23496,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F456" t="inlineStr"/>
       <c r="G456" t="inlineStr">
         <is>
           <t>In this editorial for our special issue on interorganizational collaboration (IOC), we position collaborative action in the context of the concurrent global crises that necessitate the bridging of interests, positions, competencies, and resources. We unpack the notion of IOC in terms of its conditions, phases, practices, and dynamics, and provide an overview of how the contributing authors support such understanding of cross-boundary collaboration. Through their action-oriented approaches to research and learning, they show a promising interplay of insight and impact. We underline their search for impact and aim to reinforce the potential of IOC not just to be successful, but also highly meaningful to address grand challenges. We therefore take a normative stance and describe how the intertwined notions of justice, resilience, and thriving can serve as a compass to legitimize, organize, facilitate, assess, and study IOC as an important pathway for the co-creation of a better world.</t>
@@ -25387,7 +25260,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr">
         <is>
           <t>Purpose – This study seeks to address a gap in the literature by investigating product management (PM) as a set of ﬁrm-level activities, distinct from the behaviours embedded within the market orientation (MO) construct. This research establishes PM as a set of organizational activities, which lie at the boundary between the traditional functions of the ﬁrm.</t>
@@ -25535,7 +25407,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F493" t="inlineStr"/>
       <c r="G493" t="inlineStr">
         <is>
           <t>In this paper, we present an empirical study of 1,156 open source virtual reality (VR) projects from Unity List. Our study shows that the number of open source VR software projects are steadily growing, and some large projects attracting many developers are emerging. The most popular topic of VR software is still games. We also found that VR developers often face misscommit of automatically generated ﬁles.</t>
@@ -25635,7 +25506,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>Abstract             In this study, we analyse the discursive strategies of professionalization used by psychology in Spain during its professionalization phase in the health sector in the early twenty-first century. Our primary focus is the conflict with political regulators and other healthcare professions after the Ley de Ordenación de Profesiones Sanitarias (Healthcare Professions Act) came into effect, since this Act calls into question the extent to which psychology can be viewed as health care. We use discourse analysis to determine the discursive structure of the conflict, which has an interprofessional dimension, as well as the professionalization and social closure strategies of psychology within the framework of professional relationships (boundary work). We argue that understanding this conflict requires viewing it as part of the European and international regulation context of healthcare professions. Highlighted in the analysis is the emergence of two psychology discourses divided into four modes of enunciation (professionalizing, cultural, scientific, and political–economic). Among other aspects, the conclusions focus on the dual interprofessional and intraprofessional nature of the conflict and evidence of a dual closure in psychology. The latter’s professionalization strategies in the sector occasionally resemble those employed by nursing, although at other times they are similar to those followed by some paramedical professions.</t>
@@ -25735,7 +25605,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -25783,7 +25652,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
           <t>Process Management Programs (PMPs) rely heavily on the standardization of activities to improve organizational efficiency and reliability. Standardization, however, can lead to rigidity and inertia, which may eventually inhibit exploration and innovation. While scholars have provided cognitive and routine-based arguments to cope with this dilemma, the fact that standardization is a social process that requires collaboration between individuals has been overlooked. In this paper, we propose that standardization can improve a team’s social capital and thereby facilitate the activities that enable exploration. Specifically, we hypothesize that standardization relates positively to external communication, psychological safety, and the perception of support for innovation in operational teams. These three social capital attributes mediate the relationship between standardization and exploration. We tested this multilevel mediation model by analysing 431 members of 62 operational teams in a large multinational mining company that had recently implemented a Process Management Program (Lean Management). Our multilevel mediation results confirmed that standardisation promoted exploration by enhancing the teams’ social capital. For robustness we tested our model with a second survey of 450 workers of different companies and obtained similar results. Therefore, we propose that the productivity dilemma can be balanced by improving operational teams’ social capital.</t>
@@ -25935,7 +25803,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr">
         <is>
           <t>A model of cross-functional project groups was developed and hypotheses were tested in a study of 93 research and new product development groups from four companies. The results showed that functional diversity had indirect effects through external communication on one-year-later measures. Technical quality and schedule and budget performance improved, but group cohesiveness diminished. Functional diversity also had an indirect effect through job stress on group cohesiveness, which was again reduced. Implications for the development of conceptual models of cross-functional groups and their effective management are discussed.</t>
@@ -26141,7 +26008,6 @@
           <t>0 = Exclude</t>
         </is>
       </c>
-      <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr">
         <is>
           <t>The human resource management (HRM) function has realized a considerable increase in power, influence, and reputation, but it has not been examined from the perspective of organizational boundary spanning. Because boundary spanning's function of information control provides a source of power, it is helpful in explaining HRM's growing influence in US organizations. However,